<commit_message>
up to level 14, can't get scroll glitch to work, investigation is needed
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD57DB06-27F0-477E-B226-AD10749EBAFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B33206E4-434A-45A8-B63E-96C2AF256808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50865" yWindow="3795" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,6 +21,7 @@
     <sheet name="Takanawa Comparison" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="285">
   <si>
     <t>Place</t>
   </si>
@@ -878,6 +879,18 @@
   </si>
   <si>
     <t>12 1st move</t>
+  </si>
+  <si>
+    <t>12 end</t>
+  </si>
+  <si>
+    <t>13 1st move</t>
+  </si>
+  <si>
+    <t>13 end</t>
+  </si>
+  <si>
+    <t>14 1st move</t>
   </si>
 </sst>
 </file>
@@ -887,12 +900,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1247,121 +1267,122 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1812,7 +1833,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="45" t="s">
+      <c r="A9" s="37" t="s">
         <v>243</v>
       </c>
       <c r="B9" s="7">
@@ -1830,7 +1851,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A10" s="45" t="s">
+      <c r="A10" s="37" t="s">
         <v>245</v>
       </c>
       <c r="B10" s="7">
@@ -1860,7 +1881,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="45" t="s">
+      <c r="A12" s="37" t="s">
         <v>246</v>
       </c>
       <c r="B12" s="7">
@@ -1875,13 +1896,13 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13" s="45" t="s">
+      <c r="A13" s="37" t="s">
         <v>247</v>
       </c>
       <c r="B13" s="7">
         <v>2059</v>
       </c>
-      <c r="C13" s="45">
+      <c r="C13" s="37">
         <v>2943</v>
       </c>
       <c r="D13" s="3">
@@ -1890,7 +1911,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" s="45" t="s">
+      <c r="A14" s="37" t="s">
         <v>127</v>
       </c>
       <c r="B14" s="7">
@@ -1905,7 +1926,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="45" t="s">
+      <c r="A15" s="37" t="s">
         <v>249</v>
       </c>
       <c r="B15" s="7">
@@ -1920,7 +1941,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A16" s="45" t="s">
+      <c r="A16" s="37" t="s">
         <v>248</v>
       </c>
       <c r="B16" s="7">
@@ -1935,7 +1956,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A17" s="45" t="s">
+      <c r="A17" s="37" t="s">
         <v>250</v>
       </c>
       <c r="B17" s="7">
@@ -1950,7 +1971,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" s="45" t="s">
+      <c r="A18" s="37" t="s">
         <v>251</v>
       </c>
       <c r="B18" s="7">
@@ -1965,7 +1986,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A19" s="45" t="s">
+      <c r="A19" s="37" t="s">
         <v>252</v>
       </c>
       <c r="B19" s="7">
@@ -1980,7 +2001,7 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A20" s="45" t="s">
+      <c r="A20" s="37" t="s">
         <v>127</v>
       </c>
       <c r="B20" s="7">
@@ -1995,7 +2016,7 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A21" s="45" t="s">
+      <c r="A21" s="37" t="s">
         <v>253</v>
       </c>
       <c r="B21" s="7">
@@ -2010,7 +2031,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A22" s="45" t="s">
+      <c r="A22" s="37" t="s">
         <v>254</v>
       </c>
       <c r="B22" s="7">
@@ -2025,7 +2046,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A23" s="45" t="s">
+      <c r="A23" s="37" t="s">
         <v>255</v>
       </c>
       <c r="B23" s="7">
@@ -2040,7 +2061,7 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A24" s="45" t="s">
+      <c r="A24" s="37" t="s">
         <v>256</v>
       </c>
       <c r="B24" s="7">
@@ -2055,7 +2076,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A25" s="45" t="s">
+      <c r="A25" s="37" t="s">
         <v>257</v>
       </c>
       <c r="B25" s="7">
@@ -2070,7 +2091,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A26" s="45" t="s">
+      <c r="A26" s="37" t="s">
         <v>258</v>
       </c>
       <c r="B26" s="7">
@@ -2085,7 +2106,7 @@
       </c>
     </row>
     <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="45" t="s">
+      <c r="A27" s="37" t="s">
         <v>127</v>
       </c>
       <c r="B27" s="7">
@@ -2100,7 +2121,7 @@
       </c>
     </row>
     <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="45" t="s">
+      <c r="A28" s="37" t="s">
         <v>261</v>
       </c>
       <c r="B28" s="7">
@@ -2115,7 +2136,7 @@
       </c>
     </row>
     <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="45" t="s">
+      <c r="A29" s="37" t="s">
         <v>260</v>
       </c>
       <c r="B29" s="7">
@@ -2130,7 +2151,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="45" t="s">
+      <c r="A30" s="37" t="s">
         <v>262</v>
       </c>
       <c r="B30" s="7">
@@ -2148,7 +2169,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A31" s="45" t="s">
+      <c r="A31" s="37" t="s">
         <v>259</v>
       </c>
       <c r="B31" s="7">
@@ -2163,7 +2184,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A32" s="45" t="s">
+      <c r="A32" s="37" t="s">
         <v>264</v>
       </c>
       <c r="B32" s="7">
@@ -2178,7 +2199,7 @@
       </c>
     </row>
     <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A33" s="45" t="s">
+      <c r="A33" s="37" t="s">
         <v>261</v>
       </c>
       <c r="B33" s="7">
@@ -2193,7 +2214,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A34" s="45" t="s">
+      <c r="A34" s="37" t="s">
         <v>265</v>
       </c>
       <c r="B34" s="7">
@@ -2208,7 +2229,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A35" s="45" t="s">
+      <c r="A35" s="37" t="s">
         <v>266</v>
       </c>
       <c r="B35" s="33">
@@ -2223,7 +2244,7 @@
       </c>
     </row>
     <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A36" s="45" t="s">
+      <c r="A36" s="37" t="s">
         <v>267</v>
       </c>
       <c r="B36" s="7">
@@ -2238,7 +2259,7 @@
       </c>
     </row>
     <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A37" s="45" t="s">
+      <c r="A37" s="37" t="s">
         <v>268</v>
       </c>
       <c r="B37" s="7">
@@ -2253,13 +2274,13 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A38" s="45" t="s">
+      <c r="A38" s="37" t="s">
         <v>269</v>
       </c>
       <c r="B38" s="7">
         <v>7531</v>
       </c>
-      <c r="C38" s="45">
+      <c r="C38" s="37">
         <v>10236</v>
       </c>
       <c r="D38" s="3">
@@ -2268,7 +2289,7 @@
       </c>
     </row>
     <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A39" s="45" t="s">
+      <c r="A39" s="37" t="s">
         <v>270</v>
       </c>
       <c r="B39" s="7">
@@ -2283,7 +2304,7 @@
       </c>
     </row>
     <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A40" s="45" t="s">
+      <c r="A40" s="37" t="s">
         <v>272</v>
       </c>
       <c r="B40" s="7">
@@ -2298,7 +2319,7 @@
       </c>
     </row>
     <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A41" s="45" t="s">
+      <c r="A41" s="37" t="s">
         <v>273</v>
       </c>
       <c r="B41" s="7">
@@ -2313,7 +2334,7 @@
       </c>
     </row>
     <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A42" s="45" t="s">
+      <c r="A42" s="37" t="s">
         <v>271</v>
       </c>
       <c r="B42" s="7">
@@ -2328,7 +2349,7 @@
       </c>
     </row>
     <row r="43" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A43" s="45" t="s">
+      <c r="A43" s="37" t="s">
         <v>274</v>
       </c>
       <c r="B43" s="7">
@@ -2344,7 +2365,7 @@
       <c r="E43" s="7"/>
     </row>
     <row r="44" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A44" s="45" t="s">
+      <c r="A44" s="37" t="s">
         <v>275</v>
       </c>
       <c r="B44" s="7">
@@ -2360,7 +2381,7 @@
       <c r="E44" s="7"/>
     </row>
     <row r="45" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A45" s="45" t="s">
+      <c r="A45" s="37" t="s">
         <v>276</v>
       </c>
       <c r="B45" s="7">
@@ -2375,7 +2396,7 @@
       </c>
     </row>
     <row r="46" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A46" s="45" t="s">
+      <c r="A46" s="37" t="s">
         <v>277</v>
       </c>
       <c r="B46" s="7">
@@ -2390,7 +2411,7 @@
       </c>
     </row>
     <row r="47" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A47" s="45" t="s">
+      <c r="A47" s="37" t="s">
         <v>279</v>
       </c>
       <c r="B47" s="7">
@@ -2405,7 +2426,7 @@
       </c>
     </row>
     <row r="48" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A48" s="45" t="s">
+      <c r="A48" s="37" t="s">
         <v>278</v>
       </c>
       <c r="B48" s="7">
@@ -2420,7 +2441,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A49" s="45" t="s">
+      <c r="A49" s="37" t="s">
         <v>280</v>
       </c>
       <c r="B49" s="7">
@@ -2435,39 +2456,63 @@
       </c>
     </row>
     <row r="50" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A50" s="7"/>
-      <c r="B50" s="8"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="3" t="str">
+      <c r="A50" s="46" t="s">
+        <v>281</v>
+      </c>
+      <c r="B50" s="8">
+        <v>10810</v>
+      </c>
+      <c r="C50" s="8">
+        <v>14421</v>
+      </c>
+      <c r="D50" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>3611</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A51" s="7"/>
-      <c r="B51" s="33"/>
-      <c r="C51" s="33"/>
-      <c r="D51" s="3" t="str">
+      <c r="A51" s="46" t="s">
+        <v>282</v>
+      </c>
+      <c r="B51" s="33">
+        <v>11165</v>
+      </c>
+      <c r="C51" s="33">
+        <v>15078</v>
+      </c>
+      <c r="D51" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>3913</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A52" s="7"/>
-      <c r="B52" s="7"/>
-      <c r="C52" s="7"/>
-      <c r="D52" s="3" t="str">
+      <c r="A52" s="46" t="s">
+        <v>283</v>
+      </c>
+      <c r="B52" s="7">
+        <v>11729</v>
+      </c>
+      <c r="C52" s="7">
+        <v>15652</v>
+      </c>
+      <c r="D52" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>3923</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A53" s="7"/>
-      <c r="B53" s="7"/>
-      <c r="C53" s="7"/>
-      <c r="D53" s="3" t="str">
+      <c r="A53" s="46" t="s">
+        <v>284</v>
+      </c>
+      <c r="B53" s="7">
+        <v>12384</v>
+      </c>
+      <c r="C53" s="7">
+        <v>16307</v>
+      </c>
+      <c r="D53" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>3923</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -13978,7 +14023,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="18" type="noConversion"/>
+  <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -14008,10 +14053,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="37" t="s">
+      <c r="K1" s="38" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="38"/>
+      <c r="L1" s="39"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -15863,13 +15908,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="39" t="s">
+      <c r="H53" s="40" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="40"/>
-      <c r="J53" s="40"/>
-      <c r="K53" s="40"/>
-      <c r="L53" s="41"/>
+      <c r="I53" s="41"/>
+      <c r="J53" s="41"/>
+      <c r="K53" s="41"/>
+      <c r="L53" s="42"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -15891,11 +15936,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="42"/>
-      <c r="I54" s="43"/>
-      <c r="J54" s="43"/>
-      <c r="K54" s="43"/>
-      <c r="L54" s="44"/>
+      <c r="H54" s="43"/>
+      <c r="I54" s="44"/>
+      <c r="J54" s="44"/>
+      <c r="K54" s="44"/>
+      <c r="L54" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner 14 done - 4240 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B33206E4-434A-45A8-B63E-96C2AF256808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A029EB2B-7AD9-467B-81F3-2E3F43034936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50865" yWindow="3795" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V6" sheetId="7" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <sheet name="Takanawa Comparison" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="288">
   <si>
     <t>Place</t>
   </si>
@@ -891,6 +890,15 @@
   </si>
   <si>
     <t>14 1st move</t>
+  </si>
+  <si>
+    <t>14 end</t>
+  </si>
+  <si>
+    <t>15 1st move</t>
+  </si>
+  <si>
+    <t>Gold = 20</t>
   </si>
 </sst>
 </file>
@@ -900,12 +908,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1267,122 +1282,123 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2456,7 +2472,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A50" s="46" t="s">
+      <c r="A50" s="38" t="s">
         <v>281</v>
       </c>
       <c r="B50" s="8">
@@ -2471,7 +2487,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A51" s="46" t="s">
+      <c r="A51" s="38" t="s">
         <v>282</v>
       </c>
       <c r="B51" s="33">
@@ -2486,7 +2502,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A52" s="46" t="s">
+      <c r="A52" s="38" t="s">
         <v>283</v>
       </c>
       <c r="B52" s="7">
@@ -2501,45 +2517,63 @@
       </c>
     </row>
     <row r="53" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A53" s="46" t="s">
+      <c r="A53" s="38" t="s">
         <v>284</v>
       </c>
       <c r="B53" s="7">
-        <v>12384</v>
+        <v>12383</v>
       </c>
       <c r="C53" s="7">
         <v>16307</v>
       </c>
       <c r="D53" s="3">
         <f t="shared" si="2"/>
-        <v>3923</v>
+        <v>3924</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A54" s="7"/>
-      <c r="B54" s="7"/>
-      <c r="C54" s="7"/>
-      <c r="D54" s="3" t="str">
+      <c r="A54" s="47" t="s">
+        <v>285</v>
+      </c>
+      <c r="B54" s="7">
+        <v>12889</v>
+      </c>
+      <c r="C54" s="7">
+        <v>16822</v>
+      </c>
+      <c r="D54" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>3933</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A55" s="7"/>
-      <c r="B55" s="7"/>
-      <c r="C55" s="7"/>
-      <c r="D55" s="3" t="str">
+      <c r="A55" s="47" t="s">
+        <v>286</v>
+      </c>
+      <c r="B55" s="7">
+        <v>13239</v>
+      </c>
+      <c r="C55" s="7">
+        <v>17480</v>
+      </c>
+      <c r="D55" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>4241</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A56" s="7"/>
-      <c r="B56" s="7"/>
-      <c r="C56" s="7"/>
-      <c r="D56" s="3" t="str">
+      <c r="A56" s="47" t="s">
+        <v>287</v>
+      </c>
+      <c r="B56" s="7">
+        <v>13254</v>
+      </c>
+      <c r="C56" s="7">
+        <v>17494</v>
+      </c>
+      <c r="D56" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>4240</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -14023,7 +14057,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="19" type="noConversion"/>
+  <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -14053,10 +14087,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="38" t="s">
+      <c r="K1" s="39" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="39"/>
+      <c r="L1" s="40"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -15908,13 +15942,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="40" t="s">
+      <c r="H53" s="41" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="41"/>
-      <c r="J53" s="41"/>
-      <c r="K53" s="41"/>
-      <c r="L53" s="42"/>
+      <c r="I53" s="42"/>
+      <c r="J53" s="42"/>
+      <c r="K53" s="42"/>
+      <c r="L53" s="43"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -15936,11 +15970,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="43"/>
-      <c r="I54" s="44"/>
-      <c r="J54" s="44"/>
-      <c r="K54" s="44"/>
-      <c r="L54" s="45"/>
+      <c r="H54" s="44"/>
+      <c r="I54" s="45"/>
+      <c r="J54" s="45"/>
+      <c r="K54" s="45"/>
+      <c r="L54" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - up to level 17
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A029EB2B-7AD9-467B-81F3-2E3F43034936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C23700-2EEF-4A2A-A926-5B5CC4F62DC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="297">
   <si>
     <t>Place</t>
   </si>
@@ -899,6 +899,33 @@
   </si>
   <si>
     <t>Gold = 20</t>
+  </si>
+  <si>
+    <t>15 end</t>
+  </si>
+  <si>
+    <t>Gold = 15</t>
+  </si>
+  <si>
+    <t>Gold = 10</t>
+  </si>
+  <si>
+    <t>E gets gold in air</t>
+  </si>
+  <si>
+    <t>16 gold = 10</t>
+  </si>
+  <si>
+    <t>gold = 6</t>
+  </si>
+  <si>
+    <t>16 end</t>
+  </si>
+  <si>
+    <t>17 1st move</t>
+  </si>
+  <si>
+    <t>move right</t>
   </si>
 </sst>
 </file>
@@ -1722,7 +1749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E299"/>
+  <dimension ref="A1:E300"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -2407,7 +2434,7 @@
         <v>12106</v>
       </c>
       <c r="D45" s="3">
-        <f t="shared" ref="D45:D77" si="2">IF(C45&lt;&gt;"",IF(B45&lt;&gt;"",C45-B45,"-"), "-")</f>
+        <f t="shared" ref="D45:D78" si="2">IF(C45&lt;&gt;"",IF(B45&lt;&gt;"",C45-B45,"-"), "-")</f>
         <v>2989</v>
       </c>
     </row>
@@ -2577,102 +2604,161 @@
       </c>
     </row>
     <row r="57" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A57" s="7"/>
-      <c r="B57" s="7"/>
-      <c r="C57" s="7"/>
-      <c r="D57" s="3" t="str">
+      <c r="A57" s="47" t="s">
+        <v>289</v>
+      </c>
+      <c r="B57" s="7">
+        <v>13480</v>
+      </c>
+      <c r="C57" s="7">
+        <v>17723</v>
+      </c>
+      <c r="D57" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>4243</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A58" s="7"/>
+      <c r="A58" s="47" t="s">
+        <v>290</v>
+      </c>
       <c r="B58" s="7"/>
-      <c r="C58" s="7"/>
+      <c r="C58" s="7">
+        <v>17893</v>
+      </c>
       <c r="D58" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A59" s="7"/>
-      <c r="B59" s="7"/>
-      <c r="C59" s="7"/>
-      <c r="D59" s="3" t="str">
+      <c r="A59" s="47" t="s">
+        <v>291</v>
+      </c>
+      <c r="B59" s="7">
+        <v>13801</v>
+      </c>
+      <c r="C59" s="7">
+        <v>18042</v>
+      </c>
+      <c r="D59" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>4241</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A60" s="7"/>
-      <c r="B60" s="7"/>
-      <c r="C60" s="7"/>
-      <c r="D60" s="3" t="str">
+      <c r="A60" s="47" t="s">
+        <v>288</v>
+      </c>
+      <c r="B60" s="7">
+        <v>13960</v>
+      </c>
+      <c r="C60" s="7">
+        <v>18210</v>
+      </c>
+      <c r="D60" s="3">
+        <f t="shared" ref="D60" si="3">IF(C60&lt;&gt;"",IF(B60&lt;&gt;"",C60-B60,"-"), "-")</f>
+        <v>4250</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A61" s="47" t="s">
+        <v>292</v>
+      </c>
+      <c r="B61" s="7">
+        <v>14356</v>
+      </c>
+      <c r="C61" s="7">
+        <v>18890</v>
+      </c>
+      <c r="D61" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A61" s="7"/>
-      <c r="B61" s="7"/>
-      <c r="C61" s="7"/>
-      <c r="D61" s="3" t="str">
+        <v>4534</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A62" s="47" t="s">
+        <v>293</v>
+      </c>
+      <c r="B62" s="7">
+        <v>14494</v>
+      </c>
+      <c r="C62" s="7">
+        <v>19029</v>
+      </c>
+      <c r="D62" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A62" s="7"/>
-      <c r="B62" s="7"/>
-      <c r="C62" s="7"/>
-      <c r="D62" s="3" t="str">
+        <v>4535</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A63" s="47" t="s">
+        <v>296</v>
+      </c>
+      <c r="B63" s="7">
+        <v>14532</v>
+      </c>
+      <c r="C63" s="7"/>
+      <c r="D63" s="3"/>
+    </row>
+    <row r="64" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A64" s="47" t="s">
+        <v>150</v>
+      </c>
+      <c r="B64" s="7">
+        <v>14572</v>
+      </c>
+      <c r="C64" s="7">
+        <v>19107</v>
+      </c>
+      <c r="D64" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A63" s="7"/>
-      <c r="B63" s="7"/>
-      <c r="C63" s="7"/>
-      <c r="D63" s="3" t="str">
+        <v>4535</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A65" s="47" t="s">
+        <v>250</v>
+      </c>
+      <c r="B65" s="7">
+        <v>14614</v>
+      </c>
+      <c r="C65" s="7">
+        <v>19149</v>
+      </c>
+      <c r="D65" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A64" s="7"/>
-      <c r="B64" s="7"/>
-      <c r="C64" s="7"/>
-      <c r="D64" s="3" t="str">
+        <v>4535</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A66" s="47" t="s">
+        <v>294</v>
+      </c>
+      <c r="B66" s="7">
+        <v>14669</v>
+      </c>
+      <c r="C66" s="7">
+        <v>19214</v>
+      </c>
+      <c r="D66" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A65" s="7"/>
-      <c r="B65" s="7"/>
-      <c r="C65" s="7"/>
-      <c r="D65" s="3" t="str">
+        <v>4545</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A67" s="47" t="s">
+        <v>295</v>
+      </c>
+      <c r="B67" s="7">
+        <v>15031</v>
+      </c>
+      <c r="C67" s="7">
+        <v>19868</v>
+      </c>
+      <c r="D67" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A66" s="7"/>
-      <c r="B66" s="7"/>
-      <c r="C66" s="7"/>
-      <c r="D66" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A67" s="7"/>
-      <c r="B67" s="7"/>
-      <c r="C67" s="7"/>
-      <c r="D67" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
+        <v>4837</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2730,7 +2816,7 @@
       </c>
     </row>
     <row r="74" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A74" s="34"/>
+      <c r="A74" s="7"/>
       <c r="B74" s="7"/>
       <c r="C74" s="7"/>
       <c r="D74" s="3" t="str">
@@ -2757,7 +2843,7 @@
       </c>
     </row>
     <row r="77" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A77" s="7"/>
+      <c r="A77" s="34"/>
       <c r="B77" s="7"/>
       <c r="C77" s="7"/>
       <c r="D77" s="3" t="str">
@@ -2770,43 +2856,43 @@
       <c r="B78" s="7"/>
       <c r="C78" s="7"/>
       <c r="D78" s="3" t="str">
-        <f t="shared" ref="D78:D84" si="3">IF(C78&lt;&gt;"",IF(B78&lt;&gt;"",C78-B78,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
     <row r="79" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A79" s="7"/>
-      <c r="B79" s="9"/>
-      <c r="C79" s="9"/>
+      <c r="B79" s="7"/>
+      <c r="C79" s="7"/>
       <c r="D79" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="D79:D85" si="4">IF(C79&lt;&gt;"",IF(B79&lt;&gt;"",C79-B79,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="80" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A80" s="7"/>
-      <c r="B80" s="7"/>
-      <c r="C80" s="7"/>
+      <c r="B80" s="9"/>
+      <c r="C80" s="9"/>
       <c r="D80" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A81" s="7"/>
-      <c r="B81" s="9"/>
-      <c r="C81" s="9"/>
+      <c r="B81" s="7"/>
+      <c r="C81" s="7"/>
       <c r="D81" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="82" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A82" s="7"/>
-      <c r="B82" s="7"/>
-      <c r="C82" s="7"/>
+      <c r="B82" s="9"/>
+      <c r="C82" s="9"/>
       <c r="D82" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
@@ -2815,16 +2901,16 @@
       <c r="B83" s="7"/>
       <c r="C83" s="7"/>
       <c r="D83" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A84" s="5"/>
+      <c r="A84" s="7"/>
       <c r="B84" s="7"/>
       <c r="C84" s="7"/>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
@@ -2833,7 +2919,7 @@
       <c r="B85" s="7"/>
       <c r="C85" s="7"/>
       <c r="D85" s="3" t="str">
-        <f t="shared" ref="D85:D153" si="4">IF(C85&lt;&gt;"",IF(B85&lt;&gt;"",C85-B85,"-"), "-")</f>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
@@ -2842,7 +2928,7 @@
       <c r="B86" s="7"/>
       <c r="C86" s="7"/>
       <c r="D86" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="D86:D154" si="5">IF(C86&lt;&gt;"",IF(B86&lt;&gt;"",C86-B86,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2851,7 +2937,7 @@
       <c r="B87" s="7"/>
       <c r="C87" s="7"/>
       <c r="D87" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -2860,7 +2946,7 @@
       <c r="B88" s="7"/>
       <c r="C88" s="7"/>
       <c r="D88" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -2869,7 +2955,7 @@
       <c r="B89" s="7"/>
       <c r="C89" s="7"/>
       <c r="D89" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -2878,16 +2964,16 @@
       <c r="B90" s="7"/>
       <c r="C90" s="7"/>
       <c r="D90" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A91" s="7"/>
+      <c r="A91" s="5"/>
       <c r="B91" s="7"/>
       <c r="C91" s="7"/>
       <c r="D91" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -2896,34 +2982,34 @@
       <c r="B92" s="7"/>
       <c r="C92" s="7"/>
       <c r="D92" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="93" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A93" s="34"/>
+      <c r="A93" s="7"/>
       <c r="B93" s="7"/>
       <c r="C93" s="7"/>
       <c r="D93" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A94" s="7"/>
+      <c r="A94" s="34"/>
       <c r="B94" s="7"/>
       <c r="C94" s="7"/>
       <c r="D94" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="95" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A95" s="5"/>
+      <c r="A95" s="7"/>
       <c r="B95" s="7"/>
       <c r="C95" s="7"/>
       <c r="D95" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -2932,7 +3018,7 @@
       <c r="B96" s="7"/>
       <c r="C96" s="7"/>
       <c r="D96" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -2941,7 +3027,7 @@
       <c r="B97" s="7"/>
       <c r="C97" s="7"/>
       <c r="D97" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -2950,7 +3036,7 @@
       <c r="B98" s="7"/>
       <c r="C98" s="7"/>
       <c r="D98" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -2959,7 +3045,7 @@
       <c r="B99" s="7"/>
       <c r="C99" s="7"/>
       <c r="D99" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -2968,7 +3054,7 @@
       <c r="B100" s="7"/>
       <c r="C100" s="7"/>
       <c r="D100" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -2977,7 +3063,7 @@
       <c r="B101" s="7"/>
       <c r="C101" s="7"/>
       <c r="D101" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -2986,7 +3072,7 @@
       <c r="B102" s="7"/>
       <c r="C102" s="7"/>
       <c r="D102" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -2995,7 +3081,7 @@
       <c r="B103" s="7"/>
       <c r="C103" s="7"/>
       <c r="D103" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3004,7 +3090,7 @@
       <c r="B104" s="7"/>
       <c r="C104" s="7"/>
       <c r="D104" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3013,7 +3099,7 @@
       <c r="B105" s="7"/>
       <c r="C105" s="7"/>
       <c r="D105" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3022,7 +3108,7 @@
       <c r="B106" s="7"/>
       <c r="C106" s="7"/>
       <c r="D106" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3031,7 +3117,7 @@
       <c r="B107" s="7"/>
       <c r="C107" s="7"/>
       <c r="D107" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3040,7 +3126,7 @@
       <c r="B108" s="7"/>
       <c r="C108" s="7"/>
       <c r="D108" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3049,7 +3135,7 @@
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
       <c r="D109" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3058,7 +3144,7 @@
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
       <c r="D110" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3067,43 +3153,43 @@
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
       <c r="D111" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="112" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A112" s="5"/>
-      <c r="B112" s="10"/>
-      <c r="C112" s="10"/>
+      <c r="B112" s="7"/>
+      <c r="C112" s="7"/>
       <c r="D112" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="113" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A113" s="5"/>
-      <c r="B113" s="7"/>
-      <c r="C113" s="7"/>
+      <c r="B113" s="10"/>
+      <c r="C113" s="10"/>
       <c r="D113" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="114" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A114" s="35"/>
+      <c r="A114" s="5"/>
       <c r="B114" s="7"/>
       <c r="C114" s="7"/>
       <c r="D114" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="115" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A115" s="5"/>
+      <c r="A115" s="35"/>
       <c r="B115" s="7"/>
       <c r="C115" s="7"/>
       <c r="D115" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3112,7 +3198,7 @@
       <c r="B116" s="7"/>
       <c r="C116" s="7"/>
       <c r="D116" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3121,7 +3207,7 @@
       <c r="B117" s="7"/>
       <c r="C117" s="7"/>
       <c r="D117" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3130,7 +3216,7 @@
       <c r="B118" s="7"/>
       <c r="C118" s="7"/>
       <c r="D118" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3138,7 +3224,10 @@
       <c r="A119" s="5"/>
       <c r="B119" s="7"/>
       <c r="C119" s="7"/>
-      <c r="D119" s="3"/>
+      <c r="D119" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="120" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A120" s="5"/>
@@ -3153,24 +3242,21 @@
       <c r="D121" s="3"/>
     </row>
     <row r="122" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A122" s="5" t="s">
+      <c r="A122" s="5"/>
+      <c r="B122" s="7"/>
+      <c r="C122" s="7"/>
+      <c r="D122" s="3"/>
+    </row>
+    <row r="123" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A123" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B122" s="7"/>
-      <c r="C122" s="7">
+      <c r="B123" s="7"/>
+      <c r="C123" s="7">
         <v>63782</v>
       </c>
-      <c r="D122" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A123" s="7"/>
-      <c r="B123" s="7"/>
-      <c r="C123" s="7"/>
       <c r="D123" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3179,7 +3265,7 @@
       <c r="B124" s="7"/>
       <c r="C124" s="7"/>
       <c r="D124" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3188,7 +3274,7 @@
       <c r="B125" s="7"/>
       <c r="C125" s="7"/>
       <c r="D125" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3197,7 +3283,7 @@
       <c r="B126" s="7"/>
       <c r="C126" s="7"/>
       <c r="D126" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3206,7 +3292,7 @@
       <c r="B127" s="7"/>
       <c r="C127" s="7"/>
       <c r="D127" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3215,7 +3301,7 @@
       <c r="B128" s="7"/>
       <c r="C128" s="7"/>
       <c r="D128" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3224,7 +3310,7 @@
       <c r="B129" s="7"/>
       <c r="C129" s="7"/>
       <c r="D129" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3233,7 +3319,7 @@
       <c r="B130" s="7"/>
       <c r="C130" s="7"/>
       <c r="D130" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3242,7 +3328,7 @@
       <c r="B131" s="7"/>
       <c r="C131" s="7"/>
       <c r="D131" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3251,7 +3337,7 @@
       <c r="B132" s="7"/>
       <c r="C132" s="7"/>
       <c r="D132" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3260,7 +3346,7 @@
       <c r="B133" s="7"/>
       <c r="C133" s="7"/>
       <c r="D133" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3269,7 +3355,7 @@
       <c r="B134" s="7"/>
       <c r="C134" s="7"/>
       <c r="D134" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3278,7 +3364,7 @@
       <c r="B135" s="7"/>
       <c r="C135" s="7"/>
       <c r="D135" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3287,7 +3373,7 @@
       <c r="B136" s="7"/>
       <c r="C136" s="7"/>
       <c r="D136" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3296,7 +3382,7 @@
       <c r="B137" s="7"/>
       <c r="C137" s="7"/>
       <c r="D137" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3305,7 +3391,7 @@
       <c r="B138" s="7"/>
       <c r="C138" s="7"/>
       <c r="D138" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3314,7 +3400,7 @@
       <c r="B139" s="7"/>
       <c r="C139" s="7"/>
       <c r="D139" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3323,7 +3409,7 @@
       <c r="B140" s="7"/>
       <c r="C140" s="7"/>
       <c r="D140" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3332,7 +3418,7 @@
       <c r="B141" s="7"/>
       <c r="C141" s="7"/>
       <c r="D141" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3341,7 +3427,7 @@
       <c r="B142" s="7"/>
       <c r="C142" s="7"/>
       <c r="D142" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3350,7 +3436,7 @@
       <c r="B143" s="7"/>
       <c r="C143" s="7"/>
       <c r="D143" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3359,7 +3445,7 @@
       <c r="B144" s="7"/>
       <c r="C144" s="7"/>
       <c r="D144" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3368,7 +3454,7 @@
       <c r="B145" s="7"/>
       <c r="C145" s="7"/>
       <c r="D145" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3377,7 +3463,7 @@
       <c r="B146" s="7"/>
       <c r="C146" s="7"/>
       <c r="D146" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3386,7 +3472,7 @@
       <c r="B147" s="7"/>
       <c r="C147" s="7"/>
       <c r="D147" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3395,7 +3481,7 @@
       <c r="B148" s="7"/>
       <c r="C148" s="7"/>
       <c r="D148" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3404,7 +3490,7 @@
       <c r="B149" s="7"/>
       <c r="C149" s="7"/>
       <c r="D149" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3413,7 +3499,7 @@
       <c r="B150" s="7"/>
       <c r="C150" s="7"/>
       <c r="D150" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3422,7 +3508,7 @@
       <c r="B151" s="7"/>
       <c r="C151" s="7"/>
       <c r="D151" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3431,7 +3517,7 @@
       <c r="B152" s="7"/>
       <c r="C152" s="7"/>
       <c r="D152" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3440,7 +3526,7 @@
       <c r="B153" s="7"/>
       <c r="C153" s="7"/>
       <c r="D153" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3449,7 +3535,7 @@
       <c r="B154" s="7"/>
       <c r="C154" s="7"/>
       <c r="D154" s="3" t="str">
-        <f t="shared" ref="D154:D158" si="5">IF(C154&lt;&gt;"",IF(B154&lt;&gt;"",C154-B154,"-"), "-")</f>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3458,7 +3544,7 @@
       <c r="B155" s="7"/>
       <c r="C155" s="7"/>
       <c r="D155" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="D155:D159" si="6">IF(C155&lt;&gt;"",IF(B155&lt;&gt;"",C155-B155,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3467,7 +3553,7 @@
       <c r="B156" s="7"/>
       <c r="C156" s="7"/>
       <c r="D156" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>-</v>
       </c>
     </row>
@@ -3476,7 +3562,7 @@
       <c r="B157" s="7"/>
       <c r="C157" s="7"/>
       <c r="D157" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>-</v>
       </c>
     </row>
@@ -3485,7 +3571,7 @@
       <c r="B158" s="7"/>
       <c r="C158" s="7"/>
       <c r="D158" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>-</v>
       </c>
     </row>
@@ -3494,7 +3580,7 @@
       <c r="B159" s="7"/>
       <c r="C159" s="7"/>
       <c r="D159" s="3" t="str">
-        <f t="shared" ref="D159:D160" si="6">IF(C159&lt;&gt;"",IF(B159&lt;&gt;"",B159-C159,"-"), "-")</f>
+        <f t="shared" si="6"/>
         <v>-</v>
       </c>
     </row>
@@ -3503,73 +3589,78 @@
       <c r="B160" s="7"/>
       <c r="C160" s="7"/>
       <c r="D160" s="3" t="str">
-        <f t="shared" si="6"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="161" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" ref="D160:D161" si="7">IF(C160&lt;&gt;"",IF(B160&lt;&gt;"",B160-C160,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A161" s="7"/>
       <c r="B161" s="7"/>
       <c r="C161" s="7"/>
-    </row>
-    <row r="162" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D161" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A162" s="7"/>
       <c r="B162" s="7"/>
       <c r="C162" s="7"/>
     </row>
-    <row r="163" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A163" s="7"/>
       <c r="B163" s="7"/>
       <c r="C163" s="7"/>
     </row>
-    <row r="164" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B164" s="7"/>
       <c r="C164" s="7"/>
     </row>
-    <row r="165" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B165" s="7"/>
       <c r="C165" s="7"/>
     </row>
-    <row r="166" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B166" s="7"/>
       <c r="C166" s="7"/>
     </row>
-    <row r="167" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B167" s="7"/>
       <c r="C167" s="7"/>
     </row>
-    <row r="168" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B168" s="7"/>
       <c r="C168" s="7"/>
     </row>
-    <row r="169" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B169" s="7"/>
       <c r="C169" s="7"/>
     </row>
-    <row r="170" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B170" s="7"/>
       <c r="C170" s="7"/>
     </row>
-    <row r="171" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B171" s="7"/>
       <c r="C171" s="7"/>
     </row>
-    <row r="172" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B172" s="7"/>
       <c r="C172" s="7"/>
     </row>
-    <row r="173" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B173" s="7"/>
       <c r="C173" s="7"/>
     </row>
-    <row r="174" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B174" s="7"/>
       <c r="C174" s="7"/>
     </row>
-    <row r="175" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B175" s="7"/>
       <c r="C175" s="7"/>
     </row>
-    <row r="176" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B176" s="7"/>
       <c r="C176" s="7"/>
     </row>
@@ -4064,6 +4155,10 @@
     <row r="299" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B299" s="7"/>
       <c r="C299" s="7"/>
+    </row>
+    <row r="300" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B300" s="7"/>
+      <c r="C300" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lv 18 done, 5508 frames ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C23700-2EEF-4A2A-A926-5B5CC4F62DC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A07853F7-E41D-4825-B1C6-879842AB8269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="305">
   <si>
     <t>Place</t>
   </si>
@@ -926,6 +926,30 @@
   </si>
   <si>
     <t>move right</t>
+  </si>
+  <si>
+    <t>17 end</t>
+  </si>
+  <si>
+    <t>leave ladder</t>
+  </si>
+  <si>
+    <t>18 1st move</t>
+  </si>
+  <si>
+    <t>dig 2nd cycle</t>
+  </si>
+  <si>
+    <t>18 end</t>
+  </si>
+  <si>
+    <t>gold = 3</t>
+  </si>
+  <si>
+    <t>earliest fall</t>
+  </si>
+  <si>
+    <t>19 1st move</t>
   </si>
 </sst>
 </file>
@@ -935,12 +959,26 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1309,123 +1347,125 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1749,7 +1789,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E300"/>
+  <dimension ref="A1:E305"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -2434,7 +2474,7 @@
         <v>12106</v>
       </c>
       <c r="D45" s="3">
-        <f t="shared" ref="D45:D78" si="2">IF(C45&lt;&gt;"",IF(B45&lt;&gt;"",C45-B45,"-"), "-")</f>
+        <f t="shared" ref="D45:D83" si="2">IF(C45&lt;&gt;"",IF(B45&lt;&gt;"",C45-B45,"-"), "-")</f>
         <v>2989</v>
       </c>
     </row>
@@ -2559,7 +2599,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A54" s="47" t="s">
+      <c r="A54" s="39" t="s">
         <v>285</v>
       </c>
       <c r="B54" s="7">
@@ -2574,7 +2614,7 @@
       </c>
     </row>
     <row r="55" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A55" s="47" t="s">
+      <c r="A55" s="39" t="s">
         <v>286</v>
       </c>
       <c r="B55" s="7">
@@ -2589,7 +2629,7 @@
       </c>
     </row>
     <row r="56" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A56" s="47" t="s">
+      <c r="A56" s="39" t="s">
         <v>287</v>
       </c>
       <c r="B56" s="7">
@@ -2604,7 +2644,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A57" s="47" t="s">
+      <c r="A57" s="39" t="s">
         <v>289</v>
       </c>
       <c r="B57" s="7">
@@ -2619,7 +2659,7 @@
       </c>
     </row>
     <row r="58" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A58" s="47" t="s">
+      <c r="A58" s="39" t="s">
         <v>290</v>
       </c>
       <c r="B58" s="7"/>
@@ -2632,7 +2672,7 @@
       </c>
     </row>
     <row r="59" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A59" s="47" t="s">
+      <c r="A59" s="39" t="s">
         <v>291</v>
       </c>
       <c r="B59" s="7">
@@ -2647,7 +2687,7 @@
       </c>
     </row>
     <row r="60" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A60" s="47" t="s">
+      <c r="A60" s="39" t="s">
         <v>288</v>
       </c>
       <c r="B60" s="7">
@@ -2662,7 +2702,7 @@
       </c>
     </row>
     <row r="61" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A61" s="47" t="s">
+      <c r="A61" s="39" t="s">
         <v>292</v>
       </c>
       <c r="B61" s="7">
@@ -2677,7 +2717,7 @@
       </c>
     </row>
     <row r="62" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A62" s="47" t="s">
+      <c r="A62" s="39" t="s">
         <v>293</v>
       </c>
       <c r="B62" s="7">
@@ -2692,7 +2732,7 @@
       </c>
     </row>
     <row r="63" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A63" s="47" t="s">
+      <c r="A63" s="39" t="s">
         <v>296</v>
       </c>
       <c r="B63" s="7">
@@ -2702,7 +2742,7 @@
       <c r="D63" s="3"/>
     </row>
     <row r="64" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A64" s="47" t="s">
+      <c r="A64" s="39" t="s">
         <v>150</v>
       </c>
       <c r="B64" s="7">
@@ -2717,7 +2757,7 @@
       </c>
     </row>
     <row r="65" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A65" s="47" t="s">
+      <c r="A65" s="39" t="s">
         <v>250</v>
       </c>
       <c r="B65" s="7">
@@ -2732,7 +2772,7 @@
       </c>
     </row>
     <row r="66" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A66" s="47" t="s">
+      <c r="A66" s="39" t="s">
         <v>294</v>
       </c>
       <c r="B66" s="7">
@@ -2747,7 +2787,7 @@
       </c>
     </row>
     <row r="67" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A67" s="47" t="s">
+      <c r="A67" s="39" t="s">
         <v>295</v>
       </c>
       <c r="B67" s="7">
@@ -2762,138 +2802,228 @@
       </c>
     </row>
     <row r="68" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A68" s="7"/>
-      <c r="B68" s="7"/>
-      <c r="C68" s="7"/>
-      <c r="D68" s="3" t="str">
+      <c r="A68" s="40" t="s">
+        <v>265</v>
+      </c>
+      <c r="B68" s="7">
+        <v>15051</v>
+      </c>
+      <c r="C68" s="7">
+        <v>19888</v>
+      </c>
+      <c r="D68" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>4837</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A69" s="7"/>
-      <c r="B69" s="7"/>
-      <c r="C69" s="7"/>
-      <c r="D69" s="3" t="str">
+      <c r="A69" s="40" t="s">
+        <v>279</v>
+      </c>
+      <c r="B69" s="7">
+        <v>15196</v>
+      </c>
+      <c r="C69" s="7">
+        <v>20031</v>
+      </c>
+      <c r="D69" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>4835</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A70" s="7"/>
-      <c r="B70" s="7"/>
-      <c r="C70" s="7"/>
-      <c r="D70" s="3" t="str">
+      <c r="A70" s="40" t="s">
+        <v>265</v>
+      </c>
+      <c r="B70" s="7">
+        <v>15467</v>
+      </c>
+      <c r="C70" s="7">
+        <v>20304</v>
+      </c>
+      <c r="D70" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>4837</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A71" s="7"/>
-      <c r="B71" s="7"/>
-      <c r="C71" s="7"/>
-      <c r="D71" s="3" t="str">
+      <c r="A71" s="40" t="s">
+        <v>298</v>
+      </c>
+      <c r="B71" s="7">
+        <v>15503</v>
+      </c>
+      <c r="C71" s="7">
+        <v>20337</v>
+      </c>
+      <c r="D71" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>4834</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A72" s="7"/>
-      <c r="B72" s="7"/>
-      <c r="C72" s="7"/>
-      <c r="D72" s="3" t="str">
+      <c r="A72" s="40" t="s">
+        <v>297</v>
+      </c>
+      <c r="B72" s="7">
+        <v>15844</v>
+      </c>
+      <c r="C72" s="7">
+        <v>20766</v>
+      </c>
+      <c r="D72" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>4922</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A73" s="7"/>
-      <c r="B73" s="7"/>
-      <c r="C73" s="7"/>
-      <c r="D73" s="3" t="str">
+      <c r="A73" s="40" t="s">
+        <v>299</v>
+      </c>
+      <c r="B73" s="7">
+        <v>16202</v>
+      </c>
+      <c r="C73" s="7">
+        <v>21388</v>
+      </c>
+      <c r="D73" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>5186</v>
       </c>
     </row>
     <row r="74" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A74" s="7"/>
-      <c r="B74" s="7"/>
-      <c r="C74" s="7"/>
-      <c r="D74" s="3" t="str">
+      <c r="A74" s="40" t="s">
+        <v>265</v>
+      </c>
+      <c r="B74" s="7">
+        <v>16215</v>
+      </c>
+      <c r="C74" s="7">
+        <v>21400</v>
+      </c>
+      <c r="D74" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>5185</v>
       </c>
     </row>
     <row r="75" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A75" s="34"/>
-      <c r="B75" s="7"/>
-      <c r="C75" s="7"/>
-      <c r="D75" s="3" t="str">
+      <c r="A75" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="B75" s="7">
+        <v>16317</v>
+      </c>
+      <c r="C75" s="7">
+        <v>21505</v>
+      </c>
+      <c r="D75" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>5188</v>
       </c>
     </row>
     <row r="76" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A76" s="34"/>
-      <c r="B76" s="7"/>
-      <c r="C76" s="7"/>
-      <c r="D76" s="3" t="str">
+      <c r="A76" s="40" t="s">
+        <v>300</v>
+      </c>
+      <c r="B76" s="7">
+        <v>16664</v>
+      </c>
+      <c r="C76" s="7">
+        <v>21855</v>
+      </c>
+      <c r="D76" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>5191</v>
       </c>
     </row>
     <row r="77" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A77" s="34"/>
-      <c r="B77" s="7"/>
-      <c r="C77" s="7"/>
-      <c r="D77" s="3" t="str">
+      <c r="A77" s="49" t="s">
+        <v>303</v>
+      </c>
+      <c r="B77" s="7">
+        <v>16745</v>
+      </c>
+      <c r="C77" s="7">
+        <v>21937</v>
+      </c>
+      <c r="D77" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>5192</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A78" s="7"/>
-      <c r="B78" s="7"/>
-      <c r="C78" s="7"/>
-      <c r="D78" s="3" t="str">
+      <c r="A78" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="B78" s="7">
+        <v>16848</v>
+      </c>
+      <c r="C78" s="7">
+        <v>22034</v>
+      </c>
+      <c r="D78" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>5186</v>
       </c>
     </row>
     <row r="79" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A79" s="7"/>
-      <c r="B79" s="7"/>
-      <c r="C79" s="7"/>
-      <c r="D79" s="3" t="str">
-        <f t="shared" ref="D79:D85" si="4">IF(C79&lt;&gt;"",IF(B79&lt;&gt;"",C79-B79,"-"), "-")</f>
-        <v>-</v>
+      <c r="A79" s="40" t="s">
+        <v>302</v>
+      </c>
+      <c r="B79" s="7">
+        <v>16976</v>
+      </c>
+      <c r="C79" s="7">
+        <v>22158</v>
+      </c>
+      <c r="D79" s="3">
+        <f t="shared" si="2"/>
+        <v>5182</v>
       </c>
     </row>
     <row r="80" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A80" s="7"/>
-      <c r="B80" s="9"/>
-      <c r="C80" s="9"/>
-      <c r="D80" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
+      <c r="A80" s="40" t="s">
+        <v>248</v>
+      </c>
+      <c r="B80" s="7">
+        <v>16999</v>
+      </c>
+      <c r="C80" s="7">
+        <v>22190</v>
+      </c>
+      <c r="D80" s="3">
+        <f t="shared" si="2"/>
+        <v>5191</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A81" s="7"/>
-      <c r="B81" s="7"/>
-      <c r="C81" s="7"/>
-      <c r="D81" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
+      <c r="A81" s="40" t="s">
+        <v>301</v>
+      </c>
+      <c r="B81" s="40">
+        <v>17133</v>
+      </c>
+      <c r="C81" s="7">
+        <v>22325</v>
+      </c>
+      <c r="D81" s="3">
+        <f t="shared" si="2"/>
+        <v>5192</v>
       </c>
     </row>
     <row r="82" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A82" s="7"/>
-      <c r="B82" s="9"/>
-      <c r="C82" s="9"/>
-      <c r="D82" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
+      <c r="A82" s="49" t="s">
+        <v>304</v>
+      </c>
+      <c r="B82" s="7">
+        <v>17487</v>
+      </c>
+      <c r="C82" s="7">
+        <v>22995</v>
+      </c>
+      <c r="D82" s="3">
+        <f t="shared" si="2"/>
+        <v>5508</v>
       </c>
     </row>
     <row r="83" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -2901,7 +3031,7 @@
       <c r="B83" s="7"/>
       <c r="C83" s="7"/>
       <c r="D83" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -2910,52 +3040,52 @@
       <c r="B84" s="7"/>
       <c r="C84" s="7"/>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="D84:D90" si="4">IF(C84&lt;&gt;"",IF(B84&lt;&gt;"",C84-B84,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A85" s="5"/>
-      <c r="B85" s="7"/>
-      <c r="C85" s="7"/>
+      <c r="A85" s="7"/>
+      <c r="B85" s="9"/>
+      <c r="C85" s="9"/>
       <c r="D85" s="3" t="str">
         <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A86" s="5"/>
+      <c r="A86" s="7"/>
       <c r="B86" s="7"/>
       <c r="C86" s="7"/>
       <c r="D86" s="3" t="str">
-        <f t="shared" ref="D86:D154" si="5">IF(C86&lt;&gt;"",IF(B86&lt;&gt;"",C86-B86,"-"), "-")</f>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="87" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A87" s="5"/>
-      <c r="B87" s="7"/>
-      <c r="C87" s="7"/>
+      <c r="A87" s="7"/>
+      <c r="B87" s="9"/>
+      <c r="C87" s="9"/>
       <c r="D87" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A88" s="5"/>
+      <c r="A88" s="7"/>
       <c r="B88" s="7"/>
       <c r="C88" s="7"/>
       <c r="D88" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="89" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A89" s="5"/>
+      <c r="A89" s="7"/>
       <c r="B89" s="7"/>
       <c r="C89" s="7"/>
       <c r="D89" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
@@ -2964,7 +3094,7 @@
       <c r="B90" s="7"/>
       <c r="C90" s="7"/>
       <c r="D90" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
@@ -2973,12 +3103,12 @@
       <c r="B91" s="7"/>
       <c r="C91" s="7"/>
       <c r="D91" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="D91:D159" si="5">IF(C91&lt;&gt;"",IF(B91&lt;&gt;"",C91-B91,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A92" s="7"/>
+      <c r="A92" s="5"/>
       <c r="B92" s="7"/>
       <c r="C92" s="7"/>
       <c r="D92" s="3" t="str">
@@ -2987,7 +3117,7 @@
       </c>
     </row>
     <row r="93" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A93" s="7"/>
+      <c r="A93" s="5"/>
       <c r="B93" s="7"/>
       <c r="C93" s="7"/>
       <c r="D93" s="3" t="str">
@@ -2996,7 +3126,7 @@
       </c>
     </row>
     <row r="94" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A94" s="34"/>
+      <c r="A94" s="5"/>
       <c r="B94" s="7"/>
       <c r="C94" s="7"/>
       <c r="D94" s="3" t="str">
@@ -3005,7 +3135,7 @@
       </c>
     </row>
     <row r="95" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A95" s="7"/>
+      <c r="A95" s="5"/>
       <c r="B95" s="7"/>
       <c r="C95" s="7"/>
       <c r="D95" s="3" t="str">
@@ -3023,7 +3153,7 @@
       </c>
     </row>
     <row r="97" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A97" s="5"/>
+      <c r="A97" s="7"/>
       <c r="B97" s="7"/>
       <c r="C97" s="7"/>
       <c r="D97" s="3" t="str">
@@ -3032,7 +3162,7 @@
       </c>
     </row>
     <row r="98" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A98" s="5"/>
+      <c r="A98" s="7"/>
       <c r="B98" s="7"/>
       <c r="C98" s="7"/>
       <c r="D98" s="3" t="str">
@@ -3041,7 +3171,7 @@
       </c>
     </row>
     <row r="99" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A99" s="5"/>
+      <c r="A99" s="34"/>
       <c r="B99" s="7"/>
       <c r="C99" s="7"/>
       <c r="D99" s="3" t="str">
@@ -3050,7 +3180,7 @@
       </c>
     </row>
     <row r="100" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A100" s="5"/>
+      <c r="A100" s="7"/>
       <c r="B100" s="7"/>
       <c r="C100" s="7"/>
       <c r="D100" s="3" t="str">
@@ -3168,8 +3298,8 @@
     </row>
     <row r="113" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A113" s="5"/>
-      <c r="B113" s="10"/>
-      <c r="C113" s="10"/>
+      <c r="B113" s="7"/>
+      <c r="C113" s="7"/>
       <c r="D113" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -3185,7 +3315,7 @@
       </c>
     </row>
     <row r="115" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A115" s="35"/>
+      <c r="A115" s="5"/>
       <c r="B115" s="7"/>
       <c r="C115" s="7"/>
       <c r="D115" s="3" t="str">
@@ -3213,8 +3343,8 @@
     </row>
     <row r="118" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A118" s="5"/>
-      <c r="B118" s="7"/>
-      <c r="C118" s="7"/>
+      <c r="B118" s="10"/>
+      <c r="C118" s="10"/>
       <c r="D118" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -3230,38 +3360,43 @@
       </c>
     </row>
     <row r="120" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A120" s="5"/>
+      <c r="A120" s="35"/>
       <c r="B120" s="7"/>
       <c r="C120" s="7"/>
-      <c r="D120" s="3"/>
+      <c r="D120" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="121" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A121" s="5"/>
       <c r="B121" s="7"/>
       <c r="C121" s="7"/>
-      <c r="D121" s="3"/>
+      <c r="D121" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="122" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A122" s="5"/>
       <c r="B122" s="7"/>
       <c r="C122" s="7"/>
-      <c r="D122" s="3"/>
+      <c r="D122" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="123" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A123" s="5" t="s">
-        <v>26</v>
-      </c>
+      <c r="A123" s="5"/>
       <c r="B123" s="7"/>
-      <c r="C123" s="7">
-        <v>63782</v>
-      </c>
+      <c r="C123" s="7"/>
       <c r="D123" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="124" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A124" s="7"/>
+      <c r="A124" s="5"/>
       <c r="B124" s="7"/>
       <c r="C124" s="7"/>
       <c r="D124" s="3" t="str">
@@ -3270,36 +3405,31 @@
       </c>
     </row>
     <row r="125" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A125" s="7"/>
+      <c r="A125" s="5"/>
       <c r="B125" s="7"/>
       <c r="C125" s="7"/>
-      <c r="D125" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="D125" s="3"/>
     </row>
     <row r="126" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A126" s="7"/>
+      <c r="A126" s="5"/>
       <c r="B126" s="7"/>
       <c r="C126" s="7"/>
-      <c r="D126" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="D126" s="3"/>
     </row>
     <row r="127" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A127" s="7"/>
+      <c r="A127" s="5"/>
       <c r="B127" s="7"/>
       <c r="C127" s="7"/>
-      <c r="D127" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="D127" s="3"/>
     </row>
     <row r="128" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A128" s="7"/>
+      <c r="A128" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="B128" s="7"/>
-      <c r="C128" s="7"/>
+      <c r="C128" s="7">
+        <v>63782</v>
+      </c>
       <c r="D128" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -3544,7 +3674,7 @@
       <c r="B155" s="7"/>
       <c r="C155" s="7"/>
       <c r="D155" s="3" t="str">
-        <f t="shared" ref="D155:D159" si="6">IF(C155&lt;&gt;"",IF(B155&lt;&gt;"",C155-B155,"-"), "-")</f>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3553,7 +3683,7 @@
       <c r="B156" s="7"/>
       <c r="C156" s="7"/>
       <c r="D156" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3562,7 +3692,7 @@
       <c r="B157" s="7"/>
       <c r="C157" s="7"/>
       <c r="D157" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3571,7 +3701,7 @@
       <c r="B158" s="7"/>
       <c r="C158" s="7"/>
       <c r="D158" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3580,7 +3710,7 @@
       <c r="B159" s="7"/>
       <c r="C159" s="7"/>
       <c r="D159" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3589,7 +3719,7 @@
       <c r="B160" s="7"/>
       <c r="C160" s="7"/>
       <c r="D160" s="3" t="str">
-        <f t="shared" ref="D160:D161" si="7">IF(C160&lt;&gt;"",IF(B160&lt;&gt;"",B160-C160,"-"), "-")</f>
+        <f t="shared" ref="D160:D164" si="6">IF(C160&lt;&gt;"",IF(B160&lt;&gt;"",C160-B160,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3598,7 +3728,7 @@
       <c r="B161" s="7"/>
       <c r="C161" s="7"/>
       <c r="D161" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-</v>
       </c>
     </row>
@@ -3606,29 +3736,54 @@
       <c r="A162" s="7"/>
       <c r="B162" s="7"/>
       <c r="C162" s="7"/>
+      <c r="D162" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="163" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A163" s="7"/>
       <c r="B163" s="7"/>
       <c r="C163" s="7"/>
+      <c r="D163" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="164" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A164" s="7"/>
       <c r="B164" s="7"/>
       <c r="C164" s="7"/>
+      <c r="D164" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="165" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A165" s="7"/>
       <c r="B165" s="7"/>
       <c r="C165" s="7"/>
+      <c r="D165" s="3" t="str">
+        <f t="shared" ref="D165:D166" si="7">IF(C165&lt;&gt;"",IF(B165&lt;&gt;"",B165-C165,"-"), "-")</f>
+        <v>-</v>
+      </c>
     </row>
     <row r="166" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A166" s="7"/>
       <c r="B166" s="7"/>
       <c r="C166" s="7"/>
+      <c r="D166" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="167" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A167" s="7"/>
       <c r="B167" s="7"/>
       <c r="C167" s="7"/>
     </row>
     <row r="168" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A168" s="7"/>
       <c r="B168" s="7"/>
       <c r="C168" s="7"/>
     </row>
@@ -4159,6 +4314,26 @@
     <row r="300" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B300" s="7"/>
       <c r="C300" s="7"/>
+    </row>
+    <row r="301" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B301" s="7"/>
+      <c r="C301" s="7"/>
+    </row>
+    <row r="302" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B302" s="7"/>
+      <c r="C302" s="7"/>
+    </row>
+    <row r="303" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B303" s="7"/>
+      <c r="C303" s="7"/>
+    </row>
+    <row r="304" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B304" s="7"/>
+      <c r="C304" s="7"/>
+    </row>
+    <row r="305" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B305" s="7"/>
+      <c r="C305" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14152,7 +14327,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="20" type="noConversion"/>
+  <phoneticPr fontId="22" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -14182,10 +14357,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="39" t="s">
+      <c r="K1" s="41" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="40"/>
+      <c r="L1" s="42"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -16037,13 +16212,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="41" t="s">
+      <c r="H53" s="43" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="42"/>
-      <c r="J53" s="42"/>
-      <c r="K53" s="42"/>
-      <c r="L53" s="43"/>
+      <c r="I53" s="44"/>
+      <c r="J53" s="44"/>
+      <c r="K53" s="44"/>
+      <c r="L53" s="45"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -16065,11 +16240,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="44"/>
-      <c r="I54" s="45"/>
-      <c r="J54" s="45"/>
-      <c r="K54" s="45"/>
-      <c r="L54" s="46"/>
+      <c r="H54" s="46"/>
+      <c r="I54" s="47"/>
+      <c r="J54" s="47"/>
+      <c r="K54" s="47"/>
+      <c r="L54" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lv 19 done - 5833 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A07853F7-E41D-4825-B1C6-879842AB8269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F327EA6-0A13-4F91-9CE8-86293F054B53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="308">
   <si>
     <t>Place</t>
   </si>
@@ -950,6 +950,15 @@
   </si>
   <si>
     <t>19 1st move</t>
+  </si>
+  <si>
+    <t>19 end</t>
+  </si>
+  <si>
+    <t>gold = 11</t>
+  </si>
+  <si>
+    <t>20 gold = 14</t>
   </si>
 </sst>
 </file>
@@ -1789,7 +1798,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E305"/>
+  <dimension ref="A1:E306"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -2474,7 +2483,7 @@
         <v>12106</v>
       </c>
       <c r="D45" s="3">
-        <f t="shared" ref="D45:D83" si="2">IF(C45&lt;&gt;"",IF(B45&lt;&gt;"",C45-B45,"-"), "-")</f>
+        <f t="shared" ref="D45:D84" si="2">IF(C45&lt;&gt;"",IF(B45&lt;&gt;"",C45-B45,"-"), "-")</f>
         <v>2989</v>
       </c>
     </row>
@@ -3027,36 +3036,54 @@
       </c>
     </row>
     <row r="83" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A83" s="7"/>
-      <c r="B83" s="7"/>
-      <c r="C83" s="7"/>
-      <c r="D83" s="3" t="str">
+      <c r="A83" s="49" t="s">
+        <v>306</v>
+      </c>
+      <c r="B83" s="7">
+        <v>17632</v>
+      </c>
+      <c r="C83" s="7">
+        <v>23135</v>
+      </c>
+      <c r="D83" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>5503</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A84" s="7"/>
-      <c r="B84" s="7"/>
-      <c r="C84" s="7"/>
-      <c r="D84" s="3" t="str">
-        <f t="shared" ref="D84:D90" si="4">IF(C84&lt;&gt;"",IF(B84&lt;&gt;"",C84-B84,"-"), "-")</f>
-        <v>-</v>
+      <c r="A84" s="49" t="s">
+        <v>305</v>
+      </c>
+      <c r="B84" s="7">
+        <v>17791</v>
+      </c>
+      <c r="C84" s="7">
+        <v>23287</v>
+      </c>
+      <c r="D84" s="3">
+        <f t="shared" si="2"/>
+        <v>5496</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A85" s="7"/>
-      <c r="B85" s="9"/>
-      <c r="C85" s="9"/>
-      <c r="D85" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
+      <c r="A85" s="49" t="s">
+        <v>307</v>
+      </c>
+      <c r="B85" s="7">
+        <v>18141</v>
+      </c>
+      <c r="C85" s="7">
+        <v>23974</v>
+      </c>
+      <c r="D85" s="3">
+        <f t="shared" ref="D85:D91" si="4">IF(C85&lt;&gt;"",IF(B85&lt;&gt;"",C85-B85,"-"), "-")</f>
+        <v>5833</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A86" s="7"/>
-      <c r="B86" s="7"/>
-      <c r="C86" s="7"/>
+      <c r="B86" s="9"/>
+      <c r="C86" s="9"/>
       <c r="D86" s="3" t="str">
         <f t="shared" si="4"/>
         <v>-</v>
@@ -3064,8 +3091,8 @@
     </row>
     <row r="87" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A87" s="7"/>
-      <c r="B87" s="9"/>
-      <c r="C87" s="9"/>
+      <c r="B87" s="7"/>
+      <c r="C87" s="7"/>
       <c r="D87" s="3" t="str">
         <f t="shared" si="4"/>
         <v>-</v>
@@ -3073,8 +3100,8 @@
     </row>
     <row r="88" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A88" s="7"/>
-      <c r="B88" s="7"/>
-      <c r="C88" s="7"/>
+      <c r="B88" s="9"/>
+      <c r="C88" s="9"/>
       <c r="D88" s="3" t="str">
         <f t="shared" si="4"/>
         <v>-</v>
@@ -3090,7 +3117,7 @@
       </c>
     </row>
     <row r="90" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A90" s="5"/>
+      <c r="A90" s="7"/>
       <c r="B90" s="7"/>
       <c r="C90" s="7"/>
       <c r="D90" s="3" t="str">
@@ -3103,7 +3130,7 @@
       <c r="B91" s="7"/>
       <c r="C91" s="7"/>
       <c r="D91" s="3" t="str">
-        <f t="shared" ref="D91:D159" si="5">IF(C91&lt;&gt;"",IF(B91&lt;&gt;"",C91-B91,"-"), "-")</f>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
@@ -3112,7 +3139,7 @@
       <c r="B92" s="7"/>
       <c r="C92" s="7"/>
       <c r="D92" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="D92:D160" si="5">IF(C92&lt;&gt;"",IF(B92&lt;&gt;"",C92-B92,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3153,7 +3180,7 @@
       </c>
     </row>
     <row r="97" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A97" s="7"/>
+      <c r="A97" s="5"/>
       <c r="B97" s="7"/>
       <c r="C97" s="7"/>
       <c r="D97" s="3" t="str">
@@ -3171,7 +3198,7 @@
       </c>
     </row>
     <row r="99" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A99" s="34"/>
+      <c r="A99" s="7"/>
       <c r="B99" s="7"/>
       <c r="C99" s="7"/>
       <c r="D99" s="3" t="str">
@@ -3180,7 +3207,7 @@
       </c>
     </row>
     <row r="100" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A100" s="7"/>
+      <c r="A100" s="34"/>
       <c r="B100" s="7"/>
       <c r="C100" s="7"/>
       <c r="D100" s="3" t="str">
@@ -3189,7 +3216,7 @@
       </c>
     </row>
     <row r="101" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A101" s="5"/>
+      <c r="A101" s="7"/>
       <c r="B101" s="7"/>
       <c r="C101" s="7"/>
       <c r="D101" s="3" t="str">
@@ -3343,8 +3370,8 @@
     </row>
     <row r="118" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A118" s="5"/>
-      <c r="B118" s="10"/>
-      <c r="C118" s="10"/>
+      <c r="B118" s="7"/>
+      <c r="C118" s="7"/>
       <c r="D118" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -3352,15 +3379,15 @@
     </row>
     <row r="119" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A119" s="5"/>
-      <c r="B119" s="7"/>
-      <c r="C119" s="7"/>
+      <c r="B119" s="10"/>
+      <c r="C119" s="10"/>
       <c r="D119" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="120" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A120" s="35"/>
+      <c r="A120" s="5"/>
       <c r="B120" s="7"/>
       <c r="C120" s="7"/>
       <c r="D120" s="3" t="str">
@@ -3369,7 +3396,7 @@
       </c>
     </row>
     <row r="121" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A121" s="5"/>
+      <c r="A121" s="35"/>
       <c r="B121" s="7"/>
       <c r="C121" s="7"/>
       <c r="D121" s="3" t="str">
@@ -3408,7 +3435,10 @@
       <c r="A125" s="5"/>
       <c r="B125" s="7"/>
       <c r="C125" s="7"/>
-      <c r="D125" s="3"/>
+      <c r="D125" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="126" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A126" s="5"/>
@@ -3423,22 +3453,19 @@
       <c r="D127" s="3"/>
     </row>
     <row r="128" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A128" s="5" t="s">
+      <c r="A128" s="5"/>
+      <c r="B128" s="7"/>
+      <c r="C128" s="7"/>
+      <c r="D128" s="3"/>
+    </row>
+    <row r="129" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A129" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B128" s="7"/>
-      <c r="C128" s="7">
+      <c r="B129" s="7"/>
+      <c r="C129" s="7">
         <v>63782</v>
       </c>
-      <c r="D128" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A129" s="7"/>
-      <c r="B129" s="7"/>
-      <c r="C129" s="7"/>
       <c r="D129" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -3719,7 +3746,7 @@
       <c r="B160" s="7"/>
       <c r="C160" s="7"/>
       <c r="D160" s="3" t="str">
-        <f t="shared" ref="D160:D164" si="6">IF(C160&lt;&gt;"",IF(B160&lt;&gt;"",C160-B160,"-"), "-")</f>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3728,7 +3755,7 @@
       <c r="B161" s="7"/>
       <c r="C161" s="7"/>
       <c r="D161" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="D161:D165" si="6">IF(C161&lt;&gt;"",IF(B161&lt;&gt;"",C161-B161,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3764,7 +3791,7 @@
       <c r="B165" s="7"/>
       <c r="C165" s="7"/>
       <c r="D165" s="3" t="str">
-        <f t="shared" ref="D165:D166" si="7">IF(C165&lt;&gt;"",IF(B165&lt;&gt;"",B165-C165,"-"), "-")</f>
+        <f t="shared" si="6"/>
         <v>-</v>
       </c>
     </row>
@@ -3773,7 +3800,7 @@
       <c r="B166" s="7"/>
       <c r="C166" s="7"/>
       <c r="D166" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="D166:D167" si="7">IF(C166&lt;&gt;"",IF(B166&lt;&gt;"",B166-C166,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3781,6 +3808,10 @@
       <c r="A167" s="7"/>
       <c r="B167" s="7"/>
       <c r="C167" s="7"/>
+      <c r="D167" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="168" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A168" s="7"/>
@@ -3788,6 +3819,7 @@
       <c r="C168" s="7"/>
     </row>
     <row r="169" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A169" s="7"/>
       <c r="B169" s="7"/>
       <c r="C169" s="7"/>
     </row>
@@ -4334,6 +4366,10 @@
     <row r="305" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B305" s="7"/>
       <c r="C305" s="7"/>
+    </row>
+    <row r="306" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B306" s="7"/>
+      <c r="C306" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - lv 21 done, 6443 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F327EA6-0A13-4F91-9CE8-86293F054B53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33E0942B-03F2-4C9B-A977-5F0108A37746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="316">
   <si>
     <t>Place</t>
   </si>
@@ -959,6 +959,30 @@
   </si>
   <si>
     <t>20 gold = 14</t>
+  </si>
+  <si>
+    <t>20 end</t>
+  </si>
+  <si>
+    <t>gold = 12</t>
+  </si>
+  <si>
+    <t>gold = 4</t>
+  </si>
+  <si>
+    <t>gold = 9</t>
+  </si>
+  <si>
+    <t>gold = 8</t>
+  </si>
+  <si>
+    <t>21 ladder grab</t>
+  </si>
+  <si>
+    <t>21 end</t>
+  </si>
+  <si>
+    <t>22 ladder grab</t>
   </si>
 </sst>
 </file>
@@ -1798,7 +1822,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E306"/>
+  <dimension ref="A1:E320"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -3070,184 +3094,280 @@
         <v>307</v>
       </c>
       <c r="B85" s="7">
-        <v>18141</v>
+        <v>18160</v>
       </c>
       <c r="C85" s="7">
         <v>23974</v>
       </c>
       <c r="D85" s="3">
-        <f t="shared" ref="D85:D91" si="4">IF(C85&lt;&gt;"",IF(B85&lt;&gt;"",C85-B85,"-"), "-")</f>
-        <v>5833</v>
+        <f t="shared" ref="D85:D105" si="4">IF(C85&lt;&gt;"",IF(B85&lt;&gt;"",C85-B85,"-"), "-")</f>
+        <v>5814</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A86" s="7"/>
-      <c r="B86" s="9"/>
-      <c r="C86" s="9"/>
-      <c r="D86" s="3" t="str">
+      <c r="A86" s="49" t="s">
+        <v>309</v>
+      </c>
+      <c r="B86" s="7">
+        <v>18223</v>
+      </c>
+      <c r="C86" s="7">
+        <v>24038</v>
+      </c>
+      <c r="D86" s="3">
         <f t="shared" si="4"/>
-        <v>-</v>
+        <v>5815</v>
       </c>
     </row>
     <row r="87" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A87" s="7"/>
-      <c r="B87" s="7"/>
-      <c r="C87" s="7"/>
-      <c r="D87" s="3" t="str">
+      <c r="A87" s="49" t="s">
+        <v>306</v>
+      </c>
+      <c r="B87" s="7">
+        <v>18289</v>
+      </c>
+      <c r="C87" s="7">
+        <v>24097</v>
+      </c>
+      <c r="D87" s="3">
         <f t="shared" si="4"/>
-        <v>-</v>
+        <v>5808</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A88" s="7"/>
-      <c r="B88" s="9"/>
-      <c r="C88" s="9"/>
+      <c r="A88" s="49" t="s">
+        <v>311</v>
+      </c>
+      <c r="B88" s="7"/>
+      <c r="C88" s="7">
+        <v>24186</v>
+      </c>
       <c r="D88" s="3" t="str">
         <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="89" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A89" s="7"/>
+      <c r="A89" s="49" t="s">
+        <v>312</v>
+      </c>
       <c r="B89" s="7"/>
-      <c r="C89" s="7"/>
+      <c r="C89" s="7">
+        <v>24206</v>
+      </c>
       <c r="D89" s="3" t="str">
         <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="90" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A90" s="7"/>
+      <c r="A90" s="49" t="s">
+        <v>279</v>
+      </c>
       <c r="B90" s="7"/>
-      <c r="C90" s="7"/>
+      <c r="C90" s="7">
+        <v>24244</v>
+      </c>
       <c r="D90" s="3" t="str">
         <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A91" s="5"/>
+      <c r="A91" s="49" t="s">
+        <v>293</v>
+      </c>
       <c r="B91" s="7"/>
-      <c r="C91" s="7"/>
+      <c r="C91" s="7">
+        <v>24282</v>
+      </c>
       <c r="D91" s="3" t="str">
         <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A92" s="5"/>
+      <c r="A92" s="49" t="s">
+        <v>247</v>
+      </c>
       <c r="B92" s="7"/>
-      <c r="C92" s="7"/>
+      <c r="C92" s="7">
+        <v>24297</v>
+      </c>
       <c r="D92" s="3" t="str">
-        <f t="shared" ref="D92:D160" si="5">IF(C92&lt;&gt;"",IF(B92&lt;&gt;"",C92-B92,"-"), "-")</f>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="93" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A93" s="5"/>
+      <c r="A93" s="49" t="s">
+        <v>310</v>
+      </c>
       <c r="B93" s="7"/>
-      <c r="C93" s="7"/>
+      <c r="C93" s="7">
+        <v>24357</v>
+      </c>
       <c r="D93" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A94" s="5"/>
-      <c r="B94" s="7"/>
-      <c r="C94" s="7"/>
-      <c r="D94" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
+      <c r="A94" s="49" t="s">
+        <v>308</v>
+      </c>
+      <c r="B94" s="9">
+        <v>18717</v>
+      </c>
+      <c r="C94" s="9">
+        <v>24522</v>
+      </c>
+      <c r="D94" s="3">
+        <f t="shared" si="4"/>
+        <v>5805</v>
       </c>
     </row>
     <row r="95" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A95" s="5"/>
-      <c r="B95" s="7"/>
-      <c r="C95" s="7"/>
-      <c r="D95" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
+      <c r="A95" s="49" t="s">
+        <v>313</v>
+      </c>
+      <c r="B95" s="7">
+        <v>19072</v>
+      </c>
+      <c r="C95" s="7">
+        <v>25193</v>
+      </c>
+      <c r="D95" s="3">
+        <f t="shared" si="4"/>
+        <v>6121</v>
       </c>
     </row>
     <row r="96" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A96" s="5"/>
-      <c r="B96" s="7"/>
-      <c r="C96" s="7"/>
-      <c r="D96" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
+      <c r="A96" s="49" t="s">
+        <v>306</v>
+      </c>
+      <c r="B96" s="7">
+        <v>19223</v>
+      </c>
+      <c r="C96" s="7">
+        <v>25345</v>
+      </c>
+      <c r="D96" s="3">
+        <f t="shared" si="4"/>
+        <v>6122</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A97" s="5"/>
-      <c r="B97" s="7"/>
-      <c r="C97" s="7"/>
-      <c r="D97" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
+      <c r="A97" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="B97" s="7">
+        <v>19260</v>
+      </c>
+      <c r="C97" s="7">
+        <v>25382</v>
+      </c>
+      <c r="D97" s="3">
+        <f t="shared" si="4"/>
+        <v>6122</v>
       </c>
     </row>
     <row r="98" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A98" s="7"/>
-      <c r="B98" s="7"/>
-      <c r="C98" s="7"/>
-      <c r="D98" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
+      <c r="A98" s="49" t="s">
+        <v>311</v>
+      </c>
+      <c r="B98" s="7">
+        <v>19369</v>
+      </c>
+      <c r="C98" s="7">
+        <v>25492</v>
+      </c>
+      <c r="D98" s="3">
+        <f t="shared" si="4"/>
+        <v>6123</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A99" s="7"/>
-      <c r="B99" s="7"/>
-      <c r="C99" s="7"/>
-      <c r="D99" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
+      <c r="A99" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="B99" s="7">
+        <v>19474</v>
+      </c>
+      <c r="C99" s="7">
+        <v>25596</v>
+      </c>
+      <c r="D99" s="3">
+        <f t="shared" si="4"/>
+        <v>6122</v>
       </c>
     </row>
     <row r="100" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A100" s="34"/>
-      <c r="B100" s="7"/>
-      <c r="C100" s="7"/>
-      <c r="D100" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
+      <c r="A100" s="49" t="s">
+        <v>247</v>
+      </c>
+      <c r="B100" s="7">
+        <v>19650</v>
+      </c>
+      <c r="C100" s="7">
+        <v>25772</v>
+      </c>
+      <c r="D100" s="3">
+        <f t="shared" si="4"/>
+        <v>6122</v>
       </c>
     </row>
     <row r="101" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A101" s="7"/>
-      <c r="B101" s="7"/>
-      <c r="C101" s="7"/>
-      <c r="D101" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
+      <c r="A101" s="49" t="s">
+        <v>250</v>
+      </c>
+      <c r="B101" s="7">
+        <v>19789</v>
+      </c>
+      <c r="C101" s="7">
+        <v>25913</v>
+      </c>
+      <c r="D101" s="3">
+        <f t="shared" si="4"/>
+        <v>6124</v>
       </c>
     </row>
     <row r="102" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A102" s="5"/>
-      <c r="B102" s="7"/>
-      <c r="C102" s="7"/>
-      <c r="D102" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
+      <c r="A102" s="49" t="s">
+        <v>314</v>
+      </c>
+      <c r="B102" s="9">
+        <v>19892</v>
+      </c>
+      <c r="C102" s="9">
+        <v>26016</v>
+      </c>
+      <c r="D102" s="3">
+        <f t="shared" si="4"/>
+        <v>6124</v>
       </c>
     </row>
     <row r="103" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A103" s="5"/>
-      <c r="B103" s="7"/>
-      <c r="C103" s="7"/>
-      <c r="D103" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
+      <c r="A103" s="49" t="s">
+        <v>315</v>
+      </c>
+      <c r="B103" s="7">
+        <v>20248</v>
+      </c>
+      <c r="C103" s="7">
+        <v>26691</v>
+      </c>
+      <c r="D103" s="3">
+        <f t="shared" si="4"/>
+        <v>6443</v>
       </c>
     </row>
     <row r="104" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A104" s="5"/>
+      <c r="A104" s="7"/>
       <c r="B104" s="7"/>
       <c r="C104" s="7"/>
       <c r="D104" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
@@ -3256,7 +3376,7 @@
       <c r="B105" s="7"/>
       <c r="C105" s="7"/>
       <c r="D105" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
@@ -3265,7 +3385,7 @@
       <c r="B106" s="7"/>
       <c r="C106" s="7"/>
       <c r="D106" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="D106:D174" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3315,7 +3435,7 @@
       </c>
     </row>
     <row r="112" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A112" s="5"/>
+      <c r="A112" s="7"/>
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
       <c r="D112" s="3" t="str">
@@ -3324,7 +3444,7 @@
       </c>
     </row>
     <row r="113" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A113" s="5"/>
+      <c r="A113" s="7"/>
       <c r="B113" s="7"/>
       <c r="C113" s="7"/>
       <c r="D113" s="3" t="str">
@@ -3333,7 +3453,7 @@
       </c>
     </row>
     <row r="114" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A114" s="5"/>
+      <c r="A114" s="34"/>
       <c r="B114" s="7"/>
       <c r="C114" s="7"/>
       <c r="D114" s="3" t="str">
@@ -3342,7 +3462,7 @@
       </c>
     </row>
     <row r="115" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A115" s="5"/>
+      <c r="A115" s="7"/>
       <c r="B115" s="7"/>
       <c r="C115" s="7"/>
       <c r="D115" s="3" t="str">
@@ -3379,8 +3499,8 @@
     </row>
     <row r="119" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A119" s="5"/>
-      <c r="B119" s="10"/>
-      <c r="C119" s="10"/>
+      <c r="B119" s="7"/>
+      <c r="C119" s="7"/>
       <c r="D119" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -3396,7 +3516,7 @@
       </c>
     </row>
     <row r="121" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A121" s="35"/>
+      <c r="A121" s="5"/>
       <c r="B121" s="7"/>
       <c r="C121" s="7"/>
       <c r="D121" s="3" t="str">
@@ -3444,35 +3564,40 @@
       <c r="A126" s="5"/>
       <c r="B126" s="7"/>
       <c r="C126" s="7"/>
-      <c r="D126" s="3"/>
+      <c r="D126" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="127" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A127" s="5"/>
       <c r="B127" s="7"/>
       <c r="C127" s="7"/>
-      <c r="D127" s="3"/>
+      <c r="D127" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="128" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A128" s="5"/>
       <c r="B128" s="7"/>
       <c r="C128" s="7"/>
-      <c r="D128" s="3"/>
+      <c r="D128" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="129" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A129" s="5" t="s">
-        <v>26</v>
-      </c>
+      <c r="A129" s="5"/>
       <c r="B129" s="7"/>
-      <c r="C129" s="7">
-        <v>63782</v>
-      </c>
+      <c r="C129" s="7"/>
       <c r="D129" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="130" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A130" s="7"/>
+      <c r="A130" s="5"/>
       <c r="B130" s="7"/>
       <c r="C130" s="7"/>
       <c r="D130" s="3" t="str">
@@ -3481,7 +3606,7 @@
       </c>
     </row>
     <row r="131" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A131" s="7"/>
+      <c r="A131" s="5"/>
       <c r="B131" s="7"/>
       <c r="C131" s="7"/>
       <c r="D131" s="3" t="str">
@@ -3490,7 +3615,7 @@
       </c>
     </row>
     <row r="132" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A132" s="7"/>
+      <c r="A132" s="5"/>
       <c r="B132" s="7"/>
       <c r="C132" s="7"/>
       <c r="D132" s="3" t="str">
@@ -3499,16 +3624,16 @@
       </c>
     </row>
     <row r="133" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A133" s="7"/>
-      <c r="B133" s="7"/>
-      <c r="C133" s="7"/>
+      <c r="A133" s="5"/>
+      <c r="B133" s="10"/>
+      <c r="C133" s="10"/>
       <c r="D133" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="134" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A134" s="7"/>
+      <c r="A134" s="5"/>
       <c r="B134" s="7"/>
       <c r="C134" s="7"/>
       <c r="D134" s="3" t="str">
@@ -3517,7 +3642,7 @@
       </c>
     </row>
     <row r="135" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A135" s="7"/>
+      <c r="A135" s="35"/>
       <c r="B135" s="7"/>
       <c r="C135" s="7"/>
       <c r="D135" s="3" t="str">
@@ -3526,7 +3651,7 @@
       </c>
     </row>
     <row r="136" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A136" s="7"/>
+      <c r="A136" s="5"/>
       <c r="B136" s="7"/>
       <c r="C136" s="7"/>
       <c r="D136" s="3" t="str">
@@ -3535,7 +3660,7 @@
       </c>
     </row>
     <row r="137" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A137" s="7"/>
+      <c r="A137" s="5"/>
       <c r="B137" s="7"/>
       <c r="C137" s="7"/>
       <c r="D137" s="3" t="str">
@@ -3544,7 +3669,7 @@
       </c>
     </row>
     <row r="138" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A138" s="7"/>
+      <c r="A138" s="5"/>
       <c r="B138" s="7"/>
       <c r="C138" s="7"/>
       <c r="D138" s="3" t="str">
@@ -3553,7 +3678,7 @@
       </c>
     </row>
     <row r="139" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A139" s="7"/>
+      <c r="A139" s="5"/>
       <c r="B139" s="7"/>
       <c r="C139" s="7"/>
       <c r="D139" s="3" t="str">
@@ -3562,36 +3687,31 @@
       </c>
     </row>
     <row r="140" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A140" s="7"/>
+      <c r="A140" s="5"/>
       <c r="B140" s="7"/>
       <c r="C140" s="7"/>
-      <c r="D140" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="D140" s="3"/>
     </row>
     <row r="141" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A141" s="7"/>
+      <c r="A141" s="5"/>
       <c r="B141" s="7"/>
       <c r="C141" s="7"/>
-      <c r="D141" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="D141" s="3"/>
     </row>
     <row r="142" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A142" s="7"/>
+      <c r="A142" s="5"/>
       <c r="B142" s="7"/>
       <c r="C142" s="7"/>
-      <c r="D142" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="D142" s="3"/>
     </row>
     <row r="143" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A143" s="7"/>
+      <c r="A143" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="B143" s="7"/>
-      <c r="C143" s="7"/>
+      <c r="C143" s="7">
+        <v>63782</v>
+      </c>
       <c r="D143" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -3755,7 +3875,7 @@
       <c r="B161" s="7"/>
       <c r="C161" s="7"/>
       <c r="D161" s="3" t="str">
-        <f t="shared" ref="D161:D165" si="6">IF(C161&lt;&gt;"",IF(B161&lt;&gt;"",C161-B161,"-"), "-")</f>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3764,7 +3884,7 @@
       <c r="B162" s="7"/>
       <c r="C162" s="7"/>
       <c r="D162" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3773,7 +3893,7 @@
       <c r="B163" s="7"/>
       <c r="C163" s="7"/>
       <c r="D163" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3782,7 +3902,7 @@
       <c r="B164" s="7"/>
       <c r="C164" s="7"/>
       <c r="D164" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3791,7 +3911,7 @@
       <c r="B165" s="7"/>
       <c r="C165" s="7"/>
       <c r="D165" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3800,7 +3920,7 @@
       <c r="B166" s="7"/>
       <c r="C166" s="7"/>
       <c r="D166" s="3" t="str">
-        <f t="shared" ref="D166:D167" si="7">IF(C166&lt;&gt;"",IF(B166&lt;&gt;"",B166-C166,"-"), "-")</f>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3809,7 +3929,7 @@
       <c r="B167" s="7"/>
       <c r="C167" s="7"/>
       <c r="D167" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -3817,101 +3937,171 @@
       <c r="A168" s="7"/>
       <c r="B168" s="7"/>
       <c r="C168" s="7"/>
+      <c r="D168" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="169" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A169" s="7"/>
       <c r="B169" s="7"/>
       <c r="C169" s="7"/>
+      <c r="D169" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="170" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A170" s="7"/>
       <c r="B170" s="7"/>
       <c r="C170" s="7"/>
+      <c r="D170" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="171" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A171" s="7"/>
       <c r="B171" s="7"/>
       <c r="C171" s="7"/>
+      <c r="D171" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="172" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A172" s="7"/>
       <c r="B172" s="7"/>
       <c r="C172" s="7"/>
+      <c r="D172" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="173" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A173" s="7"/>
       <c r="B173" s="7"/>
       <c r="C173" s="7"/>
+      <c r="D173" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="174" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A174" s="7"/>
       <c r="B174" s="7"/>
       <c r="C174" s="7"/>
+      <c r="D174" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="175" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A175" s="7"/>
       <c r="B175" s="7"/>
       <c r="C175" s="7"/>
+      <c r="D175" s="3" t="str">
+        <f t="shared" ref="D175:D179" si="6">IF(C175&lt;&gt;"",IF(B175&lt;&gt;"",C175-B175,"-"), "-")</f>
+        <v>-</v>
+      </c>
     </row>
     <row r="176" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A176" s="7"/>
       <c r="B176" s="7"/>
       <c r="C176" s="7"/>
-    </row>
-    <row r="177" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D176" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A177" s="7"/>
       <c r="B177" s="7"/>
       <c r="C177" s="7"/>
-    </row>
-    <row r="178" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D177" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A178" s="7"/>
       <c r="B178" s="7"/>
       <c r="C178" s="7"/>
-    </row>
-    <row r="179" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D178" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A179" s="7"/>
       <c r="B179" s="7"/>
       <c r="C179" s="7"/>
-    </row>
-    <row r="180" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D179" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A180" s="7"/>
       <c r="B180" s="7"/>
       <c r="C180" s="7"/>
-    </row>
-    <row r="181" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D180" s="3" t="str">
+        <f t="shared" ref="D180:D181" si="7">IF(C180&lt;&gt;"",IF(B180&lt;&gt;"",B180-C180,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A181" s="7"/>
       <c r="B181" s="7"/>
       <c r="C181" s="7"/>
-    </row>
-    <row r="182" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D181" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A182" s="7"/>
       <c r="B182" s="7"/>
       <c r="C182" s="7"/>
     </row>
-    <row r="183" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A183" s="7"/>
       <c r="B183" s="7"/>
       <c r="C183" s="7"/>
     </row>
-    <row r="184" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
     </row>
-    <row r="185" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B185" s="7"/>
       <c r="C185" s="7"/>
     </row>
-    <row r="186" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B186" s="7"/>
       <c r="C186" s="7"/>
     </row>
-    <row r="187" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B187" s="7"/>
       <c r="C187" s="7"/>
     </row>
-    <row r="188" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B188" s="7"/>
       <c r="C188" s="7"/>
     </row>
-    <row r="189" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B189" s="7"/>
       <c r="C189" s="7"/>
     </row>
-    <row r="190" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B190" s="7"/>
       <c r="C190" s="7"/>
     </row>
-    <row r="191" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B191" s="7"/>
       <c r="C191" s="7"/>
     </row>
-    <row r="192" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B192" s="7"/>
       <c r="C192" s="7"/>
     </row>
@@ -4370,6 +4560,62 @@
     <row r="306" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B306" s="7"/>
       <c r="C306" s="7"/>
+    </row>
+    <row r="307" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B307" s="7"/>
+      <c r="C307" s="7"/>
+    </row>
+    <row r="308" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B308" s="7"/>
+      <c r="C308" s="7"/>
+    </row>
+    <row r="309" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B309" s="7"/>
+      <c r="C309" s="7"/>
+    </row>
+    <row r="310" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B310" s="7"/>
+      <c r="C310" s="7"/>
+    </row>
+    <row r="311" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B311" s="7"/>
+      <c r="C311" s="7"/>
+    </row>
+    <row r="312" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B312" s="7"/>
+      <c r="C312" s="7"/>
+    </row>
+    <row r="313" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B313" s="7"/>
+      <c r="C313" s="7"/>
+    </row>
+    <row r="314" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B314" s="7"/>
+      <c r="C314" s="7"/>
+    </row>
+    <row r="315" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B315" s="7"/>
+      <c r="C315" s="7"/>
+    </row>
+    <row r="316" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B316" s="7"/>
+      <c r="C316" s="7"/>
+    </row>
+    <row r="317" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B317" s="7"/>
+      <c r="C317" s="7"/>
+    </row>
+    <row r="318" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B318" s="7"/>
+      <c r="C318" s="7"/>
+    </row>
+    <row r="319" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B319" s="7"/>
+      <c r="C319" s="7"/>
+    </row>
+    <row r="320" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B320" s="7"/>
+      <c r="C320" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - level 22 done
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33E0942B-03F2-4C9B-A977-5F0108A37746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA86907E-B483-40EA-9EA7-C543DD79BDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="322">
   <si>
     <t>Place</t>
   </si>
@@ -983,6 +983,24 @@
   </si>
   <si>
     <t>22 ladder grab</t>
+  </si>
+  <si>
+    <t>gold = 17</t>
+  </si>
+  <si>
+    <t>drop manip</t>
+  </si>
+  <si>
+    <t>gold = 13</t>
+  </si>
+  <si>
+    <t>gold = 10</t>
+  </si>
+  <si>
+    <t>22 end</t>
+  </si>
+  <si>
+    <t>23 ladder grab</t>
   </si>
 </sst>
 </file>
@@ -992,12 +1010,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1380,95 +1405,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1477,28 +1503,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2970,7 +2996,7 @@
       </c>
     </row>
     <row r="77" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A77" s="49" t="s">
+      <c r="A77" s="41" t="s">
         <v>303</v>
       </c>
       <c r="B77" s="7">
@@ -2985,7 +3011,7 @@
       </c>
     </row>
     <row r="78" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A78" s="49" t="s">
+      <c r="A78" s="41" t="s">
         <v>265</v>
       </c>
       <c r="B78" s="7">
@@ -3045,7 +3071,7 @@
       </c>
     </row>
     <row r="82" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A82" s="49" t="s">
+      <c r="A82" s="41" t="s">
         <v>304</v>
       </c>
       <c r="B82" s="7">
@@ -3060,7 +3086,7 @@
       </c>
     </row>
     <row r="83" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A83" s="49" t="s">
+      <c r="A83" s="41" t="s">
         <v>306</v>
       </c>
       <c r="B83" s="7">
@@ -3075,7 +3101,7 @@
       </c>
     </row>
     <row r="84" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A84" s="49" t="s">
+      <c r="A84" s="41" t="s">
         <v>305</v>
       </c>
       <c r="B84" s="7">
@@ -3090,7 +3116,7 @@
       </c>
     </row>
     <row r="85" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A85" s="49" t="s">
+      <c r="A85" s="41" t="s">
         <v>307</v>
       </c>
       <c r="B85" s="7">
@@ -3105,7 +3131,7 @@
       </c>
     </row>
     <row r="86" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A86" s="49" t="s">
+      <c r="A86" s="41" t="s">
         <v>309</v>
       </c>
       <c r="B86" s="7">
@@ -3120,7 +3146,7 @@
       </c>
     </row>
     <row r="87" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A87" s="49" t="s">
+      <c r="A87" s="41" t="s">
         <v>306</v>
       </c>
       <c r="B87" s="7">
@@ -3135,7 +3161,7 @@
       </c>
     </row>
     <row r="88" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A88" s="49" t="s">
+      <c r="A88" s="41" t="s">
         <v>311</v>
       </c>
       <c r="B88" s="7"/>
@@ -3148,7 +3174,7 @@
       </c>
     </row>
     <row r="89" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A89" s="49" t="s">
+      <c r="A89" s="41" t="s">
         <v>312</v>
       </c>
       <c r="B89" s="7"/>
@@ -3161,7 +3187,7 @@
       </c>
     </row>
     <row r="90" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A90" s="49" t="s">
+      <c r="A90" s="41" t="s">
         <v>279</v>
       </c>
       <c r="B90" s="7"/>
@@ -3174,7 +3200,7 @@
       </c>
     </row>
     <row r="91" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A91" s="49" t="s">
+      <c r="A91" s="41" t="s">
         <v>293</v>
       </c>
       <c r="B91" s="7"/>
@@ -3187,7 +3213,7 @@
       </c>
     </row>
     <row r="92" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A92" s="49" t="s">
+      <c r="A92" s="41" t="s">
         <v>247</v>
       </c>
       <c r="B92" s="7"/>
@@ -3200,7 +3226,7 @@
       </c>
     </row>
     <row r="93" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A93" s="49" t="s">
+      <c r="A93" s="41" t="s">
         <v>310</v>
       </c>
       <c r="B93" s="7"/>
@@ -3213,7 +3239,7 @@
       </c>
     </row>
     <row r="94" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A94" s="49" t="s">
+      <c r="A94" s="41" t="s">
         <v>308</v>
       </c>
       <c r="B94" s="9">
@@ -3228,7 +3254,7 @@
       </c>
     </row>
     <row r="95" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A95" s="49" t="s">
+      <c r="A95" s="41" t="s">
         <v>313</v>
       </c>
       <c r="B95" s="7">
@@ -3243,7 +3269,7 @@
       </c>
     </row>
     <row r="96" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A96" s="49" t="s">
+      <c r="A96" s="41" t="s">
         <v>306</v>
       </c>
       <c r="B96" s="7">
@@ -3257,8 +3283,8 @@
         <v>6122</v>
       </c>
     </row>
-    <row r="97" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A97" s="49" t="s">
+    <row r="97" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A97" s="41" t="s">
         <v>265</v>
       </c>
       <c r="B97" s="7">
@@ -3272,8 +3298,8 @@
         <v>6122</v>
       </c>
     </row>
-    <row r="98" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A98" s="49" t="s">
+    <row r="98" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A98" s="41" t="s">
         <v>311</v>
       </c>
       <c r="B98" s="7">
@@ -3287,8 +3313,8 @@
         <v>6123</v>
       </c>
     </row>
-    <row r="99" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A99" s="49" t="s">
+    <row r="99" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A99" s="41" t="s">
         <v>265</v>
       </c>
       <c r="B99" s="7">
@@ -3302,8 +3328,8 @@
         <v>6122</v>
       </c>
     </row>
-    <row r="100" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A100" s="49" t="s">
+    <row r="100" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A100" s="41" t="s">
         <v>247</v>
       </c>
       <c r="B100" s="7">
@@ -3317,8 +3343,8 @@
         <v>6122</v>
       </c>
     </row>
-    <row r="101" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A101" s="49" t="s">
+    <row r="101" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A101" s="41" t="s">
         <v>250</v>
       </c>
       <c r="B101" s="7">
@@ -3332,8 +3358,8 @@
         <v>6124</v>
       </c>
     </row>
-    <row r="102" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A102" s="49" t="s">
+    <row r="102" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A102" s="41" t="s">
         <v>314</v>
       </c>
       <c r="B102" s="9">
@@ -3347,8 +3373,8 @@
         <v>6124</v>
       </c>
     </row>
-    <row r="103" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A103" s="49" t="s">
+    <row r="103" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A103" s="41" t="s">
         <v>315</v>
       </c>
       <c r="B103" s="7">
@@ -3362,79 +3388,128 @@
         <v>6443</v>
       </c>
     </row>
-    <row r="104" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A104" s="7"/>
-      <c r="B104" s="7"/>
-      <c r="C104" s="7"/>
-      <c r="D104" s="3" t="str">
+    <row r="104" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A104" s="50" t="s">
+        <v>316</v>
+      </c>
+      <c r="B104" s="7">
+        <v>20300</v>
+      </c>
+      <c r="C104" s="7">
+        <v>26735</v>
+      </c>
+      <c r="D104" s="3">
         <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A105" s="5"/>
-      <c r="B105" s="7"/>
-      <c r="C105" s="7"/>
-      <c r="D105" s="3" t="str">
+        <v>6435</v>
+      </c>
+      <c r="E104" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A105" s="50" t="s">
+        <v>318</v>
+      </c>
+      <c r="B105" s="7">
+        <v>20429</v>
+      </c>
+      <c r="C105" s="7">
+        <v>26863</v>
+      </c>
+      <c r="D105" s="3">
         <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A106" s="5"/>
-      <c r="B106" s="7"/>
-      <c r="C106" s="7"/>
-      <c r="D106" s="3" t="str">
+        <v>6434</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A106" s="50" t="s">
+        <v>319</v>
+      </c>
+      <c r="B106" s="7">
+        <v>20541</v>
+      </c>
+      <c r="C106" s="7">
+        <v>26982</v>
+      </c>
+      <c r="D106" s="3">
         <f t="shared" ref="D106:D174" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A107" s="5"/>
-      <c r="B107" s="7"/>
-      <c r="C107" s="7"/>
-      <c r="D107" s="3" t="str">
+        <v>6441</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A107" s="50" t="s">
+        <v>247</v>
+      </c>
+      <c r="B107" s="7">
+        <v>20625</v>
+      </c>
+      <c r="C107" s="7">
+        <v>27062</v>
+      </c>
+      <c r="D107" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A108" s="5"/>
-      <c r="B108" s="7"/>
-      <c r="C108" s="7"/>
-      <c r="D108" s="3" t="str">
+        <v>6437</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A108" s="50" t="s">
+        <v>310</v>
+      </c>
+      <c r="B108" s="7">
+        <v>20662</v>
+      </c>
+      <c r="C108" s="7">
+        <v>27102</v>
+      </c>
+      <c r="D108" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A109" s="5"/>
-      <c r="B109" s="7"/>
-      <c r="C109" s="7"/>
-      <c r="D109" s="3" t="str">
+        <v>6440</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A109" s="50" t="s">
+        <v>248</v>
+      </c>
+      <c r="B109" s="7">
+        <v>20776</v>
+      </c>
+      <c r="C109" s="7">
+        <v>27199</v>
+      </c>
+      <c r="D109" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A110" s="5"/>
-      <c r="B110" s="7"/>
-      <c r="C110" s="7"/>
-      <c r="D110" s="3" t="str">
+        <v>6423</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A110" s="50" t="s">
+        <v>320</v>
+      </c>
+      <c r="B110" s="7">
+        <v>20800</v>
+      </c>
+      <c r="C110" s="7">
+        <v>27233</v>
+      </c>
+      <c r="D110" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A111" s="5"/>
+        <v>6433</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A111" s="50" t="s">
+        <v>321</v>
+      </c>
       <c r="B111" s="7"/>
-      <c r="C111" s="7"/>
+      <c r="C111" s="7">
+        <v>27895</v>
+      </c>
       <c r="D111" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
-    <row r="112" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A112" s="7"/>
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
@@ -14609,7 +14684,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="22" type="noConversion"/>
+  <phoneticPr fontId="23" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -14639,10 +14714,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="41" t="s">
+      <c r="K1" s="42" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="42"/>
+      <c r="L1" s="43"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -16494,13 +16569,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="43" t="s">
+      <c r="H53" s="44" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="44"/>
-      <c r="J53" s="44"/>
-      <c r="K53" s="44"/>
-      <c r="L53" s="45"/>
+      <c r="I53" s="45"/>
+      <c r="J53" s="45"/>
+      <c r="K53" s="45"/>
+      <c r="L53" s="46"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -16522,11 +16597,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="46"/>
-      <c r="I54" s="47"/>
-      <c r="J54" s="47"/>
-      <c r="K54" s="47"/>
-      <c r="L54" s="48"/>
+      <c r="H54" s="47"/>
+      <c r="I54" s="48"/>
+      <c r="J54" s="48"/>
+      <c r="K54" s="48"/>
+      <c r="L54" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - lv 24 done, 7160 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA86907E-B483-40EA-9EA7-C543DD79BDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47D5076-C857-4E53-9372-4C2E3A72DC7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="326">
   <si>
     <t>Place</t>
   </si>
@@ -1001,6 +1001,18 @@
   </si>
   <si>
     <t>23 ladder grab</t>
+  </si>
+  <si>
+    <t>23 end</t>
+  </si>
+  <si>
+    <t>24 ladder grab</t>
+  </si>
+  <si>
+    <t>24 end</t>
+  </si>
+  <si>
+    <t>25 ladder grab</t>
   </si>
 </sst>
 </file>
@@ -1010,12 +1022,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1405,95 +1424,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1503,28 +1523,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1848,7 +1868,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E320"/>
+  <dimension ref="A1:E326"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -3389,7 +3409,7 @@
       </c>
     </row>
     <row r="104" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A104" s="50" t="s">
+      <c r="A104" s="42" t="s">
         <v>316</v>
       </c>
       <c r="B104" s="7">
@@ -3407,7 +3427,7 @@
       </c>
     </row>
     <row r="105" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A105" s="50" t="s">
+      <c r="A105" s="42" t="s">
         <v>318</v>
       </c>
       <c r="B105" s="7">
@@ -3422,7 +3442,7 @@
       </c>
     </row>
     <row r="106" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A106" s="50" t="s">
+      <c r="A106" s="42" t="s">
         <v>319</v>
       </c>
       <c r="B106" s="7">
@@ -3432,12 +3452,12 @@
         <v>26982</v>
       </c>
       <c r="D106" s="3">
-        <f t="shared" ref="D106:D174" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
+        <f t="shared" ref="D106:D180" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
         <v>6441</v>
       </c>
     </row>
     <row r="107" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A107" s="50" t="s">
+      <c r="A107" s="42" t="s">
         <v>247</v>
       </c>
       <c r="B107" s="7">
@@ -3452,7 +3472,7 @@
       </c>
     </row>
     <row r="108" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A108" s="50" t="s">
+      <c r="A108" s="42" t="s">
         <v>310</v>
       </c>
       <c r="B108" s="7">
@@ -3467,7 +3487,7 @@
       </c>
     </row>
     <row r="109" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A109" s="50" t="s">
+      <c r="A109" s="42" t="s">
         <v>248</v>
       </c>
       <c r="B109" s="7">
@@ -3482,7 +3502,7 @@
       </c>
     </row>
     <row r="110" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A110" s="50" t="s">
+      <c r="A110" s="42" t="s">
         <v>320</v>
       </c>
       <c r="B110" s="7">
@@ -3497,115 +3517,176 @@
       </c>
     </row>
     <row r="111" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A111" s="50" t="s">
+      <c r="A111" s="42" t="s">
         <v>321</v>
       </c>
-      <c r="B111" s="7"/>
+      <c r="B111" s="7">
+        <v>21171</v>
+      </c>
       <c r="C111" s="7">
         <v>27895</v>
       </c>
-      <c r="D111" s="3" t="str">
+      <c r="D111" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>6724</v>
       </c>
     </row>
     <row r="112" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A112" s="7"/>
-      <c r="B112" s="7"/>
-      <c r="C112" s="7"/>
-      <c r="D112" s="3" t="str">
+      <c r="A112" s="51" t="s">
+        <v>127</v>
+      </c>
+      <c r="B112" s="7">
+        <v>21194</v>
+      </c>
+      <c r="C112" s="7">
+        <v>27918</v>
+      </c>
+      <c r="D112" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>6724</v>
       </c>
     </row>
     <row r="113" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A113" s="7"/>
-      <c r="B113" s="7"/>
+      <c r="A113" s="51"/>
+      <c r="B113" s="7">
+        <v>21266</v>
+      </c>
       <c r="C113" s="7"/>
-      <c r="D113" s="3" t="str">
+      <c r="D113" s="3"/>
+    </row>
+    <row r="114" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A114" s="51" t="s">
+        <v>322</v>
+      </c>
+      <c r="B114" s="7">
+        <v>22192</v>
+      </c>
+      <c r="C114" s="7">
+        <v>28938</v>
+      </c>
+      <c r="D114" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A114" s="34"/>
-      <c r="B114" s="7"/>
-      <c r="C114" s="7"/>
-      <c r="D114" s="3" t="str">
+        <v>6746</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A115" s="51" t="s">
+        <v>323</v>
+      </c>
+      <c r="B115" s="7">
+        <v>22549</v>
+      </c>
+      <c r="C115" s="7">
+        <v>29449</v>
+      </c>
+      <c r="D115" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A115" s="7"/>
-      <c r="B115" s="7"/>
-      <c r="C115" s="7"/>
-      <c r="D115" s="3" t="str">
+        <v>6900</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A116" s="51" t="s">
+        <v>319</v>
+      </c>
+      <c r="B116" s="7">
+        <v>22613</v>
+      </c>
+      <c r="C116" s="7">
+        <v>29514</v>
+      </c>
+      <c r="D116" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A116" s="5"/>
-      <c r="B116" s="7"/>
-      <c r="C116" s="7"/>
-      <c r="D116" s="3" t="str">
+        <v>6901</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A117" s="51" t="s">
+        <v>311</v>
+      </c>
+      <c r="B117" s="7">
+        <v>22650</v>
+      </c>
+      <c r="C117" s="7">
+        <v>29551</v>
+      </c>
+      <c r="D117" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A117" s="5"/>
-      <c r="B117" s="7"/>
-      <c r="C117" s="7"/>
-      <c r="D117" s="3" t="str">
+        <v>6901</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A118" s="51" t="s">
+        <v>312</v>
+      </c>
+      <c r="B118" s="7">
+        <v>22658</v>
+      </c>
+      <c r="C118" s="7">
+        <v>29559</v>
+      </c>
+      <c r="D118" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A118" s="5"/>
-      <c r="B118" s="7"/>
-      <c r="C118" s="7"/>
-      <c r="D118" s="3" t="str">
+        <v>6901</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A119" s="51" t="s">
+        <v>293</v>
+      </c>
+      <c r="B119" s="7">
+        <v>22684</v>
+      </c>
+      <c r="C119" s="7">
+        <v>29585</v>
+      </c>
+      <c r="D119" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A119" s="5"/>
-      <c r="B119" s="7"/>
-      <c r="C119" s="7"/>
-      <c r="D119" s="3" t="str">
+        <v>6901</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A120" s="51" t="s">
+        <v>265</v>
+      </c>
+      <c r="B120" s="7">
+        <v>22824</v>
+      </c>
+      <c r="C120" s="7">
+        <v>29726</v>
+      </c>
+      <c r="D120" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A120" s="5"/>
-      <c r="B120" s="7"/>
-      <c r="C120" s="7"/>
-      <c r="D120" s="3" t="str">
+        <v>6902</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A121" s="51" t="s">
+        <v>324</v>
+      </c>
+      <c r="B121" s="7">
+        <v>22963</v>
+      </c>
+      <c r="C121" s="7">
+        <v>29871</v>
+      </c>
+      <c r="D121" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A121" s="5"/>
-      <c r="B121" s="7"/>
-      <c r="C121" s="7"/>
-      <c r="D121" s="3" t="str">
+        <v>6908</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A122" s="51" t="s">
+        <v>325</v>
+      </c>
+      <c r="B122" s="7">
+        <v>23359</v>
+      </c>
+      <c r="C122" s="7">
+        <v>30519</v>
+      </c>
+      <c r="D122" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A122" s="5"/>
-      <c r="B122" s="7"/>
-      <c r="C122" s="7"/>
-      <c r="D122" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
+        <v>7160</v>
       </c>
     </row>
     <row r="123" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -3700,8 +3781,8 @@
     </row>
     <row r="133" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A133" s="5"/>
-      <c r="B133" s="10"/>
-      <c r="C133" s="10"/>
+      <c r="B133" s="7"/>
+      <c r="C133" s="7"/>
       <c r="D133" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -3717,7 +3798,7 @@
       </c>
     </row>
     <row r="135" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A135" s="35"/>
+      <c r="A135" s="5"/>
       <c r="B135" s="7"/>
       <c r="C135" s="7"/>
       <c r="D135" s="3" t="str">
@@ -3754,8 +3835,8 @@
     </row>
     <row r="139" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A139" s="5"/>
-      <c r="B139" s="7"/>
-      <c r="C139" s="7"/>
+      <c r="B139" s="10"/>
+      <c r="C139" s="10"/>
       <c r="D139" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -3765,35 +3846,40 @@
       <c r="A140" s="5"/>
       <c r="B140" s="7"/>
       <c r="C140" s="7"/>
-      <c r="D140" s="3"/>
+      <c r="D140" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="141" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A141" s="5"/>
+      <c r="A141" s="35"/>
       <c r="B141" s="7"/>
       <c r="C141" s="7"/>
-      <c r="D141" s="3"/>
+      <c r="D141" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="142" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A142" s="5"/>
       <c r="B142" s="7"/>
       <c r="C142" s="7"/>
-      <c r="D142" s="3"/>
+      <c r="D142" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="143" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A143" s="5" t="s">
-        <v>26</v>
-      </c>
+      <c r="A143" s="5"/>
       <c r="B143" s="7"/>
-      <c r="C143" s="7">
-        <v>63782</v>
-      </c>
+      <c r="C143" s="7"/>
       <c r="D143" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="144" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A144" s="7"/>
+      <c r="A144" s="5"/>
       <c r="B144" s="7"/>
       <c r="C144" s="7"/>
       <c r="D144" s="3" t="str">
@@ -3802,7 +3888,7 @@
       </c>
     </row>
     <row r="145" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A145" s="7"/>
+      <c r="A145" s="5"/>
       <c r="B145" s="7"/>
       <c r="C145" s="7"/>
       <c r="D145" s="3" t="str">
@@ -3811,36 +3897,31 @@
       </c>
     </row>
     <row r="146" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A146" s="7"/>
+      <c r="A146" s="5"/>
       <c r="B146" s="7"/>
       <c r="C146" s="7"/>
-      <c r="D146" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="D146" s="3"/>
     </row>
     <row r="147" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A147" s="7"/>
+      <c r="A147" s="5"/>
       <c r="B147" s="7"/>
       <c r="C147" s="7"/>
-      <c r="D147" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="D147" s="3"/>
     </row>
     <row r="148" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A148" s="7"/>
+      <c r="A148" s="5"/>
       <c r="B148" s="7"/>
       <c r="C148" s="7"/>
-      <c r="D148" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="D148" s="3"/>
     </row>
     <row r="149" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A149" s="7"/>
+      <c r="A149" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="B149" s="7"/>
-      <c r="C149" s="7"/>
+      <c r="C149" s="7">
+        <v>63782</v>
+      </c>
       <c r="D149" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -4076,7 +4157,7 @@
       <c r="B175" s="7"/>
       <c r="C175" s="7"/>
       <c r="D175" s="3" t="str">
-        <f t="shared" ref="D175:D179" si="6">IF(C175&lt;&gt;"",IF(B175&lt;&gt;"",C175-B175,"-"), "-")</f>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4085,7 +4166,7 @@
       <c r="B176" s="7"/>
       <c r="C176" s="7"/>
       <c r="D176" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4094,7 +4175,7 @@
       <c r="B177" s="7"/>
       <c r="C177" s="7"/>
       <c r="D177" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4103,7 +4184,7 @@
       <c r="B178" s="7"/>
       <c r="C178" s="7"/>
       <c r="D178" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4112,7 +4193,7 @@
       <c r="B179" s="7"/>
       <c r="C179" s="7"/>
       <c r="D179" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4121,7 +4202,7 @@
       <c r="B180" s="7"/>
       <c r="C180" s="7"/>
       <c r="D180" s="3" t="str">
-        <f t="shared" ref="D180:D181" si="7">IF(C180&lt;&gt;"",IF(B180&lt;&gt;"",B180-C180,"-"), "-")</f>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4130,7 +4211,7 @@
       <c r="B181" s="7"/>
       <c r="C181" s="7"/>
       <c r="D181" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="D181:D185" si="6">IF(C181&lt;&gt;"",IF(B181&lt;&gt;"",C181-B181,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -4138,33 +4219,63 @@
       <c r="A182" s="7"/>
       <c r="B182" s="7"/>
       <c r="C182" s="7"/>
+      <c r="D182" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="183" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A183" s="7"/>
       <c r="B183" s="7"/>
       <c r="C183" s="7"/>
+      <c r="D183" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="184" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A184" s="7"/>
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
+      <c r="D184" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="185" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A185" s="7"/>
       <c r="B185" s="7"/>
       <c r="C185" s="7"/>
+      <c r="D185" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="186" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A186" s="7"/>
       <c r="B186" s="7"/>
       <c r="C186" s="7"/>
+      <c r="D186" s="3" t="str">
+        <f t="shared" ref="D186:D187" si="7">IF(C186&lt;&gt;"",IF(B186&lt;&gt;"",B186-C186,"-"), "-")</f>
+        <v>-</v>
+      </c>
     </row>
     <row r="187" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A187" s="7"/>
       <c r="B187" s="7"/>
       <c r="C187" s="7"/>
+      <c r="D187" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="188" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A188" s="7"/>
       <c r="B188" s="7"/>
       <c r="C188" s="7"/>
     </row>
     <row r="189" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A189" s="7"/>
       <c r="B189" s="7"/>
       <c r="C189" s="7"/>
     </row>
@@ -4691,6 +4802,30 @@
     <row r="320" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B320" s="7"/>
       <c r="C320" s="7"/>
+    </row>
+    <row r="321" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B321" s="7"/>
+      <c r="C321" s="7"/>
+    </row>
+    <row r="322" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B322" s="7"/>
+      <c r="C322" s="7"/>
+    </row>
+    <row r="323" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B323" s="7"/>
+      <c r="C323" s="7"/>
+    </row>
+    <row r="324" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B324" s="7"/>
+      <c r="C324" s="7"/>
+    </row>
+    <row r="325" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B325" s="7"/>
+      <c r="C325" s="7"/>
+    </row>
+    <row r="326" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B326" s="7"/>
+      <c r="C326" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14684,7 +14819,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="23" type="noConversion"/>
+  <phoneticPr fontId="24" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -14714,10 +14849,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="42" t="s">
+      <c r="K1" s="43" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="43"/>
+      <c r="L1" s="44"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -16569,13 +16704,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="44" t="s">
+      <c r="H53" s="45" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="45"/>
-      <c r="J53" s="45"/>
-      <c r="K53" s="45"/>
-      <c r="L53" s="46"/>
+      <c r="I53" s="46"/>
+      <c r="J53" s="46"/>
+      <c r="K53" s="46"/>
+      <c r="L53" s="47"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -16597,11 +16732,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="47"/>
-      <c r="I54" s="48"/>
-      <c r="J54" s="48"/>
-      <c r="K54" s="48"/>
-      <c r="L54" s="49"/>
+      <c r="H54" s="48"/>
+      <c r="I54" s="49"/>
+      <c r="J54" s="49"/>
+      <c r="K54" s="49"/>
+      <c r="L54" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
level 26 done - 7817 frames ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47D5076-C857-4E53-9372-4C2E3A72DC7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEE96780-E60F-4048-B269-49BE0DC0CE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="330">
   <si>
     <t>Place</t>
   </si>
@@ -1013,6 +1013,18 @@
   </si>
   <si>
     <t>25 ladder grab</t>
+  </si>
+  <si>
+    <t>lv 25 end</t>
+  </si>
+  <si>
+    <t>lv 26 ladder grab</t>
+  </si>
+  <si>
+    <t>lv 26 end</t>
+  </si>
+  <si>
+    <t>lv 27 1st move</t>
   </si>
 </sst>
 </file>
@@ -1868,7 +1880,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E326"/>
+  <dimension ref="A1:E328"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -3452,7 +3464,7 @@
         <v>26982</v>
       </c>
       <c r="D106" s="3">
-        <f t="shared" ref="D106:D180" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
+        <f t="shared" ref="D106:D182" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
         <v>6441</v>
       </c>
     </row>
@@ -3690,102 +3702,168 @@
       </c>
     </row>
     <row r="123" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A123" s="5"/>
-      <c r="B123" s="7"/>
-      <c r="C123" s="7"/>
-      <c r="D123" s="3" t="str">
+      <c r="A123" s="51" t="s">
+        <v>261</v>
+      </c>
+      <c r="B123" s="7">
+        <v>23409</v>
+      </c>
+      <c r="C123" s="7">
+        <v>30570</v>
+      </c>
+      <c r="D123" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>7161</v>
       </c>
     </row>
     <row r="124" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A124" s="5"/>
-      <c r="B124" s="7"/>
-      <c r="C124" s="7"/>
-      <c r="D124" s="3" t="str">
+      <c r="A124" s="51" t="s">
+        <v>312</v>
+      </c>
+      <c r="B124" s="7">
+        <v>23500</v>
+      </c>
+      <c r="C124" s="7">
+        <v>30662</v>
+      </c>
+      <c r="D124" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>7162</v>
       </c>
     </row>
     <row r="125" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A125" s="5"/>
-      <c r="B125" s="7"/>
-      <c r="C125" s="7"/>
-      <c r="D125" s="3" t="str">
+      <c r="A125" s="51" t="s">
+        <v>247</v>
+      </c>
+      <c r="B125" s="7">
+        <v>23634</v>
+      </c>
+      <c r="C125" s="7">
+        <v>30801</v>
+      </c>
+      <c r="D125" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>7167</v>
       </c>
     </row>
     <row r="126" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A126" s="5"/>
-      <c r="B126" s="7"/>
-      <c r="C126" s="7"/>
-      <c r="D126" s="3" t="str">
+      <c r="A126" s="51" t="s">
+        <v>302</v>
+      </c>
+      <c r="B126" s="7">
+        <v>23688</v>
+      </c>
+      <c r="C126" s="7">
+        <v>30855</v>
+      </c>
+      <c r="D126" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>7167</v>
       </c>
     </row>
     <row r="127" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A127" s="5"/>
-      <c r="B127" s="7"/>
-      <c r="C127" s="7"/>
-      <c r="D127" s="3" t="str">
+      <c r="A127" s="51" t="s">
+        <v>248</v>
+      </c>
+      <c r="B127" s="7">
+        <v>23794</v>
+      </c>
+      <c r="C127" s="7">
+        <v>30962</v>
+      </c>
+      <c r="D127" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>7168</v>
       </c>
     </row>
     <row r="128" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A128" s="5"/>
-      <c r="B128" s="7"/>
-      <c r="C128" s="7"/>
-      <c r="D128" s="3" t="str">
+      <c r="A128" s="51" t="s">
+        <v>326</v>
+      </c>
+      <c r="B128" s="7">
+        <v>23863</v>
+      </c>
+      <c r="C128" s="7">
+        <v>31054</v>
+      </c>
+      <c r="D128" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>7191</v>
       </c>
     </row>
     <row r="129" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A129" s="5"/>
-      <c r="B129" s="7"/>
-      <c r="C129" s="7"/>
-      <c r="D129" s="3" t="str">
+      <c r="A129" s="51" t="s">
+        <v>327</v>
+      </c>
+      <c r="B129" s="7">
+        <v>24238</v>
+      </c>
+      <c r="C129" s="7">
+        <v>31723</v>
+      </c>
+      <c r="D129" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>7485</v>
       </c>
     </row>
     <row r="130" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A130" s="5"/>
-      <c r="B130" s="7"/>
-      <c r="C130" s="7"/>
-      <c r="D130" s="3" t="str">
+      <c r="A130" s="51" t="s">
+        <v>293</v>
+      </c>
+      <c r="B130" s="7">
+        <v>24844</v>
+      </c>
+      <c r="C130" s="7">
+        <v>32330</v>
+      </c>
+      <c r="D130" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>7486</v>
       </c>
     </row>
     <row r="131" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A131" s="5"/>
-      <c r="B131" s="7"/>
-      <c r="C131" s="7"/>
-      <c r="D131" s="3" t="str">
+      <c r="A131" s="51" t="s">
+        <v>265</v>
+      </c>
+      <c r="B131" s="7">
+        <v>24975</v>
+      </c>
+      <c r="C131" s="7">
+        <v>32473</v>
+      </c>
+      <c r="D131" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>7498</v>
       </c>
     </row>
     <row r="132" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A132" s="5"/>
-      <c r="B132" s="7"/>
-      <c r="C132" s="7"/>
-      <c r="D132" s="3" t="str">
+      <c r="A132" s="51" t="s">
+        <v>328</v>
+      </c>
+      <c r="B132" s="7">
+        <v>25098</v>
+      </c>
+      <c r="C132" s="7">
+        <v>32615</v>
+      </c>
+      <c r="D132" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>7517</v>
       </c>
     </row>
     <row r="133" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A133" s="5"/>
-      <c r="B133" s="7"/>
-      <c r="C133" s="7"/>
-      <c r="D133" s="3" t="str">
+      <c r="A133" s="51" t="s">
+        <v>329</v>
+      </c>
+      <c r="B133" s="7">
+        <v>25452</v>
+      </c>
+      <c r="C133" s="7">
+        <v>33269</v>
+      </c>
+      <c r="D133" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>7817</v>
       </c>
     </row>
     <row r="134" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -3835,8 +3913,8 @@
     </row>
     <row r="139" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A139" s="5"/>
-      <c r="B139" s="10"/>
-      <c r="C139" s="10"/>
+      <c r="B139" s="7"/>
+      <c r="C139" s="7"/>
       <c r="D139" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -3852,9 +3930,9 @@
       </c>
     </row>
     <row r="141" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A141" s="35"/>
-      <c r="B141" s="7"/>
-      <c r="C141" s="7"/>
+      <c r="A141" s="5"/>
+      <c r="B141" s="10"/>
+      <c r="C141" s="10"/>
       <c r="D141" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -3870,7 +3948,7 @@
       </c>
     </row>
     <row r="143" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A143" s="5"/>
+      <c r="A143" s="35"/>
       <c r="B143" s="7"/>
       <c r="C143" s="7"/>
       <c r="D143" s="3" t="str">
@@ -3900,13 +3978,19 @@
       <c r="A146" s="5"/>
       <c r="B146" s="7"/>
       <c r="C146" s="7"/>
-      <c r="D146" s="3"/>
+      <c r="D146" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="147" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A147" s="5"/>
       <c r="B147" s="7"/>
       <c r="C147" s="7"/>
-      <c r="D147" s="3"/>
+      <c r="D147" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="148" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A148" s="5"/>
@@ -3915,31 +3999,25 @@
       <c r="D148" s="3"/>
     </row>
     <row r="149" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A149" s="5" t="s">
-        <v>26</v>
-      </c>
+      <c r="A149" s="5"/>
       <c r="B149" s="7"/>
-      <c r="C149" s="7">
-        <v>63782</v>
-      </c>
-      <c r="D149" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="C149" s="7"/>
+      <c r="D149" s="3"/>
     </row>
     <row r="150" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A150" s="7"/>
+      <c r="A150" s="5"/>
       <c r="B150" s="7"/>
       <c r="C150" s="7"/>
-      <c r="D150" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="D150" s="3"/>
     </row>
     <row r="151" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A151" s="7"/>
+      <c r="A151" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="B151" s="7"/>
-      <c r="C151" s="7"/>
+      <c r="C151" s="7">
+        <v>63782</v>
+      </c>
       <c r="D151" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -4211,7 +4289,7 @@
       <c r="B181" s="7"/>
       <c r="C181" s="7"/>
       <c r="D181" s="3" t="str">
-        <f t="shared" ref="D181:D185" si="6">IF(C181&lt;&gt;"",IF(B181&lt;&gt;"",C181-B181,"-"), "-")</f>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4220,7 +4298,7 @@
       <c r="B182" s="7"/>
       <c r="C182" s="7"/>
       <c r="D182" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4229,7 +4307,7 @@
       <c r="B183" s="7"/>
       <c r="C183" s="7"/>
       <c r="D183" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="D183:D187" si="6">IF(C183&lt;&gt;"",IF(B183&lt;&gt;"",C183-B183,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -4256,7 +4334,7 @@
       <c r="B186" s="7"/>
       <c r="C186" s="7"/>
       <c r="D186" s="3" t="str">
-        <f t="shared" ref="D186:D187" si="7">IF(C186&lt;&gt;"",IF(B186&lt;&gt;"",B186-C186,"-"), "-")</f>
+        <f t="shared" si="6"/>
         <v>-</v>
       </c>
     </row>
@@ -4265,7 +4343,7 @@
       <c r="B187" s="7"/>
       <c r="C187" s="7"/>
       <c r="D187" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-</v>
       </c>
     </row>
@@ -4273,17 +4351,27 @@
       <c r="A188" s="7"/>
       <c r="B188" s="7"/>
       <c r="C188" s="7"/>
+      <c r="D188" s="3" t="str">
+        <f t="shared" ref="D188:D189" si="7">IF(C188&lt;&gt;"",IF(B188&lt;&gt;"",B188-C188,"-"), "-")</f>
+        <v>-</v>
+      </c>
     </row>
     <row r="189" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A189" s="7"/>
       <c r="B189" s="7"/>
       <c r="C189" s="7"/>
+      <c r="D189" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="190" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A190" s="7"/>
       <c r="B190" s="7"/>
       <c r="C190" s="7"/>
     </row>
     <row r="191" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A191" s="7"/>
       <c r="B191" s="7"/>
       <c r="C191" s="7"/>
     </row>
@@ -4826,6 +4914,14 @@
     <row r="326" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B326" s="7"/>
       <c r="C326" s="7"/>
+    </row>
+    <row r="327" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B327" s="7"/>
+      <c r="C327" s="7"/>
+    </row>
+    <row r="328" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B328" s="7"/>
+      <c r="C328" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - lv 27 done - 8121 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEE96780-E60F-4048-B269-49BE0DC0CE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85D0B2C8-E73E-47C6-8581-32D4CCAB2F67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="332">
   <si>
     <t>Place</t>
   </si>
@@ -1025,6 +1025,12 @@
   </si>
   <si>
     <t>lv 27 1st move</t>
+  </si>
+  <si>
+    <t>lv 27 end</t>
+  </si>
+  <si>
+    <t>28 1st move</t>
   </si>
 </sst>
 </file>
@@ -1034,12 +1040,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="29" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1436,95 +1449,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1535,28 +1549,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1880,7 +1894,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E328"/>
+  <dimension ref="A1:E331"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -3464,7 +3478,7 @@
         <v>26982</v>
       </c>
       <c r="D106" s="3">
-        <f t="shared" ref="D106:D182" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
+        <f t="shared" ref="D106:D185" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
         <v>6441</v>
       </c>
     </row>
@@ -3544,7 +3558,7 @@
       </c>
     </row>
     <row r="112" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A112" s="51" t="s">
+      <c r="A112" s="43" t="s">
         <v>127</v>
       </c>
       <c r="B112" s="7">
@@ -3559,7 +3573,7 @@
       </c>
     </row>
     <row r="113" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A113" s="51"/>
+      <c r="A113" s="43"/>
       <c r="B113" s="7">
         <v>21266</v>
       </c>
@@ -3567,7 +3581,7 @@
       <c r="D113" s="3"/>
     </row>
     <row r="114" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A114" s="51" t="s">
+      <c r="A114" s="43" t="s">
         <v>322</v>
       </c>
       <c r="B114" s="7">
@@ -3582,7 +3596,7 @@
       </c>
     </row>
     <row r="115" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A115" s="51" t="s">
+      <c r="A115" s="43" t="s">
         <v>323</v>
       </c>
       <c r="B115" s="7">
@@ -3597,7 +3611,7 @@
       </c>
     </row>
     <row r="116" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A116" s="51" t="s">
+      <c r="A116" s="43" t="s">
         <v>319</v>
       </c>
       <c r="B116" s="7">
@@ -3612,7 +3626,7 @@
       </c>
     </row>
     <row r="117" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A117" s="51" t="s">
+      <c r="A117" s="43" t="s">
         <v>311</v>
       </c>
       <c r="B117" s="7">
@@ -3627,7 +3641,7 @@
       </c>
     </row>
     <row r="118" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A118" s="51" t="s">
+      <c r="A118" s="43" t="s">
         <v>312</v>
       </c>
       <c r="B118" s="7">
@@ -3642,7 +3656,7 @@
       </c>
     </row>
     <row r="119" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A119" s="51" t="s">
+      <c r="A119" s="43" t="s">
         <v>293</v>
       </c>
       <c r="B119" s="7">
@@ -3657,7 +3671,7 @@
       </c>
     </row>
     <row r="120" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A120" s="51" t="s">
+      <c r="A120" s="43" t="s">
         <v>265</v>
       </c>
       <c r="B120" s="7">
@@ -3672,7 +3686,7 @@
       </c>
     </row>
     <row r="121" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A121" s="51" t="s">
+      <c r="A121" s="43" t="s">
         <v>324</v>
       </c>
       <c r="B121" s="7">
@@ -3687,7 +3701,7 @@
       </c>
     </row>
     <row r="122" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A122" s="51" t="s">
+      <c r="A122" s="43" t="s">
         <v>325</v>
       </c>
       <c r="B122" s="7">
@@ -3702,7 +3716,7 @@
       </c>
     </row>
     <row r="123" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A123" s="51" t="s">
+      <c r="A123" s="43" t="s">
         <v>261</v>
       </c>
       <c r="B123" s="7">
@@ -3717,7 +3731,7 @@
       </c>
     </row>
     <row r="124" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A124" s="51" t="s">
+      <c r="A124" s="43" t="s">
         <v>312</v>
       </c>
       <c r="B124" s="7">
@@ -3732,7 +3746,7 @@
       </c>
     </row>
     <row r="125" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A125" s="51" t="s">
+      <c r="A125" s="43" t="s">
         <v>247</v>
       </c>
       <c r="B125" s="7">
@@ -3747,7 +3761,7 @@
       </c>
     </row>
     <row r="126" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A126" s="51" t="s">
+      <c r="A126" s="43" t="s">
         <v>302</v>
       </c>
       <c r="B126" s="7">
@@ -3762,7 +3776,7 @@
       </c>
     </row>
     <row r="127" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A127" s="51" t="s">
+      <c r="A127" s="43" t="s">
         <v>248</v>
       </c>
       <c r="B127" s="7">
@@ -3777,7 +3791,7 @@
       </c>
     </row>
     <row r="128" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A128" s="51" t="s">
+      <c r="A128" s="43" t="s">
         <v>326</v>
       </c>
       <c r="B128" s="7">
@@ -3791,8 +3805,8 @@
         <v>7191</v>
       </c>
     </row>
-    <row r="129" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A129" s="51" t="s">
+    <row r="129" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A129" s="43" t="s">
         <v>327</v>
       </c>
       <c r="B129" s="7">
@@ -3806,8 +3820,8 @@
         <v>7485</v>
       </c>
     </row>
-    <row r="130" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A130" s="51" t="s">
+    <row r="130" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A130" s="43" t="s">
         <v>293</v>
       </c>
       <c r="B130" s="7">
@@ -3821,8 +3835,8 @@
         <v>7486</v>
       </c>
     </row>
-    <row r="131" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A131" s="51" t="s">
+    <row r="131" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A131" s="43" t="s">
         <v>265</v>
       </c>
       <c r="B131" s="7">
@@ -3836,8 +3850,8 @@
         <v>7498</v>
       </c>
     </row>
-    <row r="132" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A132" s="51" t="s">
+    <row r="132" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A132" s="43" t="s">
         <v>328</v>
       </c>
       <c r="B132" s="7">
@@ -3851,8 +3865,8 @@
         <v>7517</v>
       </c>
     </row>
-    <row r="133" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A133" s="51" t="s">
+    <row r="133" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A133" s="43" t="s">
         <v>329</v>
       </c>
       <c r="B133" s="7">
@@ -3866,25 +3880,38 @@
         <v>7817</v>
       </c>
     </row>
-    <row r="134" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A134" s="5"/>
-      <c r="B134" s="7"/>
-      <c r="C134" s="7"/>
-      <c r="D134" s="3" t="str">
+    <row r="134" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A134" s="52" t="s">
+        <v>330</v>
+      </c>
+      <c r="B134" s="7">
+        <v>26350</v>
+      </c>
+      <c r="C134" s="7">
+        <v>34168</v>
+      </c>
+      <c r="D134" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A135" s="5"/>
-      <c r="B135" s="7"/>
-      <c r="C135" s="7"/>
-      <c r="D135" s="3" t="str">
+        <v>7818</v>
+      </c>
+      <c r="E134" s="7"/>
+    </row>
+    <row r="135" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A135" s="52" t="s">
+        <v>331</v>
+      </c>
+      <c r="B135" s="7">
+        <v>26701</v>
+      </c>
+      <c r="C135" s="7">
+        <v>34822</v>
+      </c>
+      <c r="D135" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <v>8121</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A136" s="5"/>
       <c r="B136" s="7"/>
       <c r="C136" s="7"/>
@@ -3893,7 +3920,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="137" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A137" s="5"/>
       <c r="B137" s="7"/>
       <c r="C137" s="7"/>
@@ -3902,7 +3929,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="138" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A138" s="5"/>
       <c r="B138" s="7"/>
       <c r="C138" s="7"/>
@@ -3911,7 +3938,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="139" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A139" s="5"/>
       <c r="B139" s="7"/>
       <c r="C139" s="7"/>
@@ -3920,7 +3947,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="140" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A140" s="5"/>
       <c r="B140" s="7"/>
       <c r="C140" s="7"/>
@@ -3929,16 +3956,16 @@
         <v>-</v>
       </c>
     </row>
-    <row r="141" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A141" s="5"/>
-      <c r="B141" s="10"/>
-      <c r="C141" s="10"/>
+      <c r="B141" s="7"/>
+      <c r="C141" s="7"/>
       <c r="D141" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
-    <row r="142" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A142" s="5"/>
       <c r="B142" s="7"/>
       <c r="C142" s="7"/>
@@ -3947,8 +3974,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="143" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A143" s="35"/>
+    <row r="143" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A143" s="5"/>
       <c r="B143" s="7"/>
       <c r="C143" s="7"/>
       <c r="D143" s="3" t="str">
@@ -3956,10 +3983,10 @@
         <v>-</v>
       </c>
     </row>
-    <row r="144" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A144" s="5"/>
-      <c r="B144" s="7"/>
-      <c r="C144" s="7"/>
+      <c r="B144" s="10"/>
+      <c r="C144" s="10"/>
       <c r="D144" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -3975,7 +4002,7 @@
       </c>
     </row>
     <row r="146" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A146" s="5"/>
+      <c r="A146" s="35"/>
       <c r="B146" s="7"/>
       <c r="C146" s="7"/>
       <c r="D146" s="3" t="str">
@@ -3996,55 +4023,55 @@
       <c r="A148" s="5"/>
       <c r="B148" s="7"/>
       <c r="C148" s="7"/>
-      <c r="D148" s="3"/>
+      <c r="D148" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="149" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A149" s="5"/>
       <c r="B149" s="7"/>
       <c r="C149" s="7"/>
-      <c r="D149" s="3"/>
+      <c r="D149" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="150" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A150" s="5"/>
       <c r="B150" s="7"/>
       <c r="C150" s="7"/>
-      <c r="D150" s="3"/>
+      <c r="D150" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="151" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A151" s="5" t="s">
-        <v>26</v>
-      </c>
+      <c r="A151" s="5"/>
       <c r="B151" s="7"/>
-      <c r="C151" s="7">
-        <v>63782</v>
-      </c>
-      <c r="D151" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="C151" s="7"/>
+      <c r="D151" s="3"/>
     </row>
     <row r="152" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A152" s="7"/>
+      <c r="A152" s="5"/>
       <c r="B152" s="7"/>
       <c r="C152" s="7"/>
-      <c r="D152" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="D152" s="3"/>
     </row>
     <row r="153" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A153" s="7"/>
+      <c r="A153" s="5"/>
       <c r="B153" s="7"/>
       <c r="C153" s="7"/>
-      <c r="D153" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
+      <c r="D153" s="3"/>
     </row>
     <row r="154" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A154" s="7"/>
+      <c r="A154" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="B154" s="7"/>
-      <c r="C154" s="7"/>
+      <c r="C154" s="7">
+        <v>63782</v>
+      </c>
       <c r="D154" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
@@ -4307,7 +4334,7 @@
       <c r="B183" s="7"/>
       <c r="C183" s="7"/>
       <c r="D183" s="3" t="str">
-        <f t="shared" ref="D183:D187" si="6">IF(C183&lt;&gt;"",IF(B183&lt;&gt;"",C183-B183,"-"), "-")</f>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4316,7 +4343,7 @@
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
       <c r="D184" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4325,7 +4352,7 @@
       <c r="B185" s="7"/>
       <c r="C185" s="7"/>
       <c r="D185" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4334,7 +4361,7 @@
       <c r="B186" s="7"/>
       <c r="C186" s="7"/>
       <c r="D186" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="D186:D190" si="6">IF(C186&lt;&gt;"",IF(B186&lt;&gt;"",C186-B186,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -4352,7 +4379,7 @@
       <c r="B188" s="7"/>
       <c r="C188" s="7"/>
       <c r="D188" s="3" t="str">
-        <f t="shared" ref="D188:D189" si="7">IF(C188&lt;&gt;"",IF(B188&lt;&gt;"",B188-C188,"-"), "-")</f>
+        <f t="shared" si="6"/>
         <v>-</v>
       </c>
     </row>
@@ -4361,7 +4388,7 @@
       <c r="B189" s="7"/>
       <c r="C189" s="7"/>
       <c r="D189" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-</v>
       </c>
     </row>
@@ -4369,77 +4396,92 @@
       <c r="A190" s="7"/>
       <c r="B190" s="7"/>
       <c r="C190" s="7"/>
+      <c r="D190" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="191" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A191" s="7"/>
       <c r="B191" s="7"/>
       <c r="C191" s="7"/>
+      <c r="D191" s="3" t="str">
+        <f t="shared" ref="D191:D192" si="7">IF(C191&lt;&gt;"",IF(B191&lt;&gt;"",B191-C191,"-"), "-")</f>
+        <v>-</v>
+      </c>
     </row>
     <row r="192" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A192" s="7"/>
       <c r="B192" s="7"/>
       <c r="C192" s="7"/>
-    </row>
-    <row r="193" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D192" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A193" s="7"/>
       <c r="B193" s="7"/>
       <c r="C193" s="7"/>
     </row>
-    <row r="194" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A194" s="7"/>
       <c r="B194" s="7"/>
       <c r="C194" s="7"/>
     </row>
-    <row r="195" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B195" s="7"/>
       <c r="C195" s="7"/>
     </row>
-    <row r="196" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B196" s="7"/>
       <c r="C196" s="7"/>
     </row>
-    <row r="197" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B197" s="7"/>
       <c r="C197" s="7"/>
     </row>
-    <row r="198" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B198" s="7"/>
       <c r="C198" s="7"/>
     </row>
-    <row r="199" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B199" s="7"/>
       <c r="C199" s="7"/>
     </row>
-    <row r="200" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B200" s="7"/>
       <c r="C200" s="7"/>
     </row>
-    <row r="201" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B201" s="7"/>
       <c r="C201" s="7"/>
     </row>
-    <row r="202" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B202" s="7"/>
       <c r="C202" s="7"/>
     </row>
-    <row r="203" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B203" s="7"/>
       <c r="C203" s="7"/>
     </row>
-    <row r="204" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B204" s="7"/>
       <c r="C204" s="7"/>
     </row>
-    <row r="205" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B205" s="7"/>
       <c r="C205" s="7"/>
     </row>
-    <row r="206" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B206" s="7"/>
       <c r="C206" s="7"/>
     </row>
-    <row r="207" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B207" s="7"/>
       <c r="C207" s="7"/>
     </row>
-    <row r="208" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B208" s="7"/>
       <c r="C208" s="7"/>
     </row>
@@ -4922,6 +4964,18 @@
     <row r="328" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B328" s="7"/>
       <c r="C328" s="7"/>
+    </row>
+    <row r="329" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B329" s="7"/>
+      <c r="C329" s="7"/>
+    </row>
+    <row r="330" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B330" s="7"/>
+      <c r="C330" s="7"/>
+    </row>
+    <row r="331" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B331" s="7"/>
+      <c r="C331" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14915,7 +14969,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="24" type="noConversion"/>
+  <phoneticPr fontId="25" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -14945,10 +14999,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="44" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="44"/>
+      <c r="L1" s="45"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -16800,13 +16854,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="45" t="s">
+      <c r="H53" s="46" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="46"/>
-      <c r="J53" s="46"/>
-      <c r="K53" s="46"/>
-      <c r="L53" s="47"/>
+      <c r="I53" s="47"/>
+      <c r="J53" s="47"/>
+      <c r="K53" s="47"/>
+      <c r="L53" s="48"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -16828,11 +16882,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="48"/>
-      <c r="I54" s="49"/>
-      <c r="J54" s="49"/>
-      <c r="K54" s="49"/>
-      <c r="L54" s="50"/>
+      <c r="H54" s="49"/>
+      <c r="I54" s="50"/>
+      <c r="J54" s="50"/>
+      <c r="K54" s="50"/>
+      <c r="L54" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - 29 done, 8567 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85D0B2C8-E73E-47C6-8581-32D4CCAB2F67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D587743-AC22-41D7-91AD-FA7965B2AC03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="339">
   <si>
     <t>Place</t>
   </si>
@@ -1031,6 +1031,27 @@
   </si>
   <si>
     <t>28 1st move</t>
+  </si>
+  <si>
+    <t>28 end</t>
+  </si>
+  <si>
+    <t>fall (gold = 5)</t>
+  </si>
+  <si>
+    <t>x = 20</t>
+  </si>
+  <si>
+    <t>move left</t>
+  </si>
+  <si>
+    <t>29 1st move</t>
+  </si>
+  <si>
+    <t>29 end</t>
+  </si>
+  <si>
+    <t>30 e 1st move</t>
   </si>
 </sst>
 </file>
@@ -1894,7 +1915,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E331"/>
+  <dimension ref="A1:E336"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -3478,7 +3499,7 @@
         <v>26982</v>
       </c>
       <c r="D106" s="3">
-        <f t="shared" ref="D106:D185" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
+        <f t="shared" ref="D106:D190" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
         <v>6441</v>
       </c>
     </row>
@@ -3912,173 +3933,268 @@
       </c>
     </row>
     <row r="136" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A136" s="5"/>
-      <c r="B136" s="7"/>
-      <c r="C136" s="7"/>
-      <c r="D136" s="3" t="str">
+      <c r="A136" s="52" t="s">
+        <v>319</v>
+      </c>
+      <c r="B136" s="7">
+        <v>26782</v>
+      </c>
+      <c r="C136" s="7">
+        <v>34903</v>
+      </c>
+      <c r="D136" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8121</v>
       </c>
     </row>
     <row r="137" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A137" s="5"/>
-      <c r="B137" s="7"/>
-      <c r="C137" s="7"/>
-      <c r="D137" s="3" t="str">
+      <c r="A137" s="52" t="s">
+        <v>333</v>
+      </c>
+      <c r="B137" s="7">
+        <v>27027</v>
+      </c>
+      <c r="C137" s="7">
+        <v>35149</v>
+      </c>
+      <c r="D137" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8122</v>
       </c>
     </row>
     <row r="138" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A138" s="5"/>
-      <c r="B138" s="7"/>
-      <c r="C138" s="7"/>
-      <c r="D138" s="3" t="str">
+      <c r="A138" s="52" t="s">
+        <v>265</v>
+      </c>
+      <c r="B138" s="7">
+        <v>27090</v>
+      </c>
+      <c r="C138" s="7">
+        <v>35212</v>
+      </c>
+      <c r="D138" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8122</v>
       </c>
     </row>
     <row r="139" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A139" s="5"/>
-      <c r="B139" s="7"/>
-      <c r="C139" s="7"/>
-      <c r="D139" s="3" t="str">
+      <c r="A139" s="52" t="s">
+        <v>302</v>
+      </c>
+      <c r="B139" s="7">
+        <v>27303</v>
+      </c>
+      <c r="C139" s="7">
+        <v>35427</v>
+      </c>
+      <c r="D139" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8124</v>
       </c>
     </row>
     <row r="140" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A140" s="5"/>
-      <c r="B140" s="7"/>
-      <c r="C140" s="7"/>
-      <c r="D140" s="3" t="str">
+      <c r="A140" s="52" t="s">
+        <v>335</v>
+      </c>
+      <c r="B140" s="7">
+        <v>27326</v>
+      </c>
+      <c r="C140" s="7">
+        <v>35449</v>
+      </c>
+      <c r="D140" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8123</v>
       </c>
     </row>
     <row r="141" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A141" s="5"/>
-      <c r="B141" s="7"/>
-      <c r="C141" s="7"/>
-      <c r="D141" s="3" t="str">
+      <c r="A141" s="52" t="s">
+        <v>334</v>
+      </c>
+      <c r="B141" s="7">
+        <v>27428</v>
+      </c>
+      <c r="C141" s="7">
+        <v>35544</v>
+      </c>
+      <c r="D141" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8116</v>
       </c>
     </row>
     <row r="142" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A142" s="5"/>
-      <c r="B142" s="7"/>
-      <c r="C142" s="7"/>
-      <c r="D142" s="3" t="str">
+      <c r="A142" s="52" t="s">
+        <v>332</v>
+      </c>
+      <c r="B142" s="7">
+        <v>27490</v>
+      </c>
+      <c r="C142" s="7">
+        <v>35629</v>
+      </c>
+      <c r="D142" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8139</v>
       </c>
     </row>
     <row r="143" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A143" s="5"/>
-      <c r="B143" s="7"/>
-      <c r="C143" s="7"/>
-      <c r="D143" s="3" t="str">
+      <c r="A143" s="52" t="s">
+        <v>336</v>
+      </c>
+      <c r="B143" s="7">
+        <v>27838</v>
+      </c>
+      <c r="C143" s="7">
+        <v>36238</v>
+      </c>
+      <c r="D143" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8400</v>
       </c>
     </row>
     <row r="144" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A144" s="5"/>
-      <c r="B144" s="10"/>
-      <c r="C144" s="10"/>
-      <c r="D144" s="3" t="str">
+      <c r="A144" s="52" t="s">
+        <v>311</v>
+      </c>
+      <c r="B144" s="7">
+        <v>27984</v>
+      </c>
+      <c r="C144" s="7">
+        <v>36384</v>
+      </c>
+      <c r="D144" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8400</v>
       </c>
     </row>
     <row r="145" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A145" s="5"/>
-      <c r="B145" s="7"/>
-      <c r="C145" s="7"/>
-      <c r="D145" s="3" t="str">
+      <c r="A145" s="52" t="s">
+        <v>312</v>
+      </c>
+      <c r="B145" s="7">
+        <v>28083</v>
+      </c>
+      <c r="C145" s="7">
+        <v>36483</v>
+      </c>
+      <c r="D145" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8400</v>
       </c>
     </row>
     <row r="146" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A146" s="35"/>
-      <c r="B146" s="7"/>
-      <c r="C146" s="7"/>
-      <c r="D146" s="3" t="str">
+      <c r="A146" s="52" t="s">
+        <v>265</v>
+      </c>
+      <c r="B146" s="7">
+        <v>28111</v>
+      </c>
+      <c r="C146" s="7">
+        <v>36511</v>
+      </c>
+      <c r="D146" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8400</v>
       </c>
     </row>
     <row r="147" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A147" s="5"/>
-      <c r="B147" s="7"/>
-      <c r="C147" s="7"/>
-      <c r="D147" s="3" t="str">
+      <c r="A147" s="52" t="s">
+        <v>265</v>
+      </c>
+      <c r="B147" s="7">
+        <v>28300</v>
+      </c>
+      <c r="C147" s="7">
+        <v>36700</v>
+      </c>
+      <c r="D147" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8400</v>
       </c>
     </row>
     <row r="148" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A148" s="5"/>
-      <c r="B148" s="7"/>
-      <c r="C148" s="7"/>
-      <c r="D148" s="3" t="str">
+      <c r="A148" s="52" t="s">
+        <v>250</v>
+      </c>
+      <c r="B148" s="7">
+        <v>28832</v>
+      </c>
+      <c r="C148" s="7">
+        <v>37239</v>
+      </c>
+      <c r="D148" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8407</v>
       </c>
     </row>
     <row r="149" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A149" s="5"/>
-      <c r="B149" s="7"/>
-      <c r="C149" s="7"/>
-      <c r="D149" s="3" t="str">
+      <c r="A149" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="B149" s="10">
+        <v>28899</v>
+      </c>
+      <c r="C149" s="10">
+        <v>37318</v>
+      </c>
+      <c r="D149" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8419</v>
       </c>
     </row>
     <row r="150" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A150" s="5"/>
-      <c r="B150" s="7"/>
-      <c r="C150" s="7"/>
-      <c r="D150" s="3" t="str">
+      <c r="A150" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="B150" s="7">
+        <v>29251</v>
+      </c>
+      <c r="C150" s="7">
+        <v>37818</v>
+      </c>
+      <c r="D150" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>8567</v>
       </c>
     </row>
     <row r="151" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A151" s="5"/>
+      <c r="A151" s="35"/>
       <c r="B151" s="7"/>
       <c r="C151" s="7"/>
-      <c r="D151" s="3"/>
+      <c r="D151" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="152" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A152" s="5"/>
       <c r="B152" s="7"/>
       <c r="C152" s="7"/>
-      <c r="D152" s="3"/>
+      <c r="D152" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="153" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A153" s="5"/>
       <c r="B153" s="7"/>
       <c r="C153" s="7"/>
-      <c r="D153" s="3"/>
+      <c r="D153" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="154" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A154" s="5" t="s">
-        <v>26</v>
-      </c>
+      <c r="A154" s="5"/>
       <c r="B154" s="7"/>
-      <c r="C154" s="7">
-        <v>63782</v>
-      </c>
+      <c r="C154" s="7"/>
       <c r="D154" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
     <row r="155" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A155" s="7"/>
+      <c r="A155" s="5"/>
       <c r="B155" s="7"/>
       <c r="C155" s="7"/>
       <c r="D155" s="3" t="str">
@@ -4087,7 +4203,7 @@
       </c>
     </row>
     <row r="156" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A156" s="7"/>
+      <c r="A156" s="5"/>
       <c r="B156" s="7"/>
       <c r="C156" s="7"/>
       <c r="D156" s="3" t="str">
@@ -4096,7 +4212,7 @@
       </c>
     </row>
     <row r="157" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A157" s="7"/>
+      <c r="A157" s="5"/>
       <c r="B157" s="7"/>
       <c r="C157" s="7"/>
       <c r="D157" s="3" t="str">
@@ -4105,7 +4221,7 @@
       </c>
     </row>
     <row r="158" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A158" s="7"/>
+      <c r="A158" s="5"/>
       <c r="B158" s="7"/>
       <c r="C158" s="7"/>
       <c r="D158" s="3" t="str">
@@ -4114,7 +4230,7 @@
       </c>
     </row>
     <row r="159" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A159" s="7"/>
+      <c r="A159" s="5"/>
       <c r="B159" s="7"/>
       <c r="C159" s="7"/>
       <c r="D159" s="3" t="str">
@@ -4361,7 +4477,7 @@
       <c r="B186" s="7"/>
       <c r="C186" s="7"/>
       <c r="D186" s="3" t="str">
-        <f t="shared" ref="D186:D190" si="6">IF(C186&lt;&gt;"",IF(B186&lt;&gt;"",C186-B186,"-"), "-")</f>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4370,7 +4486,7 @@
       <c r="B187" s="7"/>
       <c r="C187" s="7"/>
       <c r="D187" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4379,7 +4495,7 @@
       <c r="B188" s="7"/>
       <c r="C188" s="7"/>
       <c r="D188" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4388,7 +4504,7 @@
       <c r="B189" s="7"/>
       <c r="C189" s="7"/>
       <c r="D189" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4397,7 +4513,7 @@
       <c r="B190" s="7"/>
       <c r="C190" s="7"/>
       <c r="D190" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4406,7 +4522,7 @@
       <c r="B191" s="7"/>
       <c r="C191" s="7"/>
       <c r="D191" s="3" t="str">
-        <f t="shared" ref="D191:D192" si="7">IF(C191&lt;&gt;"",IF(B191&lt;&gt;"",B191-C191,"-"), "-")</f>
+        <f t="shared" ref="D191:D195" si="6">IF(C191&lt;&gt;"",IF(B191&lt;&gt;"",C191-B191,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -4415,73 +4531,102 @@
       <c r="B192" s="7"/>
       <c r="C192" s="7"/>
       <c r="D192" s="3" t="str">
-        <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="193" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A193" s="7"/>
       <c r="B193" s="7"/>
       <c r="C193" s="7"/>
-    </row>
-    <row r="194" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D193" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A194" s="7"/>
       <c r="B194" s="7"/>
       <c r="C194" s="7"/>
-    </row>
-    <row r="195" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D194" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A195" s="7"/>
       <c r="B195" s="7"/>
       <c r="C195" s="7"/>
-    </row>
-    <row r="196" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D195" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A196" s="7"/>
       <c r="B196" s="7"/>
       <c r="C196" s="7"/>
-    </row>
-    <row r="197" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D196" s="3" t="str">
+        <f t="shared" ref="D196:D197" si="7">IF(C196&lt;&gt;"",IF(B196&lt;&gt;"",B196-C196,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A197" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="B197" s="7"/>
-      <c r="C197" s="7"/>
-    </row>
-    <row r="198" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C197" s="7">
+        <v>63782</v>
+      </c>
+      <c r="D197" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A198" s="7"/>
       <c r="B198" s="7"/>
       <c r="C198" s="7"/>
     </row>
-    <row r="199" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A199" s="7"/>
       <c r="B199" s="7"/>
       <c r="C199" s="7"/>
     </row>
-    <row r="200" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B200" s="7"/>
       <c r="C200" s="7"/>
     </row>
-    <row r="201" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B201" s="7"/>
       <c r="C201" s="7"/>
     </row>
-    <row r="202" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B202" s="7"/>
       <c r="C202" s="7"/>
     </row>
-    <row r="203" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B203" s="7"/>
       <c r="C203" s="7"/>
     </row>
-    <row r="204" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B204" s="7"/>
       <c r="C204" s="7"/>
     </row>
-    <row r="205" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B205" s="7"/>
       <c r="C205" s="7"/>
     </row>
-    <row r="206" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B206" s="7"/>
       <c r="C206" s="7"/>
     </row>
-    <row r="207" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B207" s="7"/>
       <c r="C207" s="7"/>
     </row>
-    <row r="208" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B208" s="7"/>
       <c r="C208" s="7"/>
     </row>
@@ -4976,6 +5121,26 @@
     <row r="331" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B331" s="7"/>
       <c r="C331" s="7"/>
+    </row>
+    <row r="332" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B332" s="7"/>
+      <c r="C332" s="7"/>
+    </row>
+    <row r="333" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B333" s="7"/>
+      <c r="C333" s="7"/>
+    </row>
+    <row r="334" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B334" s="7"/>
+      <c r="C334" s="7"/>
+    </row>
+    <row r="335" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B335" s="7"/>
+      <c r="C335" s="7"/>
+    </row>
+    <row r="336" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B336" s="7"/>
+      <c r="C336" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - 31 done, 8849 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D587743-AC22-41D7-91AD-FA7965B2AC03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CACEB26-9CCB-428A-89E7-5F707837CD14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="344">
   <si>
     <t>Place</t>
   </si>
@@ -1052,6 +1052,21 @@
   </si>
   <si>
     <t>30 e 1st move</t>
+  </si>
+  <si>
+    <t>E2 X = 15</t>
+  </si>
+  <si>
+    <t>enemy dies</t>
+  </si>
+  <si>
+    <t>luck manip</t>
+  </si>
+  <si>
+    <t>29390 if no delay</t>
+  </si>
+  <si>
+    <t>31 ladder grab</t>
   </si>
 </sst>
 </file>
@@ -1915,7 +1930,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E336"/>
+  <dimension ref="A1:E332"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -3499,7 +3514,7 @@
         <v>26982</v>
       </c>
       <c r="D106" s="3">
-        <f t="shared" ref="D106:D190" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
+        <f t="shared" ref="D106:D186" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
         <v>6441</v>
       </c>
     </row>
@@ -4067,7 +4082,7 @@
         <v>8400</v>
       </c>
     </row>
-    <row r="145" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A145" s="52" t="s">
         <v>312</v>
       </c>
@@ -4082,7 +4097,7 @@
         <v>8400</v>
       </c>
     </row>
-    <row r="146" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A146" s="52" t="s">
         <v>265</v>
       </c>
@@ -4097,7 +4112,7 @@
         <v>8400</v>
       </c>
     </row>
-    <row r="147" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A147" s="52" t="s">
         <v>265</v>
       </c>
@@ -4112,7 +4127,7 @@
         <v>8400</v>
       </c>
     </row>
-    <row r="148" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A148" s="52" t="s">
         <v>250</v>
       </c>
@@ -4127,7 +4142,7 @@
         <v>8407</v>
       </c>
     </row>
-    <row r="149" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A149" s="52" t="s">
         <v>337</v>
       </c>
@@ -4142,7 +4157,7 @@
         <v>8419</v>
       </c>
     </row>
-    <row r="150" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A150" s="52" t="s">
         <v>338</v>
       </c>
@@ -4157,80 +4172,134 @@
         <v>8567</v>
       </c>
     </row>
-    <row r="151" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A151" s="35"/>
-      <c r="B151" s="7"/>
-      <c r="C151" s="7"/>
-      <c r="D151" s="3" t="str">
+    <row r="151" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A151" s="52" t="s">
+        <v>339</v>
+      </c>
+      <c r="B151" s="7">
+        <v>29251</v>
+      </c>
+      <c r="C151" s="7">
+        <v>37818</v>
+      </c>
+      <c r="D151" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="152" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A152" s="5"/>
-      <c r="B152" s="7"/>
-      <c r="C152" s="7"/>
-      <c r="D152" s="3" t="str">
+        <v>8567</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A152" s="52" t="s">
+        <v>150</v>
+      </c>
+      <c r="B152" s="7">
+        <v>29377</v>
+      </c>
+      <c r="C152" s="7">
+        <v>37941</v>
+      </c>
+      <c r="D152" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="153" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A153" s="5"/>
-      <c r="B153" s="7"/>
-      <c r="C153" s="7"/>
-      <c r="D153" s="3" t="str">
+        <v>8564</v>
+      </c>
+      <c r="E152" s="52" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A153" s="52" t="s">
+        <v>340</v>
+      </c>
+      <c r="B153" s="7">
+        <v>29508</v>
+      </c>
+      <c r="C153" s="7">
+        <v>38068</v>
+      </c>
+      <c r="D153" s="3">
+        <f t="shared" ref="D153" si="6">IF(C153&lt;&gt;"",IF(B153&lt;&gt;"",C153-B153,"-"), "-")</f>
+        <v>8560</v>
+      </c>
+      <c r="E153" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A154" s="52" t="s">
+        <v>312</v>
+      </c>
+      <c r="B154" s="7">
+        <v>29615</v>
+      </c>
+      <c r="C154" s="7">
+        <v>38174</v>
+      </c>
+      <c r="D154" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="154" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A154" s="5"/>
-      <c r="B154" s="7"/>
-      <c r="C154" s="7"/>
-      <c r="D154" s="3" t="str">
+        <v>8559</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A155" s="52" t="s">
+        <v>150</v>
+      </c>
+      <c r="B155" s="7">
+        <v>29666</v>
+      </c>
+      <c r="C155" s="7">
+        <v>38224</v>
+      </c>
+      <c r="D155" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="155" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A155" s="5"/>
-      <c r="B155" s="7"/>
-      <c r="C155" s="7"/>
-      <c r="D155" s="3" t="str">
+        <v>8558</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A156" s="52" t="s">
+        <v>293</v>
+      </c>
+      <c r="B156" s="7">
+        <v>29771</v>
+      </c>
+      <c r="C156" s="7">
+        <v>38329</v>
+      </c>
+      <c r="D156" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="156" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A156" s="5"/>
-      <c r="B156" s="7"/>
-      <c r="C156" s="7"/>
-      <c r="D156" s="3" t="str">
+        <v>8558</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A157" s="52" t="s">
+        <v>45</v>
+      </c>
+      <c r="B157" s="7">
+        <v>29961</v>
+      </c>
+      <c r="C157" s="7">
+        <v>38519</v>
+      </c>
+      <c r="D157" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="157" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A157" s="5"/>
-      <c r="B157" s="7"/>
-      <c r="C157" s="7"/>
-      <c r="D157" s="3" t="str">
+        <v>8558</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A158" s="52" t="s">
+        <v>343</v>
+      </c>
+      <c r="B158" s="7">
+        <v>30313</v>
+      </c>
+      <c r="C158" s="7">
+        <v>39162</v>
+      </c>
+      <c r="D158" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="158" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A158" s="5"/>
-      <c r="B158" s="7"/>
-      <c r="C158" s="7"/>
-      <c r="D158" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="159" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A159" s="5"/>
+        <v>8849</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A159" s="7"/>
       <c r="B159" s="7"/>
       <c r="C159" s="7"/>
       <c r="D159" s="3" t="str">
@@ -4238,7 +4307,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="160" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A160" s="7"/>
       <c r="B160" s="7"/>
       <c r="C160" s="7"/>
@@ -4486,7 +4555,7 @@
       <c r="B187" s="7"/>
       <c r="C187" s="7"/>
       <c r="D187" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="D187:D191" si="7">IF(C187&lt;&gt;"",IF(B187&lt;&gt;"",C187-B187,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -4495,7 +4564,7 @@
       <c r="B188" s="7"/>
       <c r="C188" s="7"/>
       <c r="D188" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
@@ -4504,7 +4573,7 @@
       <c r="B189" s="7"/>
       <c r="C189" s="7"/>
       <c r="D189" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
@@ -4513,7 +4582,7 @@
       <c r="B190" s="7"/>
       <c r="C190" s="7"/>
       <c r="D190" s="3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
@@ -4522,7 +4591,7 @@
       <c r="B191" s="7"/>
       <c r="C191" s="7"/>
       <c r="D191" s="3" t="str">
-        <f t="shared" ref="D191:D195" si="6">IF(C191&lt;&gt;"",IF(B191&lt;&gt;"",C191-B191,"-"), "-")</f>
+        <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
@@ -4531,16 +4600,20 @@
       <c r="B192" s="7"/>
       <c r="C192" s="7"/>
       <c r="D192" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="D192:D193" si="8">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",B192-C192,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="193" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A193" s="7"/>
+      <c r="A193" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="B193" s="7"/>
-      <c r="C193" s="7"/>
+      <c r="C193" s="7">
+        <v>63782</v>
+      </c>
       <c r="D193" s="3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
@@ -4548,49 +4621,25 @@
       <c r="A194" s="7"/>
       <c r="B194" s="7"/>
       <c r="C194" s="7"/>
-      <c r="D194" s="3" t="str">
-        <f t="shared" si="6"/>
-        <v>-</v>
-      </c>
     </row>
     <row r="195" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A195" s="7"/>
       <c r="B195" s="7"/>
       <c r="C195" s="7"/>
-      <c r="D195" s="3" t="str">
-        <f t="shared" si="6"/>
-        <v>-</v>
-      </c>
     </row>
     <row r="196" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A196" s="7"/>
       <c r="B196" s="7"/>
       <c r="C196" s="7"/>
-      <c r="D196" s="3" t="str">
-        <f t="shared" ref="D196:D197" si="7">IF(C196&lt;&gt;"",IF(B196&lt;&gt;"",B196-C196,"-"), "-")</f>
-        <v>-</v>
-      </c>
     </row>
     <row r="197" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A197" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="B197" s="7"/>
-      <c r="C197" s="7">
-        <v>63782</v>
-      </c>
-      <c r="D197" s="3" t="str">
-        <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
+      <c r="C197" s="7"/>
     </row>
     <row r="198" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A198" s="7"/>
       <c r="B198" s="7"/>
       <c r="C198" s="7"/>
     </row>
     <row r="199" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A199" s="7"/>
       <c r="B199" s="7"/>
       <c r="C199" s="7"/>
     </row>
@@ -5125,22 +5174,6 @@
     <row r="332" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B332" s="7"/>
       <c r="C332" s="7"/>
-    </row>
-    <row r="333" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B333" s="7"/>
-      <c r="C333" s="7"/>
-    </row>
-    <row r="334" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B334" s="7"/>
-      <c r="C334" s="7"/>
-    </row>
-    <row r="335" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B335" s="7"/>
-      <c r="C335" s="7"/>
-    </row>
-    <row r="336" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B336" s="7"/>
-      <c r="C336" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - 32 done - 9148 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CACEB26-9CCB-428A-89E7-5F707837CD14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32946400-8BAA-4DDD-9CE8-34319D3B6D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="348">
   <si>
     <t>Place</t>
   </si>
@@ -1067,6 +1067,18 @@
   </si>
   <si>
     <t>31 ladder grab</t>
+  </si>
+  <si>
+    <t>32 ladder grab</t>
+  </si>
+  <si>
+    <t>dig after gold = 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dig before gold = 0 </t>
+  </si>
+  <si>
+    <t>33 gold = 7</t>
   </si>
 </sst>
 </file>
@@ -1930,7 +1942,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E332"/>
+  <dimension ref="A1:E333"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -3514,7 +3526,7 @@
         <v>26982</v>
       </c>
       <c r="D106" s="3">
-        <f t="shared" ref="D106:D186" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
+        <f t="shared" ref="D106:D187" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
         <v>6441</v>
       </c>
     </row>
@@ -4288,122 +4300,194 @@
         <v>343</v>
       </c>
       <c r="B158" s="7">
-        <v>30313</v>
+        <v>30319</v>
       </c>
       <c r="C158" s="7">
         <v>39162</v>
       </c>
       <c r="D158" s="3">
         <f t="shared" si="5"/>
+        <v>8843</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A159" s="52" t="s">
+        <v>310</v>
+      </c>
+      <c r="B159" s="7">
+        <v>30354</v>
+      </c>
+      <c r="C159" s="7">
+        <v>39201</v>
+      </c>
+      <c r="D159" s="3">
+        <f t="shared" si="5"/>
+        <v>8847</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A160" s="52" t="s">
+        <v>302</v>
+      </c>
+      <c r="B160" s="7">
+        <v>30373</v>
+      </c>
+      <c r="C160" s="7">
+        <v>39219</v>
+      </c>
+      <c r="D160" s="3">
+        <f t="shared" si="5"/>
+        <v>8846</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A161" s="52" t="s">
+        <v>249</v>
+      </c>
+      <c r="B161" s="7">
+        <v>30425</v>
+      </c>
+      <c r="C161" s="7">
+        <v>39271</v>
+      </c>
+      <c r="D161" s="3">
+        <f t="shared" si="5"/>
+        <v>8846</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A162" s="52" t="s">
+        <v>46</v>
+      </c>
+      <c r="B162" s="7">
+        <v>30479</v>
+      </c>
+      <c r="C162" s="7">
+        <v>39327</v>
+      </c>
+      <c r="D162" s="3">
+        <f t="shared" si="5"/>
+        <v>8848</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A163" s="52" t="s">
+        <v>344</v>
+      </c>
+      <c r="B163" s="7">
+        <v>31129</v>
+      </c>
+      <c r="C163" s="7">
+        <v>39979</v>
+      </c>
+      <c r="D163" s="3">
+        <f t="shared" si="5"/>
+        <v>8850</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A164" s="52" t="s">
+        <v>306</v>
+      </c>
+      <c r="B164" s="7">
+        <v>31202</v>
+      </c>
+      <c r="C164" s="7">
+        <v>40051</v>
+      </c>
+      <c r="D164" s="3">
+        <f t="shared" si="5"/>
         <v>8849</v>
       </c>
     </row>
-    <row r="159" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A159" s="7"/>
-      <c r="B159" s="7"/>
-      <c r="C159" s="7"/>
-      <c r="D159" s="3" t="str">
+    <row r="165" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A165" s="52" t="s">
+        <v>345</v>
+      </c>
+      <c r="B165" s="7">
+        <v>31269</v>
+      </c>
+      <c r="C165" s="7">
+        <v>40119</v>
+      </c>
+      <c r="D165" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="160" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A160" s="7"/>
-      <c r="B160" s="7"/>
-      <c r="C160" s="7"/>
-      <c r="D160" s="3" t="str">
+        <v>8850</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A166" s="52" t="s">
+        <v>247</v>
+      </c>
+      <c r="B166" s="7">
+        <v>31408</v>
+      </c>
+      <c r="C166" s="7">
+        <v>40257</v>
+      </c>
+      <c r="D166" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="161" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A161" s="7"/>
-      <c r="B161" s="7"/>
-      <c r="C161" s="7"/>
-      <c r="D161" s="3" t="str">
+        <v>8849</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A167" s="52" t="s">
+        <v>346</v>
+      </c>
+      <c r="B167" s="7">
+        <v>31522</v>
+      </c>
+      <c r="C167" s="7">
+        <v>40368</v>
+      </c>
+      <c r="D167" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="162" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A162" s="7"/>
-      <c r="B162" s="7"/>
-      <c r="C162" s="7"/>
-      <c r="D162" s="3" t="str">
+        <v>8846</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A168" s="52" t="s">
+        <v>150</v>
+      </c>
+      <c r="B168" s="7">
+        <v>31562</v>
+      </c>
+      <c r="C168" s="7">
+        <v>40409</v>
+      </c>
+      <c r="D168" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="163" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A163" s="7"/>
-      <c r="B163" s="7"/>
-      <c r="C163" s="7"/>
-      <c r="D163" s="3" t="str">
+        <v>8847</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A169" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="B169" s="7">
+        <v>31638</v>
+      </c>
+      <c r="C169" s="7">
+        <v>40487</v>
+      </c>
+      <c r="D169" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="164" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A164" s="7"/>
-      <c r="B164" s="7"/>
-      <c r="C164" s="7"/>
-      <c r="D164" s="3" t="str">
+        <v>8849</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A170" s="52" t="s">
+        <v>347</v>
+      </c>
+      <c r="B170" s="7">
+        <v>32035</v>
+      </c>
+      <c r="C170" s="7">
+        <v>41162</v>
+      </c>
+      <c r="D170" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A165" s="7"/>
-      <c r="B165" s="7"/>
-      <c r="C165" s="7"/>
-      <c r="D165" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="166" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A166" s="7"/>
-      <c r="B166" s="7"/>
-      <c r="C166" s="7"/>
-      <c r="D166" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="167" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A167" s="7"/>
-      <c r="B167" s="7"/>
-      <c r="C167" s="7"/>
-      <c r="D167" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="168" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A168" s="7"/>
-      <c r="B168" s="7"/>
-      <c r="C168" s="7"/>
-      <c r="D168" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="169" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A169" s="7"/>
-      <c r="B169" s="7"/>
-      <c r="C169" s="7"/>
-      <c r="D169" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="170" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A170" s="7"/>
-      <c r="B170" s="7"/>
-      <c r="C170" s="7"/>
-      <c r="D170" s="3" t="str">
-        <f t="shared" si="5"/>
-        <v>-</v>
+        <v>9127</v>
       </c>
     </row>
     <row r="171" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -4555,7 +4639,7 @@
       <c r="B187" s="7"/>
       <c r="C187" s="7"/>
       <c r="D187" s="3" t="str">
-        <f t="shared" ref="D187:D191" si="7">IF(C187&lt;&gt;"",IF(B187&lt;&gt;"",C187-B187,"-"), "-")</f>
+        <f t="shared" si="5"/>
         <v>-</v>
       </c>
     </row>
@@ -4564,7 +4648,7 @@
       <c r="B188" s="7"/>
       <c r="C188" s="7"/>
       <c r="D188" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="D188:D192" si="7">IF(C188&lt;&gt;"",IF(B188&lt;&gt;"",C188-B188,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -4600,27 +4684,31 @@
       <c r="B192" s="7"/>
       <c r="C192" s="7"/>
       <c r="D192" s="3" t="str">
-        <f t="shared" ref="D192:D193" si="8">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",B192-C192,"-"), "-")</f>
+        <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
     <row r="193" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A193" s="5" t="s">
+      <c r="A193" s="7"/>
+      <c r="B193" s="7"/>
+      <c r="C193" s="7"/>
+      <c r="D193" s="3" t="str">
+        <f t="shared" ref="D193:D194" si="8">IF(C193&lt;&gt;"",IF(B193&lt;&gt;"",B193-C193,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A194" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B193" s="7"/>
-      <c r="C193" s="7">
+      <c r="B194" s="7"/>
+      <c r="C194" s="7">
         <v>63782</v>
       </c>
-      <c r="D193" s="3" t="str">
+      <c r="D194" s="3" t="str">
         <f t="shared" si="8"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="194" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A194" s="7"/>
-      <c r="B194" s="7"/>
-      <c r="C194" s="7"/>
     </row>
     <row r="195" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A195" s="7"/>
@@ -4628,6 +4716,7 @@
       <c r="C195" s="7"/>
     </row>
     <row r="196" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A196" s="7"/>
       <c r="B196" s="7"/>
       <c r="C196" s="7"/>
     </row>
@@ -5174,6 +5263,10 @@
     <row r="332" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B332" s="7"/>
       <c r="C332" s="7"/>
+    </row>
+    <row r="333" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B333" s="7"/>
+      <c r="C333" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - 33 done
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32946400-8BAA-4DDD-9CE8-34319D3B6D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA2C02FC-FD94-4710-B810-41E8ACC21526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="349">
   <si>
     <t>Place</t>
   </si>
@@ -1079,6 +1079,9 @@
   </si>
   <si>
     <t>33 gold = 7</t>
+  </si>
+  <si>
+    <t>33 ladder grab</t>
   </si>
 </sst>
 </file>
@@ -4480,92 +4483,144 @@
         <v>347</v>
       </c>
       <c r="B170" s="7">
-        <v>32035</v>
+        <v>32014</v>
       </c>
       <c r="C170" s="7">
         <v>41162</v>
       </c>
       <c r="D170" s="3">
         <f t="shared" si="5"/>
-        <v>9127</v>
+        <v>9148</v>
       </c>
     </row>
     <row r="171" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A171" s="7"/>
-      <c r="B171" s="7"/>
-      <c r="C171" s="7"/>
-      <c r="D171" s="3" t="str">
+      <c r="A171" s="52" t="s">
+        <v>247</v>
+      </c>
+      <c r="B171" s="7">
+        <v>32090</v>
+      </c>
+      <c r="C171" s="7">
+        <v>41237</v>
+      </c>
+      <c r="D171" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>9147</v>
       </c>
     </row>
     <row r="172" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A172" s="7"/>
-      <c r="B172" s="7"/>
-      <c r="C172" s="7"/>
-      <c r="D172" s="3" t="str">
+      <c r="A172" s="52" t="s">
+        <v>150</v>
+      </c>
+      <c r="B172" s="7">
+        <v>32120</v>
+      </c>
+      <c r="C172" s="7">
+        <v>41266</v>
+      </c>
+      <c r="D172" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>9146</v>
       </c>
     </row>
     <row r="173" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A173" s="7"/>
-      <c r="B173" s="7"/>
-      <c r="C173" s="7"/>
-      <c r="D173" s="3" t="str">
+      <c r="A173" s="52" t="s">
+        <v>310</v>
+      </c>
+      <c r="B173" s="7">
+        <v>32158</v>
+      </c>
+      <c r="C173" s="7">
+        <v>41304</v>
+      </c>
+      <c r="D173" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>9146</v>
       </c>
     </row>
     <row r="174" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A174" s="7"/>
-      <c r="B174" s="7"/>
-      <c r="C174" s="7"/>
-      <c r="D174" s="3" t="str">
+      <c r="A174" s="52" t="s">
+        <v>265</v>
+      </c>
+      <c r="B174" s="7">
+        <v>32252</v>
+      </c>
+      <c r="C174" s="7">
+        <v>41401</v>
+      </c>
+      <c r="D174" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>9149</v>
       </c>
     </row>
     <row r="175" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A175" s="7"/>
-      <c r="B175" s="7"/>
-      <c r="C175" s="7"/>
-      <c r="D175" s="3" t="str">
+      <c r="A175" s="52" t="s">
+        <v>249</v>
+      </c>
+      <c r="B175" s="7">
+        <v>32338</v>
+      </c>
+      <c r="C175" s="7">
+        <v>41492</v>
+      </c>
+      <c r="D175" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>9154</v>
       </c>
     </row>
     <row r="176" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A176" s="7"/>
-      <c r="B176" s="7"/>
-      <c r="C176" s="7"/>
-      <c r="D176" s="3" t="str">
+      <c r="A176" s="52" t="s">
+        <v>248</v>
+      </c>
+      <c r="B176" s="7">
+        <v>32484</v>
+      </c>
+      <c r="C176" s="7">
+        <v>41638</v>
+      </c>
+      <c r="D176" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>9154</v>
       </c>
     </row>
     <row r="177" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A177" s="7"/>
-      <c r="B177" s="7"/>
-      <c r="C177" s="7"/>
-      <c r="D177" s="3" t="str">
+      <c r="A177" s="52" t="s">
+        <v>250</v>
+      </c>
+      <c r="B177" s="7">
+        <v>32559</v>
+      </c>
+      <c r="C177" s="7">
+        <v>41709</v>
+      </c>
+      <c r="D177" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>9150</v>
       </c>
     </row>
     <row r="178" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A178" s="7"/>
-      <c r="B178" s="7"/>
-      <c r="C178" s="7"/>
-      <c r="D178" s="3" t="str">
+      <c r="A178" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="B178" s="7">
+        <v>32586</v>
+      </c>
+      <c r="C178" s="7">
+        <v>41736</v>
+      </c>
+      <c r="D178" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
+        <v>9150</v>
       </c>
     </row>
     <row r="179" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A179" s="7"/>
+      <c r="A179" s="52" t="s">
+        <v>348</v>
+      </c>
       <c r="B179" s="7"/>
-      <c r="C179" s="7"/>
+      <c r="C179" s="7">
+        <v>42391</v>
+      </c>
       <c r="D179" s="3" t="str">
         <f t="shared" si="5"/>
         <v>-</v>

</xml_diff>

<commit_message>
lv 35 done, 9461 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA2C02FC-FD94-4710-B810-41E8ACC21526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBA9E8CC-7EE3-4000-AA2B-AD2CD5B979EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50865" yWindow="3210" windowWidth="7170" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="73800" yWindow="1920" windowWidth="13785" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V6" sheetId="7" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="361">
   <si>
     <t>Place</t>
   </si>
@@ -1082,6 +1082,42 @@
   </si>
   <si>
     <t>33 ladder grab</t>
+  </si>
+  <si>
+    <t>camx = 0</t>
+  </si>
+  <si>
+    <t>camx = 214</t>
+  </si>
+  <si>
+    <t>camx = 1</t>
+  </si>
+  <si>
+    <t>gold = 29</t>
+  </si>
+  <si>
+    <t>gold=23</t>
+  </si>
+  <si>
+    <t>gold = 22</t>
+  </si>
+  <si>
+    <t>gold = 20</t>
+  </si>
+  <si>
+    <t>gold = 16</t>
+  </si>
+  <si>
+    <t>35 ladder grab</t>
+  </si>
+  <si>
+    <t>34 appears</t>
+  </si>
+  <si>
+    <t>right ladder grab</t>
+  </si>
+  <si>
+    <t>walk over enemy</t>
   </si>
 </sst>
 </file>
@@ -1091,12 +1127,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="29" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1500,95 +1543,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1600,28 +1644,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1945,7 +1989,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E333"/>
+  <dimension ref="A1:E340"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -3529,7 +3573,7 @@
         <v>26982</v>
       </c>
       <c r="D106" s="3">
-        <f t="shared" ref="D106:D187" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
+        <f t="shared" ref="D106:D191" si="5">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
         <v>6441</v>
       </c>
     </row>
@@ -3932,7 +3976,7 @@
       </c>
     </row>
     <row r="134" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A134" s="52" t="s">
+      <c r="A134" s="44" t="s">
         <v>330</v>
       </c>
       <c r="B134" s="7">
@@ -3948,7 +3992,7 @@
       <c r="E134" s="7"/>
     </row>
     <row r="135" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A135" s="52" t="s">
+      <c r="A135" s="44" t="s">
         <v>331</v>
       </c>
       <c r="B135" s="7">
@@ -3963,7 +4007,7 @@
       </c>
     </row>
     <row r="136" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A136" s="52" t="s">
+      <c r="A136" s="44" t="s">
         <v>319</v>
       </c>
       <c r="B136" s="7">
@@ -3978,7 +4022,7 @@
       </c>
     </row>
     <row r="137" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A137" s="52" t="s">
+      <c r="A137" s="44" t="s">
         <v>333</v>
       </c>
       <c r="B137" s="7">
@@ -3993,7 +4037,7 @@
       </c>
     </row>
     <row r="138" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A138" s="52" t="s">
+      <c r="A138" s="44" t="s">
         <v>265</v>
       </c>
       <c r="B138" s="7">
@@ -4008,7 +4052,7 @@
       </c>
     </row>
     <row r="139" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A139" s="52" t="s">
+      <c r="A139" s="44" t="s">
         <v>302</v>
       </c>
       <c r="B139" s="7">
@@ -4023,7 +4067,7 @@
       </c>
     </row>
     <row r="140" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A140" s="52" t="s">
+      <c r="A140" s="44" t="s">
         <v>335</v>
       </c>
       <c r="B140" s="7">
@@ -4038,7 +4082,7 @@
       </c>
     </row>
     <row r="141" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A141" s="52" t="s">
+      <c r="A141" s="44" t="s">
         <v>334</v>
       </c>
       <c r="B141" s="7">
@@ -4053,7 +4097,7 @@
       </c>
     </row>
     <row r="142" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A142" s="52" t="s">
+      <c r="A142" s="44" t="s">
         <v>332</v>
       </c>
       <c r="B142" s="7">
@@ -4068,7 +4112,7 @@
       </c>
     </row>
     <row r="143" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A143" s="52" t="s">
+      <c r="A143" s="44" t="s">
         <v>336</v>
       </c>
       <c r="B143" s="7">
@@ -4083,7 +4127,7 @@
       </c>
     </row>
     <row r="144" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A144" s="52" t="s">
+      <c r="A144" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B144" s="7">
@@ -4098,7 +4142,7 @@
       </c>
     </row>
     <row r="145" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A145" s="52" t="s">
+      <c r="A145" s="44" t="s">
         <v>312</v>
       </c>
       <c r="B145" s="7">
@@ -4113,7 +4157,7 @@
       </c>
     </row>
     <row r="146" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A146" s="52" t="s">
+      <c r="A146" s="44" t="s">
         <v>265</v>
       </c>
       <c r="B146" s="7">
@@ -4128,7 +4172,7 @@
       </c>
     </row>
     <row r="147" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A147" s="52" t="s">
+      <c r="A147" s="44" t="s">
         <v>265</v>
       </c>
       <c r="B147" s="7">
@@ -4143,7 +4187,7 @@
       </c>
     </row>
     <row r="148" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A148" s="52" t="s">
+      <c r="A148" s="44" t="s">
         <v>250</v>
       </c>
       <c r="B148" s="7">
@@ -4158,7 +4202,7 @@
       </c>
     </row>
     <row r="149" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A149" s="52" t="s">
+      <c r="A149" s="44" t="s">
         <v>337</v>
       </c>
       <c r="B149" s="10">
@@ -4173,7 +4217,7 @@
       </c>
     </row>
     <row r="150" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A150" s="52" t="s">
+      <c r="A150" s="44" t="s">
         <v>338</v>
       </c>
       <c r="B150" s="7">
@@ -4188,7 +4232,7 @@
       </c>
     </row>
     <row r="151" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A151" s="52" t="s">
+      <c r="A151" s="44" t="s">
         <v>339</v>
       </c>
       <c r="B151" s="7">
@@ -4203,7 +4247,7 @@
       </c>
     </row>
     <row r="152" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A152" s="52" t="s">
+      <c r="A152" s="44" t="s">
         <v>150</v>
       </c>
       <c r="B152" s="7">
@@ -4216,12 +4260,12 @@
         <f t="shared" si="5"/>
         <v>8564</v>
       </c>
-      <c r="E152" s="52" t="s">
+      <c r="E152" s="44" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="153" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A153" s="52" t="s">
+      <c r="A153" s="44" t="s">
         <v>340</v>
       </c>
       <c r="B153" s="7">
@@ -4239,7 +4283,7 @@
       </c>
     </row>
     <row r="154" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A154" s="52" t="s">
+      <c r="A154" s="44" t="s">
         <v>312</v>
       </c>
       <c r="B154" s="7">
@@ -4254,7 +4298,7 @@
       </c>
     </row>
     <row r="155" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A155" s="52" t="s">
+      <c r="A155" s="44" t="s">
         <v>150</v>
       </c>
       <c r="B155" s="7">
@@ -4269,7 +4313,7 @@
       </c>
     </row>
     <row r="156" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A156" s="52" t="s">
+      <c r="A156" s="44" t="s">
         <v>293</v>
       </c>
       <c r="B156" s="7">
@@ -4284,7 +4328,7 @@
       </c>
     </row>
     <row r="157" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A157" s="52" t="s">
+      <c r="A157" s="44" t="s">
         <v>45</v>
       </c>
       <c r="B157" s="7">
@@ -4299,7 +4343,7 @@
       </c>
     </row>
     <row r="158" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A158" s="52" t="s">
+      <c r="A158" s="44" t="s">
         <v>343</v>
       </c>
       <c r="B158" s="7">
@@ -4314,7 +4358,7 @@
       </c>
     </row>
     <row r="159" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A159" s="52" t="s">
+      <c r="A159" s="44" t="s">
         <v>310</v>
       </c>
       <c r="B159" s="7">
@@ -4329,7 +4373,7 @@
       </c>
     </row>
     <row r="160" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A160" s="52" t="s">
+      <c r="A160" s="44" t="s">
         <v>302</v>
       </c>
       <c r="B160" s="7">
@@ -4344,7 +4388,7 @@
       </c>
     </row>
     <row r="161" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A161" s="52" t="s">
+      <c r="A161" s="44" t="s">
         <v>249</v>
       </c>
       <c r="B161" s="7">
@@ -4359,7 +4403,7 @@
       </c>
     </row>
     <row r="162" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A162" s="52" t="s">
+      <c r="A162" s="44" t="s">
         <v>46</v>
       </c>
       <c r="B162" s="7">
@@ -4374,7 +4418,7 @@
       </c>
     </row>
     <row r="163" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A163" s="52" t="s">
+      <c r="A163" s="44" t="s">
         <v>344</v>
       </c>
       <c r="B163" s="7">
@@ -4389,7 +4433,7 @@
       </c>
     </row>
     <row r="164" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A164" s="52" t="s">
+      <c r="A164" s="44" t="s">
         <v>306</v>
       </c>
       <c r="B164" s="7">
@@ -4404,7 +4448,7 @@
       </c>
     </row>
     <row r="165" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A165" s="52" t="s">
+      <c r="A165" s="44" t="s">
         <v>345</v>
       </c>
       <c r="B165" s="7">
@@ -4419,7 +4463,7 @@
       </c>
     </row>
     <row r="166" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A166" s="52" t="s">
+      <c r="A166" s="44" t="s">
         <v>247</v>
       </c>
       <c r="B166" s="7">
@@ -4434,7 +4478,7 @@
       </c>
     </row>
     <row r="167" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A167" s="52" t="s">
+      <c r="A167" s="44" t="s">
         <v>346</v>
       </c>
       <c r="B167" s="7">
@@ -4449,7 +4493,7 @@
       </c>
     </row>
     <row r="168" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A168" s="52" t="s">
+      <c r="A168" s="44" t="s">
         <v>150</v>
       </c>
       <c r="B168" s="7">
@@ -4464,7 +4508,7 @@
       </c>
     </row>
     <row r="169" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A169" s="52" t="s">
+      <c r="A169" s="44" t="s">
         <v>28</v>
       </c>
       <c r="B169" s="7">
@@ -4479,7 +4523,7 @@
       </c>
     </row>
     <row r="170" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A170" s="52" t="s">
+      <c r="A170" s="44" t="s">
         <v>347</v>
       </c>
       <c r="B170" s="7">
@@ -4494,7 +4538,7 @@
       </c>
     </row>
     <row r="171" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A171" s="52" t="s">
+      <c r="A171" s="44" t="s">
         <v>247</v>
       </c>
       <c r="B171" s="7">
@@ -4509,7 +4553,7 @@
       </c>
     </row>
     <row r="172" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A172" s="52" t="s">
+      <c r="A172" s="44" t="s">
         <v>150</v>
       </c>
       <c r="B172" s="7">
@@ -4524,7 +4568,7 @@
       </c>
     </row>
     <row r="173" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A173" s="52" t="s">
+      <c r="A173" s="44" t="s">
         <v>310</v>
       </c>
       <c r="B173" s="7">
@@ -4539,7 +4583,7 @@
       </c>
     </row>
     <row r="174" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A174" s="52" t="s">
+      <c r="A174" s="44" t="s">
         <v>265</v>
       </c>
       <c r="B174" s="7">
@@ -4554,7 +4598,7 @@
       </c>
     </row>
     <row r="175" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A175" s="52" t="s">
+      <c r="A175" s="44" t="s">
         <v>249</v>
       </c>
       <c r="B175" s="7">
@@ -4569,7 +4613,7 @@
       </c>
     </row>
     <row r="176" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A176" s="52" t="s">
+      <c r="A176" s="44" t="s">
         <v>248</v>
       </c>
       <c r="B176" s="7">
@@ -4584,7 +4628,7 @@
       </c>
     </row>
     <row r="177" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A177" s="52" t="s">
+      <c r="A177" s="44" t="s">
         <v>250</v>
       </c>
       <c r="B177" s="7">
@@ -4599,8 +4643,8 @@
       </c>
     </row>
     <row r="178" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A178" s="52" t="s">
-        <v>28</v>
+      <c r="A178" s="53" t="s">
+        <v>29</v>
       </c>
       <c r="B178" s="7">
         <v>32586</v>
@@ -4614,192 +4658,331 @@
       </c>
     </row>
     <row r="179" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A179" s="52" t="s">
+      <c r="A179" s="53" t="s">
+        <v>358</v>
+      </c>
+      <c r="B179" s="7">
+        <v>32930</v>
+      </c>
+      <c r="C179" s="7">
+        <v>42081</v>
+      </c>
+      <c r="D179" s="3">
+        <f t="shared" si="5"/>
+        <v>9151</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A180" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="B180" s="7">
+        <v>32931</v>
+      </c>
+      <c r="C180" s="7">
+        <v>42082</v>
+      </c>
+      <c r="D180" s="3">
+        <f t="shared" si="5"/>
+        <v>9151</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A181" s="53" t="s">
+        <v>350</v>
+      </c>
+      <c r="B181" s="7">
+        <v>33090</v>
+      </c>
+      <c r="C181" s="7">
+        <v>42234</v>
+      </c>
+      <c r="D181" s="3">
+        <f t="shared" si="5"/>
+        <v>9144</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A182" s="53" t="s">
+        <v>349</v>
+      </c>
+      <c r="B182" s="7">
+        <v>33253</v>
+      </c>
+      <c r="C182" s="7">
+        <v>42389</v>
+      </c>
+      <c r="D182" s="3">
+        <f t="shared" si="5"/>
+        <v>9136</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A183" s="44" t="s">
         <v>348</v>
       </c>
-      <c r="B179" s="7"/>
-      <c r="C179" s="7">
+      <c r="B183" s="7">
+        <v>33254</v>
+      </c>
+      <c r="C183" s="7">
         <v>42391</v>
       </c>
-      <c r="D179" s="3" t="str">
+      <c r="D183" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="180" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A180" s="7"/>
-      <c r="B180" s="7"/>
-      <c r="C180" s="7"/>
-      <c r="D180" s="3" t="str">
+        <v>9137</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A184" s="53" t="s">
+        <v>352</v>
+      </c>
+      <c r="B184" s="7">
+        <v>33300</v>
+      </c>
+      <c r="C184" s="7">
+        <v>42437</v>
+      </c>
+      <c r="D184" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="181" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A181" s="7"/>
-      <c r="B181" s="7"/>
-      <c r="C181" s="7"/>
-      <c r="D181" s="3" t="str">
+        <v>9137</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A185" s="53" t="s">
+        <v>353</v>
+      </c>
+      <c r="B185" s="7">
+        <v>33377</v>
+      </c>
+      <c r="C185" s="7">
+        <v>42515</v>
+      </c>
+      <c r="D185" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="182" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A182" s="7"/>
-      <c r="B182" s="7"/>
-      <c r="C182" s="7"/>
-      <c r="D182" s="3" t="str">
+        <v>9138</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A186" s="53" t="s">
+        <v>265</v>
+      </c>
+      <c r="B186" s="7">
+        <v>33447</v>
+      </c>
+      <c r="C186" s="7">
+        <v>42585</v>
+      </c>
+      <c r="D186" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="183" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A183" s="7"/>
-      <c r="B183" s="7"/>
-      <c r="C183" s="7"/>
-      <c r="D183" s="3" t="str">
+        <v>9138</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A187" s="53" t="s">
+        <v>354</v>
+      </c>
+      <c r="B187" s="7">
+        <v>33499</v>
+      </c>
+      <c r="C187" s="7">
+        <v>42637</v>
+      </c>
+      <c r="D187" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="184" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A184" s="7"/>
-      <c r="B184" s="7"/>
-      <c r="C184" s="7"/>
-      <c r="D184" s="3" t="str">
+        <v>9138</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A188" s="53" t="s">
+        <v>355</v>
+      </c>
+      <c r="B188" s="7">
+        <v>33539</v>
+      </c>
+      <c r="C188" s="7">
+        <v>42678</v>
+      </c>
+      <c r="D188" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="185" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A185" s="7"/>
-      <c r="B185" s="7"/>
-      <c r="C185" s="7"/>
-      <c r="D185" s="3" t="str">
+        <v>9139</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A189" s="53" t="s">
+        <v>356</v>
+      </c>
+      <c r="B189" s="7">
+        <v>33601</v>
+      </c>
+      <c r="C189" s="7">
+        <v>42740</v>
+      </c>
+      <c r="D189" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="186" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A186" s="7"/>
-      <c r="B186" s="7"/>
-      <c r="C186" s="7"/>
-      <c r="D186" s="3" t="str">
+        <v>9139</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A190" s="53" t="s">
+        <v>319</v>
+      </c>
+      <c r="B190" s="7">
+        <v>33648</v>
+      </c>
+      <c r="C190" s="7">
+        <v>42788</v>
+      </c>
+      <c r="D190" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="187" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A187" s="7"/>
-      <c r="B187" s="7"/>
-      <c r="C187" s="7"/>
-      <c r="D187" s="3" t="str">
+        <v>9140</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A191" s="53" t="s">
+        <v>31</v>
+      </c>
+      <c r="B191" s="7">
+        <v>33882</v>
+      </c>
+      <c r="C191" s="7">
+        <v>43040</v>
+      </c>
+      <c r="D191" s="3">
         <f t="shared" si="5"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="188" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A188" s="7"/>
-      <c r="B188" s="7"/>
-      <c r="C188" s="7"/>
-      <c r="D188" s="3" t="str">
-        <f t="shared" ref="D188:D192" si="7">IF(C188&lt;&gt;"",IF(B188&lt;&gt;"",C188-B188,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="189" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A189" s="7"/>
-      <c r="B189" s="7"/>
-      <c r="C189" s="7"/>
-      <c r="D189" s="3" t="str">
+        <v>9158</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A192" s="53" t="s">
+        <v>357</v>
+      </c>
+      <c r="B192" s="7">
+        <v>34259</v>
+      </c>
+      <c r="C192" s="7">
+        <v>43721</v>
+      </c>
+      <c r="D192" s="3">
+        <f t="shared" ref="D192:D199" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
+        <v>9462</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A193" s="53" t="s">
+        <v>359</v>
+      </c>
+      <c r="B193" s="7">
+        <v>34658</v>
+      </c>
+      <c r="C193" s="7">
+        <v>44120</v>
+      </c>
+      <c r="D193" s="3">
+        <f t="shared" si="7"/>
+        <v>9462</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A194" s="53" t="s">
+        <v>265</v>
+      </c>
+      <c r="B194" s="7">
+        <v>34694</v>
+      </c>
+      <c r="C194" s="7">
+        <v>44156</v>
+      </c>
+      <c r="D194" s="3">
+        <f t="shared" si="7"/>
+        <v>9462</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A195" s="53" t="s">
+        <v>360</v>
+      </c>
+      <c r="B195" s="7">
+        <v>34735</v>
+      </c>
+      <c r="C195" s="7">
+        <v>44194</v>
+      </c>
+      <c r="D195" s="3">
+        <f t="shared" si="7"/>
+        <v>9459</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A196" s="53" t="s">
+        <v>30</v>
+      </c>
+      <c r="B196" s="7">
+        <v>34861</v>
+      </c>
+      <c r="C196" s="7">
+        <v>44322</v>
+      </c>
+      <c r="D196" s="3">
+        <f t="shared" si="7"/>
+        <v>9461</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A197" s="7"/>
+      <c r="B197" s="7"/>
+      <c r="C197" s="7"/>
+      <c r="D197" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="190" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A190" s="7"/>
-      <c r="B190" s="7"/>
-      <c r="C190" s="7"/>
-      <c r="D190" s="3" t="str">
+    <row r="198" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A198" s="7"/>
+      <c r="B198" s="7"/>
+      <c r="C198" s="7"/>
+      <c r="D198" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="191" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A191" s="7"/>
-      <c r="B191" s="7"/>
-      <c r="C191" s="7"/>
-      <c r="D191" s="3" t="str">
+    <row r="199" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A199" s="7"/>
+      <c r="B199" s="7"/>
+      <c r="C199" s="7"/>
+      <c r="D199" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="192" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A192" s="7"/>
-      <c r="B192" s="7"/>
-      <c r="C192" s="7"/>
-      <c r="D192" s="3" t="str">
-        <f t="shared" si="7"/>
+    <row r="200" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A200" s="7"/>
+      <c r="B200" s="7"/>
+      <c r="C200" s="7"/>
+      <c r="D200" s="3" t="str">
+        <f t="shared" ref="D200:D201" si="8">IF(C200&lt;&gt;"",IF(B200&lt;&gt;"",B200-C200,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="193" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A193" s="7"/>
-      <c r="B193" s="7"/>
-      <c r="C193" s="7"/>
-      <c r="D193" s="3" t="str">
-        <f t="shared" ref="D193:D194" si="8">IF(C193&lt;&gt;"",IF(B193&lt;&gt;"",B193-C193,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="194" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A194" s="5" t="s">
+    <row r="201" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A201" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B194" s="7"/>
-      <c r="C194" s="7">
+      <c r="B201" s="7"/>
+      <c r="C201" s="7">
         <v>63782</v>
       </c>
-      <c r="D194" s="3" t="str">
+      <c r="D201" s="3" t="str">
         <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
-    <row r="195" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A195" s="7"/>
-      <c r="B195" s="7"/>
-      <c r="C195" s="7"/>
-    </row>
-    <row r="196" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A196" s="7"/>
-      <c r="B196" s="7"/>
-      <c r="C196" s="7"/>
-    </row>
-    <row r="197" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B197" s="7"/>
-      <c r="C197" s="7"/>
-    </row>
-    <row r="198" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B198" s="7"/>
-      <c r="C198" s="7"/>
-    </row>
-    <row r="199" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B199" s="7"/>
-      <c r="C199" s="7"/>
-    </row>
-    <row r="200" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B200" s="7"/>
-      <c r="C200" s="7"/>
-    </row>
-    <row r="201" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B201" s="7"/>
-      <c r="C201" s="7"/>
-    </row>
     <row r="202" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A202" s="7"/>
       <c r="B202" s="7"/>
       <c r="C202" s="7"/>
     </row>
     <row r="203" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A203" s="7"/>
       <c r="B203" s="7"/>
       <c r="C203" s="7"/>
     </row>
@@ -5322,6 +5505,34 @@
     <row r="333" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B333" s="7"/>
       <c r="C333" s="7"/>
+    </row>
+    <row r="334" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B334" s="7"/>
+      <c r="C334" s="7"/>
+    </row>
+    <row r="335" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B335" s="7"/>
+      <c r="C335" s="7"/>
+    </row>
+    <row r="336" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B336" s="7"/>
+      <c r="C336" s="7"/>
+    </row>
+    <row r="337" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B337" s="7"/>
+      <c r="C337" s="7"/>
+    </row>
+    <row r="338" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B338" s="7"/>
+      <c r="C338" s="7"/>
+    </row>
+    <row r="339" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B339" s="7"/>
+      <c r="C339" s="7"/>
+    </row>
+    <row r="340" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B340" s="7"/>
+      <c r="C340" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15315,7 +15526,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="25" type="noConversion"/>
+  <phoneticPr fontId="26" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -15345,10 +15556,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="44" t="s">
+      <c r="K1" s="45" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="45"/>
+      <c r="L1" s="46"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -17200,13 +17411,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="46" t="s">
+      <c r="H53" s="47" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="47"/>
-      <c r="J53" s="47"/>
-      <c r="K53" s="47"/>
-      <c r="L53" s="48"/>
+      <c r="I53" s="48"/>
+      <c r="J53" s="48"/>
+      <c r="K53" s="48"/>
+      <c r="L53" s="49"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -17228,11 +17439,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="49"/>
-      <c r="I54" s="50"/>
-      <c r="J54" s="50"/>
-      <c r="K54" s="50"/>
-      <c r="L54" s="51"/>
+      <c r="H54" s="50"/>
+      <c r="I54" s="51"/>
+      <c r="J54" s="51"/>
+      <c r="K54" s="51"/>
+      <c r="L54" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
level 36 start - 9777 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBA9E8CC-7EE3-4000-AA2B-AD2CD5B979EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC869229-0237-48FB-A10E-41ED61F7C3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="73800" yWindow="1920" windowWidth="13785" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="362">
   <si>
     <t>Place</t>
   </si>
@@ -1118,6 +1118,9 @@
   </si>
   <si>
     <t>walk over enemy</t>
+  </si>
+  <si>
+    <t>36 1st move</t>
   </si>
 </sst>
 </file>
@@ -4928,12 +4931,18 @@
       </c>
     </row>
     <row r="197" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A197" s="7"/>
-      <c r="B197" s="7"/>
-      <c r="C197" s="7"/>
-      <c r="D197" s="3" t="str">
+      <c r="A197" s="53" t="s">
+        <v>361</v>
+      </c>
+      <c r="B197" s="7">
+        <v>35214</v>
+      </c>
+      <c r="C197" s="7">
+        <v>44991</v>
+      </c>
+      <c r="D197" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>9777</v>
       </c>
     </row>
     <row r="198" spans="1:4" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - level 36 done, 10126 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC869229-0237-48FB-A10E-41ED61F7C3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1554287F-368A-4149-A112-9266E7E09D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="73800" yWindow="1920" windowWidth="13785" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="363">
   <si>
     <t>Place</t>
   </si>
@@ -1121,6 +1121,9 @@
   </si>
   <si>
     <t>36 1st move</t>
+  </si>
+  <si>
+    <t>37 ladder grab</t>
   </si>
 </sst>
 </file>
@@ -1557,7 +1560,7 @@
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1672,6 +1675,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -1992,7 +1996,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E340"/>
+  <dimension ref="A1:E337"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -4946,52 +4950,49 @@
       </c>
     </row>
     <row r="198" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A198" s="7"/>
-      <c r="B198" s="7"/>
-      <c r="C198" s="7"/>
-      <c r="D198" s="3" t="str">
+      <c r="A198" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="B198" s="7">
+        <v>35770</v>
+      </c>
+      <c r="C198" s="7">
+        <v>45580</v>
+      </c>
+      <c r="D198" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>9810</v>
       </c>
     </row>
     <row r="199" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A199" s="7"/>
-      <c r="B199" s="7"/>
-      <c r="C199" s="7"/>
-      <c r="D199" s="3" t="str">
+      <c r="A199" s="53" t="s">
+        <v>362</v>
+      </c>
+      <c r="B199" s="7">
+        <v>36129</v>
+      </c>
+      <c r="C199" s="7">
+        <v>46255</v>
+      </c>
+      <c r="D199" s="54">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>10126</v>
       </c>
     </row>
     <row r="200" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A200" s="7"/>
       <c r="B200" s="7"/>
       <c r="C200" s="7"/>
-      <c r="D200" s="3" t="str">
-        <f t="shared" ref="D200:D201" si="8">IF(C200&lt;&gt;"",IF(B200&lt;&gt;"",B200-C200,"-"), "-")</f>
-        <v>-</v>
-      </c>
     </row>
     <row r="201" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A201" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="B201" s="7"/>
-      <c r="C201" s="7">
-        <v>63782</v>
-      </c>
-      <c r="D201" s="3" t="str">
-        <f t="shared" si="8"/>
-        <v>-</v>
-      </c>
+      <c r="C201" s="7"/>
     </row>
     <row r="202" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A202" s="7"/>
       <c r="B202" s="7"/>
       <c r="C202" s="7"/>
     </row>
     <row r="203" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A203" s="7"/>
       <c r="B203" s="7"/>
       <c r="C203" s="7"/>
     </row>
@@ -5143,67 +5144,76 @@
       <c r="B240" s="7"/>
       <c r="C240" s="7"/>
     </row>
-    <row r="241" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B241" s="7"/>
       <c r="C241" s="7"/>
     </row>
-    <row r="242" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B242" s="7"/>
       <c r="C242" s="7"/>
     </row>
-    <row r="243" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A243" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="B243" s="7"/>
-      <c r="C243" s="7"/>
-    </row>
-    <row r="244" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C243" s="7">
+        <v>63782</v>
+      </c>
+      <c r="D243" s="3" t="str">
+        <f t="shared" ref="D243" si="8">IF(C243&lt;&gt;"",IF(B243&lt;&gt;"",B243-C243,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="244" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B244" s="7"/>
       <c r="C244" s="7"/>
     </row>
-    <row r="245" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B245" s="7"/>
       <c r="C245" s="7"/>
     </row>
-    <row r="246" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B246" s="7"/>
       <c r="C246" s="7"/>
     </row>
-    <row r="247" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B247" s="7"/>
       <c r="C247" s="7"/>
     </row>
-    <row r="248" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B248" s="7"/>
       <c r="C248" s="7"/>
     </row>
-    <row r="249" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B249" s="7"/>
       <c r="C249" s="7"/>
     </row>
-    <row r="250" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B250" s="7"/>
       <c r="C250" s="7"/>
     </row>
-    <row r="251" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B251" s="7"/>
       <c r="C251" s="7"/>
     </row>
-    <row r="252" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B252" s="7"/>
       <c r="C252" s="7"/>
     </row>
-    <row r="253" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B253" s="7"/>
       <c r="C253" s="7"/>
     </row>
-    <row r="254" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B254" s="7"/>
       <c r="C254" s="7"/>
     </row>
-    <row r="255" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B255" s="7"/>
       <c r="C255" s="7"/>
     </row>
-    <row r="256" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B256" s="7"/>
       <c r="C256" s="7"/>
     </row>
@@ -5530,18 +5540,6 @@
     <row r="337" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B337" s="7"/>
       <c r="C337" s="7"/>
-    </row>
-    <row r="338" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B338" s="7"/>
-      <c r="C338" s="7"/>
-    </row>
-    <row r="339" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B339" s="7"/>
-      <c r="C339" s="7"/>
-    </row>
-    <row r="340" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B340" s="7"/>
-      <c r="C340" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - lv 39 done - 10870 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1554287F-368A-4149-A112-9266E7E09D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F487DA55-4ABB-471D-9360-0AE607F8AADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="73800" yWindow="1920" windowWidth="13785" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="73650" yWindow="2610" windowWidth="13785" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V6" sheetId="7" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="367">
   <si>
     <t>Place</t>
   </si>
@@ -1124,6 +1124,18 @@
   </si>
   <si>
     <t>37 ladder grab</t>
+  </si>
+  <si>
+    <t>38 gold = 8</t>
+  </si>
+  <si>
+    <t>grab pipe</t>
+  </si>
+  <si>
+    <t>39 gold = 7</t>
+  </si>
+  <si>
+    <t>40 1st move</t>
   </si>
 </sst>
 </file>
@@ -1133,12 +1145,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="30" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1549,95 +1568,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1650,32 +1670,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -1996,7 +2015,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E337"/>
+  <dimension ref="A1:E338"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -4650,7 +4669,7 @@
       </c>
     </row>
     <row r="178" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A178" s="53" t="s">
+      <c r="A178" s="45" t="s">
         <v>29</v>
       </c>
       <c r="B178" s="7">
@@ -4665,7 +4684,7 @@
       </c>
     </row>
     <row r="179" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A179" s="53" t="s">
+      <c r="A179" s="45" t="s">
         <v>358</v>
       </c>
       <c r="B179" s="7">
@@ -4680,7 +4699,7 @@
       </c>
     </row>
     <row r="180" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A180" s="53" t="s">
+      <c r="A180" s="45" t="s">
         <v>351</v>
       </c>
       <c r="B180" s="7">
@@ -4695,7 +4714,7 @@
       </c>
     </row>
     <row r="181" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A181" s="53" t="s">
+      <c r="A181" s="45" t="s">
         <v>350</v>
       </c>
       <c r="B181" s="7">
@@ -4710,7 +4729,7 @@
       </c>
     </row>
     <row r="182" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A182" s="53" t="s">
+      <c r="A182" s="45" t="s">
         <v>349</v>
       </c>
       <c r="B182" s="7">
@@ -4740,7 +4759,7 @@
       </c>
     </row>
     <row r="184" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A184" s="53" t="s">
+      <c r="A184" s="45" t="s">
         <v>352</v>
       </c>
       <c r="B184" s="7">
@@ -4755,7 +4774,7 @@
       </c>
     </row>
     <row r="185" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A185" s="53" t="s">
+      <c r="A185" s="45" t="s">
         <v>353</v>
       </c>
       <c r="B185" s="7">
@@ -4770,7 +4789,7 @@
       </c>
     </row>
     <row r="186" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A186" s="53" t="s">
+      <c r="A186" s="45" t="s">
         <v>265</v>
       </c>
       <c r="B186" s="7">
@@ -4785,7 +4804,7 @@
       </c>
     </row>
     <row r="187" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A187" s="53" t="s">
+      <c r="A187" s="45" t="s">
         <v>354</v>
       </c>
       <c r="B187" s="7">
@@ -4800,7 +4819,7 @@
       </c>
     </row>
     <row r="188" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A188" s="53" t="s">
+      <c r="A188" s="45" t="s">
         <v>355</v>
       </c>
       <c r="B188" s="7">
@@ -4815,7 +4834,7 @@
       </c>
     </row>
     <row r="189" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A189" s="53" t="s">
+      <c r="A189" s="45" t="s">
         <v>356</v>
       </c>
       <c r="B189" s="7">
@@ -4830,7 +4849,7 @@
       </c>
     </row>
     <row r="190" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A190" s="53" t="s">
+      <c r="A190" s="45" t="s">
         <v>319</v>
       </c>
       <c r="B190" s="7">
@@ -4845,7 +4864,7 @@
       </c>
     </row>
     <row r="191" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A191" s="53" t="s">
+      <c r="A191" s="45" t="s">
         <v>31</v>
       </c>
       <c r="B191" s="7">
@@ -4860,7 +4879,7 @@
       </c>
     </row>
     <row r="192" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A192" s="53" t="s">
+      <c r="A192" s="45" t="s">
         <v>357</v>
       </c>
       <c r="B192" s="7">
@@ -4870,12 +4889,12 @@
         <v>43721</v>
       </c>
       <c r="D192" s="3">
-        <f t="shared" ref="D192:D199" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
+        <f t="shared" ref="D192:D243" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
         <v>9462</v>
       </c>
     </row>
     <row r="193" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A193" s="53" t="s">
+      <c r="A193" s="45" t="s">
         <v>359</v>
       </c>
       <c r="B193" s="7">
@@ -4890,7 +4909,7 @@
       </c>
     </row>
     <row r="194" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A194" s="53" t="s">
+      <c r="A194" s="45" t="s">
         <v>265</v>
       </c>
       <c r="B194" s="7">
@@ -4905,7 +4924,7 @@
       </c>
     </row>
     <row r="195" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A195" s="53" t="s">
+      <c r="A195" s="45" t="s">
         <v>360</v>
       </c>
       <c r="B195" s="7">
@@ -4920,7 +4939,7 @@
       </c>
     </row>
     <row r="196" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A196" s="53" t="s">
+      <c r="A196" s="45" t="s">
         <v>30</v>
       </c>
       <c r="B196" s="7">
@@ -4935,7 +4954,7 @@
       </c>
     </row>
     <row r="197" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A197" s="53" t="s">
+      <c r="A197" s="45" t="s">
         <v>361</v>
       </c>
       <c r="B197" s="7">
@@ -4950,7 +4969,7 @@
       </c>
     </row>
     <row r="198" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A198" s="53" t="s">
+      <c r="A198" s="45" t="s">
         <v>32</v>
       </c>
       <c r="B198" s="7">
@@ -4965,7 +4984,7 @@
       </c>
     </row>
     <row r="199" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A199" s="53" t="s">
+      <c r="A199" s="45" t="s">
         <v>362</v>
       </c>
       <c r="B199" s="7">
@@ -4974,200 +4993,459 @@
       <c r="C199" s="7">
         <v>46255</v>
       </c>
-      <c r="D199" s="54">
+      <c r="D199" s="3">
         <f t="shared" si="7"/>
         <v>10126</v>
       </c>
     </row>
     <row r="200" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A200" s="7"/>
-      <c r="B200" s="7"/>
-      <c r="C200" s="7"/>
+      <c r="A200" s="54" t="s">
+        <v>360</v>
+      </c>
+      <c r="B200" s="7">
+        <v>36274</v>
+      </c>
+      <c r="C200" s="7">
+        <v>46401</v>
+      </c>
+      <c r="D200" s="3">
+        <f t="shared" si="7"/>
+        <v>10127</v>
+      </c>
     </row>
     <row r="201" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B201" s="7"/>
-      <c r="C201" s="7"/>
+      <c r="A201" s="54" t="s">
+        <v>47</v>
+      </c>
+      <c r="B201" s="7">
+        <v>36893</v>
+      </c>
+      <c r="C201" s="7">
+        <v>47022</v>
+      </c>
+      <c r="D201" s="3">
+        <f t="shared" si="7"/>
+        <v>10129</v>
+      </c>
     </row>
     <row r="202" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B202" s="7"/>
-      <c r="C202" s="7"/>
+      <c r="A202" s="54" t="s">
+        <v>363</v>
+      </c>
+      <c r="B202" s="7">
+        <v>37256</v>
+      </c>
+      <c r="C202" s="7">
+        <v>47544</v>
+      </c>
+      <c r="D202" s="3">
+        <f t="shared" si="7"/>
+        <v>10288</v>
+      </c>
     </row>
     <row r="203" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B203" s="7"/>
-      <c r="C203" s="7"/>
+      <c r="A203" s="54" t="s">
+        <v>364</v>
+      </c>
+      <c r="B203" s="7">
+        <v>37318</v>
+      </c>
+      <c r="C203" s="7">
+        <v>47607</v>
+      </c>
+      <c r="D203" s="3">
+        <f t="shared" si="7"/>
+        <v>10289</v>
+      </c>
     </row>
     <row r="204" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B204" s="7"/>
-      <c r="C204" s="7"/>
+      <c r="A204" s="54" t="s">
+        <v>293</v>
+      </c>
+      <c r="B204" s="7">
+        <v>37574</v>
+      </c>
+      <c r="C204" s="7">
+        <v>47872</v>
+      </c>
+      <c r="D204" s="3">
+        <f t="shared" si="7"/>
+        <v>10298</v>
+      </c>
     </row>
     <row r="205" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B205" s="7"/>
-      <c r="C205" s="7"/>
+      <c r="A205" s="54" t="s">
+        <v>310</v>
+      </c>
+      <c r="B205" s="7">
+        <v>37603</v>
+      </c>
+      <c r="C205" s="7">
+        <v>47897</v>
+      </c>
+      <c r="D205" s="3">
+        <f t="shared" si="7"/>
+        <v>10294</v>
+      </c>
     </row>
     <row r="206" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B206" s="7"/>
-      <c r="C206" s="7"/>
+      <c r="A206" s="54" t="s">
+        <v>364</v>
+      </c>
+      <c r="B206" s="7">
+        <v>37659</v>
+      </c>
+      <c r="C206" s="7">
+        <v>47958</v>
+      </c>
+      <c r="D206" s="3">
+        <f t="shared" si="7"/>
+        <v>10299</v>
+      </c>
     </row>
     <row r="207" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B207" s="7"/>
-      <c r="C207" s="7"/>
+      <c r="A207" s="54" t="s">
+        <v>250</v>
+      </c>
+      <c r="B207" s="7">
+        <v>37993</v>
+      </c>
+      <c r="C207" s="7">
+        <v>48291</v>
+      </c>
+      <c r="D207" s="3">
+        <f t="shared" si="7"/>
+        <v>10298</v>
+      </c>
     </row>
     <row r="208" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B208" s="7"/>
-      <c r="C208" s="7"/>
-    </row>
-    <row r="209" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B209" s="7"/>
-      <c r="C209" s="7"/>
-    </row>
-    <row r="210" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B210" s="7"/>
-      <c r="C210" s="7"/>
-    </row>
-    <row r="211" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B211" s="7"/>
-      <c r="C211" s="7"/>
-    </row>
-    <row r="212" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A208" s="54" t="s">
+        <v>33</v>
+      </c>
+      <c r="B208" s="7">
+        <v>38090</v>
+      </c>
+      <c r="C208" s="7">
+        <v>48390</v>
+      </c>
+      <c r="D208" s="3">
+        <f t="shared" si="7"/>
+        <v>10300</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A209" s="54" t="s">
+        <v>365</v>
+      </c>
+      <c r="B209" s="7">
+        <v>38459</v>
+      </c>
+      <c r="C209" s="7">
+        <v>49072</v>
+      </c>
+      <c r="D209" s="3">
+        <f t="shared" si="7"/>
+        <v>10613</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A210" s="54" t="s">
+        <v>34</v>
+      </c>
+      <c r="B210" s="7">
+        <v>38692</v>
+      </c>
+      <c r="C210" s="7">
+        <v>49304</v>
+      </c>
+      <c r="D210" s="3">
+        <f t="shared" si="7"/>
+        <v>10612</v>
+      </c>
+    </row>
+    <row r="211" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A211" s="54" t="s">
+        <v>366</v>
+      </c>
+      <c r="B211" s="7">
+        <v>39043</v>
+      </c>
+      <c r="C211" s="7">
+        <v>49913</v>
+      </c>
+      <c r="D211" s="3">
+        <f t="shared" si="7"/>
+        <v>10870</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B212" s="7"/>
       <c r="C212" s="7"/>
-    </row>
-    <row r="213" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D212" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="213" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B213" s="7"/>
       <c r="C213" s="7"/>
-    </row>
-    <row r="214" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D213" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B214" s="7"/>
       <c r="C214" s="7"/>
-    </row>
-    <row r="215" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D214" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B215" s="7"/>
       <c r="C215" s="7"/>
-    </row>
-    <row r="216" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D215" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B216" s="7"/>
       <c r="C216" s="7"/>
-    </row>
-    <row r="217" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D216" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="217" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B217" s="7"/>
       <c r="C217" s="7"/>
-    </row>
-    <row r="218" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D217" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="218" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B218" s="7"/>
       <c r="C218" s="7"/>
-    </row>
-    <row r="219" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D218" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B219" s="7"/>
       <c r="C219" s="7"/>
-    </row>
-    <row r="220" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D219" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B220" s="7"/>
       <c r="C220" s="7"/>
-    </row>
-    <row r="221" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D220" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B221" s="7"/>
       <c r="C221" s="7"/>
-    </row>
-    <row r="222" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D221" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="222" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B222" s="7"/>
       <c r="C222" s="7"/>
-    </row>
-    <row r="223" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D222" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="223" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B223" s="7"/>
       <c r="C223" s="7"/>
-    </row>
-    <row r="224" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D223" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="224" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B224" s="7"/>
       <c r="C224" s="7"/>
-    </row>
-    <row r="225" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D224" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="225" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B225" s="7"/>
       <c r="C225" s="7"/>
-    </row>
-    <row r="226" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D225" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="226" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B226" s="7"/>
       <c r="C226" s="7"/>
-    </row>
-    <row r="227" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D226" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="227" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B227" s="7"/>
       <c r="C227" s="7"/>
-    </row>
-    <row r="228" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D227" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="228" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B228" s="7"/>
       <c r="C228" s="7"/>
-    </row>
-    <row r="229" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D228" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="229" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B229" s="7"/>
       <c r="C229" s="7"/>
-    </row>
-    <row r="230" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D229" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="230" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B230" s="7"/>
       <c r="C230" s="7"/>
-    </row>
-    <row r="231" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D230" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="231" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B231" s="7"/>
       <c r="C231" s="7"/>
-    </row>
-    <row r="232" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D231" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="232" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B232" s="7"/>
       <c r="C232" s="7"/>
-    </row>
-    <row r="233" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D232" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="233" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B233" s="7"/>
       <c r="C233" s="7"/>
-    </row>
-    <row r="234" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D233" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="234" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B234" s="7"/>
       <c r="C234" s="7"/>
-    </row>
-    <row r="235" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D234" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="235" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B235" s="7"/>
       <c r="C235" s="7"/>
-    </row>
-    <row r="236" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D235" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="236" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B236" s="7"/>
       <c r="C236" s="7"/>
-    </row>
-    <row r="237" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D236" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="237" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B237" s="7"/>
       <c r="C237" s="7"/>
-    </row>
-    <row r="238" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D237" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="238" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B238" s="7"/>
       <c r="C238" s="7"/>
-    </row>
-    <row r="239" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D238" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="239" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B239" s="7"/>
       <c r="C239" s="7"/>
-    </row>
-    <row r="240" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D239" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="240" spans="2:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B240" s="7"/>
       <c r="C240" s="7"/>
+      <c r="D240" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="241" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B241" s="7"/>
       <c r="C241" s="7"/>
+      <c r="D241" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="242" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B242" s="7"/>
       <c r="C242" s="7"/>
+      <c r="D242" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="243" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A243" s="5" t="s">
+      <c r="B243" s="7"/>
+      <c r="C243" s="7"/>
+      <c r="D243" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="244" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A244" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B243" s="7"/>
-      <c r="C243" s="7">
+      <c r="B244" s="7"/>
+      <c r="C244" s="7">
         <v>63782</v>
       </c>
-      <c r="D243" s="3" t="str">
-        <f t="shared" ref="D243" si="8">IF(C243&lt;&gt;"",IF(B243&lt;&gt;"",B243-C243,"-"), "-")</f>
+      <c r="D244" s="3" t="str">
+        <f t="shared" ref="D244" si="8">IF(C244&lt;&gt;"",IF(B244&lt;&gt;"",B244-C244,"-"), "-")</f>
         <v>-</v>
       </c>
-    </row>
-    <row r="244" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B244" s="7"/>
-      <c r="C244" s="7"/>
     </row>
     <row r="245" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B245" s="7"/>
@@ -5540,6 +5818,10 @@
     <row r="337" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B337" s="7"/>
       <c r="C337" s="7"/>
+    </row>
+    <row r="338" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B338" s="7"/>
+      <c r="C338" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15533,7 +15815,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="26" type="noConversion"/>
+  <phoneticPr fontId="27" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -15563,10 +15845,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="45" t="s">
+      <c r="K1" s="46" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="46"/>
+      <c r="L1" s="47"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -17418,13 +17700,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="47" t="s">
+      <c r="H53" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="48"/>
-      <c r="J53" s="48"/>
-      <c r="K53" s="48"/>
-      <c r="L53" s="49"/>
+      <c r="I53" s="49"/>
+      <c r="J53" s="49"/>
+      <c r="K53" s="49"/>
+      <c r="L53" s="50"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -17446,11 +17728,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="50"/>
-      <c r="I54" s="51"/>
-      <c r="J54" s="51"/>
-      <c r="K54" s="51"/>
-      <c r="L54" s="52"/>
+      <c r="H54" s="51"/>
+      <c r="I54" s="52"/>
+      <c r="J54" s="52"/>
+      <c r="K54" s="52"/>
+      <c r="L54" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner v40 done - 11177 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F487DA55-4ABB-471D-9360-0AE607F8AADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A42C6823-0A7D-43FB-9397-FA2D63CE56A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="73650" yWindow="2610" windowWidth="13785" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="369">
   <si>
     <t>Place</t>
   </si>
@@ -1136,6 +1136,12 @@
   </si>
   <si>
     <t>40 1st move</t>
+  </si>
+  <si>
+    <t>dig to middle</t>
+  </si>
+  <si>
+    <t>41 fall</t>
   </si>
 </sst>
 </file>
@@ -5179,51 +5185,93 @@
       </c>
     </row>
     <row r="212" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B212" s="7"/>
-      <c r="C212" s="7"/>
-      <c r="D212" s="3" t="str">
+      <c r="A212" s="54" t="s">
+        <v>367</v>
+      </c>
+      <c r="B212" s="7">
+        <v>39254</v>
+      </c>
+      <c r="C212" s="7">
+        <v>50126</v>
+      </c>
+      <c r="D212" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>10872</v>
       </c>
     </row>
     <row r="213" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B213" s="7"/>
-      <c r="C213" s="7"/>
-      <c r="D213" s="3" t="str">
+      <c r="A213" s="54" t="s">
+        <v>249</v>
+      </c>
+      <c r="B213" s="7">
+        <v>39424</v>
+      </c>
+      <c r="C213" s="7">
+        <v>50296</v>
+      </c>
+      <c r="D213" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>10872</v>
       </c>
     </row>
     <row r="214" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B214" s="7"/>
-      <c r="C214" s="7"/>
-      <c r="D214" s="3" t="str">
+      <c r="A214" s="54" t="s">
+        <v>248</v>
+      </c>
+      <c r="B214" s="7">
+        <v>39488</v>
+      </c>
+      <c r="C214" s="7">
+        <v>50360</v>
+      </c>
+      <c r="D214" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>10872</v>
       </c>
     </row>
     <row r="215" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B215" s="7"/>
-      <c r="C215" s="7"/>
-      <c r="D215" s="3" t="str">
+      <c r="A215" s="54" t="s">
+        <v>233</v>
+      </c>
+      <c r="B215" s="7">
+        <v>39772</v>
+      </c>
+      <c r="C215" s="7">
+        <v>50644</v>
+      </c>
+      <c r="D215" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>10872</v>
       </c>
     </row>
     <row r="216" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B216" s="7"/>
-      <c r="C216" s="7"/>
-      <c r="D216" s="3" t="str">
+      <c r="A216" s="54" t="s">
+        <v>35</v>
+      </c>
+      <c r="B216" s="7">
+        <v>40011</v>
+      </c>
+      <c r="C216" s="7">
+        <v>50882</v>
+      </c>
+      <c r="D216" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>10871</v>
       </c>
     </row>
     <row r="217" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B217" s="7"/>
-      <c r="C217" s="7"/>
-      <c r="D217" s="3" t="str">
+      <c r="A217" s="54" t="s">
+        <v>368</v>
+      </c>
+      <c r="B217" s="7">
+        <v>40363</v>
+      </c>
+      <c r="C217" s="7">
+        <v>51540</v>
+      </c>
+      <c r="D217" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11177</v>
       </c>
     </row>
     <row r="218" spans="1:4" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lovel 41 done, 11467 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A42C6823-0A7D-43FB-9397-FA2D63CE56A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49D01F10-6BD5-4571-B3C4-55E0EBF4F9DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="73650" yWindow="2610" windowWidth="13785" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="76140" yWindow="2100" windowWidth="8805" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V6" sheetId="7" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="373">
   <si>
     <t>Place</t>
   </si>
@@ -1142,6 +1142,18 @@
   </si>
   <si>
     <t>41 fall</t>
+  </si>
+  <si>
+    <t>gold = 24</t>
+  </si>
+  <si>
+    <t>gold = 14</t>
+  </si>
+  <si>
+    <t>end</t>
+  </si>
+  <si>
+    <t>42 ladder grab</t>
   </si>
 </sst>
 </file>
@@ -1151,12 +1163,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="31" x14ac:knownFonts="1">
+  <fonts count="32" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1574,95 +1593,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1676,28 +1696,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2021,7 +2041,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E338"/>
+  <dimension ref="A1:E337"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -4895,7 +4915,7 @@
         <v>43721</v>
       </c>
       <c r="D192" s="3">
-        <f t="shared" ref="D192:D243" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
+        <f t="shared" ref="D192:D242" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
         <v>9462</v>
       </c>
     </row>
@@ -5005,7 +5025,7 @@
       </c>
     </row>
     <row r="200" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A200" s="54" t="s">
+      <c r="A200" s="46" t="s">
         <v>360</v>
       </c>
       <c r="B200" s="7">
@@ -5020,7 +5040,7 @@
       </c>
     </row>
     <row r="201" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A201" s="54" t="s">
+      <c r="A201" s="46" t="s">
         <v>47</v>
       </c>
       <c r="B201" s="7">
@@ -5035,7 +5055,7 @@
       </c>
     </row>
     <row r="202" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A202" s="54" t="s">
+      <c r="A202" s="46" t="s">
         <v>363</v>
       </c>
       <c r="B202" s="7">
@@ -5050,7 +5070,7 @@
       </c>
     </row>
     <row r="203" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A203" s="54" t="s">
+      <c r="A203" s="46" t="s">
         <v>364</v>
       </c>
       <c r="B203" s="7">
@@ -5065,7 +5085,7 @@
       </c>
     </row>
     <row r="204" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A204" s="54" t="s">
+      <c r="A204" s="46" t="s">
         <v>293</v>
       </c>
       <c r="B204" s="7">
@@ -5080,7 +5100,7 @@
       </c>
     </row>
     <row r="205" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A205" s="54" t="s">
+      <c r="A205" s="46" t="s">
         <v>310</v>
       </c>
       <c r="B205" s="7">
@@ -5095,7 +5115,7 @@
       </c>
     </row>
     <row r="206" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A206" s="54" t="s">
+      <c r="A206" s="46" t="s">
         <v>364</v>
       </c>
       <c r="B206" s="7">
@@ -5110,7 +5130,7 @@
       </c>
     </row>
     <row r="207" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A207" s="54" t="s">
+      <c r="A207" s="46" t="s">
         <v>250</v>
       </c>
       <c r="B207" s="7">
@@ -5125,7 +5145,7 @@
       </c>
     </row>
     <row r="208" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A208" s="54" t="s">
+      <c r="A208" s="46" t="s">
         <v>33</v>
       </c>
       <c r="B208" s="7">
@@ -5140,7 +5160,7 @@
       </c>
     </row>
     <row r="209" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A209" s="54" t="s">
+      <c r="A209" s="46" t="s">
         <v>365</v>
       </c>
       <c r="B209" s="7">
@@ -5155,7 +5175,7 @@
       </c>
     </row>
     <row r="210" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A210" s="54" t="s">
+      <c r="A210" s="46" t="s">
         <v>34</v>
       </c>
       <c r="B210" s="7">
@@ -5170,7 +5190,7 @@
       </c>
     </row>
     <row r="211" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A211" s="54" t="s">
+      <c r="A211" s="46" t="s">
         <v>366</v>
       </c>
       <c r="B211" s="7">
@@ -5185,7 +5205,7 @@
       </c>
     </row>
     <row r="212" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A212" s="54" t="s">
+      <c r="A212" s="46" t="s">
         <v>367</v>
       </c>
       <c r="B212" s="7">
@@ -5200,7 +5220,7 @@
       </c>
     </row>
     <row r="213" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A213" s="54" t="s">
+      <c r="A213" s="46" t="s">
         <v>249</v>
       </c>
       <c r="B213" s="7">
@@ -5215,7 +5235,7 @@
       </c>
     </row>
     <row r="214" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A214" s="54" t="s">
+      <c r="A214" s="46" t="s">
         <v>248</v>
       </c>
       <c r="B214" s="7">
@@ -5230,7 +5250,7 @@
       </c>
     </row>
     <row r="215" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A215" s="54" t="s">
+      <c r="A215" s="46" t="s">
         <v>233</v>
       </c>
       <c r="B215" s="7">
@@ -5245,7 +5265,7 @@
       </c>
     </row>
     <row r="216" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A216" s="54" t="s">
+      <c r="A216" s="46" t="s">
         <v>35</v>
       </c>
       <c r="B216" s="7">
@@ -5260,7 +5280,7 @@
       </c>
     </row>
     <row r="217" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A217" s="54" t="s">
+      <c r="A217" s="46" t="s">
         <v>368</v>
       </c>
       <c r="B217" s="7">
@@ -5275,47 +5295,87 @@
       </c>
     </row>
     <row r="218" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B218" s="7"/>
-      <c r="C218" s="7"/>
-      <c r="D218" s="3" t="str">
+      <c r="A218" s="55" t="s">
+        <v>369</v>
+      </c>
+      <c r="B218" s="7">
+        <v>40385</v>
+      </c>
+      <c r="C218" s="7">
+        <v>51561</v>
+      </c>
+      <c r="D218" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11176</v>
       </c>
     </row>
     <row r="219" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B219" s="7"/>
-      <c r="C219" s="7"/>
-      <c r="D219" s="3" t="str">
+      <c r="A219" s="55" t="s">
+        <v>370</v>
+      </c>
+      <c r="B219" s="7">
+        <v>40498</v>
+      </c>
+      <c r="C219" s="7">
+        <v>51688</v>
+      </c>
+      <c r="D219" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11190</v>
       </c>
     </row>
     <row r="220" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B220" s="7"/>
-      <c r="C220" s="7"/>
-      <c r="D220" s="3" t="str">
+      <c r="A220" s="55" t="s">
+        <v>150</v>
+      </c>
+      <c r="B220" s="7">
+        <v>40670</v>
+      </c>
+      <c r="C220" s="7">
+        <v>51862</v>
+      </c>
+      <c r="D220" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11192</v>
       </c>
     </row>
     <row r="221" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B221" s="7"/>
-      <c r="C221" s="7"/>
-      <c r="D221" s="3" t="str">
+      <c r="A221" s="55" t="s">
+        <v>279</v>
+      </c>
+      <c r="B221" s="7">
+        <v>40837</v>
+      </c>
+      <c r="C221" s="7">
+        <v>52029</v>
+      </c>
+      <c r="D221" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11192</v>
       </c>
     </row>
     <row r="222" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B222" s="7"/>
-      <c r="C222" s="7"/>
-      <c r="D222" s="3" t="str">
+      <c r="A222" s="55" t="s">
+        <v>150</v>
+      </c>
+      <c r="B222" s="7">
+        <v>40887</v>
+      </c>
+      <c r="C222" s="7">
+        <v>52080</v>
+      </c>
+      <c r="D222" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11193</v>
       </c>
     </row>
     <row r="223" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B223" s="7"/>
+      <c r="A223" s="55" t="s">
+        <v>293</v>
+      </c>
+      <c r="B223" s="7">
+        <v>40919</v>
+      </c>
       <c r="C223" s="7"/>
       <c r="D223" s="3" t="str">
         <f t="shared" si="7"/>
@@ -5323,22 +5383,36 @@
       </c>
     </row>
     <row r="224" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B224" s="7"/>
-      <c r="C224" s="7"/>
-      <c r="D224" s="3" t="str">
+      <c r="A224" s="55" t="s">
+        <v>371</v>
+      </c>
+      <c r="B224" s="7">
+        <v>41111</v>
+      </c>
+      <c r="C224" s="7">
+        <v>52303</v>
+      </c>
+      <c r="D224" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="225" spans="2:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B225" s="7"/>
-      <c r="C225" s="7"/>
-      <c r="D225" s="3" t="str">
+        <v>11192</v>
+      </c>
+    </row>
+    <row r="225" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A225" s="55" t="s">
+        <v>372</v>
+      </c>
+      <c r="B225" s="7">
+        <v>41489</v>
+      </c>
+      <c r="C225" s="7">
+        <v>52956</v>
+      </c>
+      <c r="D225" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="226" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+        <v>11467</v>
+      </c>
+    </row>
+    <row r="226" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B226" s="7"/>
       <c r="C226" s="7"/>
       <c r="D226" s="3" t="str">
@@ -5346,7 +5420,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="227" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B227" s="7"/>
       <c r="C227" s="7"/>
       <c r="D227" s="3" t="str">
@@ -5354,7 +5428,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="228" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B228" s="7"/>
       <c r="C228" s="7"/>
       <c r="D228" s="3" t="str">
@@ -5362,7 +5436,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="229" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B229" s="7"/>
       <c r="C229" s="7"/>
       <c r="D229" s="3" t="str">
@@ -5370,7 +5444,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="230" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B230" s="7"/>
       <c r="C230" s="7"/>
       <c r="D230" s="3" t="str">
@@ -5378,7 +5452,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="231" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B231" s="7"/>
       <c r="C231" s="7"/>
       <c r="D231" s="3" t="str">
@@ -5386,7 +5460,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="232" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B232" s="7"/>
       <c r="C232" s="7"/>
       <c r="D232" s="3" t="str">
@@ -5394,7 +5468,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="233" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B233" s="7"/>
       <c r="C233" s="7"/>
       <c r="D233" s="3" t="str">
@@ -5402,7 +5476,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="234" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B234" s="7"/>
       <c r="C234" s="7"/>
       <c r="D234" s="3" t="str">
@@ -5410,7 +5484,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="235" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B235" s="7"/>
       <c r="C235" s="7"/>
       <c r="D235" s="3" t="str">
@@ -5418,7 +5492,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="236" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B236" s="7"/>
       <c r="C236" s="7"/>
       <c r="D236" s="3" t="str">
@@ -5426,7 +5500,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="237" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B237" s="7"/>
       <c r="C237" s="7"/>
       <c r="D237" s="3" t="str">
@@ -5434,7 +5508,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="238" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B238" s="7"/>
       <c r="C238" s="7"/>
       <c r="D238" s="3" t="str">
@@ -5442,7 +5516,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="239" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B239" s="7"/>
       <c r="C239" s="7"/>
       <c r="D239" s="3" t="str">
@@ -5450,7 +5524,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="240" spans="2:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B240" s="7"/>
       <c r="C240" s="7"/>
       <c r="D240" s="3" t="str">
@@ -5475,25 +5549,21 @@
       </c>
     </row>
     <row r="243" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A243" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="B243" s="7"/>
-      <c r="C243" s="7"/>
+      <c r="C243" s="7">
+        <v>63782</v>
+      </c>
       <c r="D243" s="3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="D243" si="8">IF(C243&lt;&gt;"",IF(B243&lt;&gt;"",B243-C243,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="244" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A244" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="B244" s="7"/>
-      <c r="C244" s="7">
-        <v>63782</v>
-      </c>
-      <c r="D244" s="3" t="str">
-        <f t="shared" ref="D244" si="8">IF(C244&lt;&gt;"",IF(B244&lt;&gt;"",B244-C244,"-"), "-")</f>
-        <v>-</v>
-      </c>
+      <c r="C244" s="7"/>
     </row>
     <row r="245" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B245" s="7"/>
@@ -5866,10 +5936,6 @@
     <row r="337" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B337" s="7"/>
       <c r="C337" s="7"/>
-    </row>
-    <row r="338" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B338" s="7"/>
-      <c r="C338" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15863,7 +15929,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="27" type="noConversion"/>
+  <phoneticPr fontId="28" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -15893,10 +15959,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="46" t="s">
+      <c r="K1" s="47" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="47"/>
+      <c r="L1" s="48"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -17748,13 +17814,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="48" t="s">
+      <c r="H53" s="49" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="49"/>
-      <c r="J53" s="49"/>
-      <c r="K53" s="49"/>
-      <c r="L53" s="50"/>
+      <c r="I53" s="50"/>
+      <c r="J53" s="50"/>
+      <c r="K53" s="50"/>
+      <c r="L53" s="51"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -17776,11 +17842,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="51"/>
-      <c r="I54" s="52"/>
-      <c r="J54" s="52"/>
-      <c r="K54" s="52"/>
-      <c r="L54" s="53"/>
+      <c r="H54" s="52"/>
+      <c r="I54" s="53"/>
+      <c r="J54" s="53"/>
+      <c r="K54" s="53"/>
+      <c r="L54" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - lv 42 done - 11728 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49D01F10-6BD5-4571-B3C4-55E0EBF4F9DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{765249C3-1009-4C1F-AAD8-8AE888B74A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="76140" yWindow="2100" windowWidth="8805" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="375">
   <si>
     <t>Place</t>
   </si>
@@ -1154,6 +1154,12 @@
   </si>
   <si>
     <t>42 ladder grab</t>
+  </si>
+  <si>
+    <t>gold = 18</t>
+  </si>
+  <si>
+    <t>43 dig</t>
   </si>
 </sst>
 </file>
@@ -2041,7 +2047,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E337"/>
+  <dimension ref="A1:E343"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -4915,7 +4921,7 @@
         <v>43721</v>
       </c>
       <c r="D192" s="3">
-        <f t="shared" ref="D192:D242" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
+        <f t="shared" ref="D192:D248" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
         <v>9462</v>
       </c>
     </row>
@@ -5413,99 +5419,183 @@
       </c>
     </row>
     <row r="226" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B226" s="7"/>
-      <c r="C226" s="7"/>
-      <c r="D226" s="3" t="str">
+      <c r="A226" s="55" t="s">
+        <v>373</v>
+      </c>
+      <c r="B226" s="7">
+        <v>41570</v>
+      </c>
+      <c r="C226" s="7">
+        <v>53037</v>
+      </c>
+      <c r="D226" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11467</v>
       </c>
     </row>
     <row r="227" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B227" s="7"/>
-      <c r="C227" s="7"/>
-      <c r="D227" s="3" t="str">
+      <c r="A227" s="55" t="s">
+        <v>359</v>
+      </c>
+      <c r="B227" s="7">
+        <v>41659</v>
+      </c>
+      <c r="C227" s="7">
+        <v>53126</v>
+      </c>
+      <c r="D227" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11467</v>
       </c>
     </row>
     <row r="228" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B228" s="7"/>
-      <c r="C228" s="7"/>
-      <c r="D228" s="3" t="str">
+      <c r="A228" s="55" t="s">
+        <v>318</v>
+      </c>
+      <c r="B228" s="7">
+        <v>41748</v>
+      </c>
+      <c r="C228" s="7">
+        <v>53215</v>
+      </c>
+      <c r="D228" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11467</v>
       </c>
     </row>
     <row r="229" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B229" s="7"/>
-      <c r="C229" s="7"/>
-      <c r="D229" s="3" t="str">
+      <c r="A229" s="55" t="s">
+        <v>359</v>
+      </c>
+      <c r="B229" s="7">
+        <v>41866</v>
+      </c>
+      <c r="C229" s="7">
+        <v>53333</v>
+      </c>
+      <c r="D229" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11467</v>
       </c>
     </row>
     <row r="230" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B230" s="7"/>
-      <c r="C230" s="7"/>
-      <c r="D230" s="3" t="str">
+      <c r="A230" s="55" t="s">
+        <v>311</v>
+      </c>
+      <c r="B230" s="7">
+        <v>41978</v>
+      </c>
+      <c r="C230" s="7">
+        <v>53451</v>
+      </c>
+      <c r="D230" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11473</v>
       </c>
     </row>
     <row r="231" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B231" s="7"/>
-      <c r="C231" s="7"/>
-      <c r="D231" s="3" t="str">
+      <c r="A231" s="55" t="s">
+        <v>359</v>
+      </c>
+      <c r="B231" s="7">
+        <v>42018</v>
+      </c>
+      <c r="C231" s="7">
+        <v>53489</v>
+      </c>
+      <c r="D231" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11471</v>
       </c>
     </row>
     <row r="232" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B232" s="7"/>
-      <c r="C232" s="7"/>
-      <c r="D232" s="3" t="str">
+      <c r="A232" s="55" t="s">
+        <v>312</v>
+      </c>
+      <c r="B232" s="7">
+        <v>42096</v>
+      </c>
+      <c r="C232" s="7">
+        <v>53567</v>
+      </c>
+      <c r="D232" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11471</v>
       </c>
     </row>
     <row r="233" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B233" s="7"/>
-      <c r="C233" s="7"/>
-      <c r="D233" s="3" t="str">
+      <c r="A233" s="55" t="s">
+        <v>279</v>
+      </c>
+      <c r="B233" s="7">
+        <v>42125</v>
+      </c>
+      <c r="C233" s="7">
+        <v>53598</v>
+      </c>
+      <c r="D233" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11473</v>
       </c>
     </row>
     <row r="234" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B234" s="7"/>
-      <c r="C234" s="7"/>
-      <c r="D234" s="3" t="str">
+      <c r="A234" s="55" t="s">
+        <v>265</v>
+      </c>
+      <c r="B234" s="7">
+        <v>42233</v>
+      </c>
+      <c r="C234" s="7">
+        <v>53709</v>
+      </c>
+      <c r="D234" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11476</v>
       </c>
     </row>
     <row r="235" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B235" s="7"/>
-      <c r="C235" s="7"/>
-      <c r="D235" s="3" t="str">
+      <c r="A235" s="55" t="s">
+        <v>250</v>
+      </c>
+      <c r="B235" s="7">
+        <v>42324</v>
+      </c>
+      <c r="C235" s="7">
+        <v>53801</v>
+      </c>
+      <c r="D235" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11477</v>
       </c>
     </row>
     <row r="236" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B236" s="7"/>
-      <c r="C236" s="7"/>
-      <c r="D236" s="3" t="str">
+      <c r="A236" t="s">
+        <v>37</v>
+      </c>
+      <c r="B236" s="7">
+        <v>42450</v>
+      </c>
+      <c r="C236" s="7">
+        <v>53932</v>
+      </c>
+      <c r="D236" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11482</v>
       </c>
     </row>
     <row r="237" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B237" s="7"/>
-      <c r="C237" s="7"/>
-      <c r="D237" s="3" t="str">
+      <c r="A237" s="55" t="s">
+        <v>374</v>
+      </c>
+      <c r="B237" s="7">
+        <v>42803</v>
+      </c>
+      <c r="C237" s="7">
+        <v>54531</v>
+      </c>
+      <c r="D237" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>11728</v>
       </c>
     </row>
     <row r="238" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -5549,41 +5639,65 @@
       </c>
     </row>
     <row r="243" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A243" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="B243" s="7"/>
-      <c r="C243" s="7">
-        <v>63782</v>
-      </c>
+      <c r="C243" s="7"/>
       <c r="D243" s="3" t="str">
-        <f t="shared" ref="D243" si="8">IF(C243&lt;&gt;"",IF(B243&lt;&gt;"",B243-C243,"-"), "-")</f>
+        <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
     <row r="244" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B244" s="7"/>
       <c r="C244" s="7"/>
+      <c r="D244" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="245" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B245" s="7"/>
       <c r="C245" s="7"/>
+      <c r="D245" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="246" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B246" s="7"/>
       <c r="C246" s="7"/>
+      <c r="D246" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="247" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B247" s="7"/>
       <c r="C247" s="7"/>
+      <c r="D247" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="248" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B248" s="7"/>
       <c r="C248" s="7"/>
+      <c r="D248" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="249" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A249" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="B249" s="7"/>
-      <c r="C249" s="7"/>
+      <c r="C249" s="7">
+        <v>63782</v>
+      </c>
+      <c r="D249" s="3" t="str">
+        <f t="shared" ref="D249" si="8">IF(C249&lt;&gt;"",IF(B249&lt;&gt;"",B249-C249,"-"), "-")</f>
+        <v>-</v>
+      </c>
     </row>
     <row r="250" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B250" s="7"/>
@@ -5936,6 +6050,30 @@
     <row r="337" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B337" s="7"/>
       <c r="C337" s="7"/>
+    </row>
+    <row r="338" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B338" s="7"/>
+      <c r="C338" s="7"/>
+    </row>
+    <row r="339" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B339" s="7"/>
+      <c r="C339" s="7"/>
+    </row>
+    <row r="340" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B340" s="7"/>
+      <c r="C340" s="7"/>
+    </row>
+    <row r="341" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B341" s="7"/>
+      <c r="C341" s="7"/>
+    </row>
+    <row r="342" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B342" s="7"/>
+      <c r="C342" s="7"/>
+    </row>
+    <row r="343" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B343" s="7"/>
+      <c r="C343" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - working on level 44
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{765249C3-1009-4C1F-AAD8-8AE888B74A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A516DFB6-3848-4236-BBB9-B10BE3D12050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="76140" yWindow="2100" windowWidth="8805" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="50745" yWindow="3435" windowWidth="6720" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V6" sheetId="7" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="382">
   <si>
     <t>Place</t>
   </si>
@@ -1160,6 +1160,27 @@
   </si>
   <si>
     <t>43 dig</t>
+  </si>
+  <si>
+    <t>44 1st move</t>
+  </si>
+  <si>
+    <t>45 1st move</t>
+  </si>
+  <si>
+    <t>46 1st move</t>
+  </si>
+  <si>
+    <t>47 1st move</t>
+  </si>
+  <si>
+    <t>48 1st move</t>
+  </si>
+  <si>
+    <t>49 dig</t>
+  </si>
+  <si>
+    <t>50 1st move</t>
   </si>
 </sst>
 </file>
@@ -1610,7 +1631,7 @@
     <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1727,6 +1748,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2047,7 +2069,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E343"/>
+  <dimension ref="A1:E360"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -4921,7 +4943,7 @@
         <v>43721</v>
       </c>
       <c r="D192" s="3">
-        <f t="shared" ref="D192:D248" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
+        <f t="shared" ref="D192:D265" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
         <v>9462</v>
       </c>
     </row>
@@ -5599,195 +5621,479 @@
       </c>
     </row>
     <row r="238" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B238" s="7"/>
-      <c r="C238" s="7"/>
-      <c r="D238" s="3" t="str">
+      <c r="A238" s="55" t="s">
+        <v>311</v>
+      </c>
+      <c r="B238" s="7">
+        <v>42860</v>
+      </c>
+      <c r="C238" s="7">
+        <v>54588</v>
+      </c>
+      <c r="D238" s="3">
+        <f t="shared" si="7"/>
+        <v>11728</v>
+      </c>
+    </row>
+    <row r="239" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A239" s="55" t="s">
+        <v>312</v>
+      </c>
+      <c r="B239" s="7">
+        <v>42885</v>
+      </c>
+      <c r="C239" s="7">
+        <v>54613</v>
+      </c>
+      <c r="D239" s="3">
+        <f t="shared" si="7"/>
+        <v>11728</v>
+      </c>
+    </row>
+    <row r="240" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A240" s="55" t="s">
+        <v>279</v>
+      </c>
+      <c r="B240" s="7">
+        <v>42913</v>
+      </c>
+      <c r="C240" s="7">
+        <v>54641</v>
+      </c>
+      <c r="D240" s="3">
+        <f t="shared" si="7"/>
+        <v>11728</v>
+      </c>
+    </row>
+    <row r="241" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A241" s="55" t="s">
+        <v>150</v>
+      </c>
+      <c r="B241" s="7">
+        <v>42933</v>
+      </c>
+      <c r="C241" s="7">
+        <v>54661</v>
+      </c>
+      <c r="D241" s="3">
+        <f t="shared" si="7"/>
+        <v>11728</v>
+      </c>
+    </row>
+    <row r="242" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A242" s="55" t="s">
+        <v>150</v>
+      </c>
+      <c r="B242" s="7">
+        <v>42966</v>
+      </c>
+      <c r="C242" s="7">
+        <v>54693</v>
+      </c>
+      <c r="D242" s="3">
+        <f t="shared" si="7"/>
+        <v>11727</v>
+      </c>
+    </row>
+    <row r="243" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A243" s="55" t="s">
+        <v>150</v>
+      </c>
+      <c r="B243" s="7">
+        <v>43005</v>
+      </c>
+      <c r="C243" s="7">
+        <v>54732</v>
+      </c>
+      <c r="D243" s="3">
+        <f t="shared" si="7"/>
+        <v>11727</v>
+      </c>
+    </row>
+    <row r="244" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A244" s="55" t="s">
+        <v>302</v>
+      </c>
+      <c r="B244" s="7">
+        <v>43039</v>
+      </c>
+      <c r="C244" s="7">
+        <v>54766</v>
+      </c>
+      <c r="D244" s="3">
+        <f t="shared" si="7"/>
+        <v>11727</v>
+      </c>
+    </row>
+    <row r="245" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A245" s="55" t="s">
+        <v>249</v>
+      </c>
+      <c r="B245" s="7">
+        <v>43054</v>
+      </c>
+      <c r="C245" s="7">
+        <v>54780</v>
+      </c>
+      <c r="D245" s="3">
+        <f t="shared" si="7"/>
+        <v>11726</v>
+      </c>
+    </row>
+    <row r="246" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A246" s="55" t="s">
+        <v>38</v>
+      </c>
+      <c r="B246" s="7">
+        <v>43143</v>
+      </c>
+      <c r="C246" s="7">
+        <v>54875</v>
+      </c>
+      <c r="D246" s="3">
+        <f t="shared" si="7"/>
+        <v>11732</v>
+      </c>
+    </row>
+    <row r="247" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A247" s="55" t="s">
+        <v>375</v>
+      </c>
+      <c r="B247" s="7">
+        <v>43493</v>
+      </c>
+      <c r="C247" s="7">
+        <v>55525</v>
+      </c>
+      <c r="D247" s="3">
+        <f t="shared" si="7"/>
+        <v>12032</v>
+      </c>
+    </row>
+    <row r="248" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A248" s="55" t="s">
+        <v>306</v>
+      </c>
+      <c r="B248" s="7">
+        <v>43501</v>
+      </c>
+      <c r="C248" s="7">
+        <v>55533</v>
+      </c>
+      <c r="D248" s="3">
+        <f t="shared" si="7"/>
+        <v>12032</v>
+      </c>
+    </row>
+    <row r="249" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A249" s="55" t="s">
+        <v>319</v>
+      </c>
+      <c r="B249" s="7">
+        <v>43529</v>
+      </c>
+      <c r="C249" s="7">
+        <v>55569</v>
+      </c>
+      <c r="D249" s="3">
+        <f t="shared" si="7"/>
+        <v>12040</v>
+      </c>
+    </row>
+    <row r="250" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A250" s="55" t="s">
+        <v>311</v>
+      </c>
+      <c r="B250" s="7">
+        <v>43584</v>
+      </c>
+      <c r="C250" s="7">
+        <v>55669</v>
+      </c>
+      <c r="D250" s="3">
+        <f t="shared" si="7"/>
+        <v>12085</v>
+      </c>
+    </row>
+    <row r="251" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A251" s="55" t="s">
+        <v>312</v>
+      </c>
+      <c r="B251" s="7">
+        <v>43622</v>
+      </c>
+      <c r="C251" s="7">
+        <v>55702</v>
+      </c>
+      <c r="D251" s="3">
+        <f t="shared" si="7"/>
+        <v>12080</v>
+      </c>
+    </row>
+    <row r="252" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A252" s="55" t="s">
+        <v>279</v>
+      </c>
+      <c r="B252" s="7">
+        <v>43664</v>
+      </c>
+      <c r="C252" s="7">
+        <v>55744</v>
+      </c>
+      <c r="D252" s="3">
+        <f t="shared" si="7"/>
+        <v>12080</v>
+      </c>
+    </row>
+    <row r="253" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A253" s="55" t="s">
+        <v>293</v>
+      </c>
+      <c r="B253" s="7">
+        <v>43782</v>
+      </c>
+      <c r="C253" s="7">
+        <v>55865</v>
+      </c>
+      <c r="D253" s="3">
+        <f t="shared" si="7"/>
+        <v>12083</v>
+      </c>
+    </row>
+    <row r="254" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A254" s="55" t="s">
+        <v>247</v>
+      </c>
+      <c r="B254" s="7">
+        <v>43825</v>
+      </c>
+      <c r="C254" s="7">
+        <v>55908</v>
+      </c>
+      <c r="D254" s="3">
+        <f t="shared" si="7"/>
+        <v>12083</v>
+      </c>
+    </row>
+    <row r="255" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A255" s="55" t="s">
+        <v>302</v>
+      </c>
+      <c r="B255" s="7">
+        <v>43947</v>
+      </c>
+      <c r="C255" s="7">
+        <v>56048</v>
+      </c>
+      <c r="D255" s="3">
+        <f t="shared" si="7"/>
+        <v>12101</v>
+      </c>
+    </row>
+    <row r="256" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A256" s="55" t="s">
+        <v>249</v>
+      </c>
+      <c r="B256" s="7">
+        <v>43992</v>
+      </c>
+      <c r="C256" s="7">
+        <v>56077</v>
+      </c>
+      <c r="D256" s="3">
+        <f t="shared" si="7"/>
+        <v>12085</v>
+      </c>
+    </row>
+    <row r="257" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A257" s="55"/>
+      <c r="B257" s="7"/>
+      <c r="C257" s="7"/>
+      <c r="D257" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="239" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B239" s="7"/>
-      <c r="C239" s="7"/>
-      <c r="D239" s="3" t="str">
+    <row r="258" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="B258" s="7"/>
+      <c r="C258" s="7"/>
+      <c r="D258" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="240" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B240" s="7"/>
-      <c r="C240" s="7"/>
-      <c r="D240" s="3" t="str">
+    <row r="259" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A259" s="55" t="s">
+        <v>39</v>
+      </c>
+      <c r="B259" s="7">
+        <v>44167</v>
+      </c>
+      <c r="C259" s="7">
+        <v>56197</v>
+      </c>
+      <c r="D259" s="3">
+        <f t="shared" si="7"/>
+        <v>12030</v>
+      </c>
+    </row>
+    <row r="260" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A260" s="55" t="s">
+        <v>376</v>
+      </c>
+      <c r="B260" s="7"/>
+      <c r="C260" s="7">
+        <v>45805</v>
+      </c>
+      <c r="D260" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="241" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B241" s="7"/>
-      <c r="C241" s="7"/>
-      <c r="D241" s="3" t="str">
+    <row r="261" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A261" s="55" t="s">
+        <v>40</v>
+      </c>
+      <c r="B261" s="7"/>
+      <c r="C261" s="7">
+        <v>54354</v>
+      </c>
+      <c r="D261" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="242" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B242" s="7"/>
-      <c r="C242" s="7"/>
-      <c r="D242" s="3" t="str">
+    <row r="262" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A262" s="55" t="s">
+        <v>377</v>
+      </c>
+      <c r="B262" s="7"/>
+      <c r="C262" s="7">
+        <v>57998</v>
+      </c>
+      <c r="D262" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="243" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B243" s="7"/>
-      <c r="C243" s="7"/>
-      <c r="D243" s="3" t="str">
+    <row r="263" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A263" s="55" t="s">
+        <v>41</v>
+      </c>
+      <c r="B263" s="7"/>
+      <c r="C263" s="7">
+        <v>58570</v>
+      </c>
+      <c r="D263" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="244" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B244" s="7"/>
-      <c r="C244" s="7"/>
-      <c r="D244" s="3" t="str">
+    <row r="264" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A264" s="55" t="s">
+        <v>378</v>
+      </c>
+      <c r="B264" s="7"/>
+      <c r="C264" s="7">
+        <v>59229</v>
+      </c>
+      <c r="D264" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="245" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B245" s="7"/>
-      <c r="C245" s="7"/>
-      <c r="D245" s="3" t="str">
+    <row r="265" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A265" s="55" t="s">
+        <v>42</v>
+      </c>
+      <c r="B265" s="7"/>
+      <c r="C265" s="7">
+        <v>60018</v>
+      </c>
+      <c r="D265" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="246" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B246" s="7"/>
-      <c r="C246" s="7"/>
-      <c r="D246" s="3" t="str">
-        <f t="shared" si="7"/>
+    <row r="266" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A266" s="55" t="s">
+        <v>379</v>
+      </c>
+      <c r="B266" s="7"/>
+      <c r="C266" s="7">
+        <v>60667</v>
+      </c>
+      <c r="D266" s="3" t="str">
+        <f t="shared" ref="D266:D271" si="8">IF(C266&lt;&gt;"",IF(B266&lt;&gt;"",B266-C266,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="247" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B247" s="7"/>
-      <c r="C247" s="7"/>
-      <c r="D247" s="3" t="str">
-        <f t="shared" si="7"/>
+    <row r="267" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A267" s="55" t="s">
+        <v>43</v>
+      </c>
+      <c r="B267" s="7"/>
+      <c r="C267" s="7">
+        <v>61224</v>
+      </c>
+      <c r="D267" s="56" t="str">
+        <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
-    <row r="248" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B248" s="7"/>
-      <c r="C248" s="7"/>
-      <c r="D248" s="3" t="str">
-        <f t="shared" si="7"/>
+    <row r="268" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A268" s="55" t="s">
+        <v>380</v>
+      </c>
+      <c r="B268" s="7"/>
+      <c r="C268" s="7">
+        <v>61892</v>
+      </c>
+      <c r="D268" s="56" t="str">
+        <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
-    <row r="249" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A249" s="5" t="s">
+    <row r="269" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A269" s="55" t="s">
+        <v>44</v>
+      </c>
+      <c r="B269" s="7"/>
+      <c r="C269" s="7">
+        <v>62616</v>
+      </c>
+      <c r="D269" s="56" t="str">
+        <f t="shared" si="8"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="270" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A270" s="55" t="s">
+        <v>381</v>
+      </c>
+      <c r="B270" s="7"/>
+      <c r="C270" s="7">
+        <v>63244</v>
+      </c>
+      <c r="D270" s="56" t="str">
+        <f t="shared" si="8"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="271" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A271" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="B249" s="7"/>
-      <c r="C249" s="7">
+      <c r="B271" s="7"/>
+      <c r="C271" s="7">
         <v>63782</v>
       </c>
-      <c r="D249" s="3" t="str">
-        <f t="shared" ref="D249" si="8">IF(C249&lt;&gt;"",IF(B249&lt;&gt;"",B249-C249,"-"), "-")</f>
+      <c r="D271" s="56" t="str">
+        <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
-    <row r="250" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B250" s="7"/>
-      <c r="C250" s="7"/>
-    </row>
-    <row r="251" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B251" s="7"/>
-      <c r="C251" s="7"/>
-    </row>
-    <row r="252" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B252" s="7"/>
-      <c r="C252" s="7"/>
-    </row>
-    <row r="253" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B253" s="7"/>
-      <c r="C253" s="7"/>
-    </row>
-    <row r="254" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B254" s="7"/>
-      <c r="C254" s="7"/>
-    </row>
-    <row r="255" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B255" s="7"/>
-      <c r="C255" s="7"/>
-    </row>
-    <row r="256" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B256" s="7"/>
-      <c r="C256" s="7"/>
-    </row>
-    <row r="257" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B257" s="7"/>
-      <c r="C257" s="7"/>
-    </row>
-    <row r="258" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B258" s="7"/>
-      <c r="C258" s="7"/>
-    </row>
-    <row r="259" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B259" s="7"/>
-      <c r="C259" s="7"/>
-    </row>
-    <row r="260" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B260" s="7"/>
-      <c r="C260" s="7"/>
-    </row>
-    <row r="261" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B261" s="7"/>
-      <c r="C261" s="7"/>
-    </row>
-    <row r="262" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B262" s="7"/>
-      <c r="C262" s="7"/>
-    </row>
-    <row r="263" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B263" s="7"/>
-      <c r="C263" s="7"/>
-    </row>
-    <row r="264" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B264" s="7"/>
-      <c r="C264" s="7"/>
-    </row>
-    <row r="265" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B265" s="7"/>
-      <c r="C265" s="7"/>
-    </row>
-    <row r="266" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B266" s="7"/>
-      <c r="C266" s="7"/>
-    </row>
-    <row r="267" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B267" s="7"/>
-      <c r="C267" s="7"/>
-    </row>
-    <row r="268" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B268" s="7"/>
-      <c r="C268" s="7"/>
-    </row>
-    <row r="269" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B269" s="7"/>
-      <c r="C269" s="7"/>
-    </row>
-    <row r="270" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B270" s="7"/>
-      <c r="C270" s="7"/>
-    </row>
-    <row r="271" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B271" s="7"/>
-      <c r="C271" s="7"/>
-    </row>
-    <row r="272" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B272" s="7"/>
       <c r="C272" s="7"/>
     </row>
@@ -6074,6 +6380,74 @@
     <row r="343" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B343" s="7"/>
       <c r="C343" s="7"/>
+    </row>
+    <row r="344" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B344" s="7"/>
+      <c r="C344" s="7"/>
+    </row>
+    <row r="345" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B345" s="7"/>
+      <c r="C345" s="7"/>
+    </row>
+    <row r="346" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B346" s="7"/>
+      <c r="C346" s="7"/>
+    </row>
+    <row r="347" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B347" s="7"/>
+      <c r="C347" s="7"/>
+    </row>
+    <row r="348" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B348" s="7"/>
+      <c r="C348" s="7"/>
+    </row>
+    <row r="349" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B349" s="7"/>
+      <c r="C349" s="7"/>
+    </row>
+    <row r="350" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B350" s="7"/>
+      <c r="C350" s="7"/>
+    </row>
+    <row r="351" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B351" s="7"/>
+      <c r="C351" s="7"/>
+    </row>
+    <row r="352" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B352" s="7"/>
+      <c r="C352" s="7"/>
+    </row>
+    <row r="353" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B353" s="7"/>
+      <c r="C353" s="7"/>
+    </row>
+    <row r="354" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B354" s="7"/>
+      <c r="C354" s="7"/>
+    </row>
+    <row r="355" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B355" s="7"/>
+      <c r="C355" s="7"/>
+    </row>
+    <row r="356" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B356" s="7"/>
+      <c r="C356" s="7"/>
+    </row>
+    <row r="357" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B357" s="7"/>
+      <c r="C357" s="7"/>
+    </row>
+    <row r="358" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B358" s="7"/>
+      <c r="C358" s="7"/>
+    </row>
+    <row r="359" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B359" s="7"/>
+      <c r="C359" s="7"/>
+    </row>
+    <row r="360" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B360" s="7"/>
+      <c r="C360" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - 45 done, 12589 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A516DFB6-3848-4236-BBB9-B10BE3D12050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D622F60-BDFF-4EBC-AC8C-BEFE79544249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50745" yWindow="3435" windowWidth="6720" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="50745" yWindow="3210" windowWidth="6720" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V6" sheetId="7" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="382">
   <si>
     <t>Place</t>
   </si>
@@ -1190,12 +1190,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="32" x14ac:knownFonts="1">
+  <fonts count="33" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1620,95 +1627,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1723,32 +1731,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2069,7 +2076,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E360"/>
+  <dimension ref="A1:E365"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -4943,7 +4950,7 @@
         <v>43721</v>
       </c>
       <c r="D192" s="3">
-        <f t="shared" ref="D192:D265" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
+        <f t="shared" ref="D192:D270" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
         <v>9462</v>
       </c>
     </row>
@@ -5323,7 +5330,7 @@
       </c>
     </row>
     <row r="218" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A218" s="55" t="s">
+      <c r="A218" s="47" t="s">
         <v>369</v>
       </c>
       <c r="B218" s="7">
@@ -5338,7 +5345,7 @@
       </c>
     </row>
     <row r="219" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A219" s="55" t="s">
+      <c r="A219" s="47" t="s">
         <v>370</v>
       </c>
       <c r="B219" s="7">
@@ -5353,7 +5360,7 @@
       </c>
     </row>
     <row r="220" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A220" s="55" t="s">
+      <c r="A220" s="47" t="s">
         <v>150</v>
       </c>
       <c r="B220" s="7">
@@ -5368,7 +5375,7 @@
       </c>
     </row>
     <row r="221" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A221" s="55" t="s">
+      <c r="A221" s="47" t="s">
         <v>279</v>
       </c>
       <c r="B221" s="7">
@@ -5383,7 +5390,7 @@
       </c>
     </row>
     <row r="222" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A222" s="55" t="s">
+      <c r="A222" s="47" t="s">
         <v>150</v>
       </c>
       <c r="B222" s="7">
@@ -5398,7 +5405,7 @@
       </c>
     </row>
     <row r="223" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A223" s="55" t="s">
+      <c r="A223" s="47" t="s">
         <v>293</v>
       </c>
       <c r="B223" s="7">
@@ -5411,7 +5418,7 @@
       </c>
     </row>
     <row r="224" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A224" s="55" t="s">
+      <c r="A224" s="47" t="s">
         <v>371</v>
       </c>
       <c r="B224" s="7">
@@ -5426,7 +5433,7 @@
       </c>
     </row>
     <row r="225" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A225" s="55" t="s">
+      <c r="A225" s="47" t="s">
         <v>372</v>
       </c>
       <c r="B225" s="7">
@@ -5441,7 +5448,7 @@
       </c>
     </row>
     <row r="226" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A226" s="55" t="s">
+      <c r="A226" s="47" t="s">
         <v>373</v>
       </c>
       <c r="B226" s="7">
@@ -5456,7 +5463,7 @@
       </c>
     </row>
     <row r="227" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A227" s="55" t="s">
+      <c r="A227" s="47" t="s">
         <v>359</v>
       </c>
       <c r="B227" s="7">
@@ -5471,7 +5478,7 @@
       </c>
     </row>
     <row r="228" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A228" s="55" t="s">
+      <c r="A228" s="47" t="s">
         <v>318</v>
       </c>
       <c r="B228" s="7">
@@ -5486,7 +5493,7 @@
       </c>
     </row>
     <row r="229" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A229" s="55" t="s">
+      <c r="A229" s="47" t="s">
         <v>359</v>
       </c>
       <c r="B229" s="7">
@@ -5501,7 +5508,7 @@
       </c>
     </row>
     <row r="230" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A230" s="55" t="s">
+      <c r="A230" s="47" t="s">
         <v>311</v>
       </c>
       <c r="B230" s="7">
@@ -5516,7 +5523,7 @@
       </c>
     </row>
     <row r="231" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A231" s="55" t="s">
+      <c r="A231" s="47" t="s">
         <v>359</v>
       </c>
       <c r="B231" s="7">
@@ -5531,7 +5538,7 @@
       </c>
     </row>
     <row r="232" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A232" s="55" t="s">
+      <c r="A232" s="47" t="s">
         <v>312</v>
       </c>
       <c r="B232" s="7">
@@ -5546,7 +5553,7 @@
       </c>
     </row>
     <row r="233" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A233" s="55" t="s">
+      <c r="A233" s="47" t="s">
         <v>279</v>
       </c>
       <c r="B233" s="7">
@@ -5561,7 +5568,7 @@
       </c>
     </row>
     <row r="234" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A234" s="55" t="s">
+      <c r="A234" s="47" t="s">
         <v>265</v>
       </c>
       <c r="B234" s="7">
@@ -5576,7 +5583,7 @@
       </c>
     </row>
     <row r="235" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A235" s="55" t="s">
+      <c r="A235" s="47" t="s">
         <v>250</v>
       </c>
       <c r="B235" s="7">
@@ -5606,7 +5613,7 @@
       </c>
     </row>
     <row r="237" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A237" s="55" t="s">
+      <c r="A237" s="47" t="s">
         <v>374</v>
       </c>
       <c r="B237" s="7">
@@ -5621,7 +5628,7 @@
       </c>
     </row>
     <row r="238" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A238" s="55" t="s">
+      <c r="A238" s="47" t="s">
         <v>311</v>
       </c>
       <c r="B238" s="7">
@@ -5636,7 +5643,7 @@
       </c>
     </row>
     <row r="239" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A239" s="55" t="s">
+      <c r="A239" s="47" t="s">
         <v>312</v>
       </c>
       <c r="B239" s="7">
@@ -5651,7 +5658,7 @@
       </c>
     </row>
     <row r="240" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A240" s="55" t="s">
+      <c r="A240" s="47" t="s">
         <v>279</v>
       </c>
       <c r="B240" s="7">
@@ -5666,7 +5673,7 @@
       </c>
     </row>
     <row r="241" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A241" s="55" t="s">
+      <c r="A241" s="47" t="s">
         <v>150</v>
       </c>
       <c r="B241" s="7">
@@ -5681,7 +5688,7 @@
       </c>
     </row>
     <row r="242" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A242" s="55" t="s">
+      <c r="A242" s="47" t="s">
         <v>150</v>
       </c>
       <c r="B242" s="7">
@@ -5696,7 +5703,7 @@
       </c>
     </row>
     <row r="243" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A243" s="55" t="s">
+      <c r="A243" s="47" t="s">
         <v>150</v>
       </c>
       <c r="B243" s="7">
@@ -5711,7 +5718,7 @@
       </c>
     </row>
     <row r="244" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A244" s="55" t="s">
+      <c r="A244" s="47" t="s">
         <v>302</v>
       </c>
       <c r="B244" s="7">
@@ -5726,7 +5733,7 @@
       </c>
     </row>
     <row r="245" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A245" s="55" t="s">
+      <c r="A245" s="47" t="s">
         <v>249</v>
       </c>
       <c r="B245" s="7">
@@ -5741,7 +5748,7 @@
       </c>
     </row>
     <row r="246" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A246" s="55" t="s">
+      <c r="A246" s="47" t="s">
         <v>38</v>
       </c>
       <c r="B246" s="7">
@@ -5756,7 +5763,7 @@
       </c>
     </row>
     <row r="247" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A247" s="55" t="s">
+      <c r="A247" s="47" t="s">
         <v>375</v>
       </c>
       <c r="B247" s="7">
@@ -5771,7 +5778,7 @@
       </c>
     </row>
     <row r="248" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A248" s="55" t="s">
+      <c r="A248" s="47" t="s">
         <v>306</v>
       </c>
       <c r="B248" s="7">
@@ -5786,7 +5793,7 @@
       </c>
     </row>
     <row r="249" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A249" s="55" t="s">
+      <c r="A249" s="47" t="s">
         <v>319</v>
       </c>
       <c r="B249" s="7">
@@ -5801,7 +5808,7 @@
       </c>
     </row>
     <row r="250" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A250" s="55" t="s">
+      <c r="A250" s="47" t="s">
         <v>311</v>
       </c>
       <c r="B250" s="7">
@@ -5816,7 +5823,7 @@
       </c>
     </row>
     <row r="251" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A251" s="55" t="s">
+      <c r="A251" s="47" t="s">
         <v>312</v>
       </c>
       <c r="B251" s="7">
@@ -5831,7 +5838,7 @@
       </c>
     </row>
     <row r="252" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A252" s="55" t="s">
+      <c r="A252" s="47" t="s">
         <v>279</v>
       </c>
       <c r="B252" s="7">
@@ -5846,7 +5853,7 @@
       </c>
     </row>
     <row r="253" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A253" s="55" t="s">
+      <c r="A253" s="47" t="s">
         <v>293</v>
       </c>
       <c r="B253" s="7">
@@ -5861,7 +5868,7 @@
       </c>
     </row>
     <row r="254" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A254" s="55" t="s">
+      <c r="A254" s="47" t="s">
         <v>247</v>
       </c>
       <c r="B254" s="7">
@@ -5876,7 +5883,7 @@
       </c>
     </row>
     <row r="255" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A255" s="55" t="s">
+      <c r="A255" s="47" t="s">
         <v>302</v>
       </c>
       <c r="B255" s="7">
@@ -5891,7 +5898,7 @@
       </c>
     </row>
     <row r="256" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A256" s="55" t="s">
+      <c r="A256" s="47" t="s">
         <v>249</v>
       </c>
       <c r="B256" s="7">
@@ -5906,258 +5913,332 @@
       </c>
     </row>
     <row r="257" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A257" s="55"/>
-      <c r="B257" s="7"/>
-      <c r="C257" s="7"/>
-      <c r="D257" s="3" t="str">
+      <c r="A257" s="47" t="s">
+        <v>39</v>
+      </c>
+      <c r="B257" s="7">
+        <v>44163</v>
+      </c>
+      <c r="C257" s="7">
+        <v>56197</v>
+      </c>
+      <c r="D257" s="3">
+        <f t="shared" si="7"/>
+        <v>12034</v>
+      </c>
+    </row>
+    <row r="258" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A258" s="47" t="s">
+        <v>376</v>
+      </c>
+      <c r="B258" s="7">
+        <v>44514</v>
+      </c>
+      <c r="C258" s="7">
+        <v>56805</v>
+      </c>
+      <c r="D258" s="3">
+        <f t="shared" si="7"/>
+        <v>12291</v>
+      </c>
+    </row>
+    <row r="259" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A259" s="56" t="s">
+        <v>306</v>
+      </c>
+      <c r="B259" s="7">
+        <v>44587</v>
+      </c>
+      <c r="C259" s="7">
+        <v>56878</v>
+      </c>
+      <c r="D259" s="3">
+        <f t="shared" si="7"/>
+        <v>12291</v>
+      </c>
+    </row>
+    <row r="260" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A260" s="56" t="s">
+        <v>265</v>
+      </c>
+      <c r="B260" s="7">
+        <v>44670</v>
+      </c>
+      <c r="C260" s="7">
+        <v>56962</v>
+      </c>
+      <c r="D260" s="3">
+        <f t="shared" si="7"/>
+        <v>12292</v>
+      </c>
+    </row>
+    <row r="261" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A261" s="56" t="s">
+        <v>312</v>
+      </c>
+      <c r="B261" s="7">
+        <v>44732</v>
+      </c>
+      <c r="C261" s="7">
+        <v>57026</v>
+      </c>
+      <c r="D261" s="3">
+        <f t="shared" si="7"/>
+        <v>12294</v>
+      </c>
+    </row>
+    <row r="262" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A262" s="56" t="s">
+        <v>279</v>
+      </c>
+      <c r="B262" s="7">
+        <v>44782</v>
+      </c>
+      <c r="C262" s="7">
+        <v>57076</v>
+      </c>
+      <c r="D262" s="3">
+        <f t="shared" si="7"/>
+        <v>12294</v>
+      </c>
+    </row>
+    <row r="263" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A263" s="56" t="s">
+        <v>293</v>
+      </c>
+      <c r="B263" s="7">
+        <v>44820</v>
+      </c>
+      <c r="C263" s="7">
+        <v>57112</v>
+      </c>
+      <c r="D263" s="3">
+        <f t="shared" si="7"/>
+        <v>12292</v>
+      </c>
+    </row>
+    <row r="264" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A264" s="56" t="s">
+        <v>310</v>
+      </c>
+      <c r="B264" s="7">
+        <v>44885</v>
+      </c>
+      <c r="C264" s="7">
+        <v>57179</v>
+      </c>
+      <c r="D264" s="3">
+        <f t="shared" si="7"/>
+        <v>12294</v>
+      </c>
+    </row>
+    <row r="265" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A265" s="56" t="s">
+        <v>250</v>
+      </c>
+      <c r="B265" s="7">
+        <v>45023</v>
+      </c>
+      <c r="C265" s="7">
+        <v>57317</v>
+      </c>
+      <c r="D265" s="3">
+        <f t="shared" si="7"/>
+        <v>12294</v>
+      </c>
+    </row>
+    <row r="266" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A266" s="47" t="s">
+        <v>40</v>
+      </c>
+      <c r="B266" s="7">
+        <v>45060</v>
+      </c>
+      <c r="C266" s="7">
+        <v>57354</v>
+      </c>
+      <c r="D266" s="3">
+        <f t="shared" si="7"/>
+        <v>12294</v>
+      </c>
+    </row>
+    <row r="267" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A267" s="47" t="s">
+        <v>377</v>
+      </c>
+      <c r="B267" s="7">
+        <v>45409</v>
+      </c>
+      <c r="C267" s="7">
+        <v>57998</v>
+      </c>
+      <c r="D267" s="3">
+        <f t="shared" si="7"/>
+        <v>12589</v>
+      </c>
+    </row>
+    <row r="268" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A268" s="47" t="s">
+        <v>41</v>
+      </c>
+      <c r="B268" s="7"/>
+      <c r="C268" s="7">
+        <v>58570</v>
+      </c>
+      <c r="D268" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="258" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B258" s="7"/>
-      <c r="C258" s="7"/>
-      <c r="D258" s="3" t="str">
+    <row r="269" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A269" s="47" t="s">
+        <v>378</v>
+      </c>
+      <c r="B269" s="7"/>
+      <c r="C269" s="7">
+        <v>59229</v>
+      </c>
+      <c r="D269" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="259" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A259" s="55" t="s">
-        <v>39</v>
-      </c>
-      <c r="B259" s="7">
-        <v>44167</v>
-      </c>
-      <c r="C259" s="7">
-        <v>56197</v>
-      </c>
-      <c r="D259" s="3">
-        <f t="shared" si="7"/>
-        <v>12030</v>
-      </c>
-    </row>
-    <row r="260" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A260" s="55" t="s">
-        <v>376</v>
-      </c>
-      <c r="B260" s="7"/>
-      <c r="C260" s="7">
-        <v>45805</v>
-      </c>
-      <c r="D260" s="3" t="str">
+    <row r="270" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A270" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="B270" s="7"/>
+      <c r="C270" s="7">
+        <v>60018</v>
+      </c>
+      <c r="D270" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="261" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A261" s="55" t="s">
-        <v>40</v>
-      </c>
-      <c r="B261" s="7"/>
-      <c r="C261" s="7">
-        <v>54354</v>
-      </c>
-      <c r="D261" s="3" t="str">
-        <f t="shared" si="7"/>
+    <row r="271" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A271" s="47" t="s">
+        <v>379</v>
+      </c>
+      <c r="B271" s="7"/>
+      <c r="C271" s="7">
+        <v>60667</v>
+      </c>
+      <c r="D271" s="3" t="str">
+        <f t="shared" ref="D271:D276" si="8">IF(C271&lt;&gt;"",IF(B271&lt;&gt;"",B271-C271,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="262" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A262" s="55" t="s">
-        <v>377</v>
-      </c>
-      <c r="B262" s="7"/>
-      <c r="C262" s="7">
-        <v>57998</v>
-      </c>
-      <c r="D262" s="3" t="str">
-        <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="263" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A263" s="55" t="s">
-        <v>41</v>
-      </c>
-      <c r="B263" s="7"/>
-      <c r="C263" s="7">
-        <v>58570</v>
-      </c>
-      <c r="D263" s="3" t="str">
-        <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="264" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A264" s="55" t="s">
-        <v>378</v>
-      </c>
-      <c r="B264" s="7"/>
-      <c r="C264" s="7">
-        <v>59229</v>
-      </c>
-      <c r="D264" s="3" t="str">
-        <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="265" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A265" s="55" t="s">
-        <v>42</v>
-      </c>
-      <c r="B265" s="7"/>
-      <c r="C265" s="7">
-        <v>60018</v>
-      </c>
-      <c r="D265" s="3" t="str">
-        <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="266" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A266" s="55" t="s">
-        <v>379</v>
-      </c>
-      <c r="B266" s="7"/>
-      <c r="C266" s="7">
-        <v>60667</v>
-      </c>
-      <c r="D266" s="3" t="str">
-        <f t="shared" ref="D266:D271" si="8">IF(C266&lt;&gt;"",IF(B266&lt;&gt;"",B266-C266,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="267" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A267" s="55" t="s">
+    <row r="272" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A272" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="B267" s="7"/>
-      <c r="C267" s="7">
+      <c r="B272" s="7"/>
+      <c r="C272" s="7">
         <v>61224</v>
       </c>
-      <c r="D267" s="56" t="str">
+      <c r="D272" s="3" t="str">
         <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
-    <row r="268" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A268" s="55" t="s">
+    <row r="273" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A273" s="47" t="s">
         <v>380</v>
       </c>
-      <c r="B268" s="7"/>
-      <c r="C268" s="7">
+      <c r="B273" s="7"/>
+      <c r="C273" s="7">
         <v>61892</v>
       </c>
-      <c r="D268" s="56" t="str">
+      <c r="D273" s="3" t="str">
         <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
-    <row r="269" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A269" s="55" t="s">
+    <row r="274" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A274" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="B269" s="7"/>
-      <c r="C269" s="7">
+      <c r="B274" s="7"/>
+      <c r="C274" s="7">
         <v>62616</v>
       </c>
-      <c r="D269" s="56" t="str">
+      <c r="D274" s="3" t="str">
         <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
-    <row r="270" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A270" s="55" t="s">
+    <row r="275" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A275" s="47" t="s">
         <v>381</v>
       </c>
-      <c r="B270" s="7"/>
-      <c r="C270" s="7">
+      <c r="B275" s="7"/>
+      <c r="C275" s="7">
         <v>63244</v>
       </c>
-      <c r="D270" s="56" t="str">
+      <c r="D275" s="3" t="str">
         <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
-    <row r="271" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A271" s="55" t="s">
+    <row r="276" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A276" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="B271" s="7"/>
-      <c r="C271" s="7">
+      <c r="B276" s="7"/>
+      <c r="C276" s="7">
         <v>63782</v>
       </c>
-      <c r="D271" s="56" t="str">
+      <c r="D276" s="3" t="str">
         <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
-    <row r="272" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B272" s="7"/>
-      <c r="C272" s="7"/>
-    </row>
-    <row r="273" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B273" s="7"/>
-      <c r="C273" s="7"/>
-    </row>
-    <row r="274" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B274" s="7"/>
-      <c r="C274" s="7"/>
-    </row>
-    <row r="275" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B275" s="7"/>
-      <c r="C275" s="7"/>
-    </row>
-    <row r="276" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B276" s="7"/>
-      <c r="C276" s="7"/>
-    </row>
-    <row r="277" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B277" s="7"/>
       <c r="C277" s="7"/>
     </row>
-    <row r="278" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B278" s="7"/>
       <c r="C278" s="7"/>
     </row>
-    <row r="279" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B279" s="7"/>
       <c r="C279" s="7"/>
     </row>
-    <row r="280" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B280" s="7"/>
       <c r="C280" s="7"/>
     </row>
-    <row r="281" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B281" s="7"/>
       <c r="C281" s="7"/>
     </row>
-    <row r="282" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B282" s="7"/>
       <c r="C282" s="7"/>
     </row>
-    <row r="283" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B283" s="7"/>
       <c r="C283" s="7"/>
     </row>
-    <row r="284" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B284" s="7"/>
       <c r="C284" s="7"/>
     </row>
-    <row r="285" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B285" s="7"/>
       <c r="C285" s="7"/>
     </row>
-    <row r="286" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B286" s="7"/>
       <c r="C286" s="7"/>
     </row>
-    <row r="287" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B287" s="7"/>
       <c r="C287" s="7"/>
     </row>
-    <row r="288" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B288" s="7"/>
       <c r="C288" s="7"/>
     </row>
@@ -6448,6 +6529,26 @@
     <row r="360" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B360" s="7"/>
       <c r="C360" s="7"/>
+    </row>
+    <row r="361" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B361" s="7"/>
+      <c r="C361" s="7"/>
+    </row>
+    <row r="362" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B362" s="7"/>
+      <c r="C362" s="7"/>
+    </row>
+    <row r="363" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B363" s="7"/>
+      <c r="C363" s="7"/>
+    </row>
+    <row r="364" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B364" s="7"/>
+      <c r="C364" s="7"/>
+    </row>
+    <row r="365" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B365" s="7"/>
+      <c r="C365" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16441,7 +16542,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="28" type="noConversion"/>
+  <phoneticPr fontId="29" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -16471,10 +16572,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="47" t="s">
+      <c r="K1" s="48" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="48"/>
+      <c r="L1" s="49"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -18326,13 +18427,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="49" t="s">
+      <c r="H53" s="50" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="50"/>
-      <c r="J53" s="50"/>
-      <c r="K53" s="50"/>
-      <c r="L53" s="51"/>
+      <c r="I53" s="51"/>
+      <c r="J53" s="51"/>
+      <c r="K53" s="51"/>
+      <c r="L53" s="52"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -18354,11 +18455,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="52"/>
-      <c r="I54" s="53"/>
-      <c r="J54" s="53"/>
-      <c r="K54" s="53"/>
-      <c r="L54" s="54"/>
+      <c r="H54" s="53"/>
+      <c r="I54" s="54"/>
+      <c r="J54" s="54"/>
+      <c r="K54" s="54"/>
+      <c r="L54" s="55"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - level 46 done
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D622F60-BDFF-4EBC-AC8C-BEFE79544249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4185DECF-161F-437D-8F71-3D390CE250BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50745" yWindow="3210" windowWidth="6720" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="383">
   <si>
     <t>Place</t>
   </si>
@@ -1181,6 +1181,9 @@
   </si>
   <si>
     <t>50 1st move</t>
+  </si>
+  <si>
+    <t>right dig</t>
   </si>
 </sst>
 </file>
@@ -2076,7 +2079,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E365"/>
+  <dimension ref="A1:E372"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -4950,7 +4953,7 @@
         <v>43721</v>
       </c>
       <c r="D192" s="3">
-        <f t="shared" ref="D192:D270" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
+        <f t="shared" ref="D192:D277" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
         <v>9462</v>
       </c>
     </row>
@@ -6078,149 +6081,219 @@
       </c>
     </row>
     <row r="268" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A268" s="47" t="s">
+      <c r="A268" s="56" t="s">
+        <v>306</v>
+      </c>
+      <c r="B268" s="7">
+        <v>45452</v>
+      </c>
+      <c r="C268" s="7">
+        <v>58041</v>
+      </c>
+      <c r="D268" s="3">
+        <f t="shared" si="7"/>
+        <v>12589</v>
+      </c>
+    </row>
+    <row r="269" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A269" s="56" t="s">
+        <v>319</v>
+      </c>
+      <c r="B269" s="7">
+        <v>45494</v>
+      </c>
+      <c r="C269" s="7">
+        <v>58083</v>
+      </c>
+      <c r="D269" s="3">
+        <f t="shared" si="7"/>
+        <v>12589</v>
+      </c>
+    </row>
+    <row r="270" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A270" s="56" t="s">
+        <v>311</v>
+      </c>
+      <c r="B270" s="7">
+        <v>45516</v>
+      </c>
+      <c r="C270" s="7">
+        <v>58104</v>
+      </c>
+      <c r="D270" s="3">
+        <f t="shared" si="7"/>
+        <v>12588</v>
+      </c>
+    </row>
+    <row r="271" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A271" s="56" t="s">
+        <v>150</v>
+      </c>
+      <c r="B271" s="7">
+        <v>45534</v>
+      </c>
+      <c r="C271" s="7">
+        <v>58122</v>
+      </c>
+      <c r="D271" s="3">
+        <f t="shared" si="7"/>
+        <v>12588</v>
+      </c>
+    </row>
+    <row r="272" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A272" s="56" t="s">
+        <v>233</v>
+      </c>
+      <c r="B272" s="7">
+        <v>45618</v>
+      </c>
+      <c r="C272" s="7">
+        <v>58208</v>
+      </c>
+      <c r="D272" s="3">
+        <f t="shared" si="7"/>
+        <v>12590</v>
+      </c>
+    </row>
+    <row r="273" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A273" s="56" t="s">
+        <v>382</v>
+      </c>
+      <c r="B273" s="7">
+        <v>45680</v>
+      </c>
+      <c r="C273" s="7">
+        <v>58263</v>
+      </c>
+      <c r="D273" s="3">
+        <f t="shared" si="7"/>
+        <v>12583</v>
+      </c>
+    </row>
+    <row r="274" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A274" s="47"/>
+      <c r="B274" s="7"/>
+      <c r="C274" s="7"/>
+      <c r="D274" s="3"/>
+    </row>
+    <row r="275" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A275" s="47" t="s">
         <v>41</v>
       </c>
-      <c r="B268" s="7"/>
-      <c r="C268" s="7">
+      <c r="B275" s="7">
+        <v>45990</v>
+      </c>
+      <c r="C275" s="7">
         <v>58570</v>
       </c>
-      <c r="D268" s="3" t="str">
+      <c r="D275" s="3">
+        <f t="shared" si="7"/>
+        <v>12580</v>
+      </c>
+    </row>
+    <row r="276" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A276" s="47" t="s">
+        <v>378</v>
+      </c>
+      <c r="B276" s="7"/>
+      <c r="C276" s="7">
+        <v>59229</v>
+      </c>
+      <c r="D276" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="269" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A269" s="47" t="s">
-        <v>378</v>
-      </c>
-      <c r="B269" s="7"/>
-      <c r="C269" s="7">
-        <v>59229</v>
-      </c>
-      <c r="D269" s="3" t="str">
+    <row r="277" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A277" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="B277" s="7"/>
+      <c r="C277" s="7">
+        <v>60018</v>
+      </c>
+      <c r="D277" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="270" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A270" s="47" t="s">
-        <v>42</v>
-      </c>
-      <c r="B270" s="7"/>
-      <c r="C270" s="7">
-        <v>60018</v>
-      </c>
-      <c r="D270" s="3" t="str">
-        <f t="shared" si="7"/>
+    <row r="278" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A278" s="47" t="s">
+        <v>379</v>
+      </c>
+      <c r="B278" s="7"/>
+      <c r="C278" s="7">
+        <v>60667</v>
+      </c>
+      <c r="D278" s="3" t="str">
+        <f t="shared" ref="D278:D283" si="8">IF(C278&lt;&gt;"",IF(B278&lt;&gt;"",B278-C278,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="271" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A271" s="47" t="s">
-        <v>379</v>
-      </c>
-      <c r="B271" s="7"/>
-      <c r="C271" s="7">
-        <v>60667</v>
-      </c>
-      <c r="D271" s="3" t="str">
-        <f t="shared" ref="D271:D276" si="8">IF(C271&lt;&gt;"",IF(B271&lt;&gt;"",B271-C271,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="272" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A272" s="47" t="s">
+    <row r="279" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A279" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="B272" s="7"/>
-      <c r="C272" s="7">
+      <c r="B279" s="7"/>
+      <c r="C279" s="7">
         <v>61224</v>
       </c>
-      <c r="D272" s="3" t="str">
+      <c r="D279" s="3" t="str">
         <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
-    <row r="273" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A273" s="47" t="s">
+    <row r="280" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A280" s="47" t="s">
         <v>380</v>
       </c>
-      <c r="B273" s="7"/>
-      <c r="C273" s="7">
+      <c r="B280" s="7"/>
+      <c r="C280" s="7">
         <v>61892</v>
       </c>
-      <c r="D273" s="3" t="str">
+      <c r="D280" s="3" t="str">
         <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
-    <row r="274" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A274" s="47" t="s">
+    <row r="281" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A281" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="B274" s="7"/>
-      <c r="C274" s="7">
+      <c r="B281" s="7"/>
+      <c r="C281" s="7">
         <v>62616</v>
       </c>
-      <c r="D274" s="3" t="str">
+      <c r="D281" s="3" t="str">
         <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
-    <row r="275" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A275" s="47" t="s">
+    <row r="282" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A282" s="47" t="s">
         <v>381</v>
       </c>
-      <c r="B275" s="7"/>
-      <c r="C275" s="7">
+      <c r="B282" s="7"/>
+      <c r="C282" s="7">
         <v>63244</v>
       </c>
-      <c r="D275" s="3" t="str">
+      <c r="D282" s="3" t="str">
         <f t="shared" si="8"/>
         <v>-</v>
       </c>
     </row>
-    <row r="276" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A276" s="47" t="s">
+    <row r="283" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A283" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="B276" s="7"/>
-      <c r="C276" s="7">
+      <c r="B283" s="7"/>
+      <c r="C283" s="7">
         <v>63782</v>
       </c>
-      <c r="D276" s="3" t="str">
+      <c r="D283" s="3" t="str">
         <f t="shared" si="8"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="277" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B277" s="7"/>
-      <c r="C277" s="7"/>
-    </row>
-    <row r="278" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B278" s="7"/>
-      <c r="C278" s="7"/>
-    </row>
-    <row r="279" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B279" s="7"/>
-      <c r="C279" s="7"/>
-    </row>
-    <row r="280" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B280" s="7"/>
-      <c r="C280" s="7"/>
-    </row>
-    <row r="281" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B281" s="7"/>
-      <c r="C281" s="7"/>
-    </row>
-    <row r="282" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B282" s="7"/>
-      <c r="C282" s="7"/>
-    </row>
-    <row r="283" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B283" s="7"/>
-      <c r="C283" s="7"/>
     </row>
     <row r="284" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B284" s="7"/>
@@ -6549,6 +6622,34 @@
     <row r="365" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B365" s="7"/>
       <c r="C365" s="7"/>
+    </row>
+    <row r="366" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B366" s="7"/>
+      <c r="C366" s="7"/>
+    </row>
+    <row r="367" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B367" s="7"/>
+      <c r="C367" s="7"/>
+    </row>
+    <row r="368" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B368" s="7"/>
+      <c r="C368" s="7"/>
+    </row>
+    <row r="369" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B369" s="7"/>
+      <c r="C369" s="7"/>
+    </row>
+    <row r="370" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B370" s="7"/>
+      <c r="C370" s="7"/>
+    </row>
+    <row r="371" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B371" s="7"/>
+      <c r="C371" s="7"/>
+    </row>
+    <row r="372" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B372" s="7"/>
+      <c r="C372" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - lv 47 done 12879 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4185DECF-161F-437D-8F71-3D390CE250BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F498CBE3-BCB6-4705-830E-AEA9EDD120E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50745" yWindow="3210" windowWidth="6720" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="385">
   <si>
     <t>Place</t>
   </si>
@@ -1184,6 +1184,12 @@
   </si>
   <si>
     <t>right dig</t>
+  </si>
+  <si>
+    <t>dig at 2 enemies</t>
+  </si>
+  <si>
+    <t>dig above gold = 7</t>
   </si>
 </sst>
 </file>
@@ -1193,12 +1199,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="33" x14ac:knownFonts="1">
+  <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1630,95 +1643,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="31" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1734,28 +1748,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2079,7 +2093,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E372"/>
+  <dimension ref="A1:E383"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -4953,7 +4967,7 @@
         <v>43721</v>
       </c>
       <c r="D192" s="3">
-        <f t="shared" ref="D192:D277" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
+        <f t="shared" ref="D192:D294" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
         <v>9462</v>
       </c>
     </row>
@@ -5946,7 +5960,7 @@
       </c>
     </row>
     <row r="259" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A259" s="56" t="s">
+      <c r="A259" s="48" t="s">
         <v>306</v>
       </c>
       <c r="B259" s="7">
@@ -5961,7 +5975,7 @@
       </c>
     </row>
     <row r="260" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A260" s="56" t="s">
+      <c r="A260" s="48" t="s">
         <v>265</v>
       </c>
       <c r="B260" s="7">
@@ -5976,7 +5990,7 @@
       </c>
     </row>
     <row r="261" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A261" s="56" t="s">
+      <c r="A261" s="48" t="s">
         <v>312</v>
       </c>
       <c r="B261" s="7">
@@ -5991,7 +6005,7 @@
       </c>
     </row>
     <row r="262" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A262" s="56" t="s">
+      <c r="A262" s="48" t="s">
         <v>279</v>
       </c>
       <c r="B262" s="7">
@@ -6006,7 +6020,7 @@
       </c>
     </row>
     <row r="263" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A263" s="56" t="s">
+      <c r="A263" s="48" t="s">
         <v>293</v>
       </c>
       <c r="B263" s="7">
@@ -6021,7 +6035,7 @@
       </c>
     </row>
     <row r="264" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A264" s="56" t="s">
+      <c r="A264" s="48" t="s">
         <v>310</v>
       </c>
       <c r="B264" s="7">
@@ -6036,7 +6050,7 @@
       </c>
     </row>
     <row r="265" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A265" s="56" t="s">
+      <c r="A265" s="48" t="s">
         <v>250</v>
       </c>
       <c r="B265" s="7">
@@ -6081,7 +6095,7 @@
       </c>
     </row>
     <row r="268" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A268" s="56" t="s">
+      <c r="A268" s="48" t="s">
         <v>306</v>
       </c>
       <c r="B268" s="7">
@@ -6096,7 +6110,7 @@
       </c>
     </row>
     <row r="269" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A269" s="56" t="s">
+      <c r="A269" s="48" t="s">
         <v>319</v>
       </c>
       <c r="B269" s="7">
@@ -6111,7 +6125,7 @@
       </c>
     </row>
     <row r="270" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A270" s="56" t="s">
+      <c r="A270" s="48" t="s">
         <v>311</v>
       </c>
       <c r="B270" s="7">
@@ -6126,7 +6140,7 @@
       </c>
     </row>
     <row r="271" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A271" s="56" t="s">
+      <c r="A271" s="48" t="s">
         <v>150</v>
       </c>
       <c r="B271" s="7">
@@ -6141,7 +6155,7 @@
       </c>
     </row>
     <row r="272" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A272" s="56" t="s">
+      <c r="A272" s="48" t="s">
         <v>233</v>
       </c>
       <c r="B272" s="7">
@@ -6156,7 +6170,7 @@
       </c>
     </row>
     <row r="273" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A273" s="56" t="s">
+      <c r="A273" s="48" t="s">
         <v>382</v>
       </c>
       <c r="B273" s="7">
@@ -6171,211 +6185,345 @@
       </c>
     </row>
     <row r="274" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A274" s="47"/>
-      <c r="B274" s="7"/>
-      <c r="C274" s="7"/>
-      <c r="D274" s="3"/>
+      <c r="A274" s="47" t="s">
+        <v>41</v>
+      </c>
+      <c r="B274" s="7">
+        <v>45990</v>
+      </c>
+      <c r="C274" s="7">
+        <v>58570</v>
+      </c>
+      <c r="D274" s="3">
+        <f t="shared" si="7"/>
+        <v>12580</v>
+      </c>
     </row>
     <row r="275" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A275" s="47" t="s">
-        <v>41</v>
+        <v>378</v>
       </c>
       <c r="B275" s="7">
-        <v>45990</v>
+        <v>46652</v>
       </c>
       <c r="C275" s="7">
-        <v>58570</v>
+        <v>59229</v>
       </c>
       <c r="D275" s="3">
         <f t="shared" si="7"/>
-        <v>12580</v>
+        <v>12577</v>
       </c>
     </row>
     <row r="276" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A276" s="47" t="s">
-        <v>378</v>
-      </c>
-      <c r="B276" s="7"/>
+      <c r="A276" s="57" t="s">
+        <v>265</v>
+      </c>
+      <c r="B276" s="7">
+        <v>46671</v>
+      </c>
       <c r="C276" s="7">
-        <v>59229</v>
-      </c>
-      <c r="D276" s="3" t="str">
+        <v>59247</v>
+      </c>
+      <c r="D276" s="3">
+        <f t="shared" si="7"/>
+        <v>12576</v>
+      </c>
+    </row>
+    <row r="277" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A277" s="57" t="s">
+        <v>356</v>
+      </c>
+      <c r="B277" s="7">
+        <v>46702</v>
+      </c>
+      <c r="C277" s="7">
+        <v>59276</v>
+      </c>
+      <c r="D277" s="3">
+        <f t="shared" si="7"/>
+        <v>12574</v>
+      </c>
+    </row>
+    <row r="278" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A278" s="57" t="s">
+        <v>150</v>
+      </c>
+      <c r="B278" s="7">
+        <v>46739</v>
+      </c>
+      <c r="C278" s="7">
+        <v>59316</v>
+      </c>
+      <c r="D278" s="3">
+        <f t="shared" si="7"/>
+        <v>12577</v>
+      </c>
+    </row>
+    <row r="279" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A279" s="57" t="s">
+        <v>150</v>
+      </c>
+      <c r="B279" s="7">
+        <v>46769</v>
+      </c>
+      <c r="C279" s="7">
+        <v>59346</v>
+      </c>
+      <c r="D279" s="3">
+        <f t="shared" si="7"/>
+        <v>12577</v>
+      </c>
+    </row>
+    <row r="280" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A280" s="57" t="s">
+        <v>150</v>
+      </c>
+      <c r="B280" s="7">
+        <v>46840</v>
+      </c>
+      <c r="C280" s="7">
+        <v>59417</v>
+      </c>
+      <c r="D280" s="3">
+        <f t="shared" si="7"/>
+        <v>12577</v>
+      </c>
+    </row>
+    <row r="281" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A281" s="57" t="s">
+        <v>383</v>
+      </c>
+      <c r="B281" s="7">
+        <v>46914</v>
+      </c>
+      <c r="C281" s="7">
+        <v>59491</v>
+      </c>
+      <c r="D281" s="3">
+        <f t="shared" si="7"/>
+        <v>12577</v>
+      </c>
+    </row>
+    <row r="282" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A282" s="57" t="s">
+        <v>265</v>
+      </c>
+      <c r="B282" s="7">
+        <v>46978</v>
+      </c>
+      <c r="C282" s="7">
+        <v>59555</v>
+      </c>
+      <c r="D282" s="3">
+        <f t="shared" si="7"/>
+        <v>12577</v>
+      </c>
+    </row>
+    <row r="283" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A283" s="57"/>
+      <c r="B283" s="7">
+        <v>46989</v>
+      </c>
+      <c r="C283" s="7">
+        <v>59566</v>
+      </c>
+      <c r="D283" s="3">
+        <f t="shared" si="7"/>
+        <v>12577</v>
+      </c>
+    </row>
+    <row r="284" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A284" s="57" t="s">
+        <v>384</v>
+      </c>
+      <c r="B284" s="7">
+        <v>46992</v>
+      </c>
+      <c r="C284" s="7">
+        <v>59568</v>
+      </c>
+      <c r="D284" s="3">
+        <f t="shared" si="7"/>
+        <v>12576</v>
+      </c>
+    </row>
+    <row r="285" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A285" s="57" t="s">
+        <v>279</v>
+      </c>
+      <c r="B285" s="7">
+        <v>47024</v>
+      </c>
+      <c r="C285" s="7">
+        <v>59601</v>
+      </c>
+      <c r="D285" s="3">
+        <f t="shared" si="7"/>
+        <v>12577</v>
+      </c>
+    </row>
+    <row r="286" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A286" s="57" t="s">
+        <v>265</v>
+      </c>
+      <c r="B286" s="7">
+        <v>47045</v>
+      </c>
+      <c r="C286" s="7">
+        <v>59622</v>
+      </c>
+      <c r="D286" s="3">
+        <f t="shared" si="7"/>
+        <v>12577</v>
+      </c>
+    </row>
+    <row r="287" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A287" s="57" t="s">
+        <v>247</v>
+      </c>
+      <c r="B287" s="7">
+        <v>47180</v>
+      </c>
+      <c r="C287" s="7">
+        <v>59757</v>
+      </c>
+      <c r="D287" s="3">
+        <f t="shared" si="7"/>
+        <v>12577</v>
+      </c>
+    </row>
+    <row r="288" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A288" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="B288" s="7">
+        <v>47433</v>
+      </c>
+      <c r="C288" s="7">
+        <v>60018</v>
+      </c>
+      <c r="D288" s="3">
+        <f t="shared" si="7"/>
+        <v>12585</v>
+      </c>
+    </row>
+    <row r="289" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A289" s="47" t="s">
+        <v>379</v>
+      </c>
+      <c r="B289" s="7">
+        <v>47788</v>
+      </c>
+      <c r="C289" s="7">
+        <v>60667</v>
+      </c>
+      <c r="D289" s="3">
+        <f t="shared" si="7"/>
+        <v>12879</v>
+      </c>
+    </row>
+    <row r="290" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A290" s="47" t="s">
+        <v>43</v>
+      </c>
+      <c r="B290" s="7"/>
+      <c r="C290" s="7">
+        <v>61224</v>
+      </c>
+      <c r="D290" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="277" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A277" s="47" t="s">
-        <v>42</v>
-      </c>
-      <c r="B277" s="7"/>
-      <c r="C277" s="7">
-        <v>60018</v>
-      </c>
-      <c r="D277" s="3" t="str">
+    <row r="291" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A291" s="47" t="s">
+        <v>380</v>
+      </c>
+      <c r="B291" s="7"/>
+      <c r="C291" s="7">
+        <v>61892</v>
+      </c>
+      <c r="D291" s="3" t="str">
         <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="278" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A278" s="47" t="s">
-        <v>379</v>
-      </c>
-      <c r="B278" s="7"/>
-      <c r="C278" s="7">
-        <v>60667</v>
-      </c>
-      <c r="D278" s="3" t="str">
-        <f t="shared" ref="D278:D283" si="8">IF(C278&lt;&gt;"",IF(B278&lt;&gt;"",B278-C278,"-"), "-")</f>
+    <row r="292" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A292" s="47" t="s">
+        <v>44</v>
+      </c>
+      <c r="B292" s="7"/>
+      <c r="C292" s="7">
+        <v>62616</v>
+      </c>
+      <c r="D292" s="3" t="str">
+        <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="279" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A279" s="47" t="s">
-        <v>43</v>
-      </c>
-      <c r="B279" s="7"/>
-      <c r="C279" s="7">
-        <v>61224</v>
-      </c>
-      <c r="D279" s="3" t="str">
-        <f t="shared" si="8"/>
+    <row r="293" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A293" s="47" t="s">
+        <v>381</v>
+      </c>
+      <c r="B293" s="7"/>
+      <c r="C293" s="7">
+        <v>63244</v>
+      </c>
+      <c r="D293" s="3" t="str">
+        <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="280" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A280" s="47" t="s">
-        <v>380</v>
-      </c>
-      <c r="B280" s="7"/>
-      <c r="C280" s="7">
-        <v>61892</v>
-      </c>
-      <c r="D280" s="3" t="str">
-        <f t="shared" si="8"/>
+    <row r="294" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A294" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="B294" s="7"/>
+      <c r="C294" s="7">
+        <v>63782</v>
+      </c>
+      <c r="D294" s="3" t="str">
+        <f t="shared" si="7"/>
         <v>-</v>
       </c>
     </row>
-    <row r="281" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A281" s="47" t="s">
-        <v>44</v>
-      </c>
-      <c r="B281" s="7"/>
-      <c r="C281" s="7">
-        <v>62616</v>
-      </c>
-      <c r="D281" s="3" t="str">
-        <f t="shared" si="8"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="282" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A282" s="47" t="s">
-        <v>381</v>
-      </c>
-      <c r="B282" s="7"/>
-      <c r="C282" s="7">
-        <v>63244</v>
-      </c>
-      <c r="D282" s="3" t="str">
-        <f t="shared" si="8"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="283" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A283" s="47" t="s">
-        <v>26</v>
-      </c>
-      <c r="B283" s="7"/>
-      <c r="C283" s="7">
-        <v>63782</v>
-      </c>
-      <c r="D283" s="3" t="str">
-        <f t="shared" si="8"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="284" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B284" s="7"/>
-      <c r="C284" s="7"/>
-    </row>
-    <row r="285" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B285" s="7"/>
-      <c r="C285" s="7"/>
-    </row>
-    <row r="286" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B286" s="7"/>
-      <c r="C286" s="7"/>
-    </row>
-    <row r="287" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B287" s="7"/>
-      <c r="C287" s="7"/>
-    </row>
-    <row r="288" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B288" s="7"/>
-      <c r="C288" s="7"/>
-    </row>
-    <row r="289" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B289" s="7"/>
-      <c r="C289" s="7"/>
-    </row>
-    <row r="290" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B290" s="7"/>
-      <c r="C290" s="7"/>
-    </row>
-    <row r="291" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B291" s="7"/>
-      <c r="C291" s="7"/>
-    </row>
-    <row r="292" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B292" s="7"/>
-      <c r="C292" s="7"/>
-    </row>
-    <row r="293" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B293" s="7"/>
-      <c r="C293" s="7"/>
-    </row>
-    <row r="294" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B294" s="7"/>
-      <c r="C294" s="7"/>
-    </row>
-    <row r="295" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B295" s="7"/>
       <c r="C295" s="7"/>
     </row>
-    <row r="296" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B296" s="7"/>
       <c r="C296" s="7"/>
     </row>
-    <row r="297" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B297" s="7"/>
       <c r="C297" s="7"/>
     </row>
-    <row r="298" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B298" s="7"/>
       <c r="C298" s="7"/>
     </row>
-    <row r="299" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B299" s="7"/>
       <c r="C299" s="7"/>
     </row>
-    <row r="300" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B300" s="7"/>
       <c r="C300" s="7"/>
     </row>
-    <row r="301" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B301" s="7"/>
       <c r="C301" s="7"/>
     </row>
-    <row r="302" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B302" s="7"/>
       <c r="C302" s="7"/>
     </row>
-    <row r="303" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B303" s="7"/>
       <c r="C303" s="7"/>
     </row>
-    <row r="304" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B304" s="7"/>
       <c r="C304" s="7"/>
     </row>
@@ -6650,6 +6798,50 @@
     <row r="372" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B372" s="7"/>
       <c r="C372" s="7"/>
+    </row>
+    <row r="373" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B373" s="7"/>
+      <c r="C373" s="7"/>
+    </row>
+    <row r="374" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B374" s="7"/>
+      <c r="C374" s="7"/>
+    </row>
+    <row r="375" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B375" s="7"/>
+      <c r="C375" s="7"/>
+    </row>
+    <row r="376" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B376" s="7"/>
+      <c r="C376" s="7"/>
+    </row>
+    <row r="377" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B377" s="7"/>
+      <c r="C377" s="7"/>
+    </row>
+    <row r="378" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B378" s="7"/>
+      <c r="C378" s="7"/>
+    </row>
+    <row r="379" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B379" s="7"/>
+      <c r="C379" s="7"/>
+    </row>
+    <row r="380" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B380" s="7"/>
+      <c r="C380" s="7"/>
+    </row>
+    <row r="381" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B381" s="7"/>
+      <c r="C381" s="7"/>
+    </row>
+    <row r="382" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B382" s="7"/>
+      <c r="C382" s="7"/>
+    </row>
+    <row r="383" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B383" s="7"/>
+      <c r="C383" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16643,7 +16835,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="29" type="noConversion"/>
+  <phoneticPr fontId="30" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -16673,10 +16865,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="48" t="s">
+      <c r="K1" s="49" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="49"/>
+      <c r="L1" s="50"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -18528,13 +18720,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="50" t="s">
+      <c r="H53" s="51" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="51"/>
-      <c r="J53" s="51"/>
-      <c r="K53" s="51"/>
-      <c r="L53" s="52"/>
+      <c r="I53" s="52"/>
+      <c r="J53" s="52"/>
+      <c r="K53" s="52"/>
+      <c r="L53" s="53"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -18556,11 +18748,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="53"/>
-      <c r="I54" s="54"/>
-      <c r="J54" s="54"/>
-      <c r="K54" s="54"/>
-      <c r="L54" s="55"/>
+      <c r="H54" s="54"/>
+      <c r="I54" s="55"/>
+      <c r="J54" s="55"/>
+      <c r="K54" s="55"/>
+      <c r="L54" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - lv 48 done - 13203 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F498CBE3-BCB6-4705-830E-AEA9EDD120E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64B32A49-8958-4619-811C-77C3E7F44469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50745" yWindow="3210" windowWidth="6720" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="386">
   <si>
     <t>Place</t>
   </si>
@@ -1190,6 +1190,9 @@
   </si>
   <si>
     <t>dig above gold = 7</t>
+  </si>
+  <si>
+    <t>fall from pole</t>
   </si>
 </sst>
 </file>
@@ -2093,7 +2096,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E383"/>
+  <dimension ref="A1:E385"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -4967,7 +4970,7 @@
         <v>43721</v>
       </c>
       <c r="D192" s="3">
-        <f t="shared" ref="D192:D294" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
+        <f t="shared" ref="D192:D296" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
         <v>9462</v>
       </c>
     </row>
@@ -6423,64 +6426,72 @@
       </c>
     </row>
     <row r="290" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A290" s="47" t="s">
-        <v>43</v>
-      </c>
-      <c r="B290" s="7"/>
+      <c r="A290" s="57" t="s">
+        <v>385</v>
+      </c>
+      <c r="B290" s="7">
+        <v>47875</v>
+      </c>
       <c r="C290" s="7">
-        <v>61224</v>
-      </c>
-      <c r="D290" s="3" t="str">
+        <v>60754</v>
+      </c>
+      <c r="D290" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>12879</v>
       </c>
     </row>
     <row r="291" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A291" s="47" t="s">
-        <v>380</v>
-      </c>
-      <c r="B291" s="7"/>
+      <c r="A291" s="57" t="s">
+        <v>265</v>
+      </c>
+      <c r="B291" s="7">
+        <v>48069</v>
+      </c>
       <c r="C291" s="7">
-        <v>61892</v>
-      </c>
-      <c r="D291" s="3" t="str">
+        <v>60951</v>
+      </c>
+      <c r="D291" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>12882</v>
       </c>
     </row>
     <row r="292" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A292" s="47" t="s">
-        <v>44</v>
-      </c>
-      <c r="B292" s="7"/>
+        <v>43</v>
+      </c>
+      <c r="B292" s="7">
+        <v>48337</v>
+      </c>
       <c r="C292" s="7">
-        <v>62616</v>
-      </c>
-      <c r="D292" s="3" t="str">
+        <v>61224</v>
+      </c>
+      <c r="D292" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>12887</v>
       </c>
     </row>
     <row r="293" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A293" s="47" t="s">
-        <v>381</v>
-      </c>
-      <c r="B293" s="7"/>
+        <v>380</v>
+      </c>
+      <c r="B293" s="7">
+        <v>48689</v>
+      </c>
       <c r="C293" s="7">
-        <v>63244</v>
-      </c>
-      <c r="D293" s="3" t="str">
+        <v>61892</v>
+      </c>
+      <c r="D293" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
+        <v>13203</v>
       </c>
     </row>
     <row r="294" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A294" s="47" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="B294" s="7"/>
       <c r="C294" s="7">
-        <v>63782</v>
+        <v>62616</v>
       </c>
       <c r="D294" s="3" t="str">
         <f t="shared" si="7"/>
@@ -6488,12 +6499,30 @@
       </c>
     </row>
     <row r="295" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A295" s="47" t="s">
+        <v>381</v>
+      </c>
       <c r="B295" s="7"/>
-      <c r="C295" s="7"/>
+      <c r="C295" s="7">
+        <v>63244</v>
+      </c>
+      <c r="D295" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="296" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A296" s="47" t="s">
+        <v>26</v>
+      </c>
       <c r="B296" s="7"/>
-      <c r="C296" s="7"/>
+      <c r="C296" s="7">
+        <v>63782</v>
+      </c>
+      <c r="D296" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="297" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B297" s="7"/>
@@ -6842,6 +6871,14 @@
     <row r="383" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B383" s="7"/>
       <c r="C383" s="7"/>
+    </row>
+    <row r="384" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B384" s="7"/>
+      <c r="C384" s="7"/>
+    </row>
+    <row r="385" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B385" s="7"/>
+      <c r="C385" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner v6 done - 50244 frames
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64B32A49-8958-4619-811C-77C3E7F44469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A358EEE8-2CB3-4C43-B700-1B1E186FCA36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50745" yWindow="3210" windowWidth="6720" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="387">
   <si>
     <t>Place</t>
   </si>
@@ -1193,6 +1193,9 @@
   </si>
   <si>
     <t>fall from pole</t>
+  </si>
+  <si>
+    <t>ladder grab right</t>
   </si>
 </sst>
 </file>
@@ -2096,7 +2099,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
-  <dimension ref="A1:E385"/>
+  <dimension ref="A1:E388"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.125" customWidth="1"/>
@@ -4970,7 +4973,7 @@
         <v>43721</v>
       </c>
       <c r="D192" s="3">
-        <f t="shared" ref="D192:D296" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
+        <f t="shared" ref="D192:D299" si="7">IF(C192&lt;&gt;"",IF(B192&lt;&gt;"",C192-B192,"-"), "-")</f>
         <v>9462</v>
       </c>
     </row>
@@ -6486,55 +6489,94 @@
       </c>
     </row>
     <row r="294" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A294" s="47" t="s">
+      <c r="A294" s="57" t="s">
+        <v>386</v>
+      </c>
+      <c r="B294" s="7">
+        <v>48926</v>
+      </c>
+      <c r="C294" s="7">
+        <v>62177</v>
+      </c>
+      <c r="D294" s="3">
+        <f t="shared" si="7"/>
+        <v>13251</v>
+      </c>
+    </row>
+    <row r="295" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A295" s="57" t="s">
+        <v>150</v>
+      </c>
+      <c r="B295" s="7">
+        <v>49027</v>
+      </c>
+      <c r="C295" s="7">
+        <v>62280</v>
+      </c>
+      <c r="D295" s="3">
+        <f t="shared" si="7"/>
+        <v>13253</v>
+      </c>
+    </row>
+    <row r="296" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A296" s="57" t="s">
+        <v>265</v>
+      </c>
+      <c r="B296" s="7">
+        <v>49118</v>
+      </c>
+      <c r="C296" s="7">
+        <v>62371</v>
+      </c>
+      <c r="D296" s="3">
+        <f t="shared" si="7"/>
+        <v>13253</v>
+      </c>
+    </row>
+    <row r="297" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A297" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="B294" s="7"/>
-      <c r="C294" s="7">
+      <c r="B297" s="7">
+        <v>49331</v>
+      </c>
+      <c r="C297" s="7">
         <v>62616</v>
       </c>
-      <c r="D294" s="3" t="str">
+      <c r="D297" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="295" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A295" s="47" t="s">
+        <v>13285</v>
+      </c>
+    </row>
+    <row r="298" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A298" s="47" t="s">
         <v>381</v>
       </c>
-      <c r="B295" s="7"/>
-      <c r="C295" s="7">
+      <c r="B298" s="7">
+        <v>49685</v>
+      </c>
+      <c r="C298" s="7">
         <v>63244</v>
       </c>
-      <c r="D295" s="3" t="str">
+      <c r="D298" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="296" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A296" s="47" t="s">
+        <v>13559</v>
+      </c>
+    </row>
+    <row r="299" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A299" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="B296" s="7"/>
-      <c r="C296" s="7">
+      <c r="B299" s="7">
+        <v>50244</v>
+      </c>
+      <c r="C299" s="7">
         <v>63782</v>
       </c>
-      <c r="D296" s="3" t="str">
+      <c r="D299" s="3">
         <f t="shared" si="7"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="297" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B297" s="7"/>
-      <c r="C297" s="7"/>
-    </row>
-    <row r="298" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B298" s="7"/>
-      <c r="C298" s="7"/>
-    </row>
-    <row r="299" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B299" s="7"/>
-      <c r="C299" s="7"/>
+        <v>13538</v>
+      </c>
     </row>
     <row r="300" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B300" s="7"/>
@@ -6879,6 +6921,18 @@
     <row r="385" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B385" s="7"/>
       <c r="C385" s="7"/>
+    </row>
+    <row r="386" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B386" s="7"/>
+      <c r="C386" s="7"/>
+    </row>
+    <row r="387" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B387" s="7"/>
+      <c r="C387" s="7"/>
+    </row>
+    <row r="388" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B388" s="7"/>
+      <c r="C388" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - support both tastudio and non-tastudio for botting
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6786887C-D5E4-48CE-81CB-7C78380D4293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF58CA1-2ED6-4D63-8A4C-D9457F0EB77D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="48150" yWindow="3735" windowWidth="9510" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="424">
   <si>
     <t>Place</t>
   </si>
@@ -1305,6 +1305,9 @@
   </si>
   <si>
     <t>(v6 1st move)</t>
+  </si>
+  <si>
+    <t>Emulation difference on startup</t>
   </si>
 </sst>
 </file>
@@ -1871,6 +1874,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1895,7 +1899,6 @@
     <xf numFmtId="0" fontId="34" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2225,7 +2228,7 @@
     <col min="5" max="5" width="17.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2239,21 +2242,26 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A2" s="50" t="s">
         <v>389</v>
       </c>
-      <c r="B2" s="2"/>
+      <c r="B2" s="2">
+        <v>428</v>
+      </c>
       <c r="C2" s="2">
         <v>427</v>
       </c>
-      <c r="D2" s="3" t="str">
+      <c r="D2" s="3">
         <f t="shared" ref="D2:D65" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A3" s="58" t="s">
+        <v>-1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A3" s="50" t="s">
         <v>392</v>
       </c>
       <c r="B3" s="2"/>
@@ -2265,8 +2273,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A4" s="58" t="s">
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A4" s="50" t="s">
         <v>391</v>
       </c>
       <c r="B4" s="2"/>
@@ -2278,8 +2286,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A5" s="58" t="s">
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A5" s="50" t="s">
         <v>390</v>
       </c>
       <c r="B5" s="2"/>
@@ -2291,8 +2299,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A6" s="58" t="s">
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A6" s="50" t="s">
         <v>393</v>
       </c>
       <c r="B6" s="2"/>
@@ -2304,8 +2312,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A7" s="58" t="s">
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A7" s="50" t="s">
         <v>251</v>
       </c>
       <c r="B7" s="2"/>
@@ -2317,8 +2325,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A8" s="58" t="s">
+    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A8" s="50" t="s">
         <v>394</v>
       </c>
       <c r="B8" s="7"/>
@@ -2330,8 +2338,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="58" t="s">
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A9" s="50" t="s">
         <v>253</v>
       </c>
       <c r="B9" s="7"/>
@@ -2343,8 +2351,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A10" s="58" t="s">
+    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A10" s="50" t="s">
         <v>395</v>
       </c>
       <c r="B10" s="7"/>
@@ -2356,8 +2364,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11" s="58" t="s">
+    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A11" s="50" t="s">
         <v>255</v>
       </c>
       <c r="B11" s="7"/>
@@ -2369,8 +2377,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="58" t="s">
+    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A12" s="50" t="s">
         <v>396</v>
       </c>
       <c r="B12" s="7"/>
@@ -2382,8 +2390,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13" s="58" t="s">
+    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A13" s="50" t="s">
         <v>257</v>
       </c>
       <c r="B13" s="7"/>
@@ -2395,8 +2403,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" s="58" t="s">
+    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A14" s="50" t="s">
         <v>397</v>
       </c>
       <c r="B14" s="7"/>
@@ -2408,8 +2416,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="58" t="s">
+    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A15" s="50" t="s">
         <v>259</v>
       </c>
       <c r="B15" s="7"/>
@@ -2421,8 +2429,8 @@
         <v>-</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A16" s="58" t="s">
+    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A16" s="50" t="s">
         <v>410</v>
       </c>
       <c r="B16" s="7"/>
@@ -2435,7 +2443,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A17" s="58" t="s">
+      <c r="A17" s="50" t="s">
         <v>267</v>
       </c>
       <c r="B17" s="7"/>
@@ -2448,7 +2456,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" s="58" t="s">
+      <c r="A18" s="50" t="s">
         <v>398</v>
       </c>
       <c r="B18" s="7"/>
@@ -2461,7 +2469,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A19" s="58" t="s">
+      <c r="A19" s="50" t="s">
         <v>274</v>
       </c>
       <c r="B19" s="7"/>
@@ -2474,7 +2482,7 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A20" s="58" t="s">
+      <c r="A20" s="50" t="s">
         <v>399</v>
       </c>
       <c r="B20" s="7"/>
@@ -2487,7 +2495,7 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A21" s="58" t="s">
+      <c r="A21" s="50" t="s">
         <v>276</v>
       </c>
       <c r="B21" s="7"/>
@@ -2500,7 +2508,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A22" s="58" t="s">
+      <c r="A22" s="50" t="s">
         <v>400</v>
       </c>
       <c r="B22" s="7"/>
@@ -2513,7 +2521,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A23" s="58" t="s">
+      <c r="A23" s="50" t="s">
         <v>278</v>
       </c>
       <c r="B23" s="7"/>
@@ -2526,7 +2534,7 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A24" s="58" t="s">
+      <c r="A24" s="50" t="s">
         <v>401</v>
       </c>
       <c r="B24" s="7"/>
@@ -2539,7 +2547,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A25" s="58" t="s">
+      <c r="A25" s="50" t="s">
         <v>281</v>
       </c>
       <c r="B25" s="7"/>
@@ -2552,7 +2560,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A26" s="58" t="s">
+      <c r="A26" s="50" t="s">
         <v>402</v>
       </c>
       <c r="B26" s="7"/>
@@ -2565,7 +2573,7 @@
       </c>
     </row>
     <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A27" s="58" t="s">
+      <c r="A27" s="50" t="s">
         <v>283</v>
       </c>
       <c r="B27" s="7"/>
@@ -2578,7 +2586,7 @@
       </c>
     </row>
     <row r="28" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A28" s="58" t="s">
+      <c r="A28" s="50" t="s">
         <v>403</v>
       </c>
       <c r="B28" s="7"/>
@@ -2594,7 +2602,7 @@
       </c>
     </row>
     <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="58" t="s">
+      <c r="A29" s="50" t="s">
         <v>285</v>
       </c>
       <c r="B29" s="7"/>
@@ -2607,7 +2615,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="58" t="s">
+      <c r="A30" s="50" t="s">
         <v>404</v>
       </c>
       <c r="B30" s="7"/>
@@ -2620,7 +2628,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="58" t="s">
+      <c r="A31" s="50" t="s">
         <v>288</v>
       </c>
       <c r="B31" s="7"/>
@@ -2633,7 +2641,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="58" t="s">
+      <c r="A32" s="50" t="s">
         <v>405</v>
       </c>
       <c r="B32" s="7"/>
@@ -2646,7 +2654,7 @@
       </c>
     </row>
     <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A33" s="58" t="s">
+      <c r="A33" s="50" t="s">
         <v>294</v>
       </c>
       <c r="B33" s="7"/>
@@ -2659,7 +2667,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A34" s="58" t="s">
+      <c r="A34" s="50" t="s">
         <v>406</v>
       </c>
       <c r="B34" s="7"/>
@@ -2672,7 +2680,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A35" s="58" t="s">
+      <c r="A35" s="50" t="s">
         <v>297</v>
       </c>
       <c r="B35" s="7"/>
@@ -2685,7 +2693,7 @@
       </c>
     </row>
     <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A36" s="58" t="s">
+      <c r="A36" s="50" t="s">
         <v>407</v>
       </c>
       <c r="B36" s="7"/>
@@ -2698,7 +2706,7 @@
       </c>
     </row>
     <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A37" s="58" t="s">
+      <c r="A37" s="50" t="s">
         <v>301</v>
       </c>
       <c r="B37" s="33"/>
@@ -2711,7 +2719,7 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A38" s="58" t="s">
+      <c r="A38" s="50" t="s">
         <v>408</v>
       </c>
       <c r="B38" s="7"/>
@@ -2724,7 +2732,7 @@
       </c>
     </row>
     <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A39" s="58" t="s">
+      <c r="A39" s="50" t="s">
         <v>305</v>
       </c>
       <c r="B39" s="7"/>
@@ -2737,7 +2745,7 @@
       </c>
     </row>
     <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A40" s="58" t="s">
+      <c r="A40" s="50" t="s">
         <v>409</v>
       </c>
       <c r="B40" s="7"/>
@@ -2750,7 +2758,7 @@
       </c>
     </row>
     <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A41" s="58" t="s">
+      <c r="A41" s="50" t="s">
         <v>308</v>
       </c>
       <c r="B41" s="7"/>
@@ -2763,7 +2771,7 @@
       </c>
     </row>
     <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A42" s="58" t="s">
+      <c r="A42" s="50" t="s">
         <v>411</v>
       </c>
       <c r="B42" s="7"/>
@@ -2776,7 +2784,7 @@
       </c>
     </row>
     <row r="43" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A43" s="58" t="s">
+      <c r="A43" s="50" t="s">
         <v>314</v>
       </c>
       <c r="B43" s="7"/>
@@ -2789,7 +2797,7 @@
       </c>
     </row>
     <row r="44" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A44" s="58" t="s">
+      <c r="A44" s="50" t="s">
         <v>412</v>
       </c>
       <c r="B44" s="7"/>
@@ -2802,7 +2810,7 @@
       </c>
     </row>
     <row r="45" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A45" s="58" t="s">
+      <c r="A45" s="50" t="s">
         <v>320</v>
       </c>
       <c r="B45" s="7"/>
@@ -2816,7 +2824,7 @@
       <c r="E45" s="7"/>
     </row>
     <row r="46" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A46" s="58" t="s">
+      <c r="A46" s="50" t="s">
         <v>413</v>
       </c>
       <c r="B46" s="7"/>
@@ -2830,7 +2838,7 @@
       <c r="E46" s="7"/>
     </row>
     <row r="47" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A47" s="58" t="s">
+      <c r="A47" s="50" t="s">
         <v>322</v>
       </c>
       <c r="B47" s="7"/>
@@ -2843,7 +2851,7 @@
       </c>
     </row>
     <row r="48" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A48" s="58" t="s">
+      <c r="A48" s="50" t="s">
         <v>414</v>
       </c>
       <c r="B48" s="7"/>
@@ -2856,7 +2864,7 @@
       </c>
     </row>
     <row r="49" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A49" s="58" t="s">
+      <c r="A49" s="50" t="s">
         <v>324</v>
       </c>
       <c r="B49" s="7"/>
@@ -2869,7 +2877,7 @@
       </c>
     </row>
     <row r="50" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A50" s="58" t="s">
+      <c r="A50" s="50" t="s">
         <v>415</v>
       </c>
       <c r="B50" s="7"/>
@@ -2882,7 +2890,7 @@
       </c>
     </row>
     <row r="51" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A51" s="58" t="s">
+      <c r="A51" s="50" t="s">
         <v>416</v>
       </c>
       <c r="B51" s="7"/>
@@ -2895,11 +2903,11 @@
       </c>
     </row>
     <row r="52" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A52" s="58" t="s">
+      <c r="A52" s="50" t="s">
         <v>417</v>
       </c>
       <c r="B52" s="8"/>
-      <c r="C52" s="58">
+      <c r="C52" s="50">
         <v>24221</v>
       </c>
       <c r="D52" s="3" t="str">
@@ -2908,7 +2916,7 @@
       </c>
     </row>
     <row r="53" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A53" s="58" t="s">
+      <c r="A53" s="50" t="s">
         <v>418</v>
       </c>
       <c r="B53" s="33"/>
@@ -2921,7 +2929,7 @@
       </c>
     </row>
     <row r="54" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A54" s="58" t="s">
+      <c r="A54" s="50" t="s">
         <v>419</v>
       </c>
       <c r="B54" s="7"/>
@@ -2934,7 +2942,7 @@
       </c>
     </row>
     <row r="55" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A55" s="58" t="s">
+      <c r="A55" s="50" t="s">
         <v>420</v>
       </c>
       <c r="B55" s="7"/>
@@ -2947,7 +2955,7 @@
       </c>
     </row>
     <row r="56" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A56" s="58" t="s">
+      <c r="A56" s="50" t="s">
         <v>421</v>
       </c>
       <c r="B56" s="7"/>
@@ -2960,7 +2968,7 @@
       </c>
     </row>
     <row r="57" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A57" s="58" t="s">
+      <c r="A57" s="50" t="s">
         <v>332</v>
       </c>
       <c r="B57" s="7"/>
@@ -2973,7 +2981,7 @@
       </c>
     </row>
     <row r="58" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A58" s="58" t="s">
+      <c r="A58" s="50" t="s">
         <v>5</v>
       </c>
       <c r="B58" s="7"/>
@@ -2986,7 +2994,7 @@
       </c>
     </row>
     <row r="59" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A59" s="58" t="s">
+      <c r="A59" s="50" t="s">
         <v>337</v>
       </c>
       <c r="B59" s="7"/>
@@ -2999,7 +3007,7 @@
       </c>
     </row>
     <row r="60" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A60" s="58" t="s">
+      <c r="A60" s="50" t="s">
         <v>6</v>
       </c>
       <c r="B60" s="7"/>
@@ -3012,7 +3020,7 @@
       </c>
     </row>
     <row r="61" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A61" s="58" t="s">
+      <c r="A61" s="50" t="s">
         <v>45</v>
       </c>
       <c r="B61" s="7"/>
@@ -3025,7 +3033,7 @@
       </c>
     </row>
     <row r="62" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A62" s="58" t="s">
+      <c r="A62" s="50" t="s">
         <v>7</v>
       </c>
       <c r="B62" s="7"/>
@@ -3038,7 +3046,7 @@
       </c>
     </row>
     <row r="63" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A63" s="58" t="s">
+      <c r="A63" s="50" t="s">
         <v>46</v>
       </c>
       <c r="B63" s="7"/>
@@ -3051,7 +3059,7 @@
       </c>
     </row>
     <row r="64" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A64" s="58" t="s">
+      <c r="A64" s="50" t="s">
         <v>8</v>
       </c>
       <c r="B64" s="7"/>
@@ -3067,7 +3075,7 @@
       </c>
     </row>
     <row r="65" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A65" s="58" t="s">
+      <c r="A65" s="50" t="s">
         <v>28</v>
       </c>
       <c r="B65" s="7"/>
@@ -3080,7 +3088,7 @@
       </c>
     </row>
     <row r="66" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A66" s="58" t="s">
+      <c r="A66" s="50" t="s">
         <v>9</v>
       </c>
       <c r="B66" s="7"/>
@@ -3093,7 +3101,7 @@
       </c>
     </row>
     <row r="67" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A67" s="58" t="s">
+      <c r="A67" s="50" t="s">
         <v>29</v>
       </c>
       <c r="B67" s="7"/>
@@ -3106,7 +3114,7 @@
       </c>
     </row>
     <row r="68" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A68" s="58" t="s">
+      <c r="A68" s="50" t="s">
         <v>10</v>
       </c>
       <c r="B68" s="7"/>
@@ -3122,7 +3130,7 @@
       </c>
     </row>
     <row r="69" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A69" s="58" t="s">
+      <c r="A69" s="50" t="s">
         <v>31</v>
       </c>
       <c r="B69" s="7"/>
@@ -3135,7 +3143,7 @@
       </c>
     </row>
     <row r="70" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A70" s="58" t="s">
+      <c r="A70" s="50" t="s">
         <v>11</v>
       </c>
       <c r="B70" s="7"/>
@@ -3148,7 +3156,7 @@
       </c>
     </row>
     <row r="71" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A71" s="58" t="s">
+      <c r="A71" s="50" t="s">
         <v>30</v>
       </c>
       <c r="B71" s="7"/>
@@ -3161,7 +3169,7 @@
       </c>
     </row>
     <row r="72" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A72" s="58" t="s">
+      <c r="A72" s="50" t="s">
         <v>12</v>
       </c>
       <c r="B72" s="7"/>
@@ -3174,7 +3182,7 @@
       </c>
     </row>
     <row r="73" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A73" s="58" t="s">
+      <c r="A73" s="50" t="s">
         <v>32</v>
       </c>
       <c r="B73" s="7"/>
@@ -3187,7 +3195,7 @@
       </c>
     </row>
     <row r="74" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A74" s="58" t="s">
+      <c r="A74" s="50" t="s">
         <v>13</v>
       </c>
       <c r="B74" s="7"/>
@@ -3200,7 +3208,7 @@
       </c>
     </row>
     <row r="75" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A75" s="58" t="s">
+      <c r="A75" s="50" t="s">
         <v>47</v>
       </c>
       <c r="B75" s="7"/>
@@ -3213,7 +3221,7 @@
       </c>
     </row>
     <row r="76" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A76" s="58" t="s">
+      <c r="A76" s="50" t="s">
         <v>48</v>
       </c>
       <c r="B76" s="7"/>
@@ -3226,7 +3234,7 @@
       </c>
     </row>
     <row r="77" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A77" s="58" t="s">
+      <c r="A77" s="50" t="s">
         <v>33</v>
       </c>
       <c r="B77" s="7"/>
@@ -3239,7 +3247,7 @@
       </c>
     </row>
     <row r="78" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A78" s="58" t="s">
+      <c r="A78" s="50" t="s">
         <v>14</v>
       </c>
       <c r="B78" s="7"/>
@@ -3252,7 +3260,7 @@
       </c>
     </row>
     <row r="79" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A79" s="58" t="s">
+      <c r="A79" s="50" t="s">
         <v>34</v>
       </c>
       <c r="B79" s="7"/>
@@ -3265,7 +3273,7 @@
       </c>
     </row>
     <row r="80" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A80" s="58" t="s">
+      <c r="A80" s="50" t="s">
         <v>15</v>
       </c>
       <c r="B80" s="7"/>
@@ -3278,7 +3286,7 @@
       </c>
     </row>
     <row r="81" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A81" s="58" t="s">
+      <c r="A81" s="50" t="s">
         <v>35</v>
       </c>
       <c r="B81" s="7"/>
@@ -3291,7 +3299,7 @@
       </c>
     </row>
     <row r="82" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A82" s="58" t="s">
+      <c r="A82" s="50" t="s">
         <v>16</v>
       </c>
       <c r="B82" s="7"/>
@@ -3304,7 +3312,7 @@
       </c>
     </row>
     <row r="83" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A83" s="58" t="s">
+      <c r="A83" s="50" t="s">
         <v>36</v>
       </c>
       <c r="B83" s="40"/>
@@ -3317,7 +3325,7 @@
       </c>
     </row>
     <row r="84" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A84" s="58" t="s">
+      <c r="A84" s="50" t="s">
         <v>17</v>
       </c>
       <c r="B84" s="7"/>
@@ -3330,7 +3338,7 @@
       </c>
     </row>
     <row r="85" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A85" s="58" t="s">
+      <c r="A85" s="50" t="s">
         <v>37</v>
       </c>
       <c r="B85" s="7"/>
@@ -3343,7 +3351,7 @@
       </c>
     </row>
     <row r="86" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A86" s="58" t="s">
+      <c r="A86" s="50" t="s">
         <v>18</v>
       </c>
       <c r="B86" s="7"/>
@@ -3356,7 +3364,7 @@
       </c>
     </row>
     <row r="87" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A87" s="58" t="s">
+      <c r="A87" s="50" t="s">
         <v>38</v>
       </c>
       <c r="B87" s="7"/>
@@ -3369,7 +3377,7 @@
       </c>
     </row>
     <row r="88" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A88" s="58" t="s">
+      <c r="A88" s="50" t="s">
         <v>19</v>
       </c>
       <c r="B88" s="7"/>
@@ -3382,7 +3390,7 @@
       </c>
     </row>
     <row r="89" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A89" s="58" t="s">
+      <c r="A89" s="50" t="s">
         <v>39</v>
       </c>
       <c r="B89" s="7"/>
@@ -3395,7 +3403,7 @@
       </c>
     </row>
     <row r="90" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A90" s="58" t="s">
+      <c r="A90" s="50" t="s">
         <v>20</v>
       </c>
       <c r="B90" s="7"/>
@@ -3408,7 +3416,7 @@
       </c>
     </row>
     <row r="91" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A91" s="58" t="s">
+      <c r="A91" s="50" t="s">
         <v>40</v>
       </c>
       <c r="B91" s="7"/>
@@ -3421,7 +3429,7 @@
       </c>
     </row>
     <row r="92" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A92" s="58" t="s">
+      <c r="A92" s="50" t="s">
         <v>21</v>
       </c>
       <c r="B92" s="7"/>
@@ -3434,7 +3442,7 @@
       </c>
     </row>
     <row r="93" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A93" s="58" t="s">
+      <c r="A93" s="50" t="s">
         <v>41</v>
       </c>
       <c r="B93" s="7"/>
@@ -3447,7 +3455,7 @@
       </c>
     </row>
     <row r="94" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A94" s="58" t="s">
+      <c r="A94" s="50" t="s">
         <v>22</v>
       </c>
       <c r="B94" s="7"/>
@@ -3463,7 +3471,7 @@
       </c>
     </row>
     <row r="95" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A95" s="58" t="s">
+      <c r="A95" s="50" t="s">
         <v>42</v>
       </c>
       <c r="B95" s="7"/>
@@ -3476,7 +3484,7 @@
       </c>
     </row>
     <row r="96" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A96" s="58" t="s">
+      <c r="A96" s="50" t="s">
         <v>23</v>
       </c>
       <c r="B96" s="9"/>
@@ -3489,7 +3497,7 @@
       </c>
     </row>
     <row r="97" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A97" s="58" t="s">
+      <c r="A97" s="50" t="s">
         <v>43</v>
       </c>
       <c r="B97" s="7"/>
@@ -3502,7 +3510,7 @@
       </c>
     </row>
     <row r="98" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A98" s="58" t="s">
+      <c r="A98" s="50" t="s">
         <v>24</v>
       </c>
       <c r="B98" s="7"/>
@@ -3515,7 +3523,7 @@
       </c>
     </row>
     <row r="99" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A99" s="58" t="s">
+      <c r="A99" s="50" t="s">
         <v>44</v>
       </c>
       <c r="B99" s="7"/>
@@ -3528,7 +3536,7 @@
       </c>
     </row>
     <row r="100" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A100" s="58" t="s">
+      <c r="A100" s="50" t="s">
         <v>25</v>
       </c>
       <c r="B100" s="7"/>
@@ -3541,7 +3549,7 @@
       </c>
     </row>
     <row r="101" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A101" s="58" t="s">
+      <c r="A101" s="50" t="s">
         <v>26</v>
       </c>
       <c r="B101" s="7"/>
@@ -18762,10 +18770,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="50" t="s">
+      <c r="K1" s="51" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="51"/>
+      <c r="L1" s="52"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -20617,13 +20625,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="52" t="s">
+      <c r="H53" s="53" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="53"/>
-      <c r="J53" s="53"/>
-      <c r="K53" s="53"/>
-      <c r="L53" s="54"/>
+      <c r="I53" s="54"/>
+      <c r="J53" s="54"/>
+      <c r="K53" s="54"/>
+      <c r="L53" s="55"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -20645,11 +20653,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="55"/>
-      <c r="I54" s="56"/>
-      <c r="J54" s="56"/>
-      <c r="K54" s="56"/>
-      <c r="L54" s="57"/>
+      <c r="H54" s="56"/>
+      <c r="I54" s="57"/>
+      <c r="J54" s="57"/>
+      <c r="K54" s="57"/>
+      <c r="L54" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
level 1 - 26 frames after, lost 2 on level 2, more routes need to be attempted
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF58CA1-2ED6-4D63-8A4C-D9457F0EB77D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38FB5EBB-42EB-444B-9089-28C94B284978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="48150" yWindow="3735" windowWidth="9510" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="48150" yWindow="3210" windowWidth="9510" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -2264,39 +2264,45 @@
       <c r="A3" s="50" t="s">
         <v>392</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" s="2">
+        <v>759</v>
+      </c>
       <c r="C3" s="2">
         <v>758</v>
       </c>
-      <c r="D3" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D3" s="3">
+        <f t="shared" si="0"/>
+        <v>-1</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="50" t="s">
         <v>391</v>
       </c>
-      <c r="B4" s="2"/>
+      <c r="B4" s="2">
+        <v>1081</v>
+      </c>
       <c r="C4" s="2">
         <v>1107</v>
       </c>
-      <c r="D4" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D4" s="3">
+        <f t="shared" si="0"/>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="50" t="s">
         <v>390</v>
       </c>
-      <c r="B5" s="2"/>
+      <c r="B5" s="2">
+        <v>1578</v>
+      </c>
       <c r="C5" s="2">
         <v>1602</v>
       </c>
-      <c r="D5" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D5" s="3">
+        <f t="shared" si="0"/>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - level 2 done, 27 frames ahead at beginning of lv 3
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38FB5EBB-42EB-444B-9089-28C94B284978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B45DFEA6-E3A2-4F37-9AEC-49694575A139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="48150" yWindow="3210" windowWidth="9510" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="425">
   <si>
     <t>Place</t>
   </si>
@@ -1308,6 +1308,9 @@
   </si>
   <si>
     <t>Emulation difference on startup</t>
+  </si>
+  <si>
+    <t>1081 possible, delay for spawn timer</t>
   </si>
 </sst>
 </file>
@@ -2280,14 +2283,17 @@
         <v>391</v>
       </c>
       <c r="B4" s="2">
-        <v>1081</v>
+        <v>1089</v>
       </c>
       <c r="C4" s="2">
         <v>1107</v>
       </c>
       <c r="D4" s="3">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>18</v>
+      </c>
+      <c r="E4" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -2295,27 +2301,29 @@
         <v>390</v>
       </c>
       <c r="B5" s="2">
-        <v>1578</v>
+        <v>1574</v>
       </c>
       <c r="C5" s="2">
         <v>1602</v>
       </c>
       <c r="D5" s="3">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="50" t="s">
         <v>393</v>
       </c>
-      <c r="B6" s="2"/>
+      <c r="B6" s="2">
+        <v>1923</v>
+      </c>
       <c r="C6" s="2">
         <v>1950</v>
       </c>
-      <c r="D6" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D6" s="3">
+        <f t="shared" si="0"/>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 3 done - 36 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B45DFEA6-E3A2-4F37-9AEC-49694575A139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9157829C-297F-4933-8814-DAF2ADE5C86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="48150" yWindow="3210" windowWidth="9510" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2222,7 +2222,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E184"/>
+  <dimension ref="A1:E187"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2256,7 +2256,7 @@
         <v>427</v>
       </c>
       <c r="D2" s="3">
-        <f t="shared" ref="D2:D65" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <f t="shared" ref="D2:D68" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
         <v>-1</v>
       </c>
       <c r="E2" t="s">
@@ -2327,77 +2327,81 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A7" s="50" t="s">
-        <v>251</v>
-      </c>
-      <c r="B7" s="2"/>
+      <c r="A7" s="50"/>
+      <c r="B7" s="2">
+        <v>2023</v>
+      </c>
       <c r="C7" s="2">
-        <v>2371</v>
-      </c>
-      <c r="D7" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>2052</v>
+      </c>
+      <c r="D7" s="3">
+        <f t="shared" si="0"/>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A8" s="50" t="s">
-        <v>394</v>
-      </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7">
-        <v>2719</v>
-      </c>
-      <c r="D8" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="A8" s="50"/>
+      <c r="B8" s="2">
+        <v>2052</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2080</v>
+      </c>
+      <c r="D8" s="3">
+        <f t="shared" si="0"/>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="50" t="s">
-        <v>253</v>
-      </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7">
-        <v>3195</v>
-      </c>
-      <c r="D9" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="A9" s="50"/>
+      <c r="B9" s="2">
+        <v>2209</v>
+      </c>
+      <c r="C9" s="2">
+        <v>2244</v>
+      </c>
+      <c r="D9" s="3">
+        <f t="shared" si="0"/>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="50" t="s">
-        <v>395</v>
-      </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7">
-        <v>3543</v>
-      </c>
-      <c r="D10" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>251</v>
+      </c>
+      <c r="B10" s="2">
+        <v>2334</v>
+      </c>
+      <c r="C10" s="2">
+        <v>2371</v>
+      </c>
+      <c r="D10" s="3">
+        <f t="shared" si="0"/>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="50" t="s">
-        <v>255</v>
-      </c>
-      <c r="B11" s="7"/>
+        <v>394</v>
+      </c>
+      <c r="B11" s="7">
+        <v>2683</v>
+      </c>
       <c r="C11" s="7">
-        <v>3829</v>
-      </c>
-      <c r="D11" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>2719</v>
+      </c>
+      <c r="D11" s="3">
+        <f t="shared" si="0"/>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="50" t="s">
-        <v>396</v>
+        <v>253</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7">
-        <v>4178</v>
+        <v>3195</v>
       </c>
       <c r="D12" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2406,11 +2410,11 @@
     </row>
     <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="50" t="s">
-        <v>257</v>
+        <v>395</v>
       </c>
       <c r="B13" s="7"/>
-      <c r="C13" s="37">
-        <v>5190</v>
+      <c r="C13" s="7">
+        <v>3543</v>
       </c>
       <c r="D13" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2419,11 +2423,11 @@
     </row>
     <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="50" t="s">
-        <v>397</v>
+        <v>255</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7">
-        <v>5539</v>
+        <v>3829</v>
       </c>
       <c r="D14" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2432,11 +2436,11 @@
     </row>
     <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="50" t="s">
-        <v>259</v>
+        <v>396</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7">
-        <v>6003</v>
+        <v>4178</v>
       </c>
       <c r="D15" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2445,11 +2449,11 @@
     </row>
     <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="50" t="s">
-        <v>410</v>
+        <v>257</v>
       </c>
       <c r="B16" s="7"/>
-      <c r="C16" s="7">
-        <v>6352</v>
+      <c r="C16" s="37">
+        <v>5190</v>
       </c>
       <c r="D16" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2458,11 +2462,11 @@
     </row>
     <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="50" t="s">
-        <v>267</v>
+        <v>397</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7">
-        <v>6759</v>
+        <v>5539</v>
       </c>
       <c r="D17" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2471,11 +2475,11 @@
     </row>
     <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="50" t="s">
-        <v>398</v>
+        <v>259</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7">
-        <v>7106</v>
+        <v>6003</v>
       </c>
       <c r="D18" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2484,11 +2488,11 @@
     </row>
     <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="50" t="s">
-        <v>274</v>
+        <v>410</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7">
-        <v>8196</v>
+        <v>6352</v>
       </c>
       <c r="D19" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2497,11 +2501,11 @@
     </row>
     <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="50" t="s">
-        <v>399</v>
+        <v>267</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7">
-        <v>8549</v>
+        <v>6759</v>
       </c>
       <c r="D20" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2510,11 +2514,11 @@
     </row>
     <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="50" t="s">
-        <v>276</v>
+        <v>398</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7">
-        <v>9118</v>
+        <v>7106</v>
       </c>
       <c r="D21" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2523,11 +2527,11 @@
     </row>
     <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="50" t="s">
-        <v>400</v>
+        <v>274</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7">
-        <v>9467</v>
+        <v>8196</v>
       </c>
       <c r="D22" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2536,11 +2540,11 @@
     </row>
     <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="50" t="s">
-        <v>278</v>
+        <v>399</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7">
-        <v>9778</v>
+        <v>8549</v>
       </c>
       <c r="D23" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2549,11 +2553,11 @@
     </row>
     <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A24" s="50" t="s">
-        <v>401</v>
+        <v>276</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7">
-        <v>10125</v>
+        <v>9118</v>
       </c>
       <c r="D24" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2562,11 +2566,11 @@
     </row>
     <row r="25" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="50" t="s">
-        <v>281</v>
+        <v>400</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7">
-        <v>10816</v>
+        <v>9467</v>
       </c>
       <c r="D25" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2575,11 +2579,11 @@
     </row>
     <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="50" t="s">
-        <v>402</v>
+        <v>278</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7">
-        <v>11163</v>
+        <v>9778</v>
       </c>
       <c r="D26" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2588,11 +2592,11 @@
     </row>
     <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="50" t="s">
-        <v>283</v>
+        <v>401</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7">
-        <v>11729</v>
+        <v>10125</v>
       </c>
       <c r="D27" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2601,105 +2605,105 @@
     </row>
     <row r="28" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="50" t="s">
-        <v>403</v>
+        <v>281</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7">
-        <v>12383</v>
+        <v>10816</v>
       </c>
       <c r="D28" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="E28" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="50" t="s">
-        <v>285</v>
+        <v>402</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7">
-        <v>12891</v>
+        <v>11163</v>
       </c>
       <c r="D29" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="50" t="s">
-        <v>404</v>
+        <v>283</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7">
-        <v>13269</v>
+        <v>11729</v>
       </c>
       <c r="D30" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="50" t="s">
-        <v>288</v>
+        <v>403</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7">
-        <v>13960</v>
+        <v>12383</v>
       </c>
       <c r="D31" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
+      </c>
+      <c r="E31" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="50" t="s">
-        <v>405</v>
+        <v>285</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7">
-        <v>14320</v>
+        <v>12891</v>
       </c>
       <c r="D32" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="50" t="s">
-        <v>294</v>
+        <v>404</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7">
-        <v>14679</v>
+        <v>13269</v>
       </c>
       <c r="D33" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="50" t="s">
-        <v>406</v>
+        <v>288</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7">
-        <v>15029</v>
+        <v>13960</v>
       </c>
       <c r="D34" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="50" t="s">
-        <v>297</v>
+        <v>405</v>
       </c>
       <c r="B35" s="7"/>
       <c r="C35" s="7">
-        <v>15850</v>
+        <v>14320</v>
       </c>
       <c r="D35" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2708,11 +2712,11 @@
     </row>
     <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
-        <v>407</v>
+        <v>294</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7">
-        <v>16200</v>
+        <v>14679</v>
       </c>
       <c r="D36" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2721,11 +2725,11 @@
     </row>
     <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="50" t="s">
-        <v>301</v>
-      </c>
-      <c r="B37" s="33"/>
-      <c r="C37" s="33">
-        <v>17135</v>
+        <v>406</v>
+      </c>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7">
+        <v>15029</v>
       </c>
       <c r="D37" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2734,11 +2738,11 @@
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A38" s="50" t="s">
-        <v>408</v>
+        <v>297</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="7">
-        <v>17485</v>
+        <v>15850</v>
       </c>
       <c r="D38" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2747,11 +2751,11 @@
     </row>
     <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A39" s="50" t="s">
-        <v>305</v>
+        <v>407</v>
       </c>
       <c r="B39" s="7"/>
       <c r="C39" s="7">
-        <v>17791</v>
+        <v>16200</v>
       </c>
       <c r="D39" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2760,11 +2764,11 @@
     </row>
     <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A40" s="50" t="s">
-        <v>409</v>
-      </c>
-      <c r="B40" s="7"/>
-      <c r="C40" s="37">
-        <v>18139</v>
+        <v>301</v>
+      </c>
+      <c r="B40" s="33"/>
+      <c r="C40" s="33">
+        <v>17135</v>
       </c>
       <c r="D40" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2773,11 +2777,11 @@
     </row>
     <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A41" s="50" t="s">
-        <v>308</v>
+        <v>408</v>
       </c>
       <c r="B41" s="7"/>
       <c r="C41" s="7">
-        <v>18719</v>
+        <v>17485</v>
       </c>
       <c r="D41" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2786,11 +2790,11 @@
     </row>
     <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="50" t="s">
-        <v>411</v>
+        <v>305</v>
       </c>
       <c r="B42" s="7"/>
       <c r="C42" s="7">
-        <v>19068</v>
+        <v>17791</v>
       </c>
       <c r="D42" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2799,11 +2803,11 @@
     </row>
     <row r="43" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="50" t="s">
-        <v>314</v>
+        <v>409</v>
       </c>
       <c r="B43" s="7"/>
-      <c r="C43" s="7">
-        <v>19892</v>
+      <c r="C43" s="37">
+        <v>18139</v>
       </c>
       <c r="D43" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2812,11 +2816,11 @@
     </row>
     <row r="44" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="50" t="s">
-        <v>412</v>
+        <v>308</v>
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="7">
-        <v>20240</v>
+        <v>18719</v>
       </c>
       <c r="D44" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2825,39 +2829,37 @@
     </row>
     <row r="45" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A45" s="50" t="s">
-        <v>320</v>
+        <v>411</v>
       </c>
       <c r="B45" s="7"/>
       <c r="C45" s="7">
-        <v>20813</v>
+        <v>19068</v>
       </c>
       <c r="D45" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="E45" s="7"/>
     </row>
     <row r="46" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="50" t="s">
-        <v>413</v>
+        <v>314</v>
       </c>
       <c r="B46" s="7"/>
       <c r="C46" s="7">
-        <v>21161</v>
+        <v>19892</v>
       </c>
       <c r="D46" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="E46" s="7"/>
     </row>
     <row r="47" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="50" t="s">
-        <v>322</v>
+        <v>412</v>
       </c>
       <c r="B47" s="7"/>
       <c r="C47" s="7">
-        <v>22195</v>
+        <v>20240</v>
       </c>
       <c r="D47" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2866,37 +2868,39 @@
     </row>
     <row r="48" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A48" s="50" t="s">
-        <v>414</v>
+        <v>320</v>
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="7">
-        <v>22543</v>
+        <v>20813</v>
       </c>
       <c r="D48" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
+      <c r="E48" s="7"/>
     </row>
     <row r="49" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="50" t="s">
-        <v>324</v>
+        <v>413</v>
       </c>
       <c r="B49" s="7"/>
       <c r="C49" s="7">
-        <v>22963</v>
+        <v>21161</v>
       </c>
       <c r="D49" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
+      <c r="E49" s="7"/>
     </row>
     <row r="50" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="50" t="s">
-        <v>415</v>
+        <v>322</v>
       </c>
       <c r="B50" s="7"/>
       <c r="C50" s="7">
-        <v>23346</v>
+        <v>22195</v>
       </c>
       <c r="D50" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2905,11 +2909,11 @@
     </row>
     <row r="51" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="50" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="7">
-        <v>23873</v>
+        <v>22543</v>
       </c>
       <c r="D51" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2918,11 +2922,11 @@
     </row>
     <row r="52" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A52" s="50" t="s">
-        <v>417</v>
-      </c>
-      <c r="B52" s="8"/>
-      <c r="C52" s="50">
-        <v>24221</v>
+        <v>324</v>
+      </c>
+      <c r="B52" s="7"/>
+      <c r="C52" s="7">
+        <v>22963</v>
       </c>
       <c r="D52" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2931,11 +2935,11 @@
     </row>
     <row r="53" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A53" s="50" t="s">
-        <v>418</v>
-      </c>
-      <c r="B53" s="33"/>
-      <c r="C53" s="33">
-        <v>25101</v>
+        <v>415</v>
+      </c>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7">
+        <v>23346</v>
       </c>
       <c r="D53" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2944,11 +2948,11 @@
     </row>
     <row r="54" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="50" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="7">
-        <v>25450</v>
+        <v>23873</v>
       </c>
       <c r="D54" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2957,11 +2961,11 @@
     </row>
     <row r="55" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="50" t="s">
-        <v>420</v>
-      </c>
-      <c r="B55" s="7"/>
-      <c r="C55" s="7">
-        <v>26350</v>
+        <v>417</v>
+      </c>
+      <c r="B55" s="8"/>
+      <c r="C55" s="50">
+        <v>24221</v>
       </c>
       <c r="D55" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2970,11 +2974,11 @@
     </row>
     <row r="56" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A56" s="50" t="s">
-        <v>421</v>
-      </c>
-      <c r="B56" s="7"/>
-      <c r="C56" s="7">
-        <v>26699</v>
+        <v>418</v>
+      </c>
+      <c r="B56" s="33"/>
+      <c r="C56" s="33">
+        <v>25101</v>
       </c>
       <c r="D56" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2983,11 +2987,11 @@
     </row>
     <row r="57" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A57" s="50" t="s">
-        <v>332</v>
+        <v>419</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7">
-        <v>27490</v>
+        <v>25450</v>
       </c>
       <c r="D57" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2996,11 +3000,11 @@
     </row>
     <row r="58" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
-        <v>5</v>
+        <v>420</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7">
-        <v>27836</v>
+        <v>26350</v>
       </c>
       <c r="D58" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3009,11 +3013,11 @@
     </row>
     <row r="59" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>337</v>
+        <v>421</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7">
-        <v>28899</v>
+        <v>26699</v>
       </c>
       <c r="D59" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3022,11 +3026,11 @@
     </row>
     <row r="60" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>6</v>
+        <v>332</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7">
-        <v>29248</v>
+        <v>27490</v>
       </c>
       <c r="D60" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3035,11 +3039,11 @@
     </row>
     <row r="61" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7">
-        <v>29962</v>
+        <v>27836</v>
       </c>
       <c r="D61" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3048,11 +3052,11 @@
     </row>
     <row r="62" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>7</v>
+        <v>337</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7">
-        <v>30309</v>
+        <v>28899</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3061,11 +3065,11 @@
     </row>
     <row r="63" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>46</v>
+        <v>6</v>
       </c>
       <c r="B63" s="7"/>
       <c r="C63" s="7">
-        <v>30479</v>
+        <v>29248</v>
       </c>
       <c r="D63" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3074,27 +3078,24 @@
     </row>
     <row r="64" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7">
-        <v>31125</v>
+        <v>29962</v>
       </c>
       <c r="D64" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
-      </c>
-      <c r="E64" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="B65" s="7"/>
       <c r="C65" s="7">
-        <v>31643</v>
+        <v>30309</v>
       </c>
       <c r="D65" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3103,66 +3104,66 @@
     </row>
     <row r="66" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="B66" s="7"/>
       <c r="C66" s="7">
-        <v>31991</v>
+        <v>30479</v>
       </c>
       <c r="D66" s="3" t="str">
-        <f t="shared" ref="D66:D101" si="1">IF(C66&lt;&gt;"",IF(B66&lt;&gt;"",C66-B66,"-"), "-")</f>
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>32586</v>
+        <v>31125</v>
       </c>
       <c r="D67" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E67" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7">
-        <v>33254</v>
+        <v>31643</v>
       </c>
       <c r="D68" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="E68" t="s">
-        <v>422</v>
+        <f t="shared" si="0"/>
+        <v>-</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7">
-        <v>33883</v>
+        <v>31991</v>
       </c>
       <c r="D69" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="D69:D104" si="1">IF(C69&lt;&gt;"",IF(B69&lt;&gt;"",C69-B69,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>34244</v>
+        <v>32586</v>
       </c>
       <c r="D70" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3171,24 +3172,27 @@
     </row>
     <row r="71" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>34862</v>
+        <v>33254</v>
       </c>
       <c r="D71" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
+      </c>
+      <c r="E71" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>35218</v>
+        <v>33883</v>
       </c>
       <c r="D72" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3197,11 +3201,11 @@
     </row>
     <row r="73" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>35772</v>
+        <v>34244</v>
       </c>
       <c r="D73" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3210,11 +3214,11 @@
     </row>
     <row r="74" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>36120</v>
+        <v>34862</v>
       </c>
       <c r="D74" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3223,11 +3227,11 @@
     </row>
     <row r="75" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>36893</v>
+        <v>35218</v>
       </c>
       <c r="D75" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3236,11 +3240,11 @@
     </row>
     <row r="76" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>37238</v>
+        <v>35772</v>
       </c>
       <c r="D76" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3249,11 +3253,11 @@
     </row>
     <row r="77" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>38097</v>
+        <v>36120</v>
       </c>
       <c r="D77" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3262,11 +3266,11 @@
     </row>
     <row r="78" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>38443</v>
+        <v>36893</v>
       </c>
       <c r="D78" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3275,11 +3279,11 @@
     </row>
     <row r="79" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>38692</v>
+        <v>37238</v>
       </c>
       <c r="D79" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3288,334 +3292,361 @@
     </row>
     <row r="80" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>39041</v>
+        <v>38097</v>
       </c>
       <c r="D80" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="81" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>40011</v>
+        <v>38443</v>
       </c>
       <c r="D81" s="3" t="str">
-        <f>IF(C80&lt;&gt;"",IF(B80&lt;&gt;"",C80-B80,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>40373</v>
+        <v>38692</v>
       </c>
       <c r="D82" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="83" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B83" s="40"/>
+        <v>15</v>
+      </c>
+      <c r="B83" s="7"/>
       <c r="C83" s="7">
-        <v>41117</v>
+        <v>39041</v>
       </c>
       <c r="D83" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="84" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="B84" s="7"/>
       <c r="C84" s="7">
-        <v>41465</v>
+        <v>40011</v>
       </c>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <f>IF(C83&lt;&gt;"",IF(B83&lt;&gt;"",C83-B83,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>42450</v>
+        <v>40373</v>
       </c>
       <c r="D85" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="86" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>18</v>
-      </c>
-      <c r="B86" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B86" s="40"/>
       <c r="C86" s="7">
-        <v>42799</v>
+        <v>41117</v>
       </c>
       <c r="D86" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="87" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>43144</v>
+        <v>41465</v>
       </c>
       <c r="D87" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="88" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>43491</v>
+        <v>42450</v>
       </c>
       <c r="D88" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="89" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>44165</v>
+        <v>42799</v>
       </c>
       <c r="D89" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="90" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>44512</v>
+        <v>43144</v>
       </c>
       <c r="D90" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="91" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>45061</v>
+        <v>43491</v>
       </c>
       <c r="D91" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="92" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>45443</v>
+        <v>44165</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="93" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>45990</v>
+        <v>44512</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="94" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>46652</v>
+        <v>45061</v>
       </c>
       <c r="D94" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-      <c r="E94" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="95" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>47436</v>
+        <v>45443</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="96" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B96" s="9"/>
-      <c r="C96" s="9">
-        <v>48337</v>
+        <v>41</v>
+      </c>
+      <c r="B96" s="7"/>
+      <c r="C96" s="7">
+        <v>45990</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="97" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>49334</v>
+        <v>46652</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="98" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="E97" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>48681</v>
+        <v>47436</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="99" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>44</v>
-      </c>
-      <c r="B99" s="7"/>
-      <c r="C99" s="7">
-        <v>49334</v>
+        <v>23</v>
+      </c>
+      <c r="B99" s="9"/>
+      <c r="C99" s="9">
+        <v>48337</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="100" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>49683</v>
+        <v>49334</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="101" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
+        <v>48681</v>
+      </c>
+      <c r="D101" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A102" s="50" t="s">
+        <v>44</v>
+      </c>
+      <c r="B102" s="7"/>
+      <c r="C102" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D102" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A103" s="50" t="s">
+        <v>25</v>
+      </c>
+      <c r="B103" s="7"/>
+      <c r="C103" s="7">
+        <v>49683</v>
+      </c>
+      <c r="D103" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A104" s="50" t="s">
+        <v>26</v>
+      </c>
+      <c r="B104" s="7"/>
+      <c r="C104" s="7">
         <v>50244</v>
       </c>
-      <c r="D101" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B102" s="7"/>
-      <c r="C102" s="7"/>
-    </row>
-    <row r="103" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B103" s="7"/>
-      <c r="C103" s="7"/>
-    </row>
-    <row r="104" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B104" s="7"/>
-      <c r="C104" s="7"/>
-    </row>
-    <row r="105" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="D104" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B105" s="7"/>
       <c r="C105" s="7"/>
     </row>
-    <row r="106" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B106" s="7"/>
       <c r="C106" s="7"/>
     </row>
-    <row r="107" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B107" s="7"/>
       <c r="C107" s="7"/>
     </row>
-    <row r="108" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B108" s="7"/>
       <c r="C108" s="7"/>
     </row>
-    <row r="109" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
     </row>
-    <row r="110" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
     </row>
-    <row r="111" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
     </row>
-    <row r="112" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
     </row>
@@ -3906,6 +3937,18 @@
     <row r="184" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
+    </row>
+    <row r="185" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B185" s="7"/>
+      <c r="C185" s="7"/>
+    </row>
+    <row r="186" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B186" s="7"/>
+      <c r="C186" s="7"/>
+    </row>
+    <row r="187" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B187" s="7"/>
+      <c r="C187" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - level 4 done - 64 frames ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9157829C-297F-4933-8814-DAF2ADE5C86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92282E37-2B87-4821-BE9F-3A1DBAA7B561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="48150" yWindow="3210" windowWidth="9510" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2399,26 +2399,30 @@
       <c r="A12" s="50" t="s">
         <v>253</v>
       </c>
-      <c r="B12" s="7"/>
+      <c r="B12" s="7">
+        <v>3132</v>
+      </c>
       <c r="C12" s="7">
         <v>3195</v>
       </c>
-      <c r="D12" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D12" s="3">
+        <f t="shared" si="0"/>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="50" t="s">
         <v>395</v>
       </c>
-      <c r="B13" s="7"/>
+      <c r="B13" s="7">
+        <v>3479</v>
+      </c>
       <c r="C13" s="7">
         <v>3543</v>
       </c>
-      <c r="D13" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D13" s="3">
+        <f t="shared" si="0"/>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - up to level 7, 65 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92282E37-2B87-4821-BE9F-3A1DBAA7B561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B3475A9-C6EC-4A01-A992-DBEE59FD63B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="48150" yWindow="3210" windowWidth="9510" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2222,7 +2222,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E187"/>
+  <dimension ref="A1:E194"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2256,7 +2256,7 @@
         <v>427</v>
       </c>
       <c r="D2" s="3">
-        <f t="shared" ref="D2:D68" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <f t="shared" ref="D2:D75" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
         <v>-1</v>
       </c>
       <c r="E2" t="s">
@@ -2426,288 +2426,293 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" s="50" t="s">
-        <v>255</v>
-      </c>
-      <c r="B14" s="7"/>
+      <c r="A14" s="50"/>
+      <c r="B14" s="7">
+        <v>3548</v>
+      </c>
       <c r="C14" s="7">
-        <v>3829</v>
-      </c>
-      <c r="D14" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>3612</v>
+      </c>
+      <c r="D14" s="3">
+        <f t="shared" si="0"/>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="50" t="s">
-        <v>396</v>
-      </c>
-      <c r="B15" s="7"/>
+      <c r="A15" s="50"/>
+      <c r="B15" s="7">
+        <v>3640</v>
+      </c>
       <c r="C15" s="7">
-        <v>4178</v>
-      </c>
-      <c r="D15" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>3704</v>
+      </c>
+      <c r="D15" s="3">
+        <f t="shared" si="0"/>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="50" t="s">
+        <v>255</v>
+      </c>
+      <c r="B16" s="7">
+        <v>3761</v>
+      </c>
+      <c r="C16" s="7">
+        <v>3829</v>
+      </c>
+      <c r="D16" s="3">
+        <f t="shared" si="0"/>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A17" s="50" t="s">
+        <v>396</v>
+      </c>
+      <c r="B17" s="7">
+        <v>4109</v>
+      </c>
+      <c r="C17" s="7">
+        <v>4178</v>
+      </c>
+      <c r="D17" s="3">
+        <f t="shared" si="0"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A18" s="50"/>
+      <c r="B18" s="7">
+        <v>4509</v>
+      </c>
+      <c r="C18" s="7">
+        <v>4574</v>
+      </c>
+      <c r="D18" s="3">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A19" s="50"/>
+      <c r="B19" s="7">
+        <v>4669</v>
+      </c>
+      <c r="C19" s="7">
+        <v>4731</v>
+      </c>
+      <c r="D19" s="3">
+        <f t="shared" si="0"/>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A20" s="50"/>
+      <c r="B20" s="7">
+        <v>4727</v>
+      </c>
+      <c r="C20" s="7">
+        <v>4791</v>
+      </c>
+      <c r="D20" s="3">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A21" s="50"/>
+      <c r="B21" s="7">
+        <v>4866</v>
+      </c>
+      <c r="C21" s="7">
+        <v>4926</v>
+      </c>
+      <c r="D21" s="3">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A22" s="50"/>
+      <c r="B22" s="7">
+        <v>4953</v>
+      </c>
+      <c r="C22" s="7">
+        <v>5011</v>
+      </c>
+      <c r="D22" s="3">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A23" s="50" t="s">
         <v>257</v>
       </c>
-      <c r="B16" s="7"/>
-      <c r="C16" s="37">
+      <c r="B23" s="7">
+        <v>5125</v>
+      </c>
+      <c r="C23" s="37">
         <v>5190</v>
       </c>
-      <c r="D16" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A17" s="50" t="s">
+      <c r="D23" s="3">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A24" s="50" t="s">
         <v>397</v>
       </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7">
+      <c r="B24" s="7">
+        <v>5474</v>
+      </c>
+      <c r="C24" s="7">
         <v>5539</v>
       </c>
-      <c r="D17" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" s="50" t="s">
+      <c r="D24" s="3">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A25" s="50" t="s">
         <v>259</v>
-      </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7">
-        <v>6003</v>
-      </c>
-      <c r="D18" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A19" s="50" t="s">
-        <v>410</v>
-      </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7">
-        <v>6352</v>
-      </c>
-      <c r="D19" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A20" s="50" t="s">
-        <v>267</v>
-      </c>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7">
-        <v>6759</v>
-      </c>
-      <c r="D20" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A21" s="50" t="s">
-        <v>398</v>
-      </c>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7">
-        <v>7106</v>
-      </c>
-      <c r="D21" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A22" s="50" t="s">
-        <v>274</v>
-      </c>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7">
-        <v>8196</v>
-      </c>
-      <c r="D22" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A23" s="50" t="s">
-        <v>399</v>
-      </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7">
-        <v>8549</v>
-      </c>
-      <c r="D23" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A24" s="50" t="s">
-        <v>276</v>
-      </c>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7">
-        <v>9118</v>
-      </c>
-      <c r="D24" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A25" s="50" t="s">
-        <v>400</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7">
-        <v>9467</v>
+        <v>6003</v>
       </c>
       <c r="D25" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="50" t="s">
-        <v>278</v>
+        <v>410</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7">
-        <v>9778</v>
+        <v>6352</v>
       </c>
       <c r="D26" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="50" t="s">
-        <v>401</v>
+        <v>267</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7">
-        <v>10125</v>
+        <v>6759</v>
       </c>
       <c r="D27" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="50" t="s">
-        <v>281</v>
+        <v>398</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7">
-        <v>10816</v>
+        <v>7106</v>
       </c>
       <c r="D28" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="50" t="s">
-        <v>402</v>
+        <v>274</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7">
-        <v>11163</v>
+        <v>8196</v>
       </c>
       <c r="D29" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="50" t="s">
-        <v>283</v>
+        <v>399</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7">
-        <v>11729</v>
+        <v>8549</v>
       </c>
       <c r="D30" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="50" t="s">
-        <v>403</v>
+        <v>276</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7">
-        <v>12383</v>
+        <v>9118</v>
       </c>
       <c r="D31" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="E31" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="50" t="s">
-        <v>285</v>
+        <v>400</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7">
-        <v>12891</v>
+        <v>9467</v>
       </c>
       <c r="D32" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="50" t="s">
-        <v>404</v>
+        <v>278</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7">
-        <v>13269</v>
+        <v>9778</v>
       </c>
       <c r="D33" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A34" s="50" t="s">
-        <v>288</v>
+        <v>401</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7">
-        <v>13960</v>
+        <v>10125</v>
       </c>
       <c r="D34" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A35" s="50" t="s">
-        <v>405</v>
+        <v>281</v>
       </c>
       <c r="B35" s="7"/>
       <c r="C35" s="7">
-        <v>14320</v>
+        <v>10816</v>
       </c>
       <c r="D35" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2716,11 +2721,11 @@
     </row>
     <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
-        <v>294</v>
+        <v>402</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7">
-        <v>14679</v>
+        <v>11163</v>
       </c>
       <c r="D36" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2729,11 +2734,11 @@
     </row>
     <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="50" t="s">
-        <v>406</v>
+        <v>283</v>
       </c>
       <c r="B37" s="7"/>
       <c r="C37" s="7">
-        <v>15029</v>
+        <v>11729</v>
       </c>
       <c r="D37" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2742,63 +2747,66 @@
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A38" s="50" t="s">
-        <v>297</v>
+        <v>403</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="7">
-        <v>15850</v>
+        <v>12383</v>
       </c>
       <c r="D38" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="E38" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="50" t="s">
-        <v>407</v>
+        <v>285</v>
       </c>
       <c r="B39" s="7"/>
       <c r="C39" s="7">
-        <v>16200</v>
+        <v>12891</v>
       </c>
       <c r="D39" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="50" t="s">
-        <v>301</v>
-      </c>
-      <c r="B40" s="33"/>
-      <c r="C40" s="33">
-        <v>17135</v>
+        <v>404</v>
+      </c>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7">
+        <v>13269</v>
       </c>
       <c r="D40" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="50" t="s">
-        <v>408</v>
+        <v>288</v>
       </c>
       <c r="B41" s="7"/>
       <c r="C41" s="7">
-        <v>17485</v>
+        <v>13960</v>
       </c>
       <c r="D41" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="50" t="s">
-        <v>305</v>
+        <v>405</v>
       </c>
       <c r="B42" s="7"/>
       <c r="C42" s="7">
-        <v>17791</v>
+        <v>14320</v>
       </c>
       <c r="D42" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2807,11 +2815,11 @@
     </row>
     <row r="43" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="50" t="s">
-        <v>409</v>
+        <v>294</v>
       </c>
       <c r="B43" s="7"/>
-      <c r="C43" s="37">
-        <v>18139</v>
+      <c r="C43" s="7">
+        <v>14679</v>
       </c>
       <c r="D43" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2820,11 +2828,11 @@
     </row>
     <row r="44" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="50" t="s">
-        <v>308</v>
+        <v>406</v>
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="7">
-        <v>18719</v>
+        <v>15029</v>
       </c>
       <c r="D44" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2833,11 +2841,11 @@
     </row>
     <row r="45" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A45" s="50" t="s">
-        <v>411</v>
+        <v>297</v>
       </c>
       <c r="B45" s="7"/>
       <c r="C45" s="7">
-        <v>19068</v>
+        <v>15850</v>
       </c>
       <c r="D45" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2846,11 +2854,11 @@
     </row>
     <row r="46" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="50" t="s">
-        <v>314</v>
+        <v>407</v>
       </c>
       <c r="B46" s="7"/>
       <c r="C46" s="7">
-        <v>19892</v>
+        <v>16200</v>
       </c>
       <c r="D46" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2859,11 +2867,11 @@
     </row>
     <row r="47" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="50" t="s">
-        <v>412</v>
-      </c>
-      <c r="B47" s="7"/>
-      <c r="C47" s="7">
-        <v>20240</v>
+        <v>301</v>
+      </c>
+      <c r="B47" s="33"/>
+      <c r="C47" s="33">
+        <v>17135</v>
       </c>
       <c r="D47" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2872,39 +2880,37 @@
     </row>
     <row r="48" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A48" s="50" t="s">
-        <v>320</v>
+        <v>408</v>
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="7">
-        <v>20813</v>
+        <v>17485</v>
       </c>
       <c r="D48" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="E48" s="7"/>
     </row>
     <row r="49" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="50" t="s">
-        <v>413</v>
+        <v>305</v>
       </c>
       <c r="B49" s="7"/>
       <c r="C49" s="7">
-        <v>21161</v>
+        <v>17791</v>
       </c>
       <c r="D49" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="E49" s="7"/>
     </row>
     <row r="50" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="50" t="s">
-        <v>322</v>
+        <v>409</v>
       </c>
       <c r="B50" s="7"/>
-      <c r="C50" s="7">
-        <v>22195</v>
+      <c r="C50" s="37">
+        <v>18139</v>
       </c>
       <c r="D50" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2913,11 +2919,11 @@
     </row>
     <row r="51" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="50" t="s">
-        <v>414</v>
+        <v>308</v>
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="7">
-        <v>22543</v>
+        <v>18719</v>
       </c>
       <c r="D51" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2926,11 +2932,11 @@
     </row>
     <row r="52" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A52" s="50" t="s">
-        <v>324</v>
+        <v>411</v>
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="7">
-        <v>22963</v>
+        <v>19068</v>
       </c>
       <c r="D52" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2939,11 +2945,11 @@
     </row>
     <row r="53" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A53" s="50" t="s">
-        <v>415</v>
+        <v>314</v>
       </c>
       <c r="B53" s="7"/>
       <c r="C53" s="7">
-        <v>23346</v>
+        <v>19892</v>
       </c>
       <c r="D53" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2952,11 +2958,11 @@
     </row>
     <row r="54" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="50" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="7">
-        <v>23873</v>
+        <v>20240</v>
       </c>
       <c r="D54" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2965,37 +2971,39 @@
     </row>
     <row r="55" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="50" t="s">
-        <v>417</v>
-      </c>
-      <c r="B55" s="8"/>
-      <c r="C55" s="50">
-        <v>24221</v>
+        <v>320</v>
+      </c>
+      <c r="B55" s="7"/>
+      <c r="C55" s="7">
+        <v>20813</v>
       </c>
       <c r="D55" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
+      <c r="E55" s="7"/>
     </row>
     <row r="56" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A56" s="50" t="s">
-        <v>418</v>
-      </c>
-      <c r="B56" s="33"/>
-      <c r="C56" s="33">
-        <v>25101</v>
+        <v>413</v>
+      </c>
+      <c r="B56" s="7"/>
+      <c r="C56" s="7">
+        <v>21161</v>
       </c>
       <c r="D56" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
+      <c r="E56" s="7"/>
     </row>
     <row r="57" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A57" s="50" t="s">
-        <v>419</v>
+        <v>322</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7">
-        <v>25450</v>
+        <v>22195</v>
       </c>
       <c r="D57" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3004,11 +3012,11 @@
     </row>
     <row r="58" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7">
-        <v>26350</v>
+        <v>22543</v>
       </c>
       <c r="D58" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3017,11 +3025,11 @@
     </row>
     <row r="59" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>421</v>
+        <v>324</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7">
-        <v>26699</v>
+        <v>22963</v>
       </c>
       <c r="D59" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3030,11 +3038,11 @@
     </row>
     <row r="60" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>332</v>
+        <v>415</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7">
-        <v>27490</v>
+        <v>23346</v>
       </c>
       <c r="D60" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3043,11 +3051,11 @@
     </row>
     <row r="61" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>5</v>
+        <v>416</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7">
-        <v>27836</v>
+        <v>23873</v>
       </c>
       <c r="D61" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3056,11 +3064,11 @@
     </row>
     <row r="62" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>337</v>
-      </c>
-      <c r="B62" s="7"/>
-      <c r="C62" s="7">
-        <v>28899</v>
+        <v>417</v>
+      </c>
+      <c r="B62" s="8"/>
+      <c r="C62" s="50">
+        <v>24221</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3069,11 +3077,11 @@
     </row>
     <row r="63" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>6</v>
-      </c>
-      <c r="B63" s="7"/>
-      <c r="C63" s="7">
-        <v>29248</v>
+        <v>418</v>
+      </c>
+      <c r="B63" s="33"/>
+      <c r="C63" s="33">
+        <v>25101</v>
       </c>
       <c r="D63" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3082,11 +3090,11 @@
     </row>
     <row r="64" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>45</v>
+        <v>419</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7">
-        <v>29962</v>
+        <v>25450</v>
       </c>
       <c r="D64" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3095,11 +3103,11 @@
     </row>
     <row r="65" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>7</v>
+        <v>420</v>
       </c>
       <c r="B65" s="7"/>
       <c r="C65" s="7">
-        <v>30309</v>
+        <v>26350</v>
       </c>
       <c r="D65" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3108,11 +3116,11 @@
     </row>
     <row r="66" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>46</v>
+        <v>421</v>
       </c>
       <c r="B66" s="7"/>
       <c r="C66" s="7">
-        <v>30479</v>
+        <v>26699</v>
       </c>
       <c r="D66" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3121,27 +3129,24 @@
     </row>
     <row r="67" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>8</v>
+        <v>332</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>31125</v>
+        <v>27490</v>
       </c>
       <c r="D67" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
-      </c>
-      <c r="E67" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7">
-        <v>31643</v>
+        <v>27836</v>
       </c>
       <c r="D68" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3150,118 +3155,118 @@
     </row>
     <row r="69" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>9</v>
+        <v>337</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7">
-        <v>31991</v>
+        <v>28899</v>
       </c>
       <c r="D69" s="3" t="str">
-        <f t="shared" ref="D69:D104" si="1">IF(C69&lt;&gt;"",IF(B69&lt;&gt;"",C69-B69,"-"), "-")</f>
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>32586</v>
+        <v>29248</v>
       </c>
       <c r="D70" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>33254</v>
+        <v>29962</v>
       </c>
       <c r="D71" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="E71" t="s">
-        <v>422</v>
+        <f t="shared" si="0"/>
+        <v>-</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>33883</v>
+        <v>30309</v>
       </c>
       <c r="D72" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>34244</v>
+        <v>30479</v>
       </c>
       <c r="D73" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>34862</v>
+        <v>31125</v>
       </c>
       <c r="D74" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E74" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>35218</v>
+        <v>31643</v>
       </c>
       <c r="D75" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>35772</v>
+        <v>31991</v>
       </c>
       <c r="D76" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="D76:D111" si="1">IF(C76&lt;&gt;"",IF(B76&lt;&gt;"",C76-B76,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>36120</v>
+        <v>32586</v>
       </c>
       <c r="D77" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3270,24 +3275,27 @@
     </row>
     <row r="78" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>36893</v>
+        <v>33254</v>
       </c>
       <c r="D78" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
+      </c>
+      <c r="E78" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>37238</v>
+        <v>33883</v>
       </c>
       <c r="D79" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3296,11 +3304,11 @@
     </row>
     <row r="80" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>38097</v>
+        <v>34244</v>
       </c>
       <c r="D80" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3309,11 +3317,11 @@
     </row>
     <row r="81" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>38443</v>
+        <v>34862</v>
       </c>
       <c r="D81" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3322,11 +3330,11 @@
     </row>
     <row r="82" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>38692</v>
+        <v>35218</v>
       </c>
       <c r="D82" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3335,11 +3343,11 @@
     </row>
     <row r="83" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="B83" s="7"/>
       <c r="C83" s="7">
-        <v>39041</v>
+        <v>35772</v>
       </c>
       <c r="D83" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3348,24 +3356,24 @@
     </row>
     <row r="84" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="B84" s="7"/>
       <c r="C84" s="7">
-        <v>40011</v>
+        <v>36120</v>
       </c>
       <c r="D84" s="3" t="str">
-        <f>IF(C83&lt;&gt;"",IF(B83&lt;&gt;"",C83-B83,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>40373</v>
+        <v>36893</v>
       </c>
       <c r="D85" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3374,11 +3382,11 @@
     </row>
     <row r="86" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B86" s="40"/>
+        <v>48</v>
+      </c>
+      <c r="B86" s="7"/>
       <c r="C86" s="7">
-        <v>41117</v>
+        <v>37238</v>
       </c>
       <c r="D86" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3387,11 +3395,11 @@
     </row>
     <row r="87" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>41465</v>
+        <v>38097</v>
       </c>
       <c r="D87" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3400,11 +3408,11 @@
     </row>
     <row r="88" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>42450</v>
+        <v>38443</v>
       </c>
       <c r="D88" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3413,11 +3421,11 @@
     </row>
     <row r="89" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>42799</v>
+        <v>38692</v>
       </c>
       <c r="D89" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3426,11 +3434,11 @@
     </row>
     <row r="90" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>43144</v>
+        <v>39041</v>
       </c>
       <c r="D90" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3439,24 +3447,24 @@
     </row>
     <row r="91" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>43491</v>
+        <v>40011</v>
       </c>
       <c r="D91" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C90&lt;&gt;"",IF(B90&lt;&gt;"",C90-B90,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>44165</v>
+        <v>40373</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3465,11 +3473,11 @@
     </row>
     <row r="93" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>20</v>
-      </c>
-      <c r="B93" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B93" s="40"/>
       <c r="C93" s="7">
-        <v>44512</v>
+        <v>41117</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3478,11 +3486,11 @@
     </row>
     <row r="94" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>45061</v>
+        <v>41465</v>
       </c>
       <c r="D94" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3491,11 +3499,11 @@
     </row>
     <row r="95" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>45443</v>
+        <v>42450</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3504,11 +3512,11 @@
     </row>
     <row r="96" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="B96" s="7"/>
       <c r="C96" s="7">
-        <v>45990</v>
+        <v>42799</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3517,27 +3525,24 @@
     </row>
     <row r="97" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>46652</v>
+        <v>43144</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
-      </c>
-      <c r="E97" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="98" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>47436</v>
+        <v>43491</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3546,11 +3551,11 @@
     </row>
     <row r="99" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B99" s="9"/>
-      <c r="C99" s="9">
-        <v>48337</v>
+        <v>39</v>
+      </c>
+      <c r="B99" s="7"/>
+      <c r="C99" s="7">
+        <v>44165</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3559,11 +3564,11 @@
     </row>
     <row r="100" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>49334</v>
+        <v>44512</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3572,11 +3577,11 @@
     </row>
     <row r="101" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>48681</v>
+        <v>45061</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3585,11 +3590,11 @@
     </row>
     <row r="102" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A102" s="50" t="s">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="B102" s="7"/>
       <c r="C102" s="7">
-        <v>49334</v>
+        <v>45443</v>
       </c>
       <c r="D102" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3598,11 +3603,11 @@
     </row>
     <row r="103" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A103" s="50" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="B103" s="7"/>
       <c r="C103" s="7">
-        <v>49683</v>
+        <v>45990</v>
       </c>
       <c r="D103" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3611,44 +3616,110 @@
     </row>
     <row r="104" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A104" s="50" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B104" s="7"/>
       <c r="C104" s="7">
+        <v>46652</v>
+      </c>
+      <c r="D104" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+      <c r="E104" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A105" s="50" t="s">
+        <v>42</v>
+      </c>
+      <c r="B105" s="7"/>
+      <c r="C105" s="7">
+        <v>47436</v>
+      </c>
+      <c r="D105" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A106" s="50" t="s">
+        <v>23</v>
+      </c>
+      <c r="B106" s="9"/>
+      <c r="C106" s="9">
+        <v>48337</v>
+      </c>
+      <c r="D106" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A107" s="50" t="s">
+        <v>43</v>
+      </c>
+      <c r="B107" s="7"/>
+      <c r="C107" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D107" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A108" s="50" t="s">
+        <v>24</v>
+      </c>
+      <c r="B108" s="7"/>
+      <c r="C108" s="7">
+        <v>48681</v>
+      </c>
+      <c r="D108" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A109" s="50" t="s">
+        <v>44</v>
+      </c>
+      <c r="B109" s="7"/>
+      <c r="C109" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D109" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A110" s="50" t="s">
+        <v>25</v>
+      </c>
+      <c r="B110" s="7"/>
+      <c r="C110" s="7">
+        <v>49683</v>
+      </c>
+      <c r="D110" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A111" s="50" t="s">
+        <v>26</v>
+      </c>
+      <c r="B111" s="7"/>
+      <c r="C111" s="7">
         <v>50244</v>
       </c>
-      <c r="D104" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B105" s="7"/>
-      <c r="C105" s="7"/>
-    </row>
-    <row r="106" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B106" s="7"/>
-      <c r="C106" s="7"/>
-    </row>
-    <row r="107" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B107" s="7"/>
-      <c r="C107" s="7"/>
-    </row>
-    <row r="108" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B108" s="7"/>
-      <c r="C108" s="7"/>
-    </row>
-    <row r="109" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B109" s="7"/>
-      <c r="C109" s="7"/>
-    </row>
-    <row r="110" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B110" s="7"/>
-      <c r="C110" s="7"/>
-    </row>
-    <row r="111" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B111" s="7"/>
-      <c r="C111" s="7"/>
+      <c r="D111" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="112" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
@@ -3953,6 +4024,34 @@
     <row r="187" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B187" s="7"/>
       <c r="C187" s="7"/>
+    </row>
+    <row r="188" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B188" s="7"/>
+      <c r="C188" s="7"/>
+    </row>
+    <row r="189" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B189" s="7"/>
+      <c r="C189" s="7"/>
+    </row>
+    <row r="190" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B190" s="7"/>
+      <c r="C190" s="7"/>
+    </row>
+    <row r="191" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B191" s="7"/>
+      <c r="C191" s="7"/>
+    </row>
+    <row r="192" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B192" s="7"/>
+      <c r="C192" s="7"/>
+    </row>
+    <row r="193" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B193" s="7"/>
+      <c r="C193" s="7"/>
+    </row>
+    <row r="194" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B194" s="7"/>
+      <c r="C194" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - lv 7 done, still 65 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B3475A9-C6EC-4A01-A992-DBEE59FD63B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D49A7F-E1A5-4A4F-9220-55FB6A389D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="48150" yWindow="3210" windowWidth="9510" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -2580,26 +2580,30 @@
       <c r="A25" s="50" t="s">
         <v>259</v>
       </c>
-      <c r="B25" s="7"/>
+      <c r="B25" s="7">
+        <v>5936</v>
+      </c>
       <c r="C25" s="7">
         <v>6003</v>
       </c>
-      <c r="D25" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D25" s="3">
+        <f t="shared" si="0"/>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="50" t="s">
         <v>410</v>
       </c>
-      <c r="B26" s="7"/>
+      <c r="B26" s="7">
+        <v>6287</v>
+      </c>
       <c r="C26" s="7">
         <v>6352</v>
       </c>
-      <c r="D26" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D26" s="3">
+        <f t="shared" si="0"/>
+        <v>65</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - level 8 done, 67 frames ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D49A7F-E1A5-4A4F-9220-55FB6A389D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAFC8A1A-9FEF-4418-B586-8A45C2653B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2222,7 +2222,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E194"/>
+  <dimension ref="A1:E197"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2256,7 +2256,7 @@
         <v>427</v>
       </c>
       <c r="D2" s="3">
-        <f t="shared" ref="D2:D75" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <f t="shared" ref="D2:D78" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
         <v>-1</v>
       </c>
       <c r="E2" t="s">
@@ -2607,77 +2607,81 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A27" s="50" t="s">
-        <v>267</v>
-      </c>
-      <c r="B27" s="7"/>
+      <c r="A27" s="50"/>
+      <c r="B27" s="7">
+        <v>6410</v>
+      </c>
       <c r="C27" s="7">
-        <v>6759</v>
-      </c>
-      <c r="D27" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>6476</v>
+      </c>
+      <c r="D27" s="3">
+        <f t="shared" si="0"/>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A28" s="50" t="s">
-        <v>398</v>
-      </c>
-      <c r="B28" s="7"/>
+      <c r="A28" s="50"/>
+      <c r="B28" s="7">
+        <v>6446</v>
+      </c>
       <c r="C28" s="7">
-        <v>7106</v>
-      </c>
-      <c r="D28" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>6512</v>
+      </c>
+      <c r="D28" s="3">
+        <f t="shared" si="0"/>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A29" s="50" t="s">
-        <v>274</v>
-      </c>
-      <c r="B29" s="7"/>
+      <c r="A29" s="50"/>
+      <c r="B29" s="7">
+        <v>6590</v>
+      </c>
       <c r="C29" s="7">
-        <v>8196</v>
-      </c>
-      <c r="D29" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>6657</v>
+      </c>
+      <c r="D29" s="3">
+        <f t="shared" si="0"/>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="50" t="s">
-        <v>399</v>
-      </c>
-      <c r="B30" s="7"/>
+        <v>267</v>
+      </c>
+      <c r="B30" s="7">
+        <v>6690</v>
+      </c>
       <c r="C30" s="7">
-        <v>8549</v>
-      </c>
-      <c r="D30" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>6759</v>
+      </c>
+      <c r="D30" s="3">
+        <f t="shared" si="0"/>
+        <v>69</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="50" t="s">
-        <v>276</v>
-      </c>
-      <c r="B31" s="7"/>
+        <v>398</v>
+      </c>
+      <c r="B31" s="7">
+        <v>7039</v>
+      </c>
       <c r="C31" s="7">
-        <v>9118</v>
-      </c>
-      <c r="D31" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>7106</v>
+      </c>
+      <c r="D31" s="3">
+        <f t="shared" si="0"/>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="50" t="s">
-        <v>400</v>
+        <v>274</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7">
-        <v>9467</v>
+        <v>8196</v>
       </c>
       <c r="D32" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2686,11 +2690,11 @@
     </row>
     <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="50" t="s">
-        <v>278</v>
+        <v>399</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7">
-        <v>9778</v>
+        <v>8549</v>
       </c>
       <c r="D33" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2699,11 +2703,11 @@
     </row>
     <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A34" s="50" t="s">
-        <v>401</v>
+        <v>276</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7">
-        <v>10125</v>
+        <v>9118</v>
       </c>
       <c r="D34" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2712,11 +2716,11 @@
     </row>
     <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A35" s="50" t="s">
-        <v>281</v>
+        <v>400</v>
       </c>
       <c r="B35" s="7"/>
       <c r="C35" s="7">
-        <v>10816</v>
+        <v>9467</v>
       </c>
       <c r="D35" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2725,11 +2729,11 @@
     </row>
     <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
-        <v>402</v>
+        <v>278</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7">
-        <v>11163</v>
+        <v>9778</v>
       </c>
       <c r="D36" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2738,11 +2742,11 @@
     </row>
     <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="50" t="s">
-        <v>283</v>
+        <v>401</v>
       </c>
       <c r="B37" s="7"/>
       <c r="C37" s="7">
-        <v>11729</v>
+        <v>10125</v>
       </c>
       <c r="D37" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2751,105 +2755,105 @@
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A38" s="50" t="s">
-        <v>403</v>
+        <v>281</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="7">
-        <v>12383</v>
+        <v>10816</v>
       </c>
       <c r="D38" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="E38" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A39" s="50" t="s">
-        <v>285</v>
+        <v>402</v>
       </c>
       <c r="B39" s="7"/>
       <c r="C39" s="7">
-        <v>12891</v>
+        <v>11163</v>
       </c>
       <c r="D39" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A40" s="50" t="s">
-        <v>404</v>
+        <v>283</v>
       </c>
       <c r="B40" s="7"/>
       <c r="C40" s="7">
-        <v>13269</v>
+        <v>11729</v>
       </c>
       <c r="D40" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A41" s="50" t="s">
-        <v>288</v>
+        <v>403</v>
       </c>
       <c r="B41" s="7"/>
       <c r="C41" s="7">
-        <v>13960</v>
+        <v>12383</v>
       </c>
       <c r="D41" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
+      </c>
+      <c r="E41" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="50" t="s">
-        <v>405</v>
+        <v>285</v>
       </c>
       <c r="B42" s="7"/>
       <c r="C42" s="7">
-        <v>14320</v>
+        <v>12891</v>
       </c>
       <c r="D42" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="50" t="s">
-        <v>294</v>
+        <v>404</v>
       </c>
       <c r="B43" s="7"/>
       <c r="C43" s="7">
-        <v>14679</v>
+        <v>13269</v>
       </c>
       <c r="D43" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="50" t="s">
-        <v>406</v>
+        <v>288</v>
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="7">
-        <v>15029</v>
+        <v>13960</v>
       </c>
       <c r="D44" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="50" t="s">
-        <v>297</v>
+        <v>405</v>
       </c>
       <c r="B45" s="7"/>
       <c r="C45" s="7">
-        <v>15850</v>
+        <v>14320</v>
       </c>
       <c r="D45" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2858,11 +2862,11 @@
     </row>
     <row r="46" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="50" t="s">
-        <v>407</v>
+        <v>294</v>
       </c>
       <c r="B46" s="7"/>
       <c r="C46" s="7">
-        <v>16200</v>
+        <v>14679</v>
       </c>
       <c r="D46" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2871,11 +2875,11 @@
     </row>
     <row r="47" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="50" t="s">
-        <v>301</v>
-      </c>
-      <c r="B47" s="33"/>
-      <c r="C47" s="33">
-        <v>17135</v>
+        <v>406</v>
+      </c>
+      <c r="B47" s="7"/>
+      <c r="C47" s="7">
+        <v>15029</v>
       </c>
       <c r="D47" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2884,11 +2888,11 @@
     </row>
     <row r="48" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A48" s="50" t="s">
-        <v>408</v>
+        <v>297</v>
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="7">
-        <v>17485</v>
+        <v>15850</v>
       </c>
       <c r="D48" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2897,11 +2901,11 @@
     </row>
     <row r="49" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="50" t="s">
-        <v>305</v>
+        <v>407</v>
       </c>
       <c r="B49" s="7"/>
       <c r="C49" s="7">
-        <v>17791</v>
+        <v>16200</v>
       </c>
       <c r="D49" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2910,11 +2914,11 @@
     </row>
     <row r="50" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="50" t="s">
-        <v>409</v>
-      </c>
-      <c r="B50" s="7"/>
-      <c r="C50" s="37">
-        <v>18139</v>
+        <v>301</v>
+      </c>
+      <c r="B50" s="33"/>
+      <c r="C50" s="33">
+        <v>17135</v>
       </c>
       <c r="D50" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2923,11 +2927,11 @@
     </row>
     <row r="51" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="50" t="s">
-        <v>308</v>
+        <v>408</v>
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="7">
-        <v>18719</v>
+        <v>17485</v>
       </c>
       <c r="D51" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2936,11 +2940,11 @@
     </row>
     <row r="52" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A52" s="50" t="s">
-        <v>411</v>
+        <v>305</v>
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="7">
-        <v>19068</v>
+        <v>17791</v>
       </c>
       <c r="D52" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2949,11 +2953,11 @@
     </row>
     <row r="53" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A53" s="50" t="s">
-        <v>314</v>
+        <v>409</v>
       </c>
       <c r="B53" s="7"/>
-      <c r="C53" s="7">
-        <v>19892</v>
+      <c r="C53" s="37">
+        <v>18139</v>
       </c>
       <c r="D53" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2962,11 +2966,11 @@
     </row>
     <row r="54" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="50" t="s">
-        <v>412</v>
+        <v>308</v>
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="7">
-        <v>20240</v>
+        <v>18719</v>
       </c>
       <c r="D54" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2975,39 +2979,37 @@
     </row>
     <row r="55" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="50" t="s">
-        <v>320</v>
+        <v>411</v>
       </c>
       <c r="B55" s="7"/>
       <c r="C55" s="7">
-        <v>20813</v>
+        <v>19068</v>
       </c>
       <c r="D55" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="E55" s="7"/>
     </row>
     <row r="56" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A56" s="50" t="s">
-        <v>413</v>
+        <v>314</v>
       </c>
       <c r="B56" s="7"/>
       <c r="C56" s="7">
-        <v>21161</v>
+        <v>19892</v>
       </c>
       <c r="D56" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="E56" s="7"/>
     </row>
     <row r="57" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A57" s="50" t="s">
-        <v>322</v>
+        <v>412</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7">
-        <v>22195</v>
+        <v>20240</v>
       </c>
       <c r="D57" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3016,37 +3018,39 @@
     </row>
     <row r="58" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
-        <v>414</v>
+        <v>320</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7">
-        <v>22543</v>
+        <v>20813</v>
       </c>
       <c r="D58" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
+      <c r="E58" s="7"/>
     </row>
     <row r="59" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>324</v>
+        <v>413</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7">
-        <v>22963</v>
+        <v>21161</v>
       </c>
       <c r="D59" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
+      <c r="E59" s="7"/>
     </row>
     <row r="60" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>415</v>
+        <v>322</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7">
-        <v>23346</v>
+        <v>22195</v>
       </c>
       <c r="D60" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3055,11 +3059,11 @@
     </row>
     <row r="61" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7">
-        <v>23873</v>
+        <v>22543</v>
       </c>
       <c r="D61" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3068,11 +3072,11 @@
     </row>
     <row r="62" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>417</v>
-      </c>
-      <c r="B62" s="8"/>
-      <c r="C62" s="50">
-        <v>24221</v>
+        <v>324</v>
+      </c>
+      <c r="B62" s="7"/>
+      <c r="C62" s="7">
+        <v>22963</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3081,11 +3085,11 @@
     </row>
     <row r="63" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>418</v>
-      </c>
-      <c r="B63" s="33"/>
-      <c r="C63" s="33">
-        <v>25101</v>
+        <v>415</v>
+      </c>
+      <c r="B63" s="7"/>
+      <c r="C63" s="7">
+        <v>23346</v>
       </c>
       <c r="D63" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3094,11 +3098,11 @@
     </row>
     <row r="64" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7">
-        <v>25450</v>
+        <v>23873</v>
       </c>
       <c r="D64" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3107,11 +3111,11 @@
     </row>
     <row r="65" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>420</v>
-      </c>
-      <c r="B65" s="7"/>
-      <c r="C65" s="7">
-        <v>26350</v>
+        <v>417</v>
+      </c>
+      <c r="B65" s="8"/>
+      <c r="C65" s="50">
+        <v>24221</v>
       </c>
       <c r="D65" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3120,11 +3124,11 @@
     </row>
     <row r="66" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>421</v>
-      </c>
-      <c r="B66" s="7"/>
-      <c r="C66" s="7">
-        <v>26699</v>
+        <v>418</v>
+      </c>
+      <c r="B66" s="33"/>
+      <c r="C66" s="33">
+        <v>25101</v>
       </c>
       <c r="D66" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3133,11 +3137,11 @@
     </row>
     <row r="67" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>332</v>
+        <v>419</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>27490</v>
+        <v>25450</v>
       </c>
       <c r="D67" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3146,11 +3150,11 @@
     </row>
     <row r="68" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>5</v>
+        <v>420</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7">
-        <v>27836</v>
+        <v>26350</v>
       </c>
       <c r="D68" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3159,11 +3163,11 @@
     </row>
     <row r="69" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>337</v>
+        <v>421</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7">
-        <v>28899</v>
+        <v>26699</v>
       </c>
       <c r="D69" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3172,11 +3176,11 @@
     </row>
     <row r="70" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>6</v>
+        <v>332</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>29248</v>
+        <v>27490</v>
       </c>
       <c r="D70" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3185,11 +3189,11 @@
     </row>
     <row r="71" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>29962</v>
+        <v>27836</v>
       </c>
       <c r="D71" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3198,11 +3202,11 @@
     </row>
     <row r="72" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>7</v>
+        <v>337</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>30309</v>
+        <v>28899</v>
       </c>
       <c r="D72" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3211,11 +3215,11 @@
     </row>
     <row r="73" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>46</v>
+        <v>6</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>30479</v>
+        <v>29248</v>
       </c>
       <c r="D73" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3224,27 +3228,24 @@
     </row>
     <row r="74" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>31125</v>
+        <v>29962</v>
       </c>
       <c r="D74" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
-      </c>
-      <c r="E74" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>31643</v>
+        <v>30309</v>
       </c>
       <c r="D75" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3253,274 +3254,277 @@
     </row>
     <row r="76" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>31991</v>
+        <v>30479</v>
       </c>
       <c r="D76" s="3" t="str">
-        <f t="shared" ref="D76:D111" si="1">IF(C76&lt;&gt;"",IF(B76&lt;&gt;"",C76-B76,"-"), "-")</f>
+        <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>32586</v>
+        <v>31125</v>
       </c>
       <c r="D77" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E77" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>33254</v>
+        <v>31643</v>
       </c>
       <c r="D78" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="E78" t="s">
-        <v>422</v>
+        <f t="shared" si="0"/>
+        <v>-</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>33883</v>
+        <v>31991</v>
       </c>
       <c r="D79" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="D79:D114" si="1">IF(C79&lt;&gt;"",IF(B79&lt;&gt;"",C79-B79,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>34244</v>
+        <v>32586</v>
       </c>
       <c r="D80" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>34862</v>
+        <v>33254</v>
       </c>
       <c r="D81" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="E81" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>35218</v>
+        <v>33883</v>
       </c>
       <c r="D82" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="83" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="B83" s="7"/>
       <c r="C83" s="7">
-        <v>35772</v>
+        <v>34244</v>
       </c>
       <c r="D83" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="84" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="B84" s="7"/>
       <c r="C84" s="7">
-        <v>36120</v>
+        <v>34862</v>
       </c>
       <c r="D84" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="85" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>36893</v>
+        <v>35218</v>
       </c>
       <c r="D85" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="86" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="B86" s="7"/>
       <c r="C86" s="7">
-        <v>37238</v>
+        <v>35772</v>
       </c>
       <c r="D86" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="87" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>38097</v>
+        <v>36120</v>
       </c>
       <c r="D87" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>38443</v>
+        <v>36893</v>
       </c>
       <c r="D88" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>38692</v>
+        <v>37238</v>
       </c>
       <c r="D89" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="90" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>39041</v>
+        <v>38097</v>
       </c>
       <c r="D90" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="91" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>40011</v>
+        <v>38443</v>
       </c>
       <c r="D91" s="3" t="str">
-        <f>IF(C90&lt;&gt;"",IF(B90&lt;&gt;"",C90-B90,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>40373</v>
+        <v>38692</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="93" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B93" s="40"/>
+        <v>15</v>
+      </c>
+      <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>41117</v>
+        <v>39041</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="94" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>41465</v>
+        <v>40011</v>
       </c>
       <c r="D94" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <f>IF(C93&lt;&gt;"",IF(B93&lt;&gt;"",C93-B93,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>42450</v>
+        <v>40373</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="96" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>18</v>
-      </c>
-      <c r="B96" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B96" s="40"/>
       <c r="C96" s="7">
-        <v>42799</v>
+        <v>41117</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3529,11 +3533,11 @@
     </row>
     <row r="97" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>43144</v>
+        <v>41465</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3542,11 +3546,11 @@
     </row>
     <row r="98" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>43491</v>
+        <v>42450</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3555,11 +3559,11 @@
     </row>
     <row r="99" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>44165</v>
+        <v>42799</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3568,11 +3572,11 @@
     </row>
     <row r="100" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>44512</v>
+        <v>43144</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3581,11 +3585,11 @@
     </row>
     <row r="101" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>45061</v>
+        <v>43491</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3594,11 +3598,11 @@
     </row>
     <row r="102" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A102" s="50" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="B102" s="7"/>
       <c r="C102" s="7">
-        <v>45443</v>
+        <v>44165</v>
       </c>
       <c r="D102" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3607,11 +3611,11 @@
     </row>
     <row r="103" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A103" s="50" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="B103" s="7"/>
       <c r="C103" s="7">
-        <v>45990</v>
+        <v>44512</v>
       </c>
       <c r="D103" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3620,27 +3624,24 @@
     </row>
     <row r="104" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A104" s="50" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="B104" s="7"/>
       <c r="C104" s="7">
-        <v>46652</v>
+        <v>45061</v>
       </c>
       <c r="D104" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
-      </c>
-      <c r="E104" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="105" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A105" s="50" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="B105" s="7"/>
       <c r="C105" s="7">
-        <v>47436</v>
+        <v>45443</v>
       </c>
       <c r="D105" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3649,11 +3650,11 @@
     </row>
     <row r="106" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A106" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B106" s="9"/>
-      <c r="C106" s="9">
-        <v>48337</v>
+        <v>41</v>
+      </c>
+      <c r="B106" s="7"/>
+      <c r="C106" s="7">
+        <v>45990</v>
       </c>
       <c r="D106" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3662,24 +3663,27 @@
     </row>
     <row r="107" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A107" s="50" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="B107" s="7"/>
       <c r="C107" s="7">
-        <v>49334</v>
+        <v>46652</v>
       </c>
       <c r="D107" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
+      </c>
+      <c r="E107" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="108" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A108" s="50" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="B108" s="7"/>
       <c r="C108" s="7">
-        <v>48681</v>
+        <v>47436</v>
       </c>
       <c r="D108" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3688,11 +3692,11 @@
     </row>
     <row r="109" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A109" s="50" t="s">
-        <v>44</v>
-      </c>
-      <c r="B109" s="7"/>
-      <c r="C109" s="7">
-        <v>49334</v>
+        <v>23</v>
+      </c>
+      <c r="B109" s="9"/>
+      <c r="C109" s="9">
+        <v>48337</v>
       </c>
       <c r="D109" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3701,11 +3705,11 @@
     </row>
     <row r="110" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A110" s="50" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="B110" s="7"/>
       <c r="C110" s="7">
-        <v>49683</v>
+        <v>49334</v>
       </c>
       <c r="D110" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3714,82 +3718,109 @@
     </row>
     <row r="111" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A111" s="50" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B111" s="7"/>
       <c r="C111" s="7">
+        <v>48681</v>
+      </c>
+      <c r="D111" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A112" s="50" t="s">
+        <v>44</v>
+      </c>
+      <c r="B112" s="7"/>
+      <c r="C112" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D112" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A113" s="50" t="s">
+        <v>25</v>
+      </c>
+      <c r="B113" s="7"/>
+      <c r="C113" s="7">
+        <v>49683</v>
+      </c>
+      <c r="D113" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A114" s="50" t="s">
+        <v>26</v>
+      </c>
+      <c r="B114" s="7"/>
+      <c r="C114" s="7">
         <v>50244</v>
       </c>
-      <c r="D111" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B112" s="7"/>
-      <c r="C112" s="7"/>
-    </row>
-    <row r="113" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B113" s="7"/>
-      <c r="C113" s="7"/>
-    </row>
-    <row r="114" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B114" s="7"/>
-      <c r="C114" s="7"/>
-    </row>
-    <row r="115" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="D114" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B115" s="7"/>
       <c r="C115" s="7"/>
     </row>
-    <row r="116" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B116" s="7"/>
       <c r="C116" s="7"/>
     </row>
-    <row r="117" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B117" s="7"/>
       <c r="C117" s="7"/>
     </row>
-    <row r="118" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B118" s="7"/>
       <c r="C118" s="7"/>
     </row>
-    <row r="119" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B119" s="7"/>
       <c r="C119" s="7"/>
     </row>
-    <row r="120" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B120" s="7"/>
       <c r="C120" s="7"/>
     </row>
-    <row r="121" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B121" s="7"/>
       <c r="C121" s="7"/>
     </row>
-    <row r="122" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B122" s="7"/>
       <c r="C122" s="7"/>
     </row>
-    <row r="123" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B123" s="7"/>
       <c r="C123" s="7"/>
     </row>
-    <row r="124" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B124" s="7"/>
       <c r="C124" s="7"/>
     </row>
-    <row r="125" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B125" s="7"/>
       <c r="C125" s="7"/>
     </row>
-    <row r="126" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B126" s="7"/>
       <c r="C126" s="7"/>
     </row>
-    <row r="127" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B127" s="7"/>
       <c r="C127" s="7"/>
     </row>
-    <row r="128" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B128" s="7"/>
       <c r="C128" s="7"/>
     </row>
@@ -4056,6 +4087,18 @@
     <row r="194" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B194" s="7"/>
       <c r="C194" s="7"/>
+    </row>
+    <row r="195" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B195" s="7"/>
+      <c r="C195" s="7"/>
+    </row>
+    <row r="196" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B196" s="7"/>
+      <c r="C196" s="7"/>
+    </row>
+    <row r="197" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B197" s="7"/>
+      <c r="C197" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - level 9 done 69 frames ahead but unable to do scroll skip in level 10
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAFC8A1A-9FEF-4418-B586-8A45C2653B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6620889-72F8-4672-B6CF-4EE36D92C119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2256,7 +2256,7 @@
         <v>427</v>
       </c>
       <c r="D2" s="3">
-        <f t="shared" ref="D2:D78" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <f t="shared" ref="D2:D31" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
         <v>-1</v>
       </c>
       <c r="E2" t="s">
@@ -2679,13 +2679,15 @@
       <c r="A32" s="50" t="s">
         <v>274</v>
       </c>
-      <c r="B32" s="7"/>
+      <c r="B32" s="7">
+        <v>8127</v>
+      </c>
       <c r="C32" s="7">
         <v>8196</v>
       </c>
-      <c r="D32" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D32" s="3">
+        <f>IF(C32&lt;&gt;"",IF(B32&lt;&gt;"",C32-B32,"-"), "-")</f>
+        <v>69</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -2697,7 +2699,7 @@
         <v>8549</v>
       </c>
       <c r="D33" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C33&lt;&gt;"",IF(B33&lt;&gt;"",C33-B33,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2710,7 +2712,7 @@
         <v>9118</v>
       </c>
       <c r="D34" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C34&lt;&gt;"",IF(B34&lt;&gt;"",C34-B34,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2723,7 +2725,7 @@
         <v>9467</v>
       </c>
       <c r="D35" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C35&lt;&gt;"",IF(B35&lt;&gt;"",C35-B35,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2736,7 +2738,7 @@
         <v>9778</v>
       </c>
       <c r="D36" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C36&lt;&gt;"",IF(B36&lt;&gt;"",C36-B36,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2749,7 +2751,7 @@
         <v>10125</v>
       </c>
       <c r="D37" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C37&lt;&gt;"",IF(B37&lt;&gt;"",C37-B37,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2762,7 +2764,7 @@
         <v>10816</v>
       </c>
       <c r="D38" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C38&lt;&gt;"",IF(B38&lt;&gt;"",C38-B38,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2775,7 +2777,7 @@
         <v>11163</v>
       </c>
       <c r="D39" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C39&lt;&gt;"",IF(B39&lt;&gt;"",C39-B39,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2788,7 +2790,7 @@
         <v>11729</v>
       </c>
       <c r="D40" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C40&lt;&gt;"",IF(B40&lt;&gt;"",C40-B40,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2801,7 +2803,7 @@
         <v>12383</v>
       </c>
       <c r="D41" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C41&lt;&gt;"",IF(B41&lt;&gt;"",C41-B41,"-"), "-")</f>
         <v>-</v>
       </c>
       <c r="E41" t="s">
@@ -2817,7 +2819,7 @@
         <v>12891</v>
       </c>
       <c r="D42" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C42&lt;&gt;"",IF(B42&lt;&gt;"",C42-B42,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2830,7 +2832,7 @@
         <v>13269</v>
       </c>
       <c r="D43" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C43&lt;&gt;"",IF(B43&lt;&gt;"",C43-B43,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2843,7 +2845,7 @@
         <v>13960</v>
       </c>
       <c r="D44" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C44&lt;&gt;"",IF(B44&lt;&gt;"",C44-B44,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2856,7 +2858,7 @@
         <v>14320</v>
       </c>
       <c r="D45" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C45&lt;&gt;"",IF(B45&lt;&gt;"",C45-B45,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2869,7 +2871,7 @@
         <v>14679</v>
       </c>
       <c r="D46" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C46&lt;&gt;"",IF(B46&lt;&gt;"",C46-B46,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2882,7 +2884,7 @@
         <v>15029</v>
       </c>
       <c r="D47" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C47&lt;&gt;"",IF(B47&lt;&gt;"",C47-B47,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2895,7 +2897,7 @@
         <v>15850</v>
       </c>
       <c r="D48" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C48&lt;&gt;"",IF(B48&lt;&gt;"",C48-B48,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2908,7 +2910,7 @@
         <v>16200</v>
       </c>
       <c r="D49" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C49&lt;&gt;"",IF(B49&lt;&gt;"",C49-B49,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2921,7 +2923,7 @@
         <v>17135</v>
       </c>
       <c r="D50" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C50&lt;&gt;"",IF(B50&lt;&gt;"",C50-B50,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2934,7 +2936,7 @@
         <v>17485</v>
       </c>
       <c r="D51" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2947,7 +2949,7 @@
         <v>17791</v>
       </c>
       <c r="D52" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C52&lt;&gt;"",IF(B52&lt;&gt;"",C52-B52,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2960,7 +2962,7 @@
         <v>18139</v>
       </c>
       <c r="D53" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C53&lt;&gt;"",IF(B53&lt;&gt;"",C53-B53,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2973,7 +2975,7 @@
         <v>18719</v>
       </c>
       <c r="D54" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C54&lt;&gt;"",IF(B54&lt;&gt;"",C54-B54,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2986,7 +2988,7 @@
         <v>19068</v>
       </c>
       <c r="D55" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C55&lt;&gt;"",IF(B55&lt;&gt;"",C55-B55,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -2999,7 +3001,7 @@
         <v>19892</v>
       </c>
       <c r="D56" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C56&lt;&gt;"",IF(B56&lt;&gt;"",C56-B56,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3012,7 +3014,7 @@
         <v>20240</v>
       </c>
       <c r="D57" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C57&lt;&gt;"",IF(B57&lt;&gt;"",C57-B57,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3025,7 +3027,7 @@
         <v>20813</v>
       </c>
       <c r="D58" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C58&lt;&gt;"",IF(B58&lt;&gt;"",C58-B58,"-"), "-")</f>
         <v>-</v>
       </c>
       <c r="E58" s="7"/>
@@ -3039,7 +3041,7 @@
         <v>21161</v>
       </c>
       <c r="D59" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C59&lt;&gt;"",IF(B59&lt;&gt;"",C59-B59,"-"), "-")</f>
         <v>-</v>
       </c>
       <c r="E59" s="7"/>
@@ -3053,7 +3055,7 @@
         <v>22195</v>
       </c>
       <c r="D60" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C60&lt;&gt;"",IF(B60&lt;&gt;"",C60-B60,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3066,7 +3068,7 @@
         <v>22543</v>
       </c>
       <c r="D61" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C61&lt;&gt;"",IF(B61&lt;&gt;"",C61-B61,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3079,7 +3081,7 @@
         <v>22963</v>
       </c>
       <c r="D62" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C62&lt;&gt;"",IF(B62&lt;&gt;"",C62-B62,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3092,7 +3094,7 @@
         <v>23346</v>
       </c>
       <c r="D63" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C63&lt;&gt;"",IF(B63&lt;&gt;"",C63-B63,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3105,7 +3107,7 @@
         <v>23873</v>
       </c>
       <c r="D64" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C64&lt;&gt;"",IF(B64&lt;&gt;"",C64-B64,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3118,7 +3120,7 @@
         <v>24221</v>
       </c>
       <c r="D65" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C65&lt;&gt;"",IF(B65&lt;&gt;"",C65-B65,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3131,7 +3133,7 @@
         <v>25101</v>
       </c>
       <c r="D66" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C66&lt;&gt;"",IF(B66&lt;&gt;"",C66-B66,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3144,7 +3146,7 @@
         <v>25450</v>
       </c>
       <c r="D67" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C67&lt;&gt;"",IF(B67&lt;&gt;"",C67-B67,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3157,7 +3159,7 @@
         <v>26350</v>
       </c>
       <c r="D68" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C68&lt;&gt;"",IF(B68&lt;&gt;"",C68-B68,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3170,7 +3172,7 @@
         <v>26699</v>
       </c>
       <c r="D69" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C69&lt;&gt;"",IF(B69&lt;&gt;"",C69-B69,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3183,7 +3185,7 @@
         <v>27490</v>
       </c>
       <c r="D70" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C70&lt;&gt;"",IF(B70&lt;&gt;"",C70-B70,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3196,7 +3198,7 @@
         <v>27836</v>
       </c>
       <c r="D71" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C71&lt;&gt;"",IF(B71&lt;&gt;"",C71-B71,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3209,7 +3211,7 @@
         <v>28899</v>
       </c>
       <c r="D72" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C72&lt;&gt;"",IF(B72&lt;&gt;"",C72-B72,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3222,7 +3224,7 @@
         <v>29248</v>
       </c>
       <c r="D73" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C73&lt;&gt;"",IF(B73&lt;&gt;"",C73-B73,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3235,7 +3237,7 @@
         <v>29962</v>
       </c>
       <c r="D74" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C74&lt;&gt;"",IF(B74&lt;&gt;"",C74-B74,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3248,7 +3250,7 @@
         <v>30309</v>
       </c>
       <c r="D75" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C75&lt;&gt;"",IF(B75&lt;&gt;"",C75-B75,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3261,7 +3263,7 @@
         <v>30479</v>
       </c>
       <c r="D76" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C76&lt;&gt;"",IF(B76&lt;&gt;"",C76-B76,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3274,7 +3276,7 @@
         <v>31125</v>
       </c>
       <c r="D77" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C77&lt;&gt;"",IF(B77&lt;&gt;"",C77-B77,"-"), "-")</f>
         <v>-</v>
       </c>
       <c r="E77" t="s">
@@ -3290,7 +3292,7 @@
         <v>31643</v>
       </c>
       <c r="D78" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C78&lt;&gt;"",IF(B78&lt;&gt;"",C78-B78,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3303,7 +3305,7 @@
         <v>31991</v>
       </c>
       <c r="D79" s="3" t="str">
-        <f t="shared" ref="D79:D114" si="1">IF(C79&lt;&gt;"",IF(B79&lt;&gt;"",C79-B79,"-"), "-")</f>
+        <f>IF(C79&lt;&gt;"",IF(B79&lt;&gt;"",C79-B79,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3316,7 +3318,7 @@
         <v>32586</v>
       </c>
       <c r="D80" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C80&lt;&gt;"",IF(B80&lt;&gt;"",C80-B80,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3329,7 +3331,7 @@
         <v>33254</v>
       </c>
       <c r="D81" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C81&lt;&gt;"",IF(B81&lt;&gt;"",C81-B81,"-"), "-")</f>
         <v>-</v>
       </c>
       <c r="E81" t="s">
@@ -3345,7 +3347,7 @@
         <v>33883</v>
       </c>
       <c r="D82" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3358,7 +3360,7 @@
         <v>34244</v>
       </c>
       <c r="D83" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C83&lt;&gt;"",IF(B83&lt;&gt;"",C83-B83,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3371,7 +3373,7 @@
         <v>34862</v>
       </c>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C84&lt;&gt;"",IF(B84&lt;&gt;"",C84-B84,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3384,7 +3386,7 @@
         <v>35218</v>
       </c>
       <c r="D85" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C85&lt;&gt;"",IF(B85&lt;&gt;"",C85-B85,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3397,7 +3399,7 @@
         <v>35772</v>
       </c>
       <c r="D86" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C86&lt;&gt;"",IF(B86&lt;&gt;"",C86-B86,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3410,7 +3412,7 @@
         <v>36120</v>
       </c>
       <c r="D87" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C87&lt;&gt;"",IF(B87&lt;&gt;"",C87-B87,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3423,7 +3425,7 @@
         <v>36893</v>
       </c>
       <c r="D88" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C88&lt;&gt;"",IF(B88&lt;&gt;"",C88-B88,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3436,7 +3438,7 @@
         <v>37238</v>
       </c>
       <c r="D89" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C89&lt;&gt;"",IF(B89&lt;&gt;"",C89-B89,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3449,7 +3451,7 @@
         <v>38097</v>
       </c>
       <c r="D90" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C90&lt;&gt;"",IF(B90&lt;&gt;"",C90-B90,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3462,7 +3464,7 @@
         <v>38443</v>
       </c>
       <c r="D91" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C91&lt;&gt;"",IF(B91&lt;&gt;"",C91-B91,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3475,7 +3477,7 @@
         <v>38692</v>
       </c>
       <c r="D92" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C92&lt;&gt;"",IF(B92&lt;&gt;"",C92-B92,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3488,7 +3490,7 @@
         <v>39041</v>
       </c>
       <c r="D93" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C93&lt;&gt;"",IF(B93&lt;&gt;"",C93-B93,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3514,7 +3516,7 @@
         <v>40373</v>
       </c>
       <c r="D95" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C95&lt;&gt;"",IF(B95&lt;&gt;"",C95-B95,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3527,7 +3529,7 @@
         <v>41117</v>
       </c>
       <c r="D96" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C96&lt;&gt;"",IF(B96&lt;&gt;"",C96-B96,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3540,7 +3542,7 @@
         <v>41465</v>
       </c>
       <c r="D97" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C97&lt;&gt;"",IF(B97&lt;&gt;"",C97-B97,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3553,7 +3555,7 @@
         <v>42450</v>
       </c>
       <c r="D98" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C98&lt;&gt;"",IF(B98&lt;&gt;"",C98-B98,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3566,7 +3568,7 @@
         <v>42799</v>
       </c>
       <c r="D99" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C99&lt;&gt;"",IF(B99&lt;&gt;"",C99-B99,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3579,7 +3581,7 @@
         <v>43144</v>
       </c>
       <c r="D100" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C100&lt;&gt;"",IF(B100&lt;&gt;"",C100-B100,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3592,7 +3594,7 @@
         <v>43491</v>
       </c>
       <c r="D101" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C101&lt;&gt;"",IF(B101&lt;&gt;"",C101-B101,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3605,7 +3607,7 @@
         <v>44165</v>
       </c>
       <c r="D102" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C102&lt;&gt;"",IF(B102&lt;&gt;"",C102-B102,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3618,7 +3620,7 @@
         <v>44512</v>
       </c>
       <c r="D103" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C103&lt;&gt;"",IF(B103&lt;&gt;"",C103-B103,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3631,7 +3633,7 @@
         <v>45061</v>
       </c>
       <c r="D104" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C104&lt;&gt;"",IF(B104&lt;&gt;"",C104-B104,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3644,7 +3646,7 @@
         <v>45443</v>
       </c>
       <c r="D105" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C105&lt;&gt;"",IF(B105&lt;&gt;"",C105-B105,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3657,7 +3659,7 @@
         <v>45990</v>
       </c>
       <c r="D106" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3670,7 +3672,7 @@
         <v>46652</v>
       </c>
       <c r="D107" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C107&lt;&gt;"",IF(B107&lt;&gt;"",C107-B107,"-"), "-")</f>
         <v>-</v>
       </c>
       <c r="E107" t="s">
@@ -3686,7 +3688,7 @@
         <v>47436</v>
       </c>
       <c r="D108" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C108&lt;&gt;"",IF(B108&lt;&gt;"",C108-B108,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3699,7 +3701,7 @@
         <v>48337</v>
       </c>
       <c r="D109" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C109&lt;&gt;"",IF(B109&lt;&gt;"",C109-B109,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3712,7 +3714,7 @@
         <v>49334</v>
       </c>
       <c r="D110" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C110&lt;&gt;"",IF(B110&lt;&gt;"",C110-B110,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3725,7 +3727,7 @@
         <v>48681</v>
       </c>
       <c r="D111" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C111&lt;&gt;"",IF(B111&lt;&gt;"",C111-B111,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3738,7 +3740,7 @@
         <v>49334</v>
       </c>
       <c r="D112" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C112&lt;&gt;"",IF(B112&lt;&gt;"",C112-B112,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3751,7 +3753,7 @@
         <v>49683</v>
       </c>
       <c r="D113" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C113&lt;&gt;"",IF(B113&lt;&gt;"",C113-B113,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3764,7 +3766,7 @@
         <v>50244</v>
       </c>
       <c r="D114" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(C114&lt;&gt;"",IF(B114&lt;&gt;"",C114-B114,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>

</xml_diff>

<commit_message>
lode runner - skip manipulated before level 10 but at the cost of most frames, only 22 ahead, attempts to do better have failed
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6620889-72F8-4672-B6CF-4EE36D92C119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51BC573-3801-49DC-9F19-8B116FE11613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2694,13 +2694,15 @@
       <c r="A33" s="50" t="s">
         <v>399</v>
       </c>
-      <c r="B33" s="7"/>
+      <c r="B33" s="7">
+        <v>8527</v>
+      </c>
       <c r="C33" s="7">
         <v>8549</v>
       </c>
-      <c r="D33" s="3" t="str">
+      <c r="D33" s="3">
         <f>IF(C33&lt;&gt;"",IF(B33&lt;&gt;"",C33-B33,"-"), "-")</f>
-        <v>-</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - level 11 done - 21 frames ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51BC573-3801-49DC-9F19-8B116FE11613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0DA3B36-77B9-408E-8C79-B12ABBD567B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2686,7 +2686,7 @@
         <v>8196</v>
       </c>
       <c r="D32" s="3">
-        <f>IF(C32&lt;&gt;"",IF(B32&lt;&gt;"",C32-B32,"-"), "-")</f>
+        <f t="shared" ref="D32:D63" si="1">IF(C32&lt;&gt;"",IF(B32&lt;&gt;"",C32-B32,"-"), "-")</f>
         <v>69</v>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
         <v>8549</v>
       </c>
       <c r="D33" s="3">
-        <f>IF(C33&lt;&gt;"",IF(B33&lt;&gt;"",C33-B33,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
     </row>
@@ -2709,52 +2709,60 @@
       <c r="A34" s="50" t="s">
         <v>276</v>
       </c>
-      <c r="B34" s="7"/>
+      <c r="B34" s="7">
+        <v>9099</v>
+      </c>
       <c r="C34" s="7">
         <v>9118</v>
       </c>
-      <c r="D34" s="3" t="str">
-        <f>IF(C34&lt;&gt;"",IF(B34&lt;&gt;"",C34-B34,"-"), "-")</f>
-        <v>-</v>
+      <c r="D34" s="3">
+        <f t="shared" si="1"/>
+        <v>19</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A35" s="50" t="s">
         <v>400</v>
       </c>
-      <c r="B35" s="7"/>
+      <c r="B35" s="7">
+        <v>9447</v>
+      </c>
       <c r="C35" s="7">
         <v>9467</v>
       </c>
-      <c r="D35" s="3" t="str">
-        <f>IF(C35&lt;&gt;"",IF(B35&lt;&gt;"",C35-B35,"-"), "-")</f>
-        <v>-</v>
+      <c r="D35" s="3">
+        <f t="shared" si="1"/>
+        <v>20</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
         <v>278</v>
       </c>
-      <c r="B36" s="7"/>
+      <c r="B36" s="7">
+        <v>9758</v>
+      </c>
       <c r="C36" s="7">
         <v>9778</v>
       </c>
-      <c r="D36" s="3" t="str">
-        <f>IF(C36&lt;&gt;"",IF(B36&lt;&gt;"",C36-B36,"-"), "-")</f>
-        <v>-</v>
+      <c r="D36" s="3">
+        <f t="shared" si="1"/>
+        <v>20</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="50" t="s">
         <v>401</v>
       </c>
-      <c r="B37" s="7"/>
+      <c r="B37" s="7">
+        <v>10104</v>
+      </c>
       <c r="C37" s="7">
         <v>10125</v>
       </c>
-      <c r="D37" s="3" t="str">
-        <f>IF(C37&lt;&gt;"",IF(B37&lt;&gt;"",C37-B37,"-"), "-")</f>
-        <v>-</v>
+      <c r="D37" s="3">
+        <f t="shared" si="1"/>
+        <v>21</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
@@ -2766,7 +2774,7 @@
         <v>10816</v>
       </c>
       <c r="D38" s="3" t="str">
-        <f>IF(C38&lt;&gt;"",IF(B38&lt;&gt;"",C38-B38,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2779,7 +2787,7 @@
         <v>11163</v>
       </c>
       <c r="D39" s="3" t="str">
-        <f>IF(C39&lt;&gt;"",IF(B39&lt;&gt;"",C39-B39,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2792,7 +2800,7 @@
         <v>11729</v>
       </c>
       <c r="D40" s="3" t="str">
-        <f>IF(C40&lt;&gt;"",IF(B40&lt;&gt;"",C40-B40,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2805,7 +2813,7 @@
         <v>12383</v>
       </c>
       <c r="D41" s="3" t="str">
-        <f>IF(C41&lt;&gt;"",IF(B41&lt;&gt;"",C41-B41,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="E41" t="s">
@@ -2821,7 +2829,7 @@
         <v>12891</v>
       </c>
       <c r="D42" s="3" t="str">
-        <f>IF(C42&lt;&gt;"",IF(B42&lt;&gt;"",C42-B42,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2834,7 +2842,7 @@
         <v>13269</v>
       </c>
       <c r="D43" s="3" t="str">
-        <f>IF(C43&lt;&gt;"",IF(B43&lt;&gt;"",C43-B43,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2847,7 +2855,7 @@
         <v>13960</v>
       </c>
       <c r="D44" s="3" t="str">
-        <f>IF(C44&lt;&gt;"",IF(B44&lt;&gt;"",C44-B44,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2860,7 +2868,7 @@
         <v>14320</v>
       </c>
       <c r="D45" s="3" t="str">
-        <f>IF(C45&lt;&gt;"",IF(B45&lt;&gt;"",C45-B45,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2873,7 +2881,7 @@
         <v>14679</v>
       </c>
       <c r="D46" s="3" t="str">
-        <f>IF(C46&lt;&gt;"",IF(B46&lt;&gt;"",C46-B46,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2886,7 +2894,7 @@
         <v>15029</v>
       </c>
       <c r="D47" s="3" t="str">
-        <f>IF(C47&lt;&gt;"",IF(B47&lt;&gt;"",C47-B47,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2899,7 +2907,7 @@
         <v>15850</v>
       </c>
       <c r="D48" s="3" t="str">
-        <f>IF(C48&lt;&gt;"",IF(B48&lt;&gt;"",C48-B48,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2912,7 +2920,7 @@
         <v>16200</v>
       </c>
       <c r="D49" s="3" t="str">
-        <f>IF(C49&lt;&gt;"",IF(B49&lt;&gt;"",C49-B49,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2925,7 +2933,7 @@
         <v>17135</v>
       </c>
       <c r="D50" s="3" t="str">
-        <f>IF(C50&lt;&gt;"",IF(B50&lt;&gt;"",C50-B50,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2938,7 +2946,7 @@
         <v>17485</v>
       </c>
       <c r="D51" s="3" t="str">
-        <f>IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2951,7 +2959,7 @@
         <v>17791</v>
       </c>
       <c r="D52" s="3" t="str">
-        <f>IF(C52&lt;&gt;"",IF(B52&lt;&gt;"",C52-B52,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2964,7 +2972,7 @@
         <v>18139</v>
       </c>
       <c r="D53" s="3" t="str">
-        <f>IF(C53&lt;&gt;"",IF(B53&lt;&gt;"",C53-B53,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2977,7 +2985,7 @@
         <v>18719</v>
       </c>
       <c r="D54" s="3" t="str">
-        <f>IF(C54&lt;&gt;"",IF(B54&lt;&gt;"",C54-B54,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -2990,7 +2998,7 @@
         <v>19068</v>
       </c>
       <c r="D55" s="3" t="str">
-        <f>IF(C55&lt;&gt;"",IF(B55&lt;&gt;"",C55-B55,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -3003,7 +3011,7 @@
         <v>19892</v>
       </c>
       <c r="D56" s="3" t="str">
-        <f>IF(C56&lt;&gt;"",IF(B56&lt;&gt;"",C56-B56,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -3016,7 +3024,7 @@
         <v>20240</v>
       </c>
       <c r="D57" s="3" t="str">
-        <f>IF(C57&lt;&gt;"",IF(B57&lt;&gt;"",C57-B57,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -3029,7 +3037,7 @@
         <v>20813</v>
       </c>
       <c r="D58" s="3" t="str">
-        <f>IF(C58&lt;&gt;"",IF(B58&lt;&gt;"",C58-B58,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="E58" s="7"/>
@@ -3043,7 +3051,7 @@
         <v>21161</v>
       </c>
       <c r="D59" s="3" t="str">
-        <f>IF(C59&lt;&gt;"",IF(B59&lt;&gt;"",C59-B59,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="E59" s="7"/>
@@ -3057,7 +3065,7 @@
         <v>22195</v>
       </c>
       <c r="D60" s="3" t="str">
-        <f>IF(C60&lt;&gt;"",IF(B60&lt;&gt;"",C60-B60,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -3070,7 +3078,7 @@
         <v>22543</v>
       </c>
       <c r="D61" s="3" t="str">
-        <f>IF(C61&lt;&gt;"",IF(B61&lt;&gt;"",C61-B61,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -3083,7 +3091,7 @@
         <v>22963</v>
       </c>
       <c r="D62" s="3" t="str">
-        <f>IF(C62&lt;&gt;"",IF(B62&lt;&gt;"",C62-B62,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -3096,7 +3104,7 @@
         <v>23346</v>
       </c>
       <c r="D63" s="3" t="str">
-        <f>IF(C63&lt;&gt;"",IF(B63&lt;&gt;"",C63-B63,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
@@ -3109,7 +3117,7 @@
         <v>23873</v>
       </c>
       <c r="D64" s="3" t="str">
-        <f>IF(C64&lt;&gt;"",IF(B64&lt;&gt;"",C64-B64,"-"), "-")</f>
+        <f t="shared" ref="D64:D95" si="2">IF(C64&lt;&gt;"",IF(B64&lt;&gt;"",C64-B64,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3122,7 +3130,7 @@
         <v>24221</v>
       </c>
       <c r="D65" s="3" t="str">
-        <f>IF(C65&lt;&gt;"",IF(B65&lt;&gt;"",C65-B65,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3135,7 +3143,7 @@
         <v>25101</v>
       </c>
       <c r="D66" s="3" t="str">
-        <f>IF(C66&lt;&gt;"",IF(B66&lt;&gt;"",C66-B66,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3148,7 +3156,7 @@
         <v>25450</v>
       </c>
       <c r="D67" s="3" t="str">
-        <f>IF(C67&lt;&gt;"",IF(B67&lt;&gt;"",C67-B67,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3161,7 +3169,7 @@
         <v>26350</v>
       </c>
       <c r="D68" s="3" t="str">
-        <f>IF(C68&lt;&gt;"",IF(B68&lt;&gt;"",C68-B68,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3174,7 +3182,7 @@
         <v>26699</v>
       </c>
       <c r="D69" s="3" t="str">
-        <f>IF(C69&lt;&gt;"",IF(B69&lt;&gt;"",C69-B69,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3187,7 +3195,7 @@
         <v>27490</v>
       </c>
       <c r="D70" s="3" t="str">
-        <f>IF(C70&lt;&gt;"",IF(B70&lt;&gt;"",C70-B70,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3200,7 +3208,7 @@
         <v>27836</v>
       </c>
       <c r="D71" s="3" t="str">
-        <f>IF(C71&lt;&gt;"",IF(B71&lt;&gt;"",C71-B71,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3213,7 +3221,7 @@
         <v>28899</v>
       </c>
       <c r="D72" s="3" t="str">
-        <f>IF(C72&lt;&gt;"",IF(B72&lt;&gt;"",C72-B72,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3226,7 +3234,7 @@
         <v>29248</v>
       </c>
       <c r="D73" s="3" t="str">
-        <f>IF(C73&lt;&gt;"",IF(B73&lt;&gt;"",C73-B73,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3239,7 +3247,7 @@
         <v>29962</v>
       </c>
       <c r="D74" s="3" t="str">
-        <f>IF(C74&lt;&gt;"",IF(B74&lt;&gt;"",C74-B74,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3252,7 +3260,7 @@
         <v>30309</v>
       </c>
       <c r="D75" s="3" t="str">
-        <f>IF(C75&lt;&gt;"",IF(B75&lt;&gt;"",C75-B75,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3265,7 +3273,7 @@
         <v>30479</v>
       </c>
       <c r="D76" s="3" t="str">
-        <f>IF(C76&lt;&gt;"",IF(B76&lt;&gt;"",C76-B76,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3278,7 +3286,7 @@
         <v>31125</v>
       </c>
       <c r="D77" s="3" t="str">
-        <f>IF(C77&lt;&gt;"",IF(B77&lt;&gt;"",C77-B77,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="E77" t="s">
@@ -3294,7 +3302,7 @@
         <v>31643</v>
       </c>
       <c r="D78" s="3" t="str">
-        <f>IF(C78&lt;&gt;"",IF(B78&lt;&gt;"",C78-B78,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3307,7 +3315,7 @@
         <v>31991</v>
       </c>
       <c r="D79" s="3" t="str">
-        <f>IF(C79&lt;&gt;"",IF(B79&lt;&gt;"",C79-B79,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3320,7 +3328,7 @@
         <v>32586</v>
       </c>
       <c r="D80" s="3" t="str">
-        <f>IF(C80&lt;&gt;"",IF(B80&lt;&gt;"",C80-B80,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3333,7 +3341,7 @@
         <v>33254</v>
       </c>
       <c r="D81" s="3" t="str">
-        <f>IF(C81&lt;&gt;"",IF(B81&lt;&gt;"",C81-B81,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="E81" t="s">
@@ -3349,7 +3357,7 @@
         <v>33883</v>
       </c>
       <c r="D82" s="3" t="str">
-        <f>IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3362,7 +3370,7 @@
         <v>34244</v>
       </c>
       <c r="D83" s="3" t="str">
-        <f>IF(C83&lt;&gt;"",IF(B83&lt;&gt;"",C83-B83,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3375,7 +3383,7 @@
         <v>34862</v>
       </c>
       <c r="D84" s="3" t="str">
-        <f>IF(C84&lt;&gt;"",IF(B84&lt;&gt;"",C84-B84,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3388,7 +3396,7 @@
         <v>35218</v>
       </c>
       <c r="D85" s="3" t="str">
-        <f>IF(C85&lt;&gt;"",IF(B85&lt;&gt;"",C85-B85,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3401,7 +3409,7 @@
         <v>35772</v>
       </c>
       <c r="D86" s="3" t="str">
-        <f>IF(C86&lt;&gt;"",IF(B86&lt;&gt;"",C86-B86,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3414,7 +3422,7 @@
         <v>36120</v>
       </c>
       <c r="D87" s="3" t="str">
-        <f>IF(C87&lt;&gt;"",IF(B87&lt;&gt;"",C87-B87,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3427,7 +3435,7 @@
         <v>36893</v>
       </c>
       <c r="D88" s="3" t="str">
-        <f>IF(C88&lt;&gt;"",IF(B88&lt;&gt;"",C88-B88,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3440,7 +3448,7 @@
         <v>37238</v>
       </c>
       <c r="D89" s="3" t="str">
-        <f>IF(C89&lt;&gt;"",IF(B89&lt;&gt;"",C89-B89,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3453,7 +3461,7 @@
         <v>38097</v>
       </c>
       <c r="D90" s="3" t="str">
-        <f>IF(C90&lt;&gt;"",IF(B90&lt;&gt;"",C90-B90,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3466,7 +3474,7 @@
         <v>38443</v>
       </c>
       <c r="D91" s="3" t="str">
-        <f>IF(C91&lt;&gt;"",IF(B91&lt;&gt;"",C91-B91,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3479,7 +3487,7 @@
         <v>38692</v>
       </c>
       <c r="D92" s="3" t="str">
-        <f>IF(C92&lt;&gt;"",IF(B92&lt;&gt;"",C92-B92,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3492,7 +3500,7 @@
         <v>39041</v>
       </c>
       <c r="D93" s="3" t="str">
-        <f>IF(C93&lt;&gt;"",IF(B93&lt;&gt;"",C93-B93,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
@@ -3518,7 +3526,7 @@
         <v>40373</v>
       </c>
       <c r="D95" s="3" t="str">
-        <f>IF(C95&lt;&gt;"",IF(B95&lt;&gt;"",C95-B95,"-"), "-")</f>
+        <f t="shared" ref="D95:D114" si="3">IF(C95&lt;&gt;"",IF(B95&lt;&gt;"",C95-B95,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -3531,7 +3539,7 @@
         <v>41117</v>
       </c>
       <c r="D96" s="3" t="str">
-        <f>IF(C96&lt;&gt;"",IF(B96&lt;&gt;"",C96-B96,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3544,7 +3552,7 @@
         <v>41465</v>
       </c>
       <c r="D97" s="3" t="str">
-        <f>IF(C97&lt;&gt;"",IF(B97&lt;&gt;"",C97-B97,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3557,7 +3565,7 @@
         <v>42450</v>
       </c>
       <c r="D98" s="3" t="str">
-        <f>IF(C98&lt;&gt;"",IF(B98&lt;&gt;"",C98-B98,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3570,7 +3578,7 @@
         <v>42799</v>
       </c>
       <c r="D99" s="3" t="str">
-        <f>IF(C99&lt;&gt;"",IF(B99&lt;&gt;"",C99-B99,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3583,7 +3591,7 @@
         <v>43144</v>
       </c>
       <c r="D100" s="3" t="str">
-        <f>IF(C100&lt;&gt;"",IF(B100&lt;&gt;"",C100-B100,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3596,7 +3604,7 @@
         <v>43491</v>
       </c>
       <c r="D101" s="3" t="str">
-        <f>IF(C101&lt;&gt;"",IF(B101&lt;&gt;"",C101-B101,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3609,7 +3617,7 @@
         <v>44165</v>
       </c>
       <c r="D102" s="3" t="str">
-        <f>IF(C102&lt;&gt;"",IF(B102&lt;&gt;"",C102-B102,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3622,7 +3630,7 @@
         <v>44512</v>
       </c>
       <c r="D103" s="3" t="str">
-        <f>IF(C103&lt;&gt;"",IF(B103&lt;&gt;"",C103-B103,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3635,7 +3643,7 @@
         <v>45061</v>
       </c>
       <c r="D104" s="3" t="str">
-        <f>IF(C104&lt;&gt;"",IF(B104&lt;&gt;"",C104-B104,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3648,7 +3656,7 @@
         <v>45443</v>
       </c>
       <c r="D105" s="3" t="str">
-        <f>IF(C105&lt;&gt;"",IF(B105&lt;&gt;"",C105-B105,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3661,7 +3669,7 @@
         <v>45990</v>
       </c>
       <c r="D106" s="3" t="str">
-        <f>IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3674,7 +3682,7 @@
         <v>46652</v>
       </c>
       <c r="D107" s="3" t="str">
-        <f>IF(C107&lt;&gt;"",IF(B107&lt;&gt;"",C107-B107,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
       <c r="E107" t="s">
@@ -3690,7 +3698,7 @@
         <v>47436</v>
       </c>
       <c r="D108" s="3" t="str">
-        <f>IF(C108&lt;&gt;"",IF(B108&lt;&gt;"",C108-B108,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3703,7 +3711,7 @@
         <v>48337</v>
       </c>
       <c r="D109" s="3" t="str">
-        <f>IF(C109&lt;&gt;"",IF(B109&lt;&gt;"",C109-B109,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3716,7 +3724,7 @@
         <v>49334</v>
       </c>
       <c r="D110" s="3" t="str">
-        <f>IF(C110&lt;&gt;"",IF(B110&lt;&gt;"",C110-B110,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3729,7 +3737,7 @@
         <v>48681</v>
       </c>
       <c r="D111" s="3" t="str">
-        <f>IF(C111&lt;&gt;"",IF(B111&lt;&gt;"",C111-B111,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3742,7 +3750,7 @@
         <v>49334</v>
       </c>
       <c r="D112" s="3" t="str">
-        <f>IF(C112&lt;&gt;"",IF(B112&lt;&gt;"",C112-B112,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3755,7 +3763,7 @@
         <v>49683</v>
       </c>
       <c r="D113" s="3" t="str">
-        <f>IF(C113&lt;&gt;"",IF(B113&lt;&gt;"",C113-B113,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
@@ -3768,7 +3776,7 @@
         <v>50244</v>
       </c>
       <c r="D114" s="3" t="str">
-        <f>IF(C114&lt;&gt;"",IF(B114&lt;&gt;"",C114-B114,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>

</xml_diff>

<commit_message>
up to level 14, 77 frames ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0DA3B36-77B9-408E-8C79-B12ABBD567B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E84BC021-0226-406A-9380-7D6F5B28F03C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="427">
   <si>
     <t>Place</t>
   </si>
@@ -1311,6 +1311,12 @@
   </si>
   <si>
     <t>1081 possible, delay for spawn timer</t>
+  </si>
+  <si>
+    <t>drop</t>
+  </si>
+  <si>
+    <t>land</t>
   </si>
 </sst>
 </file>
@@ -1320,12 +1326,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="35" x14ac:knownFonts="1">
+  <fonts count="36" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1771,95 +1784,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="33" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1877,31 +1891,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2222,7 +2236,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E197"/>
+  <dimension ref="A1:E200"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2686,7 +2700,7 @@
         <v>8196</v>
       </c>
       <c r="D32" s="3">
-        <f t="shared" ref="D32:D63" si="1">IF(C32&lt;&gt;"",IF(B32&lt;&gt;"",C32-B32,"-"), "-")</f>
+        <f t="shared" ref="D32:D66" si="1">IF(C32&lt;&gt;"",IF(B32&lt;&gt;"",C32-B32,"-"), "-")</f>
         <v>69</v>
       </c>
     </row>
@@ -2766,145 +2780,157 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A38" s="50" t="s">
-        <v>281</v>
-      </c>
-      <c r="B38" s="7"/>
+      <c r="A38" s="59" t="s">
+        <v>127</v>
+      </c>
+      <c r="B38" s="7">
+        <v>10305</v>
+      </c>
       <c r="C38" s="7">
-        <v>10816</v>
-      </c>
-      <c r="D38" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>10328</v>
+      </c>
+      <c r="D38" s="3">
+        <f t="shared" ref="D38" si="2">IF(C38&lt;&gt;"",IF(B38&lt;&gt;"",C38-B38,"-"), "-")</f>
+        <v>23</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A39" s="50" t="s">
-        <v>402</v>
-      </c>
-      <c r="B39" s="7"/>
+      <c r="A39" s="59" t="s">
+        <v>426</v>
+      </c>
+      <c r="B39" s="7">
+        <v>10532</v>
+      </c>
       <c r="C39" s="7">
-        <v>11163</v>
-      </c>
-      <c r="D39" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>10557</v>
+      </c>
+      <c r="D39" s="3">
+        <f t="shared" si="1"/>
+        <v>25</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A40" s="50" t="s">
-        <v>283</v>
-      </c>
-      <c r="B40" s="7"/>
+      <c r="A40" s="59" t="s">
+        <v>425</v>
+      </c>
+      <c r="B40" s="7">
+        <v>10574</v>
+      </c>
       <c r="C40" s="7">
-        <v>11729</v>
-      </c>
-      <c r="D40" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>10589</v>
+      </c>
+      <c r="D40" s="3">
+        <f t="shared" si="1"/>
+        <v>15</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A41" s="50" t="s">
+        <v>281</v>
+      </c>
+      <c r="B41" s="7">
+        <v>10743</v>
+      </c>
+      <c r="C41" s="7">
+        <v>10816</v>
+      </c>
+      <c r="D41" s="3">
+        <f t="shared" si="1"/>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A42" s="50" t="s">
+        <v>402</v>
+      </c>
+      <c r="B42" s="7">
+        <v>11094</v>
+      </c>
+      <c r="C42" s="7">
+        <v>11163</v>
+      </c>
+      <c r="D42" s="3">
+        <f t="shared" si="1"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A43" s="50" t="s">
+        <v>283</v>
+      </c>
+      <c r="B43" s="7">
+        <v>11652</v>
+      </c>
+      <c r="C43" s="7">
+        <v>11729</v>
+      </c>
+      <c r="D43" s="3">
+        <f t="shared" si="1"/>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A44" s="50" t="s">
         <v>403</v>
-      </c>
-      <c r="B41" s="7"/>
-      <c r="C41" s="7">
-        <v>12383</v>
-      </c>
-      <c r="D41" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="E41" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="50" t="s">
-        <v>285</v>
-      </c>
-      <c r="B42" s="7"/>
-      <c r="C42" s="7">
-        <v>12891</v>
-      </c>
-      <c r="D42" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="50" t="s">
-        <v>404</v>
-      </c>
-      <c r="B43" s="7"/>
-      <c r="C43" s="7">
-        <v>13269</v>
-      </c>
-      <c r="D43" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="50" t="s">
-        <v>288</v>
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="7">
-        <v>13960</v>
+        <v>12383</v>
       </c>
       <c r="D44" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
+      </c>
+      <c r="E44" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="50" t="s">
-        <v>405</v>
+        <v>285</v>
       </c>
       <c r="B45" s="7"/>
       <c r="C45" s="7">
-        <v>14320</v>
+        <v>12891</v>
       </c>
       <c r="D45" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="50" t="s">
-        <v>294</v>
+        <v>404</v>
       </c>
       <c r="B46" s="7"/>
       <c r="C46" s="7">
-        <v>14679</v>
+        <v>13269</v>
       </c>
       <c r="D46" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="50" t="s">
-        <v>406</v>
+        <v>288</v>
       </c>
       <c r="B47" s="7"/>
       <c r="C47" s="7">
-        <v>15029</v>
+        <v>13960</v>
       </c>
       <c r="D47" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="50" t="s">
-        <v>297</v>
+        <v>405</v>
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="7">
-        <v>15850</v>
+        <v>14320</v>
       </c>
       <c r="D48" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2913,11 +2939,11 @@
     </row>
     <row r="49" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="50" t="s">
-        <v>407</v>
+        <v>294</v>
       </c>
       <c r="B49" s="7"/>
       <c r="C49" s="7">
-        <v>16200</v>
+        <v>14679</v>
       </c>
       <c r="D49" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2926,11 +2952,11 @@
     </row>
     <row r="50" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="50" t="s">
-        <v>301</v>
-      </c>
-      <c r="B50" s="33"/>
-      <c r="C50" s="33">
-        <v>17135</v>
+        <v>406</v>
+      </c>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7">
+        <v>15029</v>
       </c>
       <c r="D50" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2939,11 +2965,11 @@
     </row>
     <row r="51" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="50" t="s">
-        <v>408</v>
+        <v>297</v>
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="7">
-        <v>17485</v>
+        <v>15850</v>
       </c>
       <c r="D51" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2952,11 +2978,11 @@
     </row>
     <row r="52" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A52" s="50" t="s">
-        <v>305</v>
+        <v>407</v>
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="7">
-        <v>17791</v>
+        <v>16200</v>
       </c>
       <c r="D52" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2965,11 +2991,11 @@
     </row>
     <row r="53" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A53" s="50" t="s">
-        <v>409</v>
-      </c>
-      <c r="B53" s="7"/>
-      <c r="C53" s="37">
-        <v>18139</v>
+        <v>301</v>
+      </c>
+      <c r="B53" s="33"/>
+      <c r="C53" s="33">
+        <v>17135</v>
       </c>
       <c r="D53" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2978,11 +3004,11 @@
     </row>
     <row r="54" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="50" t="s">
-        <v>308</v>
+        <v>408</v>
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="7">
-        <v>18719</v>
+        <v>17485</v>
       </c>
       <c r="D54" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2991,11 +3017,11 @@
     </row>
     <row r="55" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="50" t="s">
-        <v>411</v>
+        <v>305</v>
       </c>
       <c r="B55" s="7"/>
       <c r="C55" s="7">
-        <v>19068</v>
+        <v>17791</v>
       </c>
       <c r="D55" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3004,11 +3030,11 @@
     </row>
     <row r="56" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A56" s="50" t="s">
-        <v>314</v>
+        <v>409</v>
       </c>
       <c r="B56" s="7"/>
-      <c r="C56" s="7">
-        <v>19892</v>
+      <c r="C56" s="37">
+        <v>18139</v>
       </c>
       <c r="D56" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3017,11 +3043,11 @@
     </row>
     <row r="57" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A57" s="50" t="s">
-        <v>412</v>
+        <v>308</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7">
-        <v>20240</v>
+        <v>18719</v>
       </c>
       <c r="D57" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3030,39 +3056,37 @@
     </row>
     <row r="58" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
-        <v>320</v>
+        <v>411</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7">
-        <v>20813</v>
+        <v>19068</v>
       </c>
       <c r="D58" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-      <c r="E58" s="7"/>
     </row>
     <row r="59" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>413</v>
+        <v>314</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7">
-        <v>21161</v>
+        <v>19892</v>
       </c>
       <c r="D59" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-      <c r="E59" s="7"/>
     </row>
     <row r="60" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>322</v>
+        <v>412</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7">
-        <v>22195</v>
+        <v>20240</v>
       </c>
       <c r="D60" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3071,37 +3095,39 @@
     </row>
     <row r="61" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>414</v>
+        <v>320</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7">
-        <v>22543</v>
+        <v>20813</v>
       </c>
       <c r="D61" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
+      <c r="E61" s="7"/>
     </row>
     <row r="62" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>324</v>
+        <v>413</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7">
-        <v>22963</v>
+        <v>21161</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
+      <c r="E62" s="7"/>
     </row>
     <row r="63" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>415</v>
+        <v>322</v>
       </c>
       <c r="B63" s="7"/>
       <c r="C63" s="7">
-        <v>23346</v>
+        <v>22195</v>
       </c>
       <c r="D63" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3110,433 +3136,433 @@
     </row>
     <row r="64" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7">
-        <v>23873</v>
+        <v>22543</v>
       </c>
       <c r="D64" s="3" t="str">
-        <f t="shared" ref="D64:D95" si="2">IF(C64&lt;&gt;"",IF(B64&lt;&gt;"",C64-B64,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>417</v>
-      </c>
-      <c r="B65" s="8"/>
-      <c r="C65" s="50">
-        <v>24221</v>
+        <v>324</v>
+      </c>
+      <c r="B65" s="7"/>
+      <c r="C65" s="7">
+        <v>22963</v>
       </c>
       <c r="D65" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>418</v>
-      </c>
-      <c r="B66" s="33"/>
-      <c r="C66" s="33">
-        <v>25101</v>
+        <v>415</v>
+      </c>
+      <c r="B66" s="7"/>
+      <c r="C66" s="7">
+        <v>23346</v>
       </c>
       <c r="D66" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>25450</v>
+        <v>23873</v>
       </c>
       <c r="D67" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="D67:D98" si="3">IF(C67&lt;&gt;"",IF(B67&lt;&gt;"",C67-B67,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>420</v>
-      </c>
-      <c r="B68" s="7"/>
-      <c r="C68" s="7">
-        <v>26350</v>
+        <v>417</v>
+      </c>
+      <c r="B68" s="8"/>
+      <c r="C68" s="50">
+        <v>24221</v>
       </c>
       <c r="D68" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>421</v>
-      </c>
-      <c r="B69" s="7"/>
-      <c r="C69" s="7">
-        <v>26699</v>
+        <v>418</v>
+      </c>
+      <c r="B69" s="33"/>
+      <c r="C69" s="33">
+        <v>25101</v>
       </c>
       <c r="D69" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>332</v>
+        <v>419</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>27490</v>
+        <v>25450</v>
       </c>
       <c r="D70" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>5</v>
+        <v>420</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>27836</v>
+        <v>26350</v>
       </c>
       <c r="D71" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>337</v>
+        <v>421</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>28899</v>
+        <v>26699</v>
       </c>
       <c r="D72" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>6</v>
+        <v>332</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>29248</v>
+        <v>27490</v>
       </c>
       <c r="D73" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>29962</v>
+        <v>27836</v>
       </c>
       <c r="D74" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>7</v>
+        <v>337</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>30309</v>
+        <v>28899</v>
       </c>
       <c r="D75" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>46</v>
+        <v>6</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>30479</v>
+        <v>29248</v>
       </c>
       <c r="D76" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>31125</v>
+        <v>29962</v>
       </c>
       <c r="D77" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-      <c r="E77" t="s">
-        <v>422</v>
+        <f t="shared" si="3"/>
+        <v>-</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>31643</v>
+        <v>30309</v>
       </c>
       <c r="D78" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>31991</v>
+        <v>30479</v>
       </c>
       <c r="D79" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>32586</v>
+        <v>31125</v>
       </c>
       <c r="D80" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+      <c r="E80" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="81" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>33254</v>
+        <v>31643</v>
       </c>
       <c r="D81" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-      <c r="E81" t="s">
-        <v>422</v>
+        <f t="shared" si="3"/>
+        <v>-</v>
       </c>
     </row>
     <row r="82" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>33883</v>
+        <v>31991</v>
       </c>
       <c r="D82" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="83" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B83" s="7"/>
       <c r="C83" s="7">
-        <v>34244</v>
+        <v>32586</v>
       </c>
       <c r="D83" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B84" s="7"/>
       <c r="C84" s="7">
-        <v>34862</v>
+        <v>33254</v>
       </c>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+      <c r="E84" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="85" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>35218</v>
+        <v>33883</v>
       </c>
       <c r="D85" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="86" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="B86" s="7"/>
       <c r="C86" s="7">
-        <v>35772</v>
+        <v>34244</v>
       </c>
       <c r="D86" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="87" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>36120</v>
+        <v>34862</v>
       </c>
       <c r="D87" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>36893</v>
+        <v>35218</v>
       </c>
       <c r="D88" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="89" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>37238</v>
+        <v>35772</v>
       </c>
       <c r="D89" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="90" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>38097</v>
+        <v>36120</v>
       </c>
       <c r="D90" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>38443</v>
+        <v>36893</v>
       </c>
       <c r="D91" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="92" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>38692</v>
+        <v>37238</v>
       </c>
       <c r="D92" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="93" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>39041</v>
+        <v>38097</v>
       </c>
       <c r="D93" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="94" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>40011</v>
+        <v>38443</v>
       </c>
       <c r="D94" s="3" t="str">
-        <f>IF(C93&lt;&gt;"",IF(B93&lt;&gt;"",C93-B93,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="95" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>40373</v>
+        <v>38692</v>
       </c>
       <c r="D95" s="3" t="str">
-        <f t="shared" ref="D95:D114" si="3">IF(C95&lt;&gt;"",IF(B95&lt;&gt;"",C95-B95,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="96" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B96" s="40"/>
+        <v>15</v>
+      </c>
+      <c r="B96" s="7"/>
       <c r="C96" s="7">
-        <v>41117</v>
+        <v>39041</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3545,252 +3571,279 @@
     </row>
     <row r="97" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>41465</v>
+        <v>40011</v>
       </c>
       <c r="D97" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(C96&lt;&gt;"",IF(B96&lt;&gt;"",C96-B96,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="98" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>42450</v>
+        <v>40373</v>
       </c>
       <c r="D98" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="D98:D117" si="4">IF(C98&lt;&gt;"",IF(B98&lt;&gt;"",C98-B98,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="99" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>18</v>
-      </c>
-      <c r="B99" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B99" s="40"/>
       <c r="C99" s="7">
-        <v>42799</v>
+        <v>41117</v>
       </c>
       <c r="D99" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="100" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>43144</v>
+        <v>41465</v>
       </c>
       <c r="D100" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="101" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>43491</v>
+        <v>42450</v>
       </c>
       <c r="D101" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="102" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A102" s="50" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="B102" s="7"/>
       <c r="C102" s="7">
-        <v>44165</v>
+        <v>42799</v>
       </c>
       <c r="D102" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="103" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A103" s="50" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="B103" s="7"/>
       <c r="C103" s="7">
-        <v>44512</v>
+        <v>43144</v>
       </c>
       <c r="D103" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="104" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A104" s="50" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="B104" s="7"/>
       <c r="C104" s="7">
-        <v>45061</v>
+        <v>43491</v>
       </c>
       <c r="D104" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="105" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A105" s="50" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="B105" s="7"/>
       <c r="C105" s="7">
-        <v>45443</v>
+        <v>44165</v>
       </c>
       <c r="D105" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="106" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A106" s="50" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="B106" s="7"/>
       <c r="C106" s="7">
-        <v>45990</v>
+        <v>44512</v>
       </c>
       <c r="D106" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="107" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A107" s="50" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="B107" s="7"/>
       <c r="C107" s="7">
-        <v>46652</v>
+        <v>45061</v>
       </c>
       <c r="D107" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-      <c r="E107" t="s">
-        <v>422</v>
+        <f t="shared" si="4"/>
+        <v>-</v>
       </c>
     </row>
     <row r="108" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A108" s="50" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="B108" s="7"/>
       <c r="C108" s="7">
-        <v>47436</v>
+        <v>45443</v>
       </c>
       <c r="D108" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="109" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A109" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B109" s="9"/>
-      <c r="C109" s="9">
-        <v>48337</v>
+        <v>41</v>
+      </c>
+      <c r="B109" s="7"/>
+      <c r="C109" s="7">
+        <v>45990</v>
       </c>
       <c r="D109" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="110" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A110" s="50" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="B110" s="7"/>
       <c r="C110" s="7">
-        <v>49334</v>
+        <v>46652</v>
       </c>
       <c r="D110" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
+        <f t="shared" si="4"/>
+        <v>-</v>
+      </c>
+      <c r="E110" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="111" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A111" s="50" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="B111" s="7"/>
       <c r="C111" s="7">
-        <v>48681</v>
+        <v>47436</v>
       </c>
       <c r="D111" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="112" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A112" s="50" t="s">
-        <v>44</v>
-      </c>
-      <c r="B112" s="7"/>
-      <c r="C112" s="7">
-        <v>49334</v>
+        <v>23</v>
+      </c>
+      <c r="B112" s="9"/>
+      <c r="C112" s="9">
+        <v>48337</v>
       </c>
       <c r="D112" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="113" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A113" s="50" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="B113" s="7"/>
       <c r="C113" s="7">
-        <v>49683</v>
+        <v>49334</v>
       </c>
       <c r="D113" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-</v>
       </c>
     </row>
     <row r="114" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A114" s="50" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B114" s="7"/>
       <c r="C114" s="7">
+        <v>48681</v>
+      </c>
+      <c r="D114" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A115" s="50" t="s">
+        <v>44</v>
+      </c>
+      <c r="B115" s="7"/>
+      <c r="C115" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D115" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A116" s="50" t="s">
+        <v>25</v>
+      </c>
+      <c r="B116" s="7"/>
+      <c r="C116" s="7">
+        <v>49683</v>
+      </c>
+      <c r="D116" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A117" s="50" t="s">
+        <v>26</v>
+      </c>
+      <c r="B117" s="7"/>
+      <c r="C117" s="7">
         <v>50244</v>
       </c>
-      <c r="D114" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B115" s="7"/>
-      <c r="C115" s="7"/>
-    </row>
-    <row r="116" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B116" s="7"/>
-      <c r="C116" s="7"/>
-    </row>
-    <row r="117" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B117" s="7"/>
-      <c r="C117" s="7"/>
+      <c r="D117" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="118" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="B118" s="7"/>
@@ -4111,6 +4164,18 @@
     <row r="197" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B197" s="7"/>
       <c r="C197" s="7"/>
+    </row>
+    <row r="198" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B198" s="7"/>
+      <c r="C198" s="7"/>
+    </row>
+    <row r="199" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B199" s="7"/>
+      <c r="C199" s="7"/>
+    </row>
+    <row r="200" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B200" s="7"/>
+      <c r="C200" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18959,7 +19024,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="31" type="noConversion"/>
+  <phoneticPr fontId="32" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>

</xml_diff>

<commit_message>
14 done, 76 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E84BC021-0226-406A-9380-7D6F5B28F03C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79ADBF79-E002-41D6-9591-B55CBEB442E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2873,13 +2873,15 @@
       <c r="A44" s="50" t="s">
         <v>403</v>
       </c>
-      <c r="B44" s="7"/>
+      <c r="B44" s="7">
+        <v>12308</v>
+      </c>
       <c r="C44" s="7">
         <v>12383</v>
       </c>
-      <c r="D44" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="D44" s="3">
+        <f t="shared" si="1"/>
+        <v>75</v>
       </c>
       <c r="E44" t="s">
         <v>422</v>
@@ -2889,13 +2891,15 @@
       <c r="A45" s="50" t="s">
         <v>285</v>
       </c>
-      <c r="B45" s="7"/>
+      <c r="B45" s="7">
+        <v>12815</v>
+      </c>
       <c r="C45" s="7">
         <v>12891</v>
       </c>
-      <c r="D45" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="D45" s="3">
+        <f t="shared" si="1"/>
+        <v>76</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 14 done at a slower speed with select skip, only saves a few frames
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79ADBF79-E002-41D6-9591-B55CBEB442E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B7B7D79-810A-46A1-B28C-2995B2730AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1891,6 +1891,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1915,7 +1916,6 @@
     <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2780,7 +2780,7 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A38" s="59" t="s">
+      <c r="A38" s="51" t="s">
         <v>127</v>
       </c>
       <c r="B38" s="7">
@@ -2795,7 +2795,7 @@
       </c>
     </row>
     <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A39" s="59" t="s">
+      <c r="A39" s="51" t="s">
         <v>426</v>
       </c>
       <c r="B39" s="7">
@@ -2810,7 +2810,7 @@
       </c>
     </row>
     <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A40" s="59" t="s">
+      <c r="A40" s="51" t="s">
         <v>425</v>
       </c>
       <c r="B40" s="7">
@@ -2892,27 +2892,32 @@
         <v>285</v>
       </c>
       <c r="B45" s="7">
-        <v>12815</v>
+        <v>12806</v>
       </c>
       <c r="C45" s="7">
         <v>12891</v>
       </c>
       <c r="D45" s="3">
         <f t="shared" si="1"/>
-        <v>76</v>
+        <v>85</v>
+      </c>
+      <c r="E45" s="7">
+        <v>12815</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="50" t="s">
         <v>404</v>
       </c>
-      <c r="B46" s="7"/>
+      <c r="B46" s="7">
+        <v>13160</v>
+      </c>
       <c r="C46" s="7">
-        <v>13269</v>
-      </c>
-      <c r="D46" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>13236</v>
+      </c>
+      <c r="D46" s="3">
+        <f t="shared" si="1"/>
+        <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3186,7 +3191,7 @@
         <v>23873</v>
       </c>
       <c r="D67" s="3" t="str">
-        <f t="shared" ref="D67:D98" si="3">IF(C67&lt;&gt;"",IF(B67&lt;&gt;"",C67-B67,"-"), "-")</f>
+        <f t="shared" ref="D67:D96" si="3">IF(C67&lt;&gt;"",IF(B67&lt;&gt;"",C67-B67,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
@@ -19058,10 +19063,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="51" t="s">
+      <c r="K1" s="52" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="52"/>
+      <c r="L1" s="53"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -20913,13 +20918,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="53" t="s">
+      <c r="H53" s="54" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="54"/>
-      <c r="J53" s="54"/>
-      <c r="K53" s="54"/>
-      <c r="L53" s="55"/>
+      <c r="I53" s="55"/>
+      <c r="J53" s="55"/>
+      <c r="K53" s="55"/>
+      <c r="L53" s="56"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -20941,11 +20946,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="56"/>
-      <c r="I54" s="57"/>
-      <c r="J54" s="57"/>
-      <c r="K54" s="57"/>
-      <c r="L54" s="58"/>
+      <c r="H54" s="57"/>
+      <c r="I54" s="58"/>
+      <c r="J54" s="58"/>
+      <c r="K54" s="58"/>
+      <c r="L54" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - lv 14 done at speed 4, 116 ahead at start of lv 15
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B7B7D79-810A-46A1-B28C-2995B2730AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3EBC64E-3EBD-4892-B650-5191C72A703E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="428">
   <si>
     <t>Place</t>
   </si>
@@ -1317,6 +1317,9 @@
   </si>
   <si>
     <t>land</t>
+  </si>
+  <si>
+    <t>13162 fast mode</t>
   </si>
 </sst>
 </file>
@@ -2892,14 +2895,14 @@
         <v>285</v>
       </c>
       <c r="B45" s="7">
-        <v>12806</v>
+        <v>12768</v>
       </c>
       <c r="C45" s="7">
         <v>12891</v>
       </c>
       <c r="D45" s="3">
         <f t="shared" si="1"/>
-        <v>85</v>
+        <v>123</v>
       </c>
       <c r="E45" s="7">
         <v>12815</v>
@@ -2910,14 +2913,17 @@
         <v>404</v>
       </c>
       <c r="B46" s="7">
-        <v>13160</v>
+        <v>13120</v>
       </c>
       <c r="C46" s="7">
         <v>13236</v>
       </c>
       <c r="D46" s="3">
         <f t="shared" si="1"/>
-        <v>76</v>
+        <v>116</v>
+      </c>
+      <c r="E46" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - restart using neshawk, 1 frame saved on start up timing difference, possibly 2 more frames saved but probably not
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3EBC64E-3EBD-4892-B650-5191C72A703E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{484D956D-77AC-4121-A690-7BA0588A75D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="V7" sheetId="8" r:id="rId1"/>
-    <sheet name="V6" sheetId="7" r:id="rId2"/>
-    <sheet name="V5" sheetId="5" r:id="rId3"/>
-    <sheet name="V4" sheetId="4" r:id="rId4"/>
-    <sheet name="V3" sheetId="3" r:id="rId5"/>
-    <sheet name="V2" sheetId="1" r:id="rId6"/>
-    <sheet name="Takanawa Comparison" sheetId="6" r:id="rId7"/>
+    <sheet name="V7.1" sheetId="9" r:id="rId1"/>
+    <sheet name="V7" sheetId="8" r:id="rId2"/>
+    <sheet name="V6" sheetId="7" r:id="rId3"/>
+    <sheet name="V5" sheetId="5" r:id="rId4"/>
+    <sheet name="V4" sheetId="4" r:id="rId5"/>
+    <sheet name="V3" sheetId="3" r:id="rId6"/>
+    <sheet name="V2" sheetId="1" r:id="rId7"/>
+    <sheet name="Takanawa Comparison" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="430">
   <si>
     <t>Place</t>
   </si>
@@ -1320,6 +1321,12 @@
   </si>
   <si>
     <t>13162 fast mode</t>
+  </si>
+  <si>
+    <t>12815 fast mode</t>
+  </si>
+  <si>
+    <t>v7.1</t>
   </si>
 </sst>
 </file>
@@ -1329,12 +1336,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1787,95 +1801,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="28" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1894,31 +1909,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2238,6 +2253,945 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8465CAE6-FA0E-4F56-807B-2D9877AC152D}">
+  <dimension ref="A1:E129"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="8.75" customWidth="1"/>
+    <col min="4" max="4" width="6.625" customWidth="1"/>
+    <col min="5" max="5" width="17.625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A2" s="50" t="s">
+        <v>389</v>
+      </c>
+      <c r="B2" s="2">
+        <v>427</v>
+      </c>
+      <c r="C2" s="2">
+        <v>428</v>
+      </c>
+      <c r="D2" s="3">
+        <f t="shared" ref="D2:D46" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A3" s="50" t="s">
+        <v>392</v>
+      </c>
+      <c r="B3" s="2">
+        <v>737</v>
+      </c>
+      <c r="C3" s="2">
+        <v>739</v>
+      </c>
+      <c r="D3" s="3">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A4" s="50" t="s">
+        <v>391</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1088</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1089</v>
+      </c>
+      <c r="D4" s="3">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A5" s="50" t="s">
+        <v>390</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1573</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1574</v>
+      </c>
+      <c r="D5" s="3">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A6" s="50" t="s">
+        <v>393</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1920</v>
+      </c>
+      <c r="C6" s="2">
+        <v>1923</v>
+      </c>
+      <c r="D6" s="3">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A7" s="50"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A8" s="50"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A9" s="50"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A10" s="50" t="s">
+        <v>251</v>
+      </c>
+      <c r="B10" s="2">
+        <v>2333</v>
+      </c>
+      <c r="C10" s="2">
+        <v>2334</v>
+      </c>
+      <c r="D10" s="3">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A11" s="50" t="s">
+        <v>394</v>
+      </c>
+      <c r="B11" s="7">
+        <v>2680</v>
+      </c>
+      <c r="C11" s="7">
+        <v>2683</v>
+      </c>
+      <c r="D11" s="3">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A12" s="50" t="s">
+        <v>253</v>
+      </c>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7">
+        <v>3132</v>
+      </c>
+      <c r="D12" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A13" s="50" t="s">
+        <v>395</v>
+      </c>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7">
+        <v>3479</v>
+      </c>
+      <c r="D13" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A14" s="50"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7">
+        <v>3548</v>
+      </c>
+      <c r="D14" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A15" s="50"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7">
+        <v>3640</v>
+      </c>
+      <c r="D15" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A16" s="50" t="s">
+        <v>255</v>
+      </c>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7">
+        <v>3761</v>
+      </c>
+      <c r="D16" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A17" s="50" t="s">
+        <v>396</v>
+      </c>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7">
+        <v>4109</v>
+      </c>
+      <c r="D17" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A18" s="50"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7">
+        <v>4509</v>
+      </c>
+      <c r="D18" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A19" s="50"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7">
+        <v>4669</v>
+      </c>
+      <c r="D19" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A20" s="50"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7">
+        <v>4727</v>
+      </c>
+      <c r="D20" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A21" s="50"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7">
+        <v>4866</v>
+      </c>
+      <c r="D21" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A22" s="50"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7">
+        <v>4953</v>
+      </c>
+      <c r="D22" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A23" s="50" t="s">
+        <v>257</v>
+      </c>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7">
+        <v>5125</v>
+      </c>
+      <c r="D23" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A24" s="50" t="s">
+        <v>397</v>
+      </c>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7">
+        <v>5474</v>
+      </c>
+      <c r="D24" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A25" s="50" t="s">
+        <v>259</v>
+      </c>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7">
+        <v>5936</v>
+      </c>
+      <c r="D25" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A26" s="50" t="s">
+        <v>410</v>
+      </c>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7">
+        <v>6287</v>
+      </c>
+      <c r="D26" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A27" s="50"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7">
+        <v>6410</v>
+      </c>
+      <c r="D27" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A28" s="50"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7">
+        <v>6446</v>
+      </c>
+      <c r="D28" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A29" s="50"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7">
+        <v>6590</v>
+      </c>
+      <c r="D29" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A30" s="50" t="s">
+        <v>267</v>
+      </c>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7">
+        <v>6690</v>
+      </c>
+      <c r="D30" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A31" s="50" t="s">
+        <v>398</v>
+      </c>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7">
+        <v>7039</v>
+      </c>
+      <c r="D31" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A32" s="50" t="s">
+        <v>274</v>
+      </c>
+      <c r="B32" s="7"/>
+      <c r="C32" s="7">
+        <v>8127</v>
+      </c>
+      <c r="D32" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A33" s="50" t="s">
+        <v>399</v>
+      </c>
+      <c r="B33" s="7"/>
+      <c r="C33" s="7">
+        <v>8527</v>
+      </c>
+      <c r="D33" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A34" s="50" t="s">
+        <v>276</v>
+      </c>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7">
+        <v>9099</v>
+      </c>
+      <c r="D34" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A35" s="50" t="s">
+        <v>400</v>
+      </c>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7">
+        <v>9447</v>
+      </c>
+      <c r="D35" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A36" s="50" t="s">
+        <v>278</v>
+      </c>
+      <c r="B36" s="7"/>
+      <c r="C36" s="7">
+        <v>9758</v>
+      </c>
+      <c r="D36" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A37" s="50" t="s">
+        <v>401</v>
+      </c>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7">
+        <v>10104</v>
+      </c>
+      <c r="D37" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A38" s="51" t="s">
+        <v>127</v>
+      </c>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7">
+        <v>10305</v>
+      </c>
+      <c r="D38" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A39" s="51" t="s">
+        <v>426</v>
+      </c>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7">
+        <v>10532</v>
+      </c>
+      <c r="D39" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A40" s="51" t="s">
+        <v>425</v>
+      </c>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7">
+        <v>10574</v>
+      </c>
+      <c r="D40" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A41" s="50" t="s">
+        <v>281</v>
+      </c>
+      <c r="B41" s="7"/>
+      <c r="C41" s="7">
+        <v>10743</v>
+      </c>
+      <c r="D41" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A42" s="50" t="s">
+        <v>402</v>
+      </c>
+      <c r="B42" s="7"/>
+      <c r="C42" s="7">
+        <v>11094</v>
+      </c>
+      <c r="D42" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A43" s="50" t="s">
+        <v>283</v>
+      </c>
+      <c r="B43" s="7"/>
+      <c r="C43" s="7">
+        <v>11652</v>
+      </c>
+      <c r="D43" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A44" s="50" t="s">
+        <v>403</v>
+      </c>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7">
+        <v>12308</v>
+      </c>
+      <c r="D44" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="50" t="s">
+        <v>285</v>
+      </c>
+      <c r="B45" s="7"/>
+      <c r="C45" s="7">
+        <v>12768</v>
+      </c>
+      <c r="D45" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E45" s="60" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="50" t="s">
+        <v>404</v>
+      </c>
+      <c r="B46" s="7"/>
+      <c r="C46" s="7">
+        <v>13120</v>
+      </c>
+      <c r="D46" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E46" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="B47" s="7"/>
+      <c r="C47" s="7"/>
+    </row>
+    <row r="48" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="B48" s="7"/>
+      <c r="C48" s="7"/>
+    </row>
+    <row r="49" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B49" s="7"/>
+      <c r="C49" s="7"/>
+    </row>
+    <row r="50" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B50" s="7"/>
+      <c r="C50" s="7"/>
+    </row>
+    <row r="51" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B51" s="7"/>
+      <c r="C51" s="7"/>
+    </row>
+    <row r="52" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B52" s="7"/>
+      <c r="C52" s="7"/>
+    </row>
+    <row r="53" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+    </row>
+    <row r="54" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B54" s="7"/>
+      <c r="C54" s="7"/>
+    </row>
+    <row r="55" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B55" s="7"/>
+      <c r="C55" s="7"/>
+    </row>
+    <row r="56" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B56" s="7"/>
+      <c r="C56" s="7"/>
+    </row>
+    <row r="57" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B57" s="7"/>
+      <c r="C57" s="7"/>
+    </row>
+    <row r="58" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B58" s="7"/>
+      <c r="C58" s="7"/>
+    </row>
+    <row r="59" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B59" s="7"/>
+      <c r="C59" s="7"/>
+    </row>
+    <row r="60" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B60" s="7"/>
+      <c r="C60" s="7"/>
+    </row>
+    <row r="61" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B61" s="7"/>
+      <c r="C61" s="7"/>
+    </row>
+    <row r="62" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B62" s="7"/>
+      <c r="C62" s="7"/>
+    </row>
+    <row r="63" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B63" s="7"/>
+      <c r="C63" s="7"/>
+    </row>
+    <row r="64" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B64" s="7"/>
+      <c r="C64" s="7"/>
+    </row>
+    <row r="65" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B65" s="7"/>
+      <c r="C65" s="7"/>
+    </row>
+    <row r="66" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B66" s="7"/>
+      <c r="C66" s="7"/>
+    </row>
+    <row r="67" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B67" s="7"/>
+      <c r="C67" s="7"/>
+    </row>
+    <row r="68" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B68" s="7"/>
+      <c r="C68" s="7"/>
+    </row>
+    <row r="69" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B69" s="7"/>
+      <c r="C69" s="7"/>
+    </row>
+    <row r="70" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B70" s="7"/>
+      <c r="C70" s="7"/>
+    </row>
+    <row r="71" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B71" s="7"/>
+      <c r="C71" s="7"/>
+    </row>
+    <row r="72" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B72" s="7"/>
+      <c r="C72" s="7"/>
+    </row>
+    <row r="73" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B73" s="7"/>
+      <c r="C73" s="7"/>
+    </row>
+    <row r="74" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B74" s="7"/>
+      <c r="C74" s="7"/>
+    </row>
+    <row r="75" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B75" s="7"/>
+      <c r="C75" s="7"/>
+    </row>
+    <row r="76" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B76" s="7"/>
+      <c r="C76" s="7"/>
+    </row>
+    <row r="77" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B77" s="7"/>
+      <c r="C77" s="7"/>
+    </row>
+    <row r="78" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B78" s="7"/>
+      <c r="C78" s="7"/>
+    </row>
+    <row r="79" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B79" s="7"/>
+      <c r="C79" s="7"/>
+    </row>
+    <row r="80" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B80" s="7"/>
+      <c r="C80" s="7"/>
+    </row>
+    <row r="81" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B81" s="7"/>
+      <c r="C81" s="7"/>
+    </row>
+    <row r="82" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B82" s="7"/>
+      <c r="C82" s="7"/>
+    </row>
+    <row r="83" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B83" s="7"/>
+      <c r="C83" s="7"/>
+    </row>
+    <row r="84" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B84" s="7"/>
+      <c r="C84" s="7"/>
+    </row>
+    <row r="85" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B85" s="7"/>
+      <c r="C85" s="7"/>
+    </row>
+    <row r="86" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B86" s="7"/>
+      <c r="C86" s="7"/>
+    </row>
+    <row r="87" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B87" s="7"/>
+      <c r="C87" s="7"/>
+    </row>
+    <row r="88" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B88" s="7"/>
+      <c r="C88" s="7"/>
+    </row>
+    <row r="89" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B89" s="7"/>
+      <c r="C89" s="7"/>
+    </row>
+    <row r="90" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B90" s="7"/>
+      <c r="C90" s="7"/>
+    </row>
+    <row r="91" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B91" s="7"/>
+      <c r="C91" s="7"/>
+    </row>
+    <row r="92" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B92" s="7"/>
+      <c r="C92" s="7"/>
+    </row>
+    <row r="93" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B93" s="7"/>
+      <c r="C93" s="7"/>
+    </row>
+    <row r="94" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B94" s="7"/>
+      <c r="C94" s="7"/>
+    </row>
+    <row r="95" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B95" s="7"/>
+      <c r="C95" s="7"/>
+    </row>
+    <row r="96" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B96" s="7"/>
+      <c r="C96" s="7"/>
+    </row>
+    <row r="97" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B97" s="7"/>
+      <c r="C97" s="7"/>
+    </row>
+    <row r="98" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B98" s="7"/>
+      <c r="C98" s="7"/>
+    </row>
+    <row r="99" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B99" s="7"/>
+      <c r="C99" s="7"/>
+    </row>
+    <row r="100" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B100" s="7"/>
+      <c r="C100" s="7"/>
+    </row>
+    <row r="101" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B101" s="7"/>
+      <c r="C101" s="7"/>
+    </row>
+    <row r="102" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B102" s="7"/>
+      <c r="C102" s="7"/>
+    </row>
+    <row r="103" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B103" s="7"/>
+      <c r="C103" s="7"/>
+    </row>
+    <row r="104" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B104" s="7"/>
+      <c r="C104" s="7"/>
+    </row>
+    <row r="105" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B105" s="7"/>
+      <c r="C105" s="7"/>
+    </row>
+    <row r="106" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B106" s="7"/>
+      <c r="C106" s="7"/>
+    </row>
+    <row r="107" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B107" s="7"/>
+      <c r="C107" s="7"/>
+    </row>
+    <row r="108" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B108" s="7"/>
+      <c r="C108" s="7"/>
+    </row>
+    <row r="109" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B109" s="7"/>
+      <c r="C109" s="7"/>
+    </row>
+    <row r="110" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B110" s="7"/>
+      <c r="C110" s="7"/>
+    </row>
+    <row r="111" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B111" s="7"/>
+      <c r="C111" s="7"/>
+    </row>
+    <row r="112" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B112" s="7"/>
+      <c r="C112" s="7"/>
+    </row>
+    <row r="113" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B113" s="7"/>
+      <c r="C113" s="7"/>
+    </row>
+    <row r="114" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B114" s="7"/>
+      <c r="C114" s="7"/>
+    </row>
+    <row r="115" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B115" s="7"/>
+      <c r="C115" s="7"/>
+    </row>
+    <row r="116" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B116" s="7"/>
+      <c r="C116" s="7"/>
+    </row>
+    <row r="117" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B117" s="7"/>
+      <c r="C117" s="7"/>
+    </row>
+    <row r="118" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B118" s="7"/>
+      <c r="C118" s="7"/>
+    </row>
+    <row r="119" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B119" s="7"/>
+      <c r="C119" s="7"/>
+    </row>
+    <row r="120" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B120" s="7"/>
+      <c r="C120" s="7"/>
+    </row>
+    <row r="121" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B121" s="7"/>
+      <c r="C121" s="7"/>
+    </row>
+    <row r="122" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B122" s="7"/>
+      <c r="C122" s="7"/>
+    </row>
+    <row r="123" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B123" s="7"/>
+      <c r="C123" s="7"/>
+    </row>
+    <row r="124" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B124" s="7"/>
+      <c r="C124" s="7"/>
+    </row>
+    <row r="125" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B125" s="7"/>
+      <c r="C125" s="7"/>
+    </row>
+    <row r="126" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B126" s="7"/>
+      <c r="C126" s="7"/>
+    </row>
+    <row r="127" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B127" s="7"/>
+      <c r="C127" s="7"/>
+    </row>
+    <row r="128" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B128" s="7"/>
+      <c r="C128" s="7"/>
+    </row>
+    <row r="129" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B129" s="7"/>
+      <c r="C129" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
   <dimension ref="A1:E200"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -4198,7 +5152,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
   <dimension ref="A1:E388"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -9053,7 +10007,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39B3565E-C480-4A10-8524-B7BC06C9B703}">
   <dimension ref="A1:H287"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -13009,7 +13963,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D06DA051-0308-42D5-B7F7-51E79FAF1C31}">
   <dimension ref="A1:F292"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -15552,7 +16506,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B2A8891-531F-43A4-B044-6C02F070C564}">
   <dimension ref="A1:I278"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -17874,7 +18828,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -19039,7 +19993,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="32" type="noConversion"/>
+  <phoneticPr fontId="33" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -19049,7 +20003,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8F82A59-57DF-46F6-BCD0-E7A53E611046}">
   <dimension ref="A1:L54"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
lode runner - various script changes, and a demo movie of a strange gold drop, not sure if it is useful, but it is odd
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{484D956D-77AC-4121-A690-7BA0588A75D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAF954DD-8CFA-40F7-89DF-B6475026F76E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="431">
   <si>
     <t>Place</t>
   </si>
@@ -1327,6 +1327,9 @@
   </si>
   <si>
     <t>v7.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2679 I found manually can't recreate, bad spawn timer </t>
   </si>
 </sst>
 </file>
@@ -2254,7 +2257,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8465CAE6-FA0E-4F56-807B-2D9877AC152D}">
-  <dimension ref="A1:E129"/>
+  <dimension ref="A1:F129"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2263,7 +2266,7 @@
     <col min="5" max="5" width="17.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2277,7 +2280,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="50" t="s">
         <v>389</v>
       </c>
@@ -2292,7 +2295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="50" t="s">
         <v>392</v>
       </c>
@@ -2307,7 +2310,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="50" t="s">
         <v>391</v>
       </c>
@@ -2325,7 +2328,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="50" t="s">
         <v>390</v>
       </c>
@@ -2340,7 +2343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="50" t="s">
         <v>393</v>
       </c>
@@ -2355,7 +2358,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="50"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2364,7 +2367,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="50"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -2373,7 +2376,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="50"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -2382,7 +2385,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="50" t="s">
         <v>251</v>
       </c>
@@ -2397,22 +2400,28 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="50" t="s">
         <v>394</v>
       </c>
       <c r="B11" s="7">
-        <v>2680</v>
+        <v>2688</v>
       </c>
       <c r="C11" s="7">
         <v>2683</v>
       </c>
       <c r="D11" s="3">
         <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>-5</v>
+      </c>
+      <c r="E11">
+        <v>2680</v>
+      </c>
+      <c r="F11" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="50" t="s">
         <v>253</v>
       </c>
@@ -2425,7 +2434,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="50" t="s">
         <v>395</v>
       </c>
@@ -2438,7 +2447,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="50"/>
       <c r="B14" s="7"/>
       <c r="C14" s="7">
@@ -2449,7 +2458,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="50"/>
       <c r="B15" s="7"/>
       <c r="C15" s="7">
@@ -2460,7 +2469,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="50" t="s">
         <v>255</v>
       </c>

</xml_diff>

<commit_message>
lode runner - lv 3 improved route, about 20 frames faster
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAF954DD-8CFA-40F7-89DF-B6475026F76E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4EC116E-03F8-47E2-AE25-0E6E484D864A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1912,6 +1912,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1936,7 +1937,6 @@
     <xf numFmtId="0" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2390,14 +2390,14 @@
         <v>251</v>
       </c>
       <c r="B10" s="2">
-        <v>2333</v>
+        <v>2312</v>
       </c>
       <c r="C10" s="2">
         <v>2334</v>
       </c>
       <c r="D10" s="3">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2405,14 +2405,14 @@
         <v>394</v>
       </c>
       <c r="B11" s="7">
-        <v>2688</v>
+        <v>2661</v>
       </c>
       <c r="C11" s="7">
         <v>2683</v>
       </c>
       <c r="D11" s="3">
         <f t="shared" si="0"/>
-        <v>-5</v>
+        <v>22</v>
       </c>
       <c r="E11">
         <v>2680</v>
@@ -2425,13 +2425,15 @@
       <c r="A12" s="50" t="s">
         <v>253</v>
       </c>
-      <c r="B12" s="7"/>
+      <c r="B12" s="7">
+        <v>3144</v>
+      </c>
       <c r="C12" s="7">
         <v>3132</v>
       </c>
-      <c r="D12" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D12" s="3">
+        <f t="shared" si="0"/>
+        <v>-12</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2842,7 +2844,7 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="E45" s="60" t="s">
+      <c r="E45" s="52" t="s">
         <v>428</v>
       </c>
     </row>
@@ -20032,10 +20034,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="52" t="s">
+      <c r="K1" s="53" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="53"/>
+      <c r="L1" s="54"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -21887,13 +21889,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="54" t="s">
+      <c r="H53" s="55" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="55"/>
-      <c r="J53" s="55"/>
-      <c r="K53" s="55"/>
-      <c r="L53" s="56"/>
+      <c r="I53" s="56"/>
+      <c r="J53" s="56"/>
+      <c r="K53" s="56"/>
+      <c r="L53" s="57"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -21915,11 +21917,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="57"/>
-      <c r="I54" s="58"/>
-      <c r="J54" s="58"/>
-      <c r="K54" s="58"/>
-      <c r="L54" s="59"/>
+      <c r="H54" s="58"/>
+      <c r="I54" s="59"/>
+      <c r="J54" s="59"/>
+      <c r="K54" s="59"/>
+      <c r="L54" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - lv 4 25 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4EC116E-03F8-47E2-AE25-0E6E484D864A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{337F7624-CC3B-4DE7-BA13-8A5ED85F0ABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2405,14 +2405,14 @@
         <v>394</v>
       </c>
       <c r="B11" s="7">
-        <v>2661</v>
+        <v>2660</v>
       </c>
       <c r="C11" s="7">
         <v>2683</v>
       </c>
       <c r="D11" s="3">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E11">
         <v>2680</v>
@@ -2426,14 +2426,14 @@
         <v>253</v>
       </c>
       <c r="B12" s="7">
-        <v>3144</v>
+        <v>3107</v>
       </c>
       <c r="C12" s="7">
         <v>3132</v>
       </c>
       <c r="D12" s="3">
         <f t="shared" si="0"/>
-        <v>-12</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
level 6 done, lost 10 frames, investigating better routes
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{337F7624-CC3B-4DE7-BA13-8A5ED85F0ABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9AABBE4-1DC5-4467-A726-B85A894EAF4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2257,7 +2257,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8465CAE6-FA0E-4F56-807B-2D9877AC152D}">
-  <dimension ref="A1:F129"/>
+  <dimension ref="A1:F124"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2291,7 +2291,7 @@
         <v>428</v>
       </c>
       <c r="D2" s="3">
-        <f t="shared" ref="D2:D46" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <f t="shared" ref="D2:D41" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
         <v>1</v>
       </c>
     </row>
@@ -2359,102 +2359,119 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A7" s="50"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="A7" s="50" t="s">
+        <v>251</v>
+      </c>
+      <c r="B7" s="2">
+        <v>2312</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2334</v>
+      </c>
+      <c r="D7" s="3">
+        <f t="shared" si="0"/>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A8" s="50"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="A8" s="50" t="s">
+        <v>394</v>
+      </c>
+      <c r="B8" s="7">
+        <v>2660</v>
+      </c>
+      <c r="C8" s="7">
+        <v>2683</v>
+      </c>
+      <c r="D8" s="3">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="E8">
+        <v>2680</v>
+      </c>
+      <c r="F8" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="50"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="A9" s="50" t="s">
+        <v>253</v>
+      </c>
+      <c r="B9" s="7">
+        <v>3108</v>
+      </c>
+      <c r="C9" s="7">
+        <v>3132</v>
+      </c>
+      <c r="D9" s="3">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="E9">
+        <v>3107</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="50" t="s">
-        <v>251</v>
-      </c>
-      <c r="B10" s="2">
-        <v>2312</v>
-      </c>
-      <c r="C10" s="2">
-        <v>2334</v>
-      </c>
-      <c r="D10" s="3">
-        <f t="shared" si="0"/>
-        <v>22</v>
+        <v>395</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7">
+        <v>3479</v>
+      </c>
+      <c r="D10" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="50" t="s">
-        <v>394</v>
+        <v>255</v>
       </c>
       <c r="B11" s="7">
-        <v>2660</v>
+        <v>3739</v>
       </c>
       <c r="C11" s="7">
-        <v>2683</v>
+        <v>3761</v>
       </c>
       <c r="D11" s="3">
         <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-      <c r="E11">
-        <v>2680</v>
-      </c>
-      <c r="F11" t="s">
-        <v>430</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="50" t="s">
-        <v>253</v>
+        <v>396</v>
       </c>
       <c r="B12" s="7">
-        <v>3107</v>
+        <v>4089</v>
       </c>
       <c r="C12" s="7">
-        <v>3132</v>
+        <v>4109</v>
       </c>
       <c r="D12" s="3">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13" s="50" t="s">
-        <v>395</v>
-      </c>
-      <c r="B13" s="7"/>
+      <c r="A13" s="50"/>
+      <c r="B13" s="7">
+        <v>4644</v>
+      </c>
       <c r="C13" s="7">
-        <v>3479</v>
-      </c>
-      <c r="D13" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>4657</v>
+      </c>
+      <c r="D13" s="3">
+        <f t="shared" si="0"/>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="50"/>
       <c r="B14" s="7"/>
-      <c r="C14" s="7">
-        <v>3548</v>
-      </c>
+      <c r="C14" s="7"/>
       <c r="D14" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
@@ -2463,56 +2480,52 @@
     <row r="15" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="50"/>
       <c r="B15" s="7"/>
-      <c r="C15" s="7">
-        <v>3640</v>
-      </c>
+      <c r="C15" s="7"/>
       <c r="D15" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A16" s="50" t="s">
-        <v>255</v>
-      </c>
+      <c r="A16" s="50"/>
       <c r="B16" s="7"/>
-      <c r="C16" s="7">
-        <v>3761</v>
-      </c>
+      <c r="C16" s="7"/>
       <c r="D16" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A17" s="50" t="s">
-        <v>396</v>
-      </c>
+      <c r="A17" s="50"/>
       <c r="B17" s="7"/>
-      <c r="C17" s="7">
-        <v>4109</v>
-      </c>
+      <c r="C17" s="7"/>
       <c r="D17" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" s="50"/>
-      <c r="B18" s="7"/>
+      <c r="A18" s="50" t="s">
+        <v>257</v>
+      </c>
+      <c r="B18" s="7">
+        <v>5115</v>
+      </c>
       <c r="C18" s="7">
-        <v>4509</v>
-      </c>
-      <c r="D18" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>5125</v>
+      </c>
+      <c r="D18" s="3">
+        <f t="shared" si="0"/>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A19" s="50"/>
+      <c r="A19" s="50" t="s">
+        <v>397</v>
+      </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7">
-        <v>4669</v>
+        <v>5474</v>
       </c>
       <c r="D19" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2520,10 +2533,12 @@
       </c>
     </row>
     <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A20" s="50"/>
+      <c r="A20" s="50" t="s">
+        <v>259</v>
+      </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7">
-        <v>4727</v>
+        <v>5936</v>
       </c>
       <c r="D20" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2531,10 +2546,12 @@
       </c>
     </row>
     <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A21" s="50"/>
+      <c r="A21" s="50" t="s">
+        <v>410</v>
+      </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7">
-        <v>4866</v>
+        <v>6287</v>
       </c>
       <c r="D21" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2545,7 +2562,7 @@
       <c r="A22" s="50"/>
       <c r="B22" s="7"/>
       <c r="C22" s="7">
-        <v>4953</v>
+        <v>6410</v>
       </c>
       <c r="D22" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2553,12 +2570,10 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A23" s="50" t="s">
-        <v>257</v>
-      </c>
+      <c r="A23" s="50"/>
       <c r="B23" s="7"/>
       <c r="C23" s="7">
-        <v>5125</v>
+        <v>6446</v>
       </c>
       <c r="D23" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2566,12 +2581,10 @@
       </c>
     </row>
     <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A24" s="50" t="s">
-        <v>397</v>
-      </c>
+      <c r="A24" s="50"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7">
-        <v>5474</v>
+        <v>6590</v>
       </c>
       <c r="D24" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2580,11 +2593,11 @@
     </row>
     <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="50" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7">
-        <v>5936</v>
+        <v>6690</v>
       </c>
       <c r="D25" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2593,11 +2606,11 @@
     </row>
     <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="50" t="s">
-        <v>410</v>
+        <v>398</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7">
-        <v>6287</v>
+        <v>7039</v>
       </c>
       <c r="D26" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2605,10 +2618,12 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A27" s="50"/>
+      <c r="A27" s="50" t="s">
+        <v>274</v>
+      </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7">
-        <v>6410</v>
+        <v>8127</v>
       </c>
       <c r="D27" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2616,10 +2631,12 @@
       </c>
     </row>
     <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A28" s="50"/>
+      <c r="A28" s="50" t="s">
+        <v>399</v>
+      </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7">
-        <v>6446</v>
+        <v>8527</v>
       </c>
       <c r="D28" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2627,10 +2644,12 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A29" s="50"/>
+      <c r="A29" s="50" t="s">
+        <v>276</v>
+      </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7">
-        <v>6590</v>
+        <v>9099</v>
       </c>
       <c r="D29" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2639,11 +2658,11 @@
     </row>
     <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="50" t="s">
-        <v>267</v>
+        <v>400</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7">
-        <v>6690</v>
+        <v>9447</v>
       </c>
       <c r="D30" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2652,11 +2671,11 @@
     </row>
     <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="50" t="s">
-        <v>398</v>
+        <v>278</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7">
-        <v>7039</v>
+        <v>9758</v>
       </c>
       <c r="D31" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2665,11 +2684,11 @@
     </row>
     <row r="32" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="50" t="s">
-        <v>274</v>
+        <v>401</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7">
-        <v>8127</v>
+        <v>10104</v>
       </c>
       <c r="D32" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2677,12 +2696,12 @@
       </c>
     </row>
     <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A33" s="50" t="s">
-        <v>399</v>
+      <c r="A33" s="51" t="s">
+        <v>127</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7">
-        <v>8527</v>
+        <v>10305</v>
       </c>
       <c r="D33" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2690,12 +2709,12 @@
       </c>
     </row>
     <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A34" s="50" t="s">
-        <v>276</v>
+      <c r="A34" s="51" t="s">
+        <v>426</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7">
-        <v>9099</v>
+        <v>10532</v>
       </c>
       <c r="D34" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2703,12 +2722,12 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A35" s="50" t="s">
-        <v>400</v>
+      <c r="A35" s="51" t="s">
+        <v>425</v>
       </c>
       <c r="B35" s="7"/>
       <c r="C35" s="7">
-        <v>9447</v>
+        <v>10574</v>
       </c>
       <c r="D35" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2717,11 +2736,11 @@
     </row>
     <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7">
-        <v>9758</v>
+        <v>10743</v>
       </c>
       <c r="D36" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2730,11 +2749,11 @@
     </row>
     <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="50" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B37" s="7"/>
       <c r="C37" s="7">
-        <v>10104</v>
+        <v>11094</v>
       </c>
       <c r="D37" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2742,12 +2761,12 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A38" s="51" t="s">
-        <v>127</v>
+      <c r="A38" s="50" t="s">
+        <v>283</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="7">
-        <v>10305</v>
+        <v>11652</v>
       </c>
       <c r="D38" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2755,114 +2774,69 @@
       </c>
     </row>
     <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A39" s="51" t="s">
-        <v>426</v>
+      <c r="A39" s="50" t="s">
+        <v>403</v>
       </c>
       <c r="B39" s="7"/>
       <c r="C39" s="7">
-        <v>10532</v>
+        <v>12308</v>
       </c>
       <c r="D39" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A40" s="51" t="s">
-        <v>425</v>
+    <row r="40" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="50" t="s">
+        <v>285</v>
       </c>
       <c r="B40" s="7"/>
       <c r="C40" s="7">
-        <v>10574</v>
+        <v>12768</v>
       </c>
       <c r="D40" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="E40" s="52" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="50" t="s">
-        <v>281</v>
+        <v>404</v>
       </c>
       <c r="B41" s="7"/>
       <c r="C41" s="7">
-        <v>10743</v>
+        <v>13120</v>
       </c>
       <c r="D41" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
+      <c r="E41" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A42" s="50" t="s">
-        <v>402</v>
-      </c>
       <c r="B42" s="7"/>
-      <c r="C42" s="7">
-        <v>11094</v>
-      </c>
-      <c r="D42" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
+      <c r="C42" s="7"/>
     </row>
     <row r="43" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A43" s="50" t="s">
-        <v>283</v>
-      </c>
       <c r="B43" s="7"/>
-      <c r="C43" s="7">
-        <v>11652</v>
-      </c>
-      <c r="D43" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
+      <c r="C43" s="7"/>
     </row>
     <row r="44" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A44" s="50" t="s">
-        <v>403</v>
-      </c>
       <c r="B44" s="7"/>
-      <c r="C44" s="7">
-        <v>12308</v>
-      </c>
-      <c r="D44" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="50" t="s">
-        <v>285</v>
-      </c>
+      <c r="C44" s="7"/>
+    </row>
+    <row r="45" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B45" s="7"/>
-      <c r="C45" s="7">
-        <v>12768</v>
-      </c>
-      <c r="D45" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="E45" s="52" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="50" t="s">
-        <v>404</v>
-      </c>
+      <c r="C45" s="7"/>
+    </row>
+    <row r="46" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B46" s="7"/>
-      <c r="C46" s="7">
-        <v>13120</v>
-      </c>
-      <c r="D46" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="E46" t="s">
-        <v>427</v>
-      </c>
+      <c r="C46" s="7"/>
     </row>
     <row r="47" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B47" s="7"/>
@@ -3175,26 +3149,6 @@
     <row r="124" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B124" s="7"/>
       <c r="C124" s="7"/>
-    </row>
-    <row r="125" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B125" s="7"/>
-      <c r="C125" s="7"/>
-    </row>
-    <row r="126" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B126" s="7"/>
-      <c r="C126" s="7"/>
-    </row>
-    <row r="127" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B127" s="7"/>
-      <c r="C127" s="7"/>
-    </row>
-    <row r="128" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B128" s="7"/>
-      <c r="C128" s="7"/>
-    </row>
-    <row r="129" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B129" s="7"/>
-      <c r="C129" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - up to lv 7 27 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9AABBE4-1DC5-4467-A726-B85A894EAF4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6E36E4A-773A-4907-B158-D34C1980B122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="49050" yWindow="2325" windowWidth="8610" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="46560" yWindow="3780" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7.1" sheetId="9" r:id="rId1"/>
@@ -2257,13 +2257,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8465CAE6-FA0E-4F56-807B-2D9877AC152D}">
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F119"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="8.75" customWidth="1"/>
     <col min="4" max="4" width="6.625" customWidth="1"/>
     <col min="5" max="5" width="17.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.25" customWidth="1"/>
+    <col min="7" max="7" width="26.375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.25">
@@ -2291,7 +2293,7 @@
         <v>428</v>
       </c>
       <c r="D2" s="3">
-        <f t="shared" ref="D2:D41" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <f t="shared" ref="D2:D36" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
         <v>1</v>
       </c>
     </row>
@@ -2456,40 +2458,56 @@
       </c>
     </row>
     <row r="13" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13" s="50"/>
+      <c r="A13" s="50" t="s">
+        <v>257</v>
+      </c>
       <c r="B13" s="7">
-        <v>4644</v>
+        <v>5097</v>
       </c>
       <c r="C13" s="7">
-        <v>4657</v>
+        <v>5125</v>
       </c>
       <c r="D13" s="3">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" s="50"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="A14" s="50" t="s">
+        <v>397</v>
+      </c>
+      <c r="B14" s="7">
+        <v>5447</v>
+      </c>
+      <c r="C14" s="7">
+        <v>5474</v>
+      </c>
+      <c r="D14" s="3">
+        <f t="shared" si="0"/>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="50"/>
+      <c r="A15" s="50" t="s">
+        <v>259</v>
+      </c>
       <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
+      <c r="C15" s="7">
+        <v>5936</v>
+      </c>
       <c r="D15" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A16" s="50"/>
+      <c r="A16" s="50" t="s">
+        <v>410</v>
+      </c>
       <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
+      <c r="C16" s="7">
+        <v>6287</v>
+      </c>
       <c r="D16" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
@@ -2498,34 +2516,30 @@
     <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="50"/>
       <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
+      <c r="C17" s="7">
+        <v>6410</v>
+      </c>
       <c r="D17" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" s="50" t="s">
-        <v>257</v>
-      </c>
-      <c r="B18" s="7">
-        <v>5115</v>
-      </c>
+      <c r="A18" s="50"/>
+      <c r="B18" s="7"/>
       <c r="C18" s="7">
-        <v>5125</v>
-      </c>
-      <c r="D18" s="3">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <v>6446</v>
+      </c>
+      <c r="D18" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A19" s="50" t="s">
-        <v>397</v>
-      </c>
+      <c r="A19" s="50"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7">
-        <v>5474</v>
+        <v>6590</v>
       </c>
       <c r="D19" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2534,11 +2548,11 @@
     </row>
     <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="50" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7">
-        <v>5936</v>
+        <v>6690</v>
       </c>
       <c r="D20" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2547,11 +2561,11 @@
     </row>
     <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="50" t="s">
-        <v>410</v>
+        <v>398</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7">
-        <v>6287</v>
+        <v>7039</v>
       </c>
       <c r="D21" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2559,10 +2573,12 @@
       </c>
     </row>
     <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A22" s="50"/>
+      <c r="A22" s="50" t="s">
+        <v>274</v>
+      </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7">
-        <v>6410</v>
+        <v>8127</v>
       </c>
       <c r="D22" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2570,10 +2586,12 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A23" s="50"/>
+      <c r="A23" s="50" t="s">
+        <v>399</v>
+      </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7">
-        <v>6446</v>
+        <v>8527</v>
       </c>
       <c r="D23" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2581,10 +2599,12 @@
       </c>
     </row>
     <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A24" s="50"/>
+      <c r="A24" s="50" t="s">
+        <v>276</v>
+      </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7">
-        <v>6590</v>
+        <v>9099</v>
       </c>
       <c r="D24" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2593,11 +2613,11 @@
     </row>
     <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="50" t="s">
-        <v>267</v>
+        <v>400</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7">
-        <v>6690</v>
+        <v>9447</v>
       </c>
       <c r="D25" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2606,11 +2626,11 @@
     </row>
     <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="50" t="s">
-        <v>398</v>
+        <v>278</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7">
-        <v>7039</v>
+        <v>9758</v>
       </c>
       <c r="D26" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2619,11 +2639,11 @@
     </row>
     <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="50" t="s">
-        <v>274</v>
+        <v>401</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7">
-        <v>8127</v>
+        <v>10104</v>
       </c>
       <c r="D27" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2631,12 +2651,12 @@
       </c>
     </row>
     <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A28" s="50" t="s">
-        <v>399</v>
+      <c r="A28" s="51" t="s">
+        <v>127</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7">
-        <v>8527</v>
+        <v>10305</v>
       </c>
       <c r="D28" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2644,12 +2664,12 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A29" s="50" t="s">
-        <v>276</v>
+      <c r="A29" s="51" t="s">
+        <v>426</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7">
-        <v>9099</v>
+        <v>10532</v>
       </c>
       <c r="D29" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2657,12 +2677,12 @@
       </c>
     </row>
     <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A30" s="50" t="s">
-        <v>400</v>
+      <c r="A30" s="51" t="s">
+        <v>425</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7">
-        <v>9447</v>
+        <v>10574</v>
       </c>
       <c r="D30" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2671,11 +2691,11 @@
     </row>
     <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="50" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7">
-        <v>9758</v>
+        <v>10743</v>
       </c>
       <c r="D31" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2684,11 +2704,11 @@
     </row>
     <row r="32" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="50" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7">
-        <v>10104</v>
+        <v>11094</v>
       </c>
       <c r="D32" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2696,12 +2716,12 @@
       </c>
     </row>
     <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A33" s="51" t="s">
-        <v>127</v>
+      <c r="A33" s="50" t="s">
+        <v>283</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7">
-        <v>10305</v>
+        <v>11652</v>
       </c>
       <c r="D33" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2709,114 +2729,69 @@
       </c>
     </row>
     <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A34" s="51" t="s">
-        <v>426</v>
+      <c r="A34" s="50" t="s">
+        <v>403</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7">
-        <v>10532</v>
+        <v>12308</v>
       </c>
       <c r="D34" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A35" s="51" t="s">
-        <v>425</v>
+    <row r="35" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="50" t="s">
+        <v>285</v>
       </c>
       <c r="B35" s="7"/>
       <c r="C35" s="7">
-        <v>10574</v>
+        <v>12768</v>
       </c>
       <c r="D35" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="E35" s="52" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
-        <v>281</v>
+        <v>404</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7">
-        <v>10743</v>
+        <v>13120</v>
       </c>
       <c r="D36" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
+      <c r="E36" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A37" s="50" t="s">
-        <v>402</v>
-      </c>
       <c r="B37" s="7"/>
-      <c r="C37" s="7">
-        <v>11094</v>
-      </c>
-      <c r="D37" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
+      <c r="C37" s="7"/>
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A38" s="50" t="s">
-        <v>283</v>
-      </c>
       <c r="B38" s="7"/>
-      <c r="C38" s="7">
-        <v>11652</v>
-      </c>
-      <c r="D38" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
+      <c r="C38" s="7"/>
     </row>
     <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A39" s="50" t="s">
-        <v>403</v>
-      </c>
       <c r="B39" s="7"/>
-      <c r="C39" s="7">
-        <v>12308</v>
-      </c>
-      <c r="D39" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="50" t="s">
-        <v>285</v>
-      </c>
+      <c r="C39" s="7"/>
+    </row>
+    <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B40" s="7"/>
-      <c r="C40" s="7">
-        <v>12768</v>
-      </c>
-      <c r="D40" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="E40" s="52" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="50" t="s">
-        <v>404</v>
-      </c>
+      <c r="C40" s="7"/>
+    </row>
+    <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B41" s="7"/>
-      <c r="C41" s="7">
-        <v>13120</v>
-      </c>
-      <c r="D41" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="E41" t="s">
-        <v>427</v>
-      </c>
+      <c r="C41" s="7"/>
     </row>
     <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B42" s="7"/>
@@ -3129,26 +3104,6 @@
     <row r="119" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B119" s="7"/>
       <c r="C119" s="7"/>
-    </row>
-    <row r="120" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B120" s="7"/>
-      <c r="C120" s="7"/>
-    </row>
-    <row r="121" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B121" s="7"/>
-      <c r="C121" s="7"/>
-    </row>
-    <row r="122" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B122" s="7"/>
-      <c r="C122" s="7"/>
-    </row>
-    <row r="123" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B123" s="7"/>
-      <c r="C123" s="7"/>
-    </row>
-    <row r="124" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B124" s="7"/>
-      <c r="C124" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - lv 7 done, 27 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6E36E4A-773A-4907-B158-D34C1980B122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{751736DE-E28D-4078-8BAD-F63F87D506C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="46560" yWindow="3780" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2257,7 +2257,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8465CAE6-FA0E-4F56-807B-2D9877AC152D}">
-  <dimension ref="A1:F119"/>
+  <dimension ref="A1:F120"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2293,7 +2293,7 @@
         <v>428</v>
       </c>
       <c r="D2" s="3">
-        <f t="shared" ref="D2:D36" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <f t="shared" ref="D2:D37" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
         <v>1</v>
       </c>
     </row>
@@ -2488,47 +2488,53 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="50" t="s">
-        <v>259</v>
-      </c>
-      <c r="B15" s="7"/>
+      <c r="A15" s="50"/>
+      <c r="B15" s="7">
+        <v>5706</v>
+      </c>
       <c r="C15" s="7">
-        <v>5936</v>
-      </c>
-      <c r="D15" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>5733</v>
+      </c>
+      <c r="D15" s="3">
+        <f t="shared" si="0"/>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="50" t="s">
+        <v>259</v>
+      </c>
+      <c r="B16" s="7">
+        <v>5910</v>
+      </c>
+      <c r="C16" s="7">
+        <v>5936</v>
+      </c>
+      <c r="D16" s="3">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A17" s="50" t="s">
         <v>410</v>
       </c>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7">
+      <c r="B17" s="7">
+        <v>6260</v>
+      </c>
+      <c r="C17" s="7">
         <v>6287</v>
       </c>
-      <c r="D16" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A17" s="50"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7">
-        <v>6410</v>
-      </c>
-      <c r="D17" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D17" s="3">
+        <f t="shared" si="0"/>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="50"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7">
-        <v>6446</v>
+        <v>6410</v>
       </c>
       <c r="D18" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2539,7 +2545,7 @@
       <c r="A19" s="50"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7">
-        <v>6590</v>
+        <v>6446</v>
       </c>
       <c r="D19" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2547,12 +2553,10 @@
       </c>
     </row>
     <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A20" s="50" t="s">
-        <v>267</v>
-      </c>
+      <c r="A20" s="50"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7">
-        <v>6690</v>
+        <v>6590</v>
       </c>
       <c r="D20" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2561,11 +2565,11 @@
     </row>
     <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="50" t="s">
-        <v>398</v>
+        <v>267</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7">
-        <v>7039</v>
+        <v>6690</v>
       </c>
       <c r="D21" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2574,11 +2578,11 @@
     </row>
     <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="50" t="s">
-        <v>274</v>
+        <v>398</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7">
-        <v>8127</v>
+        <v>7039</v>
       </c>
       <c r="D22" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2587,11 +2591,11 @@
     </row>
     <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="50" t="s">
-        <v>399</v>
+        <v>274</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7">
-        <v>8527</v>
+        <v>8127</v>
       </c>
       <c r="D23" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2600,11 +2604,11 @@
     </row>
     <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A24" s="50" t="s">
-        <v>276</v>
+        <v>399</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7">
-        <v>9099</v>
+        <v>8527</v>
       </c>
       <c r="D24" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2613,11 +2617,11 @@
     </row>
     <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="50" t="s">
-        <v>400</v>
+        <v>276</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7">
-        <v>9447</v>
+        <v>9099</v>
       </c>
       <c r="D25" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2626,11 +2630,11 @@
     </row>
     <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="50" t="s">
-        <v>278</v>
+        <v>400</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7">
-        <v>9758</v>
+        <v>9447</v>
       </c>
       <c r="D26" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2639,11 +2643,11 @@
     </row>
     <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="50" t="s">
-        <v>401</v>
+        <v>278</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7">
-        <v>10104</v>
+        <v>9758</v>
       </c>
       <c r="D27" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2651,12 +2655,12 @@
       </c>
     </row>
     <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A28" s="51" t="s">
-        <v>127</v>
+      <c r="A28" s="50" t="s">
+        <v>401</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7">
-        <v>10305</v>
+        <v>10104</v>
       </c>
       <c r="D28" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2665,11 +2669,11 @@
     </row>
     <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="51" t="s">
-        <v>426</v>
+        <v>127</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7">
-        <v>10532</v>
+        <v>10305</v>
       </c>
       <c r="D29" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2678,11 +2682,11 @@
     </row>
     <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="51" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7">
-        <v>10574</v>
+        <v>10532</v>
       </c>
       <c r="D30" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2690,12 +2694,12 @@
       </c>
     </row>
     <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A31" s="50" t="s">
-        <v>281</v>
+      <c r="A31" s="51" t="s">
+        <v>425</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7">
-        <v>10743</v>
+        <v>10574</v>
       </c>
       <c r="D31" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2704,11 +2708,11 @@
     </row>
     <row r="32" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="50" t="s">
-        <v>402</v>
+        <v>281</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7">
-        <v>11094</v>
+        <v>10743</v>
       </c>
       <c r="D32" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2717,11 +2721,11 @@
     </row>
     <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="50" t="s">
-        <v>283</v>
+        <v>402</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7">
-        <v>11652</v>
+        <v>11094</v>
       </c>
       <c r="D33" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2730,52 +2734,61 @@
     </row>
     <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A34" s="50" t="s">
-        <v>403</v>
+        <v>283</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7">
-        <v>12308</v>
+        <v>11652</v>
       </c>
       <c r="D34" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A35" s="50" t="s">
-        <v>285</v>
+        <v>403</v>
       </c>
       <c r="B35" s="7"/>
       <c r="C35" s="7">
-        <v>12768</v>
+        <v>12308</v>
       </c>
       <c r="D35" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
-      </c>
-      <c r="E35" s="52" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
-        <v>404</v>
+        <v>285</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7">
+        <v>12768</v>
+      </c>
+      <c r="D36" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E36" s="52" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="50" t="s">
+        <v>404</v>
+      </c>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7">
         <v>13120</v>
       </c>
-      <c r="D36" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="E36" t="s">
+      <c r="D37" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="E37" t="s">
         <v>427</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B38" s="7"/>
@@ -3104,6 +3117,10 @@
     <row r="119" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B119" s="7"/>
       <c r="C119" s="7"/>
+    </row>
+    <row r="120" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B120" s="7"/>
+      <c r="C120" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - level 8 done - 31 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{751736DE-E28D-4078-8BAD-F63F87D506C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BABE2684-EE2E-472C-B479-B912D536E1D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="46560" yWindow="3780" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2532,21 +2532,21 @@
     </row>
     <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="50"/>
-      <c r="B18" s="7"/>
+      <c r="B18" s="7">
+        <v>6417</v>
+      </c>
       <c r="C18" s="7">
-        <v>6410</v>
-      </c>
-      <c r="D18" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>6446</v>
+      </c>
+      <c r="D18" s="3">
+        <f t="shared" si="0"/>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="50"/>
       <c r="B19" s="7"/>
-      <c r="C19" s="7">
-        <v>6446</v>
-      </c>
+      <c r="C19" s="7"/>
       <c r="D19" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
@@ -2567,26 +2567,30 @@
       <c r="A21" s="50" t="s">
         <v>267</v>
       </c>
-      <c r="B21" s="7"/>
+      <c r="B21" s="7">
+        <v>6660</v>
+      </c>
       <c r="C21" s="7">
         <v>6690</v>
       </c>
-      <c r="D21" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D21" s="3">
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="50" t="s">
         <v>398</v>
       </c>
-      <c r="B22" s="7"/>
+      <c r="B22" s="7">
+        <v>7008</v>
+      </c>
       <c r="C22" s="7">
         <v>7039</v>
       </c>
-      <c r="D22" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D22" s="3">
+        <f t="shared" si="0"/>
+        <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - levle 9 done, 74 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BABE2684-EE2E-472C-B479-B912D536E1D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E4A7E2-99BA-4E03-A345-57447F8CE365}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="46560" yWindow="3780" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2597,26 +2597,30 @@
       <c r="A23" s="50" t="s">
         <v>274</v>
       </c>
-      <c r="B23" s="7"/>
+      <c r="B23" s="7">
+        <v>8096</v>
+      </c>
       <c r="C23" s="7">
         <v>8127</v>
       </c>
-      <c r="D23" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D23" s="3">
+        <f t="shared" si="0"/>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A24" s="50" t="s">
         <v>399</v>
       </c>
-      <c r="B24" s="7"/>
+      <c r="B24" s="7">
+        <v>8453</v>
+      </c>
       <c r="C24" s="7">
         <v>8527</v>
       </c>
-      <c r="D24" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D24" s="3">
+        <f t="shared" si="0"/>
+        <v>74</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - level 11 done, 83 frames ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E4A7E2-99BA-4E03-A345-57447F8CE365}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B0157F7-0BD8-45D6-82E8-9F40216BEBA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46560" yWindow="3780" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="46560" yWindow="3210" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7.1" sheetId="9" r:id="rId1"/>
@@ -2627,52 +2627,60 @@
       <c r="A25" s="50" t="s">
         <v>276</v>
       </c>
-      <c r="B25" s="7"/>
+      <c r="B25" s="7">
+        <v>9024</v>
+      </c>
       <c r="C25" s="7">
         <v>9099</v>
       </c>
-      <c r="D25" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D25" s="3">
+        <f t="shared" si="0"/>
+        <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="50" t="s">
         <v>400</v>
       </c>
-      <c r="B26" s="7"/>
+      <c r="B26" s="7">
+        <v>9372</v>
+      </c>
       <c r="C26" s="7">
         <v>9447</v>
       </c>
-      <c r="D26" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D26" s="3">
+        <f t="shared" si="0"/>
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="50" t="s">
         <v>278</v>
       </c>
-      <c r="B27" s="7"/>
+      <c r="B27" s="7">
+        <v>9676</v>
+      </c>
       <c r="C27" s="7">
         <v>9758</v>
       </c>
-      <c r="D27" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D27" s="3">
+        <f t="shared" si="0"/>
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="50" t="s">
         <v>401</v>
       </c>
-      <c r="B28" s="7"/>
+      <c r="B28" s="7">
+        <v>10021</v>
+      </c>
       <c r="C28" s="7">
         <v>10104</v>
       </c>
-      <c r="D28" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D28" s="3">
+        <f t="shared" si="0"/>
+        <v>83</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - level 12 - route change, might be faster
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B0157F7-0BD8-45D6-82E8-9F40216BEBA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EC9BA62-EA51-4C72-B14B-8491909ED481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="46560" yWindow="3210" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="432">
   <si>
     <t>Place</t>
   </si>
@@ -1330,6 +1330,9 @@
   </si>
   <si>
     <t xml:space="preserve">2679 I found manually can't recreate, bad spawn timer </t>
+  </si>
+  <si>
+    <t>begin wait</t>
   </si>
 </sst>
 </file>
@@ -1339,12 +1342,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="37" x14ac:knownFonts="1">
+  <fonts count="38" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1804,95 +1814,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1912,31 +1923,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2257,7 +2268,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8465CAE6-FA0E-4F56-807B-2D9877AC152D}">
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F116"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2293,7 +2304,7 @@
         <v>428</v>
       </c>
       <c r="D2" s="3">
-        <f t="shared" ref="D2:D37" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <f t="shared" ref="D2:D33" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
         <v>1</v>
       </c>
     </row>
@@ -2488,323 +2499,295 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="50"/>
+      <c r="A15" s="50" t="s">
+        <v>259</v>
+      </c>
       <c r="B15" s="7">
-        <v>5706</v>
+        <v>5910</v>
       </c>
       <c r="C15" s="7">
-        <v>5733</v>
+        <v>5936</v>
       </c>
       <c r="D15" s="3">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="50" t="s">
-        <v>259</v>
+        <v>410</v>
       </c>
       <c r="B16" s="7">
-        <v>5910</v>
+        <v>6260</v>
       </c>
       <c r="C16" s="7">
-        <v>5936</v>
+        <v>6287</v>
       </c>
       <c r="D16" s="3">
         <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="50" t="s">
-        <v>410</v>
+        <v>267</v>
       </c>
       <c r="B17" s="7">
-        <v>6260</v>
+        <v>6660</v>
       </c>
       <c r="C17" s="7">
-        <v>6287</v>
+        <v>6690</v>
       </c>
       <c r="D17" s="3">
         <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" s="50"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A18" s="50" t="s">
+        <v>398</v>
+      </c>
       <c r="B18" s="7">
-        <v>6417</v>
+        <v>7008</v>
       </c>
       <c r="C18" s="7">
-        <v>6446</v>
+        <v>7039</v>
       </c>
       <c r="D18" s="3">
         <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A19" s="50"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A20" s="50"/>
-      <c r="B20" s="7"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A19" s="50" t="s">
+        <v>274</v>
+      </c>
+      <c r="B19" s="7">
+        <v>8096</v>
+      </c>
+      <c r="C19" s="7">
+        <v>8127</v>
+      </c>
+      <c r="D19" s="3">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A20" s="50" t="s">
+        <v>399</v>
+      </c>
+      <c r="B20" s="7">
+        <v>8453</v>
+      </c>
       <c r="C20" s="7">
-        <v>6590</v>
-      </c>
-      <c r="D20" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <v>8527</v>
+      </c>
+      <c r="D20" s="3">
+        <f t="shared" si="0"/>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="50" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="B21" s="7">
-        <v>6660</v>
+        <v>9024</v>
       </c>
       <c r="C21" s="7">
-        <v>6690</v>
+        <v>9099</v>
       </c>
       <c r="D21" s="3">
         <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="50" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B22" s="7">
-        <v>7008</v>
+        <v>9372</v>
       </c>
       <c r="C22" s="7">
-        <v>7039</v>
+        <v>9447</v>
       </c>
       <c r="D22" s="3">
         <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="50" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B23" s="7">
-        <v>8096</v>
+        <v>9676</v>
       </c>
       <c r="C23" s="7">
-        <v>8127</v>
+        <v>9758</v>
       </c>
       <c r="D23" s="3">
         <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A24" s="50" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B24" s="7">
-        <v>8453</v>
+        <v>10021</v>
       </c>
       <c r="C24" s="7">
-        <v>8527</v>
+        <v>10104</v>
       </c>
       <c r="D24" s="3">
         <f t="shared" si="0"/>
-        <v>74</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A25" s="50" t="s">
-        <v>276</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A25" s="61" t="s">
+        <v>127</v>
       </c>
       <c r="B25" s="7">
-        <v>9024</v>
+        <v>10222</v>
       </c>
       <c r="C25" s="7">
-        <v>9099</v>
+        <v>10305</v>
       </c>
       <c r="D25" s="3">
         <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A26" s="50" t="s">
-        <v>400</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A26" s="61" t="s">
+        <v>431</v>
       </c>
       <c r="B26" s="7">
-        <v>9372</v>
+        <v>10486</v>
       </c>
       <c r="C26" s="7">
-        <v>9447</v>
+        <v>10563</v>
       </c>
       <c r="D26" s="3">
         <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A27" s="50" t="s">
-        <v>278</v>
-      </c>
-      <c r="B27" s="7">
-        <v>9676</v>
-      </c>
-      <c r="C27" s="7">
-        <v>9758</v>
-      </c>
-      <c r="D27" s="3">
-        <f t="shared" si="0"/>
-        <v>82</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A27" s="51"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="50" t="s">
-        <v>401</v>
+        <v>281</v>
       </c>
       <c r="B28" s="7">
-        <v>10021</v>
+        <v>10658</v>
       </c>
       <c r="C28" s="7">
-        <v>10104</v>
+        <v>10743</v>
       </c>
       <c r="D28" s="3">
         <f t="shared" si="0"/>
-        <v>83</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A29" s="51" t="s">
-        <v>127</v>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A29" s="50" t="s">
+        <v>402</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7">
-        <v>10305</v>
+        <v>11094</v>
       </c>
       <c r="D29" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A30" s="51" t="s">
-        <v>426</v>
+    <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A30" s="50" t="s">
+        <v>283</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7">
-        <v>10532</v>
+        <v>11652</v>
       </c>
       <c r="D30" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A31" s="51" t="s">
-        <v>425</v>
+    <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A31" s="50" t="s">
+        <v>403</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7">
-        <v>10574</v>
+        <v>12308</v>
       </c>
       <c r="D31" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="50" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7">
-        <v>10743</v>
+        <v>12768</v>
       </c>
       <c r="D32" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="E32" s="52" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="50" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7">
-        <v>11094</v>
+        <v>13120</v>
       </c>
       <c r="D33" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
+      <c r="E33" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A34" s="50" t="s">
-        <v>283</v>
-      </c>
       <c r="B34" s="7"/>
-      <c r="C34" s="7">
-        <v>11652</v>
-      </c>
-      <c r="D34" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
+      <c r="C34" s="7"/>
     </row>
     <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A35" s="50" t="s">
-        <v>403</v>
-      </c>
       <c r="B35" s="7"/>
-      <c r="C35" s="7">
-        <v>12308</v>
-      </c>
-      <c r="D35" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="50" t="s">
-        <v>285</v>
-      </c>
+      <c r="C35" s="7"/>
+    </row>
+    <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B36" s="7"/>
-      <c r="C36" s="7">
-        <v>12768</v>
-      </c>
-      <c r="D36" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="E36" s="52" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="50" t="s">
-        <v>404</v>
-      </c>
+      <c r="C36" s="7"/>
+    </row>
+    <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B37" s="7"/>
-      <c r="C37" s="7">
-        <v>13120</v>
-      </c>
-      <c r="D37" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="E37" t="s">
-        <v>427</v>
-      </c>
+      <c r="C37" s="7"/>
     </row>
     <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B38" s="7"/>
@@ -3121,22 +3104,6 @@
     <row r="116" spans="2:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B116" s="7"/>
       <c r="C116" s="7"/>
-    </row>
-    <row r="117" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B117" s="7"/>
-      <c r="C117" s="7"/>
-    </row>
-    <row r="118" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B118" s="7"/>
-      <c r="C118" s="7"/>
-    </row>
-    <row r="119" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B119" s="7"/>
-      <c r="C119" s="7"/>
-    </row>
-    <row r="120" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B120" s="7"/>
-      <c r="C120" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19946,7 +19913,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="33" type="noConversion"/>
+  <phoneticPr fontId="34" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>

</xml_diff>

<commit_message>
lode runner - up to lv 13 - 91 frames ahead but bad spawn timer, will need to spend on it
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EC9BA62-EA51-4C72-B14B-8491909ED481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97685501-8851-493C-BCFC-A2171393976A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="46560" yWindow="3210" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2706,13 +2706,15 @@
       <c r="A29" s="50" t="s">
         <v>402</v>
       </c>
-      <c r="B29" s="7"/>
+      <c r="B29" s="7">
+        <v>11003</v>
+      </c>
       <c r="C29" s="7">
         <v>11094</v>
       </c>
-      <c r="D29" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D29" s="3">
+        <f t="shared" si="0"/>
+        <v>91</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - up to level 14, 80 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97685501-8851-493C-BCFC-A2171393976A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{275B34C3-6A7F-4B6E-ADAA-CC0C5B4FD970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="46560" yWindow="3210" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2707,40 +2707,47 @@
         <v>402</v>
       </c>
       <c r="B29" s="7">
-        <v>11003</v>
+        <v>11015</v>
       </c>
       <c r="C29" s="7">
         <v>11094</v>
       </c>
       <c r="D29" s="3">
         <f t="shared" si="0"/>
-        <v>91</v>
+        <v>79</v>
+      </c>
+      <c r="E29" s="7">
+        <v>11003</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="50" t="s">
         <v>283</v>
       </c>
-      <c r="B30" s="7"/>
+      <c r="B30" s="7">
+        <v>11573</v>
+      </c>
       <c r="C30" s="7">
         <v>11652</v>
       </c>
-      <c r="D30" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="D30" s="3">
+        <f t="shared" si="0"/>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="50" t="s">
         <v>403</v>
       </c>
-      <c r="B31" s="7"/>
+      <c r="B31" s="61">
+        <v>11928</v>
+      </c>
       <c r="C31" s="7">
-        <v>12308</v>
-      </c>
-      <c r="D31" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+        <v>12008</v>
+      </c>
+      <c r="D31" s="3">
+        <f t="shared" si="0"/>
+        <v>80</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - merge v7.1 as v7 and rework files and spreadsheet, 244 frames ahead ahead of v6 at the start of level 15
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,19 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{275B34C3-6A7F-4B6E-ADAA-CC0C5B4FD970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89B2B36A-42AE-4060-8C33-91EF5B9F4680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46560" yWindow="3210" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="V7.1" sheetId="9" r:id="rId1"/>
-    <sheet name="V7" sheetId="8" r:id="rId2"/>
-    <sheet name="V6" sheetId="7" r:id="rId3"/>
-    <sheet name="V5" sheetId="5" r:id="rId4"/>
-    <sheet name="V4" sheetId="4" r:id="rId5"/>
-    <sheet name="V3" sheetId="3" r:id="rId6"/>
-    <sheet name="V2" sheetId="1" r:id="rId7"/>
-    <sheet name="Takanawa Comparison" sheetId="6" r:id="rId8"/>
+    <sheet name="V7" sheetId="8" r:id="rId1"/>
+    <sheet name="V6" sheetId="7" r:id="rId2"/>
+    <sheet name="V5" sheetId="5" r:id="rId3"/>
+    <sheet name="V4" sheetId="4" r:id="rId4"/>
+    <sheet name="V3" sheetId="3" r:id="rId5"/>
+    <sheet name="V2" sheetId="1" r:id="rId6"/>
+    <sheet name="Takanawa Comparison" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="423">
   <si>
     <t>Place</t>
   </si>
@@ -1306,33 +1305,6 @@
   </si>
   <si>
     <t>(v6 1st move)</t>
-  </si>
-  <si>
-    <t>Emulation difference on startup</t>
-  </si>
-  <si>
-    <t>1081 possible, delay for spawn timer</t>
-  </si>
-  <si>
-    <t>drop</t>
-  </si>
-  <si>
-    <t>land</t>
-  </si>
-  <si>
-    <t>13162 fast mode</t>
-  </si>
-  <si>
-    <t>12815 fast mode</t>
-  </si>
-  <si>
-    <t>v7.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2679 I found manually can't recreate, bad spawn timer </t>
-  </si>
-  <si>
-    <t>begin wait</t>
   </si>
 </sst>
 </file>
@@ -1342,26 +1314,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="38" x14ac:knownFonts="1">
+  <fonts count="36" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1814,97 +1772,95 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="30" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="5"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="6" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1923,28 +1879,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2267,33 +2223,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8465CAE6-FA0E-4F56-807B-2D9877AC152D}">
-  <dimension ref="A1:F116"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
+  <dimension ref="A1:E184"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="8.75" customWidth="1"/>
     <col min="4" max="4" width="6.625" customWidth="1"/>
-    <col min="5" max="5" width="17.625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.25" customWidth="1"/>
-    <col min="7" max="7" width="26.375" customWidth="1"/>
+    <col min="5" max="5" width="17.625" style="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>429</v>
+        <v>388</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="50" t="s">
         <v>389</v>
       </c>
@@ -2301,14 +2255,14 @@
         <v>427</v>
       </c>
       <c r="C2" s="2">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="D2" s="3">
-        <f t="shared" ref="D2:D33" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" ref="D2:D18" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="50" t="s">
         <v>392</v>
       </c>
@@ -2316,14 +2270,14 @@
         <v>737</v>
       </c>
       <c r="C3" s="2">
-        <v>739</v>
+        <v>758</v>
       </c>
       <c r="D3" s="3">
         <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="50" t="s">
         <v>391</v>
       </c>
@@ -2331,17 +2285,14 @@
         <v>1088</v>
       </c>
       <c r="C4" s="2">
-        <v>1089</v>
+        <v>1107</v>
       </c>
       <c r="D4" s="3">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="E4" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="50" t="s">
         <v>390</v>
       </c>
@@ -2349,14 +2300,14 @@
         <v>1573</v>
       </c>
       <c r="C5" s="2">
-        <v>1574</v>
+        <v>1602</v>
       </c>
       <c r="D5" s="3">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="50" t="s">
         <v>393</v>
       </c>
@@ -2364,14 +2315,14 @@
         <v>1920</v>
       </c>
       <c r="C6" s="2">
-        <v>1923</v>
+        <v>1950</v>
       </c>
       <c r="D6" s="3">
         <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="50" t="s">
         <v>251</v>
       </c>
@@ -2379,14 +2330,14 @@
         <v>2312</v>
       </c>
       <c r="C7" s="2">
-        <v>2334</v>
+        <v>2371</v>
       </c>
       <c r="D7" s="3">
         <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="50" t="s">
         <v>394</v>
       </c>
@@ -2394,20 +2345,14 @@
         <v>2660</v>
       </c>
       <c r="C8" s="7">
-        <v>2683</v>
+        <v>2719</v>
       </c>
       <c r="D8" s="3">
         <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-      <c r="E8">
-        <v>2680</v>
-      </c>
-      <c r="F8" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="50" t="s">
         <v>253</v>
       </c>
@@ -2415,30 +2360,27 @@
         <v>3108</v>
       </c>
       <c r="C9" s="7">
-        <v>3132</v>
+        <v>3195</v>
       </c>
       <c r="D9" s="3">
         <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-      <c r="E9">
-        <v>3107</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="50" t="s">
         <v>395</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7">
-        <v>3479</v>
+        <v>3543</v>
       </c>
       <c r="D10" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="50" t="s">
         <v>255</v>
       </c>
@@ -2446,14 +2388,14 @@
         <v>3739</v>
       </c>
       <c r="C11" s="7">
-        <v>3761</v>
+        <v>3829</v>
       </c>
       <c r="D11" s="3">
         <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="50" t="s">
         <v>396</v>
       </c>
@@ -2461,29 +2403,29 @@
         <v>4089</v>
       </c>
       <c r="C12" s="7">
-        <v>4109</v>
+        <v>4178</v>
       </c>
       <c r="D12" s="3">
         <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="50" t="s">
         <v>257</v>
       </c>
       <c r="B13" s="7">
         <v>5097</v>
       </c>
-      <c r="C13" s="7">
-        <v>5125</v>
+      <c r="C13" s="37">
+        <v>5190</v>
       </c>
       <c r="D13" s="3">
         <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="50" t="s">
         <v>397</v>
       </c>
@@ -2491,14 +2433,14 @@
         <v>5447</v>
       </c>
       <c r="C14" s="7">
-        <v>5474</v>
+        <v>5539</v>
       </c>
       <c r="D14" s="3">
         <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="50" t="s">
         <v>259</v>
       </c>
@@ -2506,14 +2448,14 @@
         <v>5910</v>
       </c>
       <c r="C15" s="7">
-        <v>5936</v>
+        <v>6003</v>
       </c>
       <c r="D15" s="3">
         <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="50" t="s">
         <v>410</v>
       </c>
@@ -2521,14 +2463,14 @@
         <v>6260</v>
       </c>
       <c r="C16" s="7">
-        <v>6287</v>
+        <v>6352</v>
       </c>
       <c r="D16" s="3">
         <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="50" t="s">
         <v>267</v>
       </c>
@@ -2536,14 +2478,14 @@
         <v>6660</v>
       </c>
       <c r="C17" s="7">
-        <v>6690</v>
+        <v>6759</v>
       </c>
       <c r="D17" s="3">
         <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="50" t="s">
         <v>398</v>
       </c>
@@ -2551,14 +2493,14 @@
         <v>7008</v>
       </c>
       <c r="C18" s="7">
-        <v>7039</v>
+        <v>7106</v>
       </c>
       <c r="D18" s="3">
         <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="50" t="s">
         <v>274</v>
       </c>
@@ -2566,14 +2508,14 @@
         <v>8096</v>
       </c>
       <c r="C19" s="7">
-        <v>8127</v>
+        <v>8196</v>
       </c>
       <c r="D19" s="3">
-        <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" ref="D19:D50" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="50" t="s">
         <v>399</v>
       </c>
@@ -2581,14 +2523,14 @@
         <v>8453</v>
       </c>
       <c r="C20" s="7">
-        <v>8527</v>
+        <v>8549</v>
       </c>
       <c r="D20" s="3">
-        <f t="shared" si="0"/>
-        <v>74</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="50" t="s">
         <v>276</v>
       </c>
@@ -2596,14 +2538,14 @@
         <v>9024</v>
       </c>
       <c r="C21" s="7">
-        <v>9099</v>
+        <v>9118</v>
       </c>
       <c r="D21" s="3">
-        <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>94</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="50" t="s">
         <v>400</v>
       </c>
@@ -2611,14 +2553,14 @@
         <v>9372</v>
       </c>
       <c r="C22" s="7">
-        <v>9447</v>
+        <v>9467</v>
       </c>
       <c r="D22" s="3">
-        <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="50" t="s">
         <v>278</v>
       </c>
@@ -2626,14 +2568,14 @@
         <v>9676</v>
       </c>
       <c r="C23" s="7">
-        <v>9758</v>
+        <v>9778</v>
       </c>
       <c r="D23" s="3">
-        <f t="shared" si="0"/>
-        <v>82</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="50" t="s">
         <v>401</v>
       </c>
@@ -2641,478 +2583,1369 @@
         <v>10021</v>
       </c>
       <c r="C24" s="7">
-        <v>10104</v>
+        <v>10125</v>
       </c>
       <c r="D24" s="3">
-        <f t="shared" si="0"/>
-        <v>83</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A25" s="61" t="s">
-        <v>127</v>
+        <f t="shared" si="1"/>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="50" t="s">
+        <v>281</v>
       </c>
       <c r="B25" s="7">
-        <v>10222</v>
+        <v>10658</v>
       </c>
       <c r="C25" s="7">
-        <v>10305</v>
+        <v>10816</v>
       </c>
       <c r="D25" s="3">
-        <f t="shared" si="0"/>
-        <v>83</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A26" s="61" t="s">
-        <v>431</v>
+        <f t="shared" si="1"/>
+        <v>158</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="50" t="s">
+        <v>402</v>
       </c>
       <c r="B26" s="7">
-        <v>10486</v>
+        <v>11015</v>
       </c>
       <c r="C26" s="7">
-        <v>10563</v>
+        <v>11163</v>
       </c>
       <c r="D26" s="3">
-        <f t="shared" si="0"/>
-        <v>77</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A27" s="51"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="50" t="s">
+        <v>283</v>
+      </c>
+      <c r="B27" s="7">
+        <v>11573</v>
+      </c>
+      <c r="C27" s="7">
+        <v>11729</v>
+      </c>
+      <c r="D27" s="3">
+        <f t="shared" si="1"/>
+        <v>156</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="50" t="s">
-        <v>281</v>
-      </c>
-      <c r="B28" s="7">
-        <v>10658</v>
+        <v>403</v>
+      </c>
+      <c r="B28" s="59">
+        <v>11928</v>
       </c>
       <c r="C28" s="7">
-        <v>10743</v>
+        <v>12383</v>
       </c>
       <c r="D28" s="3">
-        <f t="shared" si="0"/>
-        <v>85</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>455</v>
+      </c>
+      <c r="E28" s="59" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="50" t="s">
-        <v>402</v>
+        <v>285</v>
       </c>
       <c r="B29" s="7">
-        <v>11015</v>
+        <v>12640</v>
       </c>
       <c r="C29" s="7">
-        <v>11094</v>
+        <v>12891</v>
       </c>
       <c r="D29" s="3">
-        <f t="shared" si="0"/>
-        <v>79</v>
-      </c>
-      <c r="E29" s="7">
-        <v>11003</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>251</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="50" t="s">
-        <v>283</v>
+        <v>404</v>
       </c>
       <c r="B30" s="7">
-        <v>11573</v>
+        <v>12992</v>
       </c>
       <c r="C30" s="7">
-        <v>11652</v>
+        <v>13236</v>
       </c>
       <c r="D30" s="3">
-        <f t="shared" si="0"/>
-        <v>79</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>244</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="50" t="s">
-        <v>403</v>
-      </c>
-      <c r="B31" s="61">
-        <v>11928</v>
-      </c>
+        <v>288</v>
+      </c>
+      <c r="B31" s="7"/>
       <c r="C31" s="7">
-        <v>12008</v>
-      </c>
-      <c r="D31" s="3">
-        <f t="shared" si="0"/>
-        <v>80</v>
+        <v>13960</v>
+      </c>
+      <c r="D31" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="50" t="s">
-        <v>285</v>
+        <v>405</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7">
-        <v>12768</v>
+        <v>14320</v>
       </c>
       <c r="D32" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="E32" s="52" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="50" t="s">
-        <v>404</v>
+        <v>294</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7">
-        <v>13120</v>
+        <v>14679</v>
       </c>
       <c r="D33" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="E33" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="50" t="s">
+        <v>406</v>
+      </c>
       <c r="B34" s="7"/>
-      <c r="C34" s="7"/>
-    </row>
-    <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="C34" s="7">
+        <v>15029</v>
+      </c>
+      <c r="D34" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="50" t="s">
+        <v>297</v>
+      </c>
       <c r="B35" s="7"/>
-      <c r="C35" s="7"/>
-    </row>
-    <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="C35" s="7">
+        <v>15850</v>
+      </c>
+      <c r="D35" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="50" t="s">
+        <v>407</v>
+      </c>
       <c r="B36" s="7"/>
-      <c r="C36" s="7"/>
-    </row>
-    <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-    </row>
-    <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="C36" s="7">
+        <v>16200</v>
+      </c>
+      <c r="D36" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="50" t="s">
+        <v>301</v>
+      </c>
+      <c r="B37" s="33"/>
+      <c r="C37" s="33">
+        <v>17135</v>
+      </c>
+      <c r="D37" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="50" t="s">
+        <v>408</v>
+      </c>
       <c r="B38" s="7"/>
-      <c r="C38" s="7"/>
-    </row>
-    <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="C38" s="7">
+        <v>17485</v>
+      </c>
+      <c r="D38" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="50" t="s">
+        <v>305</v>
+      </c>
       <c r="B39" s="7"/>
-      <c r="C39" s="7"/>
-    </row>
-    <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="C39" s="7">
+        <v>17791</v>
+      </c>
+      <c r="D39" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="50" t="s">
+        <v>409</v>
+      </c>
       <c r="B40" s="7"/>
-      <c r="C40" s="7"/>
-    </row>
-    <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="C40" s="37">
+        <v>18139</v>
+      </c>
+      <c r="D40" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="50" t="s">
+        <v>308</v>
+      </c>
       <c r="B41" s="7"/>
-      <c r="C41" s="7"/>
-    </row>
-    <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="C41" s="7">
+        <v>18719</v>
+      </c>
+      <c r="D41" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="50" t="s">
+        <v>411</v>
+      </c>
       <c r="B42" s="7"/>
-      <c r="C42" s="7"/>
-    </row>
-    <row r="43" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="C42" s="7">
+        <v>19068</v>
+      </c>
+      <c r="D42" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="50" t="s">
+        <v>314</v>
+      </c>
       <c r="B43" s="7"/>
-      <c r="C43" s="7"/>
-    </row>
-    <row r="44" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="C43" s="7">
+        <v>19892</v>
+      </c>
+      <c r="D43" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="50" t="s">
+        <v>412</v>
+      </c>
       <c r="B44" s="7"/>
-      <c r="C44" s="7"/>
-    </row>
-    <row r="45" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="C44" s="7">
+        <v>20240</v>
+      </c>
+      <c r="D44" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="50" t="s">
+        <v>320</v>
+      </c>
       <c r="B45" s="7"/>
-      <c r="C45" s="7"/>
-    </row>
-    <row r="46" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="C45" s="7">
+        <v>20813</v>
+      </c>
+      <c r="D45" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="50" t="s">
+        <v>413</v>
+      </c>
       <c r="B46" s="7"/>
-      <c r="C46" s="7"/>
-    </row>
-    <row r="47" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="C46" s="7">
+        <v>21161</v>
+      </c>
+      <c r="D46" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="50" t="s">
+        <v>322</v>
+      </c>
       <c r="B47" s="7"/>
-      <c r="C47" s="7"/>
-    </row>
-    <row r="48" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="C47" s="7">
+        <v>22195</v>
+      </c>
+      <c r="D47" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="50" t="s">
+        <v>414</v>
+      </c>
       <c r="B48" s="7"/>
-      <c r="C48" s="7"/>
-    </row>
-    <row r="49" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C48" s="7">
+        <v>22543</v>
+      </c>
+      <c r="D48" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="50" t="s">
+        <v>324</v>
+      </c>
       <c r="B49" s="7"/>
-      <c r="C49" s="7"/>
-    </row>
-    <row r="50" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C49" s="7">
+        <v>22963</v>
+      </c>
+      <c r="D49" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="50" t="s">
+        <v>415</v>
+      </c>
       <c r="B50" s="7"/>
-      <c r="C50" s="7"/>
-    </row>
-    <row r="51" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C50" s="7">
+        <v>23346</v>
+      </c>
+      <c r="D50" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="50" t="s">
+        <v>416</v>
+      </c>
       <c r="B51" s="7"/>
-      <c r="C51" s="7"/>
-    </row>
-    <row r="52" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B52" s="7"/>
-      <c r="C52" s="7"/>
-    </row>
-    <row r="53" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B53" s="7"/>
-      <c r="C53" s="7"/>
-    </row>
-    <row r="54" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C51" s="7">
+        <v>23873</v>
+      </c>
+      <c r="D51" s="3" t="str">
+        <f t="shared" ref="D51:D80" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="50" t="s">
+        <v>417</v>
+      </c>
+      <c r="B52" s="8"/>
+      <c r="C52" s="50">
+        <v>24221</v>
+      </c>
+      <c r="D52" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="50" t="s">
+        <v>418</v>
+      </c>
+      <c r="B53" s="33"/>
+      <c r="C53" s="33">
+        <v>25101</v>
+      </c>
+      <c r="D53" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="50" t="s">
+        <v>419</v>
+      </c>
       <c r="B54" s="7"/>
-      <c r="C54" s="7"/>
-    </row>
-    <row r="55" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C54" s="7">
+        <v>25450</v>
+      </c>
+      <c r="D54" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="50" t="s">
+        <v>420</v>
+      </c>
       <c r="B55" s="7"/>
-      <c r="C55" s="7"/>
-    </row>
-    <row r="56" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C55" s="7">
+        <v>26350</v>
+      </c>
+      <c r="D55" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="50" t="s">
+        <v>421</v>
+      </c>
       <c r="B56" s="7"/>
-      <c r="C56" s="7"/>
-    </row>
-    <row r="57" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C56" s="7">
+        <v>26699</v>
+      </c>
+      <c r="D56" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="50" t="s">
+        <v>332</v>
+      </c>
       <c r="B57" s="7"/>
-      <c r="C57" s="7"/>
-    </row>
-    <row r="58" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C57" s="7">
+        <v>27490</v>
+      </c>
+      <c r="D57" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="50" t="s">
+        <v>5</v>
+      </c>
       <c r="B58" s="7"/>
-      <c r="C58" s="7"/>
-    </row>
-    <row r="59" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C58" s="7">
+        <v>27836</v>
+      </c>
+      <c r="D58" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="50" t="s">
+        <v>337</v>
+      </c>
       <c r="B59" s="7"/>
-      <c r="C59" s="7"/>
-    </row>
-    <row r="60" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C59" s="7">
+        <v>28899</v>
+      </c>
+      <c r="D59" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="50" t="s">
+        <v>6</v>
+      </c>
       <c r="B60" s="7"/>
-      <c r="C60" s="7"/>
-    </row>
-    <row r="61" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C60" s="7">
+        <v>29248</v>
+      </c>
+      <c r="D60" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="50" t="s">
+        <v>45</v>
+      </c>
       <c r="B61" s="7"/>
-      <c r="C61" s="7"/>
-    </row>
-    <row r="62" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C61" s="7">
+        <v>29962</v>
+      </c>
+      <c r="D61" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="50" t="s">
+        <v>7</v>
+      </c>
       <c r="B62" s="7"/>
-      <c r="C62" s="7"/>
-    </row>
-    <row r="63" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C62" s="7">
+        <v>30309</v>
+      </c>
+      <c r="D62" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="50" t="s">
+        <v>46</v>
+      </c>
       <c r="B63" s="7"/>
-      <c r="C63" s="7"/>
-    </row>
-    <row r="64" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C63" s="7">
+        <v>30479</v>
+      </c>
+      <c r="D63" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="50" t="s">
+        <v>8</v>
+      </c>
       <c r="B64" s="7"/>
-      <c r="C64" s="7"/>
-    </row>
-    <row r="65" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C64" s="7">
+        <v>31125</v>
+      </c>
+      <c r="D64" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+      <c r="E64" s="59" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="50" t="s">
+        <v>28</v>
+      </c>
       <c r="B65" s="7"/>
-      <c r="C65" s="7"/>
-    </row>
-    <row r="66" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C65" s="7">
+        <v>31643</v>
+      </c>
+      <c r="D65" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="50" t="s">
+        <v>9</v>
+      </c>
       <c r="B66" s="7"/>
-      <c r="C66" s="7"/>
-    </row>
-    <row r="67" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C66" s="7">
+        <v>31991</v>
+      </c>
+      <c r="D66" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="50" t="s">
+        <v>29</v>
+      </c>
       <c r="B67" s="7"/>
-      <c r="C67" s="7"/>
-    </row>
-    <row r="68" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C67" s="7">
+        <v>32586</v>
+      </c>
+      <c r="D67" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="50" t="s">
+        <v>10</v>
+      </c>
       <c r="B68" s="7"/>
-      <c r="C68" s="7"/>
-    </row>
-    <row r="69" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C68" s="7">
+        <v>33254</v>
+      </c>
+      <c r="D68" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+      <c r="E68" s="59" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="50" t="s">
+        <v>31</v>
+      </c>
       <c r="B69" s="7"/>
-      <c r="C69" s="7"/>
-    </row>
-    <row r="70" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C69" s="7">
+        <v>33883</v>
+      </c>
+      <c r="D69" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="50" t="s">
+        <v>11</v>
+      </c>
       <c r="B70" s="7"/>
-      <c r="C70" s="7"/>
-    </row>
-    <row r="71" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C70" s="7">
+        <v>34244</v>
+      </c>
+      <c r="D70" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="50" t="s">
+        <v>30</v>
+      </c>
       <c r="B71" s="7"/>
-      <c r="C71" s="7"/>
-    </row>
-    <row r="72" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C71" s="7">
+        <v>34862</v>
+      </c>
+      <c r="D71" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="50" t="s">
+        <v>12</v>
+      </c>
       <c r="B72" s="7"/>
-      <c r="C72" s="7"/>
-    </row>
-    <row r="73" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C72" s="7">
+        <v>35218</v>
+      </c>
+      <c r="D72" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="50" t="s">
+        <v>32</v>
+      </c>
       <c r="B73" s="7"/>
-      <c r="C73" s="7"/>
-    </row>
-    <row r="74" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C73" s="7">
+        <v>35772</v>
+      </c>
+      <c r="D73" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="50" t="s">
+        <v>13</v>
+      </c>
       <c r="B74" s="7"/>
-      <c r="C74" s="7"/>
-    </row>
-    <row r="75" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C74" s="7">
+        <v>36120</v>
+      </c>
+      <c r="D74" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="50" t="s">
+        <v>47</v>
+      </c>
       <c r="B75" s="7"/>
-      <c r="C75" s="7"/>
-    </row>
-    <row r="76" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C75" s="7">
+        <v>36893</v>
+      </c>
+      <c r="D75" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="50" t="s">
+        <v>48</v>
+      </c>
       <c r="B76" s="7"/>
-      <c r="C76" s="7"/>
-    </row>
-    <row r="77" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C76" s="7">
+        <v>37238</v>
+      </c>
+      <c r="D76" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="50" t="s">
+        <v>33</v>
+      </c>
       <c r="B77" s="7"/>
-      <c r="C77" s="7"/>
-    </row>
-    <row r="78" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C77" s="7">
+        <v>38097</v>
+      </c>
+      <c r="D77" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="50" t="s">
+        <v>14</v>
+      </c>
       <c r="B78" s="7"/>
-      <c r="C78" s="7"/>
-    </row>
-    <row r="79" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C78" s="7">
+        <v>38443</v>
+      </c>
+      <c r="D78" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="50" t="s">
+        <v>34</v>
+      </c>
       <c r="B79" s="7"/>
-      <c r="C79" s="7"/>
-    </row>
-    <row r="80" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C79" s="7">
+        <v>38692</v>
+      </c>
+      <c r="D79" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="50" t="s">
+        <v>15</v>
+      </c>
       <c r="B80" s="7"/>
-      <c r="C80" s="7"/>
-    </row>
-    <row r="81" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C80" s="7">
+        <v>39041</v>
+      </c>
+      <c r="D80" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="50" t="s">
+        <v>35</v>
+      </c>
       <c r="B81" s="7"/>
-      <c r="C81" s="7"/>
-    </row>
-    <row r="82" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C81" s="7">
+        <v>40011</v>
+      </c>
+      <c r="D81" s="3" t="str">
+        <f>IF(C80&lt;&gt;"",IF(B80&lt;&gt;"",C80-B80,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="50" t="s">
+        <v>16</v>
+      </c>
       <c r="B82" s="7"/>
-      <c r="C82" s="7"/>
-    </row>
-    <row r="83" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B83" s="7"/>
-      <c r="C83" s="7"/>
-    </row>
-    <row r="84" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C82" s="7">
+        <v>40373</v>
+      </c>
+      <c r="D82" s="3" t="str">
+        <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="50" t="s">
+        <v>36</v>
+      </c>
+      <c r="B83" s="40"/>
+      <c r="C83" s="7">
+        <v>41117</v>
+      </c>
+      <c r="D83" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="50" t="s">
+        <v>17</v>
+      </c>
       <c r="B84" s="7"/>
-      <c r="C84" s="7"/>
-    </row>
-    <row r="85" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C84" s="7">
+        <v>41465</v>
+      </c>
+      <c r="D84" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="50" t="s">
+        <v>37</v>
+      </c>
       <c r="B85" s="7"/>
-      <c r="C85" s="7"/>
-    </row>
-    <row r="86" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C85" s="7">
+        <v>42450</v>
+      </c>
+      <c r="D85" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" s="50" t="s">
+        <v>18</v>
+      </c>
       <c r="B86" s="7"/>
-      <c r="C86" s="7"/>
-    </row>
-    <row r="87" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C86" s="7">
+        <v>42799</v>
+      </c>
+      <c r="D86" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="50" t="s">
+        <v>38</v>
+      </c>
       <c r="B87" s="7"/>
-      <c r="C87" s="7"/>
-    </row>
-    <row r="88" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C87" s="7">
+        <v>43144</v>
+      </c>
+      <c r="D87" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" s="50" t="s">
+        <v>19</v>
+      </c>
       <c r="B88" s="7"/>
-      <c r="C88" s="7"/>
-    </row>
-    <row r="89" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C88" s="7">
+        <v>43491</v>
+      </c>
+      <c r="D88" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="50" t="s">
+        <v>39</v>
+      </c>
       <c r="B89" s="7"/>
-      <c r="C89" s="7"/>
-    </row>
-    <row r="90" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C89" s="7">
+        <v>44165</v>
+      </c>
+      <c r="D89" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="50" t="s">
+        <v>20</v>
+      </c>
       <c r="B90" s="7"/>
-      <c r="C90" s="7"/>
-    </row>
-    <row r="91" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C90" s="7">
+        <v>44512</v>
+      </c>
+      <c r="D90" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="50" t="s">
+        <v>40</v>
+      </c>
       <c r="B91" s="7"/>
-      <c r="C91" s="7"/>
-    </row>
-    <row r="92" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C91" s="7">
+        <v>45061</v>
+      </c>
+      <c r="D91" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="50" t="s">
+        <v>21</v>
+      </c>
       <c r="B92" s="7"/>
-      <c r="C92" s="7"/>
-    </row>
-    <row r="93" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C92" s="7">
+        <v>45443</v>
+      </c>
+      <c r="D92" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" s="50" t="s">
+        <v>41</v>
+      </c>
       <c r="B93" s="7"/>
-      <c r="C93" s="7"/>
-    </row>
-    <row r="94" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C93" s="7">
+        <v>45990</v>
+      </c>
+      <c r="D93" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" s="50" t="s">
+        <v>22</v>
+      </c>
       <c r="B94" s="7"/>
-      <c r="C94" s="7"/>
-    </row>
-    <row r="95" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C94" s="7">
+        <v>46652</v>
+      </c>
+      <c r="D94" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+      <c r="E94" s="59" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" s="50" t="s">
+        <v>42</v>
+      </c>
       <c r="B95" s="7"/>
-      <c r="C95" s="7"/>
-    </row>
-    <row r="96" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B96" s="7"/>
-      <c r="C96" s="7"/>
-    </row>
-    <row r="97" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C95" s="7">
+        <v>47436</v>
+      </c>
+      <c r="D95" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="50" t="s">
+        <v>23</v>
+      </c>
+      <c r="B96" s="9"/>
+      <c r="C96" s="9">
+        <v>48337</v>
+      </c>
+      <c r="D96" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" s="50" t="s">
+        <v>43</v>
+      </c>
       <c r="B97" s="7"/>
-      <c r="C97" s="7"/>
-    </row>
-    <row r="98" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C97" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D97" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" s="50" t="s">
+        <v>24</v>
+      </c>
       <c r="B98" s="7"/>
-      <c r="C98" s="7"/>
-    </row>
-    <row r="99" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C98" s="7">
+        <v>48681</v>
+      </c>
+      <c r="D98" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" s="50" t="s">
+        <v>44</v>
+      </c>
       <c r="B99" s="7"/>
-      <c r="C99" s="7"/>
-    </row>
-    <row r="100" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C99" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D99" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" s="50" t="s">
+        <v>25</v>
+      </c>
       <c r="B100" s="7"/>
-      <c r="C100" s="7"/>
-    </row>
-    <row r="101" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C100" s="7">
+        <v>49683</v>
+      </c>
+      <c r="D100" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" s="50" t="s">
+        <v>26</v>
+      </c>
       <c r="B101" s="7"/>
-      <c r="C101" s="7"/>
-    </row>
-    <row r="102" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="C101" s="7">
+        <v>50244</v>
+      </c>
+      <c r="D101" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B102" s="7"/>
       <c r="C102" s="7"/>
     </row>
-    <row r="103" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B103" s="7"/>
       <c r="C103" s="7"/>
     </row>
-    <row r="104" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B104" s="7"/>
       <c r="C104" s="7"/>
     </row>
-    <row r="105" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B105" s="7"/>
       <c r="C105" s="7"/>
     </row>
-    <row r="106" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B106" s="7"/>
       <c r="C106" s="7"/>
     </row>
-    <row r="107" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B107" s="7"/>
       <c r="C107" s="7"/>
     </row>
-    <row r="108" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B108" s="7"/>
       <c r="C108" s="7"/>
     </row>
-    <row r="109" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
     </row>
-    <row r="110" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
     </row>
-    <row r="111" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
     </row>
-    <row r="112" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
     </row>
-    <row r="113" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B113" s="7"/>
       <c r="C113" s="7"/>
     </row>
-    <row r="114" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B114" s="7"/>
       <c r="C114" s="7"/>
     </row>
-    <row r="115" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B115" s="7"/>
       <c r="C115" s="7"/>
     </row>
-    <row r="116" spans="2:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B116" s="7"/>
       <c r="C116" s="7"/>
+    </row>
+    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B117" s="7"/>
+      <c r="C117" s="7"/>
+    </row>
+    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B118" s="7"/>
+      <c r="C118" s="7"/>
+    </row>
+    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B119" s="7"/>
+      <c r="C119" s="7"/>
+    </row>
+    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B120" s="7"/>
+      <c r="C120" s="7"/>
+    </row>
+    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B121" s="7"/>
+      <c r="C121" s="7"/>
+    </row>
+    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B122" s="7"/>
+      <c r="C122" s="7"/>
+    </row>
+    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B123" s="7"/>
+      <c r="C123" s="7"/>
+    </row>
+    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B124" s="7"/>
+      <c r="C124" s="7"/>
+    </row>
+    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B125" s="7"/>
+      <c r="C125" s="7"/>
+    </row>
+    <row r="126" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B126" s="7"/>
+      <c r="C126" s="7"/>
+    </row>
+    <row r="127" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B127" s="7"/>
+      <c r="C127" s="7"/>
+    </row>
+    <row r="128" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B128" s="7"/>
+      <c r="C128" s="7"/>
+    </row>
+    <row r="129" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B129" s="7"/>
+      <c r="C129" s="7"/>
+    </row>
+    <row r="130" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B130" s="7"/>
+      <c r="C130" s="7"/>
+    </row>
+    <row r="131" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B131" s="7"/>
+      <c r="C131" s="7"/>
+    </row>
+    <row r="132" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B132" s="7"/>
+      <c r="C132" s="7"/>
+    </row>
+    <row r="133" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B133" s="7"/>
+      <c r="C133" s="7"/>
+    </row>
+    <row r="134" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B134" s="7"/>
+      <c r="C134" s="7"/>
+    </row>
+    <row r="135" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B135" s="7"/>
+      <c r="C135" s="7"/>
+    </row>
+    <row r="136" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B136" s="7"/>
+      <c r="C136" s="7"/>
+    </row>
+    <row r="137" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B137" s="7"/>
+      <c r="C137" s="7"/>
+    </row>
+    <row r="138" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B138" s="7"/>
+      <c r="C138" s="7"/>
+    </row>
+    <row r="139" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B139" s="7"/>
+      <c r="C139" s="7"/>
+    </row>
+    <row r="140" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B140" s="7"/>
+      <c r="C140" s="7"/>
+    </row>
+    <row r="141" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B141" s="7"/>
+      <c r="C141" s="7"/>
+    </row>
+    <row r="142" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B142" s="7"/>
+      <c r="C142" s="7"/>
+    </row>
+    <row r="143" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B143" s="7"/>
+      <c r="C143" s="7"/>
+    </row>
+    <row r="144" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B144" s="7"/>
+      <c r="C144" s="7"/>
+    </row>
+    <row r="145" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B145" s="7"/>
+      <c r="C145" s="7"/>
+    </row>
+    <row r="146" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B146" s="7"/>
+      <c r="C146" s="7"/>
+    </row>
+    <row r="147" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B147" s="7"/>
+      <c r="C147" s="7"/>
+    </row>
+    <row r="148" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B148" s="7"/>
+      <c r="C148" s="7"/>
+    </row>
+    <row r="149" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B149" s="7"/>
+      <c r="C149" s="7"/>
+    </row>
+    <row r="150" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B150" s="7"/>
+      <c r="C150" s="7"/>
+    </row>
+    <row r="151" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B151" s="7"/>
+      <c r="C151" s="7"/>
+    </row>
+    <row r="152" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B152" s="7"/>
+      <c r="C152" s="7"/>
+    </row>
+    <row r="153" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B153" s="7"/>
+      <c r="C153" s="7"/>
+    </row>
+    <row r="154" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B154" s="7"/>
+      <c r="C154" s="7"/>
+    </row>
+    <row r="155" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B155" s="7"/>
+      <c r="C155" s="7"/>
+    </row>
+    <row r="156" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B156" s="7"/>
+      <c r="C156" s="7"/>
+    </row>
+    <row r="157" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B157" s="7"/>
+      <c r="C157" s="7"/>
+    </row>
+    <row r="158" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B158" s="7"/>
+      <c r="C158" s="7"/>
+    </row>
+    <row r="159" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B159" s="7"/>
+      <c r="C159" s="7"/>
+    </row>
+    <row r="160" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B160" s="7"/>
+      <c r="C160" s="7"/>
+    </row>
+    <row r="161" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B161" s="7"/>
+      <c r="C161" s="7"/>
+    </row>
+    <row r="162" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B162" s="7"/>
+      <c r="C162" s="7"/>
+    </row>
+    <row r="163" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B163" s="7"/>
+      <c r="C163" s="7"/>
+    </row>
+    <row r="164" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B164" s="7"/>
+      <c r="C164" s="7"/>
+    </row>
+    <row r="165" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B165" s="7"/>
+      <c r="C165" s="7"/>
+    </row>
+    <row r="166" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B166" s="7"/>
+      <c r="C166" s="7"/>
+    </row>
+    <row r="167" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B167" s="7"/>
+      <c r="C167" s="7"/>
+    </row>
+    <row r="168" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B168" s="7"/>
+      <c r="C168" s="7"/>
+    </row>
+    <row r="169" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B169" s="7"/>
+      <c r="C169" s="7"/>
+    </row>
+    <row r="170" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B170" s="7"/>
+      <c r="C170" s="7"/>
+    </row>
+    <row r="171" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B171" s="7"/>
+      <c r="C171" s="7"/>
+    </row>
+    <row r="172" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B172" s="7"/>
+      <c r="C172" s="7"/>
+    </row>
+    <row r="173" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B173" s="7"/>
+      <c r="C173" s="7"/>
+    </row>
+    <row r="174" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B174" s="7"/>
+      <c r="C174" s="7"/>
+    </row>
+    <row r="175" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B175" s="7"/>
+      <c r="C175" s="7"/>
+    </row>
+    <row r="176" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B176" s="7"/>
+      <c r="C176" s="7"/>
+    </row>
+    <row r="177" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B177" s="7"/>
+      <c r="C177" s="7"/>
+    </row>
+    <row r="178" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B178" s="7"/>
+      <c r="C178" s="7"/>
+    </row>
+    <row r="179" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B179" s="7"/>
+      <c r="C179" s="7"/>
+    </row>
+    <row r="180" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B180" s="7"/>
+      <c r="C180" s="7"/>
+    </row>
+    <row r="181" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B181" s="7"/>
+      <c r="C181" s="7"/>
+    </row>
+    <row r="182" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B182" s="7"/>
+      <c r="C182" s="7"/>
+    </row>
+    <row r="183" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B183" s="7"/>
+      <c r="C183" s="7"/>
+    </row>
+    <row r="184" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B184" s="7"/>
+      <c r="C184" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3121,1967 +3954,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E200"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="8.75" customWidth="1"/>
-    <col min="4" max="4" width="6.625" customWidth="1"/>
-    <col min="5" max="5" width="17.625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>388</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>387</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2" s="50" t="s">
-        <v>389</v>
-      </c>
-      <c r="B2" s="2">
-        <v>428</v>
-      </c>
-      <c r="C2" s="2">
-        <v>427</v>
-      </c>
-      <c r="D2" s="3">
-        <f t="shared" ref="D2:D31" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
-        <v>-1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A3" s="50" t="s">
-        <v>392</v>
-      </c>
-      <c r="B3" s="2">
-        <v>759</v>
-      </c>
-      <c r="C3" s="2">
-        <v>758</v>
-      </c>
-      <c r="D3" s="3">
-        <f t="shared" si="0"/>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A4" s="50" t="s">
-        <v>391</v>
-      </c>
-      <c r="B4" s="2">
-        <v>1089</v>
-      </c>
-      <c r="C4" s="2">
-        <v>1107</v>
-      </c>
-      <c r="D4" s="3">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A5" s="50" t="s">
-        <v>390</v>
-      </c>
-      <c r="B5" s="2">
-        <v>1574</v>
-      </c>
-      <c r="C5" s="2">
-        <v>1602</v>
-      </c>
-      <c r="D5" s="3">
-        <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A6" s="50" t="s">
-        <v>393</v>
-      </c>
-      <c r="B6" s="2">
-        <v>1923</v>
-      </c>
-      <c r="C6" s="2">
-        <v>1950</v>
-      </c>
-      <c r="D6" s="3">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A7" s="50"/>
-      <c r="B7" s="2">
-        <v>2023</v>
-      </c>
-      <c r="C7" s="2">
-        <v>2052</v>
-      </c>
-      <c r="D7" s="3">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A8" s="50"/>
-      <c r="B8" s="2">
-        <v>2052</v>
-      </c>
-      <c r="C8" s="2">
-        <v>2080</v>
-      </c>
-      <c r="D8" s="3">
-        <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="50"/>
-      <c r="B9" s="2">
-        <v>2209</v>
-      </c>
-      <c r="C9" s="2">
-        <v>2244</v>
-      </c>
-      <c r="D9" s="3">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A10" s="50" t="s">
-        <v>251</v>
-      </c>
-      <c r="B10" s="2">
-        <v>2334</v>
-      </c>
-      <c r="C10" s="2">
-        <v>2371</v>
-      </c>
-      <c r="D10" s="3">
-        <f t="shared" si="0"/>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11" s="50" t="s">
-        <v>394</v>
-      </c>
-      <c r="B11" s="7">
-        <v>2683</v>
-      </c>
-      <c r="C11" s="7">
-        <v>2719</v>
-      </c>
-      <c r="D11" s="3">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="50" t="s">
-        <v>253</v>
-      </c>
-      <c r="B12" s="7">
-        <v>3132</v>
-      </c>
-      <c r="C12" s="7">
-        <v>3195</v>
-      </c>
-      <c r="D12" s="3">
-        <f t="shared" si="0"/>
-        <v>63</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13" s="50" t="s">
-        <v>395</v>
-      </c>
-      <c r="B13" s="7">
-        <v>3479</v>
-      </c>
-      <c r="C13" s="7">
-        <v>3543</v>
-      </c>
-      <c r="D13" s="3">
-        <f t="shared" si="0"/>
-        <v>64</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" s="50"/>
-      <c r="B14" s="7">
-        <v>3548</v>
-      </c>
-      <c r="C14" s="7">
-        <v>3612</v>
-      </c>
-      <c r="D14" s="3">
-        <f t="shared" si="0"/>
-        <v>64</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="50"/>
-      <c r="B15" s="7">
-        <v>3640</v>
-      </c>
-      <c r="C15" s="7">
-        <v>3704</v>
-      </c>
-      <c r="D15" s="3">
-        <f t="shared" si="0"/>
-        <v>64</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A16" s="50" t="s">
-        <v>255</v>
-      </c>
-      <c r="B16" s="7">
-        <v>3761</v>
-      </c>
-      <c r="C16" s="7">
-        <v>3829</v>
-      </c>
-      <c r="D16" s="3">
-        <f t="shared" si="0"/>
-        <v>68</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A17" s="50" t="s">
-        <v>396</v>
-      </c>
-      <c r="B17" s="7">
-        <v>4109</v>
-      </c>
-      <c r="C17" s="7">
-        <v>4178</v>
-      </c>
-      <c r="D17" s="3">
-        <f t="shared" si="0"/>
-        <v>69</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" s="50"/>
-      <c r="B18" s="7">
-        <v>4509</v>
-      </c>
-      <c r="C18" s="7">
-        <v>4574</v>
-      </c>
-      <c r="D18" s="3">
-        <f t="shared" si="0"/>
-        <v>65</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A19" s="50"/>
-      <c r="B19" s="7">
-        <v>4669</v>
-      </c>
-      <c r="C19" s="7">
-        <v>4731</v>
-      </c>
-      <c r="D19" s="3">
-        <f t="shared" si="0"/>
-        <v>62</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A20" s="50"/>
-      <c r="B20" s="7">
-        <v>4727</v>
-      </c>
-      <c r="C20" s="7">
-        <v>4791</v>
-      </c>
-      <c r="D20" s="3">
-        <f t="shared" si="0"/>
-        <v>64</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A21" s="50"/>
-      <c r="B21" s="7">
-        <v>4866</v>
-      </c>
-      <c r="C21" s="7">
-        <v>4926</v>
-      </c>
-      <c r="D21" s="3">
-        <f t="shared" si="0"/>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A22" s="50"/>
-      <c r="B22" s="7">
-        <v>4953</v>
-      </c>
-      <c r="C22" s="7">
-        <v>5011</v>
-      </c>
-      <c r="D22" s="3">
-        <f t="shared" si="0"/>
-        <v>58</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A23" s="50" t="s">
-        <v>257</v>
-      </c>
-      <c r="B23" s="7">
-        <v>5125</v>
-      </c>
-      <c r="C23" s="37">
-        <v>5190</v>
-      </c>
-      <c r="D23" s="3">
-        <f t="shared" si="0"/>
-        <v>65</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A24" s="50" t="s">
-        <v>397</v>
-      </c>
-      <c r="B24" s="7">
-        <v>5474</v>
-      </c>
-      <c r="C24" s="7">
-        <v>5539</v>
-      </c>
-      <c r="D24" s="3">
-        <f t="shared" si="0"/>
-        <v>65</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A25" s="50" t="s">
-        <v>259</v>
-      </c>
-      <c r="B25" s="7">
-        <v>5936</v>
-      </c>
-      <c r="C25" s="7">
-        <v>6003</v>
-      </c>
-      <c r="D25" s="3">
-        <f t="shared" si="0"/>
-        <v>67</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A26" s="50" t="s">
-        <v>410</v>
-      </c>
-      <c r="B26" s="7">
-        <v>6287</v>
-      </c>
-      <c r="C26" s="7">
-        <v>6352</v>
-      </c>
-      <c r="D26" s="3">
-        <f t="shared" si="0"/>
-        <v>65</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A27" s="50"/>
-      <c r="B27" s="7">
-        <v>6410</v>
-      </c>
-      <c r="C27" s="7">
-        <v>6476</v>
-      </c>
-      <c r="D27" s="3">
-        <f t="shared" si="0"/>
-        <v>66</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A28" s="50"/>
-      <c r="B28" s="7">
-        <v>6446</v>
-      </c>
-      <c r="C28" s="7">
-        <v>6512</v>
-      </c>
-      <c r="D28" s="3">
-        <f t="shared" si="0"/>
-        <v>66</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A29" s="50"/>
-      <c r="B29" s="7">
-        <v>6590</v>
-      </c>
-      <c r="C29" s="7">
-        <v>6657</v>
-      </c>
-      <c r="D29" s="3">
-        <f t="shared" si="0"/>
-        <v>67</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A30" s="50" t="s">
-        <v>267</v>
-      </c>
-      <c r="B30" s="7">
-        <v>6690</v>
-      </c>
-      <c r="C30" s="7">
-        <v>6759</v>
-      </c>
-      <c r="D30" s="3">
-        <f t="shared" si="0"/>
-        <v>69</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A31" s="50" t="s">
-        <v>398</v>
-      </c>
-      <c r="B31" s="7">
-        <v>7039</v>
-      </c>
-      <c r="C31" s="7">
-        <v>7106</v>
-      </c>
-      <c r="D31" s="3">
-        <f t="shared" si="0"/>
-        <v>67</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A32" s="50" t="s">
-        <v>274</v>
-      </c>
-      <c r="B32" s="7">
-        <v>8127</v>
-      </c>
-      <c r="C32" s="7">
-        <v>8196</v>
-      </c>
-      <c r="D32" s="3">
-        <f t="shared" ref="D32:D66" si="1">IF(C32&lt;&gt;"",IF(B32&lt;&gt;"",C32-B32,"-"), "-")</f>
-        <v>69</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A33" s="50" t="s">
-        <v>399</v>
-      </c>
-      <c r="B33" s="7">
-        <v>8527</v>
-      </c>
-      <c r="C33" s="7">
-        <v>8549</v>
-      </c>
-      <c r="D33" s="3">
-        <f t="shared" si="1"/>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A34" s="50" t="s">
-        <v>276</v>
-      </c>
-      <c r="B34" s="7">
-        <v>9099</v>
-      </c>
-      <c r="C34" s="7">
-        <v>9118</v>
-      </c>
-      <c r="D34" s="3">
-        <f t="shared" si="1"/>
-        <v>19</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A35" s="50" t="s">
-        <v>400</v>
-      </c>
-      <c r="B35" s="7">
-        <v>9447</v>
-      </c>
-      <c r="C35" s="7">
-        <v>9467</v>
-      </c>
-      <c r="D35" s="3">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A36" s="50" t="s">
-        <v>278</v>
-      </c>
-      <c r="B36" s="7">
-        <v>9758</v>
-      </c>
-      <c r="C36" s="7">
-        <v>9778</v>
-      </c>
-      <c r="D36" s="3">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A37" s="50" t="s">
-        <v>401</v>
-      </c>
-      <c r="B37" s="7">
-        <v>10104</v>
-      </c>
-      <c r="C37" s="7">
-        <v>10125</v>
-      </c>
-      <c r="D37" s="3">
-        <f t="shared" si="1"/>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A38" s="51" t="s">
-        <v>127</v>
-      </c>
-      <c r="B38" s="7">
-        <v>10305</v>
-      </c>
-      <c r="C38" s="7">
-        <v>10328</v>
-      </c>
-      <c r="D38" s="3">
-        <f t="shared" ref="D38" si="2">IF(C38&lt;&gt;"",IF(B38&lt;&gt;"",C38-B38,"-"), "-")</f>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A39" s="51" t="s">
-        <v>426</v>
-      </c>
-      <c r="B39" s="7">
-        <v>10532</v>
-      </c>
-      <c r="C39" s="7">
-        <v>10557</v>
-      </c>
-      <c r="D39" s="3">
-        <f t="shared" si="1"/>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A40" s="51" t="s">
-        <v>425</v>
-      </c>
-      <c r="B40" s="7">
-        <v>10574</v>
-      </c>
-      <c r="C40" s="7">
-        <v>10589</v>
-      </c>
-      <c r="D40" s="3">
-        <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A41" s="50" t="s">
-        <v>281</v>
-      </c>
-      <c r="B41" s="7">
-        <v>10743</v>
-      </c>
-      <c r="C41" s="7">
-        <v>10816</v>
-      </c>
-      <c r="D41" s="3">
-        <f t="shared" si="1"/>
-        <v>73</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A42" s="50" t="s">
-        <v>402</v>
-      </c>
-      <c r="B42" s="7">
-        <v>11094</v>
-      </c>
-      <c r="C42" s="7">
-        <v>11163</v>
-      </c>
-      <c r="D42" s="3">
-        <f t="shared" si="1"/>
-        <v>69</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A43" s="50" t="s">
-        <v>283</v>
-      </c>
-      <c r="B43" s="7">
-        <v>11652</v>
-      </c>
-      <c r="C43" s="7">
-        <v>11729</v>
-      </c>
-      <c r="D43" s="3">
-        <f t="shared" si="1"/>
-        <v>77</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A44" s="50" t="s">
-        <v>403</v>
-      </c>
-      <c r="B44" s="7">
-        <v>12308</v>
-      </c>
-      <c r="C44" s="7">
-        <v>12383</v>
-      </c>
-      <c r="D44" s="3">
-        <f t="shared" si="1"/>
-        <v>75</v>
-      </c>
-      <c r="E44" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="50" t="s">
-        <v>285</v>
-      </c>
-      <c r="B45" s="7">
-        <v>12768</v>
-      </c>
-      <c r="C45" s="7">
-        <v>12891</v>
-      </c>
-      <c r="D45" s="3">
-        <f t="shared" si="1"/>
-        <v>123</v>
-      </c>
-      <c r="E45" s="7">
-        <v>12815</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="50" t="s">
-        <v>404</v>
-      </c>
-      <c r="B46" s="7">
-        <v>13120</v>
-      </c>
-      <c r="C46" s="7">
-        <v>13236</v>
-      </c>
-      <c r="D46" s="3">
-        <f t="shared" si="1"/>
-        <v>116</v>
-      </c>
-      <c r="E46" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="50" t="s">
-        <v>288</v>
-      </c>
-      <c r="B47" s="7"/>
-      <c r="C47" s="7">
-        <v>13960</v>
-      </c>
-      <c r="D47" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="50" t="s">
-        <v>405</v>
-      </c>
-      <c r="B48" s="7"/>
-      <c r="C48" s="7">
-        <v>14320</v>
-      </c>
-      <c r="D48" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A49" s="50" t="s">
-        <v>294</v>
-      </c>
-      <c r="B49" s="7"/>
-      <c r="C49" s="7">
-        <v>14679</v>
-      </c>
-      <c r="D49" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A50" s="50" t="s">
-        <v>406</v>
-      </c>
-      <c r="B50" s="7"/>
-      <c r="C50" s="7">
-        <v>15029</v>
-      </c>
-      <c r="D50" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A51" s="50" t="s">
-        <v>297</v>
-      </c>
-      <c r="B51" s="7"/>
-      <c r="C51" s="7">
-        <v>15850</v>
-      </c>
-      <c r="D51" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A52" s="50" t="s">
-        <v>407</v>
-      </c>
-      <c r="B52" s="7"/>
-      <c r="C52" s="7">
-        <v>16200</v>
-      </c>
-      <c r="D52" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A53" s="50" t="s">
-        <v>301</v>
-      </c>
-      <c r="B53" s="33"/>
-      <c r="C53" s="33">
-        <v>17135</v>
-      </c>
-      <c r="D53" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A54" s="50" t="s">
-        <v>408</v>
-      </c>
-      <c r="B54" s="7"/>
-      <c r="C54" s="7">
-        <v>17485</v>
-      </c>
-      <c r="D54" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A55" s="50" t="s">
-        <v>305</v>
-      </c>
-      <c r="B55" s="7"/>
-      <c r="C55" s="7">
-        <v>17791</v>
-      </c>
-      <c r="D55" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A56" s="50" t="s">
-        <v>409</v>
-      </c>
-      <c r="B56" s="7"/>
-      <c r="C56" s="37">
-        <v>18139</v>
-      </c>
-      <c r="D56" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A57" s="50" t="s">
-        <v>308</v>
-      </c>
-      <c r="B57" s="7"/>
-      <c r="C57" s="7">
-        <v>18719</v>
-      </c>
-      <c r="D57" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A58" s="50" t="s">
-        <v>411</v>
-      </c>
-      <c r="B58" s="7"/>
-      <c r="C58" s="7">
-        <v>19068</v>
-      </c>
-      <c r="D58" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A59" s="50" t="s">
-        <v>314</v>
-      </c>
-      <c r="B59" s="7"/>
-      <c r="C59" s="7">
-        <v>19892</v>
-      </c>
-      <c r="D59" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A60" s="50" t="s">
-        <v>412</v>
-      </c>
-      <c r="B60" s="7"/>
-      <c r="C60" s="7">
-        <v>20240</v>
-      </c>
-      <c r="D60" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A61" s="50" t="s">
-        <v>320</v>
-      </c>
-      <c r="B61" s="7"/>
-      <c r="C61" s="7">
-        <v>20813</v>
-      </c>
-      <c r="D61" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="E61" s="7"/>
-    </row>
-    <row r="62" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A62" s="50" t="s">
-        <v>413</v>
-      </c>
-      <c r="B62" s="7"/>
-      <c r="C62" s="7">
-        <v>21161</v>
-      </c>
-      <c r="D62" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-      <c r="E62" s="7"/>
-    </row>
-    <row r="63" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A63" s="50" t="s">
-        <v>322</v>
-      </c>
-      <c r="B63" s="7"/>
-      <c r="C63" s="7">
-        <v>22195</v>
-      </c>
-      <c r="D63" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A64" s="50" t="s">
-        <v>414</v>
-      </c>
-      <c r="B64" s="7"/>
-      <c r="C64" s="7">
-        <v>22543</v>
-      </c>
-      <c r="D64" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A65" s="50" t="s">
-        <v>324</v>
-      </c>
-      <c r="B65" s="7"/>
-      <c r="C65" s="7">
-        <v>22963</v>
-      </c>
-      <c r="D65" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A66" s="50" t="s">
-        <v>415</v>
-      </c>
-      <c r="B66" s="7"/>
-      <c r="C66" s="7">
-        <v>23346</v>
-      </c>
-      <c r="D66" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A67" s="50" t="s">
-        <v>416</v>
-      </c>
-      <c r="B67" s="7"/>
-      <c r="C67" s="7">
-        <v>23873</v>
-      </c>
-      <c r="D67" s="3" t="str">
-        <f t="shared" ref="D67:D96" si="3">IF(C67&lt;&gt;"",IF(B67&lt;&gt;"",C67-B67,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A68" s="50" t="s">
-        <v>417</v>
-      </c>
-      <c r="B68" s="8"/>
-      <c r="C68" s="50">
-        <v>24221</v>
-      </c>
-      <c r="D68" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A69" s="50" t="s">
-        <v>418</v>
-      </c>
-      <c r="B69" s="33"/>
-      <c r="C69" s="33">
-        <v>25101</v>
-      </c>
-      <c r="D69" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A70" s="50" t="s">
-        <v>419</v>
-      </c>
-      <c r="B70" s="7"/>
-      <c r="C70" s="7">
-        <v>25450</v>
-      </c>
-      <c r="D70" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A71" s="50" t="s">
-        <v>420</v>
-      </c>
-      <c r="B71" s="7"/>
-      <c r="C71" s="7">
-        <v>26350</v>
-      </c>
-      <c r="D71" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A72" s="50" t="s">
-        <v>421</v>
-      </c>
-      <c r="B72" s="7"/>
-      <c r="C72" s="7">
-        <v>26699</v>
-      </c>
-      <c r="D72" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A73" s="50" t="s">
-        <v>332</v>
-      </c>
-      <c r="B73" s="7"/>
-      <c r="C73" s="7">
-        <v>27490</v>
-      </c>
-      <c r="D73" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A74" s="50" t="s">
-        <v>5</v>
-      </c>
-      <c r="B74" s="7"/>
-      <c r="C74" s="7">
-        <v>27836</v>
-      </c>
-      <c r="D74" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A75" s="50" t="s">
-        <v>337</v>
-      </c>
-      <c r="B75" s="7"/>
-      <c r="C75" s="7">
-        <v>28899</v>
-      </c>
-      <c r="D75" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A76" s="50" t="s">
-        <v>6</v>
-      </c>
-      <c r="B76" s="7"/>
-      <c r="C76" s="7">
-        <v>29248</v>
-      </c>
-      <c r="D76" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A77" s="50" t="s">
-        <v>45</v>
-      </c>
-      <c r="B77" s="7"/>
-      <c r="C77" s="7">
-        <v>29962</v>
-      </c>
-      <c r="D77" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A78" s="50" t="s">
-        <v>7</v>
-      </c>
-      <c r="B78" s="7"/>
-      <c r="C78" s="7">
-        <v>30309</v>
-      </c>
-      <c r="D78" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A79" s="50" t="s">
-        <v>46</v>
-      </c>
-      <c r="B79" s="7"/>
-      <c r="C79" s="7">
-        <v>30479</v>
-      </c>
-      <c r="D79" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A80" s="50" t="s">
-        <v>8</v>
-      </c>
-      <c r="B80" s="7"/>
-      <c r="C80" s="7">
-        <v>31125</v>
-      </c>
-      <c r="D80" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-      <c r="E80" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A81" s="50" t="s">
-        <v>28</v>
-      </c>
-      <c r="B81" s="7"/>
-      <c r="C81" s="7">
-        <v>31643</v>
-      </c>
-      <c r="D81" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A82" s="50" t="s">
-        <v>9</v>
-      </c>
-      <c r="B82" s="7"/>
-      <c r="C82" s="7">
-        <v>31991</v>
-      </c>
-      <c r="D82" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A83" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="B83" s="7"/>
-      <c r="C83" s="7">
-        <v>32586</v>
-      </c>
-      <c r="D83" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A84" s="50" t="s">
-        <v>10</v>
-      </c>
-      <c r="B84" s="7"/>
-      <c r="C84" s="7">
-        <v>33254</v>
-      </c>
-      <c r="D84" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-      <c r="E84" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A85" s="50" t="s">
-        <v>31</v>
-      </c>
-      <c r="B85" s="7"/>
-      <c r="C85" s="7">
-        <v>33883</v>
-      </c>
-      <c r="D85" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A86" s="50" t="s">
-        <v>11</v>
-      </c>
-      <c r="B86" s="7"/>
-      <c r="C86" s="7">
-        <v>34244</v>
-      </c>
-      <c r="D86" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A87" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="B87" s="7"/>
-      <c r="C87" s="7">
-        <v>34862</v>
-      </c>
-      <c r="D87" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A88" s="50" t="s">
-        <v>12</v>
-      </c>
-      <c r="B88" s="7"/>
-      <c r="C88" s="7">
-        <v>35218</v>
-      </c>
-      <c r="D88" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A89" s="50" t="s">
-        <v>32</v>
-      </c>
-      <c r="B89" s="7"/>
-      <c r="C89" s="7">
-        <v>35772</v>
-      </c>
-      <c r="D89" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A90" s="50" t="s">
-        <v>13</v>
-      </c>
-      <c r="B90" s="7"/>
-      <c r="C90" s="7">
-        <v>36120</v>
-      </c>
-      <c r="D90" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A91" s="50" t="s">
-        <v>47</v>
-      </c>
-      <c r="B91" s="7"/>
-      <c r="C91" s="7">
-        <v>36893</v>
-      </c>
-      <c r="D91" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A92" s="50" t="s">
-        <v>48</v>
-      </c>
-      <c r="B92" s="7"/>
-      <c r="C92" s="7">
-        <v>37238</v>
-      </c>
-      <c r="D92" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A93" s="50" t="s">
-        <v>33</v>
-      </c>
-      <c r="B93" s="7"/>
-      <c r="C93" s="7">
-        <v>38097</v>
-      </c>
-      <c r="D93" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A94" s="50" t="s">
-        <v>14</v>
-      </c>
-      <c r="B94" s="7"/>
-      <c r="C94" s="7">
-        <v>38443</v>
-      </c>
-      <c r="D94" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A95" s="50" t="s">
-        <v>34</v>
-      </c>
-      <c r="B95" s="7"/>
-      <c r="C95" s="7">
-        <v>38692</v>
-      </c>
-      <c r="D95" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A96" s="50" t="s">
-        <v>15</v>
-      </c>
-      <c r="B96" s="7"/>
-      <c r="C96" s="7">
-        <v>39041</v>
-      </c>
-      <c r="D96" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A97" s="50" t="s">
-        <v>35</v>
-      </c>
-      <c r="B97" s="7"/>
-      <c r="C97" s="7">
-        <v>40011</v>
-      </c>
-      <c r="D97" s="3" t="str">
-        <f>IF(C96&lt;&gt;"",IF(B96&lt;&gt;"",C96-B96,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A98" s="50" t="s">
-        <v>16</v>
-      </c>
-      <c r="B98" s="7"/>
-      <c r="C98" s="7">
-        <v>40373</v>
-      </c>
-      <c r="D98" s="3" t="str">
-        <f t="shared" ref="D98:D117" si="4">IF(C98&lt;&gt;"",IF(B98&lt;&gt;"",C98-B98,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A99" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B99" s="40"/>
-      <c r="C99" s="7">
-        <v>41117</v>
-      </c>
-      <c r="D99" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A100" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="B100" s="7"/>
-      <c r="C100" s="7">
-        <v>41465</v>
-      </c>
-      <c r="D100" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A101" s="50" t="s">
-        <v>37</v>
-      </c>
-      <c r="B101" s="7"/>
-      <c r="C101" s="7">
-        <v>42450</v>
-      </c>
-      <c r="D101" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A102" s="50" t="s">
-        <v>18</v>
-      </c>
-      <c r="B102" s="7"/>
-      <c r="C102" s="7">
-        <v>42799</v>
-      </c>
-      <c r="D102" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A103" s="50" t="s">
-        <v>38</v>
-      </c>
-      <c r="B103" s="7"/>
-      <c r="C103" s="7">
-        <v>43144</v>
-      </c>
-      <c r="D103" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A104" s="50" t="s">
-        <v>19</v>
-      </c>
-      <c r="B104" s="7"/>
-      <c r="C104" s="7">
-        <v>43491</v>
-      </c>
-      <c r="D104" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A105" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="B105" s="7"/>
-      <c r="C105" s="7">
-        <v>44165</v>
-      </c>
-      <c r="D105" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A106" s="50" t="s">
-        <v>20</v>
-      </c>
-      <c r="B106" s="7"/>
-      <c r="C106" s="7">
-        <v>44512</v>
-      </c>
-      <c r="D106" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A107" s="50" t="s">
-        <v>40</v>
-      </c>
-      <c r="B107" s="7"/>
-      <c r="C107" s="7">
-        <v>45061</v>
-      </c>
-      <c r="D107" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A108" s="50" t="s">
-        <v>21</v>
-      </c>
-      <c r="B108" s="7"/>
-      <c r="C108" s="7">
-        <v>45443</v>
-      </c>
-      <c r="D108" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A109" s="50" t="s">
-        <v>41</v>
-      </c>
-      <c r="B109" s="7"/>
-      <c r="C109" s="7">
-        <v>45990</v>
-      </c>
-      <c r="D109" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A110" s="50" t="s">
-        <v>22</v>
-      </c>
-      <c r="B110" s="7"/>
-      <c r="C110" s="7">
-        <v>46652</v>
-      </c>
-      <c r="D110" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-      <c r="E110" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A111" s="50" t="s">
-        <v>42</v>
-      </c>
-      <c r="B111" s="7"/>
-      <c r="C111" s="7">
-        <v>47436</v>
-      </c>
-      <c r="D111" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A112" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B112" s="9"/>
-      <c r="C112" s="9">
-        <v>48337</v>
-      </c>
-      <c r="D112" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A113" s="50" t="s">
-        <v>43</v>
-      </c>
-      <c r="B113" s="7"/>
-      <c r="C113" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D113" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A114" s="50" t="s">
-        <v>24</v>
-      </c>
-      <c r="B114" s="7"/>
-      <c r="C114" s="7">
-        <v>48681</v>
-      </c>
-      <c r="D114" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A115" s="50" t="s">
-        <v>44</v>
-      </c>
-      <c r="B115" s="7"/>
-      <c r="C115" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D115" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A116" s="50" t="s">
-        <v>25</v>
-      </c>
-      <c r="B116" s="7"/>
-      <c r="C116" s="7">
-        <v>49683</v>
-      </c>
-      <c r="D116" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A117" s="50" t="s">
-        <v>26</v>
-      </c>
-      <c r="B117" s="7"/>
-      <c r="C117" s="7">
-        <v>50244</v>
-      </c>
-      <c r="D117" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B118" s="7"/>
-      <c r="C118" s="7"/>
-    </row>
-    <row r="119" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B119" s="7"/>
-      <c r="C119" s="7"/>
-    </row>
-    <row r="120" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B120" s="7"/>
-      <c r="C120" s="7"/>
-    </row>
-    <row r="121" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B121" s="7"/>
-      <c r="C121" s="7"/>
-    </row>
-    <row r="122" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B122" s="7"/>
-      <c r="C122" s="7"/>
-    </row>
-    <row r="123" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B123" s="7"/>
-      <c r="C123" s="7"/>
-    </row>
-    <row r="124" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B124" s="7"/>
-      <c r="C124" s="7"/>
-    </row>
-    <row r="125" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B125" s="7"/>
-      <c r="C125" s="7"/>
-    </row>
-    <row r="126" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B126" s="7"/>
-      <c r="C126" s="7"/>
-    </row>
-    <row r="127" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B127" s="7"/>
-      <c r="C127" s="7"/>
-    </row>
-    <row r="128" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="B128" s="7"/>
-      <c r="C128" s="7"/>
-    </row>
-    <row r="129" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B129" s="7"/>
-      <c r="C129" s="7"/>
-    </row>
-    <row r="130" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B130" s="7"/>
-      <c r="C130" s="7"/>
-    </row>
-    <row r="131" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B131" s="7"/>
-      <c r="C131" s="7"/>
-    </row>
-    <row r="132" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B132" s="7"/>
-      <c r="C132" s="7"/>
-    </row>
-    <row r="133" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B133" s="7"/>
-      <c r="C133" s="7"/>
-    </row>
-    <row r="134" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B134" s="7"/>
-      <c r="C134" s="7"/>
-    </row>
-    <row r="135" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B135" s="7"/>
-      <c r="C135" s="7"/>
-    </row>
-    <row r="136" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B136" s="7"/>
-      <c r="C136" s="7"/>
-    </row>
-    <row r="137" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B137" s="7"/>
-      <c r="C137" s="7"/>
-    </row>
-    <row r="138" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B138" s="7"/>
-      <c r="C138" s="7"/>
-    </row>
-    <row r="139" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B139" s="7"/>
-      <c r="C139" s="7"/>
-    </row>
-    <row r="140" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B140" s="7"/>
-      <c r="C140" s="7"/>
-    </row>
-    <row r="141" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B141" s="7"/>
-      <c r="C141" s="7"/>
-    </row>
-    <row r="142" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B142" s="7"/>
-      <c r="C142" s="7"/>
-    </row>
-    <row r="143" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B143" s="7"/>
-      <c r="C143" s="7"/>
-    </row>
-    <row r="144" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B144" s="7"/>
-      <c r="C144" s="7"/>
-    </row>
-    <row r="145" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B145" s="7"/>
-      <c r="C145" s="7"/>
-    </row>
-    <row r="146" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B146" s="7"/>
-      <c r="C146" s="7"/>
-    </row>
-    <row r="147" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B147" s="7"/>
-      <c r="C147" s="7"/>
-    </row>
-    <row r="148" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B148" s="7"/>
-      <c r="C148" s="7"/>
-    </row>
-    <row r="149" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B149" s="7"/>
-      <c r="C149" s="7"/>
-    </row>
-    <row r="150" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B150" s="7"/>
-      <c r="C150" s="7"/>
-    </row>
-    <row r="151" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B151" s="7"/>
-      <c r="C151" s="7"/>
-    </row>
-    <row r="152" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B152" s="7"/>
-      <c r="C152" s="7"/>
-    </row>
-    <row r="153" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B153" s="7"/>
-      <c r="C153" s="7"/>
-    </row>
-    <row r="154" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B154" s="7"/>
-      <c r="C154" s="7"/>
-    </row>
-    <row r="155" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B155" s="7"/>
-      <c r="C155" s="7"/>
-    </row>
-    <row r="156" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B156" s="7"/>
-      <c r="C156" s="7"/>
-    </row>
-    <row r="157" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B157" s="7"/>
-      <c r="C157" s="7"/>
-    </row>
-    <row r="158" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B158" s="7"/>
-      <c r="C158" s="7"/>
-    </row>
-    <row r="159" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B159" s="7"/>
-      <c r="C159" s="7"/>
-    </row>
-    <row r="160" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B160" s="7"/>
-      <c r="C160" s="7"/>
-    </row>
-    <row r="161" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B161" s="7"/>
-      <c r="C161" s="7"/>
-    </row>
-    <row r="162" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B162" s="7"/>
-      <c r="C162" s="7"/>
-    </row>
-    <row r="163" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B163" s="7"/>
-      <c r="C163" s="7"/>
-    </row>
-    <row r="164" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B164" s="7"/>
-      <c r="C164" s="7"/>
-    </row>
-    <row r="165" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B165" s="7"/>
-      <c r="C165" s="7"/>
-    </row>
-    <row r="166" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B166" s="7"/>
-      <c r="C166" s="7"/>
-    </row>
-    <row r="167" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B167" s="7"/>
-      <c r="C167" s="7"/>
-    </row>
-    <row r="168" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B168" s="7"/>
-      <c r="C168" s="7"/>
-    </row>
-    <row r="169" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B169" s="7"/>
-      <c r="C169" s="7"/>
-    </row>
-    <row r="170" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B170" s="7"/>
-      <c r="C170" s="7"/>
-    </row>
-    <row r="171" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B171" s="7"/>
-      <c r="C171" s="7"/>
-    </row>
-    <row r="172" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B172" s="7"/>
-      <c r="C172" s="7"/>
-    </row>
-    <row r="173" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B173" s="7"/>
-      <c r="C173" s="7"/>
-    </row>
-    <row r="174" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B174" s="7"/>
-      <c r="C174" s="7"/>
-    </row>
-    <row r="175" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B175" s="7"/>
-      <c r="C175" s="7"/>
-    </row>
-    <row r="176" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B176" s="7"/>
-      <c r="C176" s="7"/>
-    </row>
-    <row r="177" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B177" s="7"/>
-      <c r="C177" s="7"/>
-    </row>
-    <row r="178" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B178" s="7"/>
-      <c r="C178" s="7"/>
-    </row>
-    <row r="179" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B179" s="7"/>
-      <c r="C179" s="7"/>
-    </row>
-    <row r="180" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B180" s="7"/>
-      <c r="C180" s="7"/>
-    </row>
-    <row r="181" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B181" s="7"/>
-      <c r="C181" s="7"/>
-    </row>
-    <row r="182" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B182" s="7"/>
-      <c r="C182" s="7"/>
-    </row>
-    <row r="183" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B183" s="7"/>
-      <c r="C183" s="7"/>
-    </row>
-    <row r="184" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B184" s="7"/>
-      <c r="C184" s="7"/>
-    </row>
-    <row r="185" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B185" s="7"/>
-      <c r="C185" s="7"/>
-    </row>
-    <row r="186" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B186" s="7"/>
-      <c r="C186" s="7"/>
-    </row>
-    <row r="187" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B187" s="7"/>
-      <c r="C187" s="7"/>
-    </row>
-    <row r="188" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B188" s="7"/>
-      <c r="C188" s="7"/>
-    </row>
-    <row r="189" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B189" s="7"/>
-      <c r="C189" s="7"/>
-    </row>
-    <row r="190" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B190" s="7"/>
-      <c r="C190" s="7"/>
-    </row>
-    <row r="191" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B191" s="7"/>
-      <c r="C191" s="7"/>
-    </row>
-    <row r="192" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B192" s="7"/>
-      <c r="C192" s="7"/>
-    </row>
-    <row r="193" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B193" s="7"/>
-      <c r="C193" s="7"/>
-    </row>
-    <row r="194" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B194" s="7"/>
-      <c r="C194" s="7"/>
-    </row>
-    <row r="195" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B195" s="7"/>
-      <c r="C195" s="7"/>
-    </row>
-    <row r="196" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B196" s="7"/>
-      <c r="C196" s="7"/>
-    </row>
-    <row r="197" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B197" s="7"/>
-      <c r="C197" s="7"/>
-    </row>
-    <row r="198" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B198" s="7"/>
-      <c r="C198" s="7"/>
-    </row>
-    <row r="199" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B199" s="7"/>
-      <c r="C199" s="7"/>
-    </row>
-    <row r="200" spans="2:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="B200" s="7"/>
-      <c r="C200" s="7"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB48F502-AA0A-4BF9-ABA2-AA87E3F2B5E4}">
   <dimension ref="A1:E388"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -9936,7 +8808,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39B3565E-C480-4A10-8524-B7BC06C9B703}">
   <dimension ref="A1:H287"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -13892,7 +12764,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D06DA051-0308-42D5-B7F7-51E79FAF1C31}">
   <dimension ref="A1:F292"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -16435,7 +15307,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B2A8891-531F-43A4-B044-6C02F070C564}">
   <dimension ref="A1:I278"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -18757,7 +17629,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -19922,7 +18794,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="34" type="noConversion"/>
+  <phoneticPr fontId="32" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -19932,7 +18804,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8F82A59-57DF-46F6-BCD0-E7A53E611046}">
   <dimension ref="A1:L54"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -19952,10 +18824,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="53" t="s">
+      <c r="K1" s="51" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="54"/>
+      <c r="L1" s="52"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -21807,13 +20679,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="55" t="s">
+      <c r="H53" s="53" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="56"/>
-      <c r="J53" s="56"/>
-      <c r="K53" s="56"/>
-      <c r="L53" s="57"/>
+      <c r="I53" s="54"/>
+      <c r="J53" s="54"/>
+      <c r="K53" s="54"/>
+      <c r="L53" s="55"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -21835,11 +20707,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="58"/>
-      <c r="I54" s="59"/>
-      <c r="J54" s="59"/>
-      <c r="K54" s="59"/>
-      <c r="L54" s="60"/>
+      <c r="H54" s="56"/>
+      <c r="I54" s="57"/>
+      <c r="J54" s="57"/>
+      <c r="K54" s="57"/>
+      <c r="L54" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - level 17 done - 241 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89B2B36A-42AE-4060-8C33-91EF5B9F4680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E17D81F-62C2-4BD1-A485-941825B01C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="47415" yWindow="3540" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -1879,6 +1879,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1903,7 +1904,6 @@
     <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2230,7 +2230,7 @@
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="8.75" customWidth="1"/>
     <col min="4" max="4" width="6.625" customWidth="1"/>
-    <col min="5" max="5" width="17.625" style="59" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.625" style="51" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2639,7 +2639,7 @@
       <c r="A28" s="50" t="s">
         <v>403</v>
       </c>
-      <c r="B28" s="59">
+      <c r="B28" s="51">
         <v>11928</v>
       </c>
       <c r="C28" s="7">
@@ -2649,7 +2649,7 @@
         <f t="shared" si="1"/>
         <v>455</v>
       </c>
-      <c r="E28" s="59" t="s">
+      <c r="E28" s="51" t="s">
         <v>422</v>
       </c>
     </row>
@@ -2687,52 +2687,60 @@
       <c r="A31" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="B31" s="7"/>
+      <c r="B31" s="7">
+        <v>13719</v>
+      </c>
       <c r="C31" s="7">
         <v>13960</v>
       </c>
-      <c r="D31" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="D31" s="3">
+        <f t="shared" si="1"/>
+        <v>241</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="50" t="s">
         <v>405</v>
       </c>
-      <c r="B32" s="7"/>
+      <c r="B32" s="7">
+        <v>14077</v>
+      </c>
       <c r="C32" s="7">
         <v>14320</v>
       </c>
-      <c r="D32" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="D32" s="3">
+        <f t="shared" si="1"/>
+        <v>243</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="50" t="s">
         <v>294</v>
       </c>
-      <c r="B33" s="7"/>
+      <c r="B33" s="7">
+        <v>14437</v>
+      </c>
       <c r="C33" s="7">
         <v>14679</v>
       </c>
-      <c r="D33" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="D33" s="3">
+        <f t="shared" si="1"/>
+        <v>242</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="50" t="s">
         <v>406</v>
       </c>
-      <c r="B34" s="7"/>
+      <c r="B34" s="7">
+        <v>14788</v>
+      </c>
       <c r="C34" s="7">
         <v>15029</v>
       </c>
-      <c r="D34" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="D34" s="3">
+        <f t="shared" si="1"/>
+        <v>241</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -3124,7 +3132,7 @@
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E64" s="59" t="s">
+      <c r="E64" s="51" t="s">
         <v>422</v>
       </c>
     </row>
@@ -3179,7 +3187,7 @@
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E68" s="59" t="s">
+      <c r="E68" s="51" t="s">
         <v>422</v>
       </c>
     </row>
@@ -3520,7 +3528,7 @@
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E94" s="59" t="s">
+      <c r="E94" s="51" t="s">
         <v>422</v>
       </c>
     </row>
@@ -18824,10 +18832,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="51" t="s">
+      <c r="K1" s="52" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="52"/>
+      <c r="L1" s="53"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -20679,13 +20687,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="53" t="s">
+      <c r="H53" s="54" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="54"/>
-      <c r="J53" s="54"/>
-      <c r="K53" s="54"/>
-      <c r="L53" s="55"/>
+      <c r="I53" s="55"/>
+      <c r="J53" s="55"/>
+      <c r="K53" s="55"/>
+      <c r="L53" s="56"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -20707,11 +20715,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="56"/>
-      <c r="I54" s="57"/>
-      <c r="J54" s="57"/>
-      <c r="K54" s="57"/>
-      <c r="L54" s="58"/>
+      <c r="H54" s="57"/>
+      <c r="I54" s="58"/>
+      <c r="J54" s="58"/>
+      <c r="K54" s="58"/>
+      <c r="L54" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - core lua script changes
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E17D81F-62C2-4BD1-A485-941825B01C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2384BE53-FFEF-4D7D-B3B9-B0752A0F13E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="47415" yWindow="3540" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="46845" yWindow="3870" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="428">
   <si>
     <t>Place</t>
   </si>
@@ -1305,6 +1305,21 @@
   </si>
   <si>
     <t>(v6 1st move)</t>
+  </si>
+  <si>
+    <t>last ladder grab</t>
+  </si>
+  <si>
+    <t>enemy fall</t>
+  </si>
+  <si>
+    <t>x = 4.625</t>
+  </si>
+  <si>
+    <t>dig 3</t>
+  </si>
+  <si>
+    <t>dig 2</t>
   </si>
 </sst>
 </file>
@@ -1314,12 +1329,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1772,95 +1794,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="28" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1879,31 +1902,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2224,7 +2247,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E184"/>
+  <dimension ref="A1:E196"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2511,7 +2534,7 @@
         <v>8196</v>
       </c>
       <c r="D19" s="3">
-        <f t="shared" ref="D19:D50" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
+        <f t="shared" ref="D19:D62" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
         <v>100</v>
       </c>
     </row>
@@ -2744,405 +2767,392 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="50" t="s">
-        <v>297</v>
-      </c>
-      <c r="B35" s="7"/>
+      <c r="A35" s="60" t="s">
+        <v>424</v>
+      </c>
+      <c r="B35" s="7">
+        <v>14970</v>
+      </c>
       <c r="C35" s="7">
-        <v>15850</v>
-      </c>
-      <c r="D35" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>15211</v>
+      </c>
+      <c r="D35" s="3">
+        <f t="shared" si="1"/>
+        <v>241</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="50" t="s">
-        <v>407</v>
-      </c>
-      <c r="B36" s="7"/>
+      <c r="A36" s="60" t="s">
+        <v>425</v>
+      </c>
+      <c r="B36" s="7">
+        <v>14972</v>
+      </c>
       <c r="C36" s="7">
-        <v>16200</v>
-      </c>
-      <c r="D36" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>15213</v>
+      </c>
+      <c r="D36" s="3">
+        <f t="shared" si="1"/>
+        <v>241</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="50" t="s">
-        <v>301</v>
-      </c>
-      <c r="B37" s="33"/>
-      <c r="C37" s="33">
-        <v>17135</v>
-      </c>
-      <c r="D37" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="A37" s="60" t="s">
+        <v>150</v>
+      </c>
+      <c r="B37" s="7">
+        <v>14981</v>
+      </c>
+      <c r="C37" s="7">
+        <v>15222</v>
+      </c>
+      <c r="D37" s="3">
+        <f t="shared" si="1"/>
+        <v>241</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="50" t="s">
-        <v>408</v>
-      </c>
-      <c r="B38" s="7"/>
+      <c r="A38" s="60" t="s">
+        <v>427</v>
+      </c>
+      <c r="B38" s="7">
+        <v>15008</v>
+      </c>
       <c r="C38" s="7">
-        <v>17485</v>
-      </c>
-      <c r="D38" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>15248</v>
+      </c>
+      <c r="D38" s="3">
+        <f t="shared" si="1"/>
+        <v>240</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="50" t="s">
-        <v>305</v>
-      </c>
-      <c r="B39" s="7"/>
+      <c r="A39" s="60" t="s">
+        <v>426</v>
+      </c>
+      <c r="B39" s="7">
+        <v>15034</v>
+      </c>
       <c r="C39" s="7">
-        <v>17791</v>
-      </c>
-      <c r="D39" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>15274</v>
+      </c>
+      <c r="D39" s="3">
+        <f t="shared" si="1"/>
+        <v>240</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="50" t="s">
-        <v>409</v>
-      </c>
+      <c r="A40" s="60"/>
       <c r="B40" s="7"/>
-      <c r="C40" s="37">
-        <v>18139</v>
-      </c>
-      <c r="D40" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
+      <c r="C40" s="7"/>
+      <c r="D40" s="3"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="50" t="s">
-        <v>308</v>
-      </c>
-      <c r="B41" s="7"/>
+      <c r="A41" s="60" t="s">
+        <v>279</v>
+      </c>
+      <c r="B41" s="7">
+        <v>15151</v>
+      </c>
       <c r="C41" s="7">
-        <v>18719</v>
-      </c>
-      <c r="D41" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>15389</v>
+      </c>
+      <c r="D41" s="3">
+        <f t="shared" si="1"/>
+        <v>238</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="50" t="s">
-        <v>411</v>
-      </c>
+      <c r="A42" s="60"/>
       <c r="B42" s="7"/>
-      <c r="C42" s="7">
-        <v>19068</v>
-      </c>
-      <c r="D42" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
+      <c r="C42" s="7"/>
+      <c r="D42" s="3"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="50" t="s">
-        <v>314</v>
-      </c>
-      <c r="B43" s="7"/>
+      <c r="A43" s="60" t="s">
+        <v>265</v>
+      </c>
+      <c r="B43" s="7">
+        <v>15219</v>
+      </c>
       <c r="C43" s="7">
-        <v>19892</v>
-      </c>
-      <c r="D43" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>15452</v>
+      </c>
+      <c r="D43" s="3">
+        <f t="shared" si="1"/>
+        <v>233</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="50" t="s">
-        <v>412</v>
-      </c>
+      <c r="A44" s="60"/>
       <c r="B44" s="7"/>
-      <c r="C44" s="7">
-        <v>20240</v>
-      </c>
-      <c r="D44" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
+      <c r="C44" s="7"/>
+      <c r="D44" s="3"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="50" t="s">
-        <v>320</v>
-      </c>
+      <c r="A45" s="50"/>
       <c r="B45" s="7"/>
-      <c r="C45" s="7">
-        <v>20813</v>
-      </c>
-      <c r="D45" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
+      <c r="C45" s="7"/>
+      <c r="D45" s="3"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="50" t="s">
-        <v>413</v>
-      </c>
-      <c r="B46" s="7"/>
+      <c r="A46" s="60" t="s">
+        <v>423</v>
+      </c>
+      <c r="B46" s="7">
+        <v>15577</v>
+      </c>
       <c r="C46" s="7">
-        <v>21161</v>
-      </c>
-      <c r="D46" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>15812</v>
+      </c>
+      <c r="D46" s="3">
+        <f t="shared" si="1"/>
+        <v>235</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="50" t="s">
-        <v>322</v>
-      </c>
-      <c r="B47" s="7"/>
+        <v>297</v>
+      </c>
+      <c r="B47" s="7">
+        <v>15609</v>
+      </c>
       <c r="C47" s="7">
-        <v>22195</v>
-      </c>
-      <c r="D47" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>15850</v>
+      </c>
+      <c r="D47" s="3">
+        <f t="shared" si="1"/>
+        <v>241</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="50" t="s">
-        <v>414</v>
+        <v>407</v>
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="7">
-        <v>22543</v>
+        <v>16200</v>
       </c>
       <c r="D48" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="50" t="s">
-        <v>324</v>
-      </c>
-      <c r="B49" s="7"/>
-      <c r="C49" s="7">
-        <v>22963</v>
+        <v>301</v>
+      </c>
+      <c r="B49" s="33"/>
+      <c r="C49" s="33">
+        <v>17135</v>
       </c>
       <c r="D49" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="50" t="s">
-        <v>415</v>
+        <v>408</v>
       </c>
       <c r="B50" s="7"/>
       <c r="C50" s="7">
-        <v>23346</v>
+        <v>17485</v>
       </c>
       <c r="D50" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="50" t="s">
-        <v>416</v>
+        <v>305</v>
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="7">
-        <v>23873</v>
+        <v>17791</v>
       </c>
       <c r="D51" s="3" t="str">
-        <f t="shared" ref="D51:D80" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="50" t="s">
-        <v>417</v>
-      </c>
-      <c r="B52" s="8"/>
-      <c r="C52" s="50">
-        <v>24221</v>
+        <v>409</v>
+      </c>
+      <c r="B52" s="7"/>
+      <c r="C52" s="37">
+        <v>18139</v>
       </c>
       <c r="D52" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="50" t="s">
-        <v>418</v>
-      </c>
-      <c r="B53" s="33"/>
-      <c r="C53" s="33">
-        <v>25101</v>
+        <v>308</v>
+      </c>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7">
+        <v>18719</v>
       </c>
       <c r="D53" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="50" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="7">
-        <v>25450</v>
+        <v>19068</v>
       </c>
       <c r="D54" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="50" t="s">
-        <v>420</v>
+        <v>314</v>
       </c>
       <c r="B55" s="7"/>
       <c r="C55" s="7">
-        <v>26350</v>
+        <v>19892</v>
       </c>
       <c r="D55" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="50" t="s">
-        <v>421</v>
+        <v>412</v>
       </c>
       <c r="B56" s="7"/>
       <c r="C56" s="7">
-        <v>26699</v>
+        <v>20240</v>
       </c>
       <c r="D56" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="50" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7">
-        <v>27490</v>
+        <v>20813</v>
       </c>
       <c r="D57" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
-        <v>5</v>
+        <v>413</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7">
-        <v>27836</v>
+        <v>21161</v>
       </c>
       <c r="D58" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>337</v>
+        <v>322</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7">
-        <v>28899</v>
+        <v>22195</v>
       </c>
       <c r="D59" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>6</v>
+        <v>414</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7">
-        <v>29248</v>
+        <v>22543</v>
       </c>
       <c r="D60" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>45</v>
+        <v>324</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7">
-        <v>29962</v>
+        <v>22963</v>
       </c>
       <c r="D61" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>7</v>
+        <v>415</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7">
-        <v>30309</v>
+        <v>23346</v>
       </c>
       <c r="D62" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>46</v>
+        <v>416</v>
       </c>
       <c r="B63" s="7"/>
       <c r="C63" s="7">
-        <v>30479</v>
+        <v>23873</v>
       </c>
       <c r="D63" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" ref="D63:D92" si="2">IF(C63&lt;&gt;"",IF(B63&lt;&gt;"",C63-B63,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>8</v>
-      </c>
-      <c r="B64" s="7"/>
-      <c r="C64" s="7">
-        <v>31125</v>
+        <v>417</v>
+      </c>
+      <c r="B64" s="8"/>
+      <c r="C64" s="50">
+        <v>24221</v>
       </c>
       <c r="D64" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E64" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>28</v>
-      </c>
-      <c r="B65" s="7"/>
-      <c r="C65" s="7">
-        <v>31643</v>
+        <v>418</v>
+      </c>
+      <c r="B65" s="33"/>
+      <c r="C65" s="33">
+        <v>25101</v>
       </c>
       <c r="D65" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3151,11 +3161,11 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>9</v>
+        <v>419</v>
       </c>
       <c r="B66" s="7"/>
       <c r="C66" s="7">
-        <v>31991</v>
+        <v>25450</v>
       </c>
       <c r="D66" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3164,11 +3174,11 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>29</v>
+        <v>420</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>32586</v>
+        <v>26350</v>
       </c>
       <c r="D67" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3177,27 +3187,24 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>10</v>
+        <v>421</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7">
-        <v>33254</v>
+        <v>26699</v>
       </c>
       <c r="D68" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E68" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>31</v>
+        <v>332</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7">
-        <v>33883</v>
+        <v>27490</v>
       </c>
       <c r="D69" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3206,11 +3213,11 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>34244</v>
+        <v>27836</v>
       </c>
       <c r="D70" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3219,11 +3226,11 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>30</v>
+        <v>337</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>34862</v>
+        <v>28899</v>
       </c>
       <c r="D71" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3232,11 +3239,11 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>35218</v>
+        <v>29248</v>
       </c>
       <c r="D72" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3245,11 +3252,11 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>35772</v>
+        <v>29962</v>
       </c>
       <c r="D73" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3258,11 +3265,11 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>36120</v>
+        <v>30309</v>
       </c>
       <c r="D74" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3271,11 +3278,11 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>36893</v>
+        <v>30479</v>
       </c>
       <c r="D75" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3284,24 +3291,27 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>37238</v>
+        <v>31125</v>
       </c>
       <c r="D76" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E76" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>38097</v>
+        <v>31643</v>
       </c>
       <c r="D77" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3310,11 +3320,11 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>38443</v>
+        <v>31991</v>
       </c>
       <c r="D78" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3323,11 +3333,11 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>38692</v>
+        <v>32586</v>
       </c>
       <c r="D79" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3336,398 +3346,509 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>39041</v>
+        <v>33254</v>
       </c>
       <c r="D80" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E80" s="51" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>40011</v>
+        <v>33883</v>
       </c>
       <c r="D81" s="3" t="str">
-        <f>IF(C80&lt;&gt;"",IF(B80&lt;&gt;"",C80-B80,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>40373</v>
+        <v>34244</v>
       </c>
       <c r="D82" s="3" t="str">
-        <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B83" s="40"/>
+        <v>30</v>
+      </c>
+      <c r="B83" s="7"/>
       <c r="C83" s="7">
-        <v>41117</v>
+        <v>34862</v>
       </c>
       <c r="D83" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B84" s="7"/>
       <c r="C84" s="7">
-        <v>41465</v>
+        <v>35218</v>
       </c>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>42450</v>
+        <v>35772</v>
       </c>
       <c r="D85" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B86" s="7"/>
       <c r="C86" s="7">
-        <v>42799</v>
+        <v>36120</v>
       </c>
       <c r="D86" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>43144</v>
+        <v>36893</v>
       </c>
       <c r="D87" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>43491</v>
+        <v>37238</v>
       </c>
       <c r="D88" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>44165</v>
+        <v>38097</v>
       </c>
       <c r="D89" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>44512</v>
+        <v>38443</v>
       </c>
       <c r="D90" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>45061</v>
+        <v>38692</v>
       </c>
       <c r="D91" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>45443</v>
+        <v>39041</v>
       </c>
       <c r="D92" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>45990</v>
+        <v>40011</v>
       </c>
       <c r="D93" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+        <f>IF(C92&lt;&gt;"",IF(B92&lt;&gt;"",C92-B92,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>46652</v>
+        <v>40373</v>
       </c>
       <c r="D94" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-      <c r="E94" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" ref="D94:D113" si="3">IF(C94&lt;&gt;"",IF(B94&lt;&gt;"",C94-B94,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>42</v>
-      </c>
-      <c r="B95" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B95" s="40"/>
       <c r="C95" s="7">
-        <v>47436</v>
+        <v>41117</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B96" s="9"/>
-      <c r="C96" s="9">
-        <v>48337</v>
+        <v>17</v>
+      </c>
+      <c r="B96" s="7"/>
+      <c r="C96" s="7">
+        <v>41465</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>49334</v>
+        <v>42450</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>48681</v>
+        <v>42799</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>49334</v>
+        <v>43144</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>49683</v>
+        <v>43491</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>50244</v>
+        <v>44165</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="50" t="s">
+        <v>20</v>
+      </c>
       <c r="B102" s="7"/>
-      <c r="C102" s="7"/>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C102" s="7">
+        <v>44512</v>
+      </c>
+      <c r="D102" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="50" t="s">
+        <v>40</v>
+      </c>
       <c r="B103" s="7"/>
-      <c r="C103" s="7"/>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C103" s="7">
+        <v>45061</v>
+      </c>
+      <c r="D103" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="50" t="s">
+        <v>21</v>
+      </c>
       <c r="B104" s="7"/>
-      <c r="C104" s="7"/>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C104" s="7">
+        <v>45443</v>
+      </c>
+      <c r="D104" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="50" t="s">
+        <v>41</v>
+      </c>
       <c r="B105" s="7"/>
-      <c r="C105" s="7"/>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C105" s="7">
+        <v>45990</v>
+      </c>
+      <c r="D105" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="50" t="s">
+        <v>22</v>
+      </c>
       <c r="B106" s="7"/>
-      <c r="C106" s="7"/>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C106" s="7">
+        <v>46652</v>
+      </c>
+      <c r="D106" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+      <c r="E106" s="51" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="50" t="s">
+        <v>42</v>
+      </c>
       <c r="B107" s="7"/>
-      <c r="C107" s="7"/>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B108" s="7"/>
-      <c r="C108" s="7"/>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C107" s="7">
+        <v>47436</v>
+      </c>
+      <c r="D107" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" s="50" t="s">
+        <v>23</v>
+      </c>
+      <c r="B108" s="9"/>
+      <c r="C108" s="9">
+        <v>48337</v>
+      </c>
+      <c r="D108" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" s="50" t="s">
+        <v>43</v>
+      </c>
       <c r="B109" s="7"/>
-      <c r="C109" s="7"/>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C109" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D109" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" s="50" t="s">
+        <v>24</v>
+      </c>
       <c r="B110" s="7"/>
-      <c r="C110" s="7"/>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C110" s="7">
+        <v>48681</v>
+      </c>
+      <c r="D110" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A111" s="50" t="s">
+        <v>44</v>
+      </c>
       <c r="B111" s="7"/>
-      <c r="C111" s="7"/>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C111" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D111" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A112" s="50" t="s">
+        <v>25</v>
+      </c>
       <c r="B112" s="7"/>
-      <c r="C112" s="7"/>
-    </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C112" s="7">
+        <v>49683</v>
+      </c>
+      <c r="D112" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" s="50" t="s">
+        <v>26</v>
+      </c>
       <c r="B113" s="7"/>
-      <c r="C113" s="7"/>
-    </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C113" s="7">
+        <v>50244</v>
+      </c>
+      <c r="D113" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B114" s="7"/>
       <c r="C114" s="7"/>
     </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B115" s="7"/>
       <c r="C115" s="7"/>
     </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B116" s="7"/>
       <c r="C116" s="7"/>
     </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B117" s="7"/>
       <c r="C117" s="7"/>
     </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B118" s="7"/>
       <c r="C118" s="7"/>
     </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B119" s="7"/>
       <c r="C119" s="7"/>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B120" s="7"/>
       <c r="C120" s="7"/>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B121" s="7"/>
       <c r="C121" s="7"/>
     </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B122" s="7"/>
       <c r="C122" s="7"/>
     </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B123" s="7"/>
       <c r="C123" s="7"/>
     </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B124" s="7"/>
       <c r="C124" s="7"/>
     </row>
-    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B125" s="7"/>
       <c r="C125" s="7"/>
     </row>
-    <row r="126" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B126" s="7"/>
       <c r="C126" s="7"/>
     </row>
-    <row r="127" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B127" s="7"/>
       <c r="C127" s="7"/>
     </row>
-    <row r="128" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B128" s="7"/>
       <c r="C128" s="7"/>
     </row>
@@ -3954,6 +4075,54 @@
     <row r="184" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
+    </row>
+    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B185" s="7"/>
+      <c r="C185" s="7"/>
+    </row>
+    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B186" s="7"/>
+      <c r="C186" s="7"/>
+    </row>
+    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B187" s="7"/>
+      <c r="C187" s="7"/>
+    </row>
+    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B188" s="7"/>
+      <c r="C188" s="7"/>
+    </row>
+    <row r="189" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B189" s="7"/>
+      <c r="C189" s="7"/>
+    </row>
+    <row r="190" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B190" s="7"/>
+      <c r="C190" s="7"/>
+    </row>
+    <row r="191" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B191" s="7"/>
+      <c r="C191" s="7"/>
+    </row>
+    <row r="192" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B192" s="7"/>
+      <c r="C192" s="7"/>
+    </row>
+    <row r="193" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B193" s="7"/>
+      <c r="C193" s="7"/>
+    </row>
+    <row r="194" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B194" s="7"/>
+      <c r="C194" s="7"/>
+    </row>
+    <row r="195" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B195" s="7"/>
+      <c r="C195" s="7"/>
+    </row>
+    <row r="196" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B196" s="7"/>
+      <c r="C196" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18802,7 +18971,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="32" type="noConversion"/>
+  <phoneticPr fontId="33" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>

</xml_diff>

<commit_message>
lode runner - lv 17 done - 245 frames ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2384BE53-FFEF-4D7D-B3B9-B0752A0F13E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8330A113-835E-4CBA-8155-8FAE4FC9C6E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46845" yWindow="3870" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="46845" yWindow="3210" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="423">
   <si>
     <t>Place</t>
   </si>
@@ -1305,21 +1305,6 @@
   </si>
   <si>
     <t>(v6 1st move)</t>
-  </si>
-  <si>
-    <t>last ladder grab</t>
-  </si>
-  <si>
-    <t>enemy fall</t>
-  </si>
-  <si>
-    <t>x = 4.625</t>
-  </si>
-  <si>
-    <t>dig 3</t>
-  </si>
-  <si>
-    <t>dig 2</t>
   </si>
 </sst>
 </file>
@@ -1329,19 +1314,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="37" x14ac:knownFonts="1">
+  <fonts count="36" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1794,96 +1772,95 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="5"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1902,31 +1879,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2247,7 +2224,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E196"/>
+  <dimension ref="A1:E184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2534,7 +2511,7 @@
         <v>8196</v>
       </c>
       <c r="D19" s="3">
-        <f t="shared" ref="D19:D62" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
+        <f t="shared" ref="D19:D50" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
         <v>100</v>
       </c>
     </row>
@@ -2767,392 +2744,409 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="60" t="s">
-        <v>424</v>
+      <c r="A35" s="50" t="s">
+        <v>297</v>
       </c>
       <c r="B35" s="7">
-        <v>14970</v>
+        <v>15603</v>
       </c>
       <c r="C35" s="7">
-        <v>15211</v>
+        <v>15850</v>
       </c>
       <c r="D35" s="3">
         <f t="shared" si="1"/>
-        <v>241</v>
+        <v>247</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="60" t="s">
-        <v>425</v>
+      <c r="A36" s="50" t="s">
+        <v>407</v>
       </c>
       <c r="B36" s="7">
-        <v>14972</v>
+        <v>15955</v>
       </c>
       <c r="C36" s="7">
-        <v>15213</v>
+        <v>16200</v>
       </c>
       <c r="D36" s="3">
         <f t="shared" si="1"/>
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="60" t="s">
-        <v>150</v>
-      </c>
-      <c r="B37" s="7">
-        <v>14981</v>
-      </c>
-      <c r="C37" s="7">
-        <v>15222</v>
-      </c>
-      <c r="D37" s="3">
-        <f t="shared" si="1"/>
-        <v>241</v>
+      <c r="A37" s="50" t="s">
+        <v>301</v>
+      </c>
+      <c r="B37" s="33"/>
+      <c r="C37" s="33">
+        <v>17135</v>
+      </c>
+      <c r="D37" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="60" t="s">
-        <v>427</v>
-      </c>
-      <c r="B38" s="7">
-        <v>15008</v>
-      </c>
+      <c r="A38" s="50" t="s">
+        <v>408</v>
+      </c>
+      <c r="B38" s="7"/>
       <c r="C38" s="7">
-        <v>15248</v>
-      </c>
-      <c r="D38" s="3">
-        <f t="shared" si="1"/>
-        <v>240</v>
+        <v>17485</v>
+      </c>
+      <c r="D38" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="60" t="s">
-        <v>426</v>
-      </c>
-      <c r="B39" s="7">
-        <v>15034</v>
-      </c>
+      <c r="A39" s="50" t="s">
+        <v>305</v>
+      </c>
+      <c r="B39" s="7"/>
       <c r="C39" s="7">
-        <v>15274</v>
-      </c>
-      <c r="D39" s="3">
-        <f t="shared" si="1"/>
-        <v>240</v>
+        <v>17791</v>
+      </c>
+      <c r="D39" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="60"/>
+      <c r="A40" s="50" t="s">
+        <v>409</v>
+      </c>
       <c r="B40" s="7"/>
-      <c r="C40" s="7"/>
-      <c r="D40" s="3"/>
+      <c r="C40" s="37">
+        <v>18139</v>
+      </c>
+      <c r="D40" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="60" t="s">
-        <v>279</v>
-      </c>
-      <c r="B41" s="7">
-        <v>15151</v>
-      </c>
+      <c r="A41" s="50" t="s">
+        <v>308</v>
+      </c>
+      <c r="B41" s="7"/>
       <c r="C41" s="7">
-        <v>15389</v>
-      </c>
-      <c r="D41" s="3">
-        <f t="shared" si="1"/>
-        <v>238</v>
+        <v>18719</v>
+      </c>
+      <c r="D41" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="60"/>
+      <c r="A42" s="50" t="s">
+        <v>411</v>
+      </c>
       <c r="B42" s="7"/>
-      <c r="C42" s="7"/>
-      <c r="D42" s="3"/>
+      <c r="C42" s="7">
+        <v>19068</v>
+      </c>
+      <c r="D42" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="60" t="s">
-        <v>265</v>
-      </c>
-      <c r="B43" s="7">
-        <v>15219</v>
-      </c>
+      <c r="A43" s="50" t="s">
+        <v>314</v>
+      </c>
+      <c r="B43" s="7"/>
       <c r="C43" s="7">
-        <v>15452</v>
-      </c>
-      <c r="D43" s="3">
-        <f t="shared" si="1"/>
-        <v>233</v>
+        <v>19892</v>
+      </c>
+      <c r="D43" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="60"/>
+      <c r="A44" s="50" t="s">
+        <v>412</v>
+      </c>
       <c r="B44" s="7"/>
-      <c r="C44" s="7"/>
-      <c r="D44" s="3"/>
+      <c r="C44" s="7">
+        <v>20240</v>
+      </c>
+      <c r="D44" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="50"/>
+      <c r="A45" s="50" t="s">
+        <v>320</v>
+      </c>
       <c r="B45" s="7"/>
-      <c r="C45" s="7"/>
-      <c r="D45" s="3"/>
+      <c r="C45" s="7">
+        <v>20813</v>
+      </c>
+      <c r="D45" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="60" t="s">
-        <v>423</v>
-      </c>
-      <c r="B46" s="7">
-        <v>15577</v>
-      </c>
+      <c r="A46" s="50" t="s">
+        <v>413</v>
+      </c>
+      <c r="B46" s="7"/>
       <c r="C46" s="7">
-        <v>15812</v>
-      </c>
-      <c r="D46" s="3">
-        <f t="shared" si="1"/>
-        <v>235</v>
+        <v>21161</v>
+      </c>
+      <c r="D46" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="50" t="s">
-        <v>297</v>
-      </c>
-      <c r="B47" s="7">
-        <v>15609</v>
-      </c>
+        <v>322</v>
+      </c>
+      <c r="B47" s="7"/>
       <c r="C47" s="7">
-        <v>15850</v>
-      </c>
-      <c r="D47" s="3">
-        <f t="shared" si="1"/>
-        <v>241</v>
+        <v>22195</v>
+      </c>
+      <c r="D47" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="50" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="7">
-        <v>16200</v>
+        <v>22543</v>
       </c>
       <c r="D48" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="50" t="s">
-        <v>301</v>
-      </c>
-      <c r="B49" s="33"/>
-      <c r="C49" s="33">
-        <v>17135</v>
+        <v>324</v>
+      </c>
+      <c r="B49" s="7"/>
+      <c r="C49" s="7">
+        <v>22963</v>
       </c>
       <c r="D49" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="50" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="B50" s="7"/>
       <c r="C50" s="7">
-        <v>17485</v>
+        <v>23346</v>
       </c>
       <c r="D50" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="50" t="s">
-        <v>305</v>
+        <v>416</v>
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="7">
-        <v>17791</v>
+        <v>23873</v>
       </c>
       <c r="D51" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" ref="D51:D80" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="50" t="s">
-        <v>409</v>
-      </c>
-      <c r="B52" s="7"/>
-      <c r="C52" s="37">
-        <v>18139</v>
+        <v>417</v>
+      </c>
+      <c r="B52" s="8"/>
+      <c r="C52" s="50">
+        <v>24221</v>
       </c>
       <c r="D52" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="50" t="s">
-        <v>308</v>
-      </c>
-      <c r="B53" s="7"/>
-      <c r="C53" s="7">
-        <v>18719</v>
+        <v>418</v>
+      </c>
+      <c r="B53" s="33"/>
+      <c r="C53" s="33">
+        <v>25101</v>
       </c>
       <c r="D53" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="50" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="7">
-        <v>19068</v>
+        <v>25450</v>
       </c>
       <c r="D54" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="50" t="s">
-        <v>314</v>
+        <v>420</v>
       </c>
       <c r="B55" s="7"/>
       <c r="C55" s="7">
-        <v>19892</v>
+        <v>26350</v>
       </c>
       <c r="D55" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="50" t="s">
-        <v>412</v>
+        <v>421</v>
       </c>
       <c r="B56" s="7"/>
       <c r="C56" s="7">
-        <v>20240</v>
+        <v>26699</v>
       </c>
       <c r="D56" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="50" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7">
-        <v>20813</v>
+        <v>27490</v>
       </c>
       <c r="D57" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
-        <v>413</v>
+        <v>5</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7">
-        <v>21161</v>
+        <v>27836</v>
       </c>
       <c r="D58" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7">
-        <v>22195</v>
+        <v>28899</v>
       </c>
       <c r="D59" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>414</v>
+        <v>6</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7">
-        <v>22543</v>
+        <v>29248</v>
       </c>
       <c r="D60" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>324</v>
+        <v>45</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7">
-        <v>22963</v>
+        <v>29962</v>
       </c>
       <c r="D61" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>415</v>
+        <v>7</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7">
-        <v>23346</v>
+        <v>30309</v>
       </c>
       <c r="D62" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>416</v>
+        <v>46</v>
       </c>
       <c r="B63" s="7"/>
       <c r="C63" s="7">
-        <v>23873</v>
+        <v>30479</v>
       </c>
       <c r="D63" s="3" t="str">
-        <f t="shared" ref="D63:D92" si="2">IF(C63&lt;&gt;"",IF(B63&lt;&gt;"",C63-B63,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>417</v>
-      </c>
-      <c r="B64" s="8"/>
-      <c r="C64" s="50">
-        <v>24221</v>
+        <v>8</v>
+      </c>
+      <c r="B64" s="7"/>
+      <c r="C64" s="7">
+        <v>31125</v>
       </c>
       <c r="D64" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E64" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>418</v>
-      </c>
-      <c r="B65" s="33"/>
-      <c r="C65" s="33">
-        <v>25101</v>
+        <v>28</v>
+      </c>
+      <c r="B65" s="7"/>
+      <c r="C65" s="7">
+        <v>31643</v>
       </c>
       <c r="D65" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3161,11 +3155,11 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>419</v>
+        <v>9</v>
       </c>
       <c r="B66" s="7"/>
       <c r="C66" s="7">
-        <v>25450</v>
+        <v>31991</v>
       </c>
       <c r="D66" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3174,11 +3168,11 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>420</v>
+        <v>29</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>26350</v>
+        <v>32586</v>
       </c>
       <c r="D67" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3187,24 +3181,27 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>421</v>
+        <v>10</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7">
-        <v>26699</v>
+        <v>33254</v>
       </c>
       <c r="D68" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E68" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>332</v>
+        <v>31</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7">
-        <v>27490</v>
+        <v>33883</v>
       </c>
       <c r="D69" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3213,11 +3210,11 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>27836</v>
+        <v>34244</v>
       </c>
       <c r="D70" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3226,11 +3223,11 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>337</v>
+        <v>30</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>28899</v>
+        <v>34862</v>
       </c>
       <c r="D71" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3239,11 +3236,11 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>29248</v>
+        <v>35218</v>
       </c>
       <c r="D72" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3252,11 +3249,11 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>29962</v>
+        <v>35772</v>
       </c>
       <c r="D73" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3265,11 +3262,11 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>30309</v>
+        <v>36120</v>
       </c>
       <c r="D74" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3278,11 +3275,11 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>30479</v>
+        <v>36893</v>
       </c>
       <c r="D75" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3291,27 +3288,24 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>31125</v>
+        <v>37238</v>
       </c>
       <c r="D76" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E76" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>31643</v>
+        <v>38097</v>
       </c>
       <c r="D77" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3320,11 +3314,11 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>31991</v>
+        <v>38443</v>
       </c>
       <c r="D78" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3333,11 +3327,11 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>32586</v>
+        <v>38692</v>
       </c>
       <c r="D79" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3346,509 +3340,398 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>33254</v>
+        <v>39041</v>
       </c>
       <c r="D80" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E80" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>33883</v>
+        <v>40011</v>
       </c>
       <c r="D81" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+        <f>IF(C80&lt;&gt;"",IF(B80&lt;&gt;"",C80-B80,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>34244</v>
+        <v>40373</v>
       </c>
       <c r="D82" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="B83" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B83" s="40"/>
       <c r="C83" s="7">
-        <v>34862</v>
+        <v>41117</v>
       </c>
       <c r="D83" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B84" s="7"/>
       <c r="C84" s="7">
-        <v>35218</v>
+        <v>41465</v>
       </c>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>35772</v>
+        <v>42450</v>
       </c>
       <c r="D85" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B86" s="7"/>
       <c r="C86" s="7">
-        <v>36120</v>
+        <v>42799</v>
       </c>
       <c r="D86" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>36893</v>
+        <v>43144</v>
       </c>
       <c r="D87" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>37238</v>
+        <v>43491</v>
       </c>
       <c r="D88" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>38097</v>
+        <v>44165</v>
       </c>
       <c r="D89" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>38443</v>
+        <v>44512</v>
       </c>
       <c r="D90" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>38692</v>
+        <v>45061</v>
       </c>
       <c r="D91" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>39041</v>
+        <v>45443</v>
       </c>
       <c r="D92" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>40011</v>
+        <v>45990</v>
       </c>
       <c r="D93" s="3" t="str">
-        <f>IF(C92&lt;&gt;"",IF(B92&lt;&gt;"",C92-B92,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>40373</v>
+        <v>46652</v>
       </c>
       <c r="D94" s="3" t="str">
-        <f t="shared" ref="D94:D113" si="3">IF(C94&lt;&gt;"",IF(B94&lt;&gt;"",C94-B94,"-"), "-")</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+      <c r="E94" s="51" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B95" s="40"/>
+        <v>42</v>
+      </c>
+      <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>41117</v>
+        <v>47436</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="B96" s="7"/>
-      <c r="C96" s="7">
-        <v>41465</v>
+        <v>23</v>
+      </c>
+      <c r="B96" s="9"/>
+      <c r="C96" s="9">
+        <v>48337</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>42450</v>
+        <v>49334</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>42799</v>
+        <v>48681</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>43144</v>
+        <v>49334</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>43491</v>
+        <v>49683</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>44165</v>
+        <v>50244</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="50" t="s">
-        <v>20</v>
-      </c>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B102" s="7"/>
-      <c r="C102" s="7">
-        <v>44512</v>
-      </c>
-      <c r="D102" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="50" t="s">
-        <v>40</v>
-      </c>
+      <c r="C102" s="7"/>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B103" s="7"/>
-      <c r="C103" s="7">
-        <v>45061</v>
-      </c>
-      <c r="D103" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A104" s="50" t="s">
-        <v>21</v>
-      </c>
+      <c r="C103" s="7"/>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B104" s="7"/>
-      <c r="C104" s="7">
-        <v>45443</v>
-      </c>
-      <c r="D104" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="50" t="s">
-        <v>41</v>
-      </c>
+      <c r="C104" s="7"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B105" s="7"/>
-      <c r="C105" s="7">
-        <v>45990</v>
-      </c>
-      <c r="D105" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="50" t="s">
-        <v>22</v>
-      </c>
+      <c r="C105" s="7"/>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B106" s="7"/>
-      <c r="C106" s="7">
-        <v>46652</v>
-      </c>
-      <c r="D106" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-      <c r="E106" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="50" t="s">
-        <v>42</v>
-      </c>
+      <c r="C106" s="7"/>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B107" s="7"/>
-      <c r="C107" s="7">
-        <v>47436</v>
-      </c>
-      <c r="D107" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B108" s="9"/>
-      <c r="C108" s="9">
-        <v>48337</v>
-      </c>
-      <c r="D108" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A109" s="50" t="s">
-        <v>43</v>
-      </c>
+      <c r="C107" s="7"/>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B108" s="7"/>
+      <c r="C108" s="7"/>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B109" s="7"/>
-      <c r="C109" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D109" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A110" s="50" t="s">
-        <v>24</v>
-      </c>
+      <c r="C109" s="7"/>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
-      <c r="C110" s="7">
-        <v>48681</v>
-      </c>
-      <c r="D110" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A111" s="50" t="s">
-        <v>44</v>
-      </c>
+      <c r="C110" s="7"/>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
-      <c r="C111" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D111" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A112" s="50" t="s">
-        <v>25</v>
-      </c>
+      <c r="C111" s="7"/>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
-      <c r="C112" s="7">
-        <v>49683</v>
-      </c>
-      <c r="D112" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A113" s="50" t="s">
-        <v>26</v>
-      </c>
+      <c r="C112" s="7"/>
+    </row>
+    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B113" s="7"/>
-      <c r="C113" s="7">
-        <v>50244</v>
-      </c>
-      <c r="D113" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C113" s="7"/>
+    </row>
+    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B114" s="7"/>
       <c r="C114" s="7"/>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B115" s="7"/>
       <c r="C115" s="7"/>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B116" s="7"/>
       <c r="C116" s="7"/>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B117" s="7"/>
       <c r="C117" s="7"/>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B118" s="7"/>
       <c r="C118" s="7"/>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B119" s="7"/>
       <c r="C119" s="7"/>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B120" s="7"/>
       <c r="C120" s="7"/>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B121" s="7"/>
       <c r="C121" s="7"/>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B122" s="7"/>
       <c r="C122" s="7"/>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B123" s="7"/>
       <c r="C123" s="7"/>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B124" s="7"/>
       <c r="C124" s="7"/>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B125" s="7"/>
       <c r="C125" s="7"/>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B126" s="7"/>
       <c r="C126" s="7"/>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B127" s="7"/>
       <c r="C127" s="7"/>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B128" s="7"/>
       <c r="C128" s="7"/>
     </row>
@@ -4075,54 +3958,6 @@
     <row r="184" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
-    </row>
-    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B185" s="7"/>
-      <c r="C185" s="7"/>
-    </row>
-    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B186" s="7"/>
-      <c r="C186" s="7"/>
-    </row>
-    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B187" s="7"/>
-      <c r="C187" s="7"/>
-    </row>
-    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B188" s="7"/>
-      <c r="C188" s="7"/>
-    </row>
-    <row r="189" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B189" s="7"/>
-      <c r="C189" s="7"/>
-    </row>
-    <row r="190" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B190" s="7"/>
-      <c r="C190" s="7"/>
-    </row>
-    <row r="191" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B191" s="7"/>
-      <c r="C191" s="7"/>
-    </row>
-    <row r="192" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B192" s="7"/>
-      <c r="C192" s="7"/>
-    </row>
-    <row r="193" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B193" s="7"/>
-      <c r="C193" s="7"/>
-    </row>
-    <row r="194" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B194" s="7"/>
-      <c r="C194" s="7"/>
-    </row>
-    <row r="195" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B195" s="7"/>
-      <c r="C195" s="7"/>
-    </row>
-    <row r="196" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B196" s="7"/>
-      <c r="C196" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18971,7 +18806,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="33" type="noConversion"/>
+  <phoneticPr fontId="32" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>

</xml_diff>

<commit_message>
lode runner - level 18 done with new faster route, 338 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8330A113-835E-4CBA-8155-8FAE4FC9C6E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C23BFD5-9E96-4E3E-92EA-8623E69F5A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="46845" yWindow="3210" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1314,12 +1314,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1772,95 +1779,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="28" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1879,31 +1887,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2777,26 +2785,30 @@
       <c r="A37" s="50" t="s">
         <v>301</v>
       </c>
-      <c r="B37" s="33"/>
+      <c r="B37" s="7">
+        <v>16796</v>
+      </c>
       <c r="C37" s="33">
         <v>17135</v>
       </c>
-      <c r="D37" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="D37" s="3">
+        <f t="shared" si="1"/>
+        <v>339</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="50" t="s">
         <v>408</v>
       </c>
-      <c r="B38" s="7"/>
+      <c r="B38" s="60">
+        <v>17147</v>
+      </c>
       <c r="C38" s="7">
         <v>17485</v>
       </c>
-      <c r="D38" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="D38" s="3">
+        <f t="shared" si="1"/>
+        <v>338</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -18806,7 +18818,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="32" type="noConversion"/>
+  <phoneticPr fontId="33" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>

</xml_diff>

<commit_message>
lode runner - lv 19 done - 349 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C23BFD5-9E96-4E3E-92EA-8623E69F5A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{707C4E90-FE63-40DE-9658-B727A92D0D40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="46845" yWindow="3210" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2232,7 +2232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E184"/>
+  <dimension ref="A1:E185"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2519,7 +2519,7 @@
         <v>8196</v>
       </c>
       <c r="D19" s="3">
-        <f t="shared" ref="D19:D50" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
+        <f t="shared" ref="D19:D51" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
         <v>100</v>
       </c>
     </row>
@@ -2812,51 +2812,55 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="50" t="s">
-        <v>305</v>
-      </c>
-      <c r="B39" s="7"/>
+      <c r="A39" s="50"/>
+      <c r="B39" s="60">
+        <v>17287</v>
+      </c>
       <c r="C39" s="7">
-        <v>17791</v>
-      </c>
-      <c r="D39" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>17625</v>
+      </c>
+      <c r="D39" s="3">
+        <f t="shared" si="1"/>
+        <v>338</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="50" t="s">
-        <v>409</v>
-      </c>
-      <c r="B40" s="7"/>
-      <c r="C40" s="37">
-        <v>18139</v>
-      </c>
-      <c r="D40" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>305</v>
+      </c>
+      <c r="B40" s="7">
+        <v>17443</v>
+      </c>
+      <c r="C40" s="7">
+        <v>17791</v>
+      </c>
+      <c r="D40" s="3">
+        <f t="shared" si="1"/>
+        <v>348</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="50" t="s">
-        <v>308</v>
-      </c>
-      <c r="B41" s="7"/>
-      <c r="C41" s="7">
-        <v>18719</v>
-      </c>
-      <c r="D41" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>409</v>
+      </c>
+      <c r="B41" s="7">
+        <v>17790</v>
+      </c>
+      <c r="C41" s="37">
+        <v>18139</v>
+      </c>
+      <c r="D41" s="3">
+        <f t="shared" si="1"/>
+        <v>349</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="50" t="s">
-        <v>411</v>
+        <v>308</v>
       </c>
       <c r="B42" s="7"/>
       <c r="C42" s="7">
-        <v>19068</v>
+        <v>18719</v>
       </c>
       <c r="D42" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2865,11 +2869,11 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="50" t="s">
-        <v>314</v>
+        <v>411</v>
       </c>
       <c r="B43" s="7"/>
       <c r="C43" s="7">
-        <v>19892</v>
+        <v>19068</v>
       </c>
       <c r="D43" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2878,11 +2882,11 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="50" t="s">
-        <v>412</v>
+        <v>314</v>
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="7">
-        <v>20240</v>
+        <v>19892</v>
       </c>
       <c r="D44" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2891,11 +2895,11 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="50" t="s">
-        <v>320</v>
+        <v>412</v>
       </c>
       <c r="B45" s="7"/>
       <c r="C45" s="7">
-        <v>20813</v>
+        <v>20240</v>
       </c>
       <c r="D45" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2904,11 +2908,11 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="50" t="s">
-        <v>413</v>
+        <v>320</v>
       </c>
       <c r="B46" s="7"/>
       <c r="C46" s="7">
-        <v>21161</v>
+        <v>20813</v>
       </c>
       <c r="D46" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2917,11 +2921,11 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="50" t="s">
-        <v>322</v>
+        <v>413</v>
       </c>
       <c r="B47" s="7"/>
       <c r="C47" s="7">
-        <v>22195</v>
+        <v>21161</v>
       </c>
       <c r="D47" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2930,248 +2934,248 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="50" t="s">
-        <v>414</v>
+        <v>322</v>
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="7">
-        <v>22543</v>
+        <v>22195</v>
       </c>
       <c r="D48" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="50" t="s">
-        <v>324</v>
+        <v>414</v>
       </c>
       <c r="B49" s="7"/>
       <c r="C49" s="7">
-        <v>22963</v>
+        <v>22543</v>
       </c>
       <c r="D49" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="50" t="s">
-        <v>415</v>
+        <v>324</v>
       </c>
       <c r="B50" s="7"/>
       <c r="C50" s="7">
-        <v>23346</v>
+        <v>22963</v>
       </c>
       <c r="D50" s="3" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="50" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="7">
+        <v>23346</v>
+      </c>
+      <c r="D51" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="50" t="s">
+        <v>416</v>
+      </c>
+      <c r="B52" s="7"/>
+      <c r="C52" s="7">
         <v>23873</v>
       </c>
-      <c r="D51" s="3" t="str">
-        <f t="shared" ref="D51:D80" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
+      <c r="D52" s="3" t="str">
+        <f t="shared" ref="D52:D81" si="2">IF(C52&lt;&gt;"",IF(B52&lt;&gt;"",C52-B52,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="50" t="s">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="50" t="s">
         <v>417</v>
       </c>
-      <c r="B52" s="8"/>
-      <c r="C52" s="50">
+      <c r="B53" s="8"/>
+      <c r="C53" s="50">
         <v>24221</v>
-      </c>
-      <c r="D52" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="50" t="s">
-        <v>418</v>
-      </c>
-      <c r="B53" s="33"/>
-      <c r="C53" s="33">
-        <v>25101</v>
       </c>
       <c r="D53" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="50" t="s">
-        <v>419</v>
-      </c>
-      <c r="B54" s="7"/>
-      <c r="C54" s="7">
-        <v>25450</v>
+        <v>418</v>
+      </c>
+      <c r="B54" s="33"/>
+      <c r="C54" s="33">
+        <v>25101</v>
       </c>
       <c r="D54" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="50" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B55" s="7"/>
       <c r="C55" s="7">
-        <v>26350</v>
+        <v>25450</v>
       </c>
       <c r="D55" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="50" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B56" s="7"/>
       <c r="C56" s="7">
-        <v>26699</v>
+        <v>26350</v>
       </c>
       <c r="D56" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="50" t="s">
-        <v>332</v>
+        <v>421</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7">
-        <v>27490</v>
+        <v>26699</v>
       </c>
       <c r="D57" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
-        <v>5</v>
+        <v>332</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7">
-        <v>27836</v>
+        <v>27490</v>
       </c>
       <c r="D58" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>337</v>
+        <v>5</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7">
-        <v>28899</v>
+        <v>27836</v>
       </c>
       <c r="D59" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>6</v>
+        <v>337</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7">
-        <v>29248</v>
+        <v>28899</v>
       </c>
       <c r="D60" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7">
-        <v>29962</v>
+        <v>29248</v>
       </c>
       <c r="D61" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7">
-        <v>30309</v>
+        <v>29962</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="B63" s="7"/>
       <c r="C63" s="7">
-        <v>30479</v>
+        <v>30309</v>
       </c>
       <c r="D63" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7">
-        <v>31125</v>
+        <v>30479</v>
       </c>
       <c r="D64" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E64" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B65" s="7"/>
       <c r="C65" s="7">
-        <v>31643</v>
+        <v>31125</v>
       </c>
       <c r="D65" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E65" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="B66" s="7"/>
       <c r="C66" s="7">
-        <v>31991</v>
+        <v>31643</v>
       </c>
       <c r="D66" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3180,11 +3184,11 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>32586</v>
+        <v>31991</v>
       </c>
       <c r="D67" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3193,40 +3197,40 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7">
-        <v>33254</v>
+        <v>32586</v>
       </c>
       <c r="D68" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E68" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7">
-        <v>33883</v>
+        <v>33254</v>
       </c>
       <c r="D69" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E69" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>34244</v>
+        <v>33883</v>
       </c>
       <c r="D70" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3235,11 +3239,11 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>34862</v>
+        <v>34244</v>
       </c>
       <c r="D71" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3248,11 +3252,11 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>35218</v>
+        <v>34862</v>
       </c>
       <c r="D72" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3261,11 +3265,11 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>35772</v>
+        <v>35218</v>
       </c>
       <c r="D73" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3274,11 +3278,11 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>36120</v>
+        <v>35772</v>
       </c>
       <c r="D74" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3287,11 +3291,11 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>36893</v>
+        <v>36120</v>
       </c>
       <c r="D75" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3300,11 +3304,11 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>37238</v>
+        <v>36893</v>
       </c>
       <c r="D76" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3313,11 +3317,11 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>38097</v>
+        <v>37238</v>
       </c>
       <c r="D77" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3326,11 +3330,11 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>38443</v>
+        <v>38097</v>
       </c>
       <c r="D78" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3339,11 +3343,11 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>38692</v>
+        <v>38443</v>
       </c>
       <c r="D79" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3352,11 +3356,11 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>39041</v>
+        <v>38692</v>
       </c>
       <c r="D80" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3365,50 +3369,50 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>40011</v>
+        <v>39041</v>
       </c>
       <c r="D81" s="3" t="str">
-        <f>IF(C80&lt;&gt;"",IF(B80&lt;&gt;"",C80-B80,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>40373</v>
+        <v>40011</v>
       </c>
       <c r="D82" s="3" t="str">
-        <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
+        <f>IF(C81&lt;&gt;"",IF(B81&lt;&gt;"",C81-B81,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B83" s="40"/>
+        <v>16</v>
+      </c>
+      <c r="B83" s="7"/>
       <c r="C83" s="7">
-        <v>41117</v>
+        <v>40373</v>
       </c>
       <c r="D83" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="D83:D102" si="3">IF(C83&lt;&gt;"",IF(B83&lt;&gt;"",C83-B83,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="B84" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B84" s="40"/>
       <c r="C84" s="7">
-        <v>41465</v>
+        <v>41117</v>
       </c>
       <c r="D84" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3417,11 +3421,11 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>42450</v>
+        <v>41465</v>
       </c>
       <c r="D85" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3430,11 +3434,11 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="B86" s="7"/>
       <c r="C86" s="7">
-        <v>42799</v>
+        <v>42450</v>
       </c>
       <c r="D86" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3443,11 +3447,11 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>43144</v>
+        <v>42799</v>
       </c>
       <c r="D87" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3456,11 +3460,11 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>43491</v>
+        <v>43144</v>
       </c>
       <c r="D88" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3469,11 +3473,11 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>44165</v>
+        <v>43491</v>
       </c>
       <c r="D89" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3482,11 +3486,11 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>44512</v>
+        <v>44165</v>
       </c>
       <c r="D90" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3495,11 +3499,11 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>45061</v>
+        <v>44512</v>
       </c>
       <c r="D91" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3508,11 +3512,11 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>45443</v>
+        <v>45061</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3521,11 +3525,11 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>45990</v>
+        <v>45443</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3534,40 +3538,40 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>46652</v>
+        <v>45990</v>
       </c>
       <c r="D94" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E94" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>47436</v>
+        <v>46652</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
+      <c r="E95" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B96" s="9"/>
-      <c r="C96" s="9">
-        <v>48337</v>
+        <v>42</v>
+      </c>
+      <c r="B96" s="7"/>
+      <c r="C96" s="7">
+        <v>47436</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3576,11 +3580,11 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>43</v>
-      </c>
-      <c r="B97" s="7"/>
-      <c r="C97" s="7">
-        <v>49334</v>
+        <v>23</v>
+      </c>
+      <c r="B97" s="9"/>
+      <c r="C97" s="9">
+        <v>48337</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3589,11 +3593,11 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>48681</v>
+        <v>49334</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3602,11 +3606,11 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>49334</v>
+        <v>48681</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3615,11 +3619,11 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>49683</v>
+        <v>49334</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3628,11 +3632,11 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>50244</v>
+        <v>49683</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3640,8 +3644,17 @@
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="50" t="s">
+        <v>26</v>
+      </c>
       <c r="B102" s="7"/>
-      <c r="C102" s="7"/>
+      <c r="C102" s="7">
+        <v>50244</v>
+      </c>
+      <c r="D102" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B103" s="7"/>
@@ -3970,6 +3983,10 @@
     <row r="184" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
+    </row>
+    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B185" s="7"/>
+      <c r="C185" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - lv 20 done - 360 frames ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{707C4E90-FE63-40DE-9658-B727A92D0D40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D76F15E-A88D-418B-A22A-C1D9D6EAE5A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46845" yWindow="3210" windowWidth="10815" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="50250" yWindow="3210" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -2232,7 +2232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E185"/>
+  <dimension ref="A1:E192"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2519,7 +2519,7 @@
         <v>8196</v>
       </c>
       <c r="D19" s="3">
-        <f t="shared" ref="D19:D51" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
+        <f t="shared" ref="D19:D58" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
         <v>100</v>
       </c>
     </row>
@@ -2855,129 +2855,133 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="50" t="s">
-        <v>308</v>
-      </c>
-      <c r="B42" s="7"/>
-      <c r="C42" s="7">
-        <v>18719</v>
-      </c>
-      <c r="D42" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="A42" s="50"/>
+      <c r="B42" s="7">
+        <v>18193</v>
+      </c>
+      <c r="C42" s="37">
+        <v>18546</v>
+      </c>
+      <c r="D42" s="3">
+        <f t="shared" si="1"/>
+        <v>353</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="50" t="s">
-        <v>411</v>
-      </c>
-      <c r="B43" s="7"/>
-      <c r="C43" s="7">
-        <v>19068</v>
-      </c>
-      <c r="D43" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="A43" s="50"/>
+      <c r="B43" s="7">
+        <v>18226</v>
+      </c>
+      <c r="C43" s="37">
+        <v>18580</v>
+      </c>
+      <c r="D43" s="3">
+        <f t="shared" si="1"/>
+        <v>354</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="50" t="s">
-        <v>314</v>
-      </c>
-      <c r="B44" s="7"/>
-      <c r="C44" s="7">
-        <v>19892</v>
-      </c>
-      <c r="D44" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="A44" s="50"/>
+      <c r="B44" s="7">
+        <v>18255</v>
+      </c>
+      <c r="C44" s="37">
+        <v>18610</v>
+      </c>
+      <c r="D44" s="3">
+        <f t="shared" si="1"/>
+        <v>355</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="50" t="s">
-        <v>412</v>
-      </c>
-      <c r="B45" s="7"/>
-      <c r="C45" s="7">
-        <v>20240</v>
-      </c>
-      <c r="D45" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="A45" s="50"/>
+      <c r="B45" s="7">
+        <v>18270</v>
+      </c>
+      <c r="C45" s="37">
+        <v>18625</v>
+      </c>
+      <c r="D45" s="3">
+        <f t="shared" si="1"/>
+        <v>355</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="50" t="s">
-        <v>320</v>
-      </c>
-      <c r="B46" s="7"/>
-      <c r="C46" s="7">
-        <v>20813</v>
-      </c>
-      <c r="D46" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="A46" s="50"/>
+      <c r="B46" s="7">
+        <v>18291</v>
+      </c>
+      <c r="C46" s="37">
+        <v>18645</v>
+      </c>
+      <c r="D46" s="3">
+        <f t="shared" si="1"/>
+        <v>354</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="50" t="s">
-        <v>413</v>
-      </c>
-      <c r="B47" s="7"/>
-      <c r="C47" s="7">
-        <v>21161</v>
-      </c>
-      <c r="D47" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="A47" s="50"/>
+      <c r="B47" s="7">
+        <v>18326</v>
+      </c>
+      <c r="C47" s="37">
+        <v>18677</v>
+      </c>
+      <c r="D47" s="3">
+        <f t="shared" si="1"/>
+        <v>351</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="50" t="s">
-        <v>322</v>
-      </c>
-      <c r="B48" s="7"/>
-      <c r="C48" s="7">
-        <v>22195</v>
-      </c>
-      <c r="D48" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="A48" s="50"/>
+      <c r="B48" s="7">
+        <v>18339</v>
+      </c>
+      <c r="C48" s="37">
+        <v>18688</v>
+      </c>
+      <c r="D48" s="3">
+        <f t="shared" si="1"/>
+        <v>349</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="50" t="s">
-        <v>414</v>
-      </c>
-      <c r="B49" s="7"/>
+        <v>308</v>
+      </c>
+      <c r="B49" s="7">
+        <v>18359</v>
+      </c>
       <c r="C49" s="7">
-        <v>22543</v>
-      </c>
-      <c r="D49" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>18719</v>
+      </c>
+      <c r="D49" s="3">
+        <f t="shared" si="1"/>
+        <v>360</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="50" t="s">
-        <v>324</v>
-      </c>
-      <c r="B50" s="7"/>
+        <v>411</v>
+      </c>
+      <c r="B50" s="7">
+        <v>18708</v>
+      </c>
       <c r="C50" s="7">
-        <v>22963</v>
-      </c>
-      <c r="D50" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>19068</v>
+      </c>
+      <c r="D50" s="3">
+        <f t="shared" si="1"/>
+        <v>360</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="50" t="s">
-        <v>415</v>
+        <v>314</v>
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="7">
-        <v>23346</v>
+        <v>19892</v>
       </c>
       <c r="D51" s="3" t="str">
         <f t="shared" si="1"/>
@@ -2986,115 +2990,115 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="50" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="7">
-        <v>23873</v>
+        <v>20240</v>
       </c>
       <c r="D52" s="3" t="str">
-        <f t="shared" ref="D52:D81" si="2">IF(C52&lt;&gt;"",IF(B52&lt;&gt;"",C52-B52,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="50" t="s">
-        <v>417</v>
-      </c>
-      <c r="B53" s="8"/>
-      <c r="C53" s="50">
-        <v>24221</v>
+        <v>320</v>
+      </c>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7">
+        <v>20813</v>
       </c>
       <c r="D53" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="50" t="s">
-        <v>418</v>
-      </c>
-      <c r="B54" s="33"/>
-      <c r="C54" s="33">
-        <v>25101</v>
+        <v>413</v>
+      </c>
+      <c r="B54" s="7"/>
+      <c r="C54" s="7">
+        <v>21161</v>
       </c>
       <c r="D54" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="50" t="s">
-        <v>419</v>
+        <v>322</v>
       </c>
       <c r="B55" s="7"/>
       <c r="C55" s="7">
-        <v>25450</v>
+        <v>22195</v>
       </c>
       <c r="D55" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="50" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
       <c r="B56" s="7"/>
       <c r="C56" s="7">
-        <v>26350</v>
+        <v>22543</v>
       </c>
       <c r="D56" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="50" t="s">
-        <v>421</v>
+        <v>324</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7">
-        <v>26699</v>
+        <v>22963</v>
       </c>
       <c r="D57" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
-        <v>332</v>
+        <v>415</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7">
-        <v>27490</v>
+        <v>23346</v>
       </c>
       <c r="D58" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>5</v>
+        <v>416</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7">
-        <v>27836</v>
+        <v>23873</v>
       </c>
       <c r="D59" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="D59:D88" si="2">IF(C59&lt;&gt;"",IF(B59&lt;&gt;"",C59-B59,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>337</v>
-      </c>
-      <c r="B60" s="7"/>
-      <c r="C60" s="7">
-        <v>28899</v>
+        <v>417</v>
+      </c>
+      <c r="B60" s="8"/>
+      <c r="C60" s="50">
+        <v>24221</v>
       </c>
       <c r="D60" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3103,11 +3107,11 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>6</v>
-      </c>
-      <c r="B61" s="7"/>
-      <c r="C61" s="7">
-        <v>29248</v>
+        <v>418</v>
+      </c>
+      <c r="B61" s="33"/>
+      <c r="C61" s="33">
+        <v>25101</v>
       </c>
       <c r="D61" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3116,11 +3120,11 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>45</v>
+        <v>419</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7">
-        <v>29962</v>
+        <v>25450</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3129,11 +3133,11 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>7</v>
+        <v>420</v>
       </c>
       <c r="B63" s="7"/>
       <c r="C63" s="7">
-        <v>30309</v>
+        <v>26350</v>
       </c>
       <c r="D63" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3142,11 +3146,11 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>46</v>
+        <v>421</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7">
-        <v>30479</v>
+        <v>26699</v>
       </c>
       <c r="D64" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3155,27 +3159,24 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>8</v>
+        <v>332</v>
       </c>
       <c r="B65" s="7"/>
       <c r="C65" s="7">
-        <v>31125</v>
+        <v>27490</v>
       </c>
       <c r="D65" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E65" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="B66" s="7"/>
       <c r="C66" s="7">
-        <v>31643</v>
+        <v>27836</v>
       </c>
       <c r="D66" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3184,11 +3185,11 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>9</v>
+        <v>337</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>31991</v>
+        <v>28899</v>
       </c>
       <c r="D67" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3197,11 +3198,11 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7">
-        <v>32586</v>
+        <v>29248</v>
       </c>
       <c r="D68" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3210,27 +3211,24 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7">
-        <v>33254</v>
+        <v>29962</v>
       </c>
       <c r="D69" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E69" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>33883</v>
+        <v>30309</v>
       </c>
       <c r="D70" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3239,11 +3237,11 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>34244</v>
+        <v>30479</v>
       </c>
       <c r="D71" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3252,24 +3250,27 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>34862</v>
+        <v>31125</v>
       </c>
       <c r="D72" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E72" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>35218</v>
+        <v>31643</v>
       </c>
       <c r="D73" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3278,11 +3279,11 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>35772</v>
+        <v>31991</v>
       </c>
       <c r="D74" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3291,11 +3292,11 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>36120</v>
+        <v>32586</v>
       </c>
       <c r="D75" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3304,24 +3305,27 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>36893</v>
+        <v>33254</v>
       </c>
       <c r="D76" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E76" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>37238</v>
+        <v>33883</v>
       </c>
       <c r="D77" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3330,11 +3334,11 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>38097</v>
+        <v>34244</v>
       </c>
       <c r="D78" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3343,11 +3347,11 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>38443</v>
+        <v>34862</v>
       </c>
       <c r="D79" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3356,343 +3360,406 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>38692</v>
+        <v>35218</v>
       </c>
       <c r="D80" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>39041</v>
+        <v>35772</v>
       </c>
       <c r="D81" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>40011</v>
+        <v>36120</v>
       </c>
       <c r="D82" s="3" t="str">
-        <f>IF(C81&lt;&gt;"",IF(B81&lt;&gt;"",C81-B81,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="B83" s="7"/>
       <c r="C83" s="7">
-        <v>40373</v>
+        <v>36893</v>
       </c>
       <c r="D83" s="3" t="str">
-        <f t="shared" ref="D83:D102" si="3">IF(C83&lt;&gt;"",IF(B83&lt;&gt;"",C83-B83,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B84" s="40"/>
+        <v>48</v>
+      </c>
+      <c r="B84" s="7"/>
       <c r="C84" s="7">
-        <v>41117</v>
+        <v>37238</v>
       </c>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>41465</v>
+        <v>38097</v>
       </c>
       <c r="D85" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="B86" s="7"/>
       <c r="C86" s="7">
-        <v>42450</v>
+        <v>38443</v>
       </c>
       <c r="D86" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>42799</v>
+        <v>38692</v>
       </c>
       <c r="D87" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>43144</v>
+        <v>39041</v>
       </c>
       <c r="D88" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>43491</v>
+        <v>40011</v>
       </c>
       <c r="D89" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(C88&lt;&gt;"",IF(B88&lt;&gt;"",C88-B88,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>44165</v>
+        <v>40373</v>
       </c>
       <c r="D90" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="D90:D109" si="3">IF(C90&lt;&gt;"",IF(B90&lt;&gt;"",C90-B90,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>20</v>
-      </c>
-      <c r="B91" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B91" s="40"/>
       <c r="C91" s="7">
-        <v>44512</v>
+        <v>41117</v>
       </c>
       <c r="D91" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>45061</v>
+        <v>41465</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>45443</v>
+        <v>42450</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>45990</v>
+        <v>42799</v>
       </c>
       <c r="D94" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>46652</v>
+        <v>43144</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E95" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="B96" s="7"/>
       <c r="C96" s="7">
-        <v>47436</v>
+        <v>43491</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B97" s="9"/>
-      <c r="C97" s="9">
-        <v>48337</v>
+        <v>39</v>
+      </c>
+      <c r="B97" s="7"/>
+      <c r="C97" s="7">
+        <v>44165</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>49334</v>
+        <v>44512</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>48681</v>
+        <v>45061</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>49334</v>
+        <v>45443</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>49683</v>
+        <v>45990</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="50" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B102" s="7"/>
       <c r="C102" s="7">
-        <v>50244</v>
+        <v>46652</v>
       </c>
       <c r="D102" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E102" s="51" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="50" t="s">
+        <v>42</v>
+      </c>
       <c r="B103" s="7"/>
-      <c r="C103" s="7"/>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B104" s="7"/>
-      <c r="C104" s="7"/>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C103" s="7">
+        <v>47436</v>
+      </c>
+      <c r="D103" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="50" t="s">
+        <v>23</v>
+      </c>
+      <c r="B104" s="9"/>
+      <c r="C104" s="9">
+        <v>48337</v>
+      </c>
+      <c r="D104" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="50" t="s">
+        <v>43</v>
+      </c>
       <c r="B105" s="7"/>
-      <c r="C105" s="7"/>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C105" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D105" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="50" t="s">
+        <v>24</v>
+      </c>
       <c r="B106" s="7"/>
-      <c r="C106" s="7"/>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C106" s="7">
+        <v>48681</v>
+      </c>
+      <c r="D106" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="50" t="s">
+        <v>44</v>
+      </c>
       <c r="B107" s="7"/>
-      <c r="C107" s="7"/>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C107" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D107" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" s="50" t="s">
+        <v>25</v>
+      </c>
       <c r="B108" s="7"/>
-      <c r="C108" s="7"/>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C108" s="7">
+        <v>49683</v>
+      </c>
+      <c r="D108" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" s="50" t="s">
+        <v>26</v>
+      </c>
       <c r="B109" s="7"/>
-      <c r="C109" s="7"/>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C109" s="7">
+        <v>50244</v>
+      </c>
+      <c r="D109" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
     </row>
@@ -3987,6 +4054,34 @@
     <row r="185" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B185" s="7"/>
       <c r="C185" s="7"/>
+    </row>
+    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B186" s="7"/>
+      <c r="C186" s="7"/>
+    </row>
+    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B187" s="7"/>
+      <c r="C187" s="7"/>
+    </row>
+    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B188" s="7"/>
+      <c r="C188" s="7"/>
+    </row>
+    <row r="189" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B189" s="7"/>
+      <c r="C189" s="7"/>
+    </row>
+    <row r="190" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B190" s="7"/>
+      <c r="C190" s="7"/>
+    </row>
+    <row r="191" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B191" s="7"/>
+      <c r="C191" s="7"/>
+    </row>
+    <row r="192" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B192" s="7"/>
+      <c r="C192" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lde runner - lv 21 done - 372 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D76F15E-A88D-418B-A22A-C1D9D6EAE5A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55281626-403D-4563-95D6-C947EA1717AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50250" yWindow="3210" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1887,6 +1887,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1911,7 +1912,6 @@
     <xf numFmtId="0" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2800,7 +2800,7 @@
       <c r="A38" s="50" t="s">
         <v>408</v>
       </c>
-      <c r="B38" s="60">
+      <c r="B38" s="52">
         <v>17147</v>
       </c>
       <c r="C38" s="7">
@@ -2813,7 +2813,7 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="50"/>
-      <c r="B39" s="60">
+      <c r="B39" s="52">
         <v>17287</v>
       </c>
       <c r="C39" s="7">
@@ -2979,26 +2979,30 @@
       <c r="A51" s="50" t="s">
         <v>314</v>
       </c>
-      <c r="B51" s="7"/>
+      <c r="B51" s="7">
+        <v>19521</v>
+      </c>
       <c r="C51" s="7">
         <v>19892</v>
       </c>
-      <c r="D51" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="D51" s="3">
+        <f t="shared" si="1"/>
+        <v>371</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="50" t="s">
         <v>412</v>
       </c>
-      <c r="B52" s="7"/>
+      <c r="B52" s="7">
+        <v>19868</v>
+      </c>
       <c r="C52" s="7">
         <v>20240</v>
       </c>
-      <c r="D52" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+      <c r="D52" s="3">
+        <f t="shared" si="1"/>
+        <v>372</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -18960,10 +18964,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="52" t="s">
+      <c r="K1" s="53" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="53"/>
+      <c r="L1" s="54"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -20815,13 +20819,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="54" t="s">
+      <c r="H53" s="55" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="55"/>
-      <c r="J53" s="55"/>
-      <c r="K53" s="55"/>
-      <c r="L53" s="56"/>
+      <c r="I53" s="56"/>
+      <c r="J53" s="56"/>
+      <c r="K53" s="56"/>
+      <c r="L53" s="57"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -20843,11 +20847,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="57"/>
-      <c r="I54" s="58"/>
-      <c r="J54" s="58"/>
-      <c r="K54" s="58"/>
-      <c r="L54" s="59"/>
+      <c r="H54" s="58"/>
+      <c r="I54" s="59"/>
+      <c r="J54" s="59"/>
+      <c r="K54" s="59"/>
+      <c r="L54" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - level 21 done - 389 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55281626-403D-4563-95D6-C947EA1717AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11233B6-F946-401B-AF65-8B24DF352544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50250" yWindow="3210" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2232,7 +2232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E192"/>
+  <dimension ref="A1:E187"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2519,7 +2519,7 @@
         <v>8196</v>
       </c>
       <c r="D19" s="3">
-        <f t="shared" ref="D19:D58" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
+        <f t="shared" ref="D19:D53" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
         <v>100</v>
       </c>
     </row>
@@ -2812,206 +2812,210 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="50"/>
-      <c r="B39" s="52">
-        <v>17287</v>
+      <c r="A39" s="50" t="s">
+        <v>305</v>
+      </c>
+      <c r="B39" s="7">
+        <v>17443</v>
       </c>
       <c r="C39" s="7">
-        <v>17625</v>
+        <v>17791</v>
       </c>
       <c r="D39" s="3">
         <f t="shared" si="1"/>
-        <v>338</v>
+        <v>348</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="50" t="s">
-        <v>305</v>
+        <v>409</v>
       </c>
       <c r="B40" s="7">
-        <v>17443</v>
-      </c>
-      <c r="C40" s="7">
-        <v>17791</v>
+        <v>17790</v>
+      </c>
+      <c r="C40" s="37">
+        <v>18139</v>
       </c>
       <c r="D40" s="3">
         <f t="shared" si="1"/>
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="50" t="s">
-        <v>409</v>
+        <v>308</v>
       </c>
       <c r="B41" s="7">
-        <v>17790</v>
-      </c>
-      <c r="C41" s="37">
-        <v>18139</v>
+        <v>18359</v>
+      </c>
+      <c r="C41" s="7">
+        <v>18719</v>
       </c>
       <c r="D41" s="3">
         <f t="shared" si="1"/>
-        <v>349</v>
+        <v>360</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="50"/>
+      <c r="A42" s="50" t="s">
+        <v>411</v>
+      </c>
       <c r="B42" s="7">
-        <v>18193</v>
-      </c>
-      <c r="C42" s="37">
-        <v>18546</v>
+        <v>18708</v>
+      </c>
+      <c r="C42" s="7">
+        <v>19068</v>
       </c>
       <c r="D42" s="3">
         <f t="shared" si="1"/>
-        <v>353</v>
+        <v>360</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="50"/>
+      <c r="A43" s="50" t="s">
+        <v>314</v>
+      </c>
       <c r="B43" s="7">
-        <v>18226</v>
-      </c>
-      <c r="C43" s="37">
-        <v>18580</v>
+        <v>19521</v>
+      </c>
+      <c r="C43" s="7">
+        <v>19892</v>
       </c>
       <c r="D43" s="3">
         <f t="shared" si="1"/>
-        <v>354</v>
+        <v>371</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="50"/>
+      <c r="A44" s="50" t="s">
+        <v>412</v>
+      </c>
       <c r="B44" s="7">
-        <v>18255</v>
-      </c>
-      <c r="C44" s="37">
-        <v>18610</v>
+        <v>19868</v>
+      </c>
+      <c r="C44" s="7">
+        <v>20240</v>
       </c>
       <c r="D44" s="3">
         <f t="shared" si="1"/>
-        <v>355</v>
+        <v>372</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="50"/>
       <c r="B45" s="7">
-        <v>18270</v>
-      </c>
-      <c r="C45" s="37">
-        <v>18625</v>
+        <v>20112</v>
+      </c>
+      <c r="C45" s="7">
+        <v>20491</v>
       </c>
       <c r="D45" s="3">
         <f t="shared" si="1"/>
-        <v>355</v>
+        <v>379</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="50"/>
       <c r="B46" s="7">
-        <v>18291</v>
-      </c>
-      <c r="C46" s="37">
-        <v>18645</v>
+        <v>20117</v>
+      </c>
+      <c r="C46" s="7">
+        <v>20491</v>
       </c>
       <c r="D46" s="3">
         <f t="shared" si="1"/>
-        <v>354</v>
+        <v>374</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="50"/>
       <c r="B47" s="7">
-        <v>18326</v>
-      </c>
-      <c r="C47" s="37">
-        <v>18677</v>
+        <v>20155</v>
+      </c>
+      <c r="C47" s="7">
+        <v>20529</v>
       </c>
       <c r="D47" s="3">
         <f t="shared" si="1"/>
-        <v>351</v>
+        <v>374</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="50"/>
+      <c r="A48" s="50" t="s">
+        <v>320</v>
+      </c>
       <c r="B48" s="7">
-        <v>18339</v>
-      </c>
-      <c r="C48" s="37">
-        <v>18688</v>
+        <v>20425</v>
+      </c>
+      <c r="C48" s="7">
+        <v>20813</v>
       </c>
       <c r="D48" s="3">
         <f t="shared" si="1"/>
-        <v>349</v>
+        <v>388</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="50" t="s">
-        <v>308</v>
+        <v>413</v>
       </c>
       <c r="B49" s="7">
-        <v>18359</v>
+        <v>20772</v>
       </c>
       <c r="C49" s="7">
-        <v>18719</v>
+        <v>21161</v>
       </c>
       <c r="D49" s="3">
         <f t="shared" si="1"/>
-        <v>360</v>
+        <v>389</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="50" t="s">
-        <v>411</v>
-      </c>
-      <c r="B50" s="7">
-        <v>18708</v>
-      </c>
+        <v>322</v>
+      </c>
+      <c r="B50" s="7"/>
       <c r="C50" s="7">
-        <v>19068</v>
-      </c>
-      <c r="D50" s="3">
-        <f t="shared" si="1"/>
-        <v>360</v>
+        <v>22195</v>
+      </c>
+      <c r="D50" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="50" t="s">
-        <v>314</v>
-      </c>
-      <c r="B51" s="7">
-        <v>19521</v>
-      </c>
+        <v>414</v>
+      </c>
+      <c r="B51" s="7"/>
       <c r="C51" s="7">
-        <v>19892</v>
-      </c>
-      <c r="D51" s="3">
-        <f t="shared" si="1"/>
-        <v>371</v>
+        <v>22543</v>
+      </c>
+      <c r="D51" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="50" t="s">
-        <v>412</v>
-      </c>
-      <c r="B52" s="7">
-        <v>19868</v>
-      </c>
+        <v>324</v>
+      </c>
+      <c r="B52" s="7"/>
       <c r="C52" s="7">
-        <v>20240</v>
-      </c>
-      <c r="D52" s="3">
-        <f t="shared" si="1"/>
-        <v>372</v>
+        <v>22963</v>
+      </c>
+      <c r="D52" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="50" t="s">
-        <v>320</v>
+        <v>415</v>
       </c>
       <c r="B53" s="7"/>
       <c r="C53" s="7">
-        <v>20813</v>
+        <v>23346</v>
       </c>
       <c r="D53" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3020,89 +3024,89 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="50" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="7">
-        <v>21161</v>
+        <v>23873</v>
       </c>
       <c r="D54" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="D54:D83" si="2">IF(C54&lt;&gt;"",IF(B54&lt;&gt;"",C54-B54,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="50" t="s">
-        <v>322</v>
-      </c>
-      <c r="B55" s="7"/>
-      <c r="C55" s="7">
-        <v>22195</v>
+        <v>417</v>
+      </c>
+      <c r="B55" s="8"/>
+      <c r="C55" s="50">
+        <v>24221</v>
       </c>
       <c r="D55" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="50" t="s">
-        <v>414</v>
-      </c>
-      <c r="B56" s="7"/>
-      <c r="C56" s="7">
-        <v>22543</v>
+        <v>418</v>
+      </c>
+      <c r="B56" s="33"/>
+      <c r="C56" s="33">
+        <v>25101</v>
       </c>
       <c r="D56" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="50" t="s">
-        <v>324</v>
+        <v>419</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7">
-        <v>22963</v>
+        <v>25450</v>
       </c>
       <c r="D57" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7">
-        <v>23346</v>
+        <v>26350</v>
       </c>
       <c r="D58" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7">
-        <v>23873</v>
+        <v>26699</v>
       </c>
       <c r="D59" s="3" t="str">
-        <f t="shared" ref="D59:D88" si="2">IF(C59&lt;&gt;"",IF(B59&lt;&gt;"",C59-B59,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>417</v>
-      </c>
-      <c r="B60" s="8"/>
-      <c r="C60" s="50">
-        <v>24221</v>
+        <v>332</v>
+      </c>
+      <c r="B60" s="7"/>
+      <c r="C60" s="7">
+        <v>27490</v>
       </c>
       <c r="D60" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3111,11 +3115,11 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>418</v>
-      </c>
-      <c r="B61" s="33"/>
-      <c r="C61" s="33">
-        <v>25101</v>
+        <v>5</v>
+      </c>
+      <c r="B61" s="7"/>
+      <c r="C61" s="7">
+        <v>27836</v>
       </c>
       <c r="D61" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3124,11 +3128,11 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>419</v>
+        <v>337</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7">
-        <v>25450</v>
+        <v>28899</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3137,11 +3141,11 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>420</v>
+        <v>6</v>
       </c>
       <c r="B63" s="7"/>
       <c r="C63" s="7">
-        <v>26350</v>
+        <v>29248</v>
       </c>
       <c r="D63" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3150,11 +3154,11 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>421</v>
+        <v>45</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7">
-        <v>26699</v>
+        <v>29962</v>
       </c>
       <c r="D64" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3163,11 +3167,11 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>332</v>
+        <v>7</v>
       </c>
       <c r="B65" s="7"/>
       <c r="C65" s="7">
-        <v>27490</v>
+        <v>30309</v>
       </c>
       <c r="D65" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3176,11 +3180,11 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="B66" s="7"/>
       <c r="C66" s="7">
-        <v>27836</v>
+        <v>30479</v>
       </c>
       <c r="D66" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3189,24 +3193,27 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>337</v>
+        <v>8</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>28899</v>
+        <v>31125</v>
       </c>
       <c r="D67" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E67" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7">
-        <v>29248</v>
+        <v>31643</v>
       </c>
       <c r="D68" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3215,11 +3222,11 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7">
-        <v>29962</v>
+        <v>31991</v>
       </c>
       <c r="D69" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3228,11 +3235,11 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>30309</v>
+        <v>32586</v>
       </c>
       <c r="D70" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3241,40 +3248,40 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>30479</v>
+        <v>33254</v>
       </c>
       <c r="D71" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E71" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>31125</v>
+        <v>33883</v>
       </c>
       <c r="D72" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E72" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>31643</v>
+        <v>34244</v>
       </c>
       <c r="D73" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3283,11 +3290,11 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>31991</v>
+        <v>34862</v>
       </c>
       <c r="D74" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3296,11 +3303,11 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>32586</v>
+        <v>35218</v>
       </c>
       <c r="D75" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3309,27 +3316,24 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>33254</v>
+        <v>35772</v>
       </c>
       <c r="D76" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E76" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>33883</v>
+        <v>36120</v>
       </c>
       <c r="D77" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3338,11 +3342,11 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>34244</v>
+        <v>36893</v>
       </c>
       <c r="D78" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3351,11 +3355,11 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>34862</v>
+        <v>37238</v>
       </c>
       <c r="D79" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3364,11 +3368,11 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>35218</v>
+        <v>38097</v>
       </c>
       <c r="D80" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3377,11 +3381,11 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>35772</v>
+        <v>38443</v>
       </c>
       <c r="D81" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3390,11 +3394,11 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>36120</v>
+        <v>38692</v>
       </c>
       <c r="D82" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3403,11 +3407,11 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="B83" s="7"/>
       <c r="C83" s="7">
-        <v>36893</v>
+        <v>39041</v>
       </c>
       <c r="D83" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3416,102 +3420,102 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="B84" s="7"/>
       <c r="C84" s="7">
-        <v>37238</v>
+        <v>40011</v>
       </c>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(C83&lt;&gt;"",IF(B83&lt;&gt;"",C83-B83,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>38097</v>
+        <v>40373</v>
       </c>
       <c r="D85" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="D85:D104" si="3">IF(C85&lt;&gt;"",IF(B85&lt;&gt;"",C85-B85,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>14</v>
-      </c>
-      <c r="B86" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B86" s="40"/>
       <c r="C86" s="7">
-        <v>38443</v>
+        <v>41117</v>
       </c>
       <c r="D86" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>38692</v>
+        <v>41465</v>
       </c>
       <c r="D87" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>39041</v>
+        <v>42450</v>
       </c>
       <c r="D88" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>40011</v>
+        <v>42799</v>
       </c>
       <c r="D89" s="3" t="str">
-        <f>IF(C88&lt;&gt;"",IF(B88&lt;&gt;"",C88-B88,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>40373</v>
+        <v>43144</v>
       </c>
       <c r="D90" s="3" t="str">
-        <f t="shared" ref="D90:D109" si="3">IF(C90&lt;&gt;"",IF(B90&lt;&gt;"",C90-B90,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B91" s="40"/>
+        <v>19</v>
+      </c>
+      <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>41117</v>
+        <v>43491</v>
       </c>
       <c r="D91" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3520,11 +3524,11 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>41465</v>
+        <v>44165</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3533,11 +3537,11 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>42450</v>
+        <v>44512</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3546,11 +3550,11 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>42799</v>
+        <v>45061</v>
       </c>
       <c r="D94" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3559,11 +3563,11 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>43144</v>
+        <v>45443</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3572,11 +3576,11 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="B96" s="7"/>
       <c r="C96" s="7">
-        <v>43491</v>
+        <v>45990</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3585,24 +3589,27 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>44165</v>
+        <v>46652</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
+      <c r="E97" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>44512</v>
+        <v>47436</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3611,11 +3618,11 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>40</v>
-      </c>
-      <c r="B99" s="7"/>
-      <c r="C99" s="7">
-        <v>45061</v>
+        <v>23</v>
+      </c>
+      <c r="B99" s="9"/>
+      <c r="C99" s="9">
+        <v>48337</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3624,11 +3631,11 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>45443</v>
+        <v>49334</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3637,11 +3644,11 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>45990</v>
+        <v>48681</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3650,27 +3657,24 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="50" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="B102" s="7"/>
       <c r="C102" s="7">
-        <v>46652</v>
+        <v>49334</v>
       </c>
       <c r="D102" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E102" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="50" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="B103" s="7"/>
       <c r="C103" s="7">
-        <v>47436</v>
+        <v>49683</v>
       </c>
       <c r="D103" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3679,11 +3683,11 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B104" s="9"/>
-      <c r="C104" s="9">
-        <v>48337</v>
+        <v>26</v>
+      </c>
+      <c r="B104" s="7"/>
+      <c r="C104" s="7">
+        <v>50244</v>
       </c>
       <c r="D104" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3691,69 +3695,24 @@
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="50" t="s">
-        <v>43</v>
-      </c>
       <c r="B105" s="7"/>
-      <c r="C105" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D105" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
+      <c r="C105" s="7"/>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="50" t="s">
-        <v>24</v>
-      </c>
       <c r="B106" s="7"/>
-      <c r="C106" s="7">
-        <v>48681</v>
-      </c>
-      <c r="D106" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
+      <c r="C106" s="7"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="50" t="s">
-        <v>44</v>
-      </c>
       <c r="B107" s="7"/>
-      <c r="C107" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D107" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
+      <c r="C107" s="7"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" s="50" t="s">
-        <v>25</v>
-      </c>
       <c r="B108" s="7"/>
-      <c r="C108" s="7">
-        <v>49683</v>
-      </c>
-      <c r="D108" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
+      <c r="C108" s="7"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A109" s="50" t="s">
-        <v>26</v>
-      </c>
       <c r="B109" s="7"/>
-      <c r="C109" s="7">
-        <v>50244</v>
-      </c>
-      <c r="D109" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
+      <c r="C109" s="7"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
@@ -4066,26 +4025,6 @@
     <row r="187" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B187" s="7"/>
       <c r="C187" s="7"/>
-    </row>
-    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B188" s="7"/>
-      <c r="C188" s="7"/>
-    </row>
-    <row r="189" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B189" s="7"/>
-      <c r="C189" s="7"/>
-    </row>
-    <row r="190" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B190" s="7"/>
-      <c r="C190" s="7"/>
-    </row>
-    <row r="191" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B191" s="7"/>
-      <c r="C191" s="7"/>
-    </row>
-    <row r="192" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B192" s="7"/>
-      <c r="C192" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - lv 23 done - 405 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11233B6-F946-401B-AF65-8B24DF352544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC6B78AB-9D6A-46C2-BC0D-36215B9462B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50250" yWindow="3210" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2232,7 +2232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E187"/>
+  <dimension ref="A1:E188"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2519,7 +2519,7 @@
         <v>8196</v>
       </c>
       <c r="D19" s="3">
-        <f t="shared" ref="D19:D53" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
+        <f t="shared" ref="D19:D54" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
         <v>100</v>
       </c>
     </row>
@@ -2971,51 +2971,55 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="50" t="s">
-        <v>322</v>
-      </c>
-      <c r="B50" s="7"/>
+      <c r="A50" s="50"/>
+      <c r="B50" s="7">
+        <v>20983</v>
+      </c>
       <c r="C50" s="7">
-        <v>22195</v>
-      </c>
-      <c r="D50" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>21378</v>
+      </c>
+      <c r="D50" s="3">
+        <f t="shared" si="1"/>
+        <v>395</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="50" t="s">
-        <v>414</v>
-      </c>
-      <c r="B51" s="7"/>
+        <v>322</v>
+      </c>
+      <c r="B51" s="7">
+        <v>21789</v>
+      </c>
       <c r="C51" s="7">
-        <v>22543</v>
-      </c>
-      <c r="D51" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>22195</v>
+      </c>
+      <c r="D51" s="3">
+        <f t="shared" si="1"/>
+        <v>406</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="50" t="s">
-        <v>324</v>
-      </c>
-      <c r="B52" s="7"/>
+        <v>414</v>
+      </c>
+      <c r="B52" s="7">
+        <v>22138</v>
+      </c>
       <c r="C52" s="7">
-        <v>22963</v>
-      </c>
-      <c r="D52" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>-</v>
+        <v>22543</v>
+      </c>
+      <c r="D52" s="3">
+        <f t="shared" si="1"/>
+        <v>405</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="50" t="s">
-        <v>415</v>
+        <v>324</v>
       </c>
       <c r="B53" s="7"/>
       <c r="C53" s="7">
-        <v>23346</v>
+        <v>22963</v>
       </c>
       <c r="D53" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3024,37 +3028,37 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="50" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="7">
-        <v>23873</v>
+        <v>23346</v>
       </c>
       <c r="D54" s="3" t="str">
-        <f t="shared" ref="D54:D83" si="2">IF(C54&lt;&gt;"",IF(B54&lt;&gt;"",C54-B54,"-"), "-")</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="50" t="s">
-        <v>417</v>
-      </c>
-      <c r="B55" s="8"/>
-      <c r="C55" s="50">
-        <v>24221</v>
+        <v>416</v>
+      </c>
+      <c r="B55" s="7"/>
+      <c r="C55" s="7">
+        <v>23873</v>
       </c>
       <c r="D55" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="D55:D84" si="2">IF(C55&lt;&gt;"",IF(B55&lt;&gt;"",C55-B55,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="50" t="s">
-        <v>418</v>
-      </c>
-      <c r="B56" s="33"/>
-      <c r="C56" s="33">
-        <v>25101</v>
+        <v>417</v>
+      </c>
+      <c r="B56" s="8"/>
+      <c r="C56" s="50">
+        <v>24221</v>
       </c>
       <c r="D56" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3063,11 +3067,11 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="50" t="s">
-        <v>419</v>
-      </c>
-      <c r="B57" s="7"/>
-      <c r="C57" s="7">
-        <v>25450</v>
+        <v>418</v>
+      </c>
+      <c r="B57" s="33"/>
+      <c r="C57" s="33">
+        <v>25101</v>
       </c>
       <c r="D57" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3076,11 +3080,11 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7">
-        <v>26350</v>
+        <v>25450</v>
       </c>
       <c r="D58" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3089,11 +3093,11 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7">
-        <v>26699</v>
+        <v>26350</v>
       </c>
       <c r="D59" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3102,11 +3106,11 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>332</v>
+        <v>421</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7">
-        <v>27490</v>
+        <v>26699</v>
       </c>
       <c r="D60" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3115,11 +3119,11 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>5</v>
+        <v>332</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7">
-        <v>27836</v>
+        <v>27490</v>
       </c>
       <c r="D61" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3128,11 +3132,11 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>337</v>
+        <v>5</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7">
-        <v>28899</v>
+        <v>27836</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3141,11 +3145,11 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>6</v>
+        <v>337</v>
       </c>
       <c r="B63" s="7"/>
       <c r="C63" s="7">
-        <v>29248</v>
+        <v>28899</v>
       </c>
       <c r="D63" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3154,11 +3158,11 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7">
-        <v>29962</v>
+        <v>29248</v>
       </c>
       <c r="D64" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3167,11 +3171,11 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="B65" s="7"/>
       <c r="C65" s="7">
-        <v>30309</v>
+        <v>29962</v>
       </c>
       <c r="D65" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3180,11 +3184,11 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="B66" s="7"/>
       <c r="C66" s="7">
-        <v>30479</v>
+        <v>30309</v>
       </c>
       <c r="D66" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3193,40 +3197,40 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>31125</v>
+        <v>30479</v>
       </c>
       <c r="D67" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E67" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7">
-        <v>31643</v>
+        <v>31125</v>
       </c>
       <c r="D68" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E68" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7">
-        <v>31991</v>
+        <v>31643</v>
       </c>
       <c r="D69" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3235,11 +3239,11 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>32586</v>
+        <v>31991</v>
       </c>
       <c r="D70" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3248,40 +3252,40 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>33254</v>
+        <v>32586</v>
       </c>
       <c r="D71" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E71" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>33883</v>
+        <v>33254</v>
       </c>
       <c r="D72" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E72" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>34244</v>
+        <v>33883</v>
       </c>
       <c r="D73" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3290,11 +3294,11 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>34862</v>
+        <v>34244</v>
       </c>
       <c r="D74" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3303,11 +3307,11 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>35218</v>
+        <v>34862</v>
       </c>
       <c r="D75" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3316,11 +3320,11 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>35772</v>
+        <v>35218</v>
       </c>
       <c r="D76" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3329,11 +3333,11 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>36120</v>
+        <v>35772</v>
       </c>
       <c r="D77" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3342,11 +3346,11 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>36893</v>
+        <v>36120</v>
       </c>
       <c r="D78" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3355,11 +3359,11 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>37238</v>
+        <v>36893</v>
       </c>
       <c r="D79" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3368,11 +3372,11 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>38097</v>
+        <v>37238</v>
       </c>
       <c r="D80" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3381,11 +3385,11 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>38443</v>
+        <v>38097</v>
       </c>
       <c r="D81" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3394,11 +3398,11 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>38692</v>
+        <v>38443</v>
       </c>
       <c r="D82" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3407,11 +3411,11 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="B83" s="7"/>
       <c r="C83" s="7">
-        <v>39041</v>
+        <v>38692</v>
       </c>
       <c r="D83" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3420,50 +3424,50 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="B84" s="7"/>
       <c r="C84" s="7">
-        <v>40011</v>
+        <v>39041</v>
       </c>
       <c r="D84" s="3" t="str">
-        <f>IF(C83&lt;&gt;"",IF(B83&lt;&gt;"",C83-B83,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>40373</v>
+        <v>40011</v>
       </c>
       <c r="D85" s="3" t="str">
-        <f t="shared" ref="D85:D104" si="3">IF(C85&lt;&gt;"",IF(B85&lt;&gt;"",C85-B85,"-"), "-")</f>
+        <f>IF(C84&lt;&gt;"",IF(B84&lt;&gt;"",C84-B84,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B86" s="40"/>
+        <v>16</v>
+      </c>
+      <c r="B86" s="7"/>
       <c r="C86" s="7">
-        <v>41117</v>
+        <v>40373</v>
       </c>
       <c r="D86" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="D86:D105" si="3">IF(C86&lt;&gt;"",IF(B86&lt;&gt;"",C86-B86,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="B87" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B87" s="40"/>
       <c r="C87" s="7">
-        <v>41465</v>
+        <v>41117</v>
       </c>
       <c r="D87" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3472,11 +3476,11 @@
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>42450</v>
+        <v>41465</v>
       </c>
       <c r="D88" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3485,11 +3489,11 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>42799</v>
+        <v>42450</v>
       </c>
       <c r="D89" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3498,11 +3502,11 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>43144</v>
+        <v>42799</v>
       </c>
       <c r="D90" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3511,11 +3515,11 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>43491</v>
+        <v>43144</v>
       </c>
       <c r="D91" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3524,11 +3528,11 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>44165</v>
+        <v>43491</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3537,11 +3541,11 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>44512</v>
+        <v>44165</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3550,11 +3554,11 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>45061</v>
+        <v>44512</v>
       </c>
       <c r="D94" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3563,11 +3567,11 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>45443</v>
+        <v>45061</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3576,11 +3580,11 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="B96" s="7"/>
       <c r="C96" s="7">
-        <v>45990</v>
+        <v>45443</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3589,40 +3593,40 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>46652</v>
+        <v>45990</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E97" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>47436</v>
+        <v>46652</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
+      <c r="E98" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B99" s="9"/>
-      <c r="C99" s="9">
-        <v>48337</v>
+        <v>42</v>
+      </c>
+      <c r="B99" s="7"/>
+      <c r="C99" s="7">
+        <v>47436</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3631,11 +3635,11 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>43</v>
-      </c>
-      <c r="B100" s="7"/>
-      <c r="C100" s="7">
-        <v>49334</v>
+        <v>23</v>
+      </c>
+      <c r="B100" s="9"/>
+      <c r="C100" s="9">
+        <v>48337</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3644,11 +3648,11 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>48681</v>
+        <v>49334</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3657,11 +3661,11 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="50" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="B102" s="7"/>
       <c r="C102" s="7">
-        <v>49334</v>
+        <v>48681</v>
       </c>
       <c r="D102" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3670,11 +3674,11 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="50" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="B103" s="7"/>
       <c r="C103" s="7">
-        <v>49683</v>
+        <v>49334</v>
       </c>
       <c r="D103" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3683,11 +3687,11 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="50" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B104" s="7"/>
       <c r="C104" s="7">
-        <v>50244</v>
+        <v>49683</v>
       </c>
       <c r="D104" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3695,8 +3699,17 @@
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="50" t="s">
+        <v>26</v>
+      </c>
       <c r="B105" s="7"/>
-      <c r="C105" s="7"/>
+      <c r="C105" s="7">
+        <v>50244</v>
+      </c>
+      <c r="D105" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B106" s="7"/>
@@ -4025,6 +4038,10 @@
     <row r="187" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B187" s="7"/>
       <c r="C187" s="7"/>
+    </row>
+    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B188" s="7"/>
+      <c r="C188" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
level 24 done, 410 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC6B78AB-9D6A-46C2-BC0D-36215B9462B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1826C14F-7E64-4E35-9B5A-125625CFCD3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50250" yWindow="3210" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2232,7 +2232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E188"/>
+  <dimension ref="A1:E184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2519,7 +2519,7 @@
         <v>8196</v>
       </c>
       <c r="D19" s="3">
-        <f t="shared" ref="D19:D54" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
+        <f t="shared" ref="D19:D50" si="1">IF(C19&lt;&gt;"",IF(B19&lt;&gt;"",C19-B19,"-"), "-")</f>
         <v>100</v>
       </c>
     </row>
@@ -2902,280 +2902,287 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="50"/>
+      <c r="A45" s="50" t="s">
+        <v>320</v>
+      </c>
       <c r="B45" s="7">
-        <v>20112</v>
+        <v>20425</v>
       </c>
       <c r="C45" s="7">
-        <v>20491</v>
+        <v>20813</v>
       </c>
       <c r="D45" s="3">
         <f t="shared" si="1"/>
-        <v>379</v>
+        <v>388</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="50"/>
+      <c r="A46" s="50" t="s">
+        <v>413</v>
+      </c>
       <c r="B46" s="7">
-        <v>20117</v>
+        <v>20772</v>
       </c>
       <c r="C46" s="7">
-        <v>20491</v>
+        <v>21161</v>
       </c>
       <c r="D46" s="3">
         <f t="shared" si="1"/>
-        <v>374</v>
+        <v>389</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="50"/>
+      <c r="A47" s="50" t="s">
+        <v>322</v>
+      </c>
       <c r="B47" s="7">
-        <v>20155</v>
+        <v>21789</v>
       </c>
       <c r="C47" s="7">
-        <v>20529</v>
+        <v>22195</v>
       </c>
       <c r="D47" s="3">
         <f t="shared" si="1"/>
-        <v>374</v>
+        <v>406</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="50" t="s">
-        <v>320</v>
+        <v>414</v>
       </c>
       <c r="B48" s="7">
-        <v>20425</v>
+        <v>22138</v>
       </c>
       <c r="C48" s="7">
-        <v>20813</v>
+        <v>22543</v>
       </c>
       <c r="D48" s="3">
         <f t="shared" si="1"/>
-        <v>388</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="50" t="s">
-        <v>413</v>
+        <v>324</v>
       </c>
       <c r="B49" s="7">
-        <v>20772</v>
+        <v>22553</v>
       </c>
       <c r="C49" s="7">
-        <v>21161</v>
+        <v>22963</v>
       </c>
       <c r="D49" s="3">
         <f t="shared" si="1"/>
-        <v>389</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="50"/>
+        <v>410</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="50" t="s">
+        <v>415</v>
+      </c>
       <c r="B50" s="7">
-        <v>20983</v>
+        <v>22936</v>
       </c>
       <c r="C50" s="7">
-        <v>21378</v>
+        <v>23346</v>
       </c>
       <c r="D50" s="3">
         <f t="shared" si="1"/>
-        <v>395</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="50" t="s">
-        <v>322</v>
-      </c>
-      <c r="B51" s="7">
-        <v>21789</v>
-      </c>
+        <v>416</v>
+      </c>
+      <c r="B51" s="7"/>
       <c r="C51" s="7">
-        <v>22195</v>
-      </c>
-      <c r="D51" s="3">
-        <f t="shared" si="1"/>
-        <v>406</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+        <v>23873</v>
+      </c>
+      <c r="D51" s="3" t="str">
+        <f t="shared" ref="D51:D80" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="50" t="s">
-        <v>414</v>
-      </c>
-      <c r="B52" s="7">
-        <v>22138</v>
-      </c>
-      <c r="C52" s="7">
-        <v>22543</v>
-      </c>
-      <c r="D52" s="3">
-        <f t="shared" si="1"/>
-        <v>405</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+        <v>417</v>
+      </c>
+      <c r="B52" s="8"/>
+      <c r="C52" s="50">
+        <v>24221</v>
+      </c>
+      <c r="D52" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="50" t="s">
-        <v>324</v>
-      </c>
-      <c r="B53" s="7"/>
-      <c r="C53" s="7">
-        <v>22963</v>
+        <v>418</v>
+      </c>
+      <c r="B53" s="33"/>
+      <c r="C53" s="33">
+        <v>25101</v>
       </c>
       <c r="D53" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="50" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="7">
-        <v>23346</v>
+        <v>25450</v>
       </c>
       <c r="D54" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="50" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="B55" s="7"/>
       <c r="C55" s="7">
-        <v>23873</v>
+        <v>26350</v>
       </c>
       <c r="D55" s="3" t="str">
-        <f t="shared" ref="D55:D84" si="2">IF(C55&lt;&gt;"",IF(B55&lt;&gt;"",C55-B55,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="50" t="s">
-        <v>417</v>
-      </c>
-      <c r="B56" s="8"/>
-      <c r="C56" s="50">
-        <v>24221</v>
+        <v>421</v>
+      </c>
+      <c r="B56" s="7"/>
+      <c r="C56" s="7">
+        <v>26699</v>
       </c>
       <c r="D56" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="50" t="s">
-        <v>418</v>
-      </c>
-      <c r="B57" s="33"/>
-      <c r="C57" s="33">
-        <v>25101</v>
+        <v>332</v>
+      </c>
+      <c r="B57" s="7"/>
+      <c r="C57" s="7">
+        <v>27490</v>
       </c>
       <c r="D57" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
-        <v>419</v>
+        <v>5</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7">
-        <v>25450</v>
+        <v>27836</v>
       </c>
       <c r="D58" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>420</v>
+        <v>337</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7">
-        <v>26350</v>
+        <v>28899</v>
       </c>
       <c r="D59" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>421</v>
+        <v>6</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7">
-        <v>26699</v>
+        <v>29248</v>
       </c>
       <c r="D60" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>332</v>
+        <v>45</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7">
-        <v>27490</v>
+        <v>29962</v>
       </c>
       <c r="D61" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7">
-        <v>27836</v>
+        <v>30309</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>337</v>
+        <v>46</v>
       </c>
       <c r="B63" s="7"/>
       <c r="C63" s="7">
-        <v>28899</v>
+        <v>30479</v>
       </c>
       <c r="D63" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7">
-        <v>29248</v>
+        <v>31125</v>
       </c>
       <c r="D64" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E64" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="B65" s="7"/>
       <c r="C65" s="7">
-        <v>29962</v>
+        <v>31643</v>
       </c>
       <c r="D65" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3184,11 +3191,11 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B66" s="7"/>
       <c r="C66" s="7">
-        <v>30309</v>
+        <v>31991</v>
       </c>
       <c r="D66" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3197,11 +3204,11 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>30479</v>
+        <v>32586</v>
       </c>
       <c r="D67" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3210,11 +3217,11 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7">
-        <v>31125</v>
+        <v>33254</v>
       </c>
       <c r="D68" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3226,11 +3233,11 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7">
-        <v>31643</v>
+        <v>33883</v>
       </c>
       <c r="D69" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3239,11 +3246,11 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>31991</v>
+        <v>34244</v>
       </c>
       <c r="D70" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3252,11 +3259,11 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>32586</v>
+        <v>34862</v>
       </c>
       <c r="D71" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3265,27 +3272,24 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>33254</v>
+        <v>35218</v>
       </c>
       <c r="D72" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E72" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>33883</v>
+        <v>35772</v>
       </c>
       <c r="D73" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3294,11 +3298,11 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>34244</v>
+        <v>36120</v>
       </c>
       <c r="D74" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3307,11 +3311,11 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>34862</v>
+        <v>36893</v>
       </c>
       <c r="D75" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3320,11 +3324,11 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>35218</v>
+        <v>37238</v>
       </c>
       <c r="D76" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3333,11 +3337,11 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>35772</v>
+        <v>38097</v>
       </c>
       <c r="D77" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3346,11 +3350,11 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>36120</v>
+        <v>38443</v>
       </c>
       <c r="D78" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3359,11 +3363,11 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>36893</v>
+        <v>38692</v>
       </c>
       <c r="D79" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3372,370 +3376,334 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>37238</v>
+        <v>39041</v>
       </c>
       <c r="D80" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>38097</v>
+        <v>40011</v>
       </c>
       <c r="D81" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(C80&lt;&gt;"",IF(B80&lt;&gt;"",C80-B80,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>38443</v>
+        <v>40373</v>
       </c>
       <c r="D82" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>34</v>
-      </c>
-      <c r="B83" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B83" s="40"/>
       <c r="C83" s="7">
-        <v>38692</v>
+        <v>41117</v>
       </c>
       <c r="D83" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B84" s="7"/>
       <c r="C84" s="7">
-        <v>39041</v>
+        <v>41465</v>
       </c>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>40011</v>
+        <v>42450</v>
       </c>
       <c r="D85" s="3" t="str">
-        <f>IF(C84&lt;&gt;"",IF(B84&lt;&gt;"",C84-B84,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B86" s="7"/>
       <c r="C86" s="7">
-        <v>40373</v>
+        <v>42799</v>
       </c>
       <c r="D86" s="3" t="str">
-        <f t="shared" ref="D86:D105" si="3">IF(C86&lt;&gt;"",IF(B86&lt;&gt;"",C86-B86,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B87" s="40"/>
+        <v>38</v>
+      </c>
+      <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>41117</v>
+        <v>43144</v>
       </c>
       <c r="D87" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>41465</v>
+        <v>43491</v>
       </c>
       <c r="D88" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>42450</v>
+        <v>44165</v>
       </c>
       <c r="D89" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>42799</v>
+        <v>44512</v>
       </c>
       <c r="D90" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>43144</v>
+        <v>45061</v>
       </c>
       <c r="D91" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>43491</v>
+        <v>45443</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>44165</v>
+        <v>45990</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>44512</v>
+        <v>46652</v>
       </c>
       <c r="D94" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E94" s="51" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>45061</v>
+        <v>47436</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>21</v>
-      </c>
-      <c r="B96" s="7"/>
-      <c r="C96" s="7">
-        <v>45443</v>
+        <v>23</v>
+      </c>
+      <c r="B96" s="9"/>
+      <c r="C96" s="9">
+        <v>48337</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>45990</v>
+        <v>49334</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>46652</v>
+        <v>48681</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E98" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>47436</v>
+        <v>49334</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B100" s="9"/>
-      <c r="C100" s="9">
-        <v>48337</v>
+        <v>25</v>
+      </c>
+      <c r="B100" s="7"/>
+      <c r="C100" s="7">
+        <v>49683</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>49334</v>
+        <v>50244</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="50" t="s">
-        <v>24</v>
-      </c>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B102" s="7"/>
-      <c r="C102" s="7">
-        <v>48681</v>
-      </c>
-      <c r="D102" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="50" t="s">
-        <v>44</v>
-      </c>
+      <c r="C102" s="7"/>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B103" s="7"/>
-      <c r="C103" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D103" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A104" s="50" t="s">
-        <v>25</v>
-      </c>
+      <c r="C103" s="7"/>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B104" s="7"/>
-      <c r="C104" s="7">
-        <v>49683</v>
-      </c>
-      <c r="D104" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="50" t="s">
-        <v>26</v>
-      </c>
+      <c r="C104" s="7"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B105" s="7"/>
-      <c r="C105" s="7">
-        <v>50244</v>
-      </c>
-      <c r="D105" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C105" s="7"/>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B106" s="7"/>
       <c r="C106" s="7"/>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B107" s="7"/>
       <c r="C107" s="7"/>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B108" s="7"/>
       <c r="C108" s="7"/>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
     </row>
@@ -4026,22 +3994,6 @@
     <row r="184" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
-    </row>
-    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B185" s="7"/>
-      <c r="C185" s="7"/>
-    </row>
-    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B186" s="7"/>
-      <c r="C186" s="7"/>
-    </row>
-    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B187" s="7"/>
-      <c r="C187" s="7"/>
-    </row>
-    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B188" s="7"/>
-      <c r="C188" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - level 25 done - 431 frames ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1826C14F-7E64-4E35-9B5A-125625CFCD3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1A402BA-39C2-40E5-9386-76C14760A993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50250" yWindow="3210" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2995,26 +2995,30 @@
       <c r="A51" s="50" t="s">
         <v>416</v>
       </c>
-      <c r="B51" s="7"/>
+      <c r="B51" s="7">
+        <v>23443</v>
+      </c>
       <c r="C51" s="7">
         <v>23873</v>
       </c>
-      <c r="D51" s="3" t="str">
+      <c r="D51" s="3">
         <f t="shared" ref="D51:D80" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
-        <v>-</v>
+        <v>430</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="50" t="s">
         <v>417</v>
       </c>
-      <c r="B52" s="8"/>
+      <c r="B52" s="8">
+        <v>23790</v>
+      </c>
       <c r="C52" s="50">
         <v>24221</v>
       </c>
-      <c r="D52" s="3" t="str">
+      <c r="D52" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>431</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 26 done, 433 frames ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1A402BA-39C2-40E5-9386-76C14760A993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEB30724-3BB0-404F-B387-07BBF05C95A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50250" yWindow="3210" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3025,26 +3025,30 @@
       <c r="A53" s="50" t="s">
         <v>418</v>
       </c>
-      <c r="B53" s="33"/>
+      <c r="B53" s="33">
+        <v>24666</v>
+      </c>
       <c r="C53" s="33">
         <v>25101</v>
       </c>
-      <c r="D53" s="3" t="str">
+      <c r="D53" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>435</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="50" t="s">
         <v>419</v>
       </c>
-      <c r="B54" s="7"/>
+      <c r="B54" s="7">
+        <v>25017</v>
+      </c>
       <c r="C54" s="7">
         <v>25450</v>
       </c>
-      <c r="D54" s="3" t="str">
+      <c r="D54" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>433</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - 2 more frames on select skip, 435 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEB30724-3BB0-404F-B387-07BBF05C95A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{515237B5-2403-42DD-AD31-9997819E4CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50250" yWindow="3210" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3041,14 +3041,14 @@
         <v>419</v>
       </c>
       <c r="B54" s="7">
-        <v>25017</v>
+        <v>25015</v>
       </c>
       <c r="C54" s="7">
         <v>25450</v>
       </c>
       <c r="D54" s="3">
         <f t="shared" si="2"/>
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - more attempts  on level 27, including a route that is too slow but has potential to be much faster
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{515237B5-2403-42DD-AD31-9997819E4CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF67E57D-585D-4CDA-A16F-69C2B6C9EF9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50250" yWindow="3210" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2232,7 +2232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E184"/>
+  <dimension ref="A1:E185"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -3002,7 +3002,7 @@
         <v>23873</v>
       </c>
       <c r="D51" s="3">
-        <f t="shared" ref="D51:D80" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
+        <f t="shared" ref="D51:D81" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
         <v>430</v>
       </c>
     </row>
@@ -3052,38 +3052,43 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="50" t="s">
-        <v>420</v>
-      </c>
-      <c r="B55" s="7"/>
+      <c r="A55" s="50"/>
+      <c r="B55" s="7">
+        <v>25406</v>
+      </c>
       <c r="C55" s="7">
-        <v>26350</v>
-      </c>
-      <c r="D55" s="3" t="str">
+        <v>25893</v>
+      </c>
+      <c r="D55" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>487</v>
+      </c>
+      <c r="E55" s="51">
+        <v>25459</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="50" t="s">
-        <v>421</v>
-      </c>
-      <c r="B56" s="7"/>
+        <v>420</v>
+      </c>
+      <c r="B56" s="7">
+        <v>26034</v>
+      </c>
       <c r="C56" s="7">
-        <v>26699</v>
-      </c>
-      <c r="D56" s="3" t="str">
+        <v>26350</v>
+      </c>
+      <c r="D56" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>316</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="50" t="s">
-        <v>332</v>
+        <v>421</v>
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="7">
-        <v>27490</v>
+        <v>26699</v>
       </c>
       <c r="D57" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3092,11 +3097,11 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
-        <v>5</v>
+        <v>332</v>
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="7">
-        <v>27836</v>
+        <v>27490</v>
       </c>
       <c r="D58" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3105,11 +3110,11 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>337</v>
+        <v>5</v>
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="7">
-        <v>28899</v>
+        <v>27836</v>
       </c>
       <c r="D59" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3118,11 +3123,11 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>6</v>
+        <v>337</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7">
-        <v>29248</v>
+        <v>28899</v>
       </c>
       <c r="D60" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3131,11 +3136,11 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7">
-        <v>29962</v>
+        <v>29248</v>
       </c>
       <c r="D61" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3144,11 +3149,11 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7">
-        <v>30309</v>
+        <v>29962</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3157,11 +3162,11 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="B63" s="7"/>
       <c r="C63" s="7">
-        <v>30479</v>
+        <v>30309</v>
       </c>
       <c r="D63" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3170,40 +3175,40 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7">
-        <v>31125</v>
+        <v>30479</v>
       </c>
       <c r="D64" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E64" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B65" s="7"/>
       <c r="C65" s="7">
-        <v>31643</v>
+        <v>31125</v>
       </c>
       <c r="D65" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E65" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="B66" s="7"/>
       <c r="C66" s="7">
-        <v>31991</v>
+        <v>31643</v>
       </c>
       <c r="D66" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3212,11 +3217,11 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>32586</v>
+        <v>31991</v>
       </c>
       <c r="D67" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3225,40 +3230,40 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7">
-        <v>33254</v>
+        <v>32586</v>
       </c>
       <c r="D68" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E68" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7">
-        <v>33883</v>
+        <v>33254</v>
       </c>
       <c r="D69" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E69" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>34244</v>
+        <v>33883</v>
       </c>
       <c r="D70" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3267,11 +3272,11 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>34862</v>
+        <v>34244</v>
       </c>
       <c r="D71" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3280,11 +3285,11 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>35218</v>
+        <v>34862</v>
       </c>
       <c r="D72" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3293,11 +3298,11 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>35772</v>
+        <v>35218</v>
       </c>
       <c r="D73" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3306,11 +3311,11 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>36120</v>
+        <v>35772</v>
       </c>
       <c r="D74" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3319,11 +3324,11 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>36893</v>
+        <v>36120</v>
       </c>
       <c r="D75" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3332,11 +3337,11 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>37238</v>
+        <v>36893</v>
       </c>
       <c r="D76" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3345,11 +3350,11 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>38097</v>
+        <v>37238</v>
       </c>
       <c r="D77" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3358,11 +3363,11 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>38443</v>
+        <v>38097</v>
       </c>
       <c r="D78" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3371,11 +3376,11 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>38692</v>
+        <v>38443</v>
       </c>
       <c r="D79" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3384,11 +3389,11 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>39041</v>
+        <v>38692</v>
       </c>
       <c r="D80" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3397,50 +3402,50 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>40011</v>
+        <v>39041</v>
       </c>
       <c r="D81" s="3" t="str">
-        <f>IF(C80&lt;&gt;"",IF(B80&lt;&gt;"",C80-B80,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>40373</v>
+        <v>40011</v>
       </c>
       <c r="D82" s="3" t="str">
-        <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
+        <f>IF(C81&lt;&gt;"",IF(B81&lt;&gt;"",C81-B81,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B83" s="40"/>
+        <v>16</v>
+      </c>
+      <c r="B83" s="7"/>
       <c r="C83" s="7">
-        <v>41117</v>
+        <v>40373</v>
       </c>
       <c r="D83" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="D83:D102" si="3">IF(C83&lt;&gt;"",IF(B83&lt;&gt;"",C83-B83,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="B84" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B84" s="40"/>
       <c r="C84" s="7">
-        <v>41465</v>
+        <v>41117</v>
       </c>
       <c r="D84" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3449,11 +3454,11 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>42450</v>
+        <v>41465</v>
       </c>
       <c r="D85" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3462,11 +3467,11 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="B86" s="7"/>
       <c r="C86" s="7">
-        <v>42799</v>
+        <v>42450</v>
       </c>
       <c r="D86" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3475,11 +3480,11 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>43144</v>
+        <v>42799</v>
       </c>
       <c r="D87" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3488,11 +3493,11 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>43491</v>
+        <v>43144</v>
       </c>
       <c r="D88" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3501,11 +3506,11 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>44165</v>
+        <v>43491</v>
       </c>
       <c r="D89" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3514,11 +3519,11 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>44512</v>
+        <v>44165</v>
       </c>
       <c r="D90" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3527,11 +3532,11 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>45061</v>
+        <v>44512</v>
       </c>
       <c r="D91" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3540,11 +3545,11 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>45443</v>
+        <v>45061</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3553,11 +3558,11 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>45990</v>
+        <v>45443</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3566,40 +3571,40 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>46652</v>
+        <v>45990</v>
       </c>
       <c r="D94" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E94" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>47436</v>
+        <v>46652</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
+      <c r="E95" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B96" s="9"/>
-      <c r="C96" s="9">
-        <v>48337</v>
+        <v>42</v>
+      </c>
+      <c r="B96" s="7"/>
+      <c r="C96" s="7">
+        <v>47436</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3608,11 +3613,11 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>43</v>
-      </c>
-      <c r="B97" s="7"/>
-      <c r="C97" s="7">
-        <v>49334</v>
+        <v>23</v>
+      </c>
+      <c r="B97" s="9"/>
+      <c r="C97" s="9">
+        <v>48337</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3621,11 +3626,11 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>48681</v>
+        <v>49334</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3634,11 +3639,11 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>49334</v>
+        <v>48681</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3647,11 +3652,11 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>49683</v>
+        <v>49334</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3660,11 +3665,11 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>50244</v>
+        <v>49683</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3672,8 +3677,17 @@
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="50" t="s">
+        <v>26</v>
+      </c>
       <c r="B102" s="7"/>
-      <c r="C102" s="7"/>
+      <c r="C102" s="7">
+        <v>50244</v>
+      </c>
+      <c r="D102" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B103" s="7"/>
@@ -4002,6 +4016,10 @@
     <row r="184" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
+    </row>
+    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B185" s="7"/>
+      <c r="C185" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - lv 27 done - new route, 470 ahead before select skip manip
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF67E57D-585D-4CDA-A16F-69C2B6C9EF9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34C87085-3F04-4288-AB46-A955C87AA322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50250" yWindow="3210" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="425">
   <si>
     <t>Place</t>
   </si>
@@ -1305,6 +1305,12 @@
   </si>
   <si>
     <t>(v6 1st move)</t>
+  </si>
+  <si>
+    <t>mid</t>
+  </si>
+  <si>
+    <t>grab ladder</t>
   </si>
 </sst>
 </file>
@@ -1314,12 +1320,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="37" x14ac:knownFonts="1">
+  <fonts count="38" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1779,95 +1792,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1887,31 +1901,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2232,7 +2246,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E185"/>
+  <dimension ref="A1:E188"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -3002,7 +3016,7 @@
         <v>23873</v>
       </c>
       <c r="D51" s="3">
-        <f t="shared" ref="D51:D81" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
+        <f t="shared" ref="D51:D84" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
         <v>430</v>
       </c>
     </row>
@@ -3052,82 +3066,72 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="50"/>
+      <c r="A55" s="61" t="s">
+        <v>423</v>
+      </c>
       <c r="B55" s="7">
-        <v>25406</v>
+        <v>25390</v>
       </c>
       <c r="C55" s="7">
         <v>25893</v>
       </c>
       <c r="D55" s="3">
         <f t="shared" si="2"/>
-        <v>487</v>
+        <v>503</v>
       </c>
       <c r="E55" s="51">
         <v>25459</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="50" t="s">
-        <v>420</v>
+      <c r="A56" s="61" t="s">
+        <v>424</v>
       </c>
       <c r="B56" s="7">
-        <v>26034</v>
+        <v>25570</v>
       </c>
       <c r="C56" s="7">
-        <v>26350</v>
+        <v>26055</v>
       </c>
       <c r="D56" s="3">
         <f t="shared" si="2"/>
-        <v>316</v>
+        <v>485</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="50" t="s">
-        <v>421</v>
-      </c>
+      <c r="A57" s="61"/>
       <c r="B57" s="7"/>
-      <c r="C57" s="7">
-        <v>26699</v>
-      </c>
-      <c r="D57" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
+      <c r="C57" s="7"/>
+      <c r="D57" s="3"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="50" t="s">
-        <v>332</v>
-      </c>
+      <c r="A58" s="50"/>
       <c r="B58" s="7"/>
-      <c r="C58" s="7">
-        <v>27490</v>
-      </c>
-      <c r="D58" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
+      <c r="C58" s="7"/>
+      <c r="D58" s="3"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>5</v>
-      </c>
-      <c r="B59" s="7"/>
+        <v>420</v>
+      </c>
+      <c r="B59" s="7">
+        <v>25880</v>
+      </c>
       <c r="C59" s="7">
-        <v>27836</v>
-      </c>
-      <c r="D59" s="3" t="str">
+        <v>26350</v>
+      </c>
+      <c r="D59" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>470</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>337</v>
+        <v>421</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7">
-        <v>28899</v>
+        <v>26699</v>
       </c>
       <c r="D60" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3136,11 +3140,11 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>6</v>
+        <v>332</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7">
-        <v>29248</v>
+        <v>27490</v>
       </c>
       <c r="D61" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3149,11 +3153,11 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7">
-        <v>29962</v>
+        <v>27836</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3162,11 +3166,11 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>7</v>
+        <v>337</v>
       </c>
       <c r="B63" s="7"/>
       <c r="C63" s="7">
-        <v>30309</v>
+        <v>28899</v>
       </c>
       <c r="D63" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3175,11 +3179,11 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>46</v>
+        <v>6</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7">
-        <v>30479</v>
+        <v>29248</v>
       </c>
       <c r="D64" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3188,27 +3192,24 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="B65" s="7"/>
       <c r="C65" s="7">
-        <v>31125</v>
+        <v>29962</v>
       </c>
       <c r="D65" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E65" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="B66" s="7"/>
       <c r="C66" s="7">
-        <v>31643</v>
+        <v>30309</v>
       </c>
       <c r="D66" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3217,11 +3218,11 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>31991</v>
+        <v>30479</v>
       </c>
       <c r="D67" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3230,40 +3231,40 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7">
-        <v>32586</v>
+        <v>31125</v>
       </c>
       <c r="D68" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E68" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7">
-        <v>33254</v>
+        <v>31643</v>
       </c>
       <c r="D69" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E69" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>33883</v>
+        <v>31991</v>
       </c>
       <c r="D70" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3272,11 +3273,11 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>34244</v>
+        <v>32586</v>
       </c>
       <c r="D71" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3285,24 +3286,27 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>34862</v>
+        <v>33254</v>
       </c>
       <c r="D72" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E72" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>35218</v>
+        <v>33883</v>
       </c>
       <c r="D73" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3311,11 +3315,11 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>35772</v>
+        <v>34244</v>
       </c>
       <c r="D74" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3324,11 +3328,11 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>36120</v>
+        <v>34862</v>
       </c>
       <c r="D75" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3337,11 +3341,11 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>36893</v>
+        <v>35218</v>
       </c>
       <c r="D76" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3350,11 +3354,11 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>37238</v>
+        <v>35772</v>
       </c>
       <c r="D77" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3363,11 +3367,11 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>38097</v>
+        <v>36120</v>
       </c>
       <c r="D78" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3376,11 +3380,11 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>38443</v>
+        <v>36893</v>
       </c>
       <c r="D79" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3389,343 +3393,370 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>38692</v>
+        <v>37238</v>
       </c>
       <c r="D80" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>39041</v>
+        <v>38097</v>
       </c>
       <c r="D81" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>40011</v>
+        <v>38443</v>
       </c>
       <c r="D82" s="3" t="str">
-        <f>IF(C81&lt;&gt;"",IF(B81&lt;&gt;"",C81-B81,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="B83" s="7"/>
       <c r="C83" s="7">
-        <v>40373</v>
+        <v>38692</v>
       </c>
       <c r="D83" s="3" t="str">
-        <f t="shared" ref="D83:D102" si="3">IF(C83&lt;&gt;"",IF(B83&lt;&gt;"",C83-B83,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B84" s="40"/>
+        <v>15</v>
+      </c>
+      <c r="B84" s="7"/>
       <c r="C84" s="7">
-        <v>41117</v>
+        <v>39041</v>
       </c>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>41465</v>
+        <v>40011</v>
       </c>
       <c r="D85" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(C84&lt;&gt;"",IF(B84&lt;&gt;"",C84-B84,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="B86" s="7"/>
       <c r="C86" s="7">
-        <v>42450</v>
+        <v>40373</v>
       </c>
       <c r="D86" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="D86:D105" si="3">IF(C86&lt;&gt;"",IF(B86&lt;&gt;"",C86-B86,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>18</v>
-      </c>
-      <c r="B87" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B87" s="40"/>
       <c r="C87" s="7">
-        <v>42799</v>
+        <v>41117</v>
       </c>
       <c r="D87" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>43144</v>
+        <v>41465</v>
       </c>
       <c r="D88" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>43491</v>
+        <v>42450</v>
       </c>
       <c r="D89" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>44165</v>
+        <v>42799</v>
       </c>
       <c r="D90" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>44512</v>
+        <v>43144</v>
       </c>
       <c r="D91" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>45061</v>
+        <v>43491</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>45443</v>
+        <v>44165</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>45990</v>
+        <v>44512</v>
       </c>
       <c r="D94" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>46652</v>
+        <v>45061</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E95" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="B96" s="7"/>
       <c r="C96" s="7">
-        <v>47436</v>
+        <v>45443</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B97" s="9"/>
-      <c r="C97" s="9">
-        <v>48337</v>
+        <v>41</v>
+      </c>
+      <c r="B97" s="7"/>
+      <c r="C97" s="7">
+        <v>45990</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>49334</v>
+        <v>46652</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E98" s="51" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>48681</v>
+        <v>47436</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>44</v>
-      </c>
-      <c r="B100" s="7"/>
-      <c r="C100" s="7">
-        <v>49334</v>
+        <v>23</v>
+      </c>
+      <c r="B100" s="9"/>
+      <c r="C100" s="9">
+        <v>48337</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>49683</v>
+        <v>49334</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="50" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B102" s="7"/>
       <c r="C102" s="7">
-        <v>50244</v>
+        <v>48681</v>
       </c>
       <c r="D102" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="50" t="s">
+        <v>44</v>
+      </c>
       <c r="B103" s="7"/>
-      <c r="C103" s="7"/>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C103" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D103" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="50" t="s">
+        <v>25</v>
+      </c>
       <c r="B104" s="7"/>
-      <c r="C104" s="7"/>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C104" s="7">
+        <v>49683</v>
+      </c>
+      <c r="D104" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="50" t="s">
+        <v>26</v>
+      </c>
       <c r="B105" s="7"/>
-      <c r="C105" s="7"/>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C105" s="7">
+        <v>50244</v>
+      </c>
+      <c r="D105" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B106" s="7"/>
       <c r="C106" s="7"/>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B107" s="7"/>
       <c r="C107" s="7"/>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B108" s="7"/>
       <c r="C108" s="7"/>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
     </row>
@@ -4020,6 +4051,18 @@
     <row r="185" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B185" s="7"/>
       <c r="C185" s="7"/>
+    </row>
+    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B186" s="7"/>
+      <c r="C186" s="7"/>
+    </row>
+    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B187" s="7"/>
+      <c r="C187" s="7"/>
+    </row>
+    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B188" s="7"/>
+      <c r="C188" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18868,7 +18911,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="33" type="noConversion"/>
+  <phoneticPr fontId="34" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>

</xml_diff>

<commit_message>
lode runner - select skip done, 468 ahead at the start of level 28
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34C87085-3F04-4288-AB46-A955C87AA322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABE93143-AE31-402B-8FC5-B6F37D034D4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50250" yWindow="3210" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="423">
   <si>
     <t>Place</t>
   </si>
@@ -1305,12 +1305,6 @@
   </si>
   <si>
     <t>(v6 1st move)</t>
-  </si>
-  <si>
-    <t>mid</t>
-  </si>
-  <si>
-    <t>grab ladder</t>
   </si>
 </sst>
 </file>
@@ -1320,19 +1314,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="38" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1792,96 +1779,95 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="30" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="5"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1901,31 +1887,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2246,7 +2232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E188"/>
+  <dimension ref="A1:E184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -3016,7 +3002,7 @@
         <v>23873</v>
       </c>
       <c r="D51" s="3">
-        <f t="shared" ref="D51:D84" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
+        <f t="shared" ref="D51:D80" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
         <v>430</v>
       </c>
     </row>
@@ -3066,72 +3052,81 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="61" t="s">
-        <v>423</v>
+      <c r="A55" s="50" t="s">
+        <v>420</v>
       </c>
       <c r="B55" s="7">
-        <v>25390</v>
+        <v>25880</v>
       </c>
       <c r="C55" s="7">
-        <v>25893</v>
+        <v>26350</v>
       </c>
       <c r="D55" s="3">
         <f t="shared" si="2"/>
-        <v>503</v>
-      </c>
-      <c r="E55" s="51">
-        <v>25459</v>
+        <v>470</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="61" t="s">
-        <v>424</v>
+      <c r="A56" s="50" t="s">
+        <v>421</v>
       </c>
       <c r="B56" s="7">
-        <v>25570</v>
+        <v>26231</v>
       </c>
       <c r="C56" s="7">
-        <v>26055</v>
+        <v>26699</v>
       </c>
       <c r="D56" s="3">
         <f t="shared" si="2"/>
-        <v>485</v>
+        <v>468</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="61"/>
+      <c r="A57" s="50" t="s">
+        <v>332</v>
+      </c>
       <c r="B57" s="7"/>
-      <c r="C57" s="7"/>
-      <c r="D57" s="3"/>
+      <c r="C57" s="7">
+        <v>27490</v>
+      </c>
+      <c r="D57" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="50"/>
+      <c r="A58" s="50" t="s">
+        <v>5</v>
+      </c>
       <c r="B58" s="7"/>
-      <c r="C58" s="7"/>
-      <c r="D58" s="3"/>
+      <c r="C58" s="7">
+        <v>27836</v>
+      </c>
+      <c r="D58" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
-        <v>420</v>
-      </c>
-      <c r="B59" s="7">
-        <v>25880</v>
-      </c>
+        <v>337</v>
+      </c>
+      <c r="B59" s="7"/>
       <c r="C59" s="7">
-        <v>26350</v>
-      </c>
-      <c r="D59" s="3">
+        <v>28899</v>
+      </c>
+      <c r="D59" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>470</v>
+        <v>-</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>421</v>
+        <v>6</v>
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="7">
-        <v>26699</v>
+        <v>29248</v>
       </c>
       <c r="D60" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3140,11 +3135,11 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
-        <v>332</v>
+        <v>45</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7">
-        <v>27490</v>
+        <v>29962</v>
       </c>
       <c r="D61" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3153,11 +3148,11 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7">
-        <v>27836</v>
+        <v>30309</v>
       </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3166,11 +3161,11 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
-        <v>337</v>
+        <v>46</v>
       </c>
       <c r="B63" s="7"/>
       <c r="C63" s="7">
-        <v>28899</v>
+        <v>30479</v>
       </c>
       <c r="D63" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3179,24 +3174,27 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7">
-        <v>29248</v>
+        <v>31125</v>
       </c>
       <c r="D64" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
+      <c r="E64" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="B65" s="7"/>
       <c r="C65" s="7">
-        <v>29962</v>
+        <v>31643</v>
       </c>
       <c r="D65" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3205,11 +3203,11 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B66" s="7"/>
       <c r="C66" s="7">
-        <v>30309</v>
+        <v>31991</v>
       </c>
       <c r="D66" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3218,11 +3216,11 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7">
-        <v>30479</v>
+        <v>32586</v>
       </c>
       <c r="D67" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3231,11 +3229,11 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7">
-        <v>31125</v>
+        <v>33254</v>
       </c>
       <c r="D68" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3247,11 +3245,11 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7">
-        <v>31643</v>
+        <v>33883</v>
       </c>
       <c r="D69" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3260,11 +3258,11 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7">
-        <v>31991</v>
+        <v>34244</v>
       </c>
       <c r="D70" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3273,11 +3271,11 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7">
-        <v>32586</v>
+        <v>34862</v>
       </c>
       <c r="D71" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3286,27 +3284,24 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7">
-        <v>33254</v>
+        <v>35218</v>
       </c>
       <c r="D72" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E72" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7">
-        <v>33883</v>
+        <v>35772</v>
       </c>
       <c r="D73" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3315,11 +3310,11 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7">
-        <v>34244</v>
+        <v>36120</v>
       </c>
       <c r="D74" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3328,11 +3323,11 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7">
-        <v>34862</v>
+        <v>36893</v>
       </c>
       <c r="D75" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3341,11 +3336,11 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7">
-        <v>35218</v>
+        <v>37238</v>
       </c>
       <c r="D76" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3354,11 +3349,11 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7">
-        <v>35772</v>
+        <v>38097</v>
       </c>
       <c r="D77" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3367,11 +3362,11 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7">
-        <v>36120</v>
+        <v>38443</v>
       </c>
       <c r="D78" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3380,11 +3375,11 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7">
-        <v>36893</v>
+        <v>38692</v>
       </c>
       <c r="D79" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3393,370 +3388,334 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7">
-        <v>37238</v>
+        <v>39041</v>
       </c>
       <c r="D80" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="50" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7">
-        <v>38097</v>
+        <v>40011</v>
       </c>
       <c r="D81" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(C80&lt;&gt;"",IF(B80&lt;&gt;"",C80-B80,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="50" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7">
-        <v>38443</v>
+        <v>40373</v>
       </c>
       <c r="D82" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
-        <v>34</v>
-      </c>
-      <c r="B83" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B83" s="40"/>
       <c r="C83" s="7">
-        <v>38692</v>
+        <v>41117</v>
       </c>
       <c r="D83" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B84" s="7"/>
       <c r="C84" s="7">
-        <v>39041</v>
+        <v>41465</v>
       </c>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="50" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7">
-        <v>40011</v>
+        <v>42450</v>
       </c>
       <c r="D85" s="3" t="str">
-        <f>IF(C84&lt;&gt;"",IF(B84&lt;&gt;"",C84-B84,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B86" s="7"/>
       <c r="C86" s="7">
-        <v>40373</v>
+        <v>42799</v>
       </c>
       <c r="D86" s="3" t="str">
-        <f t="shared" ref="D86:D105" si="3">IF(C86&lt;&gt;"",IF(B86&lt;&gt;"",C86-B86,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B87" s="40"/>
+        <v>38</v>
+      </c>
+      <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>41117</v>
+        <v>43144</v>
       </c>
       <c r="D87" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>41465</v>
+        <v>43491</v>
       </c>
       <c r="D88" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>42450</v>
+        <v>44165</v>
       </c>
       <c r="D89" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>42799</v>
+        <v>44512</v>
       </c>
       <c r="D90" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>43144</v>
+        <v>45061</v>
       </c>
       <c r="D91" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>43491</v>
+        <v>45443</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>44165</v>
+        <v>45990</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>44512</v>
+        <v>46652</v>
       </c>
       <c r="D94" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E94" s="51" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>45061</v>
+        <v>47436</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>21</v>
-      </c>
-      <c r="B96" s="7"/>
-      <c r="C96" s="7">
-        <v>45443</v>
+        <v>23</v>
+      </c>
+      <c r="B96" s="9"/>
+      <c r="C96" s="9">
+        <v>48337</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>45990</v>
+        <v>49334</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>46652</v>
+        <v>48681</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E98" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>47436</v>
+        <v>49334</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B100" s="9"/>
-      <c r="C100" s="9">
-        <v>48337</v>
+        <v>25</v>
+      </c>
+      <c r="B100" s="7"/>
+      <c r="C100" s="7">
+        <v>49683</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>49334</v>
+        <v>50244</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="50" t="s">
-        <v>24</v>
-      </c>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B102" s="7"/>
-      <c r="C102" s="7">
-        <v>48681</v>
-      </c>
-      <c r="D102" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="50" t="s">
-        <v>44</v>
-      </c>
+      <c r="C102" s="7"/>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B103" s="7"/>
-      <c r="C103" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D103" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A104" s="50" t="s">
-        <v>25</v>
-      </c>
+      <c r="C103" s="7"/>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B104" s="7"/>
-      <c r="C104" s="7">
-        <v>49683</v>
-      </c>
-      <c r="D104" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="50" t="s">
-        <v>26</v>
-      </c>
+      <c r="C104" s="7"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B105" s="7"/>
-      <c r="C105" s="7">
-        <v>50244</v>
-      </c>
-      <c r="D105" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C105" s="7"/>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B106" s="7"/>
       <c r="C106" s="7"/>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B107" s="7"/>
       <c r="C107" s="7"/>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B108" s="7"/>
       <c r="C108" s="7"/>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
     </row>
@@ -4047,22 +4006,6 @@
     <row r="184" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
-    </row>
-    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B185" s="7"/>
-      <c r="C185" s="7"/>
-    </row>
-    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B186" s="7"/>
-      <c r="C186" s="7"/>
-    </row>
-    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B187" s="7"/>
-      <c r="C187" s="7"/>
-    </row>
-    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B188" s="7"/>
-      <c r="C188" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18911,7 +18854,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="34" type="noConversion"/>
+  <phoneticPr fontId="33" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>

</xml_diff>

<commit_message>
level 28 done - 471 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABE93143-AE31-402B-8FC5-B6F37D034D4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91702FA9-A738-435E-933D-A8F49257E84B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50250" yWindow="3210" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3085,26 +3085,30 @@
       <c r="A57" s="50" t="s">
         <v>332</v>
       </c>
-      <c r="B57" s="7"/>
+      <c r="B57" s="7">
+        <v>27018</v>
+      </c>
       <c r="C57" s="7">
         <v>27490</v>
       </c>
-      <c r="D57" s="3" t="str">
+      <c r="D57" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>472</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B58" s="7"/>
+      <c r="B58" s="7">
+        <v>27365</v>
+      </c>
       <c r="C58" s="7">
         <v>27836</v>
       </c>
-      <c r="D58" s="3" t="str">
+      <c r="D58" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>471</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 29 done - 476 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91702FA9-A738-435E-933D-A8F49257E84B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{895CC37E-5485-40F1-827C-BDAC7981C28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50250" yWindow="3210" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="50205" yWindow="4140" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -3115,26 +3115,30 @@
       <c r="A59" s="50" t="s">
         <v>337</v>
       </c>
-      <c r="B59" s="7"/>
+      <c r="B59" s="7">
+        <v>28423</v>
+      </c>
       <c r="C59" s="7">
         <v>28899</v>
       </c>
-      <c r="D59" s="3" t="str">
+      <c r="D59" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>476</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="B60" s="7"/>
+      <c r="B60" s="7">
+        <v>28772</v>
+      </c>
       <c r="C60" s="7">
         <v>29248</v>
       </c>
-      <c r="D60" s="3" t="str">
+      <c r="D60" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>476</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - level 30 done - 483 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{895CC37E-5485-40F1-827C-BDAC7981C28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45832DE4-15B3-4FE8-8874-D8BEE129FDFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50205" yWindow="4140" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3145,26 +3145,30 @@
       <c r="A61" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="B61" s="7"/>
+      <c r="B61" s="7">
+        <v>29478</v>
+      </c>
       <c r="C61" s="7">
         <v>29962</v>
       </c>
-      <c r="D61" s="3" t="str">
+      <c r="D61" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>484</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="B62" s="7"/>
+      <c r="B62" s="7">
+        <v>29826</v>
+      </c>
       <c r="C62" s="7">
         <v>30309</v>
       </c>
-      <c r="D62" s="3" t="str">
+      <c r="D62" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>483</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lv 31 done - still 483 ahead, 32 skip not manipulated yet
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45832DE4-15B3-4FE8-8874-D8BEE129FDFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E4A3A41-2FA6-4306-AAC1-EC1D845A11C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50205" yWindow="4140" windowWidth="7410" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -3175,13 +3175,15 @@
       <c r="A63" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="B63" s="7"/>
+      <c r="B63" s="7">
+        <v>29996</v>
+      </c>
       <c r="C63" s="7">
         <v>30479</v>
       </c>
-      <c r="D63" s="3" t="str">
+      <c r="D63" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>483</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lv 32 done with slower mode to get scroll skip, 558 frames ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E4A3A41-2FA6-4306-AAC1-EC1D845A11C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7EB5600-2A0A-4642-943B-A90AE20DE15C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="424">
   <si>
     <t>Place</t>
   </si>
@@ -1305,6 +1305,9 @@
   </si>
   <si>
     <t>(v6 1st move)</t>
+  </si>
+  <si>
+    <t>fast mode</t>
   </si>
 </sst>
 </file>
@@ -2232,7 +2235,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:E184"/>
+  <dimension ref="A1:F184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -2961,7 +2964,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="50" t="s">
         <v>324</v>
       </c>
@@ -2976,7 +2979,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="50" t="s">
         <v>415</v>
       </c>
@@ -2991,7 +2994,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="50" t="s">
         <v>416</v>
       </c>
@@ -3006,7 +3009,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="50" t="s">
         <v>417</v>
       </c>
@@ -3021,7 +3024,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="50" t="s">
         <v>418</v>
       </c>
@@ -3036,7 +3039,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="50" t="s">
         <v>419</v>
       </c>
@@ -3051,7 +3054,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="50" t="s">
         <v>420</v>
       </c>
@@ -3066,7 +3069,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="50" t="s">
         <v>421</v>
       </c>
@@ -3081,7 +3084,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="50" t="s">
         <v>332</v>
       </c>
@@ -3096,7 +3099,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="50" t="s">
         <v>5</v>
       </c>
@@ -3111,7 +3114,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="50" t="s">
         <v>337</v>
       </c>
@@ -3126,7 +3129,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
         <v>6</v>
       </c>
@@ -3141,7 +3144,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="50" t="s">
         <v>45</v>
       </c>
@@ -3156,7 +3159,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="50" t="s">
         <v>7</v>
       </c>
@@ -3171,7 +3174,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="50" t="s">
         <v>46</v>
       </c>
@@ -3185,50 +3188,65 @@
         <f t="shared" si="2"/>
         <v>483</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F63" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="B64" s="7"/>
+      <c r="B64" s="7">
+        <v>30361</v>
+      </c>
       <c r="C64" s="7">
         <v>31125</v>
       </c>
-      <c r="D64" s="3" t="str">
+      <c r="D64" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>764</v>
       </c>
       <c r="E64" s="51" t="s">
         <v>422</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F64" s="7">
+        <v>30642</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="B65" s="7"/>
+      <c r="B65" s="7">
+        <v>31078</v>
+      </c>
       <c r="C65" s="7">
         <v>31643</v>
       </c>
-      <c r="D65" s="3" t="str">
+      <c r="D65" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+        <v>565</v>
+      </c>
+      <c r="F65" s="7">
+        <v>31158</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="B66" s="7"/>
+      <c r="B66" s="7">
+        <v>31433</v>
+      </c>
       <c r="C66" s="7">
         <v>31991</v>
       </c>
-      <c r="D66" s="3" t="str">
+      <c r="D66" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="50" t="s">
         <v>29</v>
       </c>
@@ -3241,7 +3259,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
         <v>10</v>
       </c>
@@ -3257,7 +3275,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="50" t="s">
         <v>31</v>
       </c>
@@ -3270,7 +3288,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
         <v>11</v>
       </c>
@@ -3283,7 +3301,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
         <v>30</v>
       </c>
@@ -3296,7 +3314,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
         <v>12</v>
       </c>
@@ -3309,7 +3327,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="50" t="s">
         <v>32</v>
       </c>
@@ -3322,7 +3340,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
         <v>13</v>
       </c>
@@ -3335,7 +3353,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="50" t="s">
         <v>47</v>
       </c>
@@ -3348,7 +3366,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
         <v>48</v>
       </c>
@@ -3361,7 +3379,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="50" t="s">
         <v>33</v>
       </c>
@@ -3374,7 +3392,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
         <v>14</v>
       </c>
@@ -3387,7 +3405,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="50" t="s">
         <v>34</v>
       </c>
@@ -3400,7 +3418,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="50" t="s">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
lv 33 done (select skip not manipulated yet) - 560 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7EB5600-2A0A-4642-943B-A90AE20DE15C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{915BD990-815F-4210-A0DC-327D1FA48A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3250,13 +3250,15 @@
       <c r="A67" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="B67" s="7"/>
+      <c r="B67" s="7">
+        <v>32026</v>
+      </c>
       <c r="C67" s="7">
         <v>32586</v>
       </c>
-      <c r="D67" s="3" t="str">
+      <c r="D67" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>560</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 34 done at full speed, no select skip, 2 frames saved
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{915BD990-815F-4210-A0DC-327D1FA48A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A756C4CD-93EF-4861-8526-D2CC7B26A4D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3265,13 +3265,15 @@
       <c r="A68" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="B68" s="7"/>
+      <c r="B68" s="7">
+        <v>32694</v>
+      </c>
       <c r="C68" s="7">
         <v>33254</v>
       </c>
-      <c r="D68" s="3" t="str">
+      <c r="D68" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>560</v>
       </c>
       <c r="E68" s="51" t="s">
         <v>422</v>
@@ -3281,13 +3283,15 @@
       <c r="A69" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="B69" s="7"/>
+      <c r="B69" s="7">
+        <v>33321</v>
+      </c>
       <c r="C69" s="7">
         <v>33883</v>
       </c>
-      <c r="D69" s="3" t="str">
+      <c r="D69" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>562</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 34 done using slower mode, 681 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A756C4CD-93EF-4861-8526-D2CC7B26A4D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{884D5E83-F124-45D7-9717-E18DED229D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="424">
   <si>
     <t>Place</t>
   </si>
@@ -3260,23 +3260,29 @@
         <f t="shared" si="2"/>
         <v>560</v>
       </c>
+      <c r="F67" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="50" t="s">
         <v>10</v>
       </c>
       <c r="B68" s="7">
-        <v>32694</v>
+        <v>32379</v>
       </c>
       <c r="C68" s="7">
         <v>33254</v>
       </c>
       <c r="D68" s="3">
         <f t="shared" si="2"/>
-        <v>560</v>
+        <v>875</v>
       </c>
       <c r="E68" s="51" t="s">
         <v>422</v>
+      </c>
+      <c r="F68" s="7">
+        <v>32694</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -3284,27 +3290,32 @@
         <v>31</v>
       </c>
       <c r="B69" s="7">
-        <v>33321</v>
+        <v>33211</v>
       </c>
       <c r="C69" s="7">
         <v>33883</v>
       </c>
       <c r="D69" s="3">
         <f t="shared" si="2"/>
-        <v>562</v>
+        <v>672</v>
+      </c>
+      <c r="F69" s="7">
+        <v>33321</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="B70" s="7"/>
+      <c r="B70" s="7">
+        <v>33563</v>
+      </c>
       <c r="C70" s="7">
         <v>34244</v>
       </c>
-      <c r="D70" s="3" t="str">
+      <c r="D70" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>681</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 35 done, 672 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{884D5E83-F124-45D7-9717-E18DED229D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB8306F-2271-4DAA-82B7-7BA583F7ACD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3311,37 +3311,41 @@
         <v>33563</v>
       </c>
       <c r="C70" s="7">
-        <v>34244</v>
+        <v>34230</v>
       </c>
       <c r="D70" s="3">
         <f t="shared" si="2"/>
-        <v>681</v>
+        <v>667</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="B71" s="7"/>
+      <c r="B71" s="7">
+        <v>34198</v>
+      </c>
       <c r="C71" s="7">
         <v>34862</v>
       </c>
-      <c r="D71" s="3" t="str">
+      <c r="D71" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>664</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="B72" s="7"/>
+      <c r="B72" s="7">
+        <v>34546</v>
+      </c>
       <c r="C72" s="7">
         <v>35218</v>
       </c>
-      <c r="D72" s="3" t="str">
+      <c r="D72" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>672</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lv 36 done - 679 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB8306F-2271-4DAA-82B7-7BA583F7ACD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F2CC7F-F094-4E22-B473-1819DB135D67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3352,26 +3352,30 @@
       <c r="A73" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="B73" s="7"/>
+      <c r="B73" s="7">
+        <v>35096</v>
+      </c>
       <c r="C73" s="7">
         <v>35772</v>
       </c>
-      <c r="D73" s="3" t="str">
+      <c r="D73" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>676</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="B74" s="7"/>
+      <c r="B74" s="7">
+        <v>35441</v>
+      </c>
       <c r="C74" s="7">
         <v>36120</v>
       </c>
-      <c r="D74" s="3" t="str">
+      <c r="D74" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>679</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 38 done - 681 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F2CC7F-F094-4E22-B473-1819DB135D67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE617F92-6D02-45DF-9C1E-341351BF3E20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3382,26 +3382,30 @@
       <c r="A75" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="B75" s="7"/>
+      <c r="B75" s="7">
+        <v>36210</v>
+      </c>
       <c r="C75" s="7">
         <v>36893</v>
       </c>
-      <c r="D75" s="3" t="str">
+      <c r="D75" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>683</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="B76" s="7"/>
+      <c r="B76" s="7">
+        <v>36557</v>
+      </c>
       <c r="C76" s="7">
         <v>37238</v>
       </c>
-      <c r="D76" s="3" t="str">
+      <c r="D76" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>681</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 38 done - 703 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE617F92-6D02-45DF-9C1E-341351BF3E20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC4334D-5C5A-43EB-80EF-DA59405F377B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3412,26 +3412,30 @@
       <c r="A77" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="B77" s="7"/>
+      <c r="B77" s="7">
+        <v>37389</v>
+      </c>
       <c r="C77" s="7">
         <v>38097</v>
       </c>
-      <c r="D77" s="3" t="str">
+      <c r="D77" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>708</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="B78" s="7"/>
+      <c r="B78" s="7">
+        <v>37740</v>
+      </c>
       <c r="C78" s="7">
         <v>38443</v>
       </c>
-      <c r="D78" s="3" t="str">
+      <c r="D78" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>703</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 39 replicated with old route, 2 frames lost to random lag, going to try other routes
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC4334D-5C5A-43EB-80EF-DA59405F377B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A87A7200-43F4-4BF7-A602-CB5674DCB9DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1317,12 +1317,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="37" x14ac:knownFonts="1">
+  <fonts count="38" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1782,95 +1789,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1891,28 +1899,28 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2235,7 +2243,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:F184"/>
+  <dimension ref="A1:F191"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -3005,7 +3013,7 @@
         <v>23873</v>
       </c>
       <c r="D51" s="3">
-        <f t="shared" ref="D51:D80" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
+        <f t="shared" ref="D51:D87" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
         <v>430</v>
       </c>
     </row>
@@ -3439,348 +3447,385 @@
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A79" s="50" t="s">
-        <v>34</v>
-      </c>
+      <c r="A79" s="50"/>
       <c r="B79" s="7"/>
-      <c r="C79" s="7">
-        <v>38692</v>
-      </c>
+      <c r="C79" s="7"/>
       <c r="D79" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A80" s="50" t="s">
-        <v>15</v>
-      </c>
+      <c r="A80" s="53"/>
       <c r="B80" s="7"/>
-      <c r="C80" s="7">
-        <v>39041</v>
-      </c>
+      <c r="C80" s="7"/>
       <c r="D80" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" s="50" t="s">
-        <v>35</v>
-      </c>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="53"/>
       <c r="B81" s="7"/>
-      <c r="C81" s="7">
-        <v>40011</v>
-      </c>
+      <c r="C81" s="7"/>
       <c r="D81" s="3" t="str">
-        <f>IF(C80&lt;&gt;"",IF(B80&lt;&gt;"",C80-B80,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" s="50" t="s">
-        <v>16</v>
-      </c>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" s="53"/>
       <c r="B82" s="7"/>
-      <c r="C82" s="7">
-        <v>40373</v>
-      </c>
+      <c r="C82" s="7"/>
       <c r="D82" s="3" t="str">
-        <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B83" s="40"/>
-      <c r="C83" s="7">
-        <v>41117</v>
-      </c>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" s="53"/>
+      <c r="B83" s="7"/>
+      <c r="C83" s="7"/>
       <c r="D83" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="50" t="s">
-        <v>17</v>
-      </c>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" s="53"/>
       <c r="B84" s="7"/>
-      <c r="C84" s="7">
-        <v>41465</v>
-      </c>
+      <c r="C84" s="7"/>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" s="50" t="s">
-        <v>37</v>
-      </c>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="53"/>
       <c r="B85" s="7"/>
-      <c r="C85" s="7">
-        <v>42450</v>
-      </c>
+      <c r="C85" s="7"/>
       <c r="D85" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>18</v>
-      </c>
-      <c r="B86" s="7"/>
+        <v>34</v>
+      </c>
+      <c r="B86" s="7">
+        <v>37991</v>
+      </c>
       <c r="C86" s="7">
-        <v>42799</v>
-      </c>
-      <c r="D86" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38692</v>
+      </c>
+      <c r="D86" s="3">
+        <f t="shared" si="2"/>
+        <v>701</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>43144</v>
+        <v>39041</v>
       </c>
       <c r="D87" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>43491</v>
+        <v>40011</v>
       </c>
       <c r="D88" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(C87&lt;&gt;"",IF(B87&lt;&gt;"",C87-B87,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>44165</v>
+        <v>40373</v>
       </c>
       <c r="D89" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="D89:D108" si="3">IF(C89&lt;&gt;"",IF(B89&lt;&gt;"",C89-B89,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>20</v>
-      </c>
-      <c r="B90" s="7"/>
+        <v>36</v>
+      </c>
+      <c r="B90" s="40"/>
       <c r="C90" s="7">
-        <v>44512</v>
+        <v>41117</v>
       </c>
       <c r="D90" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>45061</v>
+        <v>41465</v>
       </c>
       <c r="D91" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>45443</v>
+        <v>42450</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>45990</v>
+        <v>42799</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>46652</v>
+        <v>43144</v>
       </c>
       <c r="D94" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E94" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>47436</v>
+        <v>43491</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B96" s="9"/>
-      <c r="C96" s="9">
-        <v>48337</v>
+        <v>39</v>
+      </c>
+      <c r="B96" s="7"/>
+      <c r="C96" s="7">
+        <v>44165</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>49334</v>
+        <v>44512</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>48681</v>
+        <v>45061</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>49334</v>
+        <v>45443</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>49683</v>
+        <v>45990</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>50244</v>
+        <v>46652</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E101" s="51" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="50" t="s">
+        <v>42</v>
+      </c>
       <c r="B102" s="7"/>
-      <c r="C102" s="7"/>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B103" s="7"/>
-      <c r="C103" s="7"/>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C102" s="7">
+        <v>47436</v>
+      </c>
+      <c r="D102" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="50" t="s">
+        <v>23</v>
+      </c>
+      <c r="B103" s="9"/>
+      <c r="C103" s="9">
+        <v>48337</v>
+      </c>
+      <c r="D103" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="50" t="s">
+        <v>43</v>
+      </c>
       <c r="B104" s="7"/>
-      <c r="C104" s="7"/>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C104" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D104" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="50" t="s">
+        <v>24</v>
+      </c>
       <c r="B105" s="7"/>
-      <c r="C105" s="7"/>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C105" s="7">
+        <v>48681</v>
+      </c>
+      <c r="D105" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="50" t="s">
+        <v>44</v>
+      </c>
       <c r="B106" s="7"/>
-      <c r="C106" s="7"/>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C106" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D106" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="50" t="s">
+        <v>25</v>
+      </c>
       <c r="B107" s="7"/>
-      <c r="C107" s="7"/>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C107" s="7">
+        <v>49683</v>
+      </c>
+      <c r="D107" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" s="50" t="s">
+        <v>26</v>
+      </c>
       <c r="B108" s="7"/>
-      <c r="C108" s="7"/>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C108" s="7">
+        <v>50244</v>
+      </c>
+      <c r="D108" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
     </row>
@@ -4071,6 +4116,34 @@
     <row r="184" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
+    </row>
+    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B185" s="7"/>
+      <c r="C185" s="7"/>
+    </row>
+    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B186" s="7"/>
+      <c r="C186" s="7"/>
+    </row>
+    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B187" s="7"/>
+      <c r="C187" s="7"/>
+    </row>
+    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B188" s="7"/>
+      <c r="C188" s="7"/>
+    </row>
+    <row r="189" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B189" s="7"/>
+      <c r="C189" s="7"/>
+    </row>
+    <row r="190" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B190" s="7"/>
+      <c r="C190" s="7"/>
+    </row>
+    <row r="191" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B191" s="7"/>
+      <c r="C191" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18919,7 +18992,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="33" type="noConversion"/>
+  <phoneticPr fontId="34" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -18949,10 +19022,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="53" t="s">
+      <c r="K1" s="54" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="54"/>
+      <c r="L1" s="55"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -20804,13 +20877,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="55" t="s">
+      <c r="H53" s="56" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="56"/>
-      <c r="J53" s="56"/>
-      <c r="K53" s="56"/>
-      <c r="L53" s="57"/>
+      <c r="I53" s="57"/>
+      <c r="J53" s="57"/>
+      <c r="K53" s="57"/>
+      <c r="L53" s="58"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -20832,11 +20905,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="58"/>
-      <c r="I54" s="59"/>
-      <c r="J54" s="59"/>
-      <c r="K54" s="59"/>
-      <c r="L54" s="60"/>
+      <c r="H54" s="59"/>
+      <c r="I54" s="60"/>
+      <c r="J54" s="60"/>
+      <c r="K54" s="60"/>
+      <c r="L54" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - lv 39 done - 701 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A87A7200-43F4-4BF7-A602-CB5674DCB9DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E53C0C-DF53-4451-B11B-2CE452716DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1317,19 +1317,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="38" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1789,96 +1782,95 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="30" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="5"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1899,28 +1891,28 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2243,7 +2235,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:F191"/>
+  <dimension ref="A1:F184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -3013,7 +3005,7 @@
         <v>23873</v>
       </c>
       <c r="D51" s="3">
-        <f t="shared" ref="D51:D87" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
+        <f t="shared" ref="D51:D81" si="2">IF(C51&lt;&gt;"",IF(B51&lt;&gt;"",C51-B51,"-"), "-")</f>
         <v>430</v>
       </c>
     </row>
@@ -3447,385 +3439,352 @@
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A79" s="50"/>
-      <c r="B79" s="7"/>
-      <c r="C79" s="7"/>
-      <c r="D79" s="3" t="str">
+      <c r="A79" s="50" t="s">
+        <v>34</v>
+      </c>
+      <c r="B79" s="7">
+        <v>37991</v>
+      </c>
+      <c r="C79" s="7">
+        <v>38692</v>
+      </c>
+      <c r="D79" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>701</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A80" s="53"/>
-      <c r="B80" s="7"/>
-      <c r="C80" s="7"/>
-      <c r="D80" s="3" t="str">
+      <c r="A80" s="50" t="s">
+        <v>15</v>
+      </c>
+      <c r="B80" s="7">
+        <v>38340</v>
+      </c>
+      <c r="C80" s="7">
+        <v>39041</v>
+      </c>
+      <c r="D80" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="53"/>
+        <v>701</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="50" t="s">
+        <v>35</v>
+      </c>
       <c r="B81" s="7"/>
-      <c r="C81" s="7"/>
+      <c r="C81" s="7">
+        <v>40011</v>
+      </c>
       <c r="D81" s="3" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="53"/>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="50" t="s">
+        <v>16</v>
+      </c>
       <c r="B82" s="7"/>
-      <c r="C82" s="7"/>
+      <c r="C82" s="7">
+        <v>40373</v>
+      </c>
       <c r="D82" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
         <v>-</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="53"/>
-      <c r="B83" s="7"/>
-      <c r="C83" s="7"/>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="50" t="s">
+        <v>36</v>
+      </c>
+      <c r="B83" s="40"/>
+      <c r="C83" s="7">
+        <v>41117</v>
+      </c>
       <c r="D83" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="53"/>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="50" t="s">
+        <v>17</v>
+      </c>
       <c r="B84" s="7"/>
-      <c r="C84" s="7"/>
+      <c r="C84" s="7">
+        <v>41465</v>
+      </c>
       <c r="D84" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="53"/>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="50" t="s">
+        <v>37</v>
+      </c>
       <c r="B85" s="7"/>
-      <c r="C85" s="7"/>
+      <c r="C85" s="7">
+        <v>42450</v>
+      </c>
       <c r="D85" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="50" t="s">
-        <v>34</v>
-      </c>
-      <c r="B86" s="7">
-        <v>37991</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="B86" s="7"/>
       <c r="C86" s="7">
-        <v>38692</v>
-      </c>
-      <c r="D86" s="3">
-        <f t="shared" si="2"/>
-        <v>701</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+        <v>42799</v>
+      </c>
+      <c r="D86" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="50" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B87" s="7"/>
       <c r="C87" s="7">
-        <v>39041</v>
+        <v>43144</v>
       </c>
       <c r="D87" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="50" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7">
-        <v>40011</v>
+        <v>43491</v>
       </c>
       <c r="D88" s="3" t="str">
-        <f>IF(C87&lt;&gt;"",IF(B87&lt;&gt;"",C87-B87,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7">
-        <v>40373</v>
+        <v>44165</v>
       </c>
       <c r="D89" s="3" t="str">
-        <f t="shared" ref="D89:D108" si="3">IF(C89&lt;&gt;"",IF(B89&lt;&gt;"",C89-B89,"-"), "-")</f>
+        <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="B90" s="40"/>
+        <v>20</v>
+      </c>
+      <c r="B90" s="7"/>
       <c r="C90" s="7">
-        <v>41117</v>
+        <v>44512</v>
       </c>
       <c r="D90" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>41465</v>
+        <v>45061</v>
       </c>
       <c r="D91" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>42450</v>
+        <v>45443</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>42799</v>
+        <v>45990</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>43144</v>
+        <v>46652</v>
       </c>
       <c r="D94" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E94" s="51" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>43491</v>
+        <v>47436</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="B96" s="7"/>
-      <c r="C96" s="7">
-        <v>44165</v>
+        <v>23</v>
+      </c>
+      <c r="B96" s="9"/>
+      <c r="C96" s="9">
+        <v>48337</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>44512</v>
+        <v>49334</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>45061</v>
+        <v>48681</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>45443</v>
+        <v>49334</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>45990</v>
+        <v>49683</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>46652</v>
+        <v>50244</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E101" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="50" t="s">
-        <v>42</v>
-      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B102" s="7"/>
-      <c r="C102" s="7">
-        <v>47436</v>
-      </c>
-      <c r="D102" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B103" s="9"/>
-      <c r="C103" s="9">
-        <v>48337</v>
-      </c>
-      <c r="D103" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A104" s="50" t="s">
-        <v>43</v>
-      </c>
+      <c r="C102" s="7"/>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B103" s="7"/>
+      <c r="C103" s="7"/>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B104" s="7"/>
-      <c r="C104" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D104" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="50" t="s">
-        <v>24</v>
-      </c>
+      <c r="C104" s="7"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B105" s="7"/>
-      <c r="C105" s="7">
-        <v>48681</v>
-      </c>
-      <c r="D105" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="50" t="s">
-        <v>44</v>
-      </c>
+      <c r="C105" s="7"/>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B106" s="7"/>
-      <c r="C106" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D106" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="50" t="s">
-        <v>25</v>
-      </c>
+      <c r="C106" s="7"/>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B107" s="7"/>
-      <c r="C107" s="7">
-        <v>49683</v>
-      </c>
-      <c r="D107" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" s="50" t="s">
-        <v>26</v>
-      </c>
+      <c r="C107" s="7"/>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B108" s="7"/>
-      <c r="C108" s="7">
-        <v>50244</v>
-      </c>
-      <c r="D108" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C108" s="7"/>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
     </row>
@@ -4116,34 +4075,6 @@
     <row r="184" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
-    </row>
-    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B185" s="7"/>
-      <c r="C185" s="7"/>
-    </row>
-    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B186" s="7"/>
-      <c r="C186" s="7"/>
-    </row>
-    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B187" s="7"/>
-      <c r="C187" s="7"/>
-    </row>
-    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B188" s="7"/>
-      <c r="C188" s="7"/>
-    </row>
-    <row r="189" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B189" s="7"/>
-      <c r="C189" s="7"/>
-    </row>
-    <row r="190" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B190" s="7"/>
-      <c r="C190" s="7"/>
-    </row>
-    <row r="191" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B191" s="7"/>
-      <c r="C191" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18992,7 +18923,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="34" type="noConversion"/>
+  <phoneticPr fontId="33" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -19022,10 +18953,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="54" t="s">
+      <c r="K1" s="53" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="55"/>
+      <c r="L1" s="54"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -20877,13 +20808,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="56" t="s">
+      <c r="H53" s="55" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="57"/>
-      <c r="J53" s="57"/>
-      <c r="K53" s="57"/>
-      <c r="L53" s="58"/>
+      <c r="I53" s="56"/>
+      <c r="J53" s="56"/>
+      <c r="K53" s="56"/>
+      <c r="L53" s="57"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -20905,11 +20836,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="59"/>
-      <c r="I54" s="60"/>
-      <c r="J54" s="60"/>
-      <c r="K54" s="60"/>
-      <c r="L54" s="61"/>
+      <c r="H54" s="58"/>
+      <c r="I54" s="59"/>
+      <c r="J54" s="59"/>
+      <c r="K54" s="59"/>
+      <c r="L54" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - lv 40 script
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E53C0C-DF53-4451-B11B-2CE452716DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{983EC914-6ADD-4A9C-9592-4642143D775F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3472,13 +3472,15 @@
       <c r="A81" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="B81" s="7"/>
+      <c r="B81" s="7">
+        <v>39308</v>
+      </c>
       <c r="C81" s="7">
         <v>40011</v>
       </c>
-      <c r="D81" s="3" t="str">
+      <c r="D81" s="3">
         <f t="shared" si="2"/>
-        <v>-</v>
+        <v>703</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 40 done - 702 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{983EC914-6ADD-4A9C-9592-4642143D775F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DC8D741-AA82-4126-9135-0A70B6B3B5DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3487,13 +3487,15 @@
       <c r="A82" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="B82" s="7"/>
+      <c r="B82" s="7">
+        <v>39656</v>
+      </c>
       <c r="C82" s="7">
-        <v>40373</v>
-      </c>
-      <c r="D82" s="3" t="str">
+        <v>40358</v>
+      </c>
+      <c r="D82" s="3">
         <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
-        <v>-</v>
+        <v>702</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 41 done - 708 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DC8D741-AA82-4126-9135-0A70B6B3B5DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6A27A13-8974-4890-AE0C-68717CD2DCEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="425">
   <si>
     <t>Place</t>
   </si>
@@ -1308,6 +1308,9 @@
   </si>
   <si>
     <t>fast mode</t>
+  </si>
+  <si>
+    <t>39656 possible, 6 frames to get exact gold drop</t>
   </si>
 </sst>
 </file>
@@ -1317,12 +1320,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="37" x14ac:knownFonts="1">
+  <fonts count="38" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1782,95 +1792,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1890,31 +1901,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -3488,40 +3499,47 @@
         <v>16</v>
       </c>
       <c r="B82" s="7">
-        <v>39656</v>
+        <v>39662</v>
       </c>
       <c r="C82" s="7">
         <v>40358</v>
       </c>
       <c r="D82" s="3">
         <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
-        <v>702</v>
+        <v>696</v>
+      </c>
+      <c r="E82" s="61" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="B83" s="40"/>
+      <c r="B83" s="61">
+        <v>40406</v>
+      </c>
       <c r="C83" s="7">
         <v>41117</v>
       </c>
-      <c r="D83" s="3" t="str">
+      <c r="D83" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>711</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="B84" s="7"/>
+      <c r="B84" s="7">
+        <v>40757</v>
+      </c>
       <c r="C84" s="7">
         <v>41465</v>
       </c>
-      <c r="D84" s="3" t="str">
+      <c r="D84" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>708</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
@@ -18927,7 +18945,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="33" type="noConversion"/>
+  <phoneticPr fontId="34" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>

</xml_diff>

<commit_message>
lode runner - lv 42 2 frames slow, more investigation needed
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6A27A13-8974-4890-AE0C-68717CD2DCEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB1398C-EE4B-4435-9C96-6320349D4669}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3546,13 +3546,15 @@
       <c r="A85" s="50" t="s">
         <v>37</v>
       </c>
-      <c r="B85" s="7"/>
+      <c r="B85" s="7">
+        <v>41744</v>
+      </c>
       <c r="C85" s="7">
         <v>42450</v>
       </c>
-      <c r="D85" s="3" t="str">
+      <c r="D85" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>706</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 42 done - 707 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB1398C-EE4B-4435-9C96-6320349D4669}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE5216E-0566-4385-AA3C-08B601375CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="49995" yWindow="2925" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="50220" yWindow="3195" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -1901,6 +1901,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1925,7 +1926,6 @@
     <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -3508,7 +3508,7 @@
         <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
         <v>696</v>
       </c>
-      <c r="E82" s="61" t="s">
+      <c r="E82" s="53" t="s">
         <v>424</v>
       </c>
     </row>
@@ -3516,7 +3516,7 @@
       <c r="A83" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="B83" s="61">
+      <c r="B83" s="53">
         <v>40406</v>
       </c>
       <c r="C83" s="7">
@@ -3561,13 +3561,15 @@
       <c r="A86" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="B86" s="7"/>
+      <c r="B86" s="7">
+        <v>42092</v>
+      </c>
       <c r="C86" s="7">
         <v>42799</v>
       </c>
-      <c r="D86" s="3" t="str">
+      <c r="D86" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>707</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
@@ -18977,10 +18979,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="53" t="s">
+      <c r="K1" s="54" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="54"/>
+      <c r="L1" s="55"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -20832,13 +20834,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="55" t="s">
+      <c r="H53" s="56" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="56"/>
-      <c r="J53" s="56"/>
-      <c r="K53" s="56"/>
-      <c r="L53" s="57"/>
+      <c r="I53" s="57"/>
+      <c r="J53" s="57"/>
+      <c r="K53" s="57"/>
+      <c r="L53" s="58"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -20860,11 +20862,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="58"/>
-      <c r="I54" s="59"/>
-      <c r="J54" s="59"/>
-      <c r="K54" s="59"/>
-      <c r="L54" s="60"/>
+      <c r="H54" s="59"/>
+      <c r="I54" s="60"/>
+      <c r="J54" s="60"/>
+      <c r="K54" s="60"/>
+      <c r="L54" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - lv 42 2 frames faster, 709 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE5216E-0566-4385-AA3C-08B601375CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D85B79-6116-4AFF-8EF3-7A8228CD4A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50220" yWindow="3195" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="49965" yWindow="2685" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -3547,14 +3547,14 @@
         <v>37</v>
       </c>
       <c r="B85" s="7">
-        <v>41744</v>
+        <v>41743</v>
       </c>
       <c r="C85" s="7">
         <v>42450</v>
       </c>
       <c r="D85" s="3">
         <f t="shared" si="3"/>
-        <v>706</v>
+        <v>707</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -3562,14 +3562,14 @@
         <v>18</v>
       </c>
       <c r="B86" s="7">
-        <v>42092</v>
+        <v>42090</v>
       </c>
       <c r="C86" s="7">
         <v>42799</v>
       </c>
       <c r="D86" s="3">
         <f t="shared" si="3"/>
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - lv 43 done - 701 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D85B79-6116-4AFF-8EF3-7A8228CD4A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D44505D7-192D-4498-833F-3A7D5E8656AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="49965" yWindow="2685" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="425">
   <si>
     <t>Place</t>
   </si>
@@ -1320,12 +1320,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="38" x14ac:knownFonts="1">
+  <fonts count="39" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1792,95 +1799,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="30" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1901,31 +1909,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2246,7 +2254,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:F184"/>
+  <dimension ref="A1:F186"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -3505,7 +3513,7 @@
         <v>40358</v>
       </c>
       <c r="D82" s="3">
-        <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
+        <f t="shared" ref="D82:D103" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
         <v>696</v>
       </c>
       <c r="E82" s="53" t="s">
@@ -3562,75 +3570,88 @@
         <v>18</v>
       </c>
       <c r="B86" s="7">
-        <v>42090</v>
+        <v>42094</v>
       </c>
       <c r="C86" s="7">
         <v>42799</v>
       </c>
       <c r="D86" s="3">
         <f t="shared" si="3"/>
-        <v>709</v>
+        <v>705</v>
+      </c>
+      <c r="E86" s="7">
+        <v>42090</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" s="50" t="s">
-        <v>38</v>
-      </c>
-      <c r="B87" s="7"/>
+      <c r="A87" s="62" t="s">
+        <v>148</v>
+      </c>
+      <c r="B87" s="7">
+        <v>42371</v>
+      </c>
       <c r="C87" s="7">
-        <v>43144</v>
-      </c>
-      <c r="D87" s="3" t="str">
+        <v>43075</v>
+      </c>
+      <c r="D87" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
+        <v>704</v>
+      </c>
+      <c r="E87" s="7"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" s="50" t="s">
-        <v>19</v>
-      </c>
-      <c r="B88" s="7"/>
+      <c r="A88" s="62" t="s">
+        <v>233</v>
+      </c>
+      <c r="B88" s="7">
+        <v>42391</v>
+      </c>
       <c r="C88" s="7">
-        <v>43491</v>
-      </c>
-      <c r="D88" s="3" t="str">
+        <v>43091</v>
+      </c>
+      <c r="D88" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
+        <v>700</v>
+      </c>
+      <c r="E88" s="7"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="B89" s="7"/>
+        <v>38</v>
+      </c>
+      <c r="B89" s="7">
+        <v>42444</v>
+      </c>
       <c r="C89" s="7">
-        <v>44165</v>
-      </c>
-      <c r="D89" s="3" t="str">
+        <v>43144</v>
+      </c>
+      <c r="D89" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>700</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="50" t="s">
-        <v>20</v>
-      </c>
-      <c r="B90" s="7"/>
+        <v>19</v>
+      </c>
+      <c r="B90" s="7">
+        <v>42790</v>
+      </c>
       <c r="C90" s="7">
-        <v>44512</v>
-      </c>
-      <c r="D90" s="3" t="str">
+        <v>43491</v>
+      </c>
+      <c r="D90" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>701</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="50" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>45061</v>
+        <v>44165</v>
       </c>
       <c r="D91" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3639,11 +3660,11 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>45443</v>
+        <v>44512</v>
       </c>
       <c r="D92" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3652,11 +3673,11 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="50" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>45990</v>
+        <v>45061</v>
       </c>
       <c r="D93" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3665,27 +3686,24 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>46652</v>
+        <v>45443</v>
       </c>
       <c r="D94" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E94" s="51" t="s">
-        <v>422</v>
-      </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>47436</v>
+        <v>45990</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3694,24 +3712,27 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B96" s="9"/>
-      <c r="C96" s="9">
-        <v>48337</v>
+        <v>22</v>
+      </c>
+      <c r="B96" s="7"/>
+      <c r="C96" s="7">
+        <v>46652</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
+      <c r="E96" s="51" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>49334</v>
+        <v>47436</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3720,11 +3741,11 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>24</v>
-      </c>
-      <c r="B98" s="7"/>
-      <c r="C98" s="7">
-        <v>48681</v>
+        <v>23</v>
+      </c>
+      <c r="B98" s="9"/>
+      <c r="C98" s="9">
+        <v>48337</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3733,7 +3754,7 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
@@ -3746,11 +3767,11 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>49683</v>
+        <v>48681</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3759,11 +3780,11 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>50244</v>
+        <v>49334</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3771,12 +3792,30 @@
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="50" t="s">
+        <v>25</v>
+      </c>
       <c r="B102" s="7"/>
-      <c r="C102" s="7"/>
+      <c r="C102" s="7">
+        <v>49683</v>
+      </c>
+      <c r="D102" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103" s="50" t="s">
+        <v>26</v>
+      </c>
       <c r="B103" s="7"/>
-      <c r="C103" s="7"/>
+      <c r="C103" s="7">
+        <v>50244</v>
+      </c>
+      <c r="D103" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B104" s="7"/>
@@ -4101,6 +4140,14 @@
     <row r="184" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
+    </row>
+    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B185" s="7"/>
+      <c r="C185" s="7"/>
+    </row>
+    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B186" s="7"/>
+      <c r="C186" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18949,7 +18996,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="34" type="noConversion"/>
+  <phoneticPr fontId="35" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>

</xml_diff>

<commit_message>
lode runner - lv 44 nominally done, 5 frames saved
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D44505D7-192D-4498-833F-3A7D5E8656AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4228D157-7341-4E10-9EDA-F90D15919099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="49965" yWindow="2685" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="50310" yWindow="3030" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="425">
   <si>
     <t>Place</t>
   </si>
@@ -2254,7 +2254,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:F186"/>
+  <dimension ref="A1:F189"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -3513,7 +3513,7 @@
         <v>40358</v>
       </c>
       <c r="D82" s="3">
-        <f t="shared" ref="D82:D103" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
+        <f t="shared" ref="D82:D106" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
         <v>696</v>
       </c>
       <c r="E82" s="53" t="s">
@@ -3584,126 +3584,128 @@
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" s="62" t="s">
-        <v>148</v>
+      <c r="A87" s="50" t="s">
+        <v>38</v>
       </c>
       <c r="B87" s="7">
-        <v>42371</v>
+        <v>42444</v>
       </c>
       <c r="C87" s="7">
-        <v>43075</v>
+        <v>43144</v>
       </c>
       <c r="D87" s="3">
         <f t="shared" si="3"/>
-        <v>704</v>
-      </c>
-      <c r="E87" s="7"/>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" s="62" t="s">
-        <v>233</v>
+        <v>700</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="50" t="s">
+        <v>19</v>
       </c>
       <c r="B88" s="7">
-        <v>42391</v>
+        <v>42790</v>
       </c>
       <c r="C88" s="7">
-        <v>43091</v>
+        <v>43491</v>
       </c>
       <c r="D88" s="3">
         <f t="shared" si="3"/>
-        <v>700</v>
-      </c>
-      <c r="E88" s="7"/>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" s="50" t="s">
-        <v>38</v>
-      </c>
+        <v>701</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="50"/>
       <c r="B89" s="7">
-        <v>42444</v>
+        <v>42798</v>
       </c>
       <c r="C89" s="7">
-        <v>43144</v>
+        <v>43499</v>
       </c>
       <c r="D89" s="3">
         <f t="shared" si="3"/>
-        <v>700</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A90" s="50" t="s">
-        <v>19</v>
-      </c>
+        <v>701</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="50"/>
       <c r="B90" s="7">
-        <v>42790</v>
+        <v>42805</v>
       </c>
       <c r="C90" s="7">
-        <v>43491</v>
+        <v>43506</v>
       </c>
       <c r="D90" s="3">
         <f t="shared" si="3"/>
         <v>701</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="B91" s="7"/>
+    <row r="91" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="62" t="s">
+        <v>265</v>
+      </c>
+      <c r="B91" s="7">
+        <v>42804</v>
+      </c>
       <c r="C91" s="7">
-        <v>44165</v>
-      </c>
-      <c r="D91" s="3" t="str">
+        <v>43505</v>
+      </c>
+      <c r="D91" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" s="50" t="s">
-        <v>20</v>
-      </c>
-      <c r="B92" s="7"/>
+        <v>701</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="62" t="s">
+        <v>319</v>
+      </c>
+      <c r="B92" s="7">
+        <v>42830</v>
+      </c>
       <c r="C92" s="7">
-        <v>44512</v>
-      </c>
-      <c r="D92" s="3" t="str">
+        <v>43529</v>
+      </c>
+      <c r="D92" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>699</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" s="50" t="s">
-        <v>40</v>
-      </c>
-      <c r="B93" s="7"/>
+      <c r="A93" s="62" t="s">
+        <v>293</v>
+      </c>
+      <c r="B93" s="7">
+        <v>43050</v>
+      </c>
       <c r="C93" s="7">
-        <v>45061</v>
-      </c>
-      <c r="D93" s="3" t="str">
+        <v>43782</v>
+      </c>
+      <c r="D93" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>732</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>21</v>
-      </c>
-      <c r="B94" s="7"/>
+        <v>39</v>
+      </c>
+      <c r="B94" s="7">
+        <v>43459</v>
+      </c>
       <c r="C94" s="7">
-        <v>45443</v>
-      </c>
-      <c r="D94" s="3" t="str">
+        <v>44165</v>
+      </c>
+      <c r="D94" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>706</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>45990</v>
+        <v>44512</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3712,144 +3714,171 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="B96" s="7"/>
       <c r="C96" s="7">
-        <v>46652</v>
+        <v>45061</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E96" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>47436</v>
+        <v>45443</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B98" s="9"/>
-      <c r="C98" s="9">
-        <v>48337</v>
+        <v>41</v>
+      </c>
+      <c r="B98" s="7"/>
+      <c r="C98" s="7">
+        <v>45990</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>49334</v>
+        <v>46652</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E99" s="51" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>48681</v>
+        <v>47436</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>44</v>
-      </c>
-      <c r="B101" s="7"/>
-      <c r="C101" s="7">
-        <v>49334</v>
+        <v>23</v>
+      </c>
+      <c r="B101" s="9"/>
+      <c r="C101" s="9">
+        <v>48337</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="50" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="B102" s="7"/>
       <c r="C102" s="7">
-        <v>49683</v>
+        <v>49334</v>
       </c>
       <c r="D102" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="50" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B103" s="7"/>
       <c r="C103" s="7">
-        <v>50244</v>
+        <v>48681</v>
       </c>
       <c r="D103" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="50" t="s">
+        <v>44</v>
+      </c>
       <c r="B104" s="7"/>
-      <c r="C104" s="7"/>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C104" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D104" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="50" t="s">
+        <v>25</v>
+      </c>
       <c r="B105" s="7"/>
-      <c r="C105" s="7"/>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C105" s="7">
+        <v>49683</v>
+      </c>
+      <c r="D105" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="50" t="s">
+        <v>26</v>
+      </c>
       <c r="B106" s="7"/>
-      <c r="C106" s="7"/>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C106" s="7">
+        <v>50244</v>
+      </c>
+      <c r="D106" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B107" s="7"/>
       <c r="C107" s="7"/>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B108" s="7"/>
       <c r="C108" s="7"/>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
     </row>
@@ -4148,6 +4177,18 @@
     <row r="186" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B186" s="7"/>
       <c r="C186" s="7"/>
+    </row>
+    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B187" s="7"/>
+      <c r="C187" s="7"/>
+    </row>
+    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B188" s="7"/>
+      <c r="C188" s="7"/>
+    </row>
+    <row r="189" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B189" s="7"/>
+      <c r="C189" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lode runner - lv 44 - new route - 797 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4228D157-7341-4E10-9EDA-F90D15919099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F027A9-FC98-4ACC-94A4-8014E41A6847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50310" yWindow="3030" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="425">
   <si>
     <t>Place</t>
   </si>
@@ -1320,19 +1320,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="39" x14ac:knownFonts="1">
+  <fonts count="38" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1799,96 +1792,95 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" xfId="5"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1909,31 +1901,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2254,7 +2246,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:F189"/>
+  <dimension ref="A1:F184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -3513,7 +3505,7 @@
         <v>40358</v>
       </c>
       <c r="D82" s="3">
-        <f t="shared" ref="D82:D106" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
+        <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
         <v>696</v>
       </c>
       <c r="E82" s="53" t="s">
@@ -3613,99 +3605,98 @@
         <v>701</v>
       </c>
     </row>
-    <row r="89" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="50"/>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="50" t="s">
+        <v>39</v>
+      </c>
       <c r="B89" s="7">
-        <v>42798</v>
+        <v>43365</v>
       </c>
       <c r="C89" s="7">
-        <v>43499</v>
+        <v>44165</v>
       </c>
       <c r="D89" s="3">
         <f t="shared" si="3"/>
-        <v>701</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="50"/>
+        <v>800</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="50" t="s">
+        <v>20</v>
+      </c>
       <c r="B90" s="7">
-        <v>42805</v>
+        <v>43715</v>
       </c>
       <c r="C90" s="7">
-        <v>43506</v>
+        <v>44512</v>
       </c>
       <c r="D90" s="3">
         <f t="shared" si="3"/>
-        <v>701</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="62" t="s">
-        <v>265</v>
-      </c>
-      <c r="B91" s="7">
-        <v>42804</v>
-      </c>
+        <v>797</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="B91" s="7"/>
       <c r="C91" s="7">
-        <v>43505</v>
-      </c>
-      <c r="D91" s="3">
+        <v>45061</v>
+      </c>
+      <c r="D91" s="3" t="str">
         <f t="shared" si="3"/>
-        <v>701</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="62" t="s">
-        <v>319</v>
-      </c>
-      <c r="B92" s="7">
-        <v>42830</v>
-      </c>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="B92" s="7"/>
       <c r="C92" s="7">
-        <v>43529</v>
-      </c>
-      <c r="D92" s="3">
+        <v>45443</v>
+      </c>
+      <c r="D92" s="3" t="str">
         <f t="shared" si="3"/>
-        <v>699</v>
+        <v>-</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" s="62" t="s">
-        <v>293</v>
-      </c>
-      <c r="B93" s="7">
-        <v>43050</v>
-      </c>
+      <c r="A93" s="50" t="s">
+        <v>41</v>
+      </c>
+      <c r="B93" s="7"/>
       <c r="C93" s="7">
-        <v>43782</v>
-      </c>
-      <c r="D93" s="3">
+        <v>45990</v>
+      </c>
+      <c r="D93" s="3" t="str">
         <f t="shared" si="3"/>
-        <v>732</v>
+        <v>-</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="B94" s="7">
-        <v>43459</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>44165</v>
-      </c>
-      <c r="D94" s="3">
+        <v>46652</v>
+      </c>
+      <c r="D94" s="3" t="str">
         <f t="shared" si="3"/>
-        <v>706</v>
+        <v>-</v>
+      </c>
+      <c r="E94" s="51" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="50" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>44512</v>
+        <v>47436</v>
       </c>
       <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
@@ -3714,171 +3705,123 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
-        <v>40</v>
-      </c>
-      <c r="B96" s="7"/>
-      <c r="C96" s="7">
-        <v>45061</v>
+        <v>23</v>
+      </c>
+      <c r="B96" s="9"/>
+      <c r="C96" s="9">
+        <v>48337</v>
       </c>
       <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>45443</v>
+        <v>49334</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7">
-        <v>45990</v>
+        <v>48681</v>
       </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>46652</v>
+        <v>49334</v>
       </c>
       <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E99" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>47436</v>
+        <v>49683</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B101" s="9"/>
-      <c r="C101" s="9">
-        <v>48337</v>
+        <v>26</v>
+      </c>
+      <c r="B101" s="7"/>
+      <c r="C101" s="7">
+        <v>50244</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="50" t="s">
-        <v>43</v>
-      </c>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B102" s="7"/>
-      <c r="C102" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D102" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="50" t="s">
-        <v>24</v>
-      </c>
+      <c r="C102" s="7"/>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B103" s="7"/>
-      <c r="C103" s="7">
-        <v>48681</v>
-      </c>
-      <c r="D103" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A104" s="50" t="s">
-        <v>44</v>
-      </c>
+      <c r="C103" s="7"/>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B104" s="7"/>
-      <c r="C104" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D104" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="50" t="s">
-        <v>25</v>
-      </c>
+      <c r="C104" s="7"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B105" s="7"/>
-      <c r="C105" s="7">
-        <v>49683</v>
-      </c>
-      <c r="D105" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="50" t="s">
-        <v>26</v>
-      </c>
+      <c r="C105" s="7"/>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B106" s="7"/>
-      <c r="C106" s="7">
-        <v>50244</v>
-      </c>
-      <c r="D106" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C106" s="7"/>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B107" s="7"/>
       <c r="C107" s="7"/>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B108" s="7"/>
       <c r="C108" s="7"/>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
     </row>
@@ -4169,26 +4112,6 @@
     <row r="184" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
-    </row>
-    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B185" s="7"/>
-      <c r="C185" s="7"/>
-    </row>
-    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B186" s="7"/>
-      <c r="C186" s="7"/>
-    </row>
-    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B187" s="7"/>
-      <c r="C187" s="7"/>
-    </row>
-    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B188" s="7"/>
-      <c r="C188" s="7"/>
-    </row>
-    <row r="189" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B189" s="7"/>
-      <c r="C189" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19037,7 +18960,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="35" type="noConversion"/>
+  <phoneticPr fontId="34" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>

</xml_diff>

<commit_message>
lode runner - lv 45 done - 800 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F027A9-FC98-4ACC-94A4-8014E41A6847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1673C97-B65D-4234-8B84-67A6D5C46732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50310" yWindow="3030" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3639,26 +3639,30 @@
       <c r="A91" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="B91" s="7"/>
+      <c r="B91" s="7">
+        <v>44263</v>
+      </c>
       <c r="C91" s="7">
         <v>45061</v>
       </c>
-      <c r="D91" s="3" t="str">
+      <c r="D91" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>798</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="B92" s="7"/>
+      <c r="B92" s="7">
+        <v>44611</v>
+      </c>
       <c r="C92" s="7">
-        <v>45443</v>
-      </c>
-      <c r="D92" s="3" t="str">
+        <v>45411</v>
+      </c>
+      <c r="D92" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>800</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lv 46 nominally done but worse lag, 786 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB08E5E9-11DC-4993-B86D-9E826E7B6590}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24AEDB3B-0458-4AA1-BCCA-974E443EC705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50310" yWindow="3030" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="426">
   <si>
     <t>Place</t>
   </si>
@@ -1313,7 +1313,7 @@
     <t>39656 possible, 6 frames to get exact gold drop</t>
   </si>
   <si>
-    <t>grab aldder</t>
+    <t>1st fall</t>
   </si>
 </sst>
 </file>
@@ -1323,12 +1323,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="39" x14ac:knownFonts="1">
+  <fonts count="40" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1802,95 +1809,96 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="37" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1912,28 +1920,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2257,7 +2265,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:F186"/>
+  <dimension ref="A1:F190"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -3516,7 +3524,7 @@
         <v>40358</v>
       </c>
       <c r="D82" s="3">
-        <f t="shared" ref="D82:D103" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
+        <f t="shared" ref="D82:D107" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
         <v>696</v>
       </c>
       <c r="E82" s="53" t="s">
@@ -3666,201 +3674,239 @@
         <v>21</v>
       </c>
       <c r="B92" s="7">
-        <v>44611</v>
+        <v>44612</v>
       </c>
       <c r="C92" s="7">
         <v>45411</v>
       </c>
       <c r="D92" s="3">
         <f t="shared" si="3"/>
-        <v>800</v>
+        <v>799</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" s="62" t="s">
-        <v>150</v>
+      <c r="A93" s="63" t="s">
+        <v>127</v>
       </c>
       <c r="B93" s="7">
-        <v>45012</v>
+        <v>44742</v>
       </c>
       <c r="C93" s="7">
-        <v>45801</v>
+        <v>45538</v>
       </c>
       <c r="D93" s="3">
         <f t="shared" si="3"/>
-        <v>789</v>
+        <v>796</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A94" s="62" t="s">
+      <c r="A94" s="63" t="s">
         <v>425</v>
       </c>
       <c r="B94" s="7">
-        <v>45134</v>
+        <v>44825</v>
       </c>
       <c r="C94" s="7">
-        <v>45920</v>
+        <v>45622</v>
       </c>
       <c r="D94" s="3">
         <f t="shared" si="3"/>
-        <v>786</v>
+        <v>797</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" s="50" t="s">
-        <v>41</v>
+      <c r="A95" s="63" t="s">
+        <v>265</v>
       </c>
       <c r="B95" s="7">
-        <v>45204</v>
+        <v>44844</v>
       </c>
       <c r="C95" s="7">
-        <v>45990</v>
+        <v>45639</v>
       </c>
       <c r="D95" s="3">
         <f t="shared" si="3"/>
-        <v>786</v>
+        <v>795</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A96" s="50" t="s">
-        <v>22</v>
-      </c>
-      <c r="B96" s="7"/>
+      <c r="A96" s="63" t="s">
+        <v>382</v>
+      </c>
+      <c r="B96" s="7">
+        <v>44888</v>
+      </c>
       <c r="C96" s="7">
-        <v>46652</v>
-      </c>
-      <c r="D96" s="3" t="str">
+        <v>45680</v>
+      </c>
+      <c r="D96" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-      <c r="E96" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="50" t="s">
-        <v>42</v>
-      </c>
-      <c r="B97" s="7"/>
+        <v>792</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" s="63" t="s">
+        <v>271</v>
+      </c>
+      <c r="B97" s="7">
+        <v>45012</v>
+      </c>
       <c r="C97" s="7">
-        <v>47436</v>
-      </c>
-      <c r="D97" s="3" t="str">
+        <v>45801</v>
+      </c>
+      <c r="D97" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B98" s="9"/>
-      <c r="C98" s="9">
-        <v>48337</v>
-      </c>
+        <v>789</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="54"/>
+      <c r="B98" s="7"/>
+      <c r="C98" s="7"/>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>43</v>
-      </c>
-      <c r="B99" s="7"/>
+        <v>41</v>
+      </c>
+      <c r="B99" s="7">
+        <v>45204</v>
+      </c>
       <c r="C99" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D99" s="3" t="str">
+        <v>45990</v>
+      </c>
+      <c r="D99" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>48681</v>
+        <v>46652</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E100" s="51" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>49334</v>
+        <v>47436</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="50" t="s">
-        <v>25</v>
-      </c>
-      <c r="B102" s="7"/>
-      <c r="C102" s="7">
-        <v>49683</v>
+        <v>23</v>
+      </c>
+      <c r="B102" s="9"/>
+      <c r="C102" s="9">
+        <v>48337</v>
       </c>
       <c r="D102" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="50" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="B103" s="7"/>
       <c r="C103" s="7">
-        <v>50244</v>
+        <v>49334</v>
       </c>
       <c r="D103" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="50" t="s">
+        <v>24</v>
+      </c>
       <c r="B104" s="7"/>
-      <c r="C104" s="7"/>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C104" s="7">
+        <v>48681</v>
+      </c>
+      <c r="D104" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="50" t="s">
+        <v>44</v>
+      </c>
       <c r="B105" s="7"/>
-      <c r="C105" s="7"/>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C105" s="7">
+        <v>49334</v>
+      </c>
+      <c r="D105" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="50" t="s">
+        <v>25</v>
+      </c>
       <c r="B106" s="7"/>
-      <c r="C106" s="7"/>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C106" s="7">
+        <v>49683</v>
+      </c>
+      <c r="D106" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="50" t="s">
+        <v>26</v>
+      </c>
       <c r="B107" s="7"/>
-      <c r="C107" s="7"/>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C107" s="7">
+        <v>50244</v>
+      </c>
+      <c r="D107" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B108" s="7"/>
       <c r="C108" s="7"/>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
     </row>
@@ -4159,6 +4205,22 @@
     <row r="186" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B186" s="7"/>
       <c r="C186" s="7"/>
+    </row>
+    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B187" s="7"/>
+      <c r="C187" s="7"/>
+    </row>
+    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B188" s="7"/>
+      <c r="C188" s="7"/>
+    </row>
+    <row r="189" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B189" s="7"/>
+      <c r="C189" s="7"/>
+    </row>
+    <row r="190" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B190" s="7"/>
+      <c r="C190" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19007,7 +19069,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="35" type="noConversion"/>
+  <phoneticPr fontId="36" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -19037,10 +19099,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="54" t="s">
+      <c r="K1" s="55" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="55"/>
+      <c r="L1" s="56"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -20892,13 +20954,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="56" t="s">
+      <c r="H53" s="57" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="57"/>
-      <c r="J53" s="57"/>
-      <c r="K53" s="57"/>
-      <c r="L53" s="58"/>
+      <c r="I53" s="58"/>
+      <c r="J53" s="58"/>
+      <c r="K53" s="58"/>
+      <c r="L53" s="59"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -20920,11 +20982,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="59"/>
-      <c r="I54" s="60"/>
-      <c r="J54" s="60"/>
-      <c r="K54" s="60"/>
-      <c r="L54" s="61"/>
+      <c r="H54" s="60"/>
+      <c r="I54" s="61"/>
+      <c r="J54" s="61"/>
+      <c r="K54" s="61"/>
+      <c r="L54" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - lv 46 done 10 frames faster, 796 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24AEDB3B-0458-4AA1-BCCA-974E443EC705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E92759FC-C8B8-4F93-8822-C297C78A956B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50310" yWindow="3030" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="425">
   <si>
     <t>Place</t>
   </si>
@@ -1311,9 +1311,6 @@
   </si>
   <si>
     <t>39656 possible, 6 frames to get exact gold drop</t>
-  </si>
-  <si>
-    <t>1st fall</t>
   </si>
 </sst>
 </file>
@@ -1323,26 +1320,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="40" x14ac:knownFonts="1">
+  <fonts count="38" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1809,97 +1792,95 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" xfId="5"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="6" applyFont="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1920,31 +1901,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2265,7 +2246,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:F190"/>
+  <dimension ref="A1:F184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -3524,7 +3505,7 @@
         <v>40358</v>
       </c>
       <c r="D82" s="3">
-        <f t="shared" ref="D82:D107" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
+        <f t="shared" ref="D82:D101" si="3">IF(C82&lt;&gt;"",IF(B82&lt;&gt;"",C82-B82,"-"), "-")</f>
         <v>696</v>
       </c>
       <c r="E82" s="53" t="s">
@@ -3674,25 +3655,25 @@
         <v>21</v>
       </c>
       <c r="B92" s="7">
-        <v>44612</v>
+        <v>44616</v>
       </c>
       <c r="C92" s="7">
         <v>45411</v>
       </c>
       <c r="D92" s="3">
         <f t="shared" si="3"/>
-        <v>799</v>
+        <v>795</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" s="63" t="s">
-        <v>127</v>
+      <c r="A93" s="50" t="s">
+        <v>41</v>
       </c>
       <c r="B93" s="7">
-        <v>44742</v>
+        <v>45194</v>
       </c>
       <c r="C93" s="7">
-        <v>45538</v>
+        <v>45990</v>
       </c>
       <c r="D93" s="3">
         <f t="shared" si="3"/>
@@ -3700,213 +3681,153 @@
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A94" s="63" t="s">
-        <v>425</v>
-      </c>
-      <c r="B94" s="7">
-        <v>44825</v>
-      </c>
+      <c r="A94" s="50" t="s">
+        <v>22</v>
+      </c>
+      <c r="B94" s="7"/>
       <c r="C94" s="7">
-        <v>45622</v>
-      </c>
-      <c r="D94" s="3">
+        <v>46652</v>
+      </c>
+      <c r="D94" s="3" t="str">
         <f t="shared" si="3"/>
-        <v>797</v>
+        <v>-</v>
+      </c>
+      <c r="E94" s="51" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" s="63" t="s">
-        <v>265</v>
-      </c>
-      <c r="B95" s="7">
-        <v>44844</v>
-      </c>
+      <c r="A95" s="50" t="s">
+        <v>42</v>
+      </c>
+      <c r="B95" s="7"/>
       <c r="C95" s="7">
-        <v>45639</v>
-      </c>
-      <c r="D95" s="3">
+        <v>47436</v>
+      </c>
+      <c r="D95" s="3" t="str">
         <f t="shared" si="3"/>
-        <v>795</v>
+        <v>-</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A96" s="63" t="s">
-        <v>382</v>
-      </c>
-      <c r="B96" s="7">
-        <v>44888</v>
-      </c>
-      <c r="C96" s="7">
-        <v>45680</v>
-      </c>
-      <c r="D96" s="3">
+      <c r="A96" s="50" t="s">
+        <v>23</v>
+      </c>
+      <c r="B96" s="9"/>
+      <c r="C96" s="9">
+        <v>48337</v>
+      </c>
+      <c r="D96" s="3" t="str">
         <f t="shared" si="3"/>
-        <v>792</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A97" s="63" t="s">
-        <v>271</v>
-      </c>
-      <c r="B97" s="7">
-        <v>45012</v>
-      </c>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" s="50" t="s">
+        <v>43</v>
+      </c>
+      <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>45801</v>
-      </c>
-      <c r="D97" s="3">
+        <v>49334</v>
+      </c>
+      <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>
-        <v>789</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A98" s="54"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" s="50" t="s">
+        <v>24</v>
+      </c>
       <c r="B98" s="7"/>
-      <c r="C98" s="7"/>
+      <c r="C98" s="7">
+        <v>48681</v>
+      </c>
       <c r="D98" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
-        <v>41</v>
-      </c>
-      <c r="B99" s="7">
-        <v>45204</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="B99" s="7"/>
       <c r="C99" s="7">
-        <v>45990</v>
-      </c>
-      <c r="D99" s="3">
+        <v>49334</v>
+      </c>
+      <c r="D99" s="3" t="str">
         <f t="shared" si="3"/>
-        <v>786</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7">
-        <v>46652</v>
+        <v>49683</v>
       </c>
       <c r="D100" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
-      <c r="E100" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7">
-        <v>47436</v>
+        <v>50244</v>
       </c>
       <c r="D101" s="3" t="str">
         <f t="shared" si="3"/>
         <v>-</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="B102" s="9"/>
-      <c r="C102" s="9">
-        <v>48337</v>
-      </c>
-      <c r="D102" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="50" t="s">
-        <v>43</v>
-      </c>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B102" s="7"/>
+      <c r="C102" s="7"/>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B103" s="7"/>
-      <c r="C103" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D103" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A104" s="50" t="s">
-        <v>24</v>
-      </c>
+      <c r="C103" s="7"/>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B104" s="7"/>
-      <c r="C104" s="7">
-        <v>48681</v>
-      </c>
-      <c r="D104" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="50" t="s">
-        <v>44</v>
-      </c>
+      <c r="C104" s="7"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B105" s="7"/>
-      <c r="C105" s="7">
-        <v>49334</v>
-      </c>
-      <c r="D105" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="50" t="s">
-        <v>25</v>
-      </c>
+      <c r="C105" s="7"/>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B106" s="7"/>
-      <c r="C106" s="7">
-        <v>49683</v>
-      </c>
-      <c r="D106" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="50" t="s">
-        <v>26</v>
-      </c>
+      <c r="C106" s="7"/>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B107" s="7"/>
-      <c r="C107" s="7">
-        <v>50244</v>
-      </c>
-      <c r="D107" s="3" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C107" s="7"/>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B108" s="7"/>
       <c r="C108" s="7"/>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
     </row>
@@ -4197,30 +4118,6 @@
     <row r="184" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
-    </row>
-    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B185" s="7"/>
-      <c r="C185" s="7"/>
-    </row>
-    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B186" s="7"/>
-      <c r="C186" s="7"/>
-    </row>
-    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B187" s="7"/>
-      <c r="C187" s="7"/>
-    </row>
-    <row r="188" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B188" s="7"/>
-      <c r="C188" s="7"/>
-    </row>
-    <row r="189" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B189" s="7"/>
-      <c r="C189" s="7"/>
-    </row>
-    <row r="190" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B190" s="7"/>
-      <c r="C190" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19069,7 +18966,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="36" type="noConversion"/>
+  <phoneticPr fontId="34" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
@@ -19099,10 +18996,10 @@
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
       <c r="J1" s="15"/>
-      <c r="K1" s="55" t="s">
+      <c r="K1" s="54" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="56"/>
+      <c r="L1" s="55"/>
     </row>
     <row r="2" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
@@ -20954,13 +20851,13 @@
       <c r="G53" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="H53" s="57" t="s">
+      <c r="H53" s="56" t="s">
         <v>165</v>
       </c>
-      <c r="I53" s="58"/>
-      <c r="J53" s="58"/>
-      <c r="K53" s="58"/>
-      <c r="L53" s="59"/>
+      <c r="I53" s="57"/>
+      <c r="J53" s="57"/>
+      <c r="K53" s="57"/>
+      <c r="L53" s="58"/>
     </row>
     <row r="54" spans="1:12" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
@@ -20982,11 +20879,11 @@
       <c r="G54" s="27">
         <v>31536</v>
       </c>
-      <c r="H54" s="60"/>
-      <c r="I54" s="61"/>
-      <c r="J54" s="61"/>
-      <c r="K54" s="61"/>
-      <c r="L54" s="62"/>
+      <c r="H54" s="59"/>
+      <c r="I54" s="60"/>
+      <c r="J54" s="60"/>
+      <c r="K54" s="60"/>
+      <c r="L54" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
lode runner - lv 47 done - 891 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E92759FC-C8B8-4F93-8822-C297C78A956B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE378083-F7AB-45B5-99C9-EB4F9B46FA20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50310" yWindow="3030" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3684,13 +3684,15 @@
       <c r="A94" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="B94" s="7"/>
+      <c r="B94" s="7">
+        <v>45555</v>
+      </c>
       <c r="C94" s="7">
         <v>46652</v>
       </c>
-      <c r="D94" s="3" t="str">
+      <c r="D94" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>1097</v>
       </c>
       <c r="E94" s="51" t="s">
         <v>422</v>
@@ -3700,26 +3702,30 @@
       <c r="A95" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="B95" s="7"/>
+      <c r="B95" s="7">
+        <v>46538</v>
+      </c>
       <c r="C95" s="7">
         <v>47436</v>
       </c>
-      <c r="D95" s="3" t="str">
+      <c r="D95" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>898</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="50" t="s">
         <v>23</v>
       </c>
-      <c r="B96" s="9"/>
+      <c r="B96" s="9">
+        <v>46895</v>
+      </c>
       <c r="C96" s="9">
-        <v>48337</v>
-      </c>
-      <c r="D96" s="3" t="str">
+        <v>47786</v>
+      </c>
+      <c r="D96" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>891</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -3728,7 +3734,7 @@
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7">
-        <v>49334</v>
+        <v>48337</v>
       </c>
       <c r="D97" s="3" t="str">
         <f t="shared" si="3"/>

</xml_diff>

<commit_message>
lode runner - lv 48 done - 894 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE378083-F7AB-45B5-99C9-EB4F9B46FA20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{144553E1-896E-48F8-A9E9-09730CF6CC3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50310" yWindow="3030" windowWidth="7500" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="42660" yWindow="3270" windowWidth="7500" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -3718,40 +3718,44 @@
         <v>23</v>
       </c>
       <c r="B96" s="9">
-        <v>46895</v>
+        <v>46894</v>
       </c>
       <c r="C96" s="9">
         <v>47786</v>
       </c>
       <c r="D96" s="3">
         <f t="shared" si="3"/>
-        <v>891</v>
+        <v>892</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="B97" s="7"/>
+      <c r="B97" s="7">
+        <v>47439</v>
+      </c>
       <c r="C97" s="7">
         <v>48337</v>
       </c>
-      <c r="D97" s="3" t="str">
+      <c r="D97" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>898</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="B98" s="7"/>
+      <c r="B98" s="7">
+        <v>47787</v>
+      </c>
       <c r="C98" s="7">
         <v>48681</v>
       </c>
-      <c r="D98" s="3" t="str">
+      <c r="D98" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>894</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - level 49 nominally done - 892 ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{144553E1-896E-48F8-A9E9-09730CF6CC3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB7235E7-2C04-4C7D-A761-61367CE4E216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42660" yWindow="3270" windowWidth="7500" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="50160" yWindow="4035" windowWidth="7500" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -3748,27 +3748,29 @@
         <v>24</v>
       </c>
       <c r="B98" s="7">
-        <v>47787</v>
+        <v>47790</v>
       </c>
       <c r="C98" s="7">
         <v>48681</v>
       </c>
       <c r="D98" s="3">
         <f t="shared" si="3"/>
-        <v>894</v>
+        <v>891</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="B99" s="7"/>
+      <c r="B99" s="7">
+        <v>48442</v>
+      </c>
       <c r="C99" s="7">
         <v>49334</v>
       </c>
-      <c r="D99" s="3" t="str">
+      <c r="D99" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>892</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - new lv 49 route, 20 frames faster
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB7235E7-2C04-4C7D-A761-61367CE4E216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8120D43-7F88-45F1-954F-D1BD05933556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50160" yWindow="4035" windowWidth="7500" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="50160" yWindow="3915" windowWidth="7500" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="425">
   <si>
     <t>Place</t>
   </si>
@@ -3728,7 +3728,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="50" t="s">
         <v>43</v>
       </c>
@@ -3743,7 +3743,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="50" t="s">
         <v>24</v>
       </c>
@@ -3758,22 +3758,28 @@
         <v>891</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="50" t="s">
         <v>44</v>
       </c>
       <c r="B99" s="7">
-        <v>48442</v>
+        <v>48423</v>
       </c>
       <c r="C99" s="7">
         <v>49334</v>
       </c>
       <c r="D99" s="3">
         <f t="shared" si="3"/>
-        <v>892</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+        <v>911</v>
+      </c>
+      <c r="E99" s="7">
+        <v>48442</v>
+      </c>
+      <c r="F99" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="50" t="s">
         <v>25</v>
       </c>
@@ -3786,7 +3792,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="50" t="s">
         <v>26</v>
       </c>
@@ -3799,47 +3805,47 @@
         <v>-</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B102" s="7"/>
       <c r="C102" s="7"/>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B103" s="7"/>
       <c r="C103" s="7"/>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B104" s="7"/>
       <c r="C104" s="7"/>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B105" s="7"/>
       <c r="C105" s="7"/>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B106" s="7"/>
       <c r="C106" s="7"/>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B107" s="7"/>
       <c r="C107" s="7"/>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B108" s="7"/>
       <c r="C108" s="7"/>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B112" s="7"/>
       <c r="C112" s="7"/>
     </row>

</xml_diff>

<commit_message>
lode runner - up to level 50 - 911 frames ahead
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8120D43-7F88-45F1-954F-D1BD05933556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC67AD2A-47D1-4340-A2DC-C7208AF747EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50160" yWindow="3915" windowWidth="7500" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3783,13 +3783,15 @@
       <c r="A100" s="50" t="s">
         <v>25</v>
       </c>
-      <c r="B100" s="7"/>
+      <c r="B100" s="7">
+        <v>48772</v>
+      </c>
       <c r="C100" s="7">
         <v>49683</v>
       </c>
-      <c r="D100" s="3" t="str">
+      <c r="D100" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>911</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lode runner - v7 nominally done, 924 frames ahead of v6, still looking at level 50 for possible improvements
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC67AD2A-47D1-4340-A2DC-C7208AF747EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C90F2F-467A-4E3B-8638-9F5761072FA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="50160" yWindow="3915" windowWidth="7500" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="427">
   <si>
     <t>Place</t>
   </si>
@@ -1311,6 +1311,12 @@
   </si>
   <si>
     <t>39656 possible, 6 frames to get exact gold drop</t>
+  </si>
+  <si>
+    <t>1st move</t>
+  </si>
+  <si>
+    <t>grab ladder</t>
   </si>
 </sst>
 </file>
@@ -3798,13 +3804,15 @@
       <c r="A101" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="B101" s="7"/>
+      <c r="B101" s="7">
+        <v>49320</v>
+      </c>
       <c r="C101" s="7">
         <v>50244</v>
       </c>
-      <c r="D101" s="3" t="str">
+      <c r="D101" s="3">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>924</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -3820,24 +3828,71 @@
       <c r="C104" s="7"/>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>387</v>
+      </c>
       <c r="B105" s="7"/>
       <c r="C105" s="7"/>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B106" s="7"/>
-      <c r="C106" s="7"/>
+      <c r="A106" t="s">
+        <v>425</v>
+      </c>
+      <c r="B106" s="7">
+        <v>48774</v>
+      </c>
+      <c r="C106" s="7">
+        <v>63244</v>
+      </c>
+      <c r="D106" s="3">
+        <f t="shared" ref="D106:D109" si="4">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
+        <v>14470</v>
+      </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B107" s="7"/>
-      <c r="C107" s="7"/>
+      <c r="A107" t="s">
+        <v>426</v>
+      </c>
+      <c r="B107" s="7">
+        <v>48863</v>
+      </c>
+      <c r="C107" s="7">
+        <v>63333</v>
+      </c>
+      <c r="D107" s="3">
+        <f t="shared" si="4"/>
+        <v>14470</v>
+      </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B108" s="7"/>
-      <c r="C108" s="7"/>
+      <c r="A108" t="s">
+        <v>426</v>
+      </c>
+      <c r="B108" s="7">
+        <v>48913</v>
+      </c>
+      <c r="C108" s="7">
+        <v>63383</v>
+      </c>
+      <c r="D108" s="3">
+        <f t="shared" si="4"/>
+        <v>14470</v>
+      </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B109" s="7"/>
-      <c r="C109" s="7"/>
+      <c r="A109" t="s">
+        <v>371</v>
+      </c>
+      <c r="B109" s="7">
+        <v>49320</v>
+      </c>
+      <c r="C109" s="7">
+        <v>63782</v>
+      </c>
+      <c r="D109" s="3">
+        <f t="shared" si="4"/>
+        <v>14462</v>
+      </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B110" s="7"/>
@@ -8646,79 +8701,115 @@
       <c r="B304" s="7"/>
       <c r="C304" s="7"/>
     </row>
-    <row r="305" spans="2:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B305" s="7">
-        <v>1381</v>
-      </c>
-      <c r="C305" s="7">
-        <v>1058</v>
-      </c>
-      <c r="D305">
-        <f>B305-C305</f>
-        <v>323</v>
-      </c>
+    <row r="305" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A305" t="s">
+        <v>387</v>
+      </c>
+      <c r="B305" s="7"/>
+      <c r="C305" s="7"/>
       <c r="E305">
         <f>D305*50</f>
-        <v>16150</v>
-      </c>
-    </row>
-    <row r="306" spans="2:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B306" s="7"/>
-      <c r="C306" s="7"/>
-    </row>
-    <row r="307" spans="2:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B307" s="7"/>
-      <c r="C307" s="7"/>
-    </row>
-    <row r="308" spans="2:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B308" s="7"/>
-      <c r="C308" s="7"/>
-    </row>
-    <row r="309" spans="2:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="B309" s="7"/>
-      <c r="C309" s="7"/>
-    </row>
-    <row r="310" spans="2:5" ht="15" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="306" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A306" t="s">
+        <v>425</v>
+      </c>
+      <c r="B306" s="7">
+        <v>48774</v>
+      </c>
+      <c r="C306" s="7">
+        <v>63244</v>
+      </c>
+      <c r="D306" s="3">
+        <f t="shared" ref="D306:D309" si="8">IF(C306&lt;&gt;"",IF(B306&lt;&gt;"",C306-B306,"-"), "-")</f>
+        <v>14470</v>
+      </c>
+    </row>
+    <row r="307" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A307" t="s">
+        <v>426</v>
+      </c>
+      <c r="B307" s="7">
+        <v>48863</v>
+      </c>
+      <c r="C307" s="7">
+        <v>63333</v>
+      </c>
+      <c r="D307" s="3">
+        <f t="shared" si="8"/>
+        <v>14470</v>
+      </c>
+    </row>
+    <row r="308" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A308" t="s">
+        <v>426</v>
+      </c>
+      <c r="B308" s="7">
+        <v>48913</v>
+      </c>
+      <c r="C308" s="7">
+        <v>63383</v>
+      </c>
+      <c r="D308" s="3">
+        <f t="shared" si="8"/>
+        <v>14470</v>
+      </c>
+    </row>
+    <row r="309" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="B309" s="7">
+        <v>49338</v>
+      </c>
+      <c r="C309" s="7">
+        <v>63782</v>
+      </c>
+      <c r="D309" s="3">
+        <f t="shared" si="8"/>
+        <v>14444</v>
+      </c>
+    </row>
+    <row r="310" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B310" s="7"/>
       <c r="C310" s="7"/>
     </row>
-    <row r="311" spans="2:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B311" s="7"/>
       <c r="C311" s="7"/>
     </row>
-    <row r="312" spans="2:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B312" s="7"/>
       <c r="C312" s="7"/>
     </row>
-    <row r="313" spans="2:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B313" s="7"/>
       <c r="C313" s="7"/>
     </row>
-    <row r="314" spans="2:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B314" s="7"/>
       <c r="C314" s="7"/>
     </row>
-    <row r="315" spans="2:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B315" s="7"/>
       <c r="C315" s="7"/>
     </row>
-    <row r="316" spans="2:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B316" s="7"/>
       <c r="C316" s="7"/>
     </row>
-    <row r="317" spans="2:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B317" s="7"/>
       <c r="C317" s="7"/>
     </row>
-    <row r="318" spans="2:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B318" s="7"/>
       <c r="C318" s="7"/>
     </row>
-    <row r="319" spans="2:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B319" s="7"/>
       <c r="C319" s="7"/>
     </row>
-    <row r="320" spans="2:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B320" s="7"/>
       <c r="C320" s="7"/>
     </row>

</xml_diff>

<commit_message>
lode runner - improved route on level 50 - 940 frames ahead of v6, 14478 head of v5 (the publsihed movie)
</commit_message>
<xml_diff>
--- a/LodeRunner/compare.xlsx
+++ b/LodeRunner/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\LodeRunner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0221E489-9B8E-4C85-B63F-DB87741B1152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF8E6A29-4E82-4EEC-BFCB-C57EBFD9CFDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50160" yWindow="3915" windowWidth="7500" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="50415" yWindow="3555" windowWidth="7500" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V7" sheetId="8" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="427">
   <si>
     <t>Place</t>
   </si>
@@ -2252,7 +2252,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7C7DF3-1A35-402E-AA40-93AF033BF7A2}">
-  <dimension ref="A1:F184"/>
+  <dimension ref="A1:F185"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -3805,14 +3805,14 @@
         <v>26</v>
       </c>
       <c r="B101" s="7">
-        <v>49320</v>
+        <v>49304</v>
       </c>
       <c r="C101" s="7">
         <v>50244</v>
       </c>
       <c r="D101" s="3">
         <f t="shared" si="3"/>
-        <v>924</v>
+        <v>940</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -3845,7 +3845,7 @@
         <v>63244</v>
       </c>
       <c r="D106" s="3">
-        <f t="shared" ref="D106:D109" si="4">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
+        <f t="shared" ref="D106:D110" si="4">IF(C106&lt;&gt;"",IF(B106&lt;&gt;"",C106-B106,"-"), "-")</f>
         <v>14468</v>
       </c>
     </row>
@@ -3881,22 +3881,33 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>371</v>
+        <v>426</v>
       </c>
       <c r="B109" s="7">
-        <v>49320</v>
+        <v>49169</v>
       </c>
       <c r="C109" s="7">
-        <v>63782</v>
+        <v>63638</v>
       </c>
       <c r="D109" s="3">
         <f t="shared" si="4"/>
-        <v>14462</v>
+        <v>14469</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B110" s="7"/>
-      <c r="C110" s="7"/>
+      <c r="A110" t="s">
+        <v>371</v>
+      </c>
+      <c r="B110" s="7">
+        <v>49304</v>
+      </c>
+      <c r="C110" s="7">
+        <v>63782</v>
+      </c>
+      <c r="D110" s="3">
+        <f t="shared" si="4"/>
+        <v>14478</v>
+      </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
@@ -4193,6 +4204,10 @@
     <row r="184" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B184" s="7"/>
       <c r="C184" s="7"/>
+    </row>
+    <row r="185" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B185" s="7"/>
+      <c r="C185" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>